<commit_message>
Scan 07.03.2026 22:35 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V28"/>
+  <dimension ref="A1:V27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -444,12 +444,12 @@
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="6" customWidth="1" min="10" max="10"/>
     <col width="6" customWidth="1" min="11" max="11"/>
-    <col width="6" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
     <col width="9" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
@@ -577,11 +577,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ACN</t>
+          <t>META</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>315.81</v>
+        <v>324.74</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,22 +614,22 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>85.90000000000001</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="J2" t="n">
-        <v>61.2</v>
+        <v>63.4</v>
       </c>
       <c r="K2" t="n">
-        <v>98.8</v>
+        <v>97.7</v>
       </c>
       <c r="L2" t="n">
-        <v>6.92</v>
+        <v>10.37</v>
       </c>
       <c r="M2" t="n">
-        <v>78.59999999999999</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="N2" t="n">
-        <v>52.6</v>
+        <v>87.8</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>51.8</v>
+        <v>58.1</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -673,11 +673,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>ITW</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>315.81</v>
+        <v>324.74</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -710,30 +710,30 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>85.90000000000001</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="J3" t="n">
-        <v>61.2</v>
+        <v>63.4</v>
       </c>
       <c r="K3" t="n">
-        <v>98.8</v>
+        <v>97.7</v>
       </c>
       <c r="L3" t="n">
-        <v>6.92</v>
+        <v>10.37</v>
       </c>
       <c r="M3" t="n">
-        <v>78.59999999999999</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="N3" t="n">
-        <v>52.6</v>
+        <v>87.8</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P3" t="n">
-        <v>34</v>
+        <v>58.1</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -769,11 +769,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ANSS</t>
+          <t>MMM</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>315.81</v>
+        <v>324.74</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -806,30 +806,30 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>85.90000000000001</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="J4" t="n">
-        <v>61.2</v>
+        <v>63.4</v>
       </c>
       <c r="K4" t="n">
-        <v>98.8</v>
+        <v>97.7</v>
       </c>
       <c r="L4" t="n">
-        <v>6.92</v>
+        <v>10.37</v>
       </c>
       <c r="M4" t="n">
-        <v>78.59999999999999</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="N4" t="n">
+        <v>87.8</v>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="P4" t="n">
         <v>52.6</v>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P4" t="n">
-        <v>51.8</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -865,11 +865,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>KHC</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>315.81</v>
+        <v>324.74</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -902,22 +902,22 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>85.90000000000001</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="J5" t="n">
-        <v>61.2</v>
+        <v>63.4</v>
       </c>
       <c r="K5" t="n">
-        <v>98.8</v>
+        <v>97.7</v>
       </c>
       <c r="L5" t="n">
-        <v>6.92</v>
+        <v>10.37</v>
       </c>
       <c r="M5" t="n">
-        <v>78.59999999999999</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="N5" t="n">
-        <v>52.6</v>
+        <v>87.8</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -925,7 +925,7 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>51.8</v>
+        <v>58.1</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -961,11 +961,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>APD</t>
+          <t>MCO</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>315.81</v>
+        <v>324.74</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -998,30 +998,30 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>85.90000000000001</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="J6" t="n">
-        <v>61.2</v>
+        <v>63.4</v>
       </c>
       <c r="K6" t="n">
-        <v>98.8</v>
+        <v>97.7</v>
       </c>
       <c r="L6" t="n">
-        <v>6.92</v>
+        <v>10.37</v>
       </c>
       <c r="M6" t="n">
-        <v>78.59999999999999</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="N6" t="n">
-        <v>52.6</v>
+        <v>87.8</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P6" t="n">
-        <v>34</v>
+        <v>58.1</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1057,30 +1057,30 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ABT</t>
+          <t>ADP</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>215</v>
+        <v>315.81</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1094,30 +1094,30 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>75.8</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="J7" t="n">
-        <v>42.2</v>
+        <v>61.2</v>
       </c>
       <c r="K7" t="n">
-        <v>81</v>
+        <v>98.8</v>
       </c>
       <c r="L7" t="n">
-        <v>4.18</v>
+        <v>6.92</v>
       </c>
       <c r="M7" t="n">
-        <v>51.5</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="N7" t="n">
-        <v>90.40000000000001</v>
+        <v>52.6</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>37</v>
+        <v>50.5</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1126,12 +1126,12 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
@@ -1139,40 +1139,44 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr"/>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ADI</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>215</v>
+        <v>315.81</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1186,22 +1190,22 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>75.8</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="J8" t="n">
-        <v>42.2</v>
+        <v>61.2</v>
       </c>
       <c r="K8" t="n">
-        <v>81</v>
+        <v>98.8</v>
       </c>
       <c r="L8" t="n">
-        <v>4.18</v>
+        <v>6.92</v>
       </c>
       <c r="M8" t="n">
-        <v>51.5</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="N8" t="n">
-        <v>90.40000000000001</v>
+        <v>52.6</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1209,7 +1213,7 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>61.2</v>
+        <v>50.5</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1218,12 +1222,12 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
@@ -1231,40 +1235,44 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U8" t="inlineStr"/>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ADBE</t>
+          <t>APH</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>215</v>
+        <v>315.81</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1278,19 +1286,19 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>75.8</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="J9" t="n">
-        <v>42.2</v>
+        <v>61.2</v>
       </c>
       <c r="K9" t="n">
-        <v>81</v>
+        <v>98.8</v>
       </c>
       <c r="L9" t="n">
-        <v>4.18</v>
+        <v>6.92</v>
       </c>
       <c r="M9" t="n">
-        <v>52.3</v>
+        <v>54.5</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1298,7 +1306,7 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>51.8</v>
+        <v>50.5</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1307,12 +1315,12 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
@@ -1320,21 +1328,25 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U9" t="inlineStr"/>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CEG</t>
+          <t>UPS</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>131.87</v>
+        <v>120.79</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1367,22 +1379,22 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>75.7</v>
+        <v>85.09999999999999</v>
       </c>
       <c r="J10" t="n">
-        <v>64.59999999999999</v>
+        <v>70.5</v>
       </c>
       <c r="K10" t="n">
-        <v>85</v>
+        <v>87.2</v>
       </c>
       <c r="L10" t="n">
-        <v>2.01</v>
+        <v>6.58</v>
       </c>
       <c r="M10" t="n">
-        <v>19</v>
+        <v>56.7</v>
       </c>
       <c r="N10" t="n">
-        <v>47.2</v>
+        <v>21.9</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1390,7 +1402,7 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>41.9</v>
+        <v>46.6</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1399,17 +1411,17 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U10" t="inlineStr"/>
@@ -1422,30 +1434,30 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>ADBE</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>131.87</v>
+        <v>215</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1459,30 +1471,30 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>75.7</v>
+        <v>75.8</v>
       </c>
       <c r="J11" t="n">
-        <v>64.59999999999999</v>
+        <v>42.2</v>
       </c>
       <c r="K11" t="n">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="L11" t="n">
-        <v>2.01</v>
+        <v>4.18</v>
       </c>
       <c r="M11" t="n">
-        <v>19</v>
+        <v>51.5</v>
       </c>
       <c r="N11" t="n">
-        <v>47.2</v>
+        <v>90.40000000000001</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>40.3</v>
+        <v>37</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1491,12 +1503,12 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
@@ -1514,30 +1526,30 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CAT</t>
+          <t>AEP</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>131.87</v>
+        <v>215</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1551,19 +1563,22 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>75.7</v>
+        <v>75.8</v>
       </c>
       <c r="J12" t="n">
-        <v>64.59999999999999</v>
+        <v>42.2</v>
       </c>
       <c r="K12" t="n">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="L12" t="n">
-        <v>2.01</v>
+        <v>4.18</v>
       </c>
       <c r="M12" t="n">
-        <v>48</v>
+        <v>51.5</v>
+      </c>
+      <c r="N12" t="n">
+        <v>90.40000000000001</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1571,7 +1586,7 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>41.9</v>
+        <v>53.3</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1580,12 +1595,12 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
@@ -1603,11 +1618,11 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>GOOG</t>
+          <t>AMGN</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>226.24</v>
+        <v>215</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -1640,30 +1655,30 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>67.5</v>
+        <v>75.8</v>
       </c>
       <c r="J13" t="n">
-        <v>34</v>
+        <v>42.2</v>
       </c>
       <c r="K13" t="n">
-        <v>98.8</v>
+        <v>81</v>
       </c>
       <c r="L13" t="n">
-        <v>6.11</v>
+        <v>4.18</v>
       </c>
       <c r="M13" t="n">
-        <v>48.3</v>
+        <v>51.5</v>
       </c>
       <c r="N13" t="n">
-        <v>100</v>
+        <v>90.40000000000001</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>57.1</v>
+        <v>37</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1695,11 +1710,11 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>INTC</t>
+          <t>ABT</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>226.24</v>
+        <v>215</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -1732,30 +1747,30 @@
         </is>
       </c>
       <c r="I14" t="n">
-        <v>67.5</v>
+        <v>75.8</v>
       </c>
       <c r="J14" t="n">
-        <v>34</v>
+        <v>42.2</v>
       </c>
       <c r="K14" t="n">
-        <v>98.8</v>
+        <v>81</v>
       </c>
       <c r="L14" t="n">
-        <v>6.11</v>
+        <v>4.18</v>
       </c>
       <c r="M14" t="n">
-        <v>48.3</v>
+        <v>51.5</v>
       </c>
       <c r="N14" t="n">
-        <v>100</v>
+        <v>90.40000000000001</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P14" t="n">
-        <v>44</v>
+        <v>40.9</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1787,30 +1802,30 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>HD</t>
+          <t>AZN</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>226.24</v>
+        <v>1292.8</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1824,22 +1839,22 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>67.5</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="J15" t="n">
-        <v>34</v>
+        <v>60</v>
       </c>
       <c r="K15" t="n">
-        <v>98.8</v>
+        <v>89.5</v>
       </c>
       <c r="L15" t="n">
-        <v>6.11</v>
+        <v>8.19</v>
       </c>
       <c r="M15" t="n">
-        <v>48.3</v>
+        <v>89</v>
       </c>
       <c r="N15" t="n">
-        <v>100</v>
+        <v>58.8</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1847,7 +1862,7 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>43.7</v>
+        <v>29.9</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1856,12 +1871,12 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
@@ -1869,40 +1884,44 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U15" t="inlineStr"/>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ICE</t>
+          <t>XLP</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>226.24</v>
+        <v>60.29</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1916,27 +1935,27 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>67.5</v>
+        <v>72.7</v>
       </c>
       <c r="J16" t="n">
-        <v>34</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="K16" t="n">
-        <v>98.8</v>
+        <v>96.5</v>
       </c>
       <c r="L16" t="n">
-        <v>6.11</v>
+        <v>4.79</v>
       </c>
       <c r="M16" t="n">
-        <v>28.3</v>
+        <v>50.7</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>43.7</v>
+        <v>50</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1950,48 +1969,52 @@
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U16" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>GILD</t>
+          <t>WDAY</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>226.24</v>
+        <v>60.29</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -2005,19 +2028,19 @@
         </is>
       </c>
       <c r="I17" t="n">
-        <v>67.5</v>
+        <v>72.7</v>
       </c>
       <c r="J17" t="n">
-        <v>34</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="K17" t="n">
-        <v>98.8</v>
+        <v>96.5</v>
       </c>
       <c r="L17" t="n">
-        <v>6.11</v>
+        <v>4.79</v>
       </c>
       <c r="M17" t="n">
-        <v>32.5</v>
+        <v>52.8</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -2025,7 +2048,7 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>57.1</v>
+        <v>50</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -2039,29 +2062,33 @@
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U17" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>VRSK</t>
+          <t>ICE</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>317.1</v>
+        <v>484.74</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -2090,31 +2117,34 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>65.8</v>
+        <v>71.3</v>
       </c>
       <c r="J18" t="n">
-        <v>61.3</v>
+        <v>52.2</v>
       </c>
       <c r="K18" t="n">
-        <v>75</v>
+        <v>93</v>
       </c>
       <c r="L18" t="n">
-        <v>2.16</v>
+        <v>2.18</v>
       </c>
       <c r="M18" t="n">
-        <v>45.5</v>
+        <v>21.1</v>
+      </c>
+      <c r="N18" t="n">
+        <v>38.7</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P18" t="n">
-        <v>47.4</v>
+        <v>47.5</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -2146,11 +2176,11 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>TLT</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>317.1</v>
+        <v>484.74</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -2179,31 +2209,34 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>65.8</v>
+        <v>71.3</v>
       </c>
       <c r="J19" t="n">
-        <v>61.3</v>
+        <v>52.2</v>
       </c>
       <c r="K19" t="n">
-        <v>75</v>
+        <v>93</v>
       </c>
       <c r="L19" t="n">
-        <v>2.16</v>
+        <v>2.18</v>
       </c>
       <c r="M19" t="n">
-        <v>12.3</v>
+        <v>21.1</v>
+      </c>
+      <c r="N19" t="n">
+        <v>38.7</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P19" t="n">
-        <v>47.4</v>
+        <v>63.4</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -2235,11 +2268,11 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ZS</t>
+          <t>MCD</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>317.1</v>
+        <v>484.74</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -2268,31 +2301,34 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I20" t="n">
-        <v>65.8</v>
+        <v>71.3</v>
       </c>
       <c r="J20" t="n">
-        <v>61.3</v>
+        <v>52.2</v>
       </c>
       <c r="K20" t="n">
-        <v>75</v>
+        <v>93</v>
       </c>
       <c r="L20" t="n">
-        <v>2.16</v>
+        <v>2.18</v>
       </c>
       <c r="M20" t="n">
-        <v>59.1</v>
+        <v>21.1</v>
+      </c>
+      <c r="N20" t="n">
+        <v>38.7</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P20" t="n">
-        <v>47.4</v>
+        <v>47.5</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
@@ -2324,11 +2360,11 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>GLD</t>
+          <t>LRCX</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>317.1</v>
+        <v>484.74</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -2357,31 +2393,31 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>65.8</v>
+        <v>71.3</v>
       </c>
       <c r="J21" t="n">
-        <v>61.3</v>
+        <v>52.2</v>
       </c>
       <c r="K21" t="n">
+        <v>93</v>
+      </c>
+      <c r="L21" t="n">
+        <v>2.18</v>
+      </c>
+      <c r="M21" t="n">
         <v>75</v>
       </c>
-      <c r="L21" t="n">
-        <v>2.16</v>
-      </c>
-      <c r="M21" t="n">
-        <v>32.5</v>
-      </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P21" t="n">
-        <v>47.4</v>
+        <v>47.5</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
@@ -2413,30 +2449,30 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>MNST</t>
+          <t>JPM</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>66.26000000000001</v>
+        <v>484.74</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -2450,27 +2486,30 @@
         </is>
       </c>
       <c r="I22" t="n">
-        <v>59.3</v>
+        <v>71.3</v>
       </c>
       <c r="J22" t="n">
-        <v>37.4</v>
+        <v>52.2</v>
       </c>
       <c r="K22" t="n">
-        <v>95.3</v>
+        <v>93</v>
       </c>
       <c r="L22" t="n">
-        <v>8.210000000000001</v>
+        <v>2.18</v>
       </c>
       <c r="M22" t="n">
-        <v>28.2</v>
+        <v>21.1</v>
+      </c>
+      <c r="N22" t="n">
+        <v>38.7</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P22" t="n">
-        <v>56</v>
+        <v>47.5</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
@@ -2484,12 +2523,12 @@
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U22" t="inlineStr"/>
@@ -2502,30 +2541,30 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>KDP</t>
+          <t>INTU</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>66.26000000000001</v>
+        <v>484.74</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2539,19 +2578,22 @@
         </is>
       </c>
       <c r="I23" t="n">
-        <v>59.3</v>
+        <v>71.3</v>
       </c>
       <c r="J23" t="n">
-        <v>37.4</v>
+        <v>52.2</v>
       </c>
       <c r="K23" t="n">
-        <v>95.3</v>
+        <v>93</v>
       </c>
       <c r="L23" t="n">
-        <v>8.210000000000001</v>
+        <v>2.18</v>
       </c>
       <c r="M23" t="n">
-        <v>30.2</v>
+        <v>21.1</v>
+      </c>
+      <c r="N23" t="n">
+        <v>38.7</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -2559,7 +2601,7 @@
         </is>
       </c>
       <c r="P23" t="n">
-        <v>61.3</v>
+        <v>63.4</v>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
@@ -2573,12 +2615,12 @@
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U23" t="inlineStr"/>
@@ -2591,59 +2633,56 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>FDX</t>
+          <t>KLAC</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>33.28</v>
+        <v>484.74</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I24" t="n">
-        <v>49.2</v>
+        <v>71.3</v>
       </c>
       <c r="J24" t="n">
-        <v>64.8</v>
+        <v>52.2</v>
       </c>
       <c r="K24" t="n">
-        <v>30</v>
+        <v>93</v>
       </c>
       <c r="L24" t="n">
-        <v>4.89</v>
+        <v>2.18</v>
       </c>
       <c r="M24" t="n">
-        <v>49.1</v>
-      </c>
-      <c r="N24" t="n">
-        <v>38.3</v>
+        <v>59.8</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
@@ -2651,7 +2690,7 @@
         </is>
       </c>
       <c r="P24" t="n">
-        <v>50.9</v>
+        <v>47.5</v>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
@@ -2660,17 +2699,17 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U24" t="inlineStr"/>
@@ -2683,35 +2722,35 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>FCX</t>
+          <t>SO</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>33.28</v>
+        <v>923.72</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -2720,30 +2759,30 @@
         </is>
       </c>
       <c r="I25" t="n">
-        <v>49.2</v>
+        <v>68.2</v>
       </c>
       <c r="J25" t="n">
-        <v>64.8</v>
+        <v>57.9</v>
       </c>
       <c r="K25" t="n">
-        <v>30</v>
+        <v>69.8</v>
       </c>
       <c r="L25" t="n">
-        <v>4.89</v>
+        <v>5.09</v>
       </c>
       <c r="M25" t="n">
-        <v>49.1</v>
+        <v>50</v>
       </c>
       <c r="N25" t="n">
-        <v>38.3</v>
+        <v>23.8</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P25" t="n">
-        <v>50.9</v>
+        <v>26.4</v>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
@@ -2752,17 +2791,17 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U25" t="inlineStr"/>
@@ -2775,35 +2814,35 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>SYK</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>33.28</v>
+        <v>923.72</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D26" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -2812,22 +2851,22 @@
         </is>
       </c>
       <c r="I26" t="n">
-        <v>49.2</v>
+        <v>68.2</v>
       </c>
       <c r="J26" t="n">
-        <v>64.8</v>
+        <v>57.9</v>
       </c>
       <c r="K26" t="n">
-        <v>30</v>
+        <v>69.8</v>
       </c>
       <c r="L26" t="n">
-        <v>4.89</v>
+        <v>5.09</v>
       </c>
       <c r="M26" t="n">
-        <v>49.1</v>
+        <v>50</v>
       </c>
       <c r="N26" t="n">
-        <v>38.3</v>
+        <v>23.8</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
@@ -2835,7 +2874,7 @@
         </is>
       </c>
       <c r="P26" t="n">
-        <v>34</v>
+        <v>26.4</v>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
@@ -2844,17 +2883,17 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U26" t="inlineStr"/>
@@ -2867,15 +2906,15 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>GD</t>
+          <t>PH</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>33.28</v>
+        <v>226.24</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -2890,36 +2929,36 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I27" t="n">
-        <v>49.2</v>
+        <v>67.5</v>
       </c>
       <c r="J27" t="n">
-        <v>64.8</v>
+        <v>34</v>
       </c>
       <c r="K27" t="n">
-        <v>30</v>
+        <v>98.8</v>
       </c>
       <c r="L27" t="n">
-        <v>4.89</v>
+        <v>6.11</v>
       </c>
       <c r="M27" t="n">
-        <v>49.1</v>
+        <v>48.3</v>
       </c>
       <c r="N27" t="n">
-        <v>38.3</v>
+        <v>100</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -2927,7 +2966,7 @@
         </is>
       </c>
       <c r="P27" t="n">
-        <v>34</v>
+        <v>45.2</v>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
@@ -2941,108 +2980,16 @@
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U27" t="inlineStr"/>
       <c r="V27" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>FICO</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
-        <v>33.28</v>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D28" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>Debit Call</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>30-60 DTE</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I28" t="n">
-        <v>49.2</v>
-      </c>
-      <c r="J28" t="n">
-        <v>64.8</v>
-      </c>
-      <c r="K28" t="n">
-        <v>30</v>
-      </c>
-      <c r="L28" t="n">
-        <v>4.89</v>
-      </c>
-      <c r="M28" t="n">
-        <v>49.1</v>
-      </c>
-      <c r="N28" t="n">
-        <v>38.3</v>
-      </c>
-      <c r="O28" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P28" t="n">
-        <v>43.7</v>
-      </c>
-      <c r="Q28" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R28" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="S28" t="inlineStr">
-        <is>
-          <t>lime</t>
-        </is>
-      </c>
-      <c r="T28" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U28" t="inlineStr"/>
-      <c r="V28" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Scan 07.03.2026 22:51 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V13"/>
+  <dimension ref="A1:V21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -448,8 +448,8 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="6" customWidth="1" min="10" max="10"/>
-    <col width="7" customWidth="1" min="11" max="11"/>
-    <col width="7" customWidth="1" min="12" max="12"/>
+    <col width="6" customWidth="1" min="11" max="11"/>
+    <col width="6" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
     <col width="9" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
@@ -577,11 +577,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>EW</t>
+          <t>PH</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>33.28</v>
+        <v>369.53</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,30 +614,30 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>90.40000000000001</v>
+        <v>87.2</v>
       </c>
       <c r="J2" t="n">
-        <v>67.7</v>
+        <v>62.3</v>
       </c>
       <c r="K2" t="n">
-        <v>100</v>
+        <v>90.7</v>
       </c>
       <c r="L2" t="n">
-        <v>9.48</v>
+        <v>5.65</v>
       </c>
       <c r="M2" t="n">
-        <v>100.9</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="N2" t="n">
-        <v>82.09999999999999</v>
+        <v>81.7</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>74.3</v>
+        <v>45.2</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -659,21 +659,25 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr"/>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>EQR</t>
+          <t>PFE</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>33.28</v>
+        <v>369.53</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -706,30 +710,30 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>90.40000000000001</v>
+        <v>87.2</v>
       </c>
       <c r="J3" t="n">
-        <v>67.7</v>
+        <v>62.3</v>
       </c>
       <c r="K3" t="n">
-        <v>100</v>
+        <v>90.7</v>
       </c>
       <c r="L3" t="n">
-        <v>9.48</v>
+        <v>5.65</v>
       </c>
       <c r="M3" t="n">
-        <v>100.9</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="N3" t="n">
-        <v>82.09999999999999</v>
+        <v>81.7</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P3" t="n">
-        <v>74.3</v>
+        <v>45.2</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -751,21 +755,25 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr"/>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>EMR</t>
+          <t>HUM</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>33.28</v>
+        <v>315.81</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -798,27 +806,27 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>90.40000000000001</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="J4" t="n">
-        <v>67.7</v>
+        <v>61.2</v>
       </c>
       <c r="K4" t="n">
-        <v>100</v>
+        <v>98.8</v>
       </c>
       <c r="L4" t="n">
-        <v>9.48</v>
+        <v>6.92</v>
       </c>
       <c r="M4" t="n">
-        <v>39.9</v>
+        <v>78.59999999999999</v>
+      </c>
+      <c r="N4" t="n">
+        <v>52.6</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P4" t="n">
-        <v>74.3</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -827,34 +835,38 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BDX</t>
+          <t>INTU</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>369.53</v>
+        <v>315.81</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -887,30 +899,27 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>87.2</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="J5" t="n">
-        <v>62.3</v>
+        <v>61.2</v>
       </c>
       <c r="K5" t="n">
-        <v>90.7</v>
+        <v>98.8</v>
       </c>
       <c r="L5" t="n">
-        <v>5.65</v>
+        <v>6.92</v>
       </c>
       <c r="M5" t="n">
-        <v>65.90000000000001</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="N5" t="n">
-        <v>81.7</v>
+        <v>52.6</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P5" t="n">
-        <v>41.9</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -919,17 +928,17 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -946,11 +955,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ANET</t>
+          <t>HON</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>324.74</v>
+        <v>315.81</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -983,30 +992,27 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>86.09999999999999</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="J6" t="n">
-        <v>63.4</v>
+        <v>61.2</v>
       </c>
       <c r="K6" t="n">
-        <v>97.7</v>
+        <v>98.8</v>
       </c>
       <c r="L6" t="n">
-        <v>10.37</v>
+        <v>6.92</v>
       </c>
       <c r="M6" t="n">
-        <v>99.09999999999999</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="N6" t="n">
-        <v>87.8</v>
+        <v>52.6</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P6" t="n">
-        <v>51.8</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1042,11 +1048,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ADI</t>
+          <t>ISRG</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>324.74</v>
+        <v>315.81</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1079,27 +1085,27 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>86.09999999999999</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="J7" t="n">
-        <v>63.4</v>
+        <v>61.2</v>
       </c>
       <c r="K7" t="n">
-        <v>97.7</v>
+        <v>98.8</v>
       </c>
       <c r="L7" t="n">
-        <v>10.37</v>
+        <v>6.92</v>
       </c>
       <c r="M7" t="n">
-        <v>43.3</v>
+        <v>78.59999999999999</v>
+      </c>
+      <c r="N7" t="n">
+        <v>52.6</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P7" t="n">
-        <v>51.8</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1135,11 +1141,11 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>BA</t>
+          <t>INTC</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>324.74</v>
+        <v>315.81</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1172,30 +1178,27 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>86.09999999999999</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="J8" t="n">
-        <v>63.4</v>
+        <v>61.2</v>
       </c>
       <c r="K8" t="n">
-        <v>97.7</v>
+        <v>98.8</v>
       </c>
       <c r="L8" t="n">
-        <v>10.37</v>
+        <v>6.92</v>
       </c>
       <c r="M8" t="n">
-        <v>99.09999999999999</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="N8" t="n">
-        <v>87.8</v>
+        <v>52.6</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P8" t="n">
-        <v>41.9</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1231,7 +1234,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>TSLA</t>
+          <t>HSY</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -1287,11 +1290,8 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P9" t="n">
-        <v>57.8</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1327,30 +1327,30 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>HD</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>215</v>
+        <v>315.81</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1364,22 +1364,19 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>75.8</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="J10" t="n">
-        <v>42.2</v>
+        <v>61.2</v>
       </c>
       <c r="K10" t="n">
-        <v>81</v>
+        <v>98.8</v>
       </c>
       <c r="L10" t="n">
-        <v>4.18</v>
+        <v>6.92</v>
       </c>
       <c r="M10" t="n">
-        <v>51.5</v>
-      </c>
-      <c r="N10" t="n">
-        <v>90.40000000000001</v>
+        <v>30.7</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1387,7 +1384,7 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>37</v>
+        <v>43.6</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1396,12 +1393,12 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -1409,40 +1406,44 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U10" t="inlineStr"/>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>ITW</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>215</v>
+        <v>315.81</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1456,30 +1457,27 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>75.8</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="J11" t="n">
-        <v>42.2</v>
+        <v>61.2</v>
       </c>
       <c r="K11" t="n">
-        <v>81</v>
+        <v>98.8</v>
       </c>
       <c r="L11" t="n">
-        <v>4.18</v>
+        <v>6.92</v>
       </c>
       <c r="M11" t="n">
-        <v>51.5</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="N11" t="n">
-        <v>90.40000000000001</v>
+        <v>52.6</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P11" t="n">
-        <v>37</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1488,12 +1486,12 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
@@ -1501,21 +1499,25 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U11" t="inlineStr"/>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>ICE</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>131.87</v>
+        <v>315.81</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1548,30 +1550,27 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>75.7</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="J12" t="n">
-        <v>64.59999999999999</v>
+        <v>61.2</v>
       </c>
       <c r="K12" t="n">
-        <v>85</v>
+        <v>98.8</v>
       </c>
       <c r="L12" t="n">
-        <v>2.01</v>
+        <v>6.92</v>
       </c>
       <c r="M12" t="n">
-        <v>19</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="N12" t="n">
-        <v>47.2</v>
+        <v>52.6</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P12" t="n">
-        <v>47.5</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1593,40 +1592,44 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U12" t="inlineStr"/>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ABNB</t>
+          <t>JPM</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>226.24</v>
+        <v>315.81</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1640,53 +1643,789 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>67.5</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="J13" t="n">
-        <v>34</v>
+        <v>61.2</v>
       </c>
       <c r="K13" t="n">
         <v>98.8</v>
       </c>
       <c r="L13" t="n">
+        <v>6.92</v>
+      </c>
+      <c r="M13" t="n">
+        <v>78.59999999999999</v>
+      </c>
+      <c r="N13" t="n">
+        <v>52.6</v>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>IBM</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>315.81</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>85.90000000000001</v>
+      </c>
+      <c r="J14" t="n">
+        <v>61.2</v>
+      </c>
+      <c r="K14" t="n">
+        <v>98.8</v>
+      </c>
+      <c r="L14" t="n">
+        <v>6.92</v>
+      </c>
+      <c r="M14" t="n">
+        <v>78.59999999999999</v>
+      </c>
+      <c r="N14" t="n">
+        <v>52.6</v>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P14" t="n">
+        <v>50.4</v>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>GS</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>315.81</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>85.90000000000001</v>
+      </c>
+      <c r="J15" t="n">
+        <v>61.2</v>
+      </c>
+      <c r="K15" t="n">
+        <v>98.8</v>
+      </c>
+      <c r="L15" t="n">
+        <v>6.92</v>
+      </c>
+      <c r="M15" t="n">
+        <v>43.6</v>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>ANSS</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>215</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>75.8</v>
+      </c>
+      <c r="J16" t="n">
+        <v>42.2</v>
+      </c>
+      <c r="K16" t="n">
+        <v>81</v>
+      </c>
+      <c r="L16" t="n">
+        <v>4.18</v>
+      </c>
+      <c r="M16" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="N16" t="n">
+        <v>90.40000000000001</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P16" t="n">
+        <v>51.6</v>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr"/>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>PSX</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>923.72</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>68.2</v>
+      </c>
+      <c r="J17" t="n">
+        <v>57.9</v>
+      </c>
+      <c r="K17" t="n">
+        <v>69.8</v>
+      </c>
+      <c r="L17" t="n">
+        <v>5.09</v>
+      </c>
+      <c r="M17" t="n">
+        <v>50</v>
+      </c>
+      <c r="N17" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P17" t="n">
+        <v>54.6</v>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr"/>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>MPC</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>226.24</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>67.5</v>
+      </c>
+      <c r="J18" t="n">
+        <v>34</v>
+      </c>
+      <c r="K18" t="n">
+        <v>98.8</v>
+      </c>
+      <c r="L18" t="n">
         <v>6.11</v>
       </c>
-      <c r="M13" t="n">
+      <c r="M18" t="n">
         <v>48.3</v>
       </c>
-      <c r="N13" t="n">
+      <c r="N18" t="n">
         <v>100</v>
       </c>
-      <c r="O13" t="inlineStr">
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P18" t="n">
+        <v>70.90000000000001</v>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr"/>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>MMM</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>226.24</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>67.5</v>
+      </c>
+      <c r="J19" t="n">
+        <v>34</v>
+      </c>
+      <c r="K19" t="n">
+        <v>98.8</v>
+      </c>
+      <c r="L19" t="n">
+        <v>6.11</v>
+      </c>
+      <c r="M19" t="n">
+        <v>48.3</v>
+      </c>
+      <c r="N19" t="n">
+        <v>100</v>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P19" t="n">
+        <v>70.90000000000001</v>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr"/>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>MO</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>226.24</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>67.5</v>
+      </c>
+      <c r="J20" t="n">
+        <v>34</v>
+      </c>
+      <c r="K20" t="n">
+        <v>98.8</v>
+      </c>
+      <c r="L20" t="n">
+        <v>6.11</v>
+      </c>
+      <c r="M20" t="n">
+        <v>48.3</v>
+      </c>
+      <c r="N20" t="n">
+        <v>100</v>
+      </c>
+      <c r="O20" t="inlineStr">
         <is>
           <t>Bearish</t>
         </is>
       </c>
-      <c r="P13" t="n">
-        <v>34.1</v>
-      </c>
-      <c r="Q13" t="inlineStr">
+      <c r="P20" t="n">
+        <v>41.7</v>
+      </c>
+      <c r="Q20" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>
       </c>
-      <c r="R13" t="inlineStr">
+      <c r="R20" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
       </c>
-      <c r="S13" t="inlineStr">
+      <c r="S20" t="inlineStr">
         <is>
           <t>maroon</t>
         </is>
       </c>
-      <c r="T13" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U13" t="inlineStr"/>
-      <c r="V13" t="inlineStr">
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr"/>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>226.24</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>67.5</v>
+      </c>
+      <c r="J21" t="n">
+        <v>34</v>
+      </c>
+      <c r="K21" t="n">
+        <v>98.8</v>
+      </c>
+      <c r="L21" t="n">
+        <v>6.11</v>
+      </c>
+      <c r="M21" t="n">
+        <v>36.1</v>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P21" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr"/>
+      <c r="V21" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Scan 09.03.2026 15:00 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V21"/>
+  <dimension ref="A1:V30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -449,7 +449,7 @@
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="6" customWidth="1" min="10" max="10"/>
     <col width="6" customWidth="1" min="11" max="11"/>
-    <col width="6" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
     <col width="9" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
@@ -577,11 +577,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>PH</t>
+          <t>GE</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>369.53</v>
+        <v>370.24</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,30 +614,30 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>87.2</v>
+        <v>87.09999999999999</v>
       </c>
       <c r="J2" t="n">
-        <v>62.3</v>
+        <v>62.6</v>
       </c>
       <c r="K2" t="n">
-        <v>90.7</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="L2" t="n">
-        <v>5.65</v>
+        <v>5.64</v>
       </c>
       <c r="M2" t="n">
-        <v>65.90000000000001</v>
+        <v>65.7</v>
       </c>
       <c r="N2" t="n">
-        <v>81.7</v>
+        <v>81.09999999999999</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>45.2</v>
+        <v>64.2</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -673,11 +673,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>PFE</t>
+          <t>HUM</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>369.53</v>
+        <v>370.24</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -710,30 +710,30 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>87.2</v>
+        <v>87.09999999999999</v>
       </c>
       <c r="J3" t="n">
-        <v>62.3</v>
+        <v>62.6</v>
       </c>
       <c r="K3" t="n">
-        <v>90.7</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="L3" t="n">
-        <v>5.65</v>
+        <v>5.64</v>
       </c>
       <c r="M3" t="n">
-        <v>65.90000000000001</v>
+        <v>65.7</v>
       </c>
       <c r="N3" t="n">
-        <v>81.7</v>
+        <v>81.09999999999999</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P3" t="n">
-        <v>45.2</v>
+        <v>70.7</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -769,11 +769,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>HUM</t>
+          <t>IBM</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>315.81</v>
+        <v>370.24</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -806,27 +806,30 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>85.90000000000001</v>
+        <v>87.09999999999999</v>
       </c>
       <c r="J4" t="n">
-        <v>61.2</v>
+        <v>62.6</v>
       </c>
       <c r="K4" t="n">
-        <v>98.8</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="L4" t="n">
-        <v>6.92</v>
+        <v>5.64</v>
       </c>
       <c r="M4" t="n">
-        <v>78.59999999999999</v>
+        <v>65.7</v>
       </c>
       <c r="N4" t="n">
-        <v>52.6</v>
+        <v>81.09999999999999</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P4" t="n">
+        <v>70.7</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -835,17 +838,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -862,11 +865,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>INTU</t>
+          <t>PAYX</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>315.81</v>
+        <v>122.98</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -899,27 +902,30 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>85.90000000000001</v>
+        <v>78.7</v>
       </c>
       <c r="J5" t="n">
-        <v>61.2</v>
+        <v>58.9</v>
       </c>
       <c r="K5" t="n">
-        <v>98.8</v>
+        <v>91.8</v>
       </c>
       <c r="L5" t="n">
-        <v>6.92</v>
+        <v>5.64</v>
       </c>
       <c r="M5" t="n">
-        <v>78.59999999999999</v>
+        <v>57.9</v>
       </c>
       <c r="N5" t="n">
-        <v>52.6</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P5" t="n">
+        <v>49.3</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -955,11 +961,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>HON</t>
+          <t>PDD</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>315.81</v>
+        <v>122.98</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -992,27 +998,30 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>85.90000000000001</v>
+        <v>78.7</v>
       </c>
       <c r="J6" t="n">
-        <v>61.2</v>
+        <v>58.9</v>
       </c>
       <c r="K6" t="n">
-        <v>98.8</v>
+        <v>91.8</v>
       </c>
       <c r="L6" t="n">
-        <v>6.92</v>
+        <v>5.64</v>
       </c>
       <c r="M6" t="n">
-        <v>78.59999999999999</v>
+        <v>57.9</v>
       </c>
       <c r="N6" t="n">
-        <v>52.6</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P6" t="n">
+        <v>49.3</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1048,11 +1057,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ISRG</t>
+          <t>MAR</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>315.81</v>
+        <v>122.98</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1085,27 +1094,30 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>85.90000000000001</v>
+        <v>78.7</v>
       </c>
       <c r="J7" t="n">
-        <v>61.2</v>
+        <v>58.9</v>
       </c>
       <c r="K7" t="n">
-        <v>98.8</v>
+        <v>91.8</v>
       </c>
       <c r="L7" t="n">
-        <v>6.92</v>
+        <v>5.64</v>
       </c>
       <c r="M7" t="n">
-        <v>78.59999999999999</v>
+        <v>57.9</v>
       </c>
       <c r="N7" t="n">
-        <v>52.6</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P7" t="n">
+        <v>49.3</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1141,11 +1153,11 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>INTC</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>315.81</v>
+        <v>122.98</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1178,27 +1190,27 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>85.90000000000001</v>
+        <v>78.7</v>
       </c>
       <c r="J8" t="n">
-        <v>61.2</v>
+        <v>58.9</v>
       </c>
       <c r="K8" t="n">
-        <v>98.8</v>
+        <v>91.8</v>
       </c>
       <c r="L8" t="n">
-        <v>6.92</v>
+        <v>5.64</v>
       </c>
       <c r="M8" t="n">
-        <v>78.59999999999999</v>
-      </c>
-      <c r="N8" t="n">
-        <v>52.6</v>
+        <v>55.6</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P8" t="n">
+        <v>49.3</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1234,11 +1246,11 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>HSY</t>
+          <t>WBD</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>315.81</v>
+        <v>122.98</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1271,27 +1283,27 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>85.90000000000001</v>
+        <v>78.7</v>
       </c>
       <c r="J9" t="n">
-        <v>61.2</v>
+        <v>58.9</v>
       </c>
       <c r="K9" t="n">
-        <v>98.8</v>
+        <v>91.8</v>
       </c>
       <c r="L9" t="n">
-        <v>6.92</v>
+        <v>5.64</v>
       </c>
       <c r="M9" t="n">
-        <v>78.59999999999999</v>
-      </c>
-      <c r="N9" t="n">
-        <v>52.6</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P9" t="n">
+        <v>49.3</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1327,11 +1339,11 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>HD</t>
+          <t>MDB</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>315.81</v>
+        <v>122.98</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1364,19 +1376,22 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>85.90000000000001</v>
+        <v>78.7</v>
       </c>
       <c r="J10" t="n">
-        <v>61.2</v>
+        <v>58.9</v>
       </c>
       <c r="K10" t="n">
-        <v>98.8</v>
+        <v>91.8</v>
       </c>
       <c r="L10" t="n">
-        <v>6.92</v>
+        <v>5.64</v>
       </c>
       <c r="M10" t="n">
-        <v>30.7</v>
+        <v>57.9</v>
+      </c>
+      <c r="N10" t="n">
+        <v>70.90000000000001</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1384,7 +1399,7 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>43.6</v>
+        <v>49.3</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1420,11 +1435,11 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ITW</t>
+          <t>COST</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>315.81</v>
+        <v>59.64</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1457,27 +1472,30 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>85.90000000000001</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="J11" t="n">
-        <v>61.2</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="K11" t="n">
-        <v>98.8</v>
+        <v>96.5</v>
       </c>
       <c r="L11" t="n">
-        <v>6.92</v>
+        <v>4.89</v>
       </c>
       <c r="M11" t="n">
-        <v>78.59999999999999</v>
+        <v>57.3</v>
       </c>
       <c r="N11" t="n">
-        <v>52.6</v>
+        <v>21.1</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P11" t="n">
+        <v>37.3</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1486,17 +1504,17 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1513,11 +1531,11 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ICE</t>
+          <t>CHTR</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>315.81</v>
+        <v>59.64</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1550,27 +1568,30 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>85.90000000000001</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="J12" t="n">
-        <v>61.2</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="K12" t="n">
-        <v>98.8</v>
+        <v>96.5</v>
       </c>
       <c r="L12" t="n">
-        <v>6.92</v>
+        <v>4.89</v>
       </c>
       <c r="M12" t="n">
-        <v>78.59999999999999</v>
+        <v>57.3</v>
       </c>
       <c r="N12" t="n">
-        <v>52.6</v>
+        <v>21.1</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P12" t="n">
+        <v>64.09999999999999</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1579,17 +1600,17 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1606,11 +1627,11 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>JPM</t>
+          <t>CME</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>315.81</v>
+        <v>59.64</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -1643,27 +1664,30 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>85.90000000000001</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="J13" t="n">
-        <v>61.2</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="K13" t="n">
-        <v>98.8</v>
+        <v>96.5</v>
       </c>
       <c r="L13" t="n">
-        <v>6.92</v>
+        <v>4.89</v>
       </c>
       <c r="M13" t="n">
-        <v>78.59999999999999</v>
+        <v>57.3</v>
       </c>
       <c r="N13" t="n">
-        <v>52.6</v>
+        <v>21.1</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P13" t="n">
+        <v>64.09999999999999</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1672,17 +1696,17 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1699,11 +1723,11 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>IBM</t>
+          <t>CAT</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>315.81</v>
+        <v>59.64</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -1736,22 +1760,19 @@
         </is>
       </c>
       <c r="I14" t="n">
-        <v>85.90000000000001</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="J14" t="n">
-        <v>61.2</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="K14" t="n">
-        <v>98.8</v>
+        <v>96.5</v>
       </c>
       <c r="L14" t="n">
-        <v>6.92</v>
+        <v>4.89</v>
       </c>
       <c r="M14" t="n">
-        <v>78.59999999999999</v>
-      </c>
-      <c r="N14" t="n">
-        <v>52.6</v>
+        <v>47.5</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1759,7 +1780,7 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>50.4</v>
+        <v>51.8</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1768,17 +1789,17 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1795,11 +1816,11 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>GS</t>
+          <t>C</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>315.81</v>
+        <v>59.64</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1832,24 +1853,30 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>85.90000000000001</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="J15" t="n">
-        <v>61.2</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="K15" t="n">
-        <v>98.8</v>
+        <v>96.5</v>
       </c>
       <c r="L15" t="n">
-        <v>6.92</v>
+        <v>4.89</v>
       </c>
       <c r="M15" t="n">
-        <v>43.6</v>
+        <v>57.3</v>
+      </c>
+      <c r="N15" t="n">
+        <v>21.1</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P15" t="n">
+        <v>37.3</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1858,17 +1885,17 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -1885,30 +1912,30 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ANSS</t>
+          <t>CEG</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>215</v>
+        <v>59.64</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1922,30 +1949,30 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>75.8</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="J16" t="n">
-        <v>42.2</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="K16" t="n">
-        <v>81</v>
+        <v>96.5</v>
       </c>
       <c r="L16" t="n">
-        <v>4.18</v>
+        <v>4.89</v>
       </c>
       <c r="M16" t="n">
-        <v>51.5</v>
+        <v>57.3</v>
       </c>
       <c r="N16" t="n">
-        <v>90.40000000000001</v>
+        <v>21.1</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>51.6</v>
+        <v>51.8</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1959,29 +1986,33 @@
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U16" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>PSX</t>
+          <t>BRK-B</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>923.72</v>
+        <v>59.64</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -2010,26 +2041,26 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>68.2</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="J17" t="n">
-        <v>57.9</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="K17" t="n">
-        <v>69.8</v>
+        <v>96.5</v>
       </c>
       <c r="L17" t="n">
-        <v>5.09</v>
+        <v>4.89</v>
       </c>
       <c r="M17" t="n">
-        <v>50</v>
+        <v>57.3</v>
       </c>
       <c r="N17" t="n">
-        <v>23.8</v>
+        <v>21.1</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -2037,7 +2068,7 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>54.6</v>
+        <v>37.3</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -2046,53 +2077,57 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U17" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>MPC</t>
+          <t>CMCSA</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>226.24</v>
+        <v>59.64</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -2106,22 +2141,22 @@
         </is>
       </c>
       <c r="I18" t="n">
-        <v>67.5</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="J18" t="n">
-        <v>34</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="K18" t="n">
-        <v>98.8</v>
+        <v>96.5</v>
       </c>
       <c r="L18" t="n">
-        <v>6.11</v>
+        <v>4.89</v>
       </c>
       <c r="M18" t="n">
-        <v>48.3</v>
+        <v>57.3</v>
       </c>
       <c r="N18" t="n">
-        <v>100</v>
+        <v>21.1</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -2129,7 +2164,7 @@
         </is>
       </c>
       <c r="P18" t="n">
-        <v>70.90000000000001</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -2143,48 +2178,52 @@
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U18" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>MMM</t>
+          <t>CCI</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>226.24</v>
+        <v>59.64</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2198,22 +2237,22 @@
         </is>
       </c>
       <c r="I19" t="n">
-        <v>67.5</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="J19" t="n">
-        <v>34</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="K19" t="n">
-        <v>98.8</v>
+        <v>96.5</v>
       </c>
       <c r="L19" t="n">
-        <v>6.11</v>
+        <v>4.89</v>
       </c>
       <c r="M19" t="n">
-        <v>48.3</v>
+        <v>57.3</v>
       </c>
       <c r="N19" t="n">
-        <v>100</v>
+        <v>21.1</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -2221,7 +2260,7 @@
         </is>
       </c>
       <c r="P19" t="n">
-        <v>70.90000000000001</v>
+        <v>57.1</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -2235,48 +2274,52 @@
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U19" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>MO</t>
+          <t>CL</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>226.24</v>
+        <v>59.64</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -2290,22 +2333,22 @@
         </is>
       </c>
       <c r="I20" t="n">
-        <v>67.5</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="J20" t="n">
-        <v>34</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="K20" t="n">
-        <v>98.8</v>
+        <v>96.5</v>
       </c>
       <c r="L20" t="n">
-        <v>6.11</v>
+        <v>4.89</v>
       </c>
       <c r="M20" t="n">
-        <v>48.3</v>
+        <v>57.3</v>
       </c>
       <c r="N20" t="n">
-        <v>100</v>
+        <v>21.1</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -2313,7 +2356,7 @@
         </is>
       </c>
       <c r="P20" t="n">
-        <v>41.7</v>
+        <v>37.6</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
@@ -2327,48 +2370,52 @@
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U20" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>D</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>226.24</v>
+        <v>131.76</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2382,27 +2429,30 @@
         </is>
       </c>
       <c r="I21" t="n">
-        <v>67.5</v>
+        <v>69.8</v>
       </c>
       <c r="J21" t="n">
-        <v>34</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="K21" t="n">
-        <v>98.8</v>
+        <v>81</v>
       </c>
       <c r="L21" t="n">
-        <v>6.11</v>
+        <v>1.88</v>
       </c>
       <c r="M21" t="n">
-        <v>36.1</v>
+        <v>18.9</v>
+      </c>
+      <c r="N21" t="n">
+        <v>46.4</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P21" t="n">
-        <v>50.5</v>
+        <v>37.6</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
@@ -2411,12 +2461,12 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
@@ -2426,6 +2476,834 @@
       </c>
       <c r="U21" t="inlineStr"/>
       <c r="V21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>SBUX</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>122.69</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>69.8</v>
+      </c>
+      <c r="J22" t="n">
+        <v>38.2</v>
+      </c>
+      <c r="K22" t="n">
+        <v>98.8</v>
+      </c>
+      <c r="L22" t="n">
+        <v>11.36</v>
+      </c>
+      <c r="M22" t="n">
+        <v>91.8</v>
+      </c>
+      <c r="N22" t="n">
+        <v>76.59999999999999</v>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P22" t="n">
+        <v>47.8</v>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr"/>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>PH</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>122.69</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>69.8</v>
+      </c>
+      <c r="J23" t="n">
+        <v>38.2</v>
+      </c>
+      <c r="K23" t="n">
+        <v>98.8</v>
+      </c>
+      <c r="L23" t="n">
+        <v>11.36</v>
+      </c>
+      <c r="M23" t="n">
+        <v>91.8</v>
+      </c>
+      <c r="N23" t="n">
+        <v>76.59999999999999</v>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P23" t="n">
+        <v>54.2</v>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr"/>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>ROST</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>122.69</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>69.8</v>
+      </c>
+      <c r="J24" t="n">
+        <v>38.2</v>
+      </c>
+      <c r="K24" t="n">
+        <v>98.8</v>
+      </c>
+      <c r="L24" t="n">
+        <v>11.36</v>
+      </c>
+      <c r="M24" t="n">
+        <v>91.8</v>
+      </c>
+      <c r="N24" t="n">
+        <v>76.59999999999999</v>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P24" t="n">
+        <v>47.8</v>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr"/>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>ROP</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>122.69</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>69.8</v>
+      </c>
+      <c r="J25" t="n">
+        <v>38.2</v>
+      </c>
+      <c r="K25" t="n">
+        <v>98.8</v>
+      </c>
+      <c r="L25" t="n">
+        <v>11.36</v>
+      </c>
+      <c r="M25" t="n">
+        <v>91.8</v>
+      </c>
+      <c r="N25" t="n">
+        <v>76.59999999999999</v>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P25" t="n">
+        <v>54.2</v>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr"/>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>PFE</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>122.69</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>69.8</v>
+      </c>
+      <c r="J26" t="n">
+        <v>38.2</v>
+      </c>
+      <c r="K26" t="n">
+        <v>98.8</v>
+      </c>
+      <c r="L26" t="n">
+        <v>11.36</v>
+      </c>
+      <c r="M26" t="n">
+        <v>91.8</v>
+      </c>
+      <c r="N26" t="n">
+        <v>76.59999999999999</v>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P26" t="n">
+        <v>47.8</v>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr"/>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>QCOM</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>122.69</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>69.8</v>
+      </c>
+      <c r="J27" t="n">
+        <v>38.2</v>
+      </c>
+      <c r="K27" t="n">
+        <v>98.8</v>
+      </c>
+      <c r="L27" t="n">
+        <v>11.36</v>
+      </c>
+      <c r="M27" t="n">
+        <v>91.8</v>
+      </c>
+      <c r="N27" t="n">
+        <v>76.59999999999999</v>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P27" t="n">
+        <v>54.2</v>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr"/>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>RTX</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>122.69</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>69.8</v>
+      </c>
+      <c r="J28" t="n">
+        <v>38.2</v>
+      </c>
+      <c r="K28" t="n">
+        <v>98.8</v>
+      </c>
+      <c r="L28" t="n">
+        <v>11.36</v>
+      </c>
+      <c r="M28" t="n">
+        <v>91.8</v>
+      </c>
+      <c r="N28" t="n">
+        <v>76.59999999999999</v>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P28" t="n">
+        <v>54.2</v>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr"/>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>PYPL</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>122.69</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>69.8</v>
+      </c>
+      <c r="J29" t="n">
+        <v>38.2</v>
+      </c>
+      <c r="K29" t="n">
+        <v>98.8</v>
+      </c>
+      <c r="L29" t="n">
+        <v>11.36</v>
+      </c>
+      <c r="M29" t="n">
+        <v>91.8</v>
+      </c>
+      <c r="N29" t="n">
+        <v>76.59999999999999</v>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P29" t="n">
+        <v>54.2</v>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr"/>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>SLB</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>122.69</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>69.8</v>
+      </c>
+      <c r="J30" t="n">
+        <v>38.2</v>
+      </c>
+      <c r="K30" t="n">
+        <v>98.8</v>
+      </c>
+      <c r="L30" t="n">
+        <v>11.36</v>
+      </c>
+      <c r="M30" t="n">
+        <v>91.8</v>
+      </c>
+      <c r="N30" t="n">
+        <v>76.59999999999999</v>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P30" t="n">
+        <v>54.2</v>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr"/>
+      <c r="V30" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Scan 09.03.2026 18:43 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,9 +32,6 @@
     </font>
     <font>
       <color rgb="00ef4444"/>
-    </font>
-    <font>
-      <color rgb="0022c55e"/>
     </font>
   </fonts>
   <fills count="3">
@@ -63,13 +60,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -435,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V30"/>
+  <dimension ref="A1:V21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -444,7 +440,7 @@
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="6" customWidth="1" min="10" max="10"/>
@@ -458,7 +454,7 @@
     <col width="15" customWidth="1" min="18" max="18"/>
     <col width="11" customWidth="1" min="19" max="19"/>
     <col width="11" customWidth="1" min="20" max="20"/>
-    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="25" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
@@ -577,11 +573,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>GE</t>
+          <t>SMCI</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>370.24</v>
+        <v>327.49</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,30 +610,30 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>87.09999999999999</v>
+        <v>86.5</v>
       </c>
       <c r="J2" t="n">
-        <v>62.6</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="K2" t="n">
-        <v>90.59999999999999</v>
+        <v>97.59999999999999</v>
       </c>
       <c r="L2" t="n">
-        <v>5.64</v>
+        <v>10.49</v>
       </c>
       <c r="M2" t="n">
-        <v>65.7</v>
+        <v>98.09999999999999</v>
       </c>
       <c r="N2" t="n">
-        <v>81.09999999999999</v>
+        <v>83.8</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>64.2</v>
+        <v>38.5</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -646,17 +642,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -673,11 +669,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>HUM</t>
+          <t>SO</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>370.24</v>
+        <v>327.49</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -710,30 +706,30 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>87.09999999999999</v>
+        <v>86.5</v>
       </c>
       <c r="J3" t="n">
-        <v>62.6</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="K3" t="n">
-        <v>90.59999999999999</v>
+        <v>97.59999999999999</v>
       </c>
       <c r="L3" t="n">
-        <v>5.64</v>
+        <v>10.49</v>
       </c>
       <c r="M3" t="n">
-        <v>65.7</v>
+        <v>98.09999999999999</v>
       </c>
       <c r="N3" t="n">
-        <v>81.09999999999999</v>
+        <v>83.8</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P3" t="n">
-        <v>70.7</v>
+        <v>38.5</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -742,17 +738,17 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -769,11 +765,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>IBM</t>
+          <t>PNC</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>370.24</v>
+        <v>327.49</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -806,30 +802,30 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>87.09999999999999</v>
+        <v>86.5</v>
       </c>
       <c r="J4" t="n">
-        <v>62.6</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="K4" t="n">
-        <v>90.59999999999999</v>
+        <v>97.59999999999999</v>
       </c>
       <c r="L4" t="n">
-        <v>5.64</v>
+        <v>10.49</v>
       </c>
       <c r="M4" t="n">
-        <v>65.7</v>
+        <v>98.09999999999999</v>
       </c>
       <c r="N4" t="n">
-        <v>81.09999999999999</v>
+        <v>83.8</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P4" t="n">
-        <v>70.7</v>
+        <v>38.5</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -838,17 +834,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -865,11 +861,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>PAYX</t>
+          <t>SPG</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>122.98</v>
+        <v>327.49</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -902,22 +898,22 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>78.7</v>
+        <v>86.5</v>
       </c>
       <c r="J5" t="n">
-        <v>58.9</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="K5" t="n">
-        <v>91.8</v>
+        <v>97.59999999999999</v>
       </c>
       <c r="L5" t="n">
-        <v>5.64</v>
+        <v>10.49</v>
       </c>
       <c r="M5" t="n">
-        <v>57.9</v>
+        <v>98.09999999999999</v>
       </c>
       <c r="N5" t="n">
-        <v>70.90000000000001</v>
+        <v>83.8</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -925,7 +921,7 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>49.3</v>
+        <v>38.5</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -961,11 +957,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>PDD</t>
+          <t>SRE</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>122.98</v>
+        <v>327.49</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -998,30 +994,30 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>78.7</v>
+        <v>86.5</v>
       </c>
       <c r="J6" t="n">
-        <v>58.9</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="K6" t="n">
-        <v>91.8</v>
+        <v>97.59999999999999</v>
       </c>
       <c r="L6" t="n">
-        <v>5.64</v>
+        <v>10.49</v>
       </c>
       <c r="M6" t="n">
-        <v>57.9</v>
+        <v>98.09999999999999</v>
       </c>
       <c r="N6" t="n">
-        <v>70.90000000000001</v>
+        <v>83.8</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P6" t="n">
-        <v>49.3</v>
+        <v>53.8</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1057,11 +1053,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>SNPS</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>122.98</v>
+        <v>327.49</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1094,22 +1090,22 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>78.7</v>
+        <v>86.5</v>
       </c>
       <c r="J7" t="n">
-        <v>58.9</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="K7" t="n">
-        <v>91.8</v>
+        <v>97.59999999999999</v>
       </c>
       <c r="L7" t="n">
-        <v>5.64</v>
+        <v>10.49</v>
       </c>
       <c r="M7" t="n">
-        <v>57.9</v>
+        <v>98.09999999999999</v>
       </c>
       <c r="N7" t="n">
-        <v>70.90000000000001</v>
+        <v>83.8</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1117,7 +1113,7 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>49.3</v>
+        <v>38.5</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1153,11 +1149,11 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>122.98</v>
+        <v>131.45</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1190,19 +1186,22 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>78.7</v>
+        <v>69.2</v>
       </c>
       <c r="J8" t="n">
-        <v>58.9</v>
+        <v>62.9</v>
       </c>
       <c r="K8" t="n">
-        <v>91.8</v>
+        <v>81</v>
       </c>
       <c r="L8" t="n">
-        <v>5.64</v>
+        <v>1.9</v>
       </c>
       <c r="M8" t="n">
-        <v>55.6</v>
+        <v>18.9</v>
+      </c>
+      <c r="N8" t="n">
+        <v>46.8</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1210,7 +1209,7 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>49.3</v>
+        <v>44.3</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1232,25 +1231,21 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>WBD</t>
+          <t>BMY</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>122.98</v>
+        <v>131.45</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1283,19 +1278,19 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>78.7</v>
+        <v>69.2</v>
       </c>
       <c r="J9" t="n">
-        <v>58.9</v>
+        <v>62.9</v>
       </c>
       <c r="K9" t="n">
-        <v>91.8</v>
+        <v>81</v>
       </c>
       <c r="L9" t="n">
-        <v>5.64</v>
+        <v>1.9</v>
       </c>
       <c r="M9" t="n">
-        <v>75.09999999999999</v>
+        <v>32.6</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1303,7 +1298,7 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>49.3</v>
+        <v>44.3</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1325,25 +1320,21 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>MDB</t>
+          <t>BK</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>122.98</v>
+        <v>131.45</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1376,22 +1367,19 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>78.7</v>
+        <v>69.2</v>
       </c>
       <c r="J10" t="n">
-        <v>58.9</v>
+        <v>62.9</v>
       </c>
       <c r="K10" t="n">
-        <v>91.8</v>
+        <v>81</v>
       </c>
       <c r="L10" t="n">
-        <v>5.64</v>
+        <v>1.9</v>
       </c>
       <c r="M10" t="n">
-        <v>57.9</v>
-      </c>
-      <c r="N10" t="n">
-        <v>70.90000000000001</v>
+        <v>44.3</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1399,7 +1387,7 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>49.3</v>
+        <v>44.3</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1421,14 +1409,10 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U10" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U10" t="inlineStr"/>
       <c r="V10" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -1439,7 +1423,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>59.64</v>
+        <v>131.45</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1472,22 +1456,19 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>72.09999999999999</v>
+        <v>69.2</v>
       </c>
       <c r="J11" t="n">
-        <v>65.40000000000001</v>
+        <v>62.9</v>
       </c>
       <c r="K11" t="n">
-        <v>96.5</v>
+        <v>81</v>
       </c>
       <c r="L11" t="n">
-        <v>4.89</v>
+        <v>1.9</v>
       </c>
       <c r="M11" t="n">
-        <v>57.3</v>
-      </c>
-      <c r="N11" t="n">
-        <v>21.1</v>
+        <v>26</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1495,7 +1476,7 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>37.3</v>
+        <v>44.3</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1504,38 +1485,34 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr"/>
+      <c r="V11" t="inlineStr">
+        <is>
           <t>No</t>
-        </is>
-      </c>
-      <c r="U11" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
-      <c r="V11" t="inlineStr">
-        <is>
-          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CHTR</t>
+          <t>C</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>59.64</v>
+        <v>131.45</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1568,30 +1545,27 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>72.09999999999999</v>
+        <v>69.2</v>
       </c>
       <c r="J12" t="n">
-        <v>65.40000000000001</v>
+        <v>62.9</v>
       </c>
       <c r="K12" t="n">
-        <v>96.5</v>
+        <v>81</v>
       </c>
       <c r="L12" t="n">
-        <v>4.89</v>
+        <v>1.9</v>
       </c>
       <c r="M12" t="n">
-        <v>57.3</v>
-      </c>
-      <c r="N12" t="n">
-        <v>21.1</v>
+        <v>42.1</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>64.09999999999999</v>
+        <v>44.4</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1600,38 +1574,34 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr"/>
+      <c r="V12" t="inlineStr">
+        <is>
           <t>No</t>
-        </is>
-      </c>
-      <c r="U12" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
-      <c r="V12" t="inlineStr">
-        <is>
-          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CME</t>
+          <t>COP</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>59.64</v>
+        <v>131.45</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -1664,30 +1634,30 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>72.09999999999999</v>
+        <v>69.2</v>
       </c>
       <c r="J13" t="n">
-        <v>65.40000000000001</v>
+        <v>62.9</v>
       </c>
       <c r="K13" t="n">
-        <v>96.5</v>
+        <v>81</v>
       </c>
       <c r="L13" t="n">
-        <v>4.89</v>
+        <v>1.9</v>
       </c>
       <c r="M13" t="n">
-        <v>57.3</v>
+        <v>18.9</v>
       </c>
       <c r="N13" t="n">
-        <v>21.1</v>
+        <v>46.8</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>64.09999999999999</v>
+        <v>44.1</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1696,38 +1666,34 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr"/>
+      <c r="V13" t="inlineStr">
+        <is>
           <t>No</t>
-        </is>
-      </c>
-      <c r="U13" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
-      <c r="V13" t="inlineStr">
-        <is>
-          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CAT</t>
+          <t>GLD</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>59.64</v>
+        <v>317.85</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -1756,23 +1722,23 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>72.09999999999999</v>
+        <v>59.8</v>
       </c>
       <c r="J14" t="n">
-        <v>65.40000000000001</v>
+        <v>54.9</v>
       </c>
       <c r="K14" t="n">
-        <v>96.5</v>
+        <v>77</v>
       </c>
       <c r="L14" t="n">
-        <v>4.89</v>
+        <v>4.3</v>
       </c>
       <c r="M14" t="n">
-        <v>47.5</v>
+        <v>30.1</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1780,7 +1746,7 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>51.8</v>
+        <v>43.7</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1802,25 +1768,21 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U14" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U14" t="inlineStr"/>
       <c r="V14" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>TTWO</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>59.64</v>
+        <v>317.85</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1849,26 +1811,26 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>72.09999999999999</v>
+        <v>59.8</v>
       </c>
       <c r="J15" t="n">
-        <v>65.40000000000001</v>
+        <v>54.9</v>
       </c>
       <c r="K15" t="n">
-        <v>96.5</v>
+        <v>77</v>
       </c>
       <c r="L15" t="n">
-        <v>4.89</v>
+        <v>4.3</v>
       </c>
       <c r="M15" t="n">
-        <v>57.3</v>
+        <v>48</v>
       </c>
       <c r="N15" t="n">
-        <v>21.1</v>
+        <v>31.4</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1876,7 +1838,7 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>37.3</v>
+        <v>47.4</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1898,25 +1860,21 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U15" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U15" t="inlineStr"/>
       <c r="V15" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CEG</t>
+          <t>TEAM</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>59.64</v>
+        <v>317.85</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -1945,34 +1903,31 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>72.09999999999999</v>
+        <v>59.8</v>
       </c>
       <c r="J16" t="n">
-        <v>65.40000000000001</v>
+        <v>54.9</v>
       </c>
       <c r="K16" t="n">
-        <v>96.5</v>
+        <v>77</v>
       </c>
       <c r="L16" t="n">
-        <v>4.89</v>
+        <v>4.3</v>
       </c>
       <c r="M16" t="n">
-        <v>57.3</v>
-      </c>
-      <c r="N16" t="n">
-        <v>21.1</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>51.8</v>
+        <v>47.4</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1994,29 +1949,25 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U16" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U16" t="inlineStr"/>
       <c r="V16" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>BRK-B</t>
+          <t>SYY</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>59.64</v>
+        <v>55.93</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -2031,68 +1982,68 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>72.09999999999999</v>
+        <v>52.6</v>
       </c>
       <c r="J17" t="n">
-        <v>65.40000000000001</v>
+        <v>38.5</v>
       </c>
       <c r="K17" t="n">
-        <v>96.5</v>
+        <v>9.4</v>
       </c>
       <c r="L17" t="n">
-        <v>4.89</v>
+        <v>8.33</v>
       </c>
       <c r="M17" t="n">
-        <v>57.3</v>
+        <v>76</v>
       </c>
       <c r="N17" t="n">
-        <v>21.1</v>
+        <v>39.2</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P17" t="n">
-        <v>37.3</v>
+        <v>50.3</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>Divergence</t>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
@@ -2104,15 +2055,15 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CMCSA</t>
+          <t>TDG</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>59.64</v>
+        <v>55.93</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -2127,36 +2078,33 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>72.09999999999999</v>
+        <v>52.6</v>
       </c>
       <c r="J18" t="n">
-        <v>65.40000000000001</v>
+        <v>38.5</v>
       </c>
       <c r="K18" t="n">
-        <v>96.5</v>
+        <v>9.4</v>
       </c>
       <c r="L18" t="n">
-        <v>4.89</v>
+        <v>8.33</v>
       </c>
       <c r="M18" t="n">
-        <v>57.3</v>
-      </c>
-      <c r="N18" t="n">
-        <v>21.1</v>
+        <v>33.5</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -2164,31 +2112,31 @@
         </is>
       </c>
       <c r="P18" t="n">
-        <v>64.09999999999999</v>
+        <v>50.3</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>Divergence</t>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
@@ -2200,15 +2148,15 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CCI</t>
+          <t>TJX</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>59.64</v>
+        <v>55.93</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -2223,36 +2171,36 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>72.09999999999999</v>
+        <v>52.6</v>
       </c>
       <c r="J19" t="n">
-        <v>65.40000000000001</v>
+        <v>38.5</v>
       </c>
       <c r="K19" t="n">
-        <v>96.5</v>
+        <v>9.4</v>
       </c>
       <c r="L19" t="n">
-        <v>4.89</v>
+        <v>8.33</v>
       </c>
       <c r="M19" t="n">
-        <v>57.3</v>
+        <v>76</v>
       </c>
       <c r="N19" t="n">
-        <v>21.1</v>
+        <v>39.2</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -2260,31 +2208,31 @@
         </is>
       </c>
       <c r="P19" t="n">
-        <v>57.1</v>
+        <v>50.3</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>Divergence</t>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
@@ -2296,15 +2244,15 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>SCHW</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>59.64</v>
+        <v>55.93</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -2319,68 +2267,68 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I20" t="n">
-        <v>72.09999999999999</v>
+        <v>52.6</v>
       </c>
       <c r="J20" t="n">
-        <v>65.40000000000001</v>
+        <v>38.5</v>
       </c>
       <c r="K20" t="n">
-        <v>96.5</v>
+        <v>9.4</v>
       </c>
       <c r="L20" t="n">
-        <v>4.89</v>
+        <v>8.33</v>
       </c>
       <c r="M20" t="n">
-        <v>57.3</v>
+        <v>76</v>
       </c>
       <c r="N20" t="n">
-        <v>21.1</v>
+        <v>39.2</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P20" t="n">
-        <v>37.6</v>
+        <v>53.8</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>Divergence</t>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
@@ -2392,15 +2340,15 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>TGT</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>131.76</v>
+        <v>55.93</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -2415,48 +2363,48 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>69.8</v>
+        <v>52.6</v>
       </c>
       <c r="J21" t="n">
-        <v>64.09999999999999</v>
+        <v>38.5</v>
       </c>
       <c r="K21" t="n">
-        <v>81</v>
+        <v>9.4</v>
       </c>
       <c r="L21" t="n">
-        <v>1.88</v>
+        <v>8.33</v>
       </c>
       <c r="M21" t="n">
-        <v>18.9</v>
+        <v>76</v>
       </c>
       <c r="N21" t="n">
-        <v>46.4</v>
+        <v>39.2</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P21" t="n">
-        <v>37.6</v>
+        <v>53.8</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
@@ -2466,7 +2414,7 @@
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
@@ -2474,838 +2422,14 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U21" t="inlineStr"/>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>SBUX</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>122.69</v>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I22" t="n">
-        <v>69.8</v>
-      </c>
-      <c r="J22" t="n">
-        <v>38.2</v>
-      </c>
-      <c r="K22" t="n">
-        <v>98.8</v>
-      </c>
-      <c r="L22" t="n">
-        <v>11.36</v>
-      </c>
-      <c r="M22" t="n">
-        <v>91.8</v>
-      </c>
-      <c r="N22" t="n">
-        <v>76.59999999999999</v>
-      </c>
-      <c r="O22" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P22" t="n">
-        <v>47.8</v>
-      </c>
-      <c r="Q22" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R22" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="S22" t="inlineStr">
-        <is>
-          <t>maroon</t>
-        </is>
-      </c>
-      <c r="T22" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U22" t="inlineStr"/>
-      <c r="V22" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>PH</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>122.69</v>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I23" t="n">
-        <v>69.8</v>
-      </c>
-      <c r="J23" t="n">
-        <v>38.2</v>
-      </c>
-      <c r="K23" t="n">
-        <v>98.8</v>
-      </c>
-      <c r="L23" t="n">
-        <v>11.36</v>
-      </c>
-      <c r="M23" t="n">
-        <v>91.8</v>
-      </c>
-      <c r="N23" t="n">
-        <v>76.59999999999999</v>
-      </c>
-      <c r="O23" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P23" t="n">
-        <v>54.2</v>
-      </c>
-      <c r="Q23" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R23" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="S23" t="inlineStr">
-        <is>
-          <t>maroon</t>
-        </is>
-      </c>
-      <c r="T23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U23" t="inlineStr"/>
-      <c r="V23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>ROST</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>122.69</v>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I24" t="n">
-        <v>69.8</v>
-      </c>
-      <c r="J24" t="n">
-        <v>38.2</v>
-      </c>
-      <c r="K24" t="n">
-        <v>98.8</v>
-      </c>
-      <c r="L24" t="n">
-        <v>11.36</v>
-      </c>
-      <c r="M24" t="n">
-        <v>91.8</v>
-      </c>
-      <c r="N24" t="n">
-        <v>76.59999999999999</v>
-      </c>
-      <c r="O24" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P24" t="n">
-        <v>47.8</v>
-      </c>
-      <c r="Q24" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R24" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="S24" t="inlineStr">
-        <is>
-          <t>maroon</t>
-        </is>
-      </c>
-      <c r="T24" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U24" t="inlineStr"/>
-      <c r="V24" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>ROP</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>122.69</v>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I25" t="n">
-        <v>69.8</v>
-      </c>
-      <c r="J25" t="n">
-        <v>38.2</v>
-      </c>
-      <c r="K25" t="n">
-        <v>98.8</v>
-      </c>
-      <c r="L25" t="n">
-        <v>11.36</v>
-      </c>
-      <c r="M25" t="n">
-        <v>91.8</v>
-      </c>
-      <c r="N25" t="n">
-        <v>76.59999999999999</v>
-      </c>
-      <c r="O25" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P25" t="n">
-        <v>54.2</v>
-      </c>
-      <c r="Q25" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R25" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="S25" t="inlineStr">
-        <is>
-          <t>maroon</t>
-        </is>
-      </c>
-      <c r="T25" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U25" t="inlineStr"/>
-      <c r="V25" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>PFE</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>122.69</v>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D26" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I26" t="n">
-        <v>69.8</v>
-      </c>
-      <c r="J26" t="n">
-        <v>38.2</v>
-      </c>
-      <c r="K26" t="n">
-        <v>98.8</v>
-      </c>
-      <c r="L26" t="n">
-        <v>11.36</v>
-      </c>
-      <c r="M26" t="n">
-        <v>91.8</v>
-      </c>
-      <c r="N26" t="n">
-        <v>76.59999999999999</v>
-      </c>
-      <c r="O26" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P26" t="n">
-        <v>47.8</v>
-      </c>
-      <c r="Q26" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R26" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="S26" t="inlineStr">
-        <is>
-          <t>maroon</t>
-        </is>
-      </c>
-      <c r="T26" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U26" t="inlineStr"/>
-      <c r="V26" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>QCOM</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>122.69</v>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D27" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I27" t="n">
-        <v>69.8</v>
-      </c>
-      <c r="J27" t="n">
-        <v>38.2</v>
-      </c>
-      <c r="K27" t="n">
-        <v>98.8</v>
-      </c>
-      <c r="L27" t="n">
-        <v>11.36</v>
-      </c>
-      <c r="M27" t="n">
-        <v>91.8</v>
-      </c>
-      <c r="N27" t="n">
-        <v>76.59999999999999</v>
-      </c>
-      <c r="O27" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P27" t="n">
-        <v>54.2</v>
-      </c>
-      <c r="Q27" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R27" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="S27" t="inlineStr">
-        <is>
-          <t>maroon</t>
-        </is>
-      </c>
-      <c r="T27" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U27" t="inlineStr"/>
-      <c r="V27" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>RTX</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
-        <v>122.69</v>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D28" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I28" t="n">
-        <v>69.8</v>
-      </c>
-      <c r="J28" t="n">
-        <v>38.2</v>
-      </c>
-      <c r="K28" t="n">
-        <v>98.8</v>
-      </c>
-      <c r="L28" t="n">
-        <v>11.36</v>
-      </c>
-      <c r="M28" t="n">
-        <v>91.8</v>
-      </c>
-      <c r="N28" t="n">
-        <v>76.59999999999999</v>
-      </c>
-      <c r="O28" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P28" t="n">
-        <v>54.2</v>
-      </c>
-      <c r="Q28" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R28" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="S28" t="inlineStr">
-        <is>
-          <t>maroon</t>
-        </is>
-      </c>
-      <c r="T28" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U28" t="inlineStr"/>
-      <c r="V28" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>PYPL</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>122.69</v>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D29" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I29" t="n">
-        <v>69.8</v>
-      </c>
-      <c r="J29" t="n">
-        <v>38.2</v>
-      </c>
-      <c r="K29" t="n">
-        <v>98.8</v>
-      </c>
-      <c r="L29" t="n">
-        <v>11.36</v>
-      </c>
-      <c r="M29" t="n">
-        <v>91.8</v>
-      </c>
-      <c r="N29" t="n">
-        <v>76.59999999999999</v>
-      </c>
-      <c r="O29" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P29" t="n">
-        <v>54.2</v>
-      </c>
-      <c r="Q29" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R29" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="S29" t="inlineStr">
-        <is>
-          <t>maroon</t>
-        </is>
-      </c>
-      <c r="T29" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U29" t="inlineStr"/>
-      <c r="V29" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>SLB</t>
-        </is>
-      </c>
-      <c r="B30" t="n">
-        <v>122.69</v>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D30" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I30" t="n">
-        <v>69.8</v>
-      </c>
-      <c r="J30" t="n">
-        <v>38.2</v>
-      </c>
-      <c r="K30" t="n">
-        <v>98.8</v>
-      </c>
-      <c r="L30" t="n">
-        <v>11.36</v>
-      </c>
-      <c r="M30" t="n">
-        <v>91.8</v>
-      </c>
-      <c r="N30" t="n">
-        <v>76.59999999999999</v>
-      </c>
-      <c r="O30" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P30" t="n">
-        <v>54.2</v>
-      </c>
-      <c r="Q30" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R30" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="S30" t="inlineStr">
-        <is>
-          <t>maroon</t>
-        </is>
-      </c>
-      <c r="T30" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U30" t="inlineStr"/>
-      <c r="V30" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan 10.03.2026 14:58 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,6 +32,9 @@
     </font>
     <font>
       <color rgb="00ef4444"/>
+    </font>
+    <font>
+      <color rgb="0022c55e"/>
     </font>
   </fonts>
   <fills count="3">
@@ -60,12 +63,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -431,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V21"/>
+  <dimension ref="A1:V36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -440,12 +444,12 @@
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="6" customWidth="1" min="10" max="10"/>
     <col width="6" customWidth="1" min="11" max="11"/>
-    <col width="7" customWidth="1" min="12" max="12"/>
+    <col width="6" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
     <col width="9" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
@@ -454,7 +458,7 @@
     <col width="15" customWidth="1" min="18" max="18"/>
     <col width="11" customWidth="1" min="19" max="19"/>
     <col width="11" customWidth="1" min="20" max="20"/>
-    <col width="25" customWidth="1" min="21" max="21"/>
+    <col width="10" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
@@ -573,11 +577,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SMCI</t>
+          <t>BKNG</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>327.49</v>
+        <v>349.44</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -610,30 +614,30 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>86.5</v>
+        <v>80.90000000000001</v>
       </c>
       <c r="J2" t="n">
-        <v>64.40000000000001</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="K2" t="n">
-        <v>97.59999999999999</v>
+        <v>95.3</v>
       </c>
       <c r="L2" t="n">
-        <v>10.49</v>
+        <v>9.609999999999999</v>
       </c>
       <c r="M2" t="n">
-        <v>98.09999999999999</v>
+        <v>90.09999999999999</v>
       </c>
       <c r="N2" t="n">
-        <v>83.8</v>
+        <v>49.6</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>38.5</v>
+        <v>48.3</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -655,25 +659,21 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SO</t>
+          <t>CAT</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>327.49</v>
+        <v>349.44</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -706,22 +706,22 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>86.5</v>
+        <v>80.90000000000001</v>
       </c>
       <c r="J3" t="n">
-        <v>64.40000000000001</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="K3" t="n">
-        <v>97.59999999999999</v>
+        <v>95.3</v>
       </c>
       <c r="L3" t="n">
-        <v>10.49</v>
+        <v>9.609999999999999</v>
       </c>
       <c r="M3" t="n">
-        <v>98.09999999999999</v>
+        <v>90.09999999999999</v>
       </c>
       <c r="N3" t="n">
-        <v>83.8</v>
+        <v>49.6</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -729,7 +729,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>38.5</v>
+        <v>39.5</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -751,25 +751,21 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U3" t="inlineStr"/>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PNC</t>
+          <t>HD</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>327.49</v>
+        <v>367.11</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -802,22 +798,22 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>86.5</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="J4" t="n">
-        <v>64.40000000000001</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="K4" t="n">
-        <v>97.59999999999999</v>
+        <v>96.5</v>
       </c>
       <c r="L4" t="n">
-        <v>10.49</v>
+        <v>5.57</v>
       </c>
       <c r="M4" t="n">
-        <v>98.09999999999999</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="N4" t="n">
-        <v>83.8</v>
+        <v>33.8</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -825,7 +821,7 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>38.5</v>
+        <v>46.9</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -834,38 +830,34 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SPG</t>
+          <t>HUM</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>327.49</v>
+        <v>367.11</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -898,22 +890,22 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>86.5</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="J5" t="n">
-        <v>64.40000000000001</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="K5" t="n">
-        <v>97.59999999999999</v>
+        <v>96.5</v>
       </c>
       <c r="L5" t="n">
-        <v>10.49</v>
+        <v>5.57</v>
       </c>
       <c r="M5" t="n">
-        <v>98.09999999999999</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="N5" t="n">
-        <v>83.8</v>
+        <v>33.8</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -921,7 +913,7 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>38.5</v>
+        <v>46.9</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -930,38 +922,34 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SRE</t>
+          <t>GS</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>327.49</v>
+        <v>367.11</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -994,30 +982,30 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>86.5</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="J6" t="n">
-        <v>64.40000000000001</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="K6" t="n">
-        <v>97.59999999999999</v>
+        <v>96.5</v>
       </c>
       <c r="L6" t="n">
-        <v>10.49</v>
+        <v>5.57</v>
       </c>
       <c r="M6" t="n">
-        <v>98.09999999999999</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="N6" t="n">
-        <v>83.8</v>
+        <v>33.8</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P6" t="n">
-        <v>53.8</v>
+        <v>46.9</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1026,38 +1014,34 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr"/>
       <c r="V6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SNPS</t>
+          <t>HSY</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>327.49</v>
+        <v>367.11</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1090,22 +1074,22 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>86.5</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="J7" t="n">
-        <v>64.40000000000001</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="K7" t="n">
-        <v>97.59999999999999</v>
+        <v>96.5</v>
       </c>
       <c r="L7" t="n">
-        <v>10.49</v>
+        <v>5.57</v>
       </c>
       <c r="M7" t="n">
-        <v>98.09999999999999</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="N7" t="n">
-        <v>83.8</v>
+        <v>33.8</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1113,7 +1097,7 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>38.5</v>
+        <v>46.9</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1122,38 +1106,34 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr"/>
       <c r="V7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>IBM</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>131.45</v>
+        <v>367.11</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1186,22 +1166,22 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>69.2</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="J8" t="n">
-        <v>62.9</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="K8" t="n">
-        <v>81</v>
+        <v>96.5</v>
       </c>
       <c r="L8" t="n">
-        <v>1.9</v>
+        <v>5.57</v>
       </c>
       <c r="M8" t="n">
-        <v>18.9</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="N8" t="n">
-        <v>46.8</v>
+        <v>33.8</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1209,7 +1189,7 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>44.3</v>
+        <v>46.9</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1218,17 +1198,17 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U8" t="inlineStr"/>
@@ -1241,11 +1221,11 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>BMY</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>131.45</v>
+        <v>367.11</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1278,19 +1258,22 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>69.2</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="J9" t="n">
-        <v>62.9</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="K9" t="n">
-        <v>81</v>
+        <v>96.5</v>
       </c>
       <c r="L9" t="n">
-        <v>1.9</v>
+        <v>5.57</v>
       </c>
       <c r="M9" t="n">
-        <v>32.6</v>
+        <v>65.90000000000001</v>
+      </c>
+      <c r="N9" t="n">
+        <v>33.8</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1298,7 +1281,7 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>44.3</v>
+        <v>46.9</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1307,17 +1290,17 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U9" t="inlineStr"/>
@@ -1330,11 +1313,11 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>BK</t>
+          <t>GPN</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>131.45</v>
+        <v>367.11</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1367,19 +1350,19 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>69.2</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="J10" t="n">
-        <v>62.9</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="K10" t="n">
-        <v>81</v>
+        <v>96.5</v>
       </c>
       <c r="L10" t="n">
-        <v>1.9</v>
+        <v>5.57</v>
       </c>
       <c r="M10" t="n">
-        <v>44.3</v>
+        <v>42.4</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1387,7 +1370,7 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>44.3</v>
+        <v>46.9</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1396,17 +1379,17 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U10" t="inlineStr"/>
@@ -1419,11 +1402,11 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>COST</t>
+          <t>ICE</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>131.45</v>
+        <v>367.11</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1456,19 +1439,19 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>69.2</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="J11" t="n">
-        <v>62.9</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="K11" t="n">
-        <v>81</v>
+        <v>96.5</v>
       </c>
       <c r="L11" t="n">
-        <v>1.9</v>
+        <v>5.57</v>
       </c>
       <c r="M11" t="n">
-        <v>26</v>
+        <v>30.3</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1476,7 +1459,7 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>44.3</v>
+        <v>46.9</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1485,17 +1468,17 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U11" t="inlineStr"/>
@@ -1508,11 +1491,11 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>GM</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>131.45</v>
+        <v>367.11</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1545,19 +1528,22 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>69.2</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="J12" t="n">
-        <v>62.9</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="K12" t="n">
-        <v>81</v>
+        <v>96.5</v>
       </c>
       <c r="L12" t="n">
-        <v>1.9</v>
+        <v>5.57</v>
       </c>
       <c r="M12" t="n">
-        <v>42.1</v>
+        <v>65.90000000000001</v>
+      </c>
+      <c r="N12" t="n">
+        <v>33.8</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1565,7 +1551,7 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>44.4</v>
+        <v>46.9</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1574,17 +1560,17 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U12" t="inlineStr"/>
@@ -1597,11 +1583,11 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>COP</t>
+          <t>HON</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>131.45</v>
+        <v>367.11</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -1634,22 +1620,19 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>69.2</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="J13" t="n">
-        <v>62.9</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="K13" t="n">
-        <v>81</v>
+        <v>96.5</v>
       </c>
       <c r="L13" t="n">
-        <v>1.9</v>
+        <v>5.57</v>
       </c>
       <c r="M13" t="n">
-        <v>18.9</v>
-      </c>
-      <c r="N13" t="n">
-        <v>46.8</v>
+        <v>27.9</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1657,7 +1640,7 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>44.1</v>
+        <v>46.9</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1666,17 +1649,17 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U13" t="inlineStr"/>
@@ -1689,11 +1672,11 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>GLD</t>
+          <t>ECL</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>317.85</v>
+        <v>375.46</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -1726,27 +1709,30 @@
         </is>
       </c>
       <c r="I14" t="n">
-        <v>59.8</v>
+        <v>76</v>
       </c>
       <c r="J14" t="n">
-        <v>54.9</v>
+        <v>63.7</v>
       </c>
       <c r="K14" t="n">
-        <v>77</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="L14" t="n">
-        <v>4.3</v>
+        <v>5.26</v>
       </c>
       <c r="M14" t="n">
-        <v>30.1</v>
+        <v>65.59999999999999</v>
+      </c>
+      <c r="N14" t="n">
+        <v>80.8</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P14" t="n">
-        <v>43.7</v>
+        <v>42</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1778,11 +1764,11 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>TTWO</t>
+          <t>EOG</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>317.85</v>
+        <v>375.46</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1815,22 +1801,22 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>59.8</v>
+        <v>76</v>
       </c>
       <c r="J15" t="n">
-        <v>54.9</v>
+        <v>63.7</v>
       </c>
       <c r="K15" t="n">
-        <v>77</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="L15" t="n">
-        <v>4.3</v>
+        <v>5.26</v>
       </c>
       <c r="M15" t="n">
-        <v>48</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="N15" t="n">
-        <v>31.4</v>
+        <v>80.8</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1838,7 +1824,7 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>47.4</v>
+        <v>41</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1870,11 +1856,11 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>TEAM</t>
+          <t>TSLA</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>317.85</v>
+        <v>724.8</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -1907,27 +1893,30 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>59.8</v>
+        <v>74.7</v>
       </c>
       <c r="J16" t="n">
-        <v>54.9</v>
+        <v>66.7</v>
       </c>
       <c r="K16" t="n">
-        <v>77</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="L16" t="n">
-        <v>4.3</v>
+        <v>7.01</v>
       </c>
       <c r="M16" t="n">
-        <v>72.90000000000001</v>
+        <v>74.59999999999999</v>
+      </c>
+      <c r="N16" t="n">
+        <v>96.5</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>47.4</v>
+        <v>55.7</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1936,17 +1925,17 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U16" t="inlineStr"/>
@@ -1959,15 +1948,15 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>SYY</t>
+          <t>TDG</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>55.93</v>
+        <v>724.8</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -1982,36 +1971,36 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>52.6</v>
+        <v>74.7</v>
       </c>
       <c r="J17" t="n">
-        <v>38.5</v>
+        <v>66.7</v>
       </c>
       <c r="K17" t="n">
-        <v>9.4</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="L17" t="n">
-        <v>8.33</v>
+        <v>7.01</v>
       </c>
       <c r="M17" t="n">
-        <v>76</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="N17" t="n">
-        <v>39.2</v>
+        <v>96.5</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -2019,11 +2008,11 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>50.3</v>
+        <v>55.7</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
@@ -2033,7 +2022,7 @@
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
@@ -2041,29 +2030,25 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U17" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U17" t="inlineStr"/>
       <c r="V17" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>TDG</t>
+          <t>TJX</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>55.93</v>
+        <v>724.8</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -2078,45 +2063,48 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>52.6</v>
+        <v>74.7</v>
       </c>
       <c r="J18" t="n">
-        <v>38.5</v>
+        <v>66.7</v>
       </c>
       <c r="K18" t="n">
-        <v>9.4</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="L18" t="n">
-        <v>8.33</v>
+        <v>7.01</v>
       </c>
       <c r="M18" t="n">
-        <v>33.5</v>
+        <v>74.59999999999999</v>
+      </c>
+      <c r="N18" t="n">
+        <v>96.5</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P18" t="n">
-        <v>50.3</v>
+        <v>37.5</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
@@ -2126,7 +2114,7 @@
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
@@ -2134,29 +2122,25 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U18" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U18" t="inlineStr"/>
       <c r="V18" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>TJX</t>
+          <t>TXN</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>55.93</v>
+        <v>724.8</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -2171,36 +2155,36 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>52.6</v>
+        <v>74.7</v>
       </c>
       <c r="J19" t="n">
-        <v>38.5</v>
+        <v>66.7</v>
       </c>
       <c r="K19" t="n">
-        <v>9.4</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="L19" t="n">
-        <v>8.33</v>
+        <v>7.01</v>
       </c>
       <c r="M19" t="n">
-        <v>76</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="N19" t="n">
-        <v>39.2</v>
+        <v>96.5</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -2208,11 +2192,11 @@
         </is>
       </c>
       <c r="P19" t="n">
-        <v>50.3</v>
+        <v>52.8</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
@@ -2222,7 +2206,7 @@
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
@@ -2230,29 +2214,25 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U19" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U19" t="inlineStr"/>
       <c r="V19" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>SCHW</t>
+          <t>TSN</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>55.93</v>
+        <v>724.8</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -2267,36 +2247,36 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I20" t="n">
-        <v>52.6</v>
+        <v>74.7</v>
       </c>
       <c r="J20" t="n">
-        <v>38.5</v>
+        <v>66.7</v>
       </c>
       <c r="K20" t="n">
-        <v>9.4</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="L20" t="n">
-        <v>8.33</v>
+        <v>7.01</v>
       </c>
       <c r="M20" t="n">
-        <v>76</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="N20" t="n">
-        <v>39.2</v>
+        <v>96.5</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -2304,11 +2284,11 @@
         </is>
       </c>
       <c r="P20" t="n">
-        <v>53.8</v>
+        <v>55.7</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
@@ -2318,7 +2298,7 @@
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
@@ -2326,29 +2306,25 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U20" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U20" t="inlineStr"/>
       <c r="V20" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>TGT</t>
+          <t>SYK</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>55.93</v>
+        <v>724.8</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -2363,36 +2339,36 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>52.6</v>
+        <v>74.7</v>
       </c>
       <c r="J21" t="n">
-        <v>38.5</v>
+        <v>66.7</v>
       </c>
       <c r="K21" t="n">
-        <v>9.4</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="L21" t="n">
-        <v>8.33</v>
+        <v>7.01</v>
       </c>
       <c r="M21" t="n">
-        <v>76</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="N21" t="n">
-        <v>39.2</v>
+        <v>96.5</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
@@ -2400,11 +2376,11 @@
         </is>
       </c>
       <c r="P21" t="n">
-        <v>53.8</v>
+        <v>52.8</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
@@ -2414,22 +2390,1386 @@
       </c>
       <c r="S21" t="inlineStr">
         <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr"/>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>SYY</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>724.8</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>74.7</v>
+      </c>
+      <c r="J22" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="K22" t="n">
+        <v>74.40000000000001</v>
+      </c>
+      <c r="L22" t="n">
+        <v>7.01</v>
+      </c>
+      <c r="M22" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P22" t="n">
+        <v>52.8</v>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr"/>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>EQR</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>326.7</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>73.40000000000001</v>
+      </c>
+      <c r="J23" t="n">
+        <v>61.6</v>
+      </c>
+      <c r="K23" t="n">
+        <v>96.5</v>
+      </c>
+      <c r="L23" t="n">
+        <v>3.78</v>
+      </c>
+      <c r="M23" t="n">
+        <v>41.3</v>
+      </c>
+      <c r="N23" t="n">
+        <v>67.8</v>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P23" t="n">
+        <v>42</v>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr"/>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>EMR</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>326.7</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>73.40000000000001</v>
+      </c>
+      <c r="J24" t="n">
+        <v>61.6</v>
+      </c>
+      <c r="K24" t="n">
+        <v>96.5</v>
+      </c>
+      <c r="L24" t="n">
+        <v>3.78</v>
+      </c>
+      <c r="M24" t="n">
+        <v>41.3</v>
+      </c>
+      <c r="N24" t="n">
+        <v>67.8</v>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P24" t="n">
+        <v>42</v>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr"/>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>MCO</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>304.8</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>64.8</v>
+      </c>
+      <c r="J25" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="K25" t="n">
+        <v>98</v>
+      </c>
+      <c r="L25" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="M25" t="n">
+        <v>37.3</v>
+      </c>
+      <c r="N25" t="n">
+        <v>42.2</v>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P25" t="n">
+        <v>56.2</v>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
           <t>red</t>
         </is>
       </c>
-      <c r="T21" t="inlineStr">
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr"/>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>MDLZ</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>304.8</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>64.8</v>
+      </c>
+      <c r="J26" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="K26" t="n">
+        <v>98</v>
+      </c>
+      <c r="L26" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="M26" t="n">
+        <v>37.3</v>
+      </c>
+      <c r="N26" t="n">
+        <v>42.2</v>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P26" t="n">
+        <v>56.2</v>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr"/>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>MDT</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>304.8</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>64.8</v>
+      </c>
+      <c r="J27" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="K27" t="n">
+        <v>98</v>
+      </c>
+      <c r="L27" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="M27" t="n">
+        <v>37.3</v>
+      </c>
+      <c r="N27" t="n">
+        <v>42.2</v>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P27" t="n">
+        <v>56.2</v>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr"/>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>MCK</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>304.8</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>64.8</v>
+      </c>
+      <c r="J28" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="K28" t="n">
+        <v>98</v>
+      </c>
+      <c r="L28" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="M28" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P28" t="n">
+        <v>56.2</v>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr"/>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>NSC</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>48.67</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>63.6</v>
+      </c>
+      <c r="J29" t="n">
+        <v>36.7</v>
+      </c>
+      <c r="K29" t="n">
+        <v>94</v>
+      </c>
+      <c r="L29" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="M29" t="n">
+        <v>28.9</v>
+      </c>
+      <c r="N29" t="n">
+        <v>39.6</v>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P29" t="n">
+        <v>54.1</v>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr"/>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>NOC</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>48.67</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>63.6</v>
+      </c>
+      <c r="J30" t="n">
+        <v>36.7</v>
+      </c>
+      <c r="K30" t="n">
+        <v>94</v>
+      </c>
+      <c r="L30" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="M30" t="n">
+        <v>28.9</v>
+      </c>
+      <c r="N30" t="n">
+        <v>39.6</v>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P30" t="n">
+        <v>54.1</v>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr"/>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>48.67</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>63.6</v>
+      </c>
+      <c r="J31" t="n">
+        <v>36.7</v>
+      </c>
+      <c r="K31" t="n">
+        <v>94</v>
+      </c>
+      <c r="L31" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="M31" t="n">
+        <v>28.9</v>
+      </c>
+      <c r="N31" t="n">
+        <v>39.6</v>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P31" t="n">
+        <v>49.2</v>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr"/>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>NKE</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>48.67</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>63.6</v>
+      </c>
+      <c r="J32" t="n">
+        <v>36.7</v>
+      </c>
+      <c r="K32" t="n">
+        <v>94</v>
+      </c>
+      <c r="L32" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="M32" t="n">
+        <v>28.9</v>
+      </c>
+      <c r="N32" t="n">
+        <v>39.6</v>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P32" t="n">
+        <v>54.1</v>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr"/>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>48.67</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>63.6</v>
+      </c>
+      <c r="J33" t="n">
+        <v>36.7</v>
+      </c>
+      <c r="K33" t="n">
+        <v>94</v>
+      </c>
+      <c r="L33" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="M33" t="n">
+        <v>51.7</v>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P33" t="n">
+        <v>54.1</v>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr"/>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>48.67</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>63.6</v>
+      </c>
+      <c r="J34" t="n">
+        <v>36.7</v>
+      </c>
+      <c r="K34" t="n">
+        <v>94</v>
+      </c>
+      <c r="L34" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="M34" t="n">
+        <v>68.5</v>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P34" t="n">
+        <v>49.2</v>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr"/>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>NEE</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>48.67</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>63.6</v>
+      </c>
+      <c r="J35" t="n">
+        <v>36.7</v>
+      </c>
+      <c r="K35" t="n">
+        <v>94</v>
+      </c>
+      <c r="L35" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="M35" t="n">
+        <v>28.9</v>
+      </c>
+      <c r="N35" t="n">
+        <v>39.6</v>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P35" t="n">
+        <v>54.1</v>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr"/>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>SPG</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>109.79</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>57.7</v>
+      </c>
+      <c r="J36" t="n">
+        <v>45.1</v>
+      </c>
+      <c r="K36" t="n">
+        <v>71</v>
+      </c>
+      <c r="L36" t="n">
+        <v>4.09</v>
+      </c>
+      <c r="M36" t="n">
+        <v>40.6</v>
+      </c>
+      <c r="N36" t="n">
+        <v>55.8</v>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P36" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="U21" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
-      <c r="V21" t="inlineStr">
-        <is>
-          <t>Yes</t>
+      <c r="U36" t="inlineStr"/>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan 11.03.2026 14:56 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V36"/>
+  <dimension ref="A1:V29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -444,7 +444,7 @@
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="6" customWidth="1" min="10" max="10"/>
@@ -458,7 +458,7 @@
     <col width="15" customWidth="1" min="18" max="18"/>
     <col width="11" customWidth="1" min="19" max="19"/>
     <col width="11" customWidth="1" min="20" max="20"/>
-    <col width="10" customWidth="1" min="21" max="21"/>
+    <col width="25" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
@@ -577,11 +577,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BKNG</t>
+          <t>GLD</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>349.44</v>
+        <v>350.23</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,30 +614,27 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>80.90000000000001</v>
+        <v>81.40000000000001</v>
       </c>
       <c r="J2" t="n">
-        <v>67.90000000000001</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="K2" t="n">
-        <v>95.3</v>
+        <v>96.5</v>
       </c>
       <c r="L2" t="n">
-        <v>9.609999999999999</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="M2" t="n">
-        <v>90.09999999999999</v>
-      </c>
-      <c r="N2" t="n">
-        <v>49.6</v>
+        <v>28.5</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>48.3</v>
+        <v>47.3</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -669,11 +666,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CAT</t>
+          <t>TSN</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>349.44</v>
+        <v>213.4</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -706,30 +703,30 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>80.90000000000001</v>
+        <v>78.3</v>
       </c>
       <c r="J3" t="n">
-        <v>67.90000000000001</v>
+        <v>85.2</v>
       </c>
       <c r="K3" t="n">
-        <v>95.3</v>
+        <v>88.40000000000001</v>
       </c>
       <c r="L3" t="n">
-        <v>9.609999999999999</v>
+        <v>4.44</v>
       </c>
       <c r="M3" t="n">
-        <v>90.09999999999999</v>
+        <v>37.3</v>
       </c>
       <c r="N3" t="n">
-        <v>49.6</v>
+        <v>0.1</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P3" t="n">
-        <v>39.5</v>
+        <v>49.4</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -738,17 +735,17 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U3" t="inlineStr"/>
@@ -761,11 +758,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>HD</t>
+          <t>V</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>367.11</v>
+        <v>213.4</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -798,30 +795,30 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>77.90000000000001</v>
+        <v>78.3</v>
       </c>
       <c r="J4" t="n">
-        <v>70.90000000000001</v>
+        <v>85.2</v>
       </c>
       <c r="K4" t="n">
-        <v>96.5</v>
+        <v>88.40000000000001</v>
       </c>
       <c r="L4" t="n">
-        <v>5.57</v>
+        <v>4.44</v>
       </c>
       <c r="M4" t="n">
-        <v>65.90000000000001</v>
+        <v>37.3</v>
       </c>
       <c r="N4" t="n">
-        <v>33.8</v>
+        <v>0.1</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P4" t="n">
-        <v>46.9</v>
+        <v>49.4</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -853,11 +850,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>HUM</t>
+          <t>UNP</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>367.11</v>
+        <v>213.4</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -890,22 +887,22 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>77.90000000000001</v>
+        <v>78.3</v>
       </c>
       <c r="J5" t="n">
-        <v>70.90000000000001</v>
+        <v>85.2</v>
       </c>
       <c r="K5" t="n">
-        <v>96.5</v>
+        <v>88.40000000000001</v>
       </c>
       <c r="L5" t="n">
-        <v>5.57</v>
+        <v>4.44</v>
       </c>
       <c r="M5" t="n">
-        <v>65.90000000000001</v>
+        <v>37.3</v>
       </c>
       <c r="N5" t="n">
-        <v>33.8</v>
+        <v>0.1</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -913,7 +910,7 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>46.9</v>
+        <v>37</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -945,11 +942,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>GS</t>
+          <t>XOM</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>367.11</v>
+        <v>100.91</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -978,26 +975,26 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>77.90000000000001</v>
+        <v>67.3</v>
       </c>
       <c r="J6" t="n">
-        <v>70.90000000000001</v>
+        <v>49.4</v>
       </c>
       <c r="K6" t="n">
-        <v>96.5</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="L6" t="n">
-        <v>5.57</v>
+        <v>6.82</v>
       </c>
       <c r="M6" t="n">
-        <v>65.90000000000001</v>
+        <v>67.5</v>
       </c>
       <c r="N6" t="n">
-        <v>33.8</v>
+        <v>48.9</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -1005,7 +1002,7 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>46.9</v>
+        <v>37</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1014,17 +1011,17 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
@@ -1037,11 +1034,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>HSY</t>
+          <t>WMT</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>367.11</v>
+        <v>100.91</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1070,26 +1067,26 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>77.90000000000001</v>
+        <v>67.3</v>
       </c>
       <c r="J7" t="n">
-        <v>70.90000000000001</v>
+        <v>49.4</v>
       </c>
       <c r="K7" t="n">
-        <v>96.5</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="L7" t="n">
-        <v>5.57</v>
+        <v>6.82</v>
       </c>
       <c r="M7" t="n">
-        <v>65.90000000000001</v>
+        <v>67.5</v>
       </c>
       <c r="N7" t="n">
-        <v>33.8</v>
+        <v>48.9</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1097,7 +1094,7 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>46.9</v>
+        <v>37</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1106,17 +1103,17 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U7" t="inlineStr"/>
@@ -1129,11 +1126,11 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>IBM</t>
+          <t>WFC</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>367.11</v>
+        <v>100.91</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1162,26 +1159,26 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>77.90000000000001</v>
+        <v>67.3</v>
       </c>
       <c r="J8" t="n">
-        <v>70.90000000000001</v>
+        <v>49.4</v>
       </c>
       <c r="K8" t="n">
-        <v>96.5</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="L8" t="n">
-        <v>5.57</v>
+        <v>6.82</v>
       </c>
       <c r="M8" t="n">
-        <v>65.90000000000001</v>
+        <v>67.5</v>
       </c>
       <c r="N8" t="n">
-        <v>33.8</v>
+        <v>48.9</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1189,7 +1186,7 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>46.9</v>
+        <v>37</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1198,17 +1195,17 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U8" t="inlineStr"/>
@@ -1221,59 +1218,59 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>CI</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>367.11</v>
+        <v>70.84999999999999</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>77.90000000000001</v>
+        <v>65.3</v>
       </c>
       <c r="J9" t="n">
-        <v>70.90000000000001</v>
+        <v>64.7</v>
       </c>
       <c r="K9" t="n">
-        <v>96.5</v>
+        <v>6</v>
       </c>
       <c r="L9" t="n">
-        <v>5.57</v>
+        <v>3</v>
       </c>
       <c r="M9" t="n">
-        <v>65.90000000000001</v>
+        <v>22.1</v>
       </c>
       <c r="N9" t="n">
-        <v>33.8</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1281,11 +1278,11 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>46.9</v>
+        <v>39.4</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -1300,10 +1297,14 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U9" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V9" t="inlineStr">
         <is>
           <t>No</t>
@@ -1313,68 +1314,71 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>GPN</t>
+          <t>CMCSA</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>367.11</v>
+        <v>70.84999999999999</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>77.90000000000001</v>
+        <v>65.3</v>
       </c>
       <c r="J10" t="n">
-        <v>70.90000000000001</v>
+        <v>64.7</v>
       </c>
       <c r="K10" t="n">
-        <v>96.5</v>
+        <v>6</v>
       </c>
       <c r="L10" t="n">
-        <v>5.57</v>
+        <v>3</v>
       </c>
       <c r="M10" t="n">
-        <v>42.4</v>
+        <v>22.1</v>
+      </c>
+      <c r="N10" t="n">
+        <v>9.199999999999999</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>46.9</v>
+        <v>49.2</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
@@ -1389,10 +1393,14 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U10" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V10" t="inlineStr">
         <is>
           <t>No</t>
@@ -1402,30 +1410,30 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ICE</t>
+          <t>TSLA</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>367.11</v>
+        <v>305.27</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1439,27 +1447,30 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>77.90000000000001</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="J11" t="n">
-        <v>70.90000000000001</v>
+        <v>34.5</v>
       </c>
       <c r="K11" t="n">
-        <v>96.5</v>
+        <v>96</v>
       </c>
       <c r="L11" t="n">
-        <v>5.57</v>
+        <v>3.24</v>
       </c>
       <c r="M11" t="n">
-        <v>30.3</v>
+        <v>37.4</v>
+      </c>
+      <c r="N11" t="n">
+        <v>42.6</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>46.9</v>
+        <v>85.2</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1468,12 +1479,12 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
@@ -1491,30 +1502,30 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>GM</t>
+          <t>SYY</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>367.11</v>
+        <v>305.27</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1528,22 +1539,22 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>77.90000000000001</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="J12" t="n">
-        <v>70.90000000000001</v>
+        <v>34.5</v>
       </c>
       <c r="K12" t="n">
-        <v>96.5</v>
+        <v>96</v>
       </c>
       <c r="L12" t="n">
-        <v>5.57</v>
+        <v>3.24</v>
       </c>
       <c r="M12" t="n">
-        <v>65.90000000000001</v>
+        <v>37.4</v>
       </c>
       <c r="N12" t="n">
-        <v>33.8</v>
+        <v>42.6</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1551,7 +1562,7 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>46.9</v>
+        <v>35.7</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1560,12 +1571,12 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
@@ -1583,30 +1594,30 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>HON</t>
+          <t>T</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>367.11</v>
+        <v>305.27</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1620,27 +1631,27 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>77.90000000000001</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="J13" t="n">
-        <v>70.90000000000001</v>
+        <v>34.5</v>
       </c>
       <c r="K13" t="n">
-        <v>96.5</v>
+        <v>96</v>
       </c>
       <c r="L13" t="n">
-        <v>5.57</v>
+        <v>3.24</v>
       </c>
       <c r="M13" t="n">
-        <v>27.9</v>
+        <v>29.2</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>46.9</v>
+        <v>85.2</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1649,12 +1660,12 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
@@ -1672,30 +1683,30 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ECL</t>
+          <t>CRWD</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>375.46</v>
+        <v>48.3</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1705,34 +1716,34 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>76</v>
+        <v>62.3</v>
       </c>
       <c r="J14" t="n">
-        <v>63.7</v>
+        <v>35.1</v>
       </c>
       <c r="K14" t="n">
-        <v>74.40000000000001</v>
+        <v>90</v>
       </c>
       <c r="L14" t="n">
-        <v>5.26</v>
+        <v>3.15</v>
       </c>
       <c r="M14" t="n">
-        <v>65.59999999999999</v>
+        <v>28.8</v>
       </c>
       <c r="N14" t="n">
-        <v>80.8</v>
+        <v>39.2</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P14" t="n">
-        <v>42</v>
+        <v>36.2</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1741,12 +1752,12 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
@@ -1764,30 +1775,30 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>EOG</t>
+          <t>BKR</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>375.46</v>
+        <v>48.3</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1797,34 +1808,34 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>76</v>
+        <v>62.3</v>
       </c>
       <c r="J15" t="n">
-        <v>63.7</v>
+        <v>35.1</v>
       </c>
       <c r="K15" t="n">
-        <v>74.40000000000001</v>
+        <v>90</v>
       </c>
       <c r="L15" t="n">
-        <v>5.26</v>
+        <v>3.15</v>
       </c>
       <c r="M15" t="n">
-        <v>65.59999999999999</v>
+        <v>28.8</v>
       </c>
       <c r="N15" t="n">
-        <v>80.8</v>
+        <v>39.2</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P15" t="n">
-        <v>41</v>
+        <v>36.2</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1833,12 +1844,12 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
@@ -1856,15 +1867,15 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>TSLA</t>
+          <t>IWM</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>724.8</v>
+        <v>491.45</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -1879,36 +1890,33 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>74.7</v>
+        <v>62.1</v>
       </c>
       <c r="J16" t="n">
-        <v>66.7</v>
+        <v>48</v>
       </c>
       <c r="K16" t="n">
-        <v>74.40000000000001</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="L16" t="n">
-        <v>7.01</v>
+        <v>3.44</v>
       </c>
       <c r="M16" t="n">
-        <v>74.59999999999999</v>
-      </c>
-      <c r="N16" t="n">
-        <v>96.5</v>
+        <v>27.7</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -1916,11 +1924,11 @@
         </is>
       </c>
       <c r="P16" t="n">
-        <v>55.7</v>
+        <v>49.8</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
@@ -1938,7 +1946,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U16" t="inlineStr"/>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V16" t="inlineStr">
         <is>
           <t>No</t>
@@ -1948,11 +1960,11 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>TDG</t>
+          <t>CSCO</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>724.8</v>
+        <v>131.93</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -1985,22 +1997,22 @@
         </is>
       </c>
       <c r="I17" t="n">
-        <v>74.7</v>
+        <v>55.9</v>
       </c>
       <c r="J17" t="n">
-        <v>66.7</v>
+        <v>63.9</v>
       </c>
       <c r="K17" t="n">
-        <v>74.40000000000001</v>
+        <v>59</v>
       </c>
       <c r="L17" t="n">
-        <v>7.01</v>
+        <v>1.74</v>
       </c>
       <c r="M17" t="n">
-        <v>74.59999999999999</v>
+        <v>18.7</v>
       </c>
       <c r="N17" t="n">
-        <v>96.5</v>
+        <v>45</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -2008,7 +2020,7 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>55.7</v>
+        <v>49.2</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -2040,11 +2052,11 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>TJX</t>
+          <t>DHR</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>724.8</v>
+        <v>131.93</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -2077,30 +2089,30 @@
         </is>
       </c>
       <c r="I18" t="n">
-        <v>74.7</v>
+        <v>55.9</v>
       </c>
       <c r="J18" t="n">
-        <v>66.7</v>
+        <v>63.9</v>
       </c>
       <c r="K18" t="n">
-        <v>74.40000000000001</v>
+        <v>59</v>
       </c>
       <c r="L18" t="n">
-        <v>7.01</v>
+        <v>1.74</v>
       </c>
       <c r="M18" t="n">
-        <v>74.59999999999999</v>
+        <v>18.7</v>
       </c>
       <c r="N18" t="n">
-        <v>96.5</v>
+        <v>45</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P18" t="n">
-        <v>37.5</v>
+        <v>49.2</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -2132,11 +2144,11 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>TXN</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>724.8</v>
+        <v>131.93</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -2169,30 +2181,30 @@
         </is>
       </c>
       <c r="I19" t="n">
-        <v>74.7</v>
+        <v>55.9</v>
       </c>
       <c r="J19" t="n">
-        <v>66.7</v>
+        <v>63.9</v>
       </c>
       <c r="K19" t="n">
-        <v>74.40000000000001</v>
+        <v>59</v>
       </c>
       <c r="L19" t="n">
-        <v>7.01</v>
+        <v>1.74</v>
       </c>
       <c r="M19" t="n">
-        <v>74.59999999999999</v>
+        <v>18.7</v>
       </c>
       <c r="N19" t="n">
-        <v>96.5</v>
+        <v>45</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P19" t="n">
-        <v>52.8</v>
+        <v>42</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -2224,11 +2236,11 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>TSN</t>
+          <t>CVS</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>724.8</v>
+        <v>131.93</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -2261,30 +2273,27 @@
         </is>
       </c>
       <c r="I20" t="n">
-        <v>74.7</v>
+        <v>55.9</v>
       </c>
       <c r="J20" t="n">
-        <v>66.7</v>
+        <v>63.9</v>
       </c>
       <c r="K20" t="n">
-        <v>74.40000000000001</v>
+        <v>59</v>
       </c>
       <c r="L20" t="n">
-        <v>7.01</v>
+        <v>1.74</v>
       </c>
       <c r="M20" t="n">
-        <v>74.59999999999999</v>
-      </c>
-      <c r="N20" t="n">
-        <v>96.5</v>
+        <v>42.8</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P20" t="n">
-        <v>55.7</v>
+        <v>42</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
@@ -2316,11 +2325,11 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>SYK</t>
+          <t>DIS</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>724.8</v>
+        <v>131.93</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -2353,30 +2362,30 @@
         </is>
       </c>
       <c r="I21" t="n">
-        <v>74.7</v>
+        <v>55.9</v>
       </c>
       <c r="J21" t="n">
-        <v>66.7</v>
+        <v>63.9</v>
       </c>
       <c r="K21" t="n">
-        <v>74.40000000000001</v>
+        <v>59</v>
       </c>
       <c r="L21" t="n">
-        <v>7.01</v>
+        <v>1.74</v>
       </c>
       <c r="M21" t="n">
-        <v>74.59999999999999</v>
+        <v>18.7</v>
       </c>
       <c r="N21" t="n">
-        <v>96.5</v>
+        <v>45</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P21" t="n">
-        <v>52.8</v>
+        <v>42</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
@@ -2408,30 +2417,30 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>SYY</t>
+          <t>NXPI</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>724.8</v>
+        <v>109.02</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -2445,27 +2454,30 @@
         </is>
       </c>
       <c r="I22" t="n">
-        <v>74.7</v>
+        <v>52.6</v>
       </c>
       <c r="J22" t="n">
-        <v>66.7</v>
+        <v>43.7</v>
       </c>
       <c r="K22" t="n">
-        <v>74.40000000000001</v>
+        <v>56</v>
       </c>
       <c r="L22" t="n">
-        <v>7.01</v>
+        <v>3.89</v>
       </c>
       <c r="M22" t="n">
-        <v>25.8</v>
+        <v>40.1</v>
+      </c>
+      <c r="N22" t="n">
+        <v>54.7</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P22" t="n">
-        <v>52.8</v>
+        <v>48</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
@@ -2479,12 +2491,12 @@
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U22" t="inlineStr"/>
@@ -2497,30 +2509,30 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>EQR</t>
+          <t>MNST</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>326.7</v>
+        <v>109.02</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2530,34 +2542,31 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I23" t="n">
-        <v>73.40000000000001</v>
+        <v>52.6</v>
       </c>
       <c r="J23" t="n">
-        <v>61.6</v>
+        <v>43.7</v>
       </c>
       <c r="K23" t="n">
-        <v>96.5</v>
+        <v>56</v>
       </c>
       <c r="L23" t="n">
-        <v>3.78</v>
+        <v>3.89</v>
       </c>
       <c r="M23" t="n">
-        <v>41.3</v>
-      </c>
-      <c r="N23" t="n">
-        <v>67.8</v>
+        <v>28.2</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P23" t="n">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
@@ -2571,12 +2580,12 @@
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U23" t="inlineStr"/>
@@ -2589,30 +2598,30 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>EMR</t>
+          <t>TEAM</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>326.7</v>
+        <v>109.02</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -2622,34 +2631,31 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I24" t="n">
+        <v>52.6</v>
+      </c>
+      <c r="J24" t="n">
+        <v>43.7</v>
+      </c>
+      <c r="K24" t="n">
+        <v>56</v>
+      </c>
+      <c r="L24" t="n">
+        <v>3.89</v>
+      </c>
+      <c r="M24" t="n">
         <v>73.40000000000001</v>
       </c>
-      <c r="J24" t="n">
-        <v>61.6</v>
-      </c>
-      <c r="K24" t="n">
-        <v>96.5</v>
-      </c>
-      <c r="L24" t="n">
-        <v>3.78</v>
-      </c>
-      <c r="M24" t="n">
-        <v>41.3</v>
-      </c>
-      <c r="N24" t="n">
-        <v>67.8</v>
-      </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P24" t="n">
-        <v>42</v>
+        <v>49.8</v>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
@@ -2663,12 +2669,12 @@
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U24" t="inlineStr"/>
@@ -2681,11 +2687,11 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>MCO</t>
+          <t>ODFL</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>304.8</v>
+        <v>109.02</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -2714,26 +2720,23 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I25" t="n">
-        <v>64.8</v>
+        <v>52.6</v>
       </c>
       <c r="J25" t="n">
-        <v>33.3</v>
+        <v>43.7</v>
       </c>
       <c r="K25" t="n">
-        <v>98</v>
+        <v>56</v>
       </c>
       <c r="L25" t="n">
-        <v>3.5</v>
+        <v>3.89</v>
       </c>
       <c r="M25" t="n">
-        <v>37.3</v>
-      </c>
-      <c r="N25" t="n">
-        <v>42.2</v>
+        <v>49.5</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
@@ -2741,7 +2744,7 @@
         </is>
       </c>
       <c r="P25" t="n">
-        <v>56.2</v>
+        <v>49.8</v>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
@@ -2773,11 +2776,11 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>MDLZ</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>304.8</v>
+        <v>109.02</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -2806,26 +2809,23 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I26" t="n">
-        <v>64.8</v>
+        <v>52.6</v>
       </c>
       <c r="J26" t="n">
-        <v>33.3</v>
+        <v>43.7</v>
       </c>
       <c r="K26" t="n">
-        <v>98</v>
+        <v>56</v>
       </c>
       <c r="L26" t="n">
-        <v>3.5</v>
+        <v>3.89</v>
       </c>
       <c r="M26" t="n">
-        <v>37.3</v>
-      </c>
-      <c r="N26" t="n">
-        <v>42.2</v>
+        <v>58.5</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
@@ -2833,7 +2833,7 @@
         </is>
       </c>
       <c r="P26" t="n">
-        <v>56.2</v>
+        <v>49.8</v>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
@@ -2865,11 +2865,11 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>MDT</t>
+          <t>PAYX</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>304.8</v>
+        <v>109.02</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -2898,26 +2898,23 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I27" t="n">
-        <v>64.8</v>
+        <v>52.6</v>
       </c>
       <c r="J27" t="n">
-        <v>33.3</v>
+        <v>43.7</v>
       </c>
       <c r="K27" t="n">
-        <v>98</v>
+        <v>56</v>
       </c>
       <c r="L27" t="n">
-        <v>3.5</v>
+        <v>3.89</v>
       </c>
       <c r="M27" t="n">
-        <v>37.3</v>
-      </c>
-      <c r="N27" t="n">
-        <v>42.2</v>
+        <v>46.8</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -2925,7 +2922,7 @@
         </is>
       </c>
       <c r="P27" t="n">
-        <v>56.2</v>
+        <v>49.8</v>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
@@ -2957,11 +2954,11 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>MCK</t>
+          <t>FANG</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>304.8</v>
+        <v>163.01</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -2994,19 +2991,22 @@
         </is>
       </c>
       <c r="I28" t="n">
-        <v>64.8</v>
+        <v>49.9</v>
       </c>
       <c r="J28" t="n">
-        <v>33.3</v>
+        <v>37.4</v>
       </c>
       <c r="K28" t="n">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="L28" t="n">
-        <v>3.5</v>
+        <v>2.71</v>
       </c>
       <c r="M28" t="n">
-        <v>28.6</v>
+        <v>29.6</v>
+      </c>
+      <c r="N28" t="n">
+        <v>28.8</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
@@ -3014,7 +3014,7 @@
         </is>
       </c>
       <c r="P28" t="n">
-        <v>56.2</v>
+        <v>42.2</v>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
@@ -3028,7 +3028,7 @@
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T28" t="inlineStr">
@@ -3036,21 +3036,25 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U28" t="inlineStr"/>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V28" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>NSC</t>
+          <t>EA</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>48.67</v>
+        <v>163.01</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -3083,30 +3087,30 @@
         </is>
       </c>
       <c r="I29" t="n">
-        <v>63.6</v>
+        <v>49.9</v>
       </c>
       <c r="J29" t="n">
-        <v>36.7</v>
+        <v>37.4</v>
       </c>
       <c r="K29" t="n">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="L29" t="n">
-        <v>3.24</v>
+        <v>2.71</v>
       </c>
       <c r="M29" t="n">
-        <v>28.9</v>
+        <v>29.6</v>
       </c>
       <c r="N29" t="n">
-        <v>39.6</v>
+        <v>28.8</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P29" t="n">
-        <v>54.1</v>
+        <v>47.3</v>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
@@ -3120,7 +3124,7 @@
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T29" t="inlineStr">
@@ -3128,648 +3132,14 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U29" t="inlineStr"/>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V29" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>NOC</t>
-        </is>
-      </c>
-      <c r="B30" t="n">
-        <v>48.67</v>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D30" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I30" t="n">
-        <v>63.6</v>
-      </c>
-      <c r="J30" t="n">
-        <v>36.7</v>
-      </c>
-      <c r="K30" t="n">
-        <v>94</v>
-      </c>
-      <c r="L30" t="n">
-        <v>3.24</v>
-      </c>
-      <c r="M30" t="n">
-        <v>28.9</v>
-      </c>
-      <c r="N30" t="n">
-        <v>39.6</v>
-      </c>
-      <c r="O30" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P30" t="n">
-        <v>54.1</v>
-      </c>
-      <c r="Q30" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R30" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S30" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T30" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U30" t="inlineStr"/>
-      <c r="V30" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>NVDA</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>48.67</v>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D31" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I31" t="n">
-        <v>63.6</v>
-      </c>
-      <c r="J31" t="n">
-        <v>36.7</v>
-      </c>
-      <c r="K31" t="n">
-        <v>94</v>
-      </c>
-      <c r="L31" t="n">
-        <v>3.24</v>
-      </c>
-      <c r="M31" t="n">
-        <v>28.9</v>
-      </c>
-      <c r="N31" t="n">
-        <v>39.6</v>
-      </c>
-      <c r="O31" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P31" t="n">
-        <v>49.2</v>
-      </c>
-      <c r="Q31" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R31" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S31" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T31" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U31" t="inlineStr"/>
-      <c r="V31" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>NKE</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>48.67</v>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D32" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I32" t="n">
-        <v>63.6</v>
-      </c>
-      <c r="J32" t="n">
-        <v>36.7</v>
-      </c>
-      <c r="K32" t="n">
-        <v>94</v>
-      </c>
-      <c r="L32" t="n">
-        <v>3.24</v>
-      </c>
-      <c r="M32" t="n">
-        <v>28.9</v>
-      </c>
-      <c r="N32" t="n">
-        <v>39.6</v>
-      </c>
-      <c r="O32" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P32" t="n">
-        <v>54.1</v>
-      </c>
-      <c r="Q32" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R32" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S32" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T32" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U32" t="inlineStr"/>
-      <c r="V32" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>NOW</t>
-        </is>
-      </c>
-      <c r="B33" t="n">
-        <v>48.67</v>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D33" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I33" t="n">
-        <v>63.6</v>
-      </c>
-      <c r="J33" t="n">
-        <v>36.7</v>
-      </c>
-      <c r="K33" t="n">
-        <v>94</v>
-      </c>
-      <c r="L33" t="n">
-        <v>3.24</v>
-      </c>
-      <c r="M33" t="n">
-        <v>51.7</v>
-      </c>
-      <c r="O33" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P33" t="n">
-        <v>54.1</v>
-      </c>
-      <c r="Q33" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R33" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S33" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T33" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U33" t="inlineStr"/>
-      <c r="V33" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>ORCL</t>
-        </is>
-      </c>
-      <c r="B34" t="n">
-        <v>48.67</v>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D34" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I34" t="n">
-        <v>63.6</v>
-      </c>
-      <c r="J34" t="n">
-        <v>36.7</v>
-      </c>
-      <c r="K34" t="n">
-        <v>94</v>
-      </c>
-      <c r="L34" t="n">
-        <v>3.24</v>
-      </c>
-      <c r="M34" t="n">
-        <v>68.5</v>
-      </c>
-      <c r="O34" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P34" t="n">
-        <v>49.2</v>
-      </c>
-      <c r="Q34" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R34" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S34" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T34" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U34" t="inlineStr"/>
-      <c r="V34" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>NEE</t>
-        </is>
-      </c>
-      <c r="B35" t="n">
-        <v>48.67</v>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D35" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I35" t="n">
-        <v>63.6</v>
-      </c>
-      <c r="J35" t="n">
-        <v>36.7</v>
-      </c>
-      <c r="K35" t="n">
-        <v>94</v>
-      </c>
-      <c r="L35" t="n">
-        <v>3.24</v>
-      </c>
-      <c r="M35" t="n">
-        <v>28.9</v>
-      </c>
-      <c r="N35" t="n">
-        <v>39.6</v>
-      </c>
-      <c r="O35" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P35" t="n">
-        <v>54.1</v>
-      </c>
-      <c r="Q35" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R35" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S35" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T35" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U35" t="inlineStr"/>
-      <c r="V35" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>SPG</t>
-        </is>
-      </c>
-      <c r="B36" t="n">
-        <v>109.79</v>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D36" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I36" t="n">
-        <v>57.7</v>
-      </c>
-      <c r="J36" t="n">
-        <v>45.1</v>
-      </c>
-      <c r="K36" t="n">
-        <v>71</v>
-      </c>
-      <c r="L36" t="n">
-        <v>4.09</v>
-      </c>
-      <c r="M36" t="n">
-        <v>40.6</v>
-      </c>
-      <c r="N36" t="n">
-        <v>55.8</v>
-      </c>
-      <c r="O36" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P36" t="n">
-        <v>66.7</v>
-      </c>
-      <c r="Q36" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R36" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="S36" t="inlineStr">
-        <is>
-          <t>maroon</t>
-        </is>
-      </c>
-      <c r="T36" t="inlineStr">
-        <is>
           <t>Yes</t>
-        </is>
-      </c>
-      <c r="U36" t="inlineStr"/>
-      <c r="V36" t="inlineStr">
-        <is>
-          <t>No</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan 11.03.2026 18:12 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V29"/>
+  <dimension ref="A1:V19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -448,7 +448,7 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="6" customWidth="1" min="10" max="10"/>
-    <col width="6" customWidth="1" min="11" max="11"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
     <col width="6" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
     <col width="9" customWidth="1" min="14" max="14"/>
@@ -577,11 +577,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>GLD</t>
+          <t>HD</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>350.23</v>
+        <v>350.19</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -626,15 +626,18 @@
         <v>9.800000000000001</v>
       </c>
       <c r="M2" t="n">
-        <v>28.5</v>
+        <v>90.2</v>
+      </c>
+      <c r="N2" t="n">
+        <v>50.1</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>47.3</v>
+        <v>51.6</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -666,11 +669,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>TSN</t>
+          <t>ITW</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>213.4</v>
+        <v>350.19</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -703,30 +706,30 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>78.3</v>
+        <v>81.40000000000001</v>
       </c>
       <c r="J3" t="n">
-        <v>85.2</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="K3" t="n">
-        <v>88.40000000000001</v>
+        <v>96.5</v>
       </c>
       <c r="L3" t="n">
-        <v>4.44</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="M3" t="n">
-        <v>37.3</v>
+        <v>90.2</v>
       </c>
       <c r="N3" t="n">
-        <v>0.1</v>
+        <v>50.1</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P3" t="n">
-        <v>49.4</v>
+        <v>29.5</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -735,17 +738,17 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U3" t="inlineStr"/>
@@ -758,11 +761,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>INTC</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>213.4</v>
+        <v>350.19</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -795,30 +798,30 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>78.3</v>
+        <v>81.40000000000001</v>
       </c>
       <c r="J4" t="n">
-        <v>85.2</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="K4" t="n">
-        <v>88.40000000000001</v>
+        <v>96.5</v>
       </c>
       <c r="L4" t="n">
-        <v>4.44</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="M4" t="n">
-        <v>37.3</v>
+        <v>90.2</v>
       </c>
       <c r="N4" t="n">
-        <v>0.1</v>
+        <v>50.1</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P4" t="n">
-        <v>49.4</v>
+        <v>51.6</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -827,17 +830,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U4" t="inlineStr"/>
@@ -850,11 +853,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>UNP</t>
+          <t>IBM</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>213.4</v>
+        <v>350.19</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -887,30 +890,27 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>78.3</v>
+        <v>81.40000000000001</v>
       </c>
       <c r="J5" t="n">
-        <v>85.2</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="K5" t="n">
-        <v>88.40000000000001</v>
+        <v>96.5</v>
       </c>
       <c r="L5" t="n">
-        <v>4.44</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="M5" t="n">
-        <v>37.3</v>
-      </c>
-      <c r="N5" t="n">
-        <v>0.1</v>
+        <v>39.1</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>37</v>
+        <v>51.6</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -919,17 +919,17 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U5" t="inlineStr"/>
@@ -942,11 +942,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>XOM</t>
+          <t>GE</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>100.91</v>
+        <v>317.51</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -975,34 +975,34 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>67.3</v>
+        <v>78.3</v>
       </c>
       <c r="J6" t="n">
-        <v>49.4</v>
+        <v>61.5</v>
       </c>
       <c r="K6" t="n">
-        <v>75.59999999999999</v>
+        <v>96.5</v>
       </c>
       <c r="L6" t="n">
-        <v>6.82</v>
+        <v>6.66</v>
       </c>
       <c r="M6" t="n">
-        <v>67.5</v>
+        <v>78.7</v>
       </c>
       <c r="N6" t="n">
-        <v>48.9</v>
+        <v>52.9</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P6" t="n">
-        <v>37</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1034,11 +1034,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>WMT</t>
+          <t>MRK</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>100.91</v>
+        <v>375.87</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1071,22 +1071,22 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>67.3</v>
+        <v>76.8</v>
       </c>
       <c r="J7" t="n">
-        <v>49.4</v>
+        <v>63.8</v>
       </c>
       <c r="K7" t="n">
-        <v>75.59999999999999</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="L7" t="n">
-        <v>6.82</v>
+        <v>5.3</v>
       </c>
       <c r="M7" t="n">
-        <v>67.5</v>
+        <v>65.7</v>
       </c>
       <c r="N7" t="n">
-        <v>48.9</v>
+        <v>80.8</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1094,7 +1094,7 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>37</v>
+        <v>40.8</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1103,17 +1103,17 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U7" t="inlineStr"/>
@@ -1126,11 +1126,11 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>WFC</t>
+          <t>LULU</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>100.91</v>
+        <v>708.15</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1163,30 +1163,30 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>67.3</v>
+        <v>73.5</v>
       </c>
       <c r="J8" t="n">
-        <v>49.4</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="K8" t="n">
-        <v>75.59999999999999</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="L8" t="n">
-        <v>6.82</v>
+        <v>7.29</v>
       </c>
       <c r="M8" t="n">
-        <v>67.5</v>
+        <v>73.7</v>
       </c>
       <c r="N8" t="n">
-        <v>48.9</v>
+        <v>91.5</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>37</v>
+        <v>40.3</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1218,15 +1218,15 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CI</t>
+          <t>KO</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>70.84999999999999</v>
+        <v>212.82</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -1241,88 +1241,88 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>65.3</v>
+        <v>68</v>
       </c>
       <c r="J9" t="n">
-        <v>64.7</v>
+        <v>29.5</v>
       </c>
       <c r="K9" t="n">
-        <v>6</v>
+        <v>100</v>
       </c>
       <c r="L9" t="n">
-        <v>3</v>
+        <v>6.55</v>
       </c>
       <c r="M9" t="n">
-        <v>22.1</v>
+        <v>50.4</v>
       </c>
       <c r="N9" t="n">
-        <v>9.199999999999999</v>
+        <v>100</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>39.4</v>
+        <v>54.6</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
           <t>Yes</t>
-        </is>
-      </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
-      <c r="V9" t="inlineStr">
-        <is>
-          <t>No</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CMCSA</t>
+          <t>LIN</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>70.84999999999999</v>
+        <v>212.82</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -1337,84 +1337,84 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>65.3</v>
+        <v>68</v>
       </c>
       <c r="J10" t="n">
-        <v>64.7</v>
+        <v>29.5</v>
       </c>
       <c r="K10" t="n">
-        <v>6</v>
+        <v>100</v>
       </c>
       <c r="L10" t="n">
-        <v>3</v>
+        <v>6.55</v>
       </c>
       <c r="M10" t="n">
-        <v>22.1</v>
+        <v>50.4</v>
       </c>
       <c r="N10" t="n">
-        <v>9.199999999999999</v>
+        <v>100</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>49.2</v>
+        <v>52</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
           <t>Yes</t>
-        </is>
-      </c>
-      <c r="U10" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
-      <c r="V10" t="inlineStr">
-        <is>
-          <t>No</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>TSLA</t>
+          <t>JNJ</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>305.27</v>
+        <v>212.82</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1447,30 +1447,30 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>65.09999999999999</v>
+        <v>68</v>
       </c>
       <c r="J11" t="n">
-        <v>34.5</v>
+        <v>29.5</v>
       </c>
       <c r="K11" t="n">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="L11" t="n">
-        <v>3.24</v>
+        <v>6.55</v>
       </c>
       <c r="M11" t="n">
-        <v>37.4</v>
+        <v>50.4</v>
       </c>
       <c r="N11" t="n">
-        <v>42.6</v>
+        <v>100</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>85.2</v>
+        <v>32.5</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1492,21 +1492,25 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U11" t="inlineStr"/>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>SYY</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>305.27</v>
+        <v>302.8</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1539,30 +1543,30 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>65.09999999999999</v>
+        <v>64.3</v>
       </c>
       <c r="J12" t="n">
-        <v>34.5</v>
+        <v>32.5</v>
       </c>
       <c r="K12" t="n">
         <v>96</v>
       </c>
       <c r="L12" t="n">
-        <v>3.24</v>
+        <v>3.33</v>
       </c>
       <c r="M12" t="n">
-        <v>37.4</v>
+        <v>37.3</v>
       </c>
       <c r="N12" t="n">
-        <v>42.6</v>
+        <v>42.2</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>35.7</v>
+        <v>63.8</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1594,11 +1598,11 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>305.27</v>
+        <v>302.8</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -1631,19 +1635,19 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>65.09999999999999</v>
+        <v>64.3</v>
       </c>
       <c r="J13" t="n">
-        <v>34.5</v>
+        <v>32.5</v>
       </c>
       <c r="K13" t="n">
         <v>96</v>
       </c>
       <c r="L13" t="n">
-        <v>3.24</v>
+        <v>3.33</v>
       </c>
       <c r="M13" t="n">
-        <v>29.2</v>
+        <v>27.7</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1651,7 +1655,7 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>85.2</v>
+        <v>63.8</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1683,15 +1687,15 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CRWD</t>
+          <t>APH</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>48.3</v>
+        <v>70.5</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
@@ -1706,36 +1710,36 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>62.3</v>
+        <v>62</v>
       </c>
       <c r="J14" t="n">
-        <v>35.1</v>
+        <v>63.6</v>
       </c>
       <c r="K14" t="n">
-        <v>90</v>
+        <v>5</v>
       </c>
       <c r="L14" t="n">
-        <v>3.15</v>
+        <v>3.12</v>
       </c>
       <c r="M14" t="n">
-        <v>28.8</v>
+        <v>21.8</v>
       </c>
       <c r="N14" t="n">
-        <v>39.2</v>
+        <v>7.6</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1743,29 +1747,33 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>36.2</v>
+        <v>50.5</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U14" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V14" t="inlineStr">
         <is>
           <t>No</t>
@@ -1775,15 +1783,15 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>BKR</t>
+          <t>AMGN</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>48.3</v>
+        <v>70.5</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -1798,36 +1806,33 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>62.3</v>
+        <v>62</v>
       </c>
       <c r="J15" t="n">
-        <v>35.1</v>
+        <v>63.6</v>
       </c>
       <c r="K15" t="n">
-        <v>90</v>
+        <v>5</v>
       </c>
       <c r="L15" t="n">
-        <v>3.15</v>
+        <v>3.12</v>
       </c>
       <c r="M15" t="n">
-        <v>28.8</v>
-      </c>
-      <c r="N15" t="n">
-        <v>39.2</v>
+        <v>32.5</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1835,29 +1840,33 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>36.2</v>
+        <v>50.5</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U15" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V15" t="inlineStr">
         <is>
           <t>No</t>
@@ -1867,30 +1876,30 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>IWM</t>
+          <t>ADSK</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>491.45</v>
+        <v>70.5</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1904,27 +1913,27 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>62.1</v>
+        <v>62</v>
       </c>
       <c r="J16" t="n">
-        <v>48</v>
+        <v>63.6</v>
       </c>
       <c r="K16" t="n">
-        <v>9.300000000000001</v>
+        <v>5</v>
       </c>
       <c r="L16" t="n">
-        <v>3.44</v>
+        <v>3.12</v>
       </c>
       <c r="M16" t="n">
-        <v>27.7</v>
+        <v>43.7</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>49.8</v>
+        <v>39.4</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1933,12 +1942,12 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
@@ -1960,30 +1969,30 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>PSA</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>131.93</v>
+        <v>162.92</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1993,34 +2002,34 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>55.9</v>
+        <v>49.8</v>
       </c>
       <c r="J17" t="n">
-        <v>63.9</v>
+        <v>37.2</v>
       </c>
       <c r="K17" t="n">
-        <v>59</v>
+        <v>86</v>
       </c>
       <c r="L17" t="n">
-        <v>1.74</v>
+        <v>2.73</v>
       </c>
       <c r="M17" t="n">
-        <v>18.7</v>
+        <v>29.6</v>
       </c>
       <c r="N17" t="n">
-        <v>45</v>
+        <v>28.9</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P17" t="n">
-        <v>49.2</v>
+        <v>36.6</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -2039,43 +2048,47 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
           <t>Yes</t>
-        </is>
-      </c>
-      <c r="U17" t="inlineStr"/>
-      <c r="V17" t="inlineStr">
-        <is>
-          <t>No</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>DHR</t>
+          <t>PFE</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>131.93</v>
+        <v>162.92</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -2085,34 +2098,31 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>55.9</v>
+        <v>49.8</v>
       </c>
       <c r="J18" t="n">
-        <v>63.9</v>
+        <v>37.2</v>
       </c>
       <c r="K18" t="n">
-        <v>59</v>
+        <v>86</v>
       </c>
       <c r="L18" t="n">
-        <v>1.74</v>
+        <v>2.73</v>
       </c>
       <c r="M18" t="n">
-        <v>18.7</v>
-      </c>
-      <c r="N18" t="n">
-        <v>45</v>
+        <v>25.8</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P18" t="n">
-        <v>49.2</v>
+        <v>36.6</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -2131,43 +2141,47 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
           <t>Yes</t>
-        </is>
-      </c>
-      <c r="U18" t="inlineStr"/>
-      <c r="V18" t="inlineStr">
-        <is>
-          <t>No</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>PEP</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>131.93</v>
+        <v>162.92</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2177,26 +2191,26 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>55.9</v>
+        <v>49.8</v>
       </c>
       <c r="J19" t="n">
-        <v>63.9</v>
+        <v>37.2</v>
       </c>
       <c r="K19" t="n">
-        <v>59</v>
+        <v>86</v>
       </c>
       <c r="L19" t="n">
-        <v>1.74</v>
+        <v>2.73</v>
       </c>
       <c r="M19" t="n">
-        <v>18.7</v>
+        <v>29.6</v>
       </c>
       <c r="N19" t="n">
-        <v>45</v>
+        <v>28.9</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -2204,7 +2218,7 @@
         </is>
       </c>
       <c r="P19" t="n">
-        <v>42</v>
+        <v>36.6</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -2223,921 +2237,15 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U19" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V19" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>CVS</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>131.93</v>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Credit Call</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I20" t="n">
-        <v>55.9</v>
-      </c>
-      <c r="J20" t="n">
-        <v>63.9</v>
-      </c>
-      <c r="K20" t="n">
-        <v>59</v>
-      </c>
-      <c r="L20" t="n">
-        <v>1.74</v>
-      </c>
-      <c r="M20" t="n">
-        <v>42.8</v>
-      </c>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P20" t="n">
-        <v>42</v>
-      </c>
-      <c r="Q20" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R20" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S20" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="T20" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U20" t="inlineStr"/>
-      <c r="V20" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>DIS</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>131.93</v>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Credit Call</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I21" t="n">
-        <v>55.9</v>
-      </c>
-      <c r="J21" t="n">
-        <v>63.9</v>
-      </c>
-      <c r="K21" t="n">
-        <v>59</v>
-      </c>
-      <c r="L21" t="n">
-        <v>1.74</v>
-      </c>
-      <c r="M21" t="n">
-        <v>18.7</v>
-      </c>
-      <c r="N21" t="n">
-        <v>45</v>
-      </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P21" t="n">
-        <v>42</v>
-      </c>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S21" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="T21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U21" t="inlineStr"/>
-      <c r="V21" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>NXPI</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>109.02</v>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I22" t="n">
-        <v>52.6</v>
-      </c>
-      <c r="J22" t="n">
-        <v>43.7</v>
-      </c>
-      <c r="K22" t="n">
-        <v>56</v>
-      </c>
-      <c r="L22" t="n">
-        <v>3.89</v>
-      </c>
-      <c r="M22" t="n">
-        <v>40.1</v>
-      </c>
-      <c r="N22" t="n">
-        <v>54.7</v>
-      </c>
-      <c r="O22" t="inlineStr">
-        <is>
-          <t>Neutral</t>
-        </is>
-      </c>
-      <c r="P22" t="n">
-        <v>48</v>
-      </c>
-      <c r="Q22" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R22" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S22" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T22" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U22" t="inlineStr"/>
-      <c r="V22" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>MNST</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>109.02</v>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I23" t="n">
-        <v>52.6</v>
-      </c>
-      <c r="J23" t="n">
-        <v>43.7</v>
-      </c>
-      <c r="K23" t="n">
-        <v>56</v>
-      </c>
-      <c r="L23" t="n">
-        <v>3.89</v>
-      </c>
-      <c r="M23" t="n">
-        <v>28.2</v>
-      </c>
-      <c r="O23" t="inlineStr">
-        <is>
-          <t>Neutral</t>
-        </is>
-      </c>
-      <c r="P23" t="n">
-        <v>48</v>
-      </c>
-      <c r="Q23" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R23" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S23" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U23" t="inlineStr"/>
-      <c r="V23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>TEAM</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>109.02</v>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I24" t="n">
-        <v>52.6</v>
-      </c>
-      <c r="J24" t="n">
-        <v>43.7</v>
-      </c>
-      <c r="K24" t="n">
-        <v>56</v>
-      </c>
-      <c r="L24" t="n">
-        <v>3.89</v>
-      </c>
-      <c r="M24" t="n">
-        <v>73.40000000000001</v>
-      </c>
-      <c r="O24" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P24" t="n">
-        <v>49.8</v>
-      </c>
-      <c r="Q24" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R24" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S24" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T24" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U24" t="inlineStr"/>
-      <c r="V24" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>ODFL</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>109.02</v>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I25" t="n">
-        <v>52.6</v>
-      </c>
-      <c r="J25" t="n">
-        <v>43.7</v>
-      </c>
-      <c r="K25" t="n">
-        <v>56</v>
-      </c>
-      <c r="L25" t="n">
-        <v>3.89</v>
-      </c>
-      <c r="M25" t="n">
-        <v>49.5</v>
-      </c>
-      <c r="O25" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P25" t="n">
-        <v>49.8</v>
-      </c>
-      <c r="Q25" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R25" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S25" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T25" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U25" t="inlineStr"/>
-      <c r="V25" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>MRVL</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>109.02</v>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D26" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I26" t="n">
-        <v>52.6</v>
-      </c>
-      <c r="J26" t="n">
-        <v>43.7</v>
-      </c>
-      <c r="K26" t="n">
-        <v>56</v>
-      </c>
-      <c r="L26" t="n">
-        <v>3.89</v>
-      </c>
-      <c r="M26" t="n">
-        <v>58.5</v>
-      </c>
-      <c r="O26" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P26" t="n">
-        <v>49.8</v>
-      </c>
-      <c r="Q26" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R26" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S26" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T26" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U26" t="inlineStr"/>
-      <c r="V26" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>PAYX</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>109.02</v>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D27" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I27" t="n">
-        <v>52.6</v>
-      </c>
-      <c r="J27" t="n">
-        <v>43.7</v>
-      </c>
-      <c r="K27" t="n">
-        <v>56</v>
-      </c>
-      <c r="L27" t="n">
-        <v>3.89</v>
-      </c>
-      <c r="M27" t="n">
-        <v>46.8</v>
-      </c>
-      <c r="O27" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P27" t="n">
-        <v>49.8</v>
-      </c>
-      <c r="Q27" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R27" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S27" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T27" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U27" t="inlineStr"/>
-      <c r="V27" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>FANG</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
-        <v>163.01</v>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D28" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I28" t="n">
-        <v>49.9</v>
-      </c>
-      <c r="J28" t="n">
-        <v>37.4</v>
-      </c>
-      <c r="K28" t="n">
-        <v>86</v>
-      </c>
-      <c r="L28" t="n">
-        <v>2.71</v>
-      </c>
-      <c r="M28" t="n">
-        <v>29.6</v>
-      </c>
-      <c r="N28" t="n">
-        <v>28.8</v>
-      </c>
-      <c r="O28" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P28" t="n">
-        <v>42.2</v>
-      </c>
-      <c r="Q28" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R28" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S28" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="T28" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U28" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
-      <c r="V28" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>EA</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>163.01</v>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D29" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I29" t="n">
-        <v>49.9</v>
-      </c>
-      <c r="J29" t="n">
-        <v>37.4</v>
-      </c>
-      <c r="K29" t="n">
-        <v>86</v>
-      </c>
-      <c r="L29" t="n">
-        <v>2.71</v>
-      </c>
-      <c r="M29" t="n">
-        <v>29.6</v>
-      </c>
-      <c r="N29" t="n">
-        <v>28.8</v>
-      </c>
-      <c r="O29" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P29" t="n">
-        <v>47.3</v>
-      </c>
-      <c r="Q29" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R29" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S29" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="T29" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U29" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
-      <c r="V29" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>

</xml_diff>

<commit_message>
Scan 12.03.2026 14:59 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V19"/>
+  <dimension ref="A1:V47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -449,7 +449,7 @@
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="6" customWidth="1" min="10" max="10"/>
     <col width="7" customWidth="1" min="11" max="11"/>
-    <col width="6" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
     <col width="9" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
@@ -577,11 +577,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>HD</t>
+          <t>FANG</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>350.19</v>
+        <v>327.74</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,30 +614,30 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>81.40000000000001</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="J2" t="n">
-        <v>68.09999999999999</v>
+        <v>62.3</v>
       </c>
       <c r="K2" t="n">
         <v>96.5</v>
       </c>
       <c r="L2" t="n">
-        <v>9.800000000000001</v>
+        <v>3.84</v>
       </c>
       <c r="M2" t="n">
-        <v>90.2</v>
+        <v>41.3</v>
       </c>
       <c r="N2" t="n">
-        <v>50.1</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>51.6</v>
+        <v>40.6</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -646,17 +646,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
@@ -669,11 +669,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ITW</t>
+          <t>FAST</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>350.19</v>
+        <v>327.74</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -706,22 +706,22 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>81.40000000000001</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="J3" t="n">
-        <v>68.09999999999999</v>
+        <v>62.3</v>
       </c>
       <c r="K3" t="n">
         <v>96.5</v>
       </c>
       <c r="L3" t="n">
-        <v>9.800000000000001</v>
+        <v>3.84</v>
       </c>
       <c r="M3" t="n">
-        <v>90.2</v>
+        <v>41.3</v>
       </c>
       <c r="N3" t="n">
-        <v>50.1</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -729,7 +729,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>29.5</v>
+        <v>40.6</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -738,17 +738,17 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U3" t="inlineStr"/>
@@ -761,11 +761,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>INTC</t>
+          <t>DDOG</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>350.19</v>
+        <v>327.74</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -798,30 +798,27 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>81.40000000000001</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="J4" t="n">
-        <v>68.09999999999999</v>
+        <v>62.3</v>
       </c>
       <c r="K4" t="n">
         <v>96.5</v>
       </c>
       <c r="L4" t="n">
-        <v>9.800000000000001</v>
+        <v>3.84</v>
       </c>
       <c r="M4" t="n">
-        <v>90.2</v>
-      </c>
-      <c r="N4" t="n">
-        <v>50.1</v>
+        <v>55.4</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P4" t="n">
-        <v>51.6</v>
+        <v>40.6</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -830,17 +827,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U4" t="inlineStr"/>
@@ -853,11 +850,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>IBM</t>
+          <t>EW</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>350.19</v>
+        <v>370.86</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -886,23 +883,23 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>81.40000000000001</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="J5" t="n">
-        <v>68.09999999999999</v>
+        <v>62.6</v>
       </c>
       <c r="K5" t="n">
-        <v>96.5</v>
+        <v>69.8</v>
       </c>
       <c r="L5" t="n">
-        <v>9.800000000000001</v>
+        <v>5.37</v>
       </c>
       <c r="M5" t="n">
-        <v>39.1</v>
+        <v>37.1</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -910,7 +907,7 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>51.6</v>
+        <v>35.7</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -919,17 +916,17 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U5" t="inlineStr"/>
@@ -942,11 +939,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>GE</t>
+          <t>GILD</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>317.51</v>
+        <v>370.86</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -975,26 +972,23 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>78.3</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="J6" t="n">
-        <v>61.5</v>
+        <v>62.6</v>
       </c>
       <c r="K6" t="n">
-        <v>96.5</v>
+        <v>69.8</v>
       </c>
       <c r="L6" t="n">
-        <v>6.66</v>
+        <v>5.37</v>
       </c>
       <c r="M6" t="n">
-        <v>78.7</v>
-      </c>
-      <c r="N6" t="n">
-        <v>52.9</v>
+        <v>34.4</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -1002,7 +996,7 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>69.59999999999999</v>
+        <v>35.7</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1011,17 +1005,17 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
@@ -1034,11 +1028,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>MRK</t>
+          <t>GOOG</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>375.87</v>
+        <v>370.86</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1071,30 +1065,27 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>76.8</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="J7" t="n">
-        <v>63.8</v>
+        <v>62.6</v>
       </c>
       <c r="K7" t="n">
-        <v>74.40000000000001</v>
+        <v>69.8</v>
       </c>
       <c r="L7" t="n">
-        <v>5.3</v>
+        <v>5.37</v>
       </c>
       <c r="M7" t="n">
-        <v>65.7</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="N7" t="n">
-        <v>80.8</v>
+        <v>80.7</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P7" t="n">
-        <v>40.8</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1126,11 +1117,11 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>LULU</t>
+          <t>EXC</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>708.15</v>
+        <v>370.86</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1163,30 +1154,27 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>73.5</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="J8" t="n">
-        <v>65.09999999999999</v>
+        <v>62.6</v>
       </c>
       <c r="K8" t="n">
-        <v>74.40000000000001</v>
+        <v>69.8</v>
       </c>
       <c r="L8" t="n">
-        <v>7.29</v>
+        <v>5.37</v>
       </c>
       <c r="M8" t="n">
-        <v>73.7</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="N8" t="n">
-        <v>91.5</v>
+        <v>80.7</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P8" t="n">
-        <v>40.3</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1195,17 +1183,17 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U8" t="inlineStr"/>
@@ -1218,30 +1206,30 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>KO</t>
+          <t>GM</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>212.82</v>
+        <v>370.86</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1251,34 +1239,31 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>68</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="J9" t="n">
-        <v>29.5</v>
+        <v>62.6</v>
       </c>
       <c r="K9" t="n">
-        <v>100</v>
+        <v>69.8</v>
       </c>
       <c r="L9" t="n">
-        <v>6.55</v>
+        <v>5.37</v>
       </c>
       <c r="M9" t="n">
-        <v>50.4</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="N9" t="n">
-        <v>100</v>
+        <v>80.7</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P9" t="n">
-        <v>54.6</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1287,12 +1272,12 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
@@ -1300,44 +1285,40 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>LIN</t>
+          <t>FCX</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>212.82</v>
+        <v>370.86</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1347,34 +1328,31 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>68</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="J10" t="n">
-        <v>29.5</v>
+        <v>62.6</v>
       </c>
       <c r="K10" t="n">
-        <v>100</v>
+        <v>69.8</v>
       </c>
       <c r="L10" t="n">
-        <v>6.55</v>
+        <v>5.37</v>
       </c>
       <c r="M10" t="n">
-        <v>50.4</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="N10" t="n">
-        <v>100</v>
+        <v>80.7</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P10" t="n">
-        <v>52</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1383,12 +1361,12 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -1396,44 +1374,40 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U10" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U10" t="inlineStr"/>
       <c r="V10" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>JNJ</t>
+          <t>GE</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>212.82</v>
+        <v>370.86</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1443,34 +1417,31 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>68</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="J11" t="n">
-        <v>29.5</v>
+        <v>62.6</v>
       </c>
       <c r="K11" t="n">
-        <v>100</v>
+        <v>69.8</v>
       </c>
       <c r="L11" t="n">
-        <v>6.55</v>
+        <v>5.37</v>
       </c>
       <c r="M11" t="n">
-        <v>50.4</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="N11" t="n">
-        <v>100</v>
+        <v>80.7</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P11" t="n">
-        <v>32.5</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1479,12 +1450,12 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
@@ -1492,44 +1463,40 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U11" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U11" t="inlineStr"/>
       <c r="V11" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>MO</t>
+          <t>ETN</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>302.8</v>
+        <v>370.86</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1539,34 +1506,31 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>64.3</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="J12" t="n">
-        <v>32.5</v>
+        <v>62.6</v>
       </c>
       <c r="K12" t="n">
-        <v>96</v>
+        <v>69.8</v>
       </c>
       <c r="L12" t="n">
-        <v>3.33</v>
+        <v>5.37</v>
       </c>
       <c r="M12" t="n">
-        <v>37.3</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="N12" t="n">
-        <v>42.2</v>
+        <v>80.7</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P12" t="n">
-        <v>63.8</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1575,12 +1539,12 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
@@ -1598,30 +1562,30 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>302.8</v>
+        <v>370.86</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1631,31 +1595,31 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>64.3</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="J13" t="n">
-        <v>32.5</v>
+        <v>62.6</v>
       </c>
       <c r="K13" t="n">
-        <v>96</v>
+        <v>69.8</v>
       </c>
       <c r="L13" t="n">
-        <v>3.33</v>
+        <v>5.37</v>
       </c>
       <c r="M13" t="n">
-        <v>27.7</v>
+        <v>65.59999999999999</v>
+      </c>
+      <c r="N13" t="n">
+        <v>80.7</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P13" t="n">
-        <v>63.8</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1664,12 +1628,12 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
@@ -1687,71 +1651,68 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>APH</t>
+          <t>F</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>70.5</v>
+        <v>370.86</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>62</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="J14" t="n">
-        <v>63.6</v>
+        <v>62.6</v>
       </c>
       <c r="K14" t="n">
-        <v>5</v>
+        <v>69.8</v>
       </c>
       <c r="L14" t="n">
-        <v>3.12</v>
+        <v>5.37</v>
       </c>
       <c r="M14" t="n">
-        <v>21.8</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="N14" t="n">
-        <v>7.6</v>
+        <v>80.7</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P14" t="n">
-        <v>50.5</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
@@ -1766,14 +1727,10 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U14" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr"/>
       <c r="V14" t="inlineStr">
         <is>
           <t>No</t>
@@ -1783,68 +1740,68 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>FI</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>70.5</v>
+        <v>370.86</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>62</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="J15" t="n">
-        <v>63.6</v>
+        <v>62.6</v>
       </c>
       <c r="K15" t="n">
-        <v>5</v>
+        <v>69.8</v>
       </c>
       <c r="L15" t="n">
-        <v>3.12</v>
+        <v>5.37</v>
       </c>
       <c r="M15" t="n">
-        <v>32.5</v>
+        <v>65.59999999999999</v>
+      </c>
+      <c r="N15" t="n">
+        <v>80.7</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P15" t="n">
-        <v>50.5</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
@@ -1859,14 +1816,10 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U15" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr"/>
       <c r="V15" t="inlineStr">
         <is>
           <t>No</t>
@@ -1876,68 +1829,68 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ADSK</t>
+          <t>GD</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>70.5</v>
+        <v>370.86</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>62</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="J16" t="n">
-        <v>63.6</v>
+        <v>62.6</v>
       </c>
       <c r="K16" t="n">
-        <v>5</v>
+        <v>69.8</v>
       </c>
       <c r="L16" t="n">
-        <v>3.12</v>
+        <v>5.37</v>
       </c>
       <c r="M16" t="n">
-        <v>43.7</v>
+        <v>65.59999999999999</v>
+      </c>
+      <c r="N16" t="n">
+        <v>80.7</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P16" t="n">
-        <v>39.4</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
@@ -1952,14 +1905,10 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U16" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr"/>
       <c r="V16" t="inlineStr">
         <is>
           <t>No</t>
@@ -1969,30 +1918,30 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>PSA</t>
+          <t>FICO</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>162.92</v>
+        <v>370.86</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -2002,34 +1951,31 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>49.8</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="J17" t="n">
-        <v>37.2</v>
+        <v>62.6</v>
       </c>
       <c r="K17" t="n">
-        <v>86</v>
+        <v>69.8</v>
       </c>
       <c r="L17" t="n">
-        <v>2.73</v>
+        <v>5.37</v>
       </c>
       <c r="M17" t="n">
-        <v>29.6</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="N17" t="n">
-        <v>28.9</v>
+        <v>80.7</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P17" t="n">
-        <v>36.6</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -2038,12 +1984,12 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
@@ -2051,44 +1997,40 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U17" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U17" t="inlineStr"/>
       <c r="V17" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>PFE</t>
+          <t>FDX</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>162.92</v>
+        <v>370.86</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -2098,31 +2040,31 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>49.8</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="J18" t="n">
-        <v>37.2</v>
+        <v>62.6</v>
       </c>
       <c r="K18" t="n">
-        <v>86</v>
+        <v>69.8</v>
       </c>
       <c r="L18" t="n">
-        <v>2.73</v>
+        <v>5.37</v>
       </c>
       <c r="M18" t="n">
-        <v>25.8</v>
+        <v>65.59999999999999</v>
+      </c>
+      <c r="N18" t="n">
+        <v>80.7</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P18" t="n">
-        <v>36.6</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -2131,12 +2073,12 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
@@ -2144,110 +2086,2678 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U18" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U18" t="inlineStr"/>
       <c r="V18" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>PEP</t>
+          <t>ZTS</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>162.92</v>
+        <v>683.85</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>71.3</v>
+      </c>
+      <c r="J19" t="n">
+        <v>62.6</v>
+      </c>
+      <c r="K19" t="n">
+        <v>74.40000000000001</v>
+      </c>
+      <c r="L19" t="n">
+        <v>7.54</v>
+      </c>
+      <c r="M19" t="n">
+        <v>40.4</v>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr"/>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>ABNB</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>683.85</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>71.3</v>
+      </c>
+      <c r="J20" t="n">
+        <v>62.6</v>
+      </c>
+      <c r="K20" t="n">
+        <v>74.40000000000001</v>
+      </c>
+      <c r="L20" t="n">
+        <v>7.54</v>
+      </c>
+      <c r="M20" t="n">
+        <v>73.59999999999999</v>
+      </c>
+      <c r="N20" t="n">
+        <v>90.8</v>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr"/>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>XEL</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>683.85</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>71.3</v>
+      </c>
+      <c r="J21" t="n">
+        <v>62.6</v>
+      </c>
+      <c r="K21" t="n">
+        <v>74.40000000000001</v>
+      </c>
+      <c r="L21" t="n">
+        <v>7.54</v>
+      </c>
+      <c r="M21" t="n">
+        <v>73.59999999999999</v>
+      </c>
+      <c r="N21" t="n">
+        <v>90.8</v>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr"/>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>683.85</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>71.3</v>
+      </c>
+      <c r="J22" t="n">
+        <v>62.6</v>
+      </c>
+      <c r="K22" t="n">
+        <v>74.40000000000001</v>
+      </c>
+      <c r="L22" t="n">
+        <v>7.54</v>
+      </c>
+      <c r="M22" t="n">
+        <v>73.59999999999999</v>
+      </c>
+      <c r="N22" t="n">
+        <v>90.8</v>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr"/>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>LMT</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>212.99</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="F23" t="inlineStr">
         <is>
           <t>Credit Put</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="G23" t="inlineStr">
         <is>
           <t>7-21 DTE</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="H23" t="inlineStr">
         <is>
           <t>EXPANSION</t>
         </is>
       </c>
-      <c r="I19" t="n">
-        <v>49.8</v>
-      </c>
-      <c r="J19" t="n">
-        <v>37.2</v>
-      </c>
-      <c r="K19" t="n">
-        <v>86</v>
-      </c>
-      <c r="L19" t="n">
-        <v>2.73</v>
-      </c>
-      <c r="M19" t="n">
+      <c r="I23" t="n">
+        <v>68</v>
+      </c>
+      <c r="J23" t="n">
         <v>29.6</v>
       </c>
-      <c r="N19" t="n">
-        <v>28.9</v>
-      </c>
-      <c r="O19" t="inlineStr">
+      <c r="K23" t="n">
+        <v>100</v>
+      </c>
+      <c r="L23" t="n">
+        <v>6.55</v>
+      </c>
+      <c r="M23" t="n">
+        <v>50.4</v>
+      </c>
+      <c r="N23" t="n">
+        <v>100</v>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="P23" t="n">
+        <v>41.7</v>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>212.99</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>68</v>
+      </c>
+      <c r="J24" t="n">
+        <v>29.6</v>
+      </c>
+      <c r="K24" t="n">
+        <v>100</v>
+      </c>
+      <c r="L24" t="n">
+        <v>6.55</v>
+      </c>
+      <c r="M24" t="n">
+        <v>50.4</v>
+      </c>
+      <c r="N24" t="n">
+        <v>100</v>
+      </c>
+      <c r="O24" t="inlineStr">
         <is>
           <t>Bearish</t>
         </is>
       </c>
-      <c r="P19" t="n">
-        <v>36.6</v>
-      </c>
-      <c r="Q19" t="inlineStr">
+      <c r="P24" t="n">
+        <v>31.3</v>
+      </c>
+      <c r="Q24" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>
       </c>
-      <c r="R19" t="inlineStr">
+      <c r="R24" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="S19" t="inlineStr">
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>LIN</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>212.99</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>68</v>
+      </c>
+      <c r="J25" t="n">
+        <v>29.6</v>
+      </c>
+      <c r="K25" t="n">
+        <v>100</v>
+      </c>
+      <c r="L25" t="n">
+        <v>6.55</v>
+      </c>
+      <c r="M25" t="n">
+        <v>27.7</v>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P25" t="n">
+        <v>31.3</v>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>TMUS</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>59.01</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>67.59999999999999</v>
+      </c>
+      <c r="J26" t="n">
+        <v>63.3</v>
+      </c>
+      <c r="K26" t="n">
+        <v>91.90000000000001</v>
+      </c>
+      <c r="L26" t="n">
+        <v>4.84</v>
+      </c>
+      <c r="M26" t="n">
+        <v>55.7</v>
+      </c>
+      <c r="N26" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P26" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr"/>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>TGT</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>59.01</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>67.59999999999999</v>
+      </c>
+      <c r="J27" t="n">
+        <v>63.3</v>
+      </c>
+      <c r="K27" t="n">
+        <v>91.90000000000001</v>
+      </c>
+      <c r="L27" t="n">
+        <v>4.84</v>
+      </c>
+      <c r="M27" t="n">
+        <v>55.7</v>
+      </c>
+      <c r="N27" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P27" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr"/>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>UNH</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>59.01</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>67.59999999999999</v>
+      </c>
+      <c r="J28" t="n">
+        <v>63.3</v>
+      </c>
+      <c r="K28" t="n">
+        <v>91.90000000000001</v>
+      </c>
+      <c r="L28" t="n">
+        <v>4.84</v>
+      </c>
+      <c r="M28" t="n">
+        <v>55.7</v>
+      </c>
+      <c r="N28" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P28" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr"/>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>TT</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>59.01</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>67.59999999999999</v>
+      </c>
+      <c r="J29" t="n">
+        <v>63.3</v>
+      </c>
+      <c r="K29" t="n">
+        <v>91.90000000000001</v>
+      </c>
+      <c r="L29" t="n">
+        <v>4.84</v>
+      </c>
+      <c r="M29" t="n">
+        <v>55.7</v>
+      </c>
+      <c r="N29" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P29" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr"/>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>UPS</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>59.01</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>67.59999999999999</v>
+      </c>
+      <c r="J30" t="n">
+        <v>63.3</v>
+      </c>
+      <c r="K30" t="n">
+        <v>91.90000000000001</v>
+      </c>
+      <c r="L30" t="n">
+        <v>4.84</v>
+      </c>
+      <c r="M30" t="n">
+        <v>55.7</v>
+      </c>
+      <c r="N30" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P30" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr"/>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>UNP</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>59.01</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>67.59999999999999</v>
+      </c>
+      <c r="J31" t="n">
+        <v>63.3</v>
+      </c>
+      <c r="K31" t="n">
+        <v>91.90000000000001</v>
+      </c>
+      <c r="L31" t="n">
+        <v>4.84</v>
+      </c>
+      <c r="M31" t="n">
+        <v>55.7</v>
+      </c>
+      <c r="N31" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P31" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr"/>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>TXN</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>59.01</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>67.59999999999999</v>
+      </c>
+      <c r="J32" t="n">
+        <v>63.3</v>
+      </c>
+      <c r="K32" t="n">
+        <v>91.90000000000001</v>
+      </c>
+      <c r="L32" t="n">
+        <v>4.84</v>
+      </c>
+      <c r="M32" t="n">
+        <v>55.7</v>
+      </c>
+      <c r="N32" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P32" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr"/>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>TSN</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>59.01</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>67.59999999999999</v>
+      </c>
+      <c r="J33" t="n">
+        <v>63.3</v>
+      </c>
+      <c r="K33" t="n">
+        <v>91.90000000000001</v>
+      </c>
+      <c r="L33" t="n">
+        <v>4.84</v>
+      </c>
+      <c r="M33" t="n">
+        <v>31.1</v>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P33" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr"/>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>TRV</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>59.01</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>67.59999999999999</v>
+      </c>
+      <c r="J34" t="n">
+        <v>63.3</v>
+      </c>
+      <c r="K34" t="n">
+        <v>91.90000000000001</v>
+      </c>
+      <c r="L34" t="n">
+        <v>4.84</v>
+      </c>
+      <c r="M34" t="n">
+        <v>55.7</v>
+      </c>
+      <c r="N34" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P34" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr"/>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>TJX</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>59.01</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>67.59999999999999</v>
+      </c>
+      <c r="J35" t="n">
+        <v>63.3</v>
+      </c>
+      <c r="K35" t="n">
+        <v>91.90000000000001</v>
+      </c>
+      <c r="L35" t="n">
+        <v>4.84</v>
+      </c>
+      <c r="M35" t="n">
+        <v>55.7</v>
+      </c>
+      <c r="N35" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P35" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr"/>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>209.34</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>66.40000000000001</v>
+      </c>
+      <c r="J36" t="n">
+        <v>60.2</v>
+      </c>
+      <c r="K36" t="n">
+        <v>81.40000000000001</v>
+      </c>
+      <c r="L36" t="n">
+        <v>11.89</v>
+      </c>
+      <c r="M36" t="n">
+        <v>76.7</v>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P36" t="n">
+        <v>57.5</v>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
         <is>
           <t>green</t>
         </is>
       </c>
-      <c r="T19" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U19" t="inlineStr">
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr"/>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>209.34</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>66.40000000000001</v>
+      </c>
+      <c r="J37" t="n">
+        <v>60.2</v>
+      </c>
+      <c r="K37" t="n">
+        <v>81.40000000000001</v>
+      </c>
+      <c r="L37" t="n">
+        <v>11.89</v>
+      </c>
+      <c r="M37" t="n">
+        <v>108.8</v>
+      </c>
+      <c r="N37" t="n">
+        <v>76.5</v>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P37" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U37" t="inlineStr"/>
+      <c r="V37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>NEE</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>209.34</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>66.40000000000001</v>
+      </c>
+      <c r="J38" t="n">
+        <v>60.2</v>
+      </c>
+      <c r="K38" t="n">
+        <v>81.40000000000001</v>
+      </c>
+      <c r="L38" t="n">
+        <v>11.89</v>
+      </c>
+      <c r="M38" t="n">
+        <v>108.8</v>
+      </c>
+      <c r="N38" t="n">
+        <v>76.5</v>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P38" t="n">
+        <v>45.7</v>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr"/>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>MSCI</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>209.34</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>66.40000000000001</v>
+      </c>
+      <c r="J39" t="n">
+        <v>60.2</v>
+      </c>
+      <c r="K39" t="n">
+        <v>81.40000000000001</v>
+      </c>
+      <c r="L39" t="n">
+        <v>11.89</v>
+      </c>
+      <c r="M39" t="n">
+        <v>108.8</v>
+      </c>
+      <c r="N39" t="n">
+        <v>76.5</v>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P39" t="n">
+        <v>57.5</v>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U39" t="inlineStr"/>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>MSI</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>209.34</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>66.40000000000001</v>
+      </c>
+      <c r="J40" t="n">
+        <v>60.2</v>
+      </c>
+      <c r="K40" t="n">
+        <v>81.40000000000001</v>
+      </c>
+      <c r="L40" t="n">
+        <v>11.89</v>
+      </c>
+      <c r="M40" t="n">
+        <v>108.8</v>
+      </c>
+      <c r="N40" t="n">
+        <v>76.5</v>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P40" t="n">
+        <v>36.4</v>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr"/>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>302.48</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>64.8</v>
+      </c>
+      <c r="J41" t="n">
+        <v>33.5</v>
+      </c>
+      <c r="K41" t="n">
+        <v>94</v>
+      </c>
+      <c r="L41" t="n">
+        <v>3.21</v>
+      </c>
+      <c r="M41" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="N41" t="n">
+        <v>42.8</v>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P41" t="n">
+        <v>29.6</v>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr"/>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>LLY</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>302.48</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>64.8</v>
+      </c>
+      <c r="J42" t="n">
+        <v>33.5</v>
+      </c>
+      <c r="K42" t="n">
+        <v>94</v>
+      </c>
+      <c r="L42" t="n">
+        <v>3.21</v>
+      </c>
+      <c r="M42" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="N42" t="n">
+        <v>42.8</v>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P42" t="n">
+        <v>29.6</v>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U42" t="inlineStr"/>
+      <c r="V42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>NSC</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>117.72</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>63.5</v>
+      </c>
+      <c r="J43" t="n">
+        <v>57.5</v>
+      </c>
+      <c r="K43" t="n">
+        <v>93</v>
+      </c>
+      <c r="L43" t="n">
+        <v>5.15</v>
+      </c>
+      <c r="M43" t="n">
+        <v>50.4</v>
+      </c>
+      <c r="N43" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P43" t="n">
+        <v>45.7</v>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U43" t="inlineStr"/>
+      <c r="V43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>117.72</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
+        <v>63.5</v>
+      </c>
+      <c r="J44" t="n">
+        <v>57.5</v>
+      </c>
+      <c r="K44" t="n">
+        <v>93</v>
+      </c>
+      <c r="L44" t="n">
+        <v>5.15</v>
+      </c>
+      <c r="M44" t="n">
+        <v>50.4</v>
+      </c>
+      <c r="N44" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P44" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U44" t="inlineStr"/>
+      <c r="V44" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>LRCX</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>47.25</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I45" t="n">
+        <v>61.8</v>
+      </c>
+      <c r="J45" t="n">
+        <v>31.3</v>
+      </c>
+      <c r="K45" t="n">
+        <v>92</v>
+      </c>
+      <c r="L45" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="M45" t="n">
+        <v>29.6</v>
+      </c>
+      <c r="N45" t="n">
+        <v>41.3</v>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P45" t="n">
+        <v>43.6</v>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U45" t="inlineStr">
         <is>
           <t>Divergence</t>
         </is>
       </c>
-      <c r="V19" t="inlineStr">
+      <c r="V45" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>MO</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>47.25</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I46" t="n">
+        <v>61.8</v>
+      </c>
+      <c r="J46" t="n">
+        <v>31.3</v>
+      </c>
+      <c r="K46" t="n">
+        <v>92</v>
+      </c>
+      <c r="L46" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="M46" t="n">
+        <v>29.6</v>
+      </c>
+      <c r="N46" t="n">
+        <v>41.3</v>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="P46" t="n">
+        <v>41.7</v>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V46" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>SYK</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>490.66</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I47" t="n">
+        <v>61</v>
+      </c>
+      <c r="J47" t="n">
+        <v>47.6</v>
+      </c>
+      <c r="K47" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="L47" t="n">
+        <v>3.47</v>
+      </c>
+      <c r="M47" t="n">
+        <v>32.2</v>
+      </c>
+      <c r="N47" t="n">
+        <v>21.3</v>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P47" t="n">
+        <v>63.3</v>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V47" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan 16.03.2026 15:10 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,11 +435,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V22"/>
+  <dimension ref="A1:V41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
@@ -577,15 +577,15 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>AXP</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>369.64</v>
+        <v>327.14</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -600,36 +600,36 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>75.40000000000001</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="J2" t="n">
-        <v>62.3</v>
+        <v>47.5</v>
       </c>
       <c r="K2" t="n">
-        <v>69.8</v>
+        <v>14</v>
       </c>
       <c r="L2" t="n">
-        <v>5.39</v>
+        <v>4.03</v>
       </c>
       <c r="M2" t="n">
-        <v>65.7</v>
+        <v>41.7</v>
       </c>
       <c r="N2" t="n">
-        <v>80.90000000000001</v>
+        <v>27.1</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -637,29 +637,33 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>47.7</v>
+        <v>52.1</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
       <c r="V2" t="inlineStr">
         <is>
           <t>No</t>
@@ -669,15 +673,15 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MCK</t>
+          <t>BRK-B</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>369.64</v>
+        <v>327.14</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -692,63 +696,70 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>75.40000000000001</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="J3" t="n">
-        <v>62.3</v>
+        <v>47.5</v>
       </c>
       <c r="K3" t="n">
-        <v>69.8</v>
+        <v>14</v>
       </c>
       <c r="L3" t="n">
-        <v>5.39</v>
+        <v>4.03</v>
       </c>
       <c r="M3" t="n">
-        <v>65.7</v>
+        <v>41.7</v>
       </c>
       <c r="N3" t="n">
-        <v>80.90000000000001</v>
+        <v>27.1</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P3" t="n">
+        <v>52.1</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
       <c r="V3" t="inlineStr">
         <is>
           <t>No</t>
@@ -758,30 +769,30 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>MCHP</t>
+          <t>GPN</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>369.64</v>
+        <v>300.41</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -791,31 +802,34 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>75.40000000000001</v>
+        <v>63.5</v>
       </c>
       <c r="J4" t="n">
-        <v>62.3</v>
+        <v>32.8</v>
       </c>
       <c r="K4" t="n">
-        <v>69.8</v>
+        <v>93</v>
       </c>
       <c r="L4" t="n">
-        <v>5.39</v>
+        <v>2.91</v>
       </c>
       <c r="M4" t="n">
-        <v>65.7</v>
+        <v>37.3</v>
       </c>
       <c r="N4" t="n">
-        <v>80.90000000000001</v>
+        <v>42.5</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="P4" t="n">
+        <v>41.4</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -829,12 +843,12 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U4" t="inlineStr"/>
@@ -847,30 +861,30 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>MCO</t>
+          <t>GILD</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>369.64</v>
+        <v>300.41</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -880,34 +894,34 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>75.40000000000001</v>
+        <v>63.5</v>
       </c>
       <c r="J5" t="n">
-        <v>62.3</v>
+        <v>32.8</v>
       </c>
       <c r="K5" t="n">
-        <v>69.8</v>
+        <v>93</v>
       </c>
       <c r="L5" t="n">
-        <v>5.39</v>
+        <v>2.91</v>
       </c>
       <c r="M5" t="n">
-        <v>65.7</v>
+        <v>37.3</v>
       </c>
       <c r="N5" t="n">
-        <v>80.90000000000001</v>
+        <v>42.5</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>47.7</v>
+        <v>41.4</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -921,12 +935,12 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U5" t="inlineStr"/>
@@ -939,30 +953,30 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>HUM</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>369.64</v>
+        <v>300.41</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -972,31 +986,34 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>75.40000000000001</v>
+        <v>63.5</v>
       </c>
       <c r="J6" t="n">
-        <v>62.3</v>
+        <v>32.8</v>
       </c>
       <c r="K6" t="n">
-        <v>69.8</v>
+        <v>93</v>
       </c>
       <c r="L6" t="n">
-        <v>5.39</v>
+        <v>2.91</v>
       </c>
       <c r="M6" t="n">
-        <v>65.7</v>
+        <v>37.3</v>
       </c>
       <c r="N6" t="n">
-        <v>80.90000000000001</v>
+        <v>42.5</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="P6" t="n">
+        <v>41.4</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1010,12 +1027,12 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
@@ -1028,30 +1045,30 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>MCD</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>369.64</v>
+        <v>300.41</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1061,31 +1078,34 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>75.40000000000001</v>
+        <v>63.5</v>
       </c>
       <c r="J7" t="n">
-        <v>62.3</v>
+        <v>32.8</v>
       </c>
       <c r="K7" t="n">
-        <v>69.8</v>
+        <v>93</v>
       </c>
       <c r="L7" t="n">
-        <v>5.39</v>
+        <v>2.91</v>
       </c>
       <c r="M7" t="n">
-        <v>65.7</v>
+        <v>37.3</v>
       </c>
       <c r="N7" t="n">
-        <v>80.90000000000001</v>
+        <v>42.5</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P7" t="n">
+        <v>34.5</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1099,12 +1119,12 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U7" t="inlineStr"/>
@@ -1117,30 +1137,30 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>MDT</t>
+          <t>HSY</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>369.64</v>
+        <v>300.41</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1150,34 +1170,31 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>75.40000000000001</v>
+        <v>63.5</v>
       </c>
       <c r="J8" t="n">
-        <v>62.3</v>
+        <v>32.8</v>
       </c>
       <c r="K8" t="n">
-        <v>69.8</v>
+        <v>93</v>
       </c>
       <c r="L8" t="n">
-        <v>5.39</v>
+        <v>2.91</v>
       </c>
       <c r="M8" t="n">
-        <v>65.7</v>
+        <v>37.3</v>
       </c>
       <c r="N8" t="n">
-        <v>80.90000000000001</v>
+        <v>42.5</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P8" t="n">
-        <v>47.7</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1191,12 +1208,12 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U8" t="inlineStr"/>
@@ -1209,30 +1226,30 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ABNB</t>
+          <t>GE</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1358.93</v>
+        <v>300.41</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1246,30 +1263,30 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>70.7</v>
+        <v>63.5</v>
       </c>
       <c r="J9" t="n">
-        <v>63.8</v>
+        <v>32.8</v>
       </c>
       <c r="K9" t="n">
-        <v>87.2</v>
+        <v>93</v>
       </c>
       <c r="L9" t="n">
-        <v>8.039999999999999</v>
+        <v>2.91</v>
       </c>
       <c r="M9" t="n">
-        <v>89.40000000000001</v>
+        <v>37.3</v>
       </c>
       <c r="N9" t="n">
-        <v>59.7</v>
+        <v>42.5</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>28.3</v>
+        <v>56.2</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1278,12 +1295,12 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
@@ -1301,11 +1318,11 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CTSH</t>
+          <t>CHTR</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1358.93</v>
+        <v/>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1334,34 +1351,28 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>70.7</v>
+        <v>50</v>
       </c>
       <c r="J10" t="n">
-        <v>63.8</v>
-      </c>
-      <c r="K10" t="n">
-        <v>87.2</v>
-      </c>
-      <c r="L10" t="n">
-        <v>8.039999999999999</v>
+        <v>62.9</v>
       </c>
       <c r="M10" t="n">
-        <v>89.40000000000001</v>
+        <v>41.2</v>
       </c>
       <c r="N10" t="n">
-        <v>59.7</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>39.2</v>
+        <v>57.3</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1370,7 +1381,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>FLAT</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1380,7 +1391,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U10" t="inlineStr"/>
@@ -1393,11 +1404,11 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>BIIB</t>
+          <t>CME</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1358.93</v>
+        <v/>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1426,26 +1437,20 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>70.7</v>
+        <v>50</v>
       </c>
       <c r="J11" t="n">
-        <v>63.8</v>
-      </c>
-      <c r="K11" t="n">
-        <v>87.2</v>
-      </c>
-      <c r="L11" t="n">
-        <v>8.039999999999999</v>
+        <v>62.9</v>
       </c>
       <c r="M11" t="n">
-        <v>89.40000000000001</v>
+        <v>41.2</v>
       </c>
       <c r="N11" t="n">
-        <v>59.7</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1453,7 +1458,7 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>28.3</v>
+        <v>48.7</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1462,7 +1467,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>FLAT</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1472,7 +1477,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U11" t="inlineStr"/>
@@ -1485,11 +1490,11 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CPRT</t>
+          <t>CI</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1358.93</v>
+        <v/>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1518,34 +1523,28 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>70.7</v>
+        <v>50</v>
       </c>
       <c r="J12" t="n">
-        <v>63.8</v>
-      </c>
-      <c r="K12" t="n">
-        <v>87.2</v>
-      </c>
-      <c r="L12" t="n">
-        <v>8.039999999999999</v>
+        <v>62.9</v>
       </c>
       <c r="M12" t="n">
-        <v>89.40000000000001</v>
+        <v>41.2</v>
       </c>
       <c r="N12" t="n">
-        <v>59.7</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>28.3</v>
+        <v>57.3</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1554,7 +1553,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>FLAT</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1564,7 +1563,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U12" t="inlineStr"/>
@@ -1577,11 +1576,11 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>AZN</t>
+          <t>CEG</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1358.93</v>
+        <v/>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -1610,34 +1609,28 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>70.7</v>
+        <v>50</v>
       </c>
       <c r="J13" t="n">
-        <v>63.8</v>
-      </c>
-      <c r="K13" t="n">
-        <v>87.2</v>
-      </c>
-      <c r="L13" t="n">
-        <v>8.039999999999999</v>
+        <v>62.9</v>
       </c>
       <c r="M13" t="n">
-        <v>89.40000000000001</v>
+        <v>41.2</v>
       </c>
       <c r="N13" t="n">
-        <v>59.7</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>28.3</v>
+        <v>57.3</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1646,7 +1639,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>FLAT</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1656,7 +1649,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U13" t="inlineStr"/>
@@ -1669,11 +1662,11 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>WMT</t>
+          <t>CMG</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1358.93</v>
+        <v/>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -1702,31 +1695,28 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>70.7</v>
+        <v>50</v>
       </c>
       <c r="J14" t="n">
-        <v>63.8</v>
-      </c>
-      <c r="K14" t="n">
-        <v>87.2</v>
-      </c>
-      <c r="L14" t="n">
-        <v>8.039999999999999</v>
+        <v>62.9</v>
       </c>
       <c r="M14" t="n">
-        <v>29.6</v>
+        <v>41.2</v>
+      </c>
+      <c r="N14" t="n">
+        <v>67.09999999999999</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P14" t="n">
-        <v>28.3</v>
+        <v>57.3</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1735,7 +1725,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>FLAT</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -1745,7 +1735,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U14" t="inlineStr"/>
@@ -1758,93 +1748,83 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>NSC</t>
+          <t>COP</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>422.44</v>
+        <v/>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>66.7</v>
+        <v>50</v>
       </c>
       <c r="J15" t="n">
-        <v>56.3</v>
-      </c>
-      <c r="K15" t="n">
-        <v>3</v>
-      </c>
-      <c r="L15" t="n">
-        <v>5.93</v>
+        <v>62.9</v>
       </c>
       <c r="M15" t="n">
-        <v>70.7</v>
+        <v>41.2</v>
       </c>
       <c r="N15" t="n">
-        <v>56</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P15" t="n">
-        <v>43.2</v>
+        <v>57.3</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>FLAT</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U15" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr"/>
       <c r="V15" t="inlineStr">
         <is>
           <t>No</t>
@@ -1854,30 +1834,30 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>302.64</v>
+        <v/>
       </c>
       <c r="C16" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1887,34 +1867,28 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>64.2</v>
+        <v>50</v>
       </c>
       <c r="J16" t="n">
-        <v>33.9</v>
-      </c>
-      <c r="K16" t="n">
-        <v>93</v>
-      </c>
-      <c r="L16" t="n">
-        <v>2.95</v>
+        <v>62.9</v>
       </c>
       <c r="M16" t="n">
-        <v>37.5</v>
+        <v>41.2</v>
       </c>
       <c r="N16" t="n">
-        <v>42.9</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>34.1</v>
+        <v>57.3</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1923,17 +1897,17 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>FLAT</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U16" t="inlineStr"/>
@@ -1946,30 +1920,30 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>OXY</t>
+          <t>DLR</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>47.57</v>
+        <v/>
       </c>
       <c r="C17" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1979,34 +1953,25 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>60.8</v>
+        <v>50</v>
       </c>
       <c r="J17" t="n">
-        <v>34.1</v>
-      </c>
-      <c r="K17" t="n">
-        <v>93</v>
-      </c>
-      <c r="L17" t="n">
-        <v>3.04</v>
+        <v>57.3</v>
       </c>
       <c r="M17" t="n">
-        <v>28.9</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="N17" t="n">
-        <v>39.5</v>
+        <v>55</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P17" t="n">
-        <v>51.2</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -2015,12 +1980,12 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>FLAT</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
@@ -2038,30 +2003,30 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>PEP</t>
+          <t>DIS</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>47.57</v>
+        <v/>
       </c>
       <c r="C18" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -2071,34 +2036,25 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>60.8</v>
+        <v>50</v>
       </c>
       <c r="J18" t="n">
-        <v>34.1</v>
-      </c>
-      <c r="K18" t="n">
-        <v>93</v>
-      </c>
-      <c r="L18" t="n">
-        <v>3.04</v>
+        <v>57.3</v>
       </c>
       <c r="M18" t="n">
-        <v>28.9</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="N18" t="n">
-        <v>39.5</v>
+        <v>55</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P18" t="n">
-        <v>51.2</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -2107,12 +2063,12 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>FLAT</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
@@ -2130,30 +2086,30 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>PCAR</t>
+          <t>COST</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>47.57</v>
+        <v/>
       </c>
       <c r="C19" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2163,34 +2119,28 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>60.8</v>
+        <v>50</v>
       </c>
       <c r="J19" t="n">
-        <v>34.1</v>
-      </c>
-      <c r="K19" t="n">
-        <v>93</v>
-      </c>
-      <c r="L19" t="n">
-        <v>3.04</v>
+        <v>62.9</v>
       </c>
       <c r="M19" t="n">
-        <v>28.9</v>
+        <v>41.2</v>
       </c>
       <c r="N19" t="n">
-        <v>39.5</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P19" t="n">
-        <v>51.2</v>
+        <v>57.3</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -2199,12 +2149,12 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>FLAT</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
@@ -2222,30 +2172,30 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ORLY</t>
+          <t>CTAS</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>47.57</v>
+        <v/>
       </c>
       <c r="C20" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -2255,34 +2205,28 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I20" t="n">
-        <v>60.8</v>
+        <v>50</v>
       </c>
       <c r="J20" t="n">
-        <v>34.1</v>
-      </c>
-      <c r="K20" t="n">
-        <v>93</v>
-      </c>
-      <c r="L20" t="n">
-        <v>3.04</v>
+        <v>57.3</v>
       </c>
       <c r="M20" t="n">
-        <v>28.9</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="N20" t="n">
-        <v>39.5</v>
+        <v>55</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P20" t="n">
-        <v>51.2</v>
+        <v>30.9</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
@@ -2291,12 +2235,12 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>FLAT</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
@@ -2314,30 +2258,30 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>NOC</t>
+          <t>CVX</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>47.57</v>
+        <v/>
       </c>
       <c r="C21" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2347,34 +2291,25 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>60.8</v>
+        <v>50</v>
       </c>
       <c r="J21" t="n">
-        <v>34.1</v>
-      </c>
-      <c r="K21" t="n">
-        <v>93</v>
-      </c>
-      <c r="L21" t="n">
-        <v>3.04</v>
+        <v>57.3</v>
       </c>
       <c r="M21" t="n">
-        <v>28.9</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="N21" t="n">
-        <v>39.5</v>
+        <v>55</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P21" t="n">
-        <v>33.2</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
@@ -2383,12 +2318,12 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>FLAT</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
@@ -2406,30 +2341,30 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ORCL</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>47.57</v>
+        <v/>
       </c>
       <c r="C22" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -2439,34 +2374,25 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I22" t="n">
-        <v>60.8</v>
+        <v>50</v>
       </c>
       <c r="J22" t="n">
-        <v>34.1</v>
-      </c>
-      <c r="K22" t="n">
-        <v>93</v>
-      </c>
-      <c r="L22" t="n">
-        <v>3.04</v>
+        <v>57.3</v>
       </c>
       <c r="M22" t="n">
-        <v>28.9</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="N22" t="n">
-        <v>39.5</v>
+        <v>55</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P22" t="n">
-        <v>51.2</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
@@ -2475,12 +2401,12 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>FLAT</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
@@ -2492,6 +2418,1656 @@
       <c r="V22" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>CAT</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v/>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>50</v>
+      </c>
+      <c r="J23" t="n">
+        <v>62.9</v>
+      </c>
+      <c r="M23" t="n">
+        <v>41.2</v>
+      </c>
+      <c r="N23" t="n">
+        <v>67.09999999999999</v>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="P23" t="n">
+        <v>57.3</v>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr"/>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v/>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>50</v>
+      </c>
+      <c r="J24" t="n">
+        <v>57.3</v>
+      </c>
+      <c r="M24" t="n">
+        <v>26.2</v>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr"/>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>DHR</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v/>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>50</v>
+      </c>
+      <c r="J25" t="n">
+        <v>57.3</v>
+      </c>
+      <c r="M25" t="n">
+        <v>79.59999999999999</v>
+      </c>
+      <c r="N25" t="n">
+        <v>55</v>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr"/>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>BLK</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v/>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>50</v>
+      </c>
+      <c r="J26" t="n">
+        <v>62.9</v>
+      </c>
+      <c r="M26" t="n">
+        <v>41.2</v>
+      </c>
+      <c r="N26" t="n">
+        <v>67.09999999999999</v>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="P26" t="n">
+        <v>57.3</v>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr"/>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>CVS</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v/>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>50</v>
+      </c>
+      <c r="J27" t="n">
+        <v>57.3</v>
+      </c>
+      <c r="M27" t="n">
+        <v>38</v>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr"/>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>CSCO</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v/>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>50</v>
+      </c>
+      <c r="J28" t="n">
+        <v>62.9</v>
+      </c>
+      <c r="M28" t="n">
+        <v>29.2</v>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="P28" t="n">
+        <v>57.3</v>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr"/>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>GD</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v/>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>50</v>
+      </c>
+      <c r="J29" t="n">
+        <v>41.4</v>
+      </c>
+      <c r="M29" t="n">
+        <v>32.6</v>
+      </c>
+      <c r="N29" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>GS</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v/>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>50</v>
+      </c>
+      <c r="J30" t="n">
+        <v>41.4</v>
+      </c>
+      <c r="M30" t="n">
+        <v>32.6</v>
+      </c>
+      <c r="N30" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>ICE</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v/>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>50</v>
+      </c>
+      <c r="J31" t="n">
+        <v>41.4</v>
+      </c>
+      <c r="M31" t="n">
+        <v>32.6</v>
+      </c>
+      <c r="N31" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>HON</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v/>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>50</v>
+      </c>
+      <c r="J32" t="n">
+        <v>41.4</v>
+      </c>
+      <c r="M32" t="n">
+        <v>32.6</v>
+      </c>
+      <c r="N32" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>IBM</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v/>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>50</v>
+      </c>
+      <c r="J33" t="n">
+        <v>41.4</v>
+      </c>
+      <c r="M33" t="n">
+        <v>32.6</v>
+      </c>
+      <c r="N33" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P33" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v/>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>50</v>
+      </c>
+      <c r="J34" t="n">
+        <v>47.3</v>
+      </c>
+      <c r="M34" t="n">
+        <v>32.2</v>
+      </c>
+      <c r="N34" t="n">
+        <v>21.6</v>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="P34" t="n">
+        <v>71.8</v>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>FIRED</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>Squeeze Fired, Divergence</t>
+        </is>
+      </c>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v/>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>50</v>
+      </c>
+      <c r="J35" t="n">
+        <v>47.3</v>
+      </c>
+      <c r="M35" t="n">
+        <v>32.2</v>
+      </c>
+      <c r="N35" t="n">
+        <v>21.6</v>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="P35" t="n">
+        <v>71.8</v>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>FIRED</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>Squeeze Fired, Divergence</t>
+        </is>
+      </c>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>NKE</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v/>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>50</v>
+      </c>
+      <c r="J36" t="n">
+        <v>47.3</v>
+      </c>
+      <c r="M36" t="n">
+        <v>32.2</v>
+      </c>
+      <c r="N36" t="n">
+        <v>21.6</v>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="P36" t="n">
+        <v>71.8</v>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>FIRED</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>Squeeze Fired, Divergence</t>
+        </is>
+      </c>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>NSC</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v/>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>50</v>
+      </c>
+      <c r="J37" t="n">
+        <v>47.3</v>
+      </c>
+      <c r="M37" t="n">
+        <v>32.2</v>
+      </c>
+      <c r="N37" t="n">
+        <v>21.6</v>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="P37" t="n">
+        <v>71.8</v>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>FIRED</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>Squeeze Fired, Divergence</t>
+        </is>
+      </c>
+      <c r="V37" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>MPC</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v/>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>50</v>
+      </c>
+      <c r="J38" t="n">
+        <v>47.3</v>
+      </c>
+      <c r="M38" t="n">
+        <v>40.7</v>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="P38" t="n">
+        <v>71.8</v>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>FIRED</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>Squeeze Fired, Divergence</t>
+        </is>
+      </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>NOC</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v/>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>50</v>
+      </c>
+      <c r="J39" t="n">
+        <v>47.3</v>
+      </c>
+      <c r="M39" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="P39" t="n">
+        <v>71.8</v>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>FIRED</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>Squeeze Fired, Divergence</t>
+        </is>
+      </c>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v/>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>50</v>
+      </c>
+      <c r="J40" t="n">
+        <v>47.3</v>
+      </c>
+      <c r="M40" t="n">
+        <v>32.2</v>
+      </c>
+      <c r="N40" t="n">
+        <v>21.6</v>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P40" t="n">
+        <v>43.1</v>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>FIRED</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>Squeeze Fired, Divergence</t>
+        </is>
+      </c>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v/>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>50</v>
+      </c>
+      <c r="J41" t="n">
+        <v>47.3</v>
+      </c>
+      <c r="M41" t="n">
+        <v>32.2</v>
+      </c>
+      <c r="N41" t="n">
+        <v>21.6</v>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="P41" t="n">
+        <v>44.9</v>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>FIRED</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>Squeeze Fired, Divergence</t>
+        </is>
+      </c>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan 17.03.2026 15:06 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V41"/>
+  <dimension ref="A1:V54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -448,7 +448,7 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="6" customWidth="1" min="10" max="10"/>
-    <col width="6" customWidth="1" min="11" max="11"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
     <col width="6" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
     <col width="9" customWidth="1" min="14" max="14"/>
@@ -577,15 +577,15 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AXP</t>
+          <t>ABNB</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>327.14</v>
+        <v>239.01</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -600,70 +600,66 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>67.59999999999999</v>
+        <v>87.90000000000001</v>
       </c>
       <c r="J2" t="n">
-        <v>47.5</v>
+        <v>61.2</v>
       </c>
       <c r="K2" t="n">
-        <v>14</v>
+        <v>97.7</v>
       </c>
       <c r="L2" t="n">
-        <v>4.03</v>
+        <v>3.98</v>
       </c>
       <c r="M2" t="n">
-        <v>41.7</v>
+        <v>39.2</v>
       </c>
       <c r="N2" t="n">
-        <v>27.1</v>
+        <v>47.3</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>52.1</v>
+        <v>51.1</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>TTM Squeeze</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr">
         <is>
           <t>No</t>
@@ -673,15 +669,15 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BRK-B</t>
+          <t>ASML</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>327.14</v>
+        <v>239.01</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -696,70 +692,66 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>67.59999999999999</v>
+        <v>87.90000000000001</v>
       </c>
       <c r="J3" t="n">
-        <v>47.5</v>
+        <v>61.2</v>
       </c>
       <c r="K3" t="n">
-        <v>14</v>
+        <v>97.7</v>
       </c>
       <c r="L3" t="n">
-        <v>4.03</v>
+        <v>3.98</v>
       </c>
       <c r="M3" t="n">
-        <v>41.7</v>
+        <v>39.2</v>
       </c>
       <c r="N3" t="n">
-        <v>27.1</v>
+        <v>47.3</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P3" t="n">
-        <v>52.1</v>
+        <v>57.2</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>TTM Squeeze</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr"/>
       <c r="V3" t="inlineStr">
         <is>
           <t>No</t>
@@ -769,30 +761,30 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>GPN</t>
+          <t>CTSH</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>300.41</v>
+        <v>239.01</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -806,22 +798,22 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>63.5</v>
+        <v>87.90000000000001</v>
       </c>
       <c r="J4" t="n">
-        <v>32.8</v>
+        <v>61.2</v>
       </c>
       <c r="K4" t="n">
-        <v>93</v>
+        <v>97.7</v>
       </c>
       <c r="L4" t="n">
-        <v>2.91</v>
+        <v>3.98</v>
       </c>
       <c r="M4" t="n">
-        <v>37.3</v>
+        <v>39.2</v>
       </c>
       <c r="N4" t="n">
-        <v>42.5</v>
+        <v>47.3</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -829,7 +821,7 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>41.4</v>
+        <v>51.1</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -843,12 +835,12 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U4" t="inlineStr"/>
@@ -861,30 +853,30 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>GILD</t>
+          <t>CPRT</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>300.41</v>
+        <v>239.01</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -898,30 +890,30 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>63.5</v>
+        <v>87.90000000000001</v>
       </c>
       <c r="J5" t="n">
-        <v>32.8</v>
+        <v>61.2</v>
       </c>
       <c r="K5" t="n">
-        <v>93</v>
+        <v>97.7</v>
       </c>
       <c r="L5" t="n">
-        <v>2.91</v>
+        <v>3.98</v>
       </c>
       <c r="M5" t="n">
-        <v>37.3</v>
+        <v>39.2</v>
       </c>
       <c r="N5" t="n">
-        <v>42.5</v>
+        <v>47.3</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>41.4</v>
+        <v>57.2</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -935,12 +927,12 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U5" t="inlineStr"/>
@@ -953,30 +945,30 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>HUM</t>
+          <t>CRWD</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>300.41</v>
+        <v>239.01</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -990,30 +982,30 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>63.5</v>
+        <v>87.90000000000001</v>
       </c>
       <c r="J6" t="n">
-        <v>32.8</v>
+        <v>61.2</v>
       </c>
       <c r="K6" t="n">
-        <v>93</v>
+        <v>97.7</v>
       </c>
       <c r="L6" t="n">
-        <v>2.91</v>
+        <v>3.98</v>
       </c>
       <c r="M6" t="n">
-        <v>37.3</v>
+        <v>39.2</v>
       </c>
       <c r="N6" t="n">
-        <v>42.5</v>
+        <v>47.3</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P6" t="n">
-        <v>41.4</v>
+        <v>57.2</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1027,12 +1019,12 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
@@ -1045,30 +1037,30 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>ZTS</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>300.41</v>
+        <v>239.01</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1082,30 +1074,30 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>63.5</v>
+        <v>87.90000000000001</v>
       </c>
       <c r="J7" t="n">
-        <v>32.8</v>
+        <v>61.2</v>
       </c>
       <c r="K7" t="n">
-        <v>93</v>
+        <v>97.7</v>
       </c>
       <c r="L7" t="n">
-        <v>2.91</v>
+        <v>3.98</v>
       </c>
       <c r="M7" t="n">
-        <v>37.3</v>
+        <v>39.2</v>
       </c>
       <c r="N7" t="n">
-        <v>42.5</v>
+        <v>47.3</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>34.5</v>
+        <v>51.1</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1119,12 +1111,12 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U7" t="inlineStr"/>
@@ -1137,30 +1129,30 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>HSY</t>
+          <t>BKR</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>300.41</v>
+        <v>239.01</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1174,27 +1166,30 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>63.5</v>
+        <v>87.90000000000001</v>
       </c>
       <c r="J8" t="n">
-        <v>32.8</v>
+        <v>61.2</v>
       </c>
       <c r="K8" t="n">
-        <v>93</v>
+        <v>97.7</v>
       </c>
       <c r="L8" t="n">
-        <v>2.91</v>
+        <v>3.98</v>
       </c>
       <c r="M8" t="n">
-        <v>37.3</v>
+        <v>39.2</v>
       </c>
       <c r="N8" t="n">
-        <v>42.5</v>
+        <v>47.3</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P8" t="n">
+        <v>83.59999999999999</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1208,12 +1203,12 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U8" t="inlineStr"/>
@@ -1226,30 +1221,30 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>GE</t>
+          <t>AZN</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>300.41</v>
+        <v>239.01</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1263,22 +1258,22 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>63.5</v>
+        <v>87.90000000000001</v>
       </c>
       <c r="J9" t="n">
-        <v>32.8</v>
+        <v>61.2</v>
       </c>
       <c r="K9" t="n">
-        <v>93</v>
+        <v>97.7</v>
       </c>
       <c r="L9" t="n">
-        <v>2.91</v>
+        <v>3.98</v>
       </c>
       <c r="M9" t="n">
-        <v>37.3</v>
+        <v>39.2</v>
       </c>
       <c r="N9" t="n">
-        <v>42.5</v>
+        <v>47.3</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1286,7 +1281,7 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>56.2</v>
+        <v>51.1</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1300,12 +1295,12 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U9" t="inlineStr"/>
@@ -1318,11 +1313,11 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CHTR</t>
+          <t>CDW</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v/>
+        <v>239.01</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1351,28 +1346,34 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>50</v>
+        <v>87.90000000000001</v>
       </c>
       <c r="J10" t="n">
-        <v>62.9</v>
+        <v>61.2</v>
+      </c>
+      <c r="K10" t="n">
+        <v>97.7</v>
+      </c>
+      <c r="L10" t="n">
+        <v>3.98</v>
       </c>
       <c r="M10" t="n">
-        <v>41.2</v>
+        <v>39.2</v>
       </c>
       <c r="N10" t="n">
-        <v>67.09999999999999</v>
+        <v>47.3</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>57.3</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1381,12 +1382,12 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>FLAT</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -1404,11 +1405,11 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CME</t>
+          <t>MELI</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v/>
+        <v>333.14</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1437,20 +1438,26 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>50</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="J11" t="n">
-        <v>62.9</v>
+        <v>65</v>
+      </c>
+      <c r="K11" t="n">
+        <v>89.5</v>
+      </c>
+      <c r="L11" t="n">
+        <v>3.7</v>
       </c>
       <c r="M11" t="n">
-        <v>41.2</v>
+        <v>41.3</v>
       </c>
       <c r="N11" t="n">
-        <v>67.09999999999999</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1458,7 +1465,7 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>48.7</v>
+        <v>44.6</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1467,12 +1474,12 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>FLAT</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
@@ -1490,11 +1497,11 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CI</t>
+          <t>ADM</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v/>
+        <v>347.71</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1523,28 +1530,31 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>50</v>
+        <v>69.5</v>
       </c>
       <c r="J12" t="n">
-        <v>62.9</v>
+        <v>67.7</v>
+      </c>
+      <c r="K12" t="n">
+        <v>87.2</v>
+      </c>
+      <c r="L12" t="n">
+        <v>8.93</v>
       </c>
       <c r="M12" t="n">
-        <v>41.2</v>
-      </c>
-      <c r="N12" t="n">
-        <v>67.09999999999999</v>
+        <v>38.8</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>57.3</v>
+        <v>49.8</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1553,7 +1563,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>FLAT</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1563,7 +1573,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U12" t="inlineStr"/>
@@ -1576,11 +1586,11 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CEG</t>
+          <t>BSX</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v/>
+        <v>347.71</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -1609,28 +1619,34 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>50</v>
+        <v>69.5</v>
       </c>
       <c r="J13" t="n">
-        <v>62.9</v>
+        <v>67.7</v>
+      </c>
+      <c r="K13" t="n">
+        <v>87.2</v>
+      </c>
+      <c r="L13" t="n">
+        <v>8.93</v>
       </c>
       <c r="M13" t="n">
-        <v>41.2</v>
+        <v>89</v>
       </c>
       <c r="N13" t="n">
-        <v>67.09999999999999</v>
+        <v>45.1</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>57.3</v>
+        <v>49.8</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1639,7 +1655,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>FLAT</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1649,7 +1665,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U13" t="inlineStr"/>
@@ -1662,11 +1678,11 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CMG</t>
+          <t>BA</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v/>
+        <v>347.71</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -1695,28 +1711,31 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>50</v>
+        <v>69.5</v>
       </c>
       <c r="J14" t="n">
-        <v>62.9</v>
+        <v>67.7</v>
+      </c>
+      <c r="K14" t="n">
+        <v>87.2</v>
+      </c>
+      <c r="L14" t="n">
+        <v>8.93</v>
       </c>
       <c r="M14" t="n">
-        <v>41.2</v>
-      </c>
-      <c r="N14" t="n">
-        <v>67.09999999999999</v>
+        <v>38.7</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P14" t="n">
-        <v>57.3</v>
+        <v>35.7</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1725,7 +1744,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>FLAT</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -1735,7 +1754,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U14" t="inlineStr"/>
@@ -1748,11 +1767,11 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>COP</t>
+          <t>AON</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v/>
+        <v>347.71</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1781,28 +1800,34 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>50</v>
+        <v>69.5</v>
       </c>
       <c r="J15" t="n">
-        <v>62.9</v>
+        <v>67.7</v>
+      </c>
+      <c r="K15" t="n">
+        <v>87.2</v>
+      </c>
+      <c r="L15" t="n">
+        <v>8.93</v>
       </c>
       <c r="M15" t="n">
-        <v>41.2</v>
+        <v>89</v>
       </c>
       <c r="N15" t="n">
-        <v>67.09999999999999</v>
+        <v>45.1</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P15" t="n">
-        <v>57.3</v>
+        <v>45</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1811,7 +1836,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>FLAT</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -1821,7 +1846,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U15" t="inlineStr"/>
@@ -1834,11 +1859,11 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>AMP</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v/>
+        <v>347.71</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -1867,28 +1892,34 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>50</v>
+        <v>69.5</v>
       </c>
       <c r="J16" t="n">
-        <v>62.9</v>
+        <v>67.7</v>
+      </c>
+      <c r="K16" t="n">
+        <v>87.2</v>
+      </c>
+      <c r="L16" t="n">
+        <v>8.93</v>
       </c>
       <c r="M16" t="n">
-        <v>41.2</v>
+        <v>89</v>
       </c>
       <c r="N16" t="n">
-        <v>67.09999999999999</v>
+        <v>45.1</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>57.3</v>
+        <v>49.8</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1897,7 +1928,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>FLAT</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -1907,7 +1938,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U16" t="inlineStr"/>
@@ -1920,11 +1951,11 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>DLR</t>
+          <t>C</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v/>
+        <v>347.71</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -1953,25 +1984,34 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>50</v>
+        <v>69.5</v>
       </c>
       <c r="J17" t="n">
-        <v>57.3</v>
+        <v>67.7</v>
+      </c>
+      <c r="K17" t="n">
+        <v>87.2</v>
+      </c>
+      <c r="L17" t="n">
+        <v>8.93</v>
       </c>
       <c r="M17" t="n">
-        <v>79.59999999999999</v>
+        <v>89</v>
       </c>
       <c r="N17" t="n">
-        <v>55</v>
+        <v>45.1</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P17" t="n">
+        <v>49.8</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -1980,7 +2020,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>FLAT</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -1990,7 +2030,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U17" t="inlineStr"/>
@@ -2003,11 +2043,11 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>DIS</t>
+          <t>BDX</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v/>
+        <v>347.71</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -2036,25 +2076,31 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>50</v>
+        <v>69.5</v>
       </c>
       <c r="J18" t="n">
-        <v>57.3</v>
+        <v>67.7</v>
+      </c>
+      <c r="K18" t="n">
+        <v>87.2</v>
+      </c>
+      <c r="L18" t="n">
+        <v>8.93</v>
       </c>
       <c r="M18" t="n">
-        <v>79.59999999999999</v>
-      </c>
-      <c r="N18" t="n">
-        <v>55</v>
+        <v>36</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P18" t="n">
+        <v>49.8</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -2063,7 +2109,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>FLAT</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -2073,7 +2119,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U18" t="inlineStr"/>
@@ -2086,11 +2132,11 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>COST</t>
+          <t>BRK-B</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v/>
+        <v>347.71</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -2119,28 +2165,31 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>50</v>
+        <v>69.5</v>
       </c>
       <c r="J19" t="n">
-        <v>62.9</v>
+        <v>67.7</v>
+      </c>
+      <c r="K19" t="n">
+        <v>87.2</v>
+      </c>
+      <c r="L19" t="n">
+        <v>8.93</v>
       </c>
       <c r="M19" t="n">
-        <v>41.2</v>
-      </c>
-      <c r="N19" t="n">
-        <v>67.09999999999999</v>
+        <v>19.1</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P19" t="n">
-        <v>57.3</v>
+        <v>49.8</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -2149,7 +2198,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>FLAT</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -2159,7 +2208,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U19" t="inlineStr"/>
@@ -2172,11 +2221,11 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CTAS</t>
+          <t>ADBE</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v/>
+        <v>347.71</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -2205,28 +2254,31 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I20" t="n">
-        <v>50</v>
+        <v>69.5</v>
       </c>
       <c r="J20" t="n">
-        <v>57.3</v>
+        <v>67.7</v>
+      </c>
+      <c r="K20" t="n">
+        <v>87.2</v>
+      </c>
+      <c r="L20" t="n">
+        <v>8.93</v>
       </c>
       <c r="M20" t="n">
-        <v>79.59999999999999</v>
-      </c>
-      <c r="N20" t="n">
-        <v>55</v>
+        <v>38.9</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P20" t="n">
-        <v>30.9</v>
+        <v>49.8</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
@@ -2235,7 +2287,7 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>FLAT</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -2245,7 +2297,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U20" t="inlineStr"/>
@@ -2258,11 +2310,11 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CVX</t>
+          <t>BKNG</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v/>
+        <v>347.71</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -2291,25 +2343,31 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>50</v>
+        <v>69.5</v>
       </c>
       <c r="J21" t="n">
-        <v>57.3</v>
+        <v>67.7</v>
+      </c>
+      <c r="K21" t="n">
+        <v>87.2</v>
+      </c>
+      <c r="L21" t="n">
+        <v>8.93</v>
       </c>
       <c r="M21" t="n">
-        <v>79.59999999999999</v>
-      </c>
-      <c r="N21" t="n">
-        <v>55</v>
+        <v>36.4</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P21" t="n">
+        <v>49.8</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
@@ -2318,7 +2376,7 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>FLAT</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -2328,7 +2386,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U21" t="inlineStr"/>
@@ -2341,11 +2399,11 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BAC</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v/>
+        <v>347.71</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -2374,25 +2432,31 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I22" t="n">
-        <v>50</v>
+        <v>69.5</v>
       </c>
       <c r="J22" t="n">
-        <v>57.3</v>
+        <v>67.7</v>
+      </c>
+      <c r="K22" t="n">
+        <v>87.2</v>
+      </c>
+      <c r="L22" t="n">
+        <v>8.93</v>
       </c>
       <c r="M22" t="n">
-        <v>79.59999999999999</v>
-      </c>
-      <c r="N22" t="n">
-        <v>55</v>
+        <v>31</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P22" t="n">
+        <v>49.8</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
@@ -2401,7 +2465,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>FLAT</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -2411,7 +2475,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U22" t="inlineStr"/>
@@ -2428,7 +2492,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v/>
+        <v>347.71</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -2457,28 +2521,31 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I23" t="n">
-        <v>50</v>
+        <v>69.5</v>
       </c>
       <c r="J23" t="n">
-        <v>62.9</v>
+        <v>67.7</v>
+      </c>
+      <c r="K23" t="n">
+        <v>87.2</v>
+      </c>
+      <c r="L23" t="n">
+        <v>8.93</v>
       </c>
       <c r="M23" t="n">
-        <v>41.2</v>
-      </c>
-      <c r="N23" t="n">
-        <v>67.09999999999999</v>
+        <v>40.3</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P23" t="n">
-        <v>57.3</v>
+        <v>49.8</v>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
@@ -2487,7 +2554,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>FLAT</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -2497,7 +2564,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U23" t="inlineStr"/>
@@ -2510,15 +2577,15 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>SYK</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v/>
+        <v>492.52</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -2533,41 +2600,53 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I24" t="n">
-        <v>50</v>
+        <v>69</v>
       </c>
       <c r="J24" t="n">
-        <v>57.3</v>
+        <v>48.6</v>
+      </c>
+      <c r="K24" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="L24" t="n">
+        <v>3.19</v>
       </c>
       <c r="M24" t="n">
-        <v>26.2</v>
+        <v>31.5</v>
+      </c>
+      <c r="N24" t="n">
+        <v>17.9</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P24" t="n">
+        <v>47</v>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>FLAT</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
@@ -2577,10 +2656,14 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U24" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
       <c r="V24" t="inlineStr">
         <is>
           <t>No</t>
@@ -2590,15 +2673,15 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>DHR</t>
+          <t>SYY</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v/>
+        <v>492.52</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -2613,44 +2696,53 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I25" t="n">
-        <v>50</v>
+        <v>69</v>
       </c>
       <c r="J25" t="n">
-        <v>57.3</v>
+        <v>48.6</v>
+      </c>
+      <c r="K25" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="L25" t="n">
+        <v>3.19</v>
       </c>
       <c r="M25" t="n">
-        <v>79.59999999999999</v>
+        <v>31.5</v>
       </c>
       <c r="N25" t="n">
-        <v>55</v>
+        <v>17.9</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P25" t="n">
+        <v>64.7</v>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>FLAT</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
@@ -2660,10 +2752,14 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U25" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
       <c r="V25" t="inlineStr">
         <is>
           <t>No</t>
@@ -2673,30 +2769,30 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>BLK</t>
+          <t>AMGN</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v/>
+        <v>211.93</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -2706,28 +2802,34 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I26" t="n">
-        <v>50</v>
+        <v>68</v>
       </c>
       <c r="J26" t="n">
-        <v>62.9</v>
+        <v>31.9</v>
+      </c>
+      <c r="K26" t="n">
+        <v>100</v>
+      </c>
+      <c r="L26" t="n">
+        <v>6.39</v>
       </c>
       <c r="M26" t="n">
-        <v>41.2</v>
+        <v>52.5</v>
       </c>
       <c r="N26" t="n">
-        <v>67.09999999999999</v>
+        <v>100</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P26" t="n">
-        <v>57.3</v>
+        <v>67.7</v>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
@@ -2736,12 +2838,12 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>FLAT</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
@@ -2759,11 +2861,11 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CVS</t>
+          <t>DOW</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v/>
+        <v>311.3</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -2792,22 +2894,34 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I27" t="n">
-        <v>50</v>
+        <v>68</v>
       </c>
       <c r="J27" t="n">
-        <v>57.3</v>
+        <v>58.8</v>
+      </c>
+      <c r="K27" t="n">
+        <v>94.2</v>
+      </c>
+      <c r="L27" t="n">
+        <v>6.42</v>
       </c>
       <c r="M27" t="n">
-        <v>38</v>
+        <v>76.09999999999999</v>
+      </c>
+      <c r="N27" t="n">
+        <v>46.4</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P27" t="n">
+        <v>39.5</v>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
@@ -2816,7 +2930,7 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>FLAT</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
@@ -2826,7 +2940,7 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U27" t="inlineStr"/>
@@ -2839,11 +2953,11 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>DLR</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v/>
+        <v>311.3</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -2872,25 +2986,34 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I28" t="n">
-        <v>50</v>
+        <v>68</v>
       </c>
       <c r="J28" t="n">
-        <v>62.9</v>
+        <v>58.8</v>
+      </c>
+      <c r="K28" t="n">
+        <v>94.2</v>
+      </c>
+      <c r="L28" t="n">
+        <v>6.42</v>
       </c>
       <c r="M28" t="n">
-        <v>29.2</v>
+        <v>76.09999999999999</v>
+      </c>
+      <c r="N28" t="n">
+        <v>46.4</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P28" t="n">
-        <v>57.3</v>
+        <v>39.5</v>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
@@ -2899,7 +3022,7 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>FLAT</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
@@ -2909,7 +3032,7 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U28" t="inlineStr"/>
@@ -2922,15 +3045,15 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>GD</t>
+          <t>DIS</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v/>
+        <v>311.3</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -2945,35 +3068,44 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I29" t="n">
-        <v>50</v>
+        <v>68</v>
       </c>
       <c r="J29" t="n">
-        <v>41.4</v>
+        <v>58.8</v>
+      </c>
+      <c r="K29" t="n">
+        <v>94.2</v>
+      </c>
+      <c r="L29" t="n">
+        <v>6.42</v>
       </c>
       <c r="M29" t="n">
-        <v>32.6</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="N29" t="n">
-        <v>7.3</v>
+        <v>46.4</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P29" t="n">
+        <v>39.5</v>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
@@ -2982,38 +3114,34 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>FLAT</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U29" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr"/>
       <c r="V29" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>GS</t>
+          <t>HSY</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v/>
+        <v>322.15</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -3042,34 +3170,43 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I30" t="n">
-        <v>50</v>
+        <v>66</v>
       </c>
       <c r="J30" t="n">
-        <v>41.4</v>
+        <v>44.6</v>
+      </c>
+      <c r="K30" t="n">
+        <v>17</v>
+      </c>
+      <c r="L30" t="n">
+        <v>3.86</v>
       </c>
       <c r="M30" t="n">
-        <v>32.6</v>
+        <v>41.6</v>
       </c>
       <c r="N30" t="n">
-        <v>7.3</v>
+        <v>26.9</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P30" t="n">
+        <v>51.8</v>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>FLAT</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
@@ -3079,28 +3216,28 @@
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
         <is>
-          <t>Divergence</t>
+          <t>TTM Squeeze, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V30" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ICE</t>
+          <t>KLAC</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v/>
+        <v>322.15</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -3129,34 +3266,43 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I31" t="n">
-        <v>50</v>
+        <v>66</v>
       </c>
       <c r="J31" t="n">
-        <v>41.4</v>
+        <v>44.6</v>
+      </c>
+      <c r="K31" t="n">
+        <v>17</v>
+      </c>
+      <c r="L31" t="n">
+        <v>3.86</v>
       </c>
       <c r="M31" t="n">
-        <v>32.6</v>
+        <v>41.6</v>
       </c>
       <c r="N31" t="n">
-        <v>7.3</v>
+        <v>26.9</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P31" t="n">
+        <v>51.8</v>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>FLAT</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
@@ -3166,28 +3312,28 @@
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
         <is>
-          <t>Divergence</t>
+          <t>TTM Squeeze, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V31" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>HON</t>
+          <t>GPN</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v/>
+        <v>322.15</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -3216,34 +3362,43 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I32" t="n">
-        <v>50</v>
+        <v>66</v>
       </c>
       <c r="J32" t="n">
-        <v>41.4</v>
+        <v>44.6</v>
+      </c>
+      <c r="K32" t="n">
+        <v>17</v>
+      </c>
+      <c r="L32" t="n">
+        <v>3.86</v>
       </c>
       <c r="M32" t="n">
-        <v>32.6</v>
+        <v>41.6</v>
       </c>
       <c r="N32" t="n">
-        <v>7.3</v>
+        <v>26.9</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P32" t="n">
+        <v>51.8</v>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>FLAT</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
@@ -3253,28 +3408,28 @@
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
         <is>
-          <t>Divergence</t>
+          <t>TTM Squeeze, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V32" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>IBM</t>
+          <t>JNJ</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v/>
+        <v>322.15</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -3303,37 +3458,43 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I33" t="n">
-        <v>50</v>
+        <v>66</v>
       </c>
       <c r="J33" t="n">
-        <v>41.4</v>
+        <v>44.6</v>
+      </c>
+      <c r="K33" t="n">
+        <v>17</v>
+      </c>
+      <c r="L33" t="n">
+        <v>3.86</v>
       </c>
       <c r="M33" t="n">
-        <v>32.6</v>
+        <v>41.6</v>
       </c>
       <c r="N33" t="n">
-        <v>7.3</v>
+        <v>26.9</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P33" t="n">
-        <v>34.5</v>
+        <v>51.8</v>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>FLAT</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
@@ -3343,479 +3504,486 @@
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
         <is>
-          <t>Divergence</t>
+          <t>TTM Squeeze, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V33" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>NOW</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v/>
+        <v>301.68</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I34" t="n">
-        <v>50</v>
+        <v>63.4</v>
       </c>
       <c r="J34" t="n">
-        <v>47.3</v>
+        <v>35</v>
+      </c>
+      <c r="K34" t="n">
+        <v>90</v>
+      </c>
+      <c r="L34" t="n">
+        <v>2.96</v>
       </c>
       <c r="M34" t="n">
-        <v>32.2</v>
+        <v>37.6</v>
       </c>
       <c r="N34" t="n">
-        <v>21.6</v>
+        <v>43</v>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P34" t="n">
-        <v>71.8</v>
+        <v>50.2</v>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>FIRED</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>FLAT</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U34" t="inlineStr">
-        <is>
-          <t>Squeeze Fired, Divergence</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr"/>
       <c r="V34" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>NFLX</t>
+          <t>NOC</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v/>
+        <v>301.68</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I35" t="n">
-        <v>50</v>
+        <v>63.4</v>
       </c>
       <c r="J35" t="n">
-        <v>47.3</v>
+        <v>35</v>
+      </c>
+      <c r="K35" t="n">
+        <v>90</v>
+      </c>
+      <c r="L35" t="n">
+        <v>2.96</v>
       </c>
       <c r="M35" t="n">
-        <v>32.2</v>
+        <v>37.6</v>
       </c>
       <c r="N35" t="n">
-        <v>21.6</v>
+        <v>43</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P35" t="n">
-        <v>71.8</v>
+        <v>50.2</v>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>FIRED</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>FLAT</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U35" t="inlineStr">
-        <is>
-          <t>Squeeze Fired, Divergence</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr"/>
       <c r="V35" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>NKE</t>
+          <t>NFLX</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v/>
+        <v>301.68</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D36" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I36" t="n">
-        <v>50</v>
+        <v>63.4</v>
       </c>
       <c r="J36" t="n">
-        <v>47.3</v>
+        <v>35</v>
+      </c>
+      <c r="K36" t="n">
+        <v>90</v>
+      </c>
+      <c r="L36" t="n">
+        <v>2.96</v>
       </c>
       <c r="M36" t="n">
-        <v>32.2</v>
-      </c>
-      <c r="N36" t="n">
-        <v>21.6</v>
+        <v>40.7</v>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P36" t="n">
-        <v>71.8</v>
+        <v>50.2</v>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>FIRED</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>FLAT</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U36" t="inlineStr">
-        <is>
-          <t>Squeeze Fired, Divergence</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr"/>
       <c r="V36" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>NSC</t>
+          <t>NEE</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v/>
+        <v>301.68</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I37" t="n">
-        <v>50</v>
+        <v>63.4</v>
       </c>
       <c r="J37" t="n">
-        <v>47.3</v>
+        <v>35</v>
+      </c>
+      <c r="K37" t="n">
+        <v>90</v>
+      </c>
+      <c r="L37" t="n">
+        <v>2.96</v>
       </c>
       <c r="M37" t="n">
-        <v>32.2</v>
+        <v>37.6</v>
       </c>
       <c r="N37" t="n">
-        <v>21.6</v>
+        <v>43</v>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P37" t="n">
-        <v>71.8</v>
+        <v>50.2</v>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>FIRED</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>FLAT</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U37" t="inlineStr">
-        <is>
-          <t>Squeeze Fired, Divergence</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U37" t="inlineStr"/>
       <c r="V37" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>MPC</t>
+          <t>MU</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v/>
+        <v>301.68</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I38" t="n">
-        <v>50</v>
+        <v>63.4</v>
       </c>
       <c r="J38" t="n">
-        <v>47.3</v>
+        <v>35</v>
+      </c>
+      <c r="K38" t="n">
+        <v>90</v>
+      </c>
+      <c r="L38" t="n">
+        <v>2.96</v>
       </c>
       <c r="M38" t="n">
-        <v>40.7</v>
+        <v>71.5</v>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P38" t="n">
-        <v>71.8</v>
+        <v>50.2</v>
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>FIRED</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>FLAT</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U38" t="inlineStr">
-        <is>
-          <t>Squeeze Fired, Divergence</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr"/>
       <c r="V38" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>NOC</t>
+          <t>REGN</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v/>
+        <v>60.55</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -3830,49 +3998,58 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I39" t="n">
-        <v>50</v>
+        <v>60.2</v>
       </c>
       <c r="J39" t="n">
-        <v>47.3</v>
+        <v>66</v>
+      </c>
+      <c r="K39" t="n">
+        <v>82.59999999999999</v>
+      </c>
+      <c r="L39" t="n">
+        <v>4.51</v>
       </c>
       <c r="M39" t="n">
-        <v>34.5</v>
+        <v>55.6</v>
+      </c>
+      <c r="N39" t="n">
+        <v>15</v>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P39" t="n">
-        <v>71.8</v>
+        <v>39.4</v>
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>FIRED</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>FLAT</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T39" t="inlineStr">
@@ -3880,29 +4057,25 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U39" t="inlineStr">
-        <is>
-          <t>Squeeze Fired, Divergence</t>
-        </is>
-      </c>
+      <c r="U39" t="inlineStr"/>
       <c r="V39" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>QCOM</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v/>
+        <v>60.55</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -3917,52 +4090,58 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I40" t="n">
-        <v>50</v>
+        <v>60.2</v>
       </c>
       <c r="J40" t="n">
-        <v>47.3</v>
+        <v>66</v>
+      </c>
+      <c r="K40" t="n">
+        <v>82.59999999999999</v>
+      </c>
+      <c r="L40" t="n">
+        <v>4.51</v>
       </c>
       <c r="M40" t="n">
-        <v>32.2</v>
+        <v>55.6</v>
       </c>
       <c r="N40" t="n">
-        <v>21.6</v>
+        <v>15</v>
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P40" t="n">
-        <v>43.1</v>
+        <v>39.4</v>
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>FIRED</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>FLAT</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T40" t="inlineStr">
@@ -3970,29 +4149,25 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U40" t="inlineStr">
-        <is>
-          <t>Squeeze Fired, Divergence</t>
-        </is>
-      </c>
+      <c r="U40" t="inlineStr"/>
       <c r="V40" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>ROP</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v/>
+        <v>60.55</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -4007,67 +4182,1259 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>60.2</v>
+      </c>
+      <c r="J41" t="n">
+        <v>66</v>
+      </c>
+      <c r="K41" t="n">
+        <v>82.59999999999999</v>
+      </c>
+      <c r="L41" t="n">
+        <v>4.51</v>
+      </c>
+      <c r="M41" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="N41" t="n">
+        <v>15</v>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P41" t="n">
+        <v>39.4</v>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr"/>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>RTX</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>60.55</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>60.2</v>
+      </c>
+      <c r="J42" t="n">
+        <v>66</v>
+      </c>
+      <c r="K42" t="n">
+        <v>82.59999999999999</v>
+      </c>
+      <c r="L42" t="n">
+        <v>4.51</v>
+      </c>
+      <c r="M42" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="N42" t="n">
+        <v>15</v>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P42" t="n">
+        <v>39.4</v>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U42" t="inlineStr"/>
+      <c r="V42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>ROST</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>60.55</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>60.2</v>
+      </c>
+      <c r="J43" t="n">
+        <v>66</v>
+      </c>
+      <c r="K43" t="n">
+        <v>82.59999999999999</v>
+      </c>
+      <c r="L43" t="n">
+        <v>4.51</v>
+      </c>
+      <c r="M43" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="N43" t="n">
+        <v>15</v>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P43" t="n">
+        <v>39.4</v>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U43" t="inlineStr"/>
+      <c r="V43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>PYPL</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>60.55</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
+        <v>60.2</v>
+      </c>
+      <c r="J44" t="n">
+        <v>66</v>
+      </c>
+      <c r="K44" t="n">
+        <v>82.59999999999999</v>
+      </c>
+      <c r="L44" t="n">
+        <v>4.51</v>
+      </c>
+      <c r="M44" t="n">
+        <v>38.3</v>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P44" t="n">
+        <v>39.4</v>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U44" t="inlineStr"/>
+      <c r="V44" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>SCHW</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>60.55</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I45" t="n">
+        <v>60.2</v>
+      </c>
+      <c r="J45" t="n">
+        <v>66</v>
+      </c>
+      <c r="K45" t="n">
+        <v>82.59999999999999</v>
+      </c>
+      <c r="L45" t="n">
+        <v>4.51</v>
+      </c>
+      <c r="M45" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="N45" t="n">
+        <v>15</v>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P45" t="n">
+        <v>39.4</v>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U45" t="inlineStr"/>
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>PSX</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>60.55</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I46" t="n">
+        <v>60.2</v>
+      </c>
+      <c r="J46" t="n">
+        <v>66</v>
+      </c>
+      <c r="K46" t="n">
+        <v>82.59999999999999</v>
+      </c>
+      <c r="L46" t="n">
+        <v>4.51</v>
+      </c>
+      <c r="M46" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="N46" t="n">
+        <v>15</v>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P46" t="n">
+        <v>39.4</v>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U46" t="inlineStr"/>
+      <c r="V46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>SBUX</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>60.55</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I47" t="n">
+        <v>60.2</v>
+      </c>
+      <c r="J47" t="n">
+        <v>66</v>
+      </c>
+      <c r="K47" t="n">
+        <v>82.59999999999999</v>
+      </c>
+      <c r="L47" t="n">
+        <v>4.51</v>
+      </c>
+      <c r="M47" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="N47" t="n">
+        <v>15</v>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P47" t="n">
+        <v>39.4</v>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U47" t="inlineStr"/>
+      <c r="V47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>MMC</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>47.51</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I48" t="n">
+        <v>59.6</v>
+      </c>
+      <c r="J48" t="n">
+        <v>35.5</v>
+      </c>
+      <c r="K48" t="n">
+        <v>94</v>
+      </c>
+      <c r="L48" t="n">
+        <v>2.91</v>
+      </c>
+      <c r="M48" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="N48" t="n">
+        <v>38.6</v>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P48" t="n">
+        <v>35</v>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U48" t="inlineStr"/>
+      <c r="V48" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>MRK</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>47.51</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
+        <v>59.6</v>
+      </c>
+      <c r="J49" t="n">
+        <v>35.5</v>
+      </c>
+      <c r="K49" t="n">
+        <v>94</v>
+      </c>
+      <c r="L49" t="n">
+        <v>2.91</v>
+      </c>
+      <c r="M49" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="N49" t="n">
+        <v>38.6</v>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P49" t="n">
+        <v>35</v>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U49" t="inlineStr"/>
+      <c r="V49" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>MPC</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>47.51</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I50" t="n">
+        <v>59.6</v>
+      </c>
+      <c r="J50" t="n">
+        <v>35.5</v>
+      </c>
+      <c r="K50" t="n">
+        <v>94</v>
+      </c>
+      <c r="L50" t="n">
+        <v>2.91</v>
+      </c>
+      <c r="M50" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="N50" t="n">
+        <v>38.6</v>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P50" t="n">
+        <v>40.5</v>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U50" t="inlineStr"/>
+      <c r="V50" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>MS</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>47.51</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I51" t="n">
+        <v>59.6</v>
+      </c>
+      <c r="J51" t="n">
+        <v>35.5</v>
+      </c>
+      <c r="K51" t="n">
+        <v>94</v>
+      </c>
+      <c r="L51" t="n">
+        <v>2.91</v>
+      </c>
+      <c r="M51" t="n">
+        <v>39.6</v>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P51" t="n">
+        <v>35</v>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U51" t="inlineStr"/>
+      <c r="V51" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>MO</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>47.51</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I52" t="n">
+        <v>59.6</v>
+      </c>
+      <c r="J52" t="n">
+        <v>35.5</v>
+      </c>
+      <c r="K52" t="n">
+        <v>94</v>
+      </c>
+      <c r="L52" t="n">
+        <v>2.91</v>
+      </c>
+      <c r="M52" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="N52" t="n">
+        <v>38.6</v>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P52" t="n">
+        <v>40.5</v>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U52" t="inlineStr"/>
+      <c r="V52" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>MMM</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>47.51</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I53" t="n">
+        <v>59.6</v>
+      </c>
+      <c r="J53" t="n">
+        <v>35.5</v>
+      </c>
+      <c r="K53" t="n">
+        <v>94</v>
+      </c>
+      <c r="L53" t="n">
+        <v>2.91</v>
+      </c>
+      <c r="M53" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="N53" t="n">
+        <v>38.6</v>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P53" t="n">
+        <v>35</v>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U53" t="inlineStr"/>
+      <c r="V53" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>BMY</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>364.42</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
           <t>NEUTRAL</t>
         </is>
       </c>
-      <c r="I41" t="n">
-        <v>50</v>
-      </c>
-      <c r="J41" t="n">
-        <v>47.3</v>
-      </c>
-      <c r="M41" t="n">
-        <v>32.2</v>
-      </c>
-      <c r="N41" t="n">
-        <v>21.6</v>
-      </c>
-      <c r="O41" t="inlineStr">
-        <is>
-          <t>Neutral</t>
-        </is>
-      </c>
-      <c r="P41" t="n">
-        <v>44.9</v>
-      </c>
-      <c r="Q41" t="inlineStr">
-        <is>
-          <t>FIRED</t>
-        </is>
-      </c>
-      <c r="R41" t="inlineStr">
-        <is>
-          <t>FLAT</t>
-        </is>
-      </c>
-      <c r="S41" t="inlineStr">
+      <c r="I54" t="n">
+        <v>58.5</v>
+      </c>
+      <c r="J54" t="n">
+        <v>60.2</v>
+      </c>
+      <c r="K54" t="n">
+        <v>52.3</v>
+      </c>
+      <c r="L54" t="n">
+        <v>5.01</v>
+      </c>
+      <c r="M54" t="n">
+        <v>65.7</v>
+      </c>
+      <c r="N54" t="n">
+        <v>81.2</v>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P54" t="n">
+        <v>67.7</v>
+      </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S54" t="inlineStr">
         <is>
           <t>green</t>
         </is>
       </c>
-      <c r="T41" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U41" t="inlineStr">
-        <is>
-          <t>Squeeze Fired, Divergence</t>
-        </is>
-      </c>
-      <c r="V41" t="inlineStr">
+      <c r="T54" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="U54" t="inlineStr"/>
+      <c r="V54" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan 19.03.2026 14:56 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V19"/>
+  <dimension ref="A1:V36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -448,7 +448,7 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="6" customWidth="1" min="10" max="10"/>
-    <col width="6" customWidth="1" min="11" max="11"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
     <col width="6" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
     <col width="9" customWidth="1" min="14" max="14"/>
@@ -577,11 +577,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>356.27</v>
+        <v>354.57</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,22 +614,22 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>72</v>
+        <v>73.5</v>
       </c>
       <c r="J2" t="n">
-        <v>69.2</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="K2" t="n">
         <v>90.7</v>
       </c>
       <c r="L2" t="n">
-        <v>8.94</v>
+        <v>9.140000000000001</v>
       </c>
       <c r="M2" t="n">
-        <v>89.09999999999999</v>
+        <v>89</v>
       </c>
       <c r="N2" t="n">
-        <v>45.4</v>
+        <v>45.1</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>57</v>
+        <v>54.8</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -669,11 +669,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MO</t>
+          <t>CVX</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>316.89</v>
+        <v>354.57</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -706,30 +706,30 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>69</v>
+        <v>73.5</v>
       </c>
       <c r="J3" t="n">
-        <v>60.3</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="K3" t="n">
-        <v>94.2</v>
+        <v>90.7</v>
       </c>
       <c r="L3" t="n">
-        <v>6.37</v>
+        <v>9.140000000000001</v>
       </c>
       <c r="M3" t="n">
-        <v>76.5</v>
+        <v>89</v>
       </c>
       <c r="N3" t="n">
-        <v>47.3</v>
+        <v>45.1</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P3" t="n">
-        <v>36.5</v>
+        <v>54.8</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -738,17 +738,17 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U3" t="inlineStr"/>
@@ -761,11 +761,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>MMM</t>
+          <t>CVS</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>316.89</v>
+        <v>354.57</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -798,30 +798,30 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>69</v>
+        <v>73.5</v>
       </c>
       <c r="J4" t="n">
-        <v>60.3</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="K4" t="n">
-        <v>94.2</v>
+        <v>90.7</v>
       </c>
       <c r="L4" t="n">
-        <v>6.37</v>
+        <v>9.140000000000001</v>
       </c>
       <c r="M4" t="n">
-        <v>76.5</v>
+        <v>89</v>
       </c>
       <c r="N4" t="n">
-        <v>47.3</v>
+        <v>45.1</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P4" t="n">
-        <v>36.5</v>
+        <v>54.8</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -830,17 +830,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U4" t="inlineStr"/>
@@ -853,11 +853,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>MMC</t>
+          <t>CSCO</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>316.89</v>
+        <v>354.57</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -890,30 +890,30 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>69</v>
+        <v>73.5</v>
       </c>
       <c r="J5" t="n">
-        <v>60.3</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="K5" t="n">
-        <v>94.2</v>
+        <v>90.7</v>
       </c>
       <c r="L5" t="n">
-        <v>6.37</v>
+        <v>9.140000000000001</v>
       </c>
       <c r="M5" t="n">
-        <v>76.5</v>
+        <v>89</v>
       </c>
       <c r="N5" t="n">
-        <v>47.3</v>
+        <v>45.1</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>36.5</v>
+        <v>54.8</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -922,17 +922,17 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U5" t="inlineStr"/>
@@ -945,11 +945,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>MCO</t>
+          <t>CTAS</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>316.89</v>
+        <v>354.57</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -982,30 +982,30 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>69</v>
+        <v>73.5</v>
       </c>
       <c r="J6" t="n">
-        <v>60.3</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="K6" t="n">
-        <v>94.2</v>
+        <v>90.7</v>
       </c>
       <c r="L6" t="n">
-        <v>6.37</v>
+        <v>9.140000000000001</v>
       </c>
       <c r="M6" t="n">
-        <v>76.5</v>
+        <v>89</v>
       </c>
       <c r="N6" t="n">
-        <v>47.3</v>
+        <v>45.1</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P6" t="n">
-        <v>38.9</v>
+        <v>54.8</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1014,17 +1014,17 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
@@ -1037,11 +1037,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>D</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>316.89</v>
+        <v>354.57</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1074,27 +1074,30 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>69</v>
+        <v>73.5</v>
       </c>
       <c r="J7" t="n">
-        <v>60.3</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="K7" t="n">
-        <v>94.2</v>
+        <v>90.7</v>
       </c>
       <c r="L7" t="n">
-        <v>6.37</v>
+        <v>9.140000000000001</v>
       </c>
       <c r="M7" t="n">
-        <v>31.3</v>
+        <v>89</v>
+      </c>
+      <c r="N7" t="n">
+        <v>45.1</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>36.5</v>
+        <v>54.8</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1103,17 +1106,17 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U7" t="inlineStr"/>
@@ -1126,30 +1129,30 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SO</t>
+          <t>COST</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>970.72</v>
+        <v>354.57</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1163,22 +1166,19 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>66.8</v>
+        <v>73.5</v>
       </c>
       <c r="J8" t="n">
-        <v>39.6</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="K8" t="n">
-        <v>98</v>
+        <v>90.7</v>
       </c>
       <c r="L8" t="n">
-        <v>3.13</v>
+        <v>9.140000000000001</v>
       </c>
       <c r="M8" t="n">
-        <v>31.8</v>
-      </c>
-      <c r="N8" t="n">
-        <v>48.3</v>
+        <v>23.6</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1186,7 +1186,7 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>54.3</v>
+        <v>54.8</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1200,12 +1200,12 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U8" t="inlineStr"/>
@@ -1218,11 +1218,11 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>BSX</t>
+          <t>AAPL</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>354.89</v>
+        <v>306.62</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1251,34 +1251,34 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>63</v>
+        <v>69.8</v>
       </c>
       <c r="J9" t="n">
-        <v>56.5</v>
+        <v>57.5</v>
       </c>
       <c r="K9" t="n">
-        <v>51.2</v>
+        <v>94.2</v>
       </c>
       <c r="L9" t="n">
-        <v>5.55</v>
+        <v>6.81</v>
       </c>
       <c r="M9" t="n">
-        <v>66.59999999999999</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="N9" t="n">
-        <v>85.2</v>
+        <v>46.4</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>50.5</v>
+        <v>49.8</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1310,11 +1310,11 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>BDX</t>
+          <t>AIG</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>354.89</v>
+        <v>306.62</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1343,34 +1343,34 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>63</v>
+        <v>69.8</v>
       </c>
       <c r="J10" t="n">
-        <v>56.5</v>
+        <v>57.5</v>
       </c>
       <c r="K10" t="n">
-        <v>51.2</v>
+        <v>94.2</v>
       </c>
       <c r="L10" t="n">
-        <v>5.55</v>
+        <v>6.81</v>
       </c>
       <c r="M10" t="n">
-        <v>66.59999999999999</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="N10" t="n">
-        <v>85.2</v>
+        <v>46.4</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>50.5</v>
+        <v>49.8</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1402,11 +1402,11 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>BMY</t>
+          <t>AEP</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>354.89</v>
+        <v>306.62</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1435,26 +1435,26 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>63</v>
+        <v>69.8</v>
       </c>
       <c r="J11" t="n">
-        <v>56.5</v>
+        <v>57.5</v>
       </c>
       <c r="K11" t="n">
-        <v>51.2</v>
+        <v>94.2</v>
       </c>
       <c r="L11" t="n">
-        <v>5.55</v>
+        <v>6.81</v>
       </c>
       <c r="M11" t="n">
-        <v>66.59999999999999</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="N11" t="n">
-        <v>85.2</v>
+        <v>46.4</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1462,7 +1462,7 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>48.1</v>
+        <v>53.7</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1494,11 +1494,11 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CAT</t>
+          <t>ADP</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>354.89</v>
+        <v>306.62</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1527,31 +1527,34 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>63</v>
+        <v>69.8</v>
       </c>
       <c r="J12" t="n">
-        <v>56.5</v>
+        <v>57.5</v>
       </c>
       <c r="K12" t="n">
-        <v>51.2</v>
+        <v>94.2</v>
       </c>
       <c r="L12" t="n">
-        <v>5.55</v>
+        <v>6.81</v>
       </c>
       <c r="M12" t="n">
-        <v>40.7</v>
+        <v>76.09999999999999</v>
+      </c>
+      <c r="N12" t="n">
+        <v>46.4</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>48.1</v>
+        <v>36.6</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1583,30 +1586,30 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>MDT</t>
+          <t>AON</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>47.59</v>
+        <v>306.62</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1620,22 +1623,22 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>59.6</v>
+        <v>69.8</v>
       </c>
       <c r="J13" t="n">
-        <v>36.2</v>
+        <v>57.5</v>
       </c>
       <c r="K13" t="n">
-        <v>90</v>
+        <v>94.2</v>
       </c>
       <c r="L13" t="n">
-        <v>2.75</v>
+        <v>6.81</v>
       </c>
       <c r="M13" t="n">
-        <v>28.3</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="N13" t="n">
-        <v>38.1</v>
+        <v>46.4</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1643,7 +1646,7 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>58</v>
+        <v>45.8</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1652,12 +1655,12 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
@@ -1679,7 +1682,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>47.59</v>
+        <v>210.83</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -1712,30 +1715,30 @@
         </is>
       </c>
       <c r="I14" t="n">
-        <v>59.6</v>
+        <v>67.7</v>
       </c>
       <c r="J14" t="n">
-        <v>36.2</v>
+        <v>31.2</v>
       </c>
       <c r="K14" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="L14" t="n">
-        <v>2.75</v>
+        <v>6.48</v>
       </c>
       <c r="M14" t="n">
-        <v>28.3</v>
+        <v>52.2</v>
       </c>
       <c r="N14" t="n">
-        <v>38.1</v>
+        <v>99.8</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P14" t="n">
-        <v>36.5</v>
+        <v>50</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1744,17 +1747,17 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U14" t="inlineStr"/>
@@ -1767,30 +1770,30 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CDW</t>
+          <t>JPM</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>59.4</v>
+        <v>210.83</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1804,30 +1807,27 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>58.6</v>
+        <v>67.7</v>
       </c>
       <c r="J15" t="n">
-        <v>64.09999999999999</v>
+        <v>31.2</v>
       </c>
       <c r="K15" t="n">
-        <v>81.40000000000001</v>
+        <v>100</v>
       </c>
       <c r="L15" t="n">
-        <v>4.61</v>
+        <v>6.48</v>
       </c>
       <c r="M15" t="n">
-        <v>55.4</v>
-      </c>
-      <c r="N15" t="n">
-        <v>14.4</v>
+        <v>34.7</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P15" t="n">
-        <v>44.3</v>
+        <v>50</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1841,12 +1841,12 @@
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U15" t="inlineStr"/>
@@ -1859,30 +1859,30 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CTSH</t>
+          <t>KLAC</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>59.4</v>
+        <v>210.83</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1896,22 +1896,22 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>58.6</v>
+        <v>67.7</v>
       </c>
       <c r="J16" t="n">
-        <v>64.09999999999999</v>
+        <v>31.2</v>
       </c>
       <c r="K16" t="n">
-        <v>81.40000000000001</v>
+        <v>100</v>
       </c>
       <c r="L16" t="n">
-        <v>4.61</v>
+        <v>6.48</v>
       </c>
       <c r="M16" t="n">
-        <v>55.4</v>
+        <v>52.2</v>
       </c>
       <c r="N16" t="n">
-        <v>14.4</v>
+        <v>99.8</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -1919,7 +1919,7 @@
         </is>
       </c>
       <c r="P16" t="n">
-        <v>52.4</v>
+        <v>50</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1933,12 +1933,12 @@
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U16" t="inlineStr"/>
@@ -1951,30 +1951,30 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>PH</t>
+          <t>KO</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>94.34999999999999</v>
+        <v>210.83</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1988,22 +1988,22 @@
         </is>
       </c>
       <c r="I17" t="n">
-        <v>55.5</v>
+        <v>67.7</v>
       </c>
       <c r="J17" t="n">
-        <v>59.1</v>
+        <v>31.2</v>
       </c>
       <c r="K17" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="L17" t="n">
-        <v>2.57</v>
+        <v>6.48</v>
       </c>
       <c r="M17" t="n">
-        <v>50.8</v>
+        <v>52.2</v>
       </c>
       <c r="N17" t="n">
-        <v>92.2</v>
+        <v>99.8</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -2011,7 +2011,7 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>52.5</v>
+        <v>50</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -2025,12 +2025,12 @@
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U17" t="inlineStr"/>
@@ -2043,30 +2043,30 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>PEP</t>
+          <t>PH</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>94.34999999999999</v>
+        <v>953</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -2080,22 +2080,22 @@
         </is>
       </c>
       <c r="I18" t="n">
-        <v>55.5</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="J18" t="n">
-        <v>59.1</v>
+        <v>36.4</v>
       </c>
       <c r="K18" t="n">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="L18" t="n">
-        <v>2.57</v>
+        <v>3.03</v>
       </c>
       <c r="M18" t="n">
-        <v>50.8</v>
+        <v>31.8</v>
       </c>
       <c r="N18" t="n">
-        <v>92.2</v>
+        <v>48.6</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -2103,7 +2103,7 @@
         </is>
       </c>
       <c r="P18" t="n">
-        <v>52.5</v>
+        <v>51.8</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -2117,12 +2117,12 @@
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U18" t="inlineStr"/>
@@ -2135,30 +2135,30 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>PFE</t>
+          <t>ISRG</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>94.34999999999999</v>
+        <v>128.38</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2172,30 +2172,30 @@
         </is>
       </c>
       <c r="I19" t="n">
-        <v>55.5</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="J19" t="n">
-        <v>59.1</v>
+        <v>39.3</v>
       </c>
       <c r="K19" t="n">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="L19" t="n">
-        <v>2.57</v>
+        <v>5.28</v>
       </c>
       <c r="M19" t="n">
-        <v>50.8</v>
+        <v>48.4</v>
       </c>
       <c r="N19" t="n">
-        <v>92.2</v>
+        <v>59.7</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P19" t="n">
-        <v>52.5</v>
+        <v>31.2</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -2209,16 +2209,1580 @@
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U19" t="inlineStr"/>
       <c r="V19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>INTU</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>128.38</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>64.40000000000001</v>
+      </c>
+      <c r="J20" t="n">
+        <v>39.3</v>
+      </c>
+      <c r="K20" t="n">
+        <v>92</v>
+      </c>
+      <c r="L20" t="n">
+        <v>5.28</v>
+      </c>
+      <c r="M20" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="N20" t="n">
+        <v>59.7</v>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P20" t="n">
+        <v>31.2</v>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr"/>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>ICE</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>128.38</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>64.40000000000001</v>
+      </c>
+      <c r="J21" t="n">
+        <v>39.3</v>
+      </c>
+      <c r="K21" t="n">
+        <v>92</v>
+      </c>
+      <c r="L21" t="n">
+        <v>5.28</v>
+      </c>
+      <c r="M21" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="N21" t="n">
+        <v>59.7</v>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P21" t="n">
+        <v>31.2</v>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr"/>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>INTC</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>128.38</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>64.40000000000001</v>
+      </c>
+      <c r="J22" t="n">
+        <v>39.3</v>
+      </c>
+      <c r="K22" t="n">
+        <v>92</v>
+      </c>
+      <c r="L22" t="n">
+        <v>5.28</v>
+      </c>
+      <c r="M22" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="N22" t="n">
+        <v>59.7</v>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P22" t="n">
+        <v>44.7</v>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr"/>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>HSY</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>128.38</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>64.40000000000001</v>
+      </c>
+      <c r="J23" t="n">
+        <v>39.3</v>
+      </c>
+      <c r="K23" t="n">
+        <v>92</v>
+      </c>
+      <c r="L23" t="n">
+        <v>5.28</v>
+      </c>
+      <c r="M23" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="N23" t="n">
+        <v>59.7</v>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P23" t="n">
+        <v>31.2</v>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr"/>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>JNJ</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>128.38</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>64.40000000000001</v>
+      </c>
+      <c r="J24" t="n">
+        <v>39.3</v>
+      </c>
+      <c r="K24" t="n">
+        <v>92</v>
+      </c>
+      <c r="L24" t="n">
+        <v>5.28</v>
+      </c>
+      <c r="M24" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="N24" t="n">
+        <v>59.7</v>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P24" t="n">
+        <v>31.2</v>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr"/>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>ITW</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>128.38</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>64.40000000000001</v>
+      </c>
+      <c r="J25" t="n">
+        <v>39.3</v>
+      </c>
+      <c r="K25" t="n">
+        <v>92</v>
+      </c>
+      <c r="L25" t="n">
+        <v>5.28</v>
+      </c>
+      <c r="M25" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="N25" t="n">
+        <v>59.7</v>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P25" t="n">
+        <v>44.7</v>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr"/>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>HUM</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>128.38</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>64.40000000000001</v>
+      </c>
+      <c r="J26" t="n">
+        <v>39.3</v>
+      </c>
+      <c r="K26" t="n">
+        <v>92</v>
+      </c>
+      <c r="L26" t="n">
+        <v>5.28</v>
+      </c>
+      <c r="M26" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="N26" t="n">
+        <v>59.7</v>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P26" t="n">
+        <v>31.2</v>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr"/>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>HON</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>128.38</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>64.40000000000001</v>
+      </c>
+      <c r="J27" t="n">
+        <v>39.3</v>
+      </c>
+      <c r="K27" t="n">
+        <v>92</v>
+      </c>
+      <c r="L27" t="n">
+        <v>5.28</v>
+      </c>
+      <c r="M27" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="N27" t="n">
+        <v>59.7</v>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P27" t="n">
+        <v>44.7</v>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr"/>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>IBM</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>128.38</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>64.40000000000001</v>
+      </c>
+      <c r="J28" t="n">
+        <v>39.3</v>
+      </c>
+      <c r="K28" t="n">
+        <v>92</v>
+      </c>
+      <c r="L28" t="n">
+        <v>5.28</v>
+      </c>
+      <c r="M28" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="N28" t="n">
+        <v>59.7</v>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P28" t="n">
+        <v>44.7</v>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr"/>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>352.39</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>63.4</v>
+      </c>
+      <c r="J29" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="K29" t="n">
+        <v>51.2</v>
+      </c>
+      <c r="L29" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="M29" t="n">
+        <v>67</v>
+      </c>
+      <c r="N29" t="n">
+        <v>86.90000000000001</v>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P29" t="n">
+        <v>42</v>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr"/>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>352.39</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>63.4</v>
+      </c>
+      <c r="J30" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="K30" t="n">
+        <v>51.2</v>
+      </c>
+      <c r="L30" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="M30" t="n">
+        <v>67</v>
+      </c>
+      <c r="N30" t="n">
+        <v>86.90000000000001</v>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P30" t="n">
+        <v>42</v>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr"/>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>MSCI</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>352.39</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>63.4</v>
+      </c>
+      <c r="J31" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="K31" t="n">
+        <v>51.2</v>
+      </c>
+      <c r="L31" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="M31" t="n">
+        <v>67</v>
+      </c>
+      <c r="N31" t="n">
+        <v>86.90000000000001</v>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P31" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr"/>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>MS</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>352.39</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>63.4</v>
+      </c>
+      <c r="J32" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="K32" t="n">
+        <v>51.2</v>
+      </c>
+      <c r="L32" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="M32" t="n">
+        <v>67</v>
+      </c>
+      <c r="N32" t="n">
+        <v>86.90000000000001</v>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P32" t="n">
+        <v>42</v>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr"/>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>MMM</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>46.38</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>56.4</v>
+      </c>
+      <c r="J33" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="K33" t="n">
+        <v>90</v>
+      </c>
+      <c r="L33" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="M33" t="n">
+        <v>27.4</v>
+      </c>
+      <c r="N33" t="n">
+        <v>35.8</v>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P33" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr"/>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>MPC</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>46.38</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>56.4</v>
+      </c>
+      <c r="J34" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="K34" t="n">
+        <v>90</v>
+      </c>
+      <c r="L34" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="M34" t="n">
+        <v>27.4</v>
+      </c>
+      <c r="N34" t="n">
+        <v>35.8</v>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P34" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr"/>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>MO</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>46.38</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>56.4</v>
+      </c>
+      <c r="J35" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="K35" t="n">
+        <v>90</v>
+      </c>
+      <c r="L35" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="M35" t="n">
+        <v>27.4</v>
+      </c>
+      <c r="N35" t="n">
+        <v>35.8</v>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P35" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr"/>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>MMC</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>46.38</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>56.4</v>
+      </c>
+      <c r="J36" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="K36" t="n">
+        <v>90</v>
+      </c>
+      <c r="L36" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="M36" t="n">
+        <v>27.4</v>
+      </c>
+      <c r="N36" t="n">
+        <v>35.8</v>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P36" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr"/>
+      <c r="V36" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Scan 20.03.2026 14:52 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V36"/>
+  <dimension ref="A1:V43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -444,11 +444,11 @@
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="6" customWidth="1" min="10" max="10"/>
-    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="6" customWidth="1" min="11" max="11"/>
     <col width="6" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
     <col width="9" customWidth="1" min="14" max="14"/>
@@ -458,7 +458,7 @@
     <col width="15" customWidth="1" min="18" max="18"/>
     <col width="11" customWidth="1" min="19" max="19"/>
     <col width="11" customWidth="1" min="20" max="20"/>
-    <col width="10" customWidth="1" min="21" max="21"/>
+    <col width="25" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
@@ -577,11 +577,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>MCHP</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>354.57</v>
+        <v>347.73</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,16 +614,16 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>73.5</v>
+        <v>73.3</v>
       </c>
       <c r="J2" t="n">
-        <v>68.90000000000001</v>
+        <v>67.7</v>
       </c>
       <c r="K2" t="n">
-        <v>90.7</v>
+        <v>87.2</v>
       </c>
       <c r="L2" t="n">
-        <v>9.140000000000001</v>
+        <v>9.470000000000001</v>
       </c>
       <c r="M2" t="n">
         <v>89</v>
@@ -633,11 +633,11 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>54.8</v>
+        <v>32.9</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -646,17 +646,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
@@ -669,11 +669,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CVX</t>
+          <t>LIN</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>354.57</v>
+        <v>347.73</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -706,16 +706,16 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>73.5</v>
+        <v>73.3</v>
       </c>
       <c r="J3" t="n">
-        <v>68.90000000000001</v>
+        <v>67.7</v>
       </c>
       <c r="K3" t="n">
-        <v>90.7</v>
+        <v>87.2</v>
       </c>
       <c r="L3" t="n">
-        <v>9.140000000000001</v>
+        <v>9.470000000000001</v>
       </c>
       <c r="M3" t="n">
         <v>89</v>
@@ -725,11 +725,11 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P3" t="n">
-        <v>54.8</v>
+        <v>32.9</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -738,17 +738,17 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U3" t="inlineStr"/>
@@ -761,15 +761,15 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CVS</t>
+          <t>EW</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>354.57</v>
+        <v>132.13</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -784,44 +784,44 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>73.5</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="J4" t="n">
-        <v>68.90000000000001</v>
+        <v>46.9</v>
       </c>
       <c r="K4" t="n">
-        <v>90.7</v>
+        <v>15</v>
       </c>
       <c r="L4" t="n">
-        <v>9.140000000000001</v>
+        <v>3.99</v>
       </c>
       <c r="M4" t="n">
-        <v>89</v>
+        <v>52.9</v>
       </c>
       <c r="N4" t="n">
-        <v>45.1</v>
+        <v>46.4</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P4" t="n">
-        <v>54.8</v>
+        <v>43.5</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -830,12 +830,12 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -843,25 +843,29 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr"/>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>FCX</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>354.57</v>
+        <v>132.13</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -876,44 +880,41 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>73.5</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="J5" t="n">
-        <v>68.90000000000001</v>
+        <v>46.9</v>
       </c>
       <c r="K5" t="n">
-        <v>90.7</v>
+        <v>15</v>
       </c>
       <c r="L5" t="n">
-        <v>9.140000000000001</v>
+        <v>3.99</v>
       </c>
       <c r="M5" t="n">
-        <v>89</v>
-      </c>
-      <c r="N5" t="n">
-        <v>45.1</v>
+        <v>58.8</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>54.8</v>
+        <v>43.5</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -922,12 +923,12 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -935,25 +936,29 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr"/>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CTAS</t>
+          <t>ETN</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>354.57</v>
+        <v>132.13</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -968,44 +973,41 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>73.5</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="J6" t="n">
-        <v>68.90000000000001</v>
+        <v>46.9</v>
       </c>
       <c r="K6" t="n">
-        <v>90.7</v>
+        <v>15</v>
       </c>
       <c r="L6" t="n">
-        <v>9.140000000000001</v>
+        <v>3.99</v>
       </c>
       <c r="M6" t="n">
-        <v>89</v>
-      </c>
-      <c r="N6" t="n">
-        <v>45.1</v>
+        <v>38.8</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P6" t="n">
-        <v>54.8</v>
+        <v>43.5</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1014,12 +1016,12 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
@@ -1027,25 +1029,29 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr"/>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>FICO</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>354.57</v>
+        <v>132.13</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -1060,44 +1066,41 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>73.5</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="J7" t="n">
-        <v>68.90000000000001</v>
+        <v>46.9</v>
       </c>
       <c r="K7" t="n">
-        <v>90.7</v>
+        <v>15</v>
       </c>
       <c r="L7" t="n">
-        <v>9.140000000000001</v>
+        <v>3.99</v>
       </c>
       <c r="M7" t="n">
-        <v>89</v>
-      </c>
-      <c r="N7" t="n">
-        <v>45.1</v>
+        <v>58.5</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>54.8</v>
+        <v>43.5</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1106,12 +1109,12 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
@@ -1119,40 +1122,44 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr"/>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>COST</t>
+          <t>SYK</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>354.57</v>
+        <v>962.77</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1166,27 +1173,30 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>73.5</v>
+        <v>67.5</v>
       </c>
       <c r="J8" t="n">
-        <v>68.90000000000001</v>
+        <v>38.2</v>
       </c>
       <c r="K8" t="n">
-        <v>90.7</v>
+        <v>96</v>
       </c>
       <c r="L8" t="n">
-        <v>9.140000000000001</v>
+        <v>2.84</v>
       </c>
       <c r="M8" t="n">
-        <v>23.6</v>
+        <v>31.3</v>
+      </c>
+      <c r="N8" t="n">
+        <v>47.1</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>54.8</v>
+        <v>39.9</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1200,12 +1210,12 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U8" t="inlineStr"/>
@@ -1218,11 +1228,11 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>GE</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>306.62</v>
+        <v>347.69</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1251,34 +1261,31 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>69.8</v>
+        <v>62.8</v>
       </c>
       <c r="J9" t="n">
-        <v>57.5</v>
+        <v>54</v>
       </c>
       <c r="K9" t="n">
-        <v>94.2</v>
+        <v>51.2</v>
       </c>
       <c r="L9" t="n">
-        <v>6.81</v>
+        <v>5.92</v>
       </c>
       <c r="M9" t="n">
-        <v>76.09999999999999</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="N9" t="n">
-        <v>46.4</v>
+        <v>90.8</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P9" t="n">
-        <v>49.8</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1300,21 +1307,25 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U9" t="inlineStr"/>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AIG</t>
+          <t>GS</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>306.62</v>
+        <v>347.69</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1343,34 +1354,31 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>69.8</v>
+        <v>62.8</v>
       </c>
       <c r="J10" t="n">
-        <v>57.5</v>
+        <v>54</v>
       </c>
       <c r="K10" t="n">
-        <v>94.2</v>
+        <v>51.2</v>
       </c>
       <c r="L10" t="n">
-        <v>6.81</v>
+        <v>5.92</v>
       </c>
       <c r="M10" t="n">
-        <v>76.09999999999999</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="N10" t="n">
-        <v>46.4</v>
+        <v>90.8</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P10" t="n">
-        <v>49.8</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1392,21 +1400,25 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U10" t="inlineStr"/>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>AEP</t>
+          <t>HD</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>306.62</v>
+        <v>347.69</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1435,34 +1447,31 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>69.8</v>
+        <v>62.8</v>
       </c>
       <c r="J11" t="n">
-        <v>57.5</v>
+        <v>54</v>
       </c>
       <c r="K11" t="n">
-        <v>94.2</v>
+        <v>51.2</v>
       </c>
       <c r="L11" t="n">
-        <v>6.81</v>
+        <v>5.92</v>
       </c>
       <c r="M11" t="n">
-        <v>76.09999999999999</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="N11" t="n">
-        <v>46.4</v>
+        <v>90.8</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P11" t="n">
-        <v>53.7</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1484,21 +1493,25 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U11" t="inlineStr"/>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ADP</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>306.62</v>
+        <v>112.58</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1531,30 +1544,30 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>69.8</v>
+        <v>59.6</v>
       </c>
       <c r="J12" t="n">
-        <v>57.5</v>
+        <v>50.3</v>
       </c>
       <c r="K12" t="n">
-        <v>94.2</v>
+        <v>90.7</v>
       </c>
       <c r="L12" t="n">
-        <v>6.81</v>
+        <v>5.41</v>
       </c>
       <c r="M12" t="n">
-        <v>76.09999999999999</v>
+        <v>51.7</v>
       </c>
       <c r="N12" t="n">
-        <v>46.4</v>
+        <v>27</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>36.6</v>
+        <v>46.6</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1586,11 +1599,11 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>AON</t>
+          <t>REGN</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>306.62</v>
+        <v>112.58</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -1623,30 +1636,30 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>69.8</v>
+        <v>59.6</v>
       </c>
       <c r="J13" t="n">
-        <v>57.5</v>
+        <v>50.3</v>
       </c>
       <c r="K13" t="n">
-        <v>94.2</v>
+        <v>90.7</v>
       </c>
       <c r="L13" t="n">
-        <v>6.81</v>
+        <v>5.41</v>
       </c>
       <c r="M13" t="n">
-        <v>76.09999999999999</v>
+        <v>51.7</v>
       </c>
       <c r="N13" t="n">
-        <v>46.4</v>
+        <v>27</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>45.8</v>
+        <v>30.3</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1678,30 +1691,30 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>KHC</t>
+          <t>PSX</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>210.83</v>
+        <v>112.58</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1715,30 +1728,30 @@
         </is>
       </c>
       <c r="I14" t="n">
-        <v>67.7</v>
+        <v>59.6</v>
       </c>
       <c r="J14" t="n">
-        <v>31.2</v>
+        <v>50.3</v>
       </c>
       <c r="K14" t="n">
-        <v>100</v>
+        <v>90.7</v>
       </c>
       <c r="L14" t="n">
-        <v>6.48</v>
+        <v>5.41</v>
       </c>
       <c r="M14" t="n">
-        <v>52.2</v>
+        <v>51.7</v>
       </c>
       <c r="N14" t="n">
-        <v>99.8</v>
+        <v>27</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P14" t="n">
-        <v>50</v>
+        <v>30.3</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1752,12 +1765,12 @@
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U14" t="inlineStr"/>
@@ -1770,30 +1783,30 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>JPM</t>
+          <t>PYPL</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>210.83</v>
+        <v>112.58</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1807,27 +1820,30 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>67.7</v>
+        <v>59.6</v>
       </c>
       <c r="J15" t="n">
-        <v>31.2</v>
+        <v>50.3</v>
       </c>
       <c r="K15" t="n">
-        <v>100</v>
+        <v>90.7</v>
       </c>
       <c r="L15" t="n">
-        <v>6.48</v>
+        <v>5.41</v>
       </c>
       <c r="M15" t="n">
-        <v>34.7</v>
+        <v>51.7</v>
+      </c>
+      <c r="N15" t="n">
+        <v>27</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P15" t="n">
-        <v>50</v>
+        <v>30.3</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1841,12 +1857,12 @@
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U15" t="inlineStr"/>
@@ -1859,30 +1875,30 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>KLAC</t>
+          <t>PH</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>210.83</v>
+        <v>112.58</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1896,30 +1912,30 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>67.7</v>
+        <v>59.6</v>
       </c>
       <c r="J16" t="n">
-        <v>31.2</v>
+        <v>50.3</v>
       </c>
       <c r="K16" t="n">
-        <v>100</v>
+        <v>90.7</v>
       </c>
       <c r="L16" t="n">
-        <v>6.48</v>
+        <v>5.41</v>
       </c>
       <c r="M16" t="n">
-        <v>52.2</v>
+        <v>51.7</v>
       </c>
       <c r="N16" t="n">
-        <v>99.8</v>
+        <v>27</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>50</v>
+        <v>32.7</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1933,12 +1949,12 @@
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U16" t="inlineStr"/>
@@ -1951,30 +1967,30 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>KO</t>
+          <t>PSA</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>210.83</v>
+        <v>112.58</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1988,30 +2004,30 @@
         </is>
       </c>
       <c r="I17" t="n">
-        <v>67.7</v>
+        <v>59.6</v>
       </c>
       <c r="J17" t="n">
-        <v>31.2</v>
+        <v>50.3</v>
       </c>
       <c r="K17" t="n">
-        <v>100</v>
+        <v>90.7</v>
       </c>
       <c r="L17" t="n">
-        <v>6.48</v>
+        <v>5.41</v>
       </c>
       <c r="M17" t="n">
-        <v>52.2</v>
+        <v>51.7</v>
       </c>
       <c r="N17" t="n">
-        <v>99.8</v>
+        <v>27</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P17" t="n">
-        <v>50</v>
+        <v>30.3</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -2025,12 +2041,12 @@
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U17" t="inlineStr"/>
@@ -2043,30 +2059,30 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>PH</t>
+          <t>PG</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>953</v>
+        <v>112.58</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -2080,22 +2096,22 @@
         </is>
       </c>
       <c r="I18" t="n">
-        <v>65.90000000000001</v>
+        <v>59.6</v>
       </c>
       <c r="J18" t="n">
-        <v>36.4</v>
+        <v>50.3</v>
       </c>
       <c r="K18" t="n">
-        <v>98</v>
+        <v>90.7</v>
       </c>
       <c r="L18" t="n">
-        <v>3.03</v>
+        <v>5.41</v>
       </c>
       <c r="M18" t="n">
-        <v>31.8</v>
+        <v>51.7</v>
       </c>
       <c r="N18" t="n">
-        <v>48.6</v>
+        <v>27</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -2103,7 +2119,7 @@
         </is>
       </c>
       <c r="P18" t="n">
-        <v>51.8</v>
+        <v>46.6</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -2117,12 +2133,12 @@
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U18" t="inlineStr"/>
@@ -2135,30 +2151,30 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ISRG</t>
+          <t>PM</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>128.38</v>
+        <v>112.58</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2172,22 +2188,22 @@
         </is>
       </c>
       <c r="I19" t="n">
-        <v>64.40000000000001</v>
+        <v>59.6</v>
       </c>
       <c r="J19" t="n">
-        <v>39.3</v>
+        <v>50.3</v>
       </c>
       <c r="K19" t="n">
-        <v>92</v>
+        <v>90.7</v>
       </c>
       <c r="L19" t="n">
-        <v>5.28</v>
+        <v>5.41</v>
       </c>
       <c r="M19" t="n">
-        <v>48.4</v>
+        <v>51.7</v>
       </c>
       <c r="N19" t="n">
-        <v>59.7</v>
+        <v>27</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -2195,7 +2211,7 @@
         </is>
       </c>
       <c r="P19" t="n">
-        <v>31.2</v>
+        <v>32.7</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -2209,12 +2225,12 @@
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U19" t="inlineStr"/>
@@ -2227,30 +2243,30 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>INTU</t>
+          <t>PNC</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>128.38</v>
+        <v>112.58</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -2264,22 +2280,22 @@
         </is>
       </c>
       <c r="I20" t="n">
-        <v>64.40000000000001</v>
+        <v>59.6</v>
       </c>
       <c r="J20" t="n">
-        <v>39.3</v>
+        <v>50.3</v>
       </c>
       <c r="K20" t="n">
-        <v>92</v>
+        <v>90.7</v>
       </c>
       <c r="L20" t="n">
-        <v>5.28</v>
+        <v>5.41</v>
       </c>
       <c r="M20" t="n">
-        <v>48.4</v>
+        <v>51.7</v>
       </c>
       <c r="N20" t="n">
-        <v>59.7</v>
+        <v>27</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -2287,7 +2303,7 @@
         </is>
       </c>
       <c r="P20" t="n">
-        <v>31.2</v>
+        <v>32.7</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
@@ -2301,12 +2317,12 @@
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U20" t="inlineStr"/>
@@ -2319,30 +2335,30 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ICE</t>
+          <t>QCOM</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>128.38</v>
+        <v>112.58</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2356,22 +2372,22 @@
         </is>
       </c>
       <c r="I21" t="n">
-        <v>64.40000000000001</v>
+        <v>59.6</v>
       </c>
       <c r="J21" t="n">
-        <v>39.3</v>
+        <v>50.3</v>
       </c>
       <c r="K21" t="n">
-        <v>92</v>
+        <v>90.7</v>
       </c>
       <c r="L21" t="n">
-        <v>5.28</v>
+        <v>5.41</v>
       </c>
       <c r="M21" t="n">
-        <v>48.4</v>
+        <v>51.7</v>
       </c>
       <c r="N21" t="n">
-        <v>59.7</v>
+        <v>27</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
@@ -2379,7 +2395,7 @@
         </is>
       </c>
       <c r="P21" t="n">
-        <v>31.2</v>
+        <v>32.7</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
@@ -2393,12 +2409,12 @@
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U21" t="inlineStr"/>
@@ -2411,30 +2427,30 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>INTC</t>
+          <t>PGR</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>128.38</v>
+        <v>112.58</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -2448,30 +2464,30 @@
         </is>
       </c>
       <c r="I22" t="n">
-        <v>64.40000000000001</v>
+        <v>59.6</v>
       </c>
       <c r="J22" t="n">
-        <v>39.3</v>
+        <v>50.3</v>
       </c>
       <c r="K22" t="n">
-        <v>92</v>
+        <v>90.7</v>
       </c>
       <c r="L22" t="n">
-        <v>5.28</v>
+        <v>5.41</v>
       </c>
       <c r="M22" t="n">
-        <v>48.4</v>
+        <v>51.7</v>
       </c>
       <c r="N22" t="n">
-        <v>59.7</v>
+        <v>27</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P22" t="n">
-        <v>44.7</v>
+        <v>32.7</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
@@ -2485,12 +2501,12 @@
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U22" t="inlineStr"/>
@@ -2503,71 +2519,71 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>HSY</t>
+          <t>GEHC</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>128.38</v>
+        <v>481.02</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I23" t="n">
-        <v>64.40000000000001</v>
+        <v>55.3</v>
       </c>
       <c r="J23" t="n">
-        <v>39.3</v>
+        <v>43.5</v>
       </c>
       <c r="K23" t="n">
-        <v>92</v>
+        <v>7</v>
       </c>
       <c r="L23" t="n">
-        <v>5.28</v>
+        <v>3.58</v>
       </c>
       <c r="M23" t="n">
-        <v>48.4</v>
+        <v>31.9</v>
       </c>
       <c r="N23" t="n">
-        <v>59.7</v>
+        <v>20</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P23" t="n">
-        <v>31.2</v>
+        <v>53.1</v>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
@@ -2577,89 +2593,93 @@
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U23" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence</t>
+        </is>
+      </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>JNJ</t>
+          <t>FANG</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>128.38</v>
+        <v>481.02</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I24" t="n">
-        <v>64.40000000000001</v>
+        <v>55.3</v>
       </c>
       <c r="J24" t="n">
-        <v>39.3</v>
+        <v>43.5</v>
       </c>
       <c r="K24" t="n">
-        <v>92</v>
+        <v>7</v>
       </c>
       <c r="L24" t="n">
-        <v>5.28</v>
+        <v>3.58</v>
       </c>
       <c r="M24" t="n">
-        <v>48.4</v>
+        <v>31.9</v>
       </c>
       <c r="N24" t="n">
-        <v>59.7</v>
+        <v>20</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P24" t="n">
-        <v>31.2</v>
+        <v>53.1</v>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
@@ -2669,77 +2689,81 @@
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U24" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence</t>
+        </is>
+      </c>
       <c r="V24" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>ITW</t>
+          <t>EA</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>128.38</v>
+        <v>481.02</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I25" t="n">
-        <v>64.40000000000001</v>
+        <v>55.3</v>
       </c>
       <c r="J25" t="n">
-        <v>39.3</v>
+        <v>43.5</v>
       </c>
       <c r="K25" t="n">
-        <v>92</v>
+        <v>7</v>
       </c>
       <c r="L25" t="n">
-        <v>5.28</v>
+        <v>3.58</v>
       </c>
       <c r="M25" t="n">
-        <v>48.4</v>
+        <v>31.9</v>
       </c>
       <c r="N25" t="n">
-        <v>59.7</v>
+        <v>20</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
@@ -2747,11 +2771,11 @@
         </is>
       </c>
       <c r="P25" t="n">
-        <v>44.7</v>
+        <v>53.1</v>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
@@ -2761,89 +2785,93 @@
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U25" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence</t>
+        </is>
+      </c>
       <c r="V25" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>HUM</t>
+          <t>DXCM</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>128.38</v>
+        <v>481.02</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D26" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I26" t="n">
-        <v>64.40000000000001</v>
+        <v>55.3</v>
       </c>
       <c r="J26" t="n">
-        <v>39.3</v>
+        <v>43.5</v>
       </c>
       <c r="K26" t="n">
-        <v>92</v>
+        <v>7</v>
       </c>
       <c r="L26" t="n">
-        <v>5.28</v>
+        <v>3.58</v>
       </c>
       <c r="M26" t="n">
-        <v>48.4</v>
+        <v>31.9</v>
       </c>
       <c r="N26" t="n">
-        <v>59.7</v>
+        <v>20</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P26" t="n">
-        <v>31.2</v>
+        <v>53.4</v>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
@@ -2853,77 +2881,78 @@
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U26" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence</t>
+        </is>
+      </c>
       <c r="V26" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>HON</t>
+          <t>KDP</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>128.38</v>
+        <v>481.02</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D27" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I27" t="n">
-        <v>64.40000000000001</v>
+        <v>55.3</v>
       </c>
       <c r="J27" t="n">
-        <v>39.3</v>
+        <v>43.5</v>
       </c>
       <c r="K27" t="n">
-        <v>92</v>
+        <v>7</v>
       </c>
       <c r="L27" t="n">
-        <v>5.28</v>
+        <v>3.58</v>
       </c>
       <c r="M27" t="n">
-        <v>48.4</v>
-      </c>
-      <c r="N27" t="n">
-        <v>59.7</v>
+        <v>30.3</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -2931,11 +2960,11 @@
         </is>
       </c>
       <c r="P27" t="n">
-        <v>44.7</v>
+        <v>53.4</v>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
@@ -2945,77 +2974,78 @@
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U27" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence</t>
+        </is>
+      </c>
       <c r="V27" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>IBM</t>
+          <t>DDOG</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>128.38</v>
+        <v>481.02</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D28" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I28" t="n">
-        <v>64.40000000000001</v>
+        <v>55.3</v>
       </c>
       <c r="J28" t="n">
-        <v>39.3</v>
+        <v>43.5</v>
       </c>
       <c r="K28" t="n">
-        <v>92</v>
+        <v>7</v>
       </c>
       <c r="L28" t="n">
-        <v>5.28</v>
+        <v>3.58</v>
       </c>
       <c r="M28" t="n">
-        <v>48.4</v>
-      </c>
-      <c r="N28" t="n">
-        <v>59.7</v>
+        <v>55</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
@@ -3023,11 +3053,11 @@
         </is>
       </c>
       <c r="P28" t="n">
-        <v>44.7</v>
+        <v>53.1</v>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
@@ -3037,33 +3067,37 @@
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U28" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence</t>
+        </is>
+      </c>
       <c r="V28" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>DLTR</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>352.39</v>
+        <v>481.02</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -3078,48 +3112,45 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I29" t="n">
-        <v>63.4</v>
+        <v>55.3</v>
       </c>
       <c r="J29" t="n">
-        <v>55.6</v>
+        <v>43.5</v>
       </c>
       <c r="K29" t="n">
-        <v>51.2</v>
+        <v>7</v>
       </c>
       <c r="L29" t="n">
-        <v>5.7</v>
+        <v>3.58</v>
       </c>
       <c r="M29" t="n">
-        <v>67</v>
-      </c>
-      <c r="N29" t="n">
-        <v>86.90000000000001</v>
+        <v>42.1</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P29" t="n">
-        <v>42</v>
+        <v>53.4</v>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
@@ -3137,25 +3168,29 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U29" t="inlineStr"/>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence</t>
+        </is>
+      </c>
       <c r="V29" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>CTSH</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>352.39</v>
+        <v>481.02</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -3170,48 +3205,48 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I30" t="n">
-        <v>63.4</v>
+        <v>55.3</v>
       </c>
       <c r="J30" t="n">
-        <v>55.6</v>
+        <v>43.5</v>
       </c>
       <c r="K30" t="n">
-        <v>51.2</v>
+        <v>7</v>
       </c>
       <c r="L30" t="n">
-        <v>5.7</v>
+        <v>3.58</v>
       </c>
       <c r="M30" t="n">
-        <v>67</v>
+        <v>31.9</v>
       </c>
       <c r="N30" t="n">
-        <v>86.90000000000001</v>
+        <v>20</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P30" t="n">
-        <v>42</v>
+        <v>53.1</v>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
@@ -3229,25 +3264,29 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U30" t="inlineStr"/>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence</t>
+        </is>
+      </c>
       <c r="V30" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>FTNT</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>352.39</v>
+        <v>481.02</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -3262,48 +3301,48 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I31" t="n">
-        <v>63.4</v>
+        <v>55.3</v>
       </c>
       <c r="J31" t="n">
-        <v>55.6</v>
+        <v>43.5</v>
       </c>
       <c r="K31" t="n">
-        <v>51.2</v>
+        <v>7</v>
       </c>
       <c r="L31" t="n">
-        <v>5.7</v>
+        <v>3.58</v>
       </c>
       <c r="M31" t="n">
-        <v>67</v>
+        <v>31.9</v>
       </c>
       <c r="N31" t="n">
-        <v>86.90000000000001</v>
+        <v>20</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P31" t="n">
-        <v>33.3</v>
+        <v>53.1</v>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R31" t="inlineStr">
@@ -3321,25 +3360,29 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U31" t="inlineStr"/>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence</t>
+        </is>
+      </c>
       <c r="V31" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>GFS</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>352.39</v>
+        <v>481.02</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -3354,48 +3397,45 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I32" t="n">
-        <v>63.4</v>
+        <v>55.3</v>
       </c>
       <c r="J32" t="n">
-        <v>55.6</v>
+        <v>43.5</v>
       </c>
       <c r="K32" t="n">
-        <v>51.2</v>
+        <v>7</v>
       </c>
       <c r="L32" t="n">
-        <v>5.7</v>
+        <v>3.58</v>
       </c>
       <c r="M32" t="n">
-        <v>67</v>
-      </c>
-      <c r="N32" t="n">
-        <v>86.90000000000001</v>
+        <v>53.2</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P32" t="n">
-        <v>42</v>
+        <v>53.1</v>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
@@ -3413,69 +3453,73 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U32" t="inlineStr"/>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence</t>
+        </is>
+      </c>
       <c r="V32" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>MMM</t>
+          <t>ILMN</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>46.38</v>
+        <v>481.02</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D33" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I33" t="n">
-        <v>56.4</v>
+        <v>55.3</v>
       </c>
       <c r="J33" t="n">
-        <v>30.5</v>
+        <v>43.5</v>
       </c>
       <c r="K33" t="n">
-        <v>90</v>
+        <v>7</v>
       </c>
       <c r="L33" t="n">
-        <v>2.75</v>
+        <v>3.58</v>
       </c>
       <c r="M33" t="n">
-        <v>27.4</v>
+        <v>31.9</v>
       </c>
       <c r="N33" t="n">
-        <v>35.8</v>
+        <v>20</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
@@ -3483,11 +3527,11 @@
         </is>
       </c>
       <c r="P33" t="n">
-        <v>55.6</v>
+        <v>53.1</v>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
@@ -3497,77 +3541,81 @@
       </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U33" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence</t>
+        </is>
+      </c>
       <c r="V33" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>MPC</t>
+          <t>DASH</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>46.38</v>
+        <v>481.02</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D34" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I34" t="n">
-        <v>56.4</v>
+        <v>55.3</v>
       </c>
       <c r="J34" t="n">
-        <v>30.5</v>
+        <v>43.5</v>
       </c>
       <c r="K34" t="n">
-        <v>90</v>
+        <v>7</v>
       </c>
       <c r="L34" t="n">
-        <v>2.75</v>
+        <v>3.58</v>
       </c>
       <c r="M34" t="n">
-        <v>27.4</v>
+        <v>31.9</v>
       </c>
       <c r="N34" t="n">
-        <v>35.8</v>
+        <v>20</v>
       </c>
       <c r="O34" t="inlineStr">
         <is>
@@ -3575,11 +3623,11 @@
         </is>
       </c>
       <c r="P34" t="n">
-        <v>55.6</v>
+        <v>53.1</v>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
@@ -3589,77 +3637,78 @@
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U34" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence</t>
+        </is>
+      </c>
       <c r="V34" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>MO</t>
+          <t>FAST</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>46.38</v>
+        <v>481.02</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D35" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I35" t="n">
-        <v>56.4</v>
+        <v>55.3</v>
       </c>
       <c r="J35" t="n">
-        <v>30.5</v>
+        <v>43.5</v>
       </c>
       <c r="K35" t="n">
-        <v>90</v>
+        <v>7</v>
       </c>
       <c r="L35" t="n">
-        <v>2.75</v>
+        <v>3.58</v>
       </c>
       <c r="M35" t="n">
-        <v>27.4</v>
-      </c>
-      <c r="N35" t="n">
-        <v>35.8</v>
+        <v>40.3</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
@@ -3667,11 +3716,11 @@
         </is>
       </c>
       <c r="P35" t="n">
-        <v>55.6</v>
+        <v>53.4</v>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
@@ -3681,108 +3730,757 @@
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U35" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence</t>
+        </is>
+      </c>
       <c r="V35" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>MMC</t>
+          <t>IDXX</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>46.38</v>
+        <v>481.02</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>55.3</v>
+      </c>
+      <c r="J36" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="K36" t="n">
+        <v>7</v>
+      </c>
+      <c r="L36" t="n">
+        <v>3.58</v>
+      </c>
+      <c r="M36" t="n">
+        <v>39.6</v>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P36" t="n">
+        <v>53.1</v>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence</t>
+        </is>
+      </c>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>ROST</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>292.95</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D36" s="3" t="inlineStr">
+      <c r="D37" s="3" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="E37" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="F37" t="inlineStr">
         <is>
           <t>Credit Put</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
+      <c r="G37" t="inlineStr">
         <is>
           <t>7-21 DTE</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr">
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>53.5</v>
+      </c>
+      <c r="J37" t="n">
+        <v>30.3</v>
+      </c>
+      <c r="K37" t="n">
+        <v>74</v>
+      </c>
+      <c r="L37" t="n">
+        <v>2.66</v>
+      </c>
+      <c r="M37" t="n">
+        <v>37.3</v>
+      </c>
+      <c r="N37" t="n">
+        <v>42.3</v>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P37" t="n">
+        <v>46.6</v>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U37" t="inlineStr"/>
+      <c r="V37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>RTX</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>292.95</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>53.5</v>
+      </c>
+      <c r="J38" t="n">
+        <v>30.3</v>
+      </c>
+      <c r="K38" t="n">
+        <v>74</v>
+      </c>
+      <c r="L38" t="n">
+        <v>2.66</v>
+      </c>
+      <c r="M38" t="n">
+        <v>37.3</v>
+      </c>
+      <c r="N38" t="n">
+        <v>42.3</v>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P38" t="n">
+        <v>32.7</v>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr"/>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>ROP</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>292.95</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>53.5</v>
+      </c>
+      <c r="J39" t="n">
+        <v>30.3</v>
+      </c>
+      <c r="K39" t="n">
+        <v>74</v>
+      </c>
+      <c r="L39" t="n">
+        <v>2.66</v>
+      </c>
+      <c r="M39" t="n">
+        <v>37.3</v>
+      </c>
+      <c r="N39" t="n">
+        <v>42.3</v>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P39" t="n">
+        <v>32.7</v>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U39" t="inlineStr"/>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>SYY</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>156.98</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
         <is>
           <t>EXPANSION</t>
         </is>
       </c>
-      <c r="I36" t="n">
-        <v>56.4</v>
-      </c>
-      <c r="J36" t="n">
-        <v>30.5</v>
-      </c>
-      <c r="K36" t="n">
-        <v>90</v>
-      </c>
-      <c r="L36" t="n">
-        <v>2.75</v>
-      </c>
-      <c r="M36" t="n">
-        <v>27.4</v>
-      </c>
-      <c r="N36" t="n">
-        <v>35.8</v>
-      </c>
-      <c r="O36" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P36" t="n">
-        <v>55.6</v>
-      </c>
-      <c r="Q36" t="inlineStr">
+      <c r="I40" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="J40" t="n">
+        <v>32.7</v>
+      </c>
+      <c r="K40" t="n">
+        <v>91</v>
+      </c>
+      <c r="L40" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="M40" t="n">
+        <v>30</v>
+      </c>
+      <c r="N40" t="n">
+        <v>29.8</v>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P40" t="n">
+        <v>38.2</v>
+      </c>
+      <c r="Q40" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>
       </c>
-      <c r="R36" t="inlineStr">
+      <c r="R40" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="S36" t="inlineStr">
+      <c r="S40" t="inlineStr">
         <is>
           <t>red</t>
         </is>
       </c>
-      <c r="T36" t="inlineStr">
+      <c r="T40" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="U36" t="inlineStr"/>
-      <c r="V36" t="inlineStr">
+      <c r="U40" t="inlineStr"/>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>156.98</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="J41" t="n">
+        <v>32.7</v>
+      </c>
+      <c r="K41" t="n">
+        <v>91</v>
+      </c>
+      <c r="L41" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="M41" t="n">
+        <v>30</v>
+      </c>
+      <c r="N41" t="n">
+        <v>29.8</v>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P41" t="n">
+        <v>38.2</v>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr"/>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>SPG</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>156.98</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="J42" t="n">
+        <v>32.7</v>
+      </c>
+      <c r="K42" t="n">
+        <v>91</v>
+      </c>
+      <c r="L42" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="M42" t="n">
+        <v>30</v>
+      </c>
+      <c r="N42" t="n">
+        <v>29.8</v>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P42" t="n">
+        <v>38.2</v>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U42" t="inlineStr"/>
+      <c r="V42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>SRE</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>156.98</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="J43" t="n">
+        <v>32.7</v>
+      </c>
+      <c r="K43" t="n">
+        <v>91</v>
+      </c>
+      <c r="L43" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="M43" t="n">
+        <v>30</v>
+      </c>
+      <c r="N43" t="n">
+        <v>29.8</v>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P43" t="n">
+        <v>38.2</v>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U43" t="inlineStr"/>
+      <c r="V43" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Scan 24.03.2026 15:08 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -31,10 +31,10 @@
       <sz val="11"/>
     </font>
     <font>
-      <color rgb="0022c55e"/>
+      <color rgb="00ef4444"/>
     </font>
     <font>
-      <color rgb="00ef4444"/>
+      <color rgb="0022c55e"/>
     </font>
   </fonts>
   <fills count="3">
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V21"/>
+  <dimension ref="A1:V19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -444,12 +444,12 @@
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="6" customWidth="1" min="10" max="10"/>
     <col width="6" customWidth="1" min="11" max="11"/>
-    <col width="6" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
     <col width="9" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
@@ -458,7 +458,7 @@
     <col width="15" customWidth="1" min="18" max="18"/>
     <col width="11" customWidth="1" min="19" max="19"/>
     <col width="11" customWidth="1" min="20" max="20"/>
-    <col width="13" customWidth="1" min="21" max="21"/>
+    <col width="10" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
@@ -577,11 +577,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ORCL</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>167.75</v>
+        <v>70.68000000000001</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -590,17 +590,17 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>BULLISH</t>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -614,30 +614,30 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>76.09999999999999</v>
+        <v>78.3</v>
       </c>
       <c r="J2" t="n">
-        <v>53.8</v>
+        <v>62</v>
       </c>
       <c r="K2" t="n">
-        <v>87</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="L2" t="n">
-        <v>3.21</v>
+        <v>6.92</v>
       </c>
       <c r="M2" t="n">
-        <v>38.7</v>
+        <v>57.9</v>
       </c>
       <c r="N2" t="n">
-        <v>55.4</v>
+        <v>46.1</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>54.4</v>
+        <v>45.3</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -651,12 +651,12 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
@@ -669,18 +669,18 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>DUK</t>
+          <t>MRK</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>137.79</v>
+        <v>70.68000000000001</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
@@ -692,48 +692,48 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>73.5</v>
+        <v>78.3</v>
       </c>
       <c r="J3" t="n">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="K3" t="n">
-        <v>9</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="L3" t="n">
-        <v>4.19</v>
+        <v>6.92</v>
       </c>
       <c r="M3" t="n">
-        <v>51.5</v>
+        <v>57.9</v>
       </c>
       <c r="N3" t="n">
-        <v>42.7</v>
+        <v>46.1</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P3" t="n">
-        <v>41.8</v>
+        <v>42.3</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -751,11 +751,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>TTM Squeeze</t>
-        </is>
-      </c>
+      <c r="U3" t="inlineStr"/>
       <c r="V3" t="inlineStr">
         <is>
           <t>No</t>
@@ -765,81 +761,81 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>DIS</t>
+          <t>PSA</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>137.79</v>
+        <v>106.38</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>BEARISH</t>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>73.5</v>
+        <v>70.5</v>
       </c>
       <c r="J4" t="n">
-        <v>53</v>
+        <v>33</v>
       </c>
       <c r="K4" t="n">
-        <v>9</v>
+        <v>96.5</v>
       </c>
       <c r="L4" t="n">
-        <v>4.19</v>
+        <v>11.93</v>
       </c>
       <c r="M4" t="n">
-        <v>51.5</v>
+        <v>95.2</v>
       </c>
       <c r="N4" t="n">
-        <v>42.7</v>
+        <v>84.09999999999999</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P4" t="n">
-        <v>41.8</v>
+        <v>44.7</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -847,11 +843,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>TTM Squeeze</t>
-        </is>
-      </c>
+      <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr">
         <is>
           <t>No</t>
@@ -861,81 +853,81 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ECL</t>
+          <t>PG</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>137.79</v>
+        <v>106.38</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>BEARISH</t>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>73.5</v>
+        <v>70.5</v>
       </c>
       <c r="J5" t="n">
-        <v>53</v>
+        <v>33</v>
       </c>
       <c r="K5" t="n">
-        <v>9</v>
+        <v>96.5</v>
       </c>
       <c r="L5" t="n">
-        <v>4.19</v>
+        <v>11.93</v>
       </c>
       <c r="M5" t="n">
-        <v>51.5</v>
+        <v>95.2</v>
       </c>
       <c r="N5" t="n">
-        <v>42.7</v>
+        <v>84.09999999999999</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>41.8</v>
+        <v>44.7</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -943,11 +935,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>TTM Squeeze</t>
-        </is>
-      </c>
+      <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr">
         <is>
           <t>No</t>
@@ -957,81 +945,81 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>EL</t>
+          <t>PNC</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>137.79</v>
+        <v>106.38</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>BEARISH</t>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>73.5</v>
+        <v>70.5</v>
       </c>
       <c r="J6" t="n">
-        <v>53</v>
+        <v>33</v>
       </c>
       <c r="K6" t="n">
-        <v>9</v>
+        <v>96.5</v>
       </c>
       <c r="L6" t="n">
-        <v>4.19</v>
+        <v>11.93</v>
       </c>
       <c r="M6" t="n">
-        <v>51.5</v>
+        <v>95.2</v>
       </c>
       <c r="N6" t="n">
-        <v>42.7</v>
+        <v>84.09999999999999</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P6" t="n">
-        <v>48.1</v>
+        <v>44.7</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
@@ -1039,11 +1027,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>TTM Squeeze</t>
-        </is>
-      </c>
+      <c r="U6" t="inlineStr"/>
       <c r="V6" t="inlineStr">
         <is>
           <t>No</t>
@@ -1053,81 +1037,81 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>DOW</t>
+          <t>PGR</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>137.79</v>
+        <v>106.38</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>BEARISH</t>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>73.5</v>
+        <v>70.5</v>
       </c>
       <c r="J7" t="n">
-        <v>53</v>
+        <v>33</v>
       </c>
       <c r="K7" t="n">
-        <v>9</v>
+        <v>96.5</v>
       </c>
       <c r="L7" t="n">
-        <v>4.19</v>
+        <v>11.93</v>
       </c>
       <c r="M7" t="n">
-        <v>51.5</v>
+        <v>95.2</v>
       </c>
       <c r="N7" t="n">
-        <v>42.7</v>
+        <v>84.09999999999999</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>48.1</v>
+        <v>38.4</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
@@ -1135,11 +1119,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>TTM Squeeze</t>
-        </is>
-      </c>
+      <c r="U7" t="inlineStr"/>
       <c r="V7" t="inlineStr">
         <is>
           <t>No</t>
@@ -1149,81 +1129,81 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>EMR</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>137.79</v>
+        <v>106.38</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>BEARISH</t>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>73.5</v>
+        <v>70.5</v>
       </c>
       <c r="J8" t="n">
-        <v>53</v>
+        <v>33</v>
       </c>
       <c r="K8" t="n">
-        <v>9</v>
+        <v>96.5</v>
       </c>
       <c r="L8" t="n">
-        <v>4.19</v>
+        <v>11.93</v>
       </c>
       <c r="M8" t="n">
-        <v>51.5</v>
+        <v>95.2</v>
       </c>
       <c r="N8" t="n">
-        <v>42.7</v>
+        <v>84.09999999999999</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>55.2</v>
+        <v>38.4</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
@@ -1231,11 +1211,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>TTM Squeeze</t>
-        </is>
-      </c>
+      <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr">
         <is>
           <t>No</t>
@@ -1245,18 +1221,18 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>986.08</v>
+        <v>106.38</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
@@ -1282,22 +1258,22 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>70.59999999999999</v>
+        <v>70.5</v>
       </c>
       <c r="J9" t="n">
-        <v>45.4</v>
+        <v>33</v>
       </c>
       <c r="K9" t="n">
-        <v>94</v>
+        <v>96.5</v>
       </c>
       <c r="L9" t="n">
-        <v>2.96</v>
+        <v>11.93</v>
       </c>
       <c r="M9" t="n">
-        <v>32.7</v>
+        <v>95.2</v>
       </c>
       <c r="N9" t="n">
-        <v>51</v>
+        <v>84.09999999999999</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1305,7 +1281,7 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>39.2</v>
+        <v>38.4</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1314,17 +1290,17 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U9" t="inlineStr"/>
@@ -1337,18 +1313,18 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>TMUS</t>
+          <t>PSX</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>986.08</v>
+        <v>106.38</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
@@ -1374,22 +1350,22 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>70.59999999999999</v>
+        <v>70.5</v>
       </c>
       <c r="J10" t="n">
-        <v>45.4</v>
+        <v>33</v>
       </c>
       <c r="K10" t="n">
-        <v>94</v>
+        <v>96.5</v>
       </c>
       <c r="L10" t="n">
-        <v>2.96</v>
+        <v>11.93</v>
       </c>
       <c r="M10" t="n">
-        <v>32.7</v>
+        <v>95.2</v>
       </c>
       <c r="N10" t="n">
-        <v>51</v>
+        <v>84.09999999999999</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1397,7 +1373,7 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>50.2</v>
+        <v>38.4</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1406,17 +1382,17 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U10" t="inlineStr"/>
@@ -1429,18 +1405,18 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>TMO</t>
+          <t>PFE</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>986.08</v>
+        <v>106.38</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
@@ -1466,19 +1442,22 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>70.59999999999999</v>
+        <v>70.5</v>
       </c>
       <c r="J11" t="n">
-        <v>45.4</v>
+        <v>33</v>
       </c>
       <c r="K11" t="n">
-        <v>94</v>
+        <v>96.5</v>
       </c>
       <c r="L11" t="n">
-        <v>2.96</v>
+        <v>11.93</v>
       </c>
       <c r="M11" t="n">
-        <v>39.9</v>
+        <v>95.2</v>
+      </c>
+      <c r="N11" t="n">
+        <v>84.09999999999999</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1486,7 +1465,7 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>50.2</v>
+        <v>44.7</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1495,17 +1474,17 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U11" t="inlineStr"/>
@@ -1518,18 +1497,18 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>PNC</t>
+          <t>PH</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>133.07</v>
+        <v>106.38</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
@@ -1551,26 +1530,26 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>62.8</v>
+        <v>70.5</v>
       </c>
       <c r="J12" t="n">
-        <v>46.1</v>
+        <v>33</v>
       </c>
       <c r="K12" t="n">
-        <v>77</v>
+        <v>96.5</v>
       </c>
       <c r="L12" t="n">
-        <v>5.18</v>
+        <v>11.93</v>
       </c>
       <c r="M12" t="n">
-        <v>47.5</v>
+        <v>95.2</v>
       </c>
       <c r="N12" t="n">
-        <v>58.1</v>
+        <v>84.09999999999999</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1578,7 +1557,7 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>48.9</v>
+        <v>44.7</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1587,17 +1566,17 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U12" t="inlineStr"/>
@@ -1610,18 +1589,18 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>PG</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>133.07</v>
+        <v>106.38</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D13" s="3" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
@@ -1643,34 +1622,34 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>62.8</v>
+        <v>70.5</v>
       </c>
       <c r="J13" t="n">
-        <v>46.1</v>
+        <v>33</v>
       </c>
       <c r="K13" t="n">
-        <v>77</v>
+        <v>96.5</v>
       </c>
       <c r="L13" t="n">
-        <v>5.18</v>
+        <v>11.93</v>
       </c>
       <c r="M13" t="n">
-        <v>47.5</v>
+        <v>95.2</v>
       </c>
       <c r="N13" t="n">
-        <v>58.1</v>
+        <v>84.09999999999999</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>43.4</v>
+        <v>38.4</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1679,17 +1658,17 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U13" t="inlineStr"/>
@@ -1702,18 +1681,18 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>PEP</t>
+          <t>SCHW</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>133.07</v>
+        <v>971.1</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
@@ -1735,26 +1714,23 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>62.8</v>
+        <v>69.8</v>
       </c>
       <c r="J14" t="n">
-        <v>46.1</v>
+        <v>41.6</v>
       </c>
       <c r="K14" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="L14" t="n">
-        <v>5.18</v>
+        <v>2.85</v>
       </c>
       <c r="M14" t="n">
-        <v>47.5</v>
-      </c>
-      <c r="N14" t="n">
-        <v>58.1</v>
+        <v>37.1</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1762,7 +1738,7 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>48.9</v>
+        <v>44.7</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1794,11 +1770,11 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>PYPL</t>
+          <t>DDOG</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>133.07</v>
+        <v>328.18</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1807,17 +1783,17 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>BULLISH</t>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1831,30 +1807,30 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>62.8</v>
+        <v>63.5</v>
       </c>
       <c r="J15" t="n">
-        <v>46.1</v>
+        <v>61.7</v>
       </c>
       <c r="K15" t="n">
-        <v>77</v>
+        <v>76.7</v>
       </c>
       <c r="L15" t="n">
-        <v>5.18</v>
+        <v>3.78</v>
       </c>
       <c r="M15" t="n">
-        <v>47.5</v>
+        <v>41.6</v>
       </c>
       <c r="N15" t="n">
-        <v>58.1</v>
+        <v>69.5</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P15" t="n">
-        <v>41.6</v>
+        <v>65</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1863,12 +1839,12 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
@@ -1886,18 +1862,18 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>QCOM</t>
+          <t>ALL</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>133.07</v>
+        <v>321.1</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D16" s="3" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
@@ -1919,26 +1895,26 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>62.8</v>
+        <v>57.6</v>
       </c>
       <c r="J16" t="n">
-        <v>46.1</v>
+        <v>50.3</v>
       </c>
       <c r="K16" t="n">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="L16" t="n">
-        <v>5.18</v>
+        <v>2.89</v>
       </c>
       <c r="M16" t="n">
-        <v>47.5</v>
+        <v>31.5</v>
       </c>
       <c r="N16" t="n">
-        <v>58.1</v>
+        <v>25.9</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -1946,7 +1922,7 @@
         </is>
       </c>
       <c r="P16" t="n">
-        <v>41.6</v>
+        <v>30.9</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1978,18 +1954,18 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>PFE</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>133.07</v>
+        <v>321.1</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D17" s="3" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
@@ -2011,26 +1987,26 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>62.8</v>
+        <v>57.6</v>
       </c>
       <c r="J17" t="n">
-        <v>46.1</v>
+        <v>50.3</v>
       </c>
       <c r="K17" t="n">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="L17" t="n">
-        <v>5.18</v>
+        <v>2.89</v>
       </c>
       <c r="M17" t="n">
-        <v>47.5</v>
+        <v>31.5</v>
       </c>
       <c r="N17" t="n">
-        <v>58.1</v>
+        <v>25.9</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -2038,7 +2014,7 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>41.6</v>
+        <v>37.7</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -2070,11 +2046,11 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>BLK</t>
+          <t>MAR</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>317.45</v>
+        <v>57.32</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -2083,17 +2059,17 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>BULLISH</t>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -2103,26 +2079,26 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>55.3</v>
+        <v>48.8</v>
       </c>
       <c r="J18" t="n">
-        <v>47.1</v>
+        <v>58.2</v>
       </c>
       <c r="K18" t="n">
-        <v>84</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="L18" t="n">
-        <v>2.89</v>
+        <v>4.94</v>
       </c>
       <c r="M18" t="n">
-        <v>31.3</v>
+        <v>56</v>
       </c>
       <c r="N18" t="n">
-        <v>25.5</v>
+        <v>16.9</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -2130,7 +2106,7 @@
         </is>
       </c>
       <c r="P18" t="n">
-        <v>48.4</v>
+        <v>64.7</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -2144,12 +2120,12 @@
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U18" t="inlineStr"/>
@@ -2162,11 +2138,11 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>BDX</t>
+          <t>ILMN</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>317.45</v>
+        <v>57.32</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -2175,17 +2151,17 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>BULLISH</t>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2195,34 +2171,34 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>55.3</v>
+        <v>48.8</v>
       </c>
       <c r="J19" t="n">
-        <v>47.1</v>
+        <v>58.2</v>
       </c>
       <c r="K19" t="n">
-        <v>84</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="L19" t="n">
-        <v>2.89</v>
+        <v>4.94</v>
       </c>
       <c r="M19" t="n">
-        <v>31.3</v>
+        <v>56</v>
       </c>
       <c r="N19" t="n">
-        <v>25.5</v>
+        <v>16.9</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P19" t="n">
-        <v>42.4</v>
+        <v>46.1</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -2236,188 +2212,16 @@
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U19" t="inlineStr"/>
       <c r="V19" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>ITW</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v/>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Credit Call</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I20" t="n">
-        <v>50</v>
-      </c>
-      <c r="J20" t="n">
-        <v>56.8</v>
-      </c>
-      <c r="M20" t="n">
-        <v>51.4</v>
-      </c>
-      <c r="N20" t="n">
-        <v>37</v>
-      </c>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t>Neutral</t>
-        </is>
-      </c>
-      <c r="P20" t="n">
-        <v>38.1</v>
-      </c>
-      <c r="Q20" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R20" t="inlineStr">
-        <is>
-          <t>FLAT</t>
-        </is>
-      </c>
-      <c r="S20" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="T20" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U20" t="inlineStr"/>
-      <c r="V20" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>JNJ</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v/>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Credit Call</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I21" t="n">
-        <v>50</v>
-      </c>
-      <c r="J21" t="n">
-        <v>56.8</v>
-      </c>
-      <c r="M21" t="n">
-        <v>51.4</v>
-      </c>
-      <c r="N21" t="n">
-        <v>37</v>
-      </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P21" t="n">
-        <v>46.2</v>
-      </c>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t>FLAT</t>
-        </is>
-      </c>
-      <c r="S21" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="T21" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U21" t="inlineStr"/>
-      <c r="V21" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Scan 25.03.2026 15:10 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V19"/>
+  <dimension ref="A1:V25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -449,7 +449,7 @@
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="6" customWidth="1" min="10" max="10"/>
     <col width="6" customWidth="1" min="11" max="11"/>
-    <col width="7" customWidth="1" min="12" max="12"/>
+    <col width="6" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
     <col width="9" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
@@ -577,11 +577,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>MO</t>
+          <t>VLO</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>70.68000000000001</v>
+        <v>371.69</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,30 +614,30 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>78.3</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="J2" t="n">
-        <v>62</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="K2" t="n">
         <v>84.90000000000001</v>
       </c>
       <c r="L2" t="n">
-        <v>6.92</v>
+        <v>8.5</v>
       </c>
       <c r="M2" t="n">
-        <v>57.9</v>
+        <v>88.5</v>
       </c>
       <c r="N2" t="n">
-        <v>46.1</v>
+        <v>43</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>45.3</v>
+        <v>51.5</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -669,30 +669,30 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MRK</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>70.68000000000001</v>
+        <v>235.85</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -702,26 +702,26 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>78.3</v>
+        <v>63.6</v>
       </c>
       <c r="J3" t="n">
-        <v>62</v>
+        <v>37</v>
       </c>
       <c r="K3" t="n">
-        <v>84.90000000000001</v>
+        <v>79</v>
       </c>
       <c r="L3" t="n">
-        <v>6.92</v>
+        <v>2.92</v>
       </c>
       <c r="M3" t="n">
-        <v>57.9</v>
+        <v>29.8</v>
       </c>
       <c r="N3" t="n">
-        <v>46.1</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -729,7 +729,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>42.3</v>
+        <v>27.3</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -743,12 +743,12 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U3" t="inlineStr"/>
@@ -761,11 +761,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PSA</t>
+          <t>NFLX</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>106.38</v>
+        <v>235.85</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -794,34 +794,34 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>70.5</v>
+        <v>63.6</v>
       </c>
       <c r="J4" t="n">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="K4" t="n">
-        <v>96.5</v>
+        <v>79</v>
       </c>
       <c r="L4" t="n">
-        <v>11.93</v>
+        <v>2.92</v>
       </c>
       <c r="M4" t="n">
-        <v>95.2</v>
+        <v>29.8</v>
       </c>
       <c r="N4" t="n">
-        <v>84.09999999999999</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P4" t="n">
-        <v>44.7</v>
+        <v>45.1</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -830,17 +830,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U4" t="inlineStr"/>
@@ -853,11 +853,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>PG</t>
+          <t>MU</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>106.38</v>
+        <v>235.85</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -886,34 +886,31 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>70.5</v>
+        <v>63.6</v>
       </c>
       <c r="J5" t="n">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="K5" t="n">
-        <v>96.5</v>
+        <v>79</v>
       </c>
       <c r="L5" t="n">
-        <v>11.93</v>
+        <v>2.92</v>
       </c>
       <c r="M5" t="n">
-        <v>95.2</v>
-      </c>
-      <c r="N5" t="n">
-        <v>84.09999999999999</v>
+        <v>62.3</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>44.7</v>
+        <v>29.1</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -922,17 +919,17 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U5" t="inlineStr"/>
@@ -945,11 +942,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>PNC</t>
+          <t>MSI</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>106.38</v>
+        <v>235.85</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -978,34 +975,34 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>70.5</v>
+        <v>63.6</v>
       </c>
       <c r="J6" t="n">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="K6" t="n">
-        <v>96.5</v>
+        <v>79</v>
       </c>
       <c r="L6" t="n">
-        <v>11.93</v>
+        <v>2.92</v>
       </c>
       <c r="M6" t="n">
-        <v>95.2</v>
+        <v>29.8</v>
       </c>
       <c r="N6" t="n">
-        <v>84.09999999999999</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P6" t="n">
-        <v>44.7</v>
+        <v>45.1</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1014,17 +1011,17 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
@@ -1037,11 +1034,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>PGR</t>
+          <t>NOC</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>106.38</v>
+        <v>235.85</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1070,34 +1067,34 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>70.5</v>
+        <v>63.6</v>
       </c>
       <c r="J7" t="n">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="K7" t="n">
-        <v>96.5</v>
+        <v>79</v>
       </c>
       <c r="L7" t="n">
-        <v>11.93</v>
+        <v>2.92</v>
       </c>
       <c r="M7" t="n">
-        <v>95.2</v>
+        <v>29.8</v>
       </c>
       <c r="N7" t="n">
-        <v>84.09999999999999</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>38.4</v>
+        <v>36.3</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1106,17 +1103,17 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U7" t="inlineStr"/>
@@ -1129,11 +1126,11 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>ORLY</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>106.38</v>
+        <v>235.85</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1162,34 +1159,34 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>70.5</v>
+        <v>63.6</v>
       </c>
       <c r="J8" t="n">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="K8" t="n">
-        <v>96.5</v>
+        <v>79</v>
       </c>
       <c r="L8" t="n">
-        <v>11.93</v>
+        <v>2.92</v>
       </c>
       <c r="M8" t="n">
-        <v>95.2</v>
+        <v>29.8</v>
       </c>
       <c r="N8" t="n">
-        <v>84.09999999999999</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>38.4</v>
+        <v>45.1</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1198,17 +1195,17 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U8" t="inlineStr"/>
@@ -1221,30 +1218,30 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>COST</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>106.38</v>
+        <v>58.76</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1254,34 +1251,34 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>70.5</v>
+        <v>51.1</v>
       </c>
       <c r="J9" t="n">
-        <v>33</v>
+        <v>61.2</v>
       </c>
       <c r="K9" t="n">
-        <v>96.5</v>
+        <v>66.3</v>
       </c>
       <c r="L9" t="n">
-        <v>11.93</v>
+        <v>4.95</v>
       </c>
       <c r="M9" t="n">
-        <v>95.2</v>
+        <v>56.1</v>
       </c>
       <c r="N9" t="n">
-        <v>84.09999999999999</v>
+        <v>17.1</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>38.4</v>
+        <v>43.5</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1295,12 +1292,12 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U9" t="inlineStr"/>
@@ -1313,30 +1310,30 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>PSX</t>
+          <t>CMG</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>106.38</v>
+        <v>58.76</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1346,34 +1343,31 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>70.5</v>
+        <v>51.1</v>
       </c>
       <c r="J10" t="n">
-        <v>33</v>
+        <v>61.2</v>
       </c>
       <c r="K10" t="n">
-        <v>96.5</v>
+        <v>66.3</v>
       </c>
       <c r="L10" t="n">
-        <v>11.93</v>
+        <v>4.95</v>
       </c>
       <c r="M10" t="n">
-        <v>95.2</v>
+        <v>56.1</v>
       </c>
       <c r="N10" t="n">
-        <v>84.09999999999999</v>
+        <v>17.1</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P10" t="n">
-        <v>38.4</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1387,12 +1381,12 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U10" t="inlineStr"/>
@@ -1405,30 +1399,30 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>PFE</t>
+          <t>CMCSA</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>106.38</v>
+        <v>58.76</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1438,34 +1432,31 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>70.5</v>
+        <v>51.1</v>
       </c>
       <c r="J11" t="n">
-        <v>33</v>
+        <v>61.2</v>
       </c>
       <c r="K11" t="n">
-        <v>96.5</v>
+        <v>66.3</v>
       </c>
       <c r="L11" t="n">
-        <v>11.93</v>
+        <v>4.95</v>
       </c>
       <c r="M11" t="n">
-        <v>95.2</v>
+        <v>56.1</v>
       </c>
       <c r="N11" t="n">
-        <v>84.09999999999999</v>
+        <v>17.1</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P11" t="n">
-        <v>44.7</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1479,12 +1470,12 @@
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U11" t="inlineStr"/>
@@ -1497,30 +1488,30 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>PH</t>
+          <t>CTAS</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>106.38</v>
+        <v>58.76</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1530,34 +1521,31 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>70.5</v>
+        <v>51.1</v>
       </c>
       <c r="J12" t="n">
-        <v>33</v>
+        <v>61.2</v>
       </c>
       <c r="K12" t="n">
-        <v>96.5</v>
+        <v>66.3</v>
       </c>
       <c r="L12" t="n">
-        <v>11.93</v>
+        <v>4.95</v>
       </c>
       <c r="M12" t="n">
-        <v>95.2</v>
+        <v>56.1</v>
       </c>
       <c r="N12" t="n">
-        <v>84.09999999999999</v>
+        <v>17.1</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P12" t="n">
-        <v>44.7</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1571,12 +1559,12 @@
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U12" t="inlineStr"/>
@@ -1589,30 +1577,30 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>CVX</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>106.38</v>
+        <v>58.76</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1622,34 +1610,31 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>70.5</v>
+        <v>51.1</v>
       </c>
       <c r="J13" t="n">
-        <v>33</v>
+        <v>61.2</v>
       </c>
       <c r="K13" t="n">
-        <v>96.5</v>
+        <v>66.3</v>
       </c>
       <c r="L13" t="n">
-        <v>11.93</v>
+        <v>4.95</v>
       </c>
       <c r="M13" t="n">
-        <v>95.2</v>
+        <v>56.1</v>
       </c>
       <c r="N13" t="n">
-        <v>84.09999999999999</v>
+        <v>17.1</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P13" t="n">
-        <v>38.4</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1663,12 +1648,12 @@
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U13" t="inlineStr"/>
@@ -1681,30 +1666,30 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SCHW</t>
+          <t>CL</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>971.1</v>
+        <v>58.76</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1714,23 +1699,26 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>69.8</v>
+        <v>51.1</v>
       </c>
       <c r="J14" t="n">
-        <v>41.6</v>
+        <v>61.2</v>
       </c>
       <c r="K14" t="n">
-        <v>93</v>
+        <v>66.3</v>
       </c>
       <c r="L14" t="n">
-        <v>2.85</v>
+        <v>4.95</v>
       </c>
       <c r="M14" t="n">
-        <v>37.1</v>
+        <v>56.1</v>
+      </c>
+      <c r="N14" t="n">
+        <v>17.1</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1738,7 +1726,7 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>44.7</v>
+        <v>49.5</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1747,12 +1735,12 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
@@ -1770,11 +1758,11 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>DDOG</t>
+          <t>CVS</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>328.18</v>
+        <v>58.76</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1807,30 +1795,27 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>63.5</v>
+        <v>51.1</v>
       </c>
       <c r="J15" t="n">
-        <v>61.7</v>
+        <v>61.2</v>
       </c>
       <c r="K15" t="n">
-        <v>76.7</v>
+        <v>66.3</v>
       </c>
       <c r="L15" t="n">
-        <v>3.78</v>
+        <v>4.95</v>
       </c>
       <c r="M15" t="n">
-        <v>41.6</v>
+        <v>56.1</v>
       </c>
       <c r="N15" t="n">
-        <v>69.5</v>
+        <v>17.1</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P15" t="n">
-        <v>65</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1862,30 +1847,30 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ALL</t>
+          <t>CME</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>321.1</v>
+        <v>58.76</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1895,34 +1880,34 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>57.6</v>
+        <v>51.1</v>
       </c>
       <c r="J16" t="n">
-        <v>50.3</v>
+        <v>61.2</v>
       </c>
       <c r="K16" t="n">
-        <v>82</v>
+        <v>66.3</v>
       </c>
       <c r="L16" t="n">
-        <v>2.89</v>
+        <v>4.95</v>
       </c>
       <c r="M16" t="n">
-        <v>31.5</v>
+        <v>56.1</v>
       </c>
       <c r="N16" t="n">
-        <v>25.9</v>
+        <v>17.1</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>30.9</v>
+        <v>77.5</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1931,12 +1916,12 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
@@ -1954,11 +1939,11 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>TGT</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>321.1</v>
+        <v>156.49</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -1991,22 +1976,22 @@
         </is>
       </c>
       <c r="I17" t="n">
-        <v>57.6</v>
+        <v>48.1</v>
       </c>
       <c r="J17" t="n">
-        <v>50.3</v>
+        <v>35.3</v>
       </c>
       <c r="K17" t="n">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="L17" t="n">
-        <v>2.89</v>
+        <v>2.35</v>
       </c>
       <c r="M17" t="n">
-        <v>31.5</v>
+        <v>25.2</v>
       </c>
       <c r="N17" t="n">
-        <v>25.9</v>
+        <v>19.6</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -2014,7 +1999,7 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>37.7</v>
+        <v>44</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -2023,17 +2008,17 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U17" t="inlineStr"/>
@@ -2046,30 +2031,30 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>TSLA</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>57.32</v>
+        <v>156.49</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -2079,34 +2064,34 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>48.8</v>
+        <v>48.1</v>
       </c>
       <c r="J18" t="n">
-        <v>58.2</v>
+        <v>35.3</v>
       </c>
       <c r="K18" t="n">
-        <v>65.09999999999999</v>
+        <v>81</v>
       </c>
       <c r="L18" t="n">
-        <v>4.94</v>
+        <v>2.35</v>
       </c>
       <c r="M18" t="n">
-        <v>56</v>
+        <v>25.2</v>
       </c>
       <c r="N18" t="n">
-        <v>16.9</v>
+        <v>19.6</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P18" t="n">
-        <v>64.7</v>
+        <v>44</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -2120,12 +2105,12 @@
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U18" t="inlineStr"/>
@@ -2138,30 +2123,30 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ILMN</t>
+          <t>TMO</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>57.32</v>
+        <v>156.49</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2171,26 +2156,26 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>48.8</v>
+        <v>48.1</v>
       </c>
       <c r="J19" t="n">
-        <v>58.2</v>
+        <v>35.3</v>
       </c>
       <c r="K19" t="n">
-        <v>65.09999999999999</v>
+        <v>81</v>
       </c>
       <c r="L19" t="n">
-        <v>4.94</v>
+        <v>2.35</v>
       </c>
       <c r="M19" t="n">
-        <v>56</v>
+        <v>25.2</v>
       </c>
       <c r="N19" t="n">
-        <v>16.9</v>
+        <v>19.6</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -2198,7 +2183,7 @@
         </is>
       </c>
       <c r="P19" t="n">
-        <v>46.1</v>
+        <v>44</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -2212,16 +2197,562 @@
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U19" t="inlineStr"/>
       <c r="V19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>TDG</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>156.49</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="J20" t="n">
+        <v>35.3</v>
+      </c>
+      <c r="K20" t="n">
+        <v>81</v>
+      </c>
+      <c r="L20" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="M20" t="n">
+        <v>25.2</v>
+      </c>
+      <c r="N20" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P20" t="n">
+        <v>44</v>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr"/>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>TMUS</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>156.49</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="J21" t="n">
+        <v>35.3</v>
+      </c>
+      <c r="K21" t="n">
+        <v>81</v>
+      </c>
+      <c r="L21" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="M21" t="n">
+        <v>25.2</v>
+      </c>
+      <c r="N21" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P21" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr"/>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>TSN</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>156.49</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="J22" t="n">
+        <v>35.3</v>
+      </c>
+      <c r="K22" t="n">
+        <v>81</v>
+      </c>
+      <c r="L22" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="M22" t="n">
+        <v>25.2</v>
+      </c>
+      <c r="N22" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P22" t="n">
+        <v>44</v>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr"/>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>156.49</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="J23" t="n">
+        <v>35.3</v>
+      </c>
+      <c r="K23" t="n">
+        <v>81</v>
+      </c>
+      <c r="L23" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="M23" t="n">
+        <v>25.2</v>
+      </c>
+      <c r="N23" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P23" t="n">
+        <v>44</v>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr"/>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>TJX</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>156.49</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="J24" t="n">
+        <v>35.3</v>
+      </c>
+      <c r="K24" t="n">
+        <v>81</v>
+      </c>
+      <c r="L24" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="M24" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P24" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr"/>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>TRV</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>156.49</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="J25" t="n">
+        <v>35.3</v>
+      </c>
+      <c r="K25" t="n">
+        <v>81</v>
+      </c>
+      <c r="L25" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="M25" t="n">
+        <v>30</v>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P25" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr"/>
+      <c r="V25" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Scan 26.03.2026 15:15 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V25"/>
+  <dimension ref="A1:V26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -444,7 +444,7 @@
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="6" customWidth="1" min="10" max="10"/>
@@ -458,7 +458,7 @@
     <col width="15" customWidth="1" min="18" max="18"/>
     <col width="11" customWidth="1" min="19" max="19"/>
     <col width="11" customWidth="1" min="20" max="20"/>
-    <col width="10" customWidth="1" min="21" max="21"/>
+    <col width="25" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
@@ -577,11 +577,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>VLO</t>
+          <t>ORCL</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>371.69</v>
+        <v>318.25</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,22 +614,22 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>69.90000000000001</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="J2" t="n">
-        <v>71.59999999999999</v>
+        <v>60.9</v>
       </c>
       <c r="K2" t="n">
-        <v>84.90000000000001</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="L2" t="n">
-        <v>8.5</v>
+        <v>6.47</v>
       </c>
       <c r="M2" t="n">
-        <v>88.5</v>
+        <v>76.2</v>
       </c>
       <c r="N2" t="n">
-        <v>43</v>
+        <v>46.7</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>51.5</v>
+        <v>67</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -646,17 +646,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
@@ -669,30 +669,30 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>PFE</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>235.85</v>
+        <v>318.25</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -702,34 +702,34 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>63.6</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="J3" t="n">
-        <v>37</v>
+        <v>60.9</v>
       </c>
       <c r="K3" t="n">
-        <v>79</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="L3" t="n">
-        <v>2.92</v>
+        <v>6.47</v>
       </c>
       <c r="M3" t="n">
-        <v>29.8</v>
+        <v>76.2</v>
       </c>
       <c r="N3" t="n">
-        <v>69.90000000000001</v>
+        <v>46.7</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P3" t="n">
-        <v>27.3</v>
+        <v>67</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -738,12 +738,12 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -761,30 +761,30 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>NFLX</t>
+          <t>NOC</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>235.85</v>
+        <v>318.25</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -794,34 +794,34 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>63.6</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="J4" t="n">
-        <v>37</v>
+        <v>60.9</v>
       </c>
       <c r="K4" t="n">
-        <v>79</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="L4" t="n">
-        <v>2.92</v>
+        <v>6.47</v>
       </c>
       <c r="M4" t="n">
-        <v>29.8</v>
+        <v>76.2</v>
       </c>
       <c r="N4" t="n">
-        <v>69.90000000000001</v>
+        <v>46.7</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P4" t="n">
-        <v>45.1</v>
+        <v>67</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -830,12 +830,12 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -853,30 +853,30 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>PCAR</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>235.85</v>
+        <v>119.86</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -890,27 +890,30 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>63.6</v>
+        <v>60.5</v>
       </c>
       <c r="J5" t="n">
-        <v>37</v>
+        <v>67</v>
       </c>
       <c r="K5" t="n">
-        <v>79</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="L5" t="n">
-        <v>2.92</v>
+        <v>5.07</v>
       </c>
       <c r="M5" t="n">
-        <v>62.3</v>
+        <v>71.5</v>
+      </c>
+      <c r="N5" t="n">
+        <v>89.7</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>29.1</v>
+        <v>63.7</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -924,12 +927,12 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U5" t="inlineStr"/>
@@ -942,30 +945,30 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>MSI</t>
+          <t>NSC</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>235.85</v>
+        <v>119.86</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -979,30 +982,30 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>63.6</v>
+        <v>60.5</v>
       </c>
       <c r="J6" t="n">
-        <v>37</v>
+        <v>67</v>
       </c>
       <c r="K6" t="n">
-        <v>79</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="L6" t="n">
-        <v>2.92</v>
+        <v>5.07</v>
       </c>
       <c r="M6" t="n">
-        <v>29.8</v>
+        <v>71.5</v>
       </c>
       <c r="N6" t="n">
-        <v>69.90000000000001</v>
+        <v>89.7</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P6" t="n">
-        <v>45.1</v>
+        <v>63.7</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1016,12 +1019,12 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
@@ -1034,30 +1037,30 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>NOC</t>
+          <t>MU</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>235.85</v>
+        <v>119.86</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1071,30 +1074,30 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>63.6</v>
+        <v>60.5</v>
       </c>
       <c r="J7" t="n">
-        <v>37</v>
+        <v>67</v>
       </c>
       <c r="K7" t="n">
-        <v>79</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="L7" t="n">
-        <v>2.92</v>
+        <v>5.07</v>
       </c>
       <c r="M7" t="n">
-        <v>29.8</v>
+        <v>71.5</v>
       </c>
       <c r="N7" t="n">
-        <v>69.90000000000001</v>
+        <v>89.7</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>36.3</v>
+        <v>63.7</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1108,12 +1111,12 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U7" t="inlineStr"/>
@@ -1126,30 +1129,30 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ORLY</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>235.85</v>
+        <v>119.86</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1163,30 +1166,30 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>63.6</v>
+        <v>60.5</v>
       </c>
       <c r="J8" t="n">
-        <v>37</v>
+        <v>67</v>
       </c>
       <c r="K8" t="n">
-        <v>79</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="L8" t="n">
-        <v>2.92</v>
+        <v>5.07</v>
       </c>
       <c r="M8" t="n">
-        <v>29.8</v>
+        <v>71.5</v>
       </c>
       <c r="N8" t="n">
-        <v>69.90000000000001</v>
+        <v>89.7</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>45.1</v>
+        <v>63.7</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1200,12 +1203,12 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U8" t="inlineStr"/>
@@ -1218,11 +1221,11 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>COST</t>
+          <t>NKE</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>58.76</v>
+        <v>119.86</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1255,30 +1258,30 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>51.1</v>
+        <v>60.5</v>
       </c>
       <c r="J9" t="n">
-        <v>61.2</v>
+        <v>67</v>
       </c>
       <c r="K9" t="n">
-        <v>66.3</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="L9" t="n">
-        <v>4.95</v>
+        <v>5.07</v>
       </c>
       <c r="M9" t="n">
-        <v>56.1</v>
+        <v>71.5</v>
       </c>
       <c r="N9" t="n">
-        <v>17.1</v>
+        <v>89.7</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>43.5</v>
+        <v>62.7</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1287,17 +1290,17 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U9" t="inlineStr"/>
@@ -1310,11 +1313,11 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CMG</t>
+          <t>PEP</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>58.76</v>
+        <v>119.86</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1347,27 +1350,27 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>51.1</v>
+        <v>60.5</v>
       </c>
       <c r="J10" t="n">
-        <v>61.2</v>
+        <v>67</v>
       </c>
       <c r="K10" t="n">
-        <v>66.3</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="L10" t="n">
-        <v>4.95</v>
+        <v>5.07</v>
       </c>
       <c r="M10" t="n">
-        <v>56.1</v>
-      </c>
-      <c r="N10" t="n">
-        <v>17.1</v>
+        <v>29.4</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P10" t="n">
+        <v>63.7</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1376,17 +1379,17 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U10" t="inlineStr"/>
@@ -1399,11 +1402,11 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CMCSA</t>
+          <t>MSI</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>58.76</v>
+        <v>119.86</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1436,27 +1439,30 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>51.1</v>
+        <v>60.5</v>
       </c>
       <c r="J11" t="n">
-        <v>61.2</v>
+        <v>67</v>
       </c>
       <c r="K11" t="n">
-        <v>66.3</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="L11" t="n">
-        <v>4.95</v>
+        <v>5.07</v>
       </c>
       <c r="M11" t="n">
-        <v>56.1</v>
+        <v>71.5</v>
       </c>
       <c r="N11" t="n">
-        <v>17.1</v>
+        <v>89.7</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P11" t="n">
+        <v>63.7</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1465,17 +1471,17 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U11" t="inlineStr"/>
@@ -1488,35 +1494,35 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CTAS</t>
+          <t>QCOM</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>58.76</v>
+        <v>294.34</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1525,27 +1531,27 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>51.1</v>
+        <v>58.2</v>
       </c>
       <c r="J12" t="n">
-        <v>61.2</v>
+        <v>63.7</v>
       </c>
       <c r="K12" t="n">
-        <v>66.3</v>
+        <v>28</v>
       </c>
       <c r="L12" t="n">
-        <v>4.95</v>
+        <v>2.55</v>
       </c>
       <c r="M12" t="n">
-        <v>56.1</v>
-      </c>
-      <c r="N12" t="n">
-        <v>17.1</v>
+        <v>38.4</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P12" t="n">
+        <v>35.8</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1554,17 +1560,17 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U12" t="inlineStr"/>
@@ -1577,35 +1583,35 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CVX</t>
+          <t>PYPL</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>58.76</v>
+        <v>294.34</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1614,27 +1620,27 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>51.1</v>
+        <v>58.2</v>
       </c>
       <c r="J13" t="n">
-        <v>61.2</v>
+        <v>63.7</v>
       </c>
       <c r="K13" t="n">
-        <v>66.3</v>
+        <v>28</v>
       </c>
       <c r="L13" t="n">
-        <v>4.95</v>
+        <v>2.55</v>
       </c>
       <c r="M13" t="n">
-        <v>56.1</v>
-      </c>
-      <c r="N13" t="n">
-        <v>17.1</v>
+        <v>43.6</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P13" t="n">
+        <v>35.8</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1643,17 +1649,17 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U13" t="inlineStr"/>
@@ -1666,35 +1672,35 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>PNC</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>58.76</v>
+        <v>294.34</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1703,30 +1709,27 @@
         </is>
       </c>
       <c r="I14" t="n">
-        <v>51.1</v>
+        <v>58.2</v>
       </c>
       <c r="J14" t="n">
-        <v>61.2</v>
+        <v>63.7</v>
       </c>
       <c r="K14" t="n">
-        <v>66.3</v>
+        <v>28</v>
       </c>
       <c r="L14" t="n">
-        <v>4.95</v>
+        <v>2.55</v>
       </c>
       <c r="M14" t="n">
-        <v>56.1</v>
-      </c>
-      <c r="N14" t="n">
-        <v>17.1</v>
+        <v>36.6</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P14" t="n">
-        <v>49.5</v>
+        <v>35.8</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1735,17 +1738,17 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U14" t="inlineStr"/>
@@ -1758,15 +1761,15 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CVS</t>
+          <t>GM</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>58.76</v>
+        <v>126.96</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -1781,45 +1784,48 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>51.1</v>
+        <v>54.9</v>
       </c>
       <c r="J15" t="n">
-        <v>61.2</v>
+        <v>43.2</v>
       </c>
       <c r="K15" t="n">
-        <v>66.3</v>
+        <v>13</v>
       </c>
       <c r="L15" t="n">
-        <v>4.95</v>
+        <v>4.82</v>
       </c>
       <c r="M15" t="n">
-        <v>56.1</v>
+        <v>54</v>
       </c>
       <c r="N15" t="n">
-        <v>17.1</v>
+        <v>49.3</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P15" t="n">
+        <v>51.8</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
@@ -1829,7 +1835,7 @@
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
@@ -1837,25 +1843,29 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U15" t="inlineStr"/>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CME</t>
+          <t>HD</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>58.76</v>
+        <v>126.96</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -1870,48 +1880,48 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>51.1</v>
+        <v>54.9</v>
       </c>
       <c r="J16" t="n">
-        <v>61.2</v>
+        <v>43.2</v>
       </c>
       <c r="K16" t="n">
-        <v>66.3</v>
+        <v>13</v>
       </c>
       <c r="L16" t="n">
-        <v>4.95</v>
+        <v>4.82</v>
       </c>
       <c r="M16" t="n">
-        <v>56.1</v>
+        <v>54</v>
       </c>
       <c r="N16" t="n">
-        <v>17.1</v>
+        <v>49.3</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>77.5</v>
+        <v>29.1</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
@@ -1921,7 +1931,7 @@
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
@@ -1929,69 +1939,73 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U16" t="inlineStr"/>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>TGT</t>
+          <t>GPN</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>156.49</v>
+        <v>126.96</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>48.1</v>
+        <v>54.9</v>
       </c>
       <c r="J17" t="n">
-        <v>35.3</v>
+        <v>43.2</v>
       </c>
       <c r="K17" t="n">
-        <v>81</v>
+        <v>13</v>
       </c>
       <c r="L17" t="n">
-        <v>2.35</v>
+        <v>4.82</v>
       </c>
       <c r="M17" t="n">
-        <v>25.2</v>
+        <v>54</v>
       </c>
       <c r="N17" t="n">
-        <v>19.6</v>
+        <v>49.3</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -1999,11 +2013,11 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>44</v>
+        <v>29.1</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
@@ -2018,72 +2032,76 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U17" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>TSLA</t>
+          <t>GOOG</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>156.49</v>
+        <v>126.96</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>48.1</v>
+        <v>54.9</v>
       </c>
       <c r="J18" t="n">
-        <v>35.3</v>
+        <v>43.2</v>
       </c>
       <c r="K18" t="n">
-        <v>81</v>
+        <v>13</v>
       </c>
       <c r="L18" t="n">
-        <v>2.35</v>
+        <v>4.82</v>
       </c>
       <c r="M18" t="n">
-        <v>25.2</v>
+        <v>54</v>
       </c>
       <c r="N18" t="n">
-        <v>19.6</v>
+        <v>49.3</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -2091,11 +2109,11 @@
         </is>
       </c>
       <c r="P18" t="n">
-        <v>44</v>
+        <v>29.7</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
@@ -2110,72 +2128,76 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U18" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>TMO</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>156.49</v>
+        <v>126.96</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>48.1</v>
+        <v>54.9</v>
       </c>
       <c r="J19" t="n">
-        <v>35.3</v>
+        <v>43.2</v>
       </c>
       <c r="K19" t="n">
-        <v>81</v>
+        <v>13</v>
       </c>
       <c r="L19" t="n">
-        <v>2.35</v>
+        <v>4.82</v>
       </c>
       <c r="M19" t="n">
-        <v>25.2</v>
+        <v>54</v>
       </c>
       <c r="N19" t="n">
-        <v>19.6</v>
+        <v>49.3</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -2183,11 +2205,11 @@
         </is>
       </c>
       <c r="P19" t="n">
-        <v>44</v>
+        <v>29.1</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
@@ -2202,84 +2224,88 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U19" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>TDG</t>
+          <t>HON</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>156.49</v>
+        <v>126.96</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I20" t="n">
-        <v>48.1</v>
+        <v>54.9</v>
       </c>
       <c r="J20" t="n">
-        <v>35.3</v>
+        <v>43.2</v>
       </c>
       <c r="K20" t="n">
-        <v>81</v>
+        <v>13</v>
       </c>
       <c r="L20" t="n">
-        <v>2.35</v>
+        <v>4.82</v>
       </c>
       <c r="M20" t="n">
-        <v>25.2</v>
+        <v>54</v>
       </c>
       <c r="N20" t="n">
-        <v>19.6</v>
+        <v>49.3</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P20" t="n">
-        <v>44</v>
+        <v>51.8</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
@@ -2294,84 +2320,88 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U20" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>TMUS</t>
+          <t>GS</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>156.49</v>
+        <v>126.96</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>48.1</v>
+        <v>54.9</v>
       </c>
       <c r="J21" t="n">
-        <v>35.3</v>
+        <v>43.2</v>
       </c>
       <c r="K21" t="n">
-        <v>81</v>
+        <v>13</v>
       </c>
       <c r="L21" t="n">
-        <v>2.35</v>
+        <v>4.82</v>
       </c>
       <c r="M21" t="n">
-        <v>25.2</v>
+        <v>54</v>
       </c>
       <c r="N21" t="n">
-        <v>19.6</v>
+        <v>49.3</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P21" t="n">
-        <v>51.5</v>
+        <v>29.1</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
@@ -2386,72 +2416,76 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U21" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>TSN</t>
+          <t>GILD</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>156.49</v>
+        <v>126.96</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I22" t="n">
-        <v>48.1</v>
+        <v>54.9</v>
       </c>
       <c r="J22" t="n">
-        <v>35.3</v>
+        <v>43.2</v>
       </c>
       <c r="K22" t="n">
-        <v>81</v>
+        <v>13</v>
       </c>
       <c r="L22" t="n">
-        <v>2.35</v>
+        <v>4.82</v>
       </c>
       <c r="M22" t="n">
-        <v>25.2</v>
+        <v>54</v>
       </c>
       <c r="N22" t="n">
-        <v>19.6</v>
+        <v>49.3</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
@@ -2459,11 +2493,11 @@
         </is>
       </c>
       <c r="P22" t="n">
-        <v>44</v>
+        <v>29.7</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
@@ -2478,43 +2512,47 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U22" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>TTD</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>156.49</v>
+        <v>59.17</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2524,26 +2562,23 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I23" t="n">
-        <v>48.1</v>
+        <v>52.4</v>
       </c>
       <c r="J23" t="n">
-        <v>35.3</v>
+        <v>61.9</v>
       </c>
       <c r="K23" t="n">
-        <v>81</v>
+        <v>66.3</v>
       </c>
       <c r="L23" t="n">
-        <v>2.35</v>
+        <v>5.06</v>
       </c>
       <c r="M23" t="n">
-        <v>25.2</v>
-      </c>
-      <c r="N23" t="n">
-        <v>19.6</v>
+        <v>65.2</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -2551,7 +2586,7 @@
         </is>
       </c>
       <c r="P23" t="n">
-        <v>44</v>
+        <v>39.9</v>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
@@ -2565,12 +2600,12 @@
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U23" t="inlineStr"/>
@@ -2583,30 +2618,30 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>TJX</t>
+          <t>PAYX</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>156.49</v>
+        <v>59.17</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -2616,23 +2651,23 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I24" t="n">
-        <v>48.1</v>
+        <v>52.4</v>
       </c>
       <c r="J24" t="n">
-        <v>35.3</v>
+        <v>61.9</v>
       </c>
       <c r="K24" t="n">
-        <v>81</v>
+        <v>66.3</v>
       </c>
       <c r="L24" t="n">
-        <v>2.35</v>
+        <v>5.06</v>
       </c>
       <c r="M24" t="n">
-        <v>26.5</v>
+        <v>38.4</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
@@ -2640,7 +2675,7 @@
         </is>
       </c>
       <c r="P24" t="n">
-        <v>51.5</v>
+        <v>57.7</v>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
@@ -2654,12 +2689,12 @@
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U24" t="inlineStr"/>
@@ -2672,30 +2707,30 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>TRV</t>
+          <t>BKR</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>156.49</v>
+        <v>59.17</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -2705,31 +2740,31 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I25" t="n">
-        <v>48.1</v>
+        <v>52.4</v>
       </c>
       <c r="J25" t="n">
-        <v>35.3</v>
+        <v>61.9</v>
       </c>
       <c r="K25" t="n">
-        <v>81</v>
+        <v>66.3</v>
       </c>
       <c r="L25" t="n">
-        <v>2.35</v>
+        <v>5.06</v>
       </c>
       <c r="M25" t="n">
-        <v>30</v>
+        <v>46.7</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P25" t="n">
-        <v>51.5</v>
+        <v>27.9</v>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
@@ -2743,16 +2778,109 @@
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U25" t="inlineStr"/>
       <c r="V25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>ODFL</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>476.82</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>49.4</v>
+      </c>
+      <c r="J26" t="n">
+        <v>41.8</v>
+      </c>
+      <c r="K26" t="n">
+        <v>22.1</v>
+      </c>
+      <c r="L26" t="n">
+        <v>3.43</v>
+      </c>
+      <c r="M26" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P26" t="n">
+        <v>57.7</v>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
+      <c r="V26" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Scan 27.03.2026 14:59 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V26"/>
+  <dimension ref="A1:V20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -449,7 +449,7 @@
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="6" customWidth="1" min="10" max="10"/>
     <col width="6" customWidth="1" min="11" max="11"/>
-    <col width="6" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
     <col width="9" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
@@ -458,7 +458,7 @@
     <col width="15" customWidth="1" min="18" max="18"/>
     <col width="11" customWidth="1" min="19" max="19"/>
     <col width="11" customWidth="1" min="20" max="20"/>
-    <col width="25" customWidth="1" min="21" max="21"/>
+    <col width="13" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
@@ -577,11 +577,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ORCL</t>
+          <t>PFE</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>318.25</v>
+        <v>339.61</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,30 +614,30 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>66.59999999999999</v>
+        <v>71.2</v>
       </c>
       <c r="J2" t="n">
-        <v>60.9</v>
+        <v>63.2</v>
       </c>
       <c r="K2" t="n">
-        <v>91.90000000000001</v>
+        <v>81.40000000000001</v>
       </c>
       <c r="L2" t="n">
-        <v>6.47</v>
+        <v>10.13</v>
       </c>
       <c r="M2" t="n">
-        <v>76.2</v>
+        <v>91.3</v>
       </c>
       <c r="N2" t="n">
-        <v>46.7</v>
+        <v>54.9</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>67</v>
+        <v>35.6</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -659,40 +659,44 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr"/>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>PFE</t>
+          <t>VRSK</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>318.25</v>
+        <v>92</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -706,30 +710,27 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>66.59999999999999</v>
+        <v>69.5</v>
       </c>
       <c r="J3" t="n">
-        <v>60.9</v>
+        <v>31.8</v>
       </c>
       <c r="K3" t="n">
         <v>91.90000000000001</v>
       </c>
       <c r="L3" t="n">
-        <v>6.47</v>
+        <v>7.41</v>
       </c>
       <c r="M3" t="n">
-        <v>76.2</v>
-      </c>
-      <c r="N3" t="n">
-        <v>46.7</v>
+        <v>46.5</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P3" t="n">
-        <v>67</v>
+        <v>48.7</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -738,12 +739,12 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -751,40 +752,44 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr"/>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>NOC</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>318.25</v>
+        <v>92</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -798,22 +803,19 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>66.59999999999999</v>
+        <v>69.5</v>
       </c>
       <c r="J4" t="n">
-        <v>60.9</v>
+        <v>31.8</v>
       </c>
       <c r="K4" t="n">
         <v>91.90000000000001</v>
       </c>
       <c r="L4" t="n">
-        <v>6.47</v>
+        <v>7.41</v>
       </c>
       <c r="M4" t="n">
-        <v>76.2</v>
-      </c>
-      <c r="N4" t="n">
-        <v>46.7</v>
+        <v>25.5</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -821,7 +823,7 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>67</v>
+        <v>54.2</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -830,12 +832,12 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -843,40 +845,44 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr"/>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>PCAR</t>
+          <t>ROP</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>119.86</v>
+        <v>44.17</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -886,34 +892,34 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>60.5</v>
+        <v>69</v>
       </c>
       <c r="J5" t="n">
-        <v>67</v>
+        <v>30.8</v>
       </c>
       <c r="K5" t="n">
-        <v>79.09999999999999</v>
+        <v>96.5</v>
       </c>
       <c r="L5" t="n">
-        <v>5.07</v>
+        <v>9.220000000000001</v>
       </c>
       <c r="M5" t="n">
-        <v>71.5</v>
+        <v>85.3</v>
       </c>
       <c r="N5" t="n">
-        <v>89.7</v>
+        <v>76.3</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>63.7</v>
+        <v>39</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -927,12 +933,12 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U5" t="inlineStr"/>
@@ -945,30 +951,30 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>NSC</t>
+          <t>PH</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>119.86</v>
+        <v>44.17</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -978,34 +984,34 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>60.5</v>
+        <v>69</v>
       </c>
       <c r="J6" t="n">
-        <v>67</v>
+        <v>30.8</v>
       </c>
       <c r="K6" t="n">
-        <v>79.09999999999999</v>
+        <v>96.5</v>
       </c>
       <c r="L6" t="n">
-        <v>5.07</v>
+        <v>9.220000000000001</v>
       </c>
       <c r="M6" t="n">
-        <v>71.5</v>
+        <v>85.3</v>
       </c>
       <c r="N6" t="n">
-        <v>89.7</v>
+        <v>76.3</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P6" t="n">
-        <v>63.7</v>
+        <v>39</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1019,12 +1025,12 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
@@ -1037,30 +1043,30 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>PNC</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>119.86</v>
+        <v>44.17</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1070,34 +1076,31 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>60.5</v>
+        <v>69</v>
       </c>
       <c r="J7" t="n">
-        <v>67</v>
+        <v>30.8</v>
       </c>
       <c r="K7" t="n">
-        <v>79.09999999999999</v>
+        <v>96.5</v>
       </c>
       <c r="L7" t="n">
-        <v>5.07</v>
+        <v>9.220000000000001</v>
       </c>
       <c r="M7" t="n">
-        <v>71.5</v>
-      </c>
-      <c r="N7" t="n">
-        <v>89.7</v>
+        <v>42</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>63.7</v>
+        <v>39</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1111,12 +1114,12 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U7" t="inlineStr"/>
@@ -1129,30 +1132,30 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>RTX</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>119.86</v>
+        <v>44.17</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1162,34 +1165,34 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>60.5</v>
+        <v>69</v>
       </c>
       <c r="J8" t="n">
-        <v>67</v>
+        <v>30.8</v>
       </c>
       <c r="K8" t="n">
-        <v>79.09999999999999</v>
+        <v>96.5</v>
       </c>
       <c r="L8" t="n">
-        <v>5.07</v>
+        <v>9.220000000000001</v>
       </c>
       <c r="M8" t="n">
-        <v>71.5</v>
+        <v>85.3</v>
       </c>
       <c r="N8" t="n">
-        <v>89.7</v>
+        <v>76.3</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>63.7</v>
+        <v>39</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1203,12 +1206,12 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U8" t="inlineStr"/>
@@ -1221,30 +1224,30 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>NKE</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>119.86</v>
+        <v>44.17</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1254,34 +1257,34 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>60.5</v>
+        <v>69</v>
       </c>
       <c r="J9" t="n">
-        <v>67</v>
+        <v>30.8</v>
       </c>
       <c r="K9" t="n">
-        <v>79.09999999999999</v>
+        <v>96.5</v>
       </c>
       <c r="L9" t="n">
-        <v>5.07</v>
+        <v>9.220000000000001</v>
       </c>
       <c r="M9" t="n">
-        <v>71.5</v>
+        <v>85.3</v>
       </c>
       <c r="N9" t="n">
-        <v>89.7</v>
+        <v>76.3</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>62.7</v>
+        <v>39</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1295,12 +1298,12 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U9" t="inlineStr"/>
@@ -1313,30 +1316,30 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>PEP</t>
+          <t>REGN</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>119.86</v>
+        <v>44.17</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1346,31 +1349,34 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>60.5</v>
+        <v>69</v>
       </c>
       <c r="J10" t="n">
-        <v>67</v>
+        <v>30.8</v>
       </c>
       <c r="K10" t="n">
-        <v>79.09999999999999</v>
+        <v>96.5</v>
       </c>
       <c r="L10" t="n">
-        <v>5.07</v>
+        <v>9.220000000000001</v>
       </c>
       <c r="M10" t="n">
-        <v>29.4</v>
+        <v>85.3</v>
+      </c>
+      <c r="N10" t="n">
+        <v>76.3</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>63.7</v>
+        <v>39</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1384,12 +1390,12 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U10" t="inlineStr"/>
@@ -1402,30 +1408,30 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>MSI</t>
+          <t>ROST</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>119.86</v>
+        <v>44.17</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1435,34 +1441,34 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>60.5</v>
+        <v>69</v>
       </c>
       <c r="J11" t="n">
-        <v>67</v>
+        <v>30.8</v>
       </c>
       <c r="K11" t="n">
-        <v>79.09999999999999</v>
+        <v>96.5</v>
       </c>
       <c r="L11" t="n">
-        <v>5.07</v>
+        <v>9.220000000000001</v>
       </c>
       <c r="M11" t="n">
-        <v>71.5</v>
+        <v>85.3</v>
       </c>
       <c r="N11" t="n">
-        <v>89.7</v>
+        <v>76.3</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>63.7</v>
+        <v>39</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1476,12 +1482,12 @@
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U11" t="inlineStr"/>
@@ -1494,35 +1500,35 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>QCOM</t>
+          <t>ETN</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>294.34</v>
+        <v>324.96</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1531,19 +1537,22 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>58.2</v>
+        <v>64.3</v>
       </c>
       <c r="J12" t="n">
-        <v>63.7</v>
+        <v>60.2</v>
       </c>
       <c r="K12" t="n">
-        <v>28</v>
+        <v>76.7</v>
       </c>
       <c r="L12" t="n">
-        <v>2.55</v>
+        <v>3.83</v>
       </c>
       <c r="M12" t="n">
-        <v>38.4</v>
+        <v>41.5</v>
+      </c>
+      <c r="N12" t="n">
+        <v>68.7</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1551,7 +1560,7 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>35.8</v>
+        <v>41.5</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1560,17 +1569,17 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U12" t="inlineStr"/>
@@ -1583,15 +1592,15 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>PYPL</t>
+          <t>ABBV</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>294.34</v>
+        <v>104.47</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -1606,12 +1615,12 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1620,27 +1629,30 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>58.2</v>
+        <v>56.9</v>
       </c>
       <c r="J13" t="n">
-        <v>63.7</v>
+        <v>33.9</v>
       </c>
       <c r="K13" t="n">
-        <v>28</v>
+        <v>78</v>
       </c>
       <c r="L13" t="n">
-        <v>2.55</v>
+        <v>2.11</v>
       </c>
       <c r="M13" t="n">
-        <v>43.6</v>
+        <v>20.6</v>
+      </c>
+      <c r="N13" t="n">
+        <v>28.9</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>35.8</v>
+        <v>44</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1649,12 +1661,12 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
@@ -1672,15 +1684,15 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>PNC</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>294.34</v>
+        <v>104.47</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
@@ -1695,12 +1707,12 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1709,27 +1721,30 @@
         </is>
       </c>
       <c r="I14" t="n">
-        <v>58.2</v>
+        <v>56.9</v>
       </c>
       <c r="J14" t="n">
-        <v>63.7</v>
+        <v>33.9</v>
       </c>
       <c r="K14" t="n">
-        <v>28</v>
+        <v>78</v>
       </c>
       <c r="L14" t="n">
-        <v>2.55</v>
+        <v>2.11</v>
       </c>
       <c r="M14" t="n">
-        <v>36.6</v>
+        <v>20.6</v>
+      </c>
+      <c r="N14" t="n">
+        <v>28.9</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P14" t="n">
-        <v>35.8</v>
+        <v>48.8</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1738,12 +1753,12 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
@@ -1761,59 +1776,59 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>GM</t>
+          <t>ADP</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>126.96</v>
+        <v>104.47</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>54.9</v>
+        <v>56.9</v>
       </c>
       <c r="J15" t="n">
-        <v>43.2</v>
+        <v>33.9</v>
       </c>
       <c r="K15" t="n">
-        <v>13</v>
+        <v>78</v>
       </c>
       <c r="L15" t="n">
-        <v>4.82</v>
+        <v>2.11</v>
       </c>
       <c r="M15" t="n">
-        <v>54</v>
+        <v>20.6</v>
       </c>
       <c r="N15" t="n">
-        <v>49.3</v>
+        <v>28.9</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1821,11 +1836,11 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>51.8</v>
+        <v>44</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
@@ -1840,28 +1855,24 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U15" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr"/>
       <c r="V15" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>HD</t>
+          <t>GOOG</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>126.96</v>
+        <v>59.41</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -1894,30 +1905,27 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>54.9</v>
+        <v>51.4</v>
       </c>
       <c r="J16" t="n">
-        <v>43.2</v>
+        <v>41.8</v>
       </c>
       <c r="K16" t="n">
-        <v>13</v>
+        <v>10.5</v>
       </c>
       <c r="L16" t="n">
-        <v>4.82</v>
+        <v>4.44</v>
       </c>
       <c r="M16" t="n">
-        <v>54</v>
-      </c>
-      <c r="N16" t="n">
-        <v>49.3</v>
+        <v>35.3</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>29.1</v>
+        <v>52.5</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1941,23 +1949,23 @@
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+          <t>TTM Squeeze</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>GPN</t>
+          <t>KO</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>126.96</v>
+        <v>22.15</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -1986,26 +1994,26 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>54.9</v>
+        <v>39.2</v>
       </c>
       <c r="J17" t="n">
-        <v>43.2</v>
+        <v>36.8</v>
       </c>
       <c r="K17" t="n">
-        <v>13</v>
+        <v>29.1</v>
       </c>
       <c r="L17" t="n">
-        <v>4.82</v>
+        <v>6.11</v>
       </c>
       <c r="M17" t="n">
-        <v>54</v>
+        <v>38.2</v>
       </c>
       <c r="N17" t="n">
-        <v>49.3</v>
+        <v>33</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -2013,7 +2021,7 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>29.1</v>
+        <v>28.5</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -2037,23 +2045,23 @@
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+          <t>TTM Squeeze</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>GOOG</t>
+          <t>MCHP</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>126.96</v>
+        <v>22.15</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -2082,26 +2090,26 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>54.9</v>
+        <v>39.2</v>
       </c>
       <c r="J18" t="n">
-        <v>43.2</v>
+        <v>36.8</v>
       </c>
       <c r="K18" t="n">
-        <v>13</v>
+        <v>29.1</v>
       </c>
       <c r="L18" t="n">
-        <v>4.82</v>
+        <v>6.11</v>
       </c>
       <c r="M18" t="n">
-        <v>54</v>
+        <v>38.2</v>
       </c>
       <c r="N18" t="n">
-        <v>49.3</v>
+        <v>33</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -2109,7 +2117,7 @@
         </is>
       </c>
       <c r="P18" t="n">
-        <v>29.7</v>
+        <v>28.5</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -2133,23 +2141,23 @@
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+          <t>TTM Squeeze</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>LMT</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>126.96</v>
+        <v>22.15</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -2178,26 +2186,23 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>54.9</v>
+        <v>39.2</v>
       </c>
       <c r="J19" t="n">
-        <v>43.2</v>
+        <v>36.8</v>
       </c>
       <c r="K19" t="n">
-        <v>13</v>
+        <v>29.1</v>
       </c>
       <c r="L19" t="n">
-        <v>4.82</v>
+        <v>6.11</v>
       </c>
       <c r="M19" t="n">
-        <v>54</v>
-      </c>
-      <c r="N19" t="n">
-        <v>49.3</v>
+        <v>41.2</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -2205,7 +2210,7 @@
         </is>
       </c>
       <c r="P19" t="n">
-        <v>29.1</v>
+        <v>28.5</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -2229,23 +2234,23 @@
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+          <t>TTM Squeeze</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>HON</t>
+          <t>MET</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>126.96</v>
+        <v>22.15</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -2274,34 +2279,31 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I20" t="n">
-        <v>54.9</v>
+        <v>39.2</v>
       </c>
       <c r="J20" t="n">
-        <v>43.2</v>
+        <v>36.8</v>
       </c>
       <c r="K20" t="n">
-        <v>13</v>
+        <v>29.1</v>
       </c>
       <c r="L20" t="n">
-        <v>4.82</v>
+        <v>6.11</v>
       </c>
       <c r="M20" t="n">
-        <v>54</v>
-      </c>
-      <c r="N20" t="n">
-        <v>49.3</v>
+        <v>41.8</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P20" t="n">
-        <v>51.8</v>
+        <v>28.5</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
@@ -2325,562 +2327,10 @@
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+          <t>TTM Squeeze</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>GS</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>126.96</v>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Debit Put</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>30-60 DTE</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>SQUEEZE</t>
-        </is>
-      </c>
-      <c r="I21" t="n">
-        <v>54.9</v>
-      </c>
-      <c r="J21" t="n">
-        <v>43.2</v>
-      </c>
-      <c r="K21" t="n">
-        <v>13</v>
-      </c>
-      <c r="L21" t="n">
-        <v>4.82</v>
-      </c>
-      <c r="M21" t="n">
-        <v>54</v>
-      </c>
-      <c r="N21" t="n">
-        <v>49.3</v>
-      </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P21" t="n">
-        <v>29.1</v>
-      </c>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S21" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U21" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
-      <c r="V21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>GILD</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>126.96</v>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Debit Put</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>30-60 DTE</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>SQUEEZE</t>
-        </is>
-      </c>
-      <c r="I22" t="n">
-        <v>54.9</v>
-      </c>
-      <c r="J22" t="n">
-        <v>43.2</v>
-      </c>
-      <c r="K22" t="n">
-        <v>13</v>
-      </c>
-      <c r="L22" t="n">
-        <v>4.82</v>
-      </c>
-      <c r="M22" t="n">
-        <v>54</v>
-      </c>
-      <c r="N22" t="n">
-        <v>49.3</v>
-      </c>
-      <c r="O22" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P22" t="n">
-        <v>29.7</v>
-      </c>
-      <c r="Q22" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="R22" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S22" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T22" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U22" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
-      <c r="V22" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>TTD</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>59.17</v>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>Credit Call</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I23" t="n">
-        <v>52.4</v>
-      </c>
-      <c r="J23" t="n">
-        <v>61.9</v>
-      </c>
-      <c r="K23" t="n">
-        <v>66.3</v>
-      </c>
-      <c r="L23" t="n">
-        <v>5.06</v>
-      </c>
-      <c r="M23" t="n">
-        <v>65.2</v>
-      </c>
-      <c r="O23" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P23" t="n">
-        <v>39.9</v>
-      </c>
-      <c r="Q23" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R23" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S23" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="T23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U23" t="inlineStr"/>
-      <c r="V23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>PAYX</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>59.17</v>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>Credit Call</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I24" t="n">
-        <v>52.4</v>
-      </c>
-      <c r="J24" t="n">
-        <v>61.9</v>
-      </c>
-      <c r="K24" t="n">
-        <v>66.3</v>
-      </c>
-      <c r="L24" t="n">
-        <v>5.06</v>
-      </c>
-      <c r="M24" t="n">
-        <v>38.4</v>
-      </c>
-      <c r="O24" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P24" t="n">
-        <v>57.7</v>
-      </c>
-      <c r="Q24" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R24" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S24" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="T24" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U24" t="inlineStr"/>
-      <c r="V24" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>BKR</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>59.17</v>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>Credit Call</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I25" t="n">
-        <v>52.4</v>
-      </c>
-      <c r="J25" t="n">
-        <v>61.9</v>
-      </c>
-      <c r="K25" t="n">
-        <v>66.3</v>
-      </c>
-      <c r="L25" t="n">
-        <v>5.06</v>
-      </c>
-      <c r="M25" t="n">
-        <v>46.7</v>
-      </c>
-      <c r="O25" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P25" t="n">
-        <v>27.9</v>
-      </c>
-      <c r="Q25" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R25" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S25" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="T25" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U25" t="inlineStr"/>
-      <c r="V25" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>ODFL</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>476.82</v>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>Debit Put</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>30-60 DTE</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I26" t="n">
-        <v>49.4</v>
-      </c>
-      <c r="J26" t="n">
-        <v>41.8</v>
-      </c>
-      <c r="K26" t="n">
-        <v>22.1</v>
-      </c>
-      <c r="L26" t="n">
-        <v>3.43</v>
-      </c>
-      <c r="M26" t="n">
-        <v>49.1</v>
-      </c>
-      <c r="O26" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P26" t="n">
-        <v>57.7</v>
-      </c>
-      <c r="Q26" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="R26" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S26" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T26" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U26" t="inlineStr">
-        <is>
-          <t>TTM Squeeze</t>
-        </is>
-      </c>
-      <c r="V26" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Scan 30.03.2026 15:13 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V20"/>
+  <dimension ref="A1:V23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -445,7 +445,7 @@
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="6" customWidth="1" min="10" max="10"/>
     <col width="6" customWidth="1" min="11" max="11"/>
@@ -458,7 +458,7 @@
     <col width="15" customWidth="1" min="18" max="18"/>
     <col width="11" customWidth="1" min="19" max="19"/>
     <col width="11" customWidth="1" min="20" max="20"/>
-    <col width="13" customWidth="1" min="21" max="21"/>
+    <col width="25" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
@@ -577,11 +577,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>PFE</t>
+          <t>EOG</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>339.61</v>
+        <v>326.17</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -610,34 +610,31 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>71.2</v>
+        <v>65.2</v>
       </c>
       <c r="J2" t="n">
-        <v>63.2</v>
+        <v>58.9</v>
       </c>
       <c r="K2" t="n">
-        <v>81.40000000000001</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="L2" t="n">
-        <v>10.13</v>
+        <v>10.07</v>
       </c>
       <c r="M2" t="n">
-        <v>91.3</v>
+        <v>93.3</v>
       </c>
       <c r="N2" t="n">
-        <v>54.9</v>
+        <v>63.5</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P2" t="n">
-        <v>35.6</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -659,44 +656,40 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>VRSK</t>
+          <t>EL</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>92</v>
+        <v>326.17</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -706,23 +699,26 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>69.5</v>
+        <v>65.2</v>
       </c>
       <c r="J3" t="n">
-        <v>31.8</v>
+        <v>58.9</v>
       </c>
       <c r="K3" t="n">
-        <v>91.90000000000001</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="L3" t="n">
-        <v>7.41</v>
+        <v>10.07</v>
       </c>
       <c r="M3" t="n">
-        <v>46.5</v>
+        <v>93.3</v>
+      </c>
+      <c r="N3" t="n">
+        <v>63.5</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -730,7 +726,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>48.7</v>
+        <v>32</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -739,12 +735,12 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -752,44 +748,40 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U3" t="inlineStr"/>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>DIS</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>92</v>
+        <v>326.17</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -799,31 +791,31 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>69.5</v>
+        <v>65.2</v>
       </c>
       <c r="J4" t="n">
-        <v>31.8</v>
+        <v>58.9</v>
       </c>
       <c r="K4" t="n">
-        <v>91.90000000000001</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="L4" t="n">
-        <v>7.41</v>
+        <v>10.07</v>
       </c>
       <c r="M4" t="n">
-        <v>25.5</v>
+        <v>93.3</v>
+      </c>
+      <c r="N4" t="n">
+        <v>63.5</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P4" t="n">
-        <v>54.2</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -832,12 +824,12 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -845,44 +837,40 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ROP</t>
+          <t>EMR</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>44.17</v>
+        <v>326.17</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -892,34 +880,34 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>69</v>
+        <v>65.2</v>
       </c>
       <c r="J5" t="n">
-        <v>30.8</v>
+        <v>58.9</v>
       </c>
       <c r="K5" t="n">
-        <v>96.5</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="L5" t="n">
-        <v>9.220000000000001</v>
+        <v>10.07</v>
       </c>
       <c r="M5" t="n">
-        <v>85.3</v>
+        <v>93.3</v>
       </c>
       <c r="N5" t="n">
-        <v>76.3</v>
+        <v>63.5</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -928,12 +916,12 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -951,30 +939,30 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>PH</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>44.17</v>
+        <v>326.17</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -984,34 +972,31 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>69</v>
+        <v>65.2</v>
       </c>
       <c r="J6" t="n">
-        <v>30.8</v>
+        <v>58.9</v>
       </c>
       <c r="K6" t="n">
-        <v>96.5</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="L6" t="n">
-        <v>9.220000000000001</v>
+        <v>10.07</v>
       </c>
       <c r="M6" t="n">
-        <v>85.3</v>
+        <v>93.3</v>
       </c>
       <c r="N6" t="n">
-        <v>76.3</v>
+        <v>63.5</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P6" t="n">
-        <v>39</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1020,12 +1005,12 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
@@ -1043,30 +1028,30 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>PNC</t>
+          <t>D</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>44.17</v>
+        <v>326.17</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1076,31 +1061,34 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>69</v>
+        <v>65.2</v>
       </c>
       <c r="J7" t="n">
-        <v>30.8</v>
+        <v>58.9</v>
       </c>
       <c r="K7" t="n">
-        <v>96.5</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="L7" t="n">
-        <v>9.220000000000001</v>
+        <v>10.07</v>
       </c>
       <c r="M7" t="n">
-        <v>42</v>
+        <v>93.3</v>
+      </c>
+      <c r="N7" t="n">
+        <v>63.5</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>39</v>
+        <v>45.1</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1109,12 +1097,12 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
@@ -1132,30 +1120,30 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>RTX</t>
+          <t>DOW</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>44.17</v>
+        <v>326.17</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1165,26 +1153,26 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>69</v>
+        <v>65.2</v>
       </c>
       <c r="J8" t="n">
-        <v>30.8</v>
+        <v>58.9</v>
       </c>
       <c r="K8" t="n">
-        <v>96.5</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="L8" t="n">
-        <v>9.220000000000001</v>
+        <v>10.07</v>
       </c>
       <c r="M8" t="n">
-        <v>85.3</v>
+        <v>93.3</v>
       </c>
       <c r="N8" t="n">
-        <v>76.3</v>
+        <v>63.5</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1192,7 +1180,7 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1201,12 +1189,12 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
@@ -1224,30 +1212,30 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>ECL</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>44.17</v>
+        <v>326.17</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1257,34 +1245,34 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>69</v>
+        <v>65.2</v>
       </c>
       <c r="J9" t="n">
-        <v>30.8</v>
+        <v>58.9</v>
       </c>
       <c r="K9" t="n">
-        <v>96.5</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="L9" t="n">
-        <v>9.220000000000001</v>
+        <v>10.07</v>
       </c>
       <c r="M9" t="n">
-        <v>85.3</v>
+        <v>93.3</v>
       </c>
       <c r="N9" t="n">
-        <v>76.3</v>
+        <v>63.5</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>39</v>
+        <v>45.1</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1293,12 +1281,12 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
@@ -1316,30 +1304,30 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>REGN</t>
+          <t>DHR</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>44.17</v>
+        <v>326.17</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1349,34 +1337,31 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>69</v>
+        <v>65.2</v>
       </c>
       <c r="J10" t="n">
-        <v>30.8</v>
+        <v>58.9</v>
       </c>
       <c r="K10" t="n">
-        <v>96.5</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="L10" t="n">
-        <v>9.220000000000001</v>
+        <v>10.07</v>
       </c>
       <c r="M10" t="n">
-        <v>85.3</v>
+        <v>93.3</v>
       </c>
       <c r="N10" t="n">
-        <v>76.3</v>
+        <v>63.5</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P10" t="n">
-        <v>39</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1385,12 +1370,12 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -1408,11 +1393,11 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ROST</t>
+          <t>AAPL</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>44.17</v>
+        <v>103.14</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1441,34 +1426,34 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>69</v>
+        <v>56.6</v>
       </c>
       <c r="J11" t="n">
-        <v>30.8</v>
+        <v>31.1</v>
       </c>
       <c r="K11" t="n">
-        <v>96.5</v>
+        <v>78</v>
       </c>
       <c r="L11" t="n">
-        <v>9.220000000000001</v>
+        <v>2.17</v>
       </c>
       <c r="M11" t="n">
-        <v>85.3</v>
+        <v>20.3</v>
       </c>
       <c r="N11" t="n">
-        <v>76.3</v>
+        <v>27.5</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>39</v>
+        <v>58.1</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1477,17 +1462,17 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U11" t="inlineStr"/>
@@ -1500,15 +1485,15 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ETN</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>324.96</v>
+        <v>119.53</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -1523,48 +1508,48 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>64.3</v>
+        <v>54.6</v>
       </c>
       <c r="J12" t="n">
-        <v>60.2</v>
+        <v>42.3</v>
       </c>
       <c r="K12" t="n">
-        <v>76.7</v>
+        <v>3.5</v>
       </c>
       <c r="L12" t="n">
-        <v>3.83</v>
+        <v>10.6</v>
       </c>
       <c r="M12" t="n">
-        <v>41.5</v>
+        <v>92.8</v>
       </c>
       <c r="N12" t="n">
-        <v>68.7</v>
+        <v>17.7</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>41.5</v>
+        <v>45.8</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
@@ -1574,7 +1559,7 @@
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
@@ -1582,7 +1567,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U12" t="inlineStr"/>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V12" t="inlineStr">
         <is>
           <t>No</t>
@@ -1592,71 +1581,71 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ABBV</t>
+          <t>NSC</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>104.47</v>
+        <v>119.53</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>56.9</v>
+        <v>54.6</v>
       </c>
       <c r="J13" t="n">
-        <v>33.9</v>
+        <v>42.3</v>
       </c>
       <c r="K13" t="n">
-        <v>78</v>
+        <v>3.5</v>
       </c>
       <c r="L13" t="n">
-        <v>2.11</v>
+        <v>10.6</v>
       </c>
       <c r="M13" t="n">
-        <v>20.6</v>
+        <v>92.8</v>
       </c>
       <c r="N13" t="n">
-        <v>28.9</v>
+        <v>17.7</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>44</v>
+        <v>40.2</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
@@ -1671,10 +1660,14 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U13" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V13" t="inlineStr">
         <is>
           <t>No</t>
@@ -1684,71 +1677,71 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>104.47</v>
+        <v>119.53</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>56.9</v>
+        <v>54.6</v>
       </c>
       <c r="J14" t="n">
-        <v>33.9</v>
+        <v>42.3</v>
       </c>
       <c r="K14" t="n">
-        <v>78</v>
+        <v>3.5</v>
       </c>
       <c r="L14" t="n">
-        <v>2.11</v>
+        <v>10.6</v>
       </c>
       <c r="M14" t="n">
-        <v>20.6</v>
+        <v>92.8</v>
       </c>
       <c r="N14" t="n">
-        <v>28.9</v>
+        <v>17.7</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P14" t="n">
-        <v>48.8</v>
+        <v>40.2</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
@@ -1763,10 +1756,14 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U14" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V14" t="inlineStr">
         <is>
           <t>No</t>
@@ -1776,71 +1773,71 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ADP</t>
+          <t>MU</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>104.47</v>
+        <v>119.53</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>56.9</v>
+        <v>54.6</v>
       </c>
       <c r="J15" t="n">
-        <v>33.9</v>
+        <v>42.3</v>
       </c>
       <c r="K15" t="n">
-        <v>78</v>
+        <v>3.5</v>
       </c>
       <c r="L15" t="n">
-        <v>2.11</v>
+        <v>10.6</v>
       </c>
       <c r="M15" t="n">
-        <v>20.6</v>
+        <v>92.8</v>
       </c>
       <c r="N15" t="n">
-        <v>28.9</v>
+        <v>17.7</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P15" t="n">
-        <v>44</v>
+        <v>33.7</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
@@ -1855,10 +1852,14 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U15" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V15" t="inlineStr">
         <is>
           <t>No</t>
@@ -1868,11 +1869,11 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>GOOG</t>
+          <t>ORCL</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>59.41</v>
+        <v>119.53</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -1905,19 +1906,22 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>51.4</v>
+        <v>54.6</v>
       </c>
       <c r="J16" t="n">
-        <v>41.8</v>
+        <v>42.3</v>
       </c>
       <c r="K16" t="n">
-        <v>10.5</v>
+        <v>3.5</v>
       </c>
       <c r="L16" t="n">
-        <v>4.44</v>
+        <v>10.6</v>
       </c>
       <c r="M16" t="n">
-        <v>35.3</v>
+        <v>92.8</v>
+      </c>
+      <c r="N16" t="n">
+        <v>17.7</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -1925,7 +1929,7 @@
         </is>
       </c>
       <c r="P16" t="n">
-        <v>52.5</v>
+        <v>45.8</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1949,7 +1953,7 @@
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>TTM Squeeze</t>
+          <t>TTM Squeeze, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
@@ -1961,11 +1965,11 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>KO</t>
+          <t>NFLX</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>22.15</v>
+        <v>119.53</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -1994,26 +1998,23 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>39.2</v>
+        <v>54.6</v>
       </c>
       <c r="J17" t="n">
-        <v>36.8</v>
+        <v>42.3</v>
       </c>
       <c r="K17" t="n">
-        <v>29.1</v>
+        <v>3.5</v>
       </c>
       <c r="L17" t="n">
-        <v>6.11</v>
+        <v>10.6</v>
       </c>
       <c r="M17" t="n">
-        <v>38.2</v>
-      </c>
-      <c r="N17" t="n">
-        <v>33</v>
+        <v>44.7</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -2021,7 +2022,7 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>28.5</v>
+        <v>40.2</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -2045,7 +2046,7 @@
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>TTM Squeeze</t>
+          <t>TTM Squeeze, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
@@ -2057,11 +2058,11 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>MCHP</t>
+          <t>NKE</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>22.15</v>
+        <v>119.53</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -2090,34 +2091,34 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>39.2</v>
+        <v>54.6</v>
       </c>
       <c r="J18" t="n">
-        <v>36.8</v>
+        <v>42.3</v>
       </c>
       <c r="K18" t="n">
-        <v>29.1</v>
+        <v>3.5</v>
       </c>
       <c r="L18" t="n">
-        <v>6.11</v>
+        <v>10.6</v>
       </c>
       <c r="M18" t="n">
-        <v>38.2</v>
+        <v>92.8</v>
       </c>
       <c r="N18" t="n">
-        <v>33</v>
+        <v>17.7</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P18" t="n">
-        <v>28.5</v>
+        <v>45.8</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -2141,7 +2142,7 @@
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>TTM Squeeze</t>
+          <t>TTM Squeeze, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
@@ -2153,11 +2154,11 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>LMT</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>22.15</v>
+        <v>119.53</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -2186,23 +2187,26 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>39.2</v>
+        <v>54.6</v>
       </c>
       <c r="J19" t="n">
-        <v>36.8</v>
+        <v>42.3</v>
       </c>
       <c r="K19" t="n">
-        <v>29.1</v>
+        <v>3.5</v>
       </c>
       <c r="L19" t="n">
-        <v>6.11</v>
+        <v>10.6</v>
       </c>
       <c r="M19" t="n">
-        <v>41.2</v>
+        <v>92.8</v>
+      </c>
+      <c r="N19" t="n">
+        <v>17.7</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -2210,7 +2214,7 @@
         </is>
       </c>
       <c r="P19" t="n">
-        <v>28.5</v>
+        <v>40.2</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -2234,7 +2238,7 @@
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>TTM Squeeze</t>
+          <t>TTM Squeeze, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
@@ -2246,11 +2250,11 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>MET</t>
+          <t>BAC</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>22.15</v>
+        <v>202.76</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -2283,19 +2287,22 @@
         </is>
       </c>
       <c r="I20" t="n">
-        <v>39.2</v>
+        <v>52.2</v>
       </c>
       <c r="J20" t="n">
-        <v>36.8</v>
+        <v>41.9</v>
       </c>
       <c r="K20" t="n">
-        <v>29.1</v>
+        <v>30</v>
       </c>
       <c r="L20" t="n">
-        <v>6.11</v>
+        <v>2.73</v>
       </c>
       <c r="M20" t="n">
-        <v>41.8</v>
+        <v>29.4</v>
+      </c>
+      <c r="N20" t="n">
+        <v>23.3</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -2303,11 +2310,11 @@
         </is>
       </c>
       <c r="P20" t="n">
-        <v>28.5</v>
+        <v>44.5</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
@@ -2322,15 +2329,284 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr"/>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>WM</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>165.15</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>39.7</v>
+      </c>
+      <c r="J21" t="n">
+        <v>42</v>
+      </c>
+      <c r="K21" t="n">
+        <v>38</v>
+      </c>
+      <c r="L21" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="M21" t="n">
+        <v>29.4</v>
+      </c>
+      <c r="N21" t="n">
+        <v>78.2</v>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P21" t="n">
+        <v>81.90000000000001</v>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="U20" t="inlineStr">
-        <is>
-          <t>TTM Squeeze</t>
-        </is>
-      </c>
-      <c r="V20" t="inlineStr">
+      <c r="U21" t="inlineStr"/>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>VLO</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>165.15</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>39.7</v>
+      </c>
+      <c r="J22" t="n">
+        <v>42</v>
+      </c>
+      <c r="K22" t="n">
+        <v>38</v>
+      </c>
+      <c r="L22" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="M22" t="n">
+        <v>29.4</v>
+      </c>
+      <c r="N22" t="n">
+        <v>78.2</v>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P22" t="n">
+        <v>46.7</v>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr"/>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>WFC</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>165.15</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>39.7</v>
+      </c>
+      <c r="J23" t="n">
+        <v>42</v>
+      </c>
+      <c r="K23" t="n">
+        <v>38</v>
+      </c>
+      <c r="L23" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="M23" t="n">
+        <v>43.7</v>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P23" t="n">
+        <v>81.90000000000001</v>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr"/>
+      <c r="V23" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Scan 31.03.2026 15:11 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,9 +29,6 @@
       <b val="1"/>
       <color rgb="00f1f5f9"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <color rgb="00ef4444"/>
     </font>
     <font>
       <color rgb="0022c55e"/>
@@ -63,13 +60,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -435,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V23"/>
+  <dimension ref="A1:V14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -444,12 +440,12 @@
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="6" customWidth="1" min="10" max="10"/>
     <col width="6" customWidth="1" min="11" max="11"/>
-    <col width="7" customWidth="1" min="12" max="12"/>
+    <col width="6" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
     <col width="9" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
@@ -458,7 +454,7 @@
     <col width="15" customWidth="1" min="18" max="18"/>
     <col width="11" customWidth="1" min="19" max="19"/>
     <col width="11" customWidth="1" min="20" max="20"/>
-    <col width="25" customWidth="1" min="21" max="21"/>
+    <col width="10" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
@@ -577,11 +573,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>EOG</t>
+          <t>SMCI</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>326.17</v>
+        <v>157.96</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -590,17 +586,17 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>BEARISH</t>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -610,31 +606,34 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>65.2</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="J2" t="n">
-        <v>58.9</v>
+        <v>42.1</v>
       </c>
       <c r="K2" t="n">
-        <v>79.09999999999999</v>
+        <v>93</v>
       </c>
       <c r="L2" t="n">
-        <v>10.07</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="M2" t="n">
-        <v>93.3</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="N2" t="n">
-        <v>63.5</v>
+        <v>96.7</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P2" t="n">
+        <v>49.9</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -648,12 +647,12 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
@@ -666,11 +665,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>EL</t>
+          <t>SBUX</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>326.17</v>
+        <v>157.96</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -679,17 +678,17 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>BEARISH</t>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -699,34 +698,34 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>65.2</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="J3" t="n">
-        <v>58.9</v>
+        <v>42.1</v>
       </c>
       <c r="K3" t="n">
-        <v>79.09999999999999</v>
+        <v>93</v>
       </c>
       <c r="L3" t="n">
-        <v>10.07</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="M3" t="n">
-        <v>93.3</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="N3" t="n">
-        <v>63.5</v>
+        <v>96.7</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P3" t="n">
-        <v>32</v>
+        <v>49.9</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -740,12 +739,12 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U3" t="inlineStr"/>
@@ -758,11 +757,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>DIS</t>
+          <t>SYY</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>326.17</v>
+        <v>157.96</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -771,17 +770,17 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>BEARISH</t>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -791,31 +790,31 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>65.2</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="J4" t="n">
-        <v>58.9</v>
+        <v>42.1</v>
       </c>
       <c r="K4" t="n">
-        <v>79.09999999999999</v>
+        <v>93</v>
       </c>
       <c r="L4" t="n">
-        <v>10.07</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="M4" t="n">
-        <v>93.3</v>
-      </c>
-      <c r="N4" t="n">
-        <v>63.5</v>
+        <v>36.4</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P4" t="n">
+        <v>33.5</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -829,12 +828,12 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U4" t="inlineStr"/>
@@ -847,11 +846,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>EMR</t>
+          <t>T</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>326.17</v>
+        <v>157.96</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -860,17 +859,17 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>BEARISH</t>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -880,34 +879,34 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>65.2</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="J5" t="n">
-        <v>58.9</v>
+        <v>42.1</v>
       </c>
       <c r="K5" t="n">
-        <v>79.09999999999999</v>
+        <v>93</v>
       </c>
       <c r="L5" t="n">
-        <v>10.07</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="M5" t="n">
-        <v>93.3</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="N5" t="n">
-        <v>63.5</v>
+        <v>96.7</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>34</v>
+        <v>39.2</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -921,12 +920,12 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U5" t="inlineStr"/>
@@ -939,11 +938,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>SHW</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>326.17</v>
+        <v>157.96</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -952,17 +951,17 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>BEARISH</t>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -972,31 +971,34 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>65.2</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="J6" t="n">
-        <v>58.9</v>
+        <v>42.1</v>
       </c>
       <c r="K6" t="n">
-        <v>79.09999999999999</v>
+        <v>93</v>
       </c>
       <c r="L6" t="n">
-        <v>10.07</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="M6" t="n">
-        <v>93.3</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="N6" t="n">
-        <v>63.5</v>
+        <v>96.7</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P6" t="n">
+        <v>49.9</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1010,12 +1012,12 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
@@ -1028,11 +1030,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>SO</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>326.17</v>
+        <v>157.96</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1041,17 +1043,17 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>BEARISH</t>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1061,34 +1063,31 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>65.2</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="J7" t="n">
-        <v>58.9</v>
+        <v>42.1</v>
       </c>
       <c r="K7" t="n">
-        <v>79.09999999999999</v>
+        <v>93</v>
       </c>
       <c r="L7" t="n">
-        <v>10.07</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="M7" t="n">
-        <v>93.3</v>
-      </c>
-      <c r="N7" t="n">
-        <v>63.5</v>
+        <v>27.4</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>45.1</v>
+        <v>33.5</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1102,12 +1101,12 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U7" t="inlineStr"/>
@@ -1120,11 +1119,11 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>DOW</t>
+          <t>SNPS</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>326.17</v>
+        <v>157.96</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1133,17 +1132,17 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>BEARISH</t>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1153,34 +1152,34 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>65.2</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="J8" t="n">
-        <v>58.9</v>
+        <v>42.1</v>
       </c>
       <c r="K8" t="n">
-        <v>79.09999999999999</v>
+        <v>93</v>
       </c>
       <c r="L8" t="n">
-        <v>10.07</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="M8" t="n">
-        <v>93.3</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="N8" t="n">
-        <v>63.5</v>
+        <v>96.7</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>32</v>
+        <v>42.9</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1194,12 +1193,12 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U8" t="inlineStr"/>
@@ -1212,11 +1211,11 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ECL</t>
+          <t>TSLA</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>326.17</v>
+        <v>45.01</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1225,17 +1224,17 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>BEARISH</t>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1245,34 +1244,34 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>65.2</v>
+        <v>67.8</v>
       </c>
       <c r="J9" t="n">
-        <v>58.9</v>
+        <v>33.5</v>
       </c>
       <c r="K9" t="n">
-        <v>79.09999999999999</v>
+        <v>95.3</v>
       </c>
       <c r="L9" t="n">
-        <v>10.07</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="M9" t="n">
-        <v>93.3</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="N9" t="n">
-        <v>63.5</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>45.1</v>
+        <v>49.9</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1281,12 +1280,12 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
@@ -1304,11 +1303,11 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>DHR</t>
+          <t>SRE</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>326.17</v>
+        <v>45.01</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1317,17 +1316,17 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>BEARISH</t>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1337,31 +1336,31 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>65.2</v>
+        <v>67.8</v>
       </c>
       <c r="J10" t="n">
-        <v>58.9</v>
+        <v>33.5</v>
       </c>
       <c r="K10" t="n">
-        <v>79.09999999999999</v>
+        <v>95.3</v>
       </c>
       <c r="L10" t="n">
-        <v>10.07</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="M10" t="n">
-        <v>93.3</v>
-      </c>
-      <c r="N10" t="n">
-        <v>63.5</v>
+        <v>33.7</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P10" t="n">
+        <v>49.9</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1370,12 +1369,12 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -1393,18 +1392,18 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>TGT</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>103.14</v>
+        <v>45.01</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
@@ -1426,34 +1425,34 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>56.6</v>
+        <v>67.8</v>
       </c>
       <c r="J11" t="n">
-        <v>31.1</v>
+        <v>33.5</v>
       </c>
       <c r="K11" t="n">
-        <v>78</v>
+        <v>95.3</v>
       </c>
       <c r="L11" t="n">
-        <v>2.17</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="M11" t="n">
-        <v>20.3</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="N11" t="n">
-        <v>27.5</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>58.1</v>
+        <v>39.2</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1462,17 +1461,17 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U11" t="inlineStr"/>
@@ -1485,81 +1484,81 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>TJX</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>119.53</v>
+        <v>45.01</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>BEARISH</t>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>54.6</v>
+        <v>67.8</v>
       </c>
       <c r="J12" t="n">
-        <v>42.3</v>
+        <v>33.5</v>
       </c>
       <c r="K12" t="n">
-        <v>3.5</v>
+        <v>95.3</v>
       </c>
       <c r="L12" t="n">
-        <v>10.6</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="M12" t="n">
-        <v>92.8</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="N12" t="n">
-        <v>17.7</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>45.8</v>
+        <v>39.4</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
@@ -1567,11 +1566,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U12" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U12" t="inlineStr"/>
       <c r="V12" t="inlineStr">
         <is>
           <t>No</t>
@@ -1581,59 +1576,59 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>NSC</t>
+          <t>TMO</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>119.53</v>
+        <v>45.01</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>BEARISH</t>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>54.6</v>
+        <v>67.8</v>
       </c>
       <c r="J13" t="n">
-        <v>42.3</v>
+        <v>33.5</v>
       </c>
       <c r="K13" t="n">
-        <v>3.5</v>
+        <v>95.3</v>
       </c>
       <c r="L13" t="n">
-        <v>10.6</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="M13" t="n">
-        <v>92.8</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="N13" t="n">
-        <v>17.7</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1641,21 +1636,21 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>40.2</v>
+        <v>39.4</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
@@ -1663,11 +1658,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U13" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U13" t="inlineStr"/>
       <c r="V13" t="inlineStr">
         <is>
           <t>No</t>
@@ -1677,59 +1668,59 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>TXN</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>119.53</v>
+        <v>947.98</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>BEARISH</t>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>54.6</v>
+        <v>59.3</v>
       </c>
       <c r="J14" t="n">
-        <v>42.3</v>
+        <v>39.2</v>
       </c>
       <c r="K14" t="n">
-        <v>3.5</v>
+        <v>75</v>
       </c>
       <c r="L14" t="n">
-        <v>10.6</v>
+        <v>2.79</v>
       </c>
       <c r="M14" t="n">
-        <v>92.8</v>
+        <v>31.9</v>
       </c>
       <c r="N14" t="n">
-        <v>17.7</v>
+        <v>48.8</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1737,21 +1728,21 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>40.2</v>
+        <v>39.4</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
@@ -1759,854 +1750,8 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U14" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U14" t="inlineStr"/>
       <c r="V14" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>MU</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>119.53</v>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Debit Put</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>30-60 DTE</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>SQUEEZE</t>
-        </is>
-      </c>
-      <c r="I15" t="n">
-        <v>54.6</v>
-      </c>
-      <c r="J15" t="n">
-        <v>42.3</v>
-      </c>
-      <c r="K15" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="L15" t="n">
-        <v>10.6</v>
-      </c>
-      <c r="M15" t="n">
-        <v>92.8</v>
-      </c>
-      <c r="N15" t="n">
-        <v>17.7</v>
-      </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P15" t="n">
-        <v>33.7</v>
-      </c>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="R15" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S15" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T15" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U15" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
-      <c r="V15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>ORCL</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>119.53</v>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Debit Put</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>30-60 DTE</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>SQUEEZE</t>
-        </is>
-      </c>
-      <c r="I16" t="n">
-        <v>54.6</v>
-      </c>
-      <c r="J16" t="n">
-        <v>42.3</v>
-      </c>
-      <c r="K16" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="L16" t="n">
-        <v>10.6</v>
-      </c>
-      <c r="M16" t="n">
-        <v>92.8</v>
-      </c>
-      <c r="N16" t="n">
-        <v>17.7</v>
-      </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P16" t="n">
-        <v>45.8</v>
-      </c>
-      <c r="Q16" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="R16" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S16" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T16" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U16" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
-      <c r="V16" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>NFLX</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>119.53</v>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Debit Put</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>30-60 DTE</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>SQUEEZE</t>
-        </is>
-      </c>
-      <c r="I17" t="n">
-        <v>54.6</v>
-      </c>
-      <c r="J17" t="n">
-        <v>42.3</v>
-      </c>
-      <c r="K17" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="L17" t="n">
-        <v>10.6</v>
-      </c>
-      <c r="M17" t="n">
-        <v>44.7</v>
-      </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P17" t="n">
-        <v>40.2</v>
-      </c>
-      <c r="Q17" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="R17" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S17" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T17" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U17" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
-      <c r="V17" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>NKE</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>119.53</v>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Debit Put</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>30-60 DTE</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>SQUEEZE</t>
-        </is>
-      </c>
-      <c r="I18" t="n">
-        <v>54.6</v>
-      </c>
-      <c r="J18" t="n">
-        <v>42.3</v>
-      </c>
-      <c r="K18" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="L18" t="n">
-        <v>10.6</v>
-      </c>
-      <c r="M18" t="n">
-        <v>92.8</v>
-      </c>
-      <c r="N18" t="n">
-        <v>17.7</v>
-      </c>
-      <c r="O18" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P18" t="n">
-        <v>45.8</v>
-      </c>
-      <c r="Q18" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="R18" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S18" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T18" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U18" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
-      <c r="V18" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>MSCI</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>119.53</v>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Debit Put</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>30-60 DTE</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>SQUEEZE</t>
-        </is>
-      </c>
-      <c r="I19" t="n">
-        <v>54.6</v>
-      </c>
-      <c r="J19" t="n">
-        <v>42.3</v>
-      </c>
-      <c r="K19" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="L19" t="n">
-        <v>10.6</v>
-      </c>
-      <c r="M19" t="n">
-        <v>92.8</v>
-      </c>
-      <c r="N19" t="n">
-        <v>17.7</v>
-      </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P19" t="n">
-        <v>40.2</v>
-      </c>
-      <c r="Q19" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="R19" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S19" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T19" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U19" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
-      <c r="V19" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>BAC</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>202.76</v>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Debit Put</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>30-60 DTE</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I20" t="n">
-        <v>52.2</v>
-      </c>
-      <c r="J20" t="n">
-        <v>41.9</v>
-      </c>
-      <c r="K20" t="n">
-        <v>30</v>
-      </c>
-      <c r="L20" t="n">
-        <v>2.73</v>
-      </c>
-      <c r="M20" t="n">
-        <v>29.4</v>
-      </c>
-      <c r="N20" t="n">
-        <v>23.3</v>
-      </c>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P20" t="n">
-        <v>44.5</v>
-      </c>
-      <c r="Q20" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R20" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S20" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T20" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U20" t="inlineStr"/>
-      <c r="V20" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>WM</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>165.15</v>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I21" t="n">
-        <v>39.7</v>
-      </c>
-      <c r="J21" t="n">
-        <v>42</v>
-      </c>
-      <c r="K21" t="n">
-        <v>38</v>
-      </c>
-      <c r="L21" t="n">
-        <v>2.36</v>
-      </c>
-      <c r="M21" t="n">
-        <v>29.4</v>
-      </c>
-      <c r="N21" t="n">
-        <v>78.2</v>
-      </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P21" t="n">
-        <v>81.90000000000001</v>
-      </c>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="S21" t="inlineStr">
-        <is>
-          <t>maroon</t>
-        </is>
-      </c>
-      <c r="T21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U21" t="inlineStr"/>
-      <c r="V21" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>VLO</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>165.15</v>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I22" t="n">
-        <v>39.7</v>
-      </c>
-      <c r="J22" t="n">
-        <v>42</v>
-      </c>
-      <c r="K22" t="n">
-        <v>38</v>
-      </c>
-      <c r="L22" t="n">
-        <v>2.36</v>
-      </c>
-      <c r="M22" t="n">
-        <v>29.4</v>
-      </c>
-      <c r="N22" t="n">
-        <v>78.2</v>
-      </c>
-      <c r="O22" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P22" t="n">
-        <v>46.7</v>
-      </c>
-      <c r="Q22" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R22" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="S22" t="inlineStr">
-        <is>
-          <t>maroon</t>
-        </is>
-      </c>
-      <c r="T22" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U22" t="inlineStr"/>
-      <c r="V22" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>WFC</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>165.15</v>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I23" t="n">
-        <v>39.7</v>
-      </c>
-      <c r="J23" t="n">
-        <v>42</v>
-      </c>
-      <c r="K23" t="n">
-        <v>38</v>
-      </c>
-      <c r="L23" t="n">
-        <v>2.36</v>
-      </c>
-      <c r="M23" t="n">
-        <v>43.7</v>
-      </c>
-      <c r="O23" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P23" t="n">
-        <v>81.90000000000001</v>
-      </c>
-      <c r="Q23" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R23" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="S23" t="inlineStr">
-        <is>
-          <t>maroon</t>
-        </is>
-      </c>
-      <c r="T23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U23" t="inlineStr"/>
-      <c r="V23" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Scan 01.04.2026 15:14 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,6 +32,9 @@
     </font>
     <font>
       <color rgb="0022c55e"/>
+    </font>
+    <font>
+      <color rgb="00ef4444"/>
     </font>
   </fonts>
   <fills count="3">
@@ -60,12 +63,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -431,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V14"/>
+  <dimension ref="A1:V17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -440,12 +444,12 @@
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="6" customWidth="1" min="10" max="10"/>
     <col width="6" customWidth="1" min="11" max="11"/>
-    <col width="6" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
     <col width="9" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
@@ -454,7 +458,7 @@
     <col width="15" customWidth="1" min="18" max="18"/>
     <col width="11" customWidth="1" min="19" max="19"/>
     <col width="11" customWidth="1" min="20" max="20"/>
-    <col width="10" customWidth="1" min="21" max="21"/>
+    <col width="25" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
@@ -573,15 +577,15 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SMCI</t>
+          <t>UPS</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>157.96</v>
+        <v>121.44</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -596,36 +600,36 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>68.59999999999999</v>
+        <v>66.8</v>
       </c>
       <c r="J2" t="n">
-        <v>42.1</v>
+        <v>61.3</v>
       </c>
       <c r="K2" t="n">
-        <v>93</v>
+        <v>14</v>
       </c>
       <c r="L2" t="n">
-        <v>9.390000000000001</v>
+        <v>2.28</v>
       </c>
       <c r="M2" t="n">
-        <v>86.09999999999999</v>
+        <v>22</v>
       </c>
       <c r="N2" t="n">
-        <v>96.7</v>
+        <v>30</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -633,29 +637,33 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>49.9</v>
+        <v>61</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V2" t="inlineStr">
         <is>
           <t>No</t>
@@ -665,15 +673,15 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SBUX</t>
+          <t>VRTX</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>157.96</v>
+        <v>121.44</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -688,36 +696,36 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>68.59999999999999</v>
+        <v>66.8</v>
       </c>
       <c r="J3" t="n">
-        <v>42.1</v>
+        <v>61.3</v>
       </c>
       <c r="K3" t="n">
-        <v>93</v>
+        <v>14</v>
       </c>
       <c r="L3" t="n">
-        <v>9.390000000000001</v>
+        <v>2.28</v>
       </c>
       <c r="M3" t="n">
-        <v>86.09999999999999</v>
+        <v>22</v>
       </c>
       <c r="N3" t="n">
-        <v>96.7</v>
+        <v>30</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -725,29 +733,33 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>49.9</v>
+        <v>61</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V3" t="inlineStr">
         <is>
           <t>No</t>
@@ -757,15 +769,15 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SYY</t>
+          <t>WMT</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>157.96</v>
+        <v>121.44</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -780,63 +792,70 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>68.59999999999999</v>
+        <v>66.8</v>
       </c>
       <c r="J4" t="n">
-        <v>42.1</v>
+        <v>61.3</v>
       </c>
       <c r="K4" t="n">
-        <v>93</v>
+        <v>14</v>
       </c>
       <c r="L4" t="n">
-        <v>9.390000000000001</v>
+        <v>2.28</v>
       </c>
       <c r="M4" t="n">
-        <v>36.4</v>
+        <v>22</v>
+      </c>
+      <c r="N4" t="n">
+        <v>30</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P4" t="n">
-        <v>33.5</v>
+        <v>41.1</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V4" t="inlineStr">
         <is>
           <t>No</t>
@@ -846,15 +865,15 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>157.96</v>
+        <v>121.44</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -869,66 +888,70 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>68.59999999999999</v>
+        <v>66.8</v>
       </c>
       <c r="J5" t="n">
-        <v>42.1</v>
+        <v>61.3</v>
       </c>
       <c r="K5" t="n">
-        <v>93</v>
+        <v>14</v>
       </c>
       <c r="L5" t="n">
-        <v>9.390000000000001</v>
+        <v>2.28</v>
       </c>
       <c r="M5" t="n">
-        <v>86.09999999999999</v>
+        <v>22</v>
       </c>
       <c r="N5" t="n">
-        <v>96.7</v>
+        <v>30</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>39.2</v>
+        <v>61</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V5" t="inlineStr">
         <is>
           <t>No</t>
@@ -938,11 +961,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SHW</t>
+          <t>BK</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>157.96</v>
+        <v>241.89</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -975,22 +998,22 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>68.59999999999999</v>
+        <v>65</v>
       </c>
       <c r="J6" t="n">
-        <v>42.1</v>
+        <v>38.7</v>
       </c>
       <c r="K6" t="n">
         <v>93</v>
       </c>
       <c r="L6" t="n">
-        <v>9.390000000000001</v>
+        <v>3.48</v>
       </c>
       <c r="M6" t="n">
-        <v>86.09999999999999</v>
+        <v>38.7</v>
       </c>
       <c r="N6" t="n">
-        <v>96.7</v>
+        <v>80</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -998,7 +1021,7 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>49.9</v>
+        <v>54.8</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1007,17 +1030,17 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
@@ -1030,11 +1053,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SO</t>
+          <t>BA</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>157.96</v>
+        <v>241.89</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1067,27 +1090,30 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>68.59999999999999</v>
+        <v>65</v>
       </c>
       <c r="J7" t="n">
-        <v>42.1</v>
+        <v>38.7</v>
       </c>
       <c r="K7" t="n">
         <v>93</v>
       </c>
       <c r="L7" t="n">
-        <v>9.390000000000001</v>
+        <v>3.48</v>
       </c>
       <c r="M7" t="n">
-        <v>27.4</v>
+        <v>38.7</v>
+      </c>
+      <c r="N7" t="n">
+        <v>80</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>33.5</v>
+        <v>54.8</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1096,17 +1122,17 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U7" t="inlineStr"/>
@@ -1119,30 +1145,30 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SNPS</t>
+          <t>CAT</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>157.96</v>
+        <v>325.14</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1156,30 +1182,30 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>68.59999999999999</v>
+        <v>63.8</v>
       </c>
       <c r="J8" t="n">
-        <v>42.1</v>
+        <v>62.7</v>
       </c>
       <c r="K8" t="n">
-        <v>93</v>
+        <v>80.2</v>
       </c>
       <c r="L8" t="n">
-        <v>9.390000000000001</v>
+        <v>6.62</v>
       </c>
       <c r="M8" t="n">
-        <v>86.09999999999999</v>
+        <v>77</v>
       </c>
       <c r="N8" t="n">
-        <v>96.7</v>
+        <v>48.7</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>42.9</v>
+        <v>39.5</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1188,12 +1214,12 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
@@ -1211,81 +1237,81 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>TSLA</t>
+          <t>META</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>45.01</v>
+        <v>126.69</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>67.8</v>
+        <v>56.7</v>
       </c>
       <c r="J9" t="n">
-        <v>33.5</v>
+        <v>47.4</v>
       </c>
       <c r="K9" t="n">
-        <v>95.3</v>
+        <v>3.5</v>
       </c>
       <c r="L9" t="n">
-        <v>8.390000000000001</v>
+        <v>10.78</v>
       </c>
       <c r="M9" t="n">
-        <v>86.09999999999999</v>
+        <v>94</v>
       </c>
       <c r="N9" t="n">
-        <v>78.59999999999999</v>
+        <v>19.7</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>49.9</v>
+        <v>43.3</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
@@ -1293,7 +1319,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U9" t="inlineStr"/>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V9" t="inlineStr">
         <is>
           <t>No</t>
@@ -1303,78 +1333,81 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SRE</t>
+          <t>LRCX</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>45.01</v>
+        <v>126.69</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>67.8</v>
+        <v>56.7</v>
       </c>
       <c r="J10" t="n">
-        <v>33.5</v>
+        <v>47.4</v>
       </c>
       <c r="K10" t="n">
-        <v>95.3</v>
+        <v>3.5</v>
       </c>
       <c r="L10" t="n">
-        <v>8.390000000000001</v>
+        <v>10.78</v>
       </c>
       <c r="M10" t="n">
-        <v>33.7</v>
+        <v>94</v>
+      </c>
+      <c r="N10" t="n">
+        <v>19.7</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>49.9</v>
+        <v>43.3</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -1382,7 +1415,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U10" t="inlineStr"/>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V10" t="inlineStr">
         <is>
           <t>No</t>
@@ -1392,59 +1429,59 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>TGT</t>
+          <t>MMC</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>45.01</v>
+        <v>126.69</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>67.8</v>
+        <v>56.7</v>
       </c>
       <c r="J11" t="n">
-        <v>33.5</v>
+        <v>47.4</v>
       </c>
       <c r="K11" t="n">
-        <v>95.3</v>
+        <v>3.5</v>
       </c>
       <c r="L11" t="n">
-        <v>8.390000000000001</v>
+        <v>10.78</v>
       </c>
       <c r="M11" t="n">
-        <v>86.09999999999999</v>
+        <v>94</v>
       </c>
       <c r="N11" t="n">
-        <v>78.59999999999999</v>
+        <v>19.7</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1452,21 +1489,21 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>39.2</v>
+        <v>43.3</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
@@ -1474,7 +1511,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U11" t="inlineStr"/>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V11" t="inlineStr">
         <is>
           <t>No</t>
@@ -1484,59 +1525,59 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TJX</t>
+          <t>MMM</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>45.01</v>
+        <v>126.69</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>67.8</v>
+        <v>56.7</v>
       </c>
       <c r="J12" t="n">
-        <v>33.5</v>
+        <v>47.4</v>
       </c>
       <c r="K12" t="n">
-        <v>95.3</v>
+        <v>3.5</v>
       </c>
       <c r="L12" t="n">
-        <v>8.390000000000001</v>
+        <v>10.78</v>
       </c>
       <c r="M12" t="n">
-        <v>86.09999999999999</v>
+        <v>94</v>
       </c>
       <c r="N12" t="n">
-        <v>78.59999999999999</v>
+        <v>19.7</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1544,21 +1585,21 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>39.4</v>
+        <v>43.3</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
@@ -1566,7 +1607,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U12" t="inlineStr"/>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V12" t="inlineStr">
         <is>
           <t>No</t>
@@ -1576,59 +1621,59 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TMO</t>
+          <t>MCHP</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>45.01</v>
+        <v>126.69</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>67.8</v>
+        <v>56.7</v>
       </c>
       <c r="J13" t="n">
-        <v>33.5</v>
+        <v>47.4</v>
       </c>
       <c r="K13" t="n">
-        <v>95.3</v>
+        <v>3.5</v>
       </c>
       <c r="L13" t="n">
-        <v>8.390000000000001</v>
+        <v>10.78</v>
       </c>
       <c r="M13" t="n">
-        <v>86.09999999999999</v>
+        <v>94</v>
       </c>
       <c r="N13" t="n">
-        <v>78.59999999999999</v>
+        <v>19.7</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1636,21 +1681,21 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>39.4</v>
+        <v>43.3</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
@@ -1658,7 +1703,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U13" t="inlineStr"/>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V13" t="inlineStr">
         <is>
           <t>No</t>
@@ -1668,90 +1717,378 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>TXN</t>
+          <t>MET</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>947.98</v>
+        <v>126.69</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>56.7</v>
+      </c>
+      <c r="J14" t="n">
+        <v>47.4</v>
+      </c>
+      <c r="K14" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="L14" t="n">
+        <v>10.78</v>
+      </c>
+      <c r="M14" t="n">
+        <v>94</v>
+      </c>
+      <c r="N14" t="n">
+        <v>19.7</v>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P14" t="n">
+        <v>43.3</v>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>MDLZ</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>126.69</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>56.7</v>
+      </c>
+      <c r="J15" t="n">
+        <v>47.4</v>
+      </c>
+      <c r="K15" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="L15" t="n">
+        <v>10.78</v>
+      </c>
+      <c r="M15" t="n">
+        <v>94</v>
+      </c>
+      <c r="N15" t="n">
+        <v>19.7</v>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P15" t="n">
+        <v>43.3</v>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>MDT</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>126.69</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>56.7</v>
+      </c>
+      <c r="J16" t="n">
+        <v>47.4</v>
+      </c>
+      <c r="K16" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="L16" t="n">
+        <v>10.78</v>
+      </c>
+      <c r="M16" t="n">
+        <v>94</v>
+      </c>
+      <c r="N16" t="n">
+        <v>19.7</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P16" t="n">
+        <v>43.3</v>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>GS</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>169.68</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
           <t>NEUTRAL</t>
         </is>
       </c>
-      <c r="I14" t="n">
-        <v>59.3</v>
-      </c>
-      <c r="J14" t="n">
-        <v>39.2</v>
-      </c>
-      <c r="K14" t="n">
-        <v>75</v>
-      </c>
-      <c r="L14" t="n">
-        <v>2.79</v>
-      </c>
-      <c r="M14" t="n">
-        <v>31.9</v>
-      </c>
-      <c r="N14" t="n">
+      <c r="I17" t="n">
+        <v>30.6</v>
+      </c>
+      <c r="J17" t="n">
+        <v>34</v>
+      </c>
+      <c r="K17" t="n">
+        <v>36</v>
+      </c>
+      <c r="L17" t="n">
+        <v>6.21</v>
+      </c>
+      <c r="M17" t="n">
         <v>48.8</v>
       </c>
-      <c r="O14" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P14" t="n">
-        <v>39.4</v>
-      </c>
-      <c r="Q14" t="inlineStr">
+      <c r="N17" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P17" t="n">
+        <v>51.4</v>
+      </c>
+      <c r="Q17" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>
       </c>
-      <c r="R14" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="S14" t="inlineStr">
-        <is>
-          <t>maroon</t>
-        </is>
-      </c>
-      <c r="T14" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U14" t="inlineStr"/>
-      <c r="V14" t="inlineStr">
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr"/>
+      <c r="V17" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Scan 02.04.2026 15:06 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,9 +29,6 @@
       <b val="1"/>
       <color rgb="00f1f5f9"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <color rgb="0022c55e"/>
     </font>
     <font>
       <color rgb="00ef4444"/>
@@ -63,13 +60,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -435,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V17"/>
+  <dimension ref="A1:V16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -577,81 +573,81 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>UPS</t>
+          <t>QCOM</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>121.44</v>
+        <v>624.34</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>BULLISH</t>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>66.8</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="J2" t="n">
-        <v>61.3</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="K2" t="n">
-        <v>14</v>
+        <v>94.2</v>
       </c>
       <c r="L2" t="n">
-        <v>2.28</v>
+        <v>5.39</v>
       </c>
       <c r="M2" t="n">
-        <v>22</v>
+        <v>56.1</v>
       </c>
       <c r="N2" t="n">
-        <v>30</v>
+        <v>60.6</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>61</v>
+        <v>45.5</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -659,11 +655,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr">
         <is>
           <t>No</t>
@@ -673,81 +665,81 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>VRTX</t>
+          <t>PGR</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>121.44</v>
+        <v>624.34</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>BULLISH</t>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>66.8</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="J3" t="n">
-        <v>61.3</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="K3" t="n">
-        <v>14</v>
+        <v>94.2</v>
       </c>
       <c r="L3" t="n">
-        <v>2.28</v>
+        <v>5.39</v>
       </c>
       <c r="M3" t="n">
-        <v>22</v>
+        <v>56.1</v>
       </c>
       <c r="N3" t="n">
-        <v>30</v>
+        <v>60.6</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P3" t="n">
-        <v>61</v>
+        <v>31.4</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -755,11 +747,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U3" t="inlineStr"/>
       <c r="V3" t="inlineStr">
         <is>
           <t>No</t>
@@ -769,11 +757,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>WMT</t>
+          <t>TDG</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>121.44</v>
+        <v>126.21</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -782,17 +770,17 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>BULLISH</t>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -806,30 +794,27 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>66.8</v>
+        <v>56.3</v>
       </c>
       <c r="J4" t="n">
-        <v>61.3</v>
+        <v>47</v>
       </c>
       <c r="K4" t="n">
-        <v>14</v>
+        <v>3.5</v>
       </c>
       <c r="L4" t="n">
-        <v>2.28</v>
+        <v>10.82</v>
       </c>
       <c r="M4" t="n">
-        <v>22</v>
+        <v>93.8</v>
       </c>
       <c r="N4" t="n">
-        <v>30</v>
+        <v>19.4</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Neutral</t>
-        </is>
-      </c>
-      <c r="P4" t="n">
-        <v>41.1</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -838,12 +823,12 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -865,11 +850,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>SLB</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>121.44</v>
+        <v>126.21</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -878,17 +863,17 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>BULLISH</t>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -902,30 +887,27 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>66.8</v>
+        <v>56.3</v>
       </c>
       <c r="J5" t="n">
-        <v>61.3</v>
+        <v>47</v>
       </c>
       <c r="K5" t="n">
-        <v>14</v>
+        <v>3.5</v>
       </c>
       <c r="L5" t="n">
-        <v>2.28</v>
+        <v>10.82</v>
       </c>
       <c r="M5" t="n">
-        <v>22</v>
+        <v>93.8</v>
       </c>
       <c r="N5" t="n">
-        <v>30</v>
+        <v>19.4</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P5" t="n">
-        <v>61</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -934,12 +916,12 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -961,81 +943,75 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BK</t>
+          <t>SNPS</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>241.89</v>
+        <v>126.21</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>BULLISH</t>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>65</v>
+        <v>56.3</v>
       </c>
       <c r="J6" t="n">
-        <v>38.7</v>
+        <v>47</v>
       </c>
       <c r="K6" t="n">
-        <v>93</v>
+        <v>3.5</v>
       </c>
       <c r="L6" t="n">
-        <v>3.48</v>
+        <v>10.82</v>
       </c>
       <c r="M6" t="n">
-        <v>38.7</v>
-      </c>
-      <c r="N6" t="n">
-        <v>80</v>
+        <v>49.8</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P6" t="n">
-        <v>54.8</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
@@ -1043,7 +1019,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr"/>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V6" t="inlineStr">
         <is>
           <t>No</t>
@@ -1053,81 +1033,78 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BA</t>
+          <t>SPG</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>241.89</v>
+        <v>126.21</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>BULLISH</t>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>65</v>
+        <v>56.3</v>
       </c>
       <c r="J7" t="n">
-        <v>38.7</v>
+        <v>47</v>
       </c>
       <c r="K7" t="n">
-        <v>93</v>
+        <v>3.5</v>
       </c>
       <c r="L7" t="n">
-        <v>3.48</v>
+        <v>10.82</v>
       </c>
       <c r="M7" t="n">
-        <v>38.7</v>
+        <v>93.8</v>
       </c>
       <c r="N7" t="n">
-        <v>80</v>
+        <v>19.4</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P7" t="n">
-        <v>54.8</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
@@ -1135,7 +1112,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr"/>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V7" t="inlineStr">
         <is>
           <t>No</t>
@@ -1145,18 +1126,18 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CAT</t>
+          <t>SHW</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>325.14</v>
+        <v>126.21</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
@@ -1168,66 +1149,67 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>63.8</v>
+        <v>56.3</v>
       </c>
       <c r="J8" t="n">
-        <v>62.7</v>
+        <v>47</v>
       </c>
       <c r="K8" t="n">
-        <v>80.2</v>
+        <v>3.5</v>
       </c>
       <c r="L8" t="n">
-        <v>6.62</v>
+        <v>10.82</v>
       </c>
       <c r="M8" t="n">
-        <v>77</v>
+        <v>93.8</v>
       </c>
       <c r="N8" t="n">
-        <v>48.7</v>
+        <v>19.4</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P8" t="n">
-        <v>39.5</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U8" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V8" t="inlineStr">
         <is>
           <t>No</t>
@@ -1237,18 +1219,18 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>TGT</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>126.69</v>
+        <v>126.21</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
@@ -1274,30 +1256,27 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>56.7</v>
+        <v>56.3</v>
       </c>
       <c r="J9" t="n">
-        <v>47.4</v>
+        <v>47</v>
       </c>
       <c r="K9" t="n">
         <v>3.5</v>
       </c>
       <c r="L9" t="n">
-        <v>10.78</v>
+        <v>10.82</v>
       </c>
       <c r="M9" t="n">
-        <v>94</v>
+        <v>93.8</v>
       </c>
       <c r="N9" t="n">
-        <v>19.7</v>
+        <v>19.4</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P9" t="n">
-        <v>43.3</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1333,18 +1312,18 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>LRCX</t>
+          <t>SYK</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>126.69</v>
+        <v>126.21</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
@@ -1370,30 +1349,24 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>56.7</v>
+        <v>56.3</v>
       </c>
       <c r="J10" t="n">
-        <v>47.4</v>
+        <v>47</v>
       </c>
       <c r="K10" t="n">
         <v>3.5</v>
       </c>
       <c r="L10" t="n">
-        <v>10.78</v>
+        <v>10.82</v>
       </c>
       <c r="M10" t="n">
-        <v>94</v>
-      </c>
-      <c r="N10" t="n">
-        <v>19.7</v>
+        <v>34.4</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P10" t="n">
-        <v>43.3</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1429,18 +1402,18 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>MMC</t>
+          <t>SO</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>126.69</v>
+        <v>126.21</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
@@ -1466,30 +1439,27 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>56.7</v>
+        <v>56.3</v>
       </c>
       <c r="J11" t="n">
-        <v>47.4</v>
+        <v>47</v>
       </c>
       <c r="K11" t="n">
         <v>3.5</v>
       </c>
       <c r="L11" t="n">
-        <v>10.78</v>
+        <v>10.82</v>
       </c>
       <c r="M11" t="n">
-        <v>94</v>
+        <v>93.8</v>
       </c>
       <c r="N11" t="n">
-        <v>19.7</v>
+        <v>19.4</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P11" t="n">
-        <v>43.3</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1525,18 +1495,18 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>MMM</t>
+          <t>PCAR</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>126.69</v>
+        <v>126.21</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
@@ -1562,30 +1532,27 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>56.7</v>
+        <v>56.3</v>
       </c>
       <c r="J12" t="n">
-        <v>47.4</v>
+        <v>47</v>
       </c>
       <c r="K12" t="n">
         <v>3.5</v>
       </c>
       <c r="L12" t="n">
-        <v>10.78</v>
+        <v>10.82</v>
       </c>
       <c r="M12" t="n">
-        <v>94</v>
+        <v>93.8</v>
       </c>
       <c r="N12" t="n">
-        <v>19.7</v>
+        <v>19.4</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P12" t="n">
-        <v>43.3</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1621,18 +1588,18 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>MCHP</t>
+          <t>SYY</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>126.69</v>
+        <v>126.21</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
@@ -1658,30 +1625,24 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>56.7</v>
+        <v>56.3</v>
       </c>
       <c r="J13" t="n">
-        <v>47.4</v>
+        <v>47</v>
       </c>
       <c r="K13" t="n">
         <v>3.5</v>
       </c>
       <c r="L13" t="n">
-        <v>10.78</v>
+        <v>10.82</v>
       </c>
       <c r="M13" t="n">
-        <v>94</v>
-      </c>
-      <c r="N13" t="n">
-        <v>19.7</v>
+        <v>33.7</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P13" t="n">
-        <v>43.3</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1717,18 +1678,18 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>MET</t>
+          <t>SRE</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>126.69</v>
+        <v>126.21</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
@@ -1754,30 +1715,27 @@
         </is>
       </c>
       <c r="I14" t="n">
-        <v>56.7</v>
+        <v>56.3</v>
       </c>
       <c r="J14" t="n">
-        <v>47.4</v>
+        <v>47</v>
       </c>
       <c r="K14" t="n">
         <v>3.5</v>
       </c>
       <c r="L14" t="n">
-        <v>10.78</v>
+        <v>10.82</v>
       </c>
       <c r="M14" t="n">
-        <v>94</v>
+        <v>93.8</v>
       </c>
       <c r="N14" t="n">
-        <v>19.7</v>
+        <v>19.4</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P14" t="n">
-        <v>43.3</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1813,18 +1771,18 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>MDLZ</t>
+          <t>SMCI</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>126.69</v>
+        <v>126.21</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
@@ -1850,30 +1808,24 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>56.7</v>
+        <v>56.3</v>
       </c>
       <c r="J15" t="n">
-        <v>47.4</v>
+        <v>47</v>
       </c>
       <c r="K15" t="n">
         <v>3.5</v>
       </c>
       <c r="L15" t="n">
-        <v>10.78</v>
+        <v>10.82</v>
       </c>
       <c r="M15" t="n">
-        <v>94</v>
-      </c>
-      <c r="N15" t="n">
-        <v>19.7</v>
+        <v>80.90000000000001</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P15" t="n">
-        <v>43.3</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1909,18 +1861,18 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>MDT</t>
+          <t>PFE</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>126.69</v>
+        <v>126.21</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
@@ -1946,30 +1898,24 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>56.7</v>
+        <v>56.3</v>
       </c>
       <c r="J16" t="n">
-        <v>47.4</v>
+        <v>47</v>
       </c>
       <c r="K16" t="n">
         <v>3.5</v>
       </c>
       <c r="L16" t="n">
-        <v>10.78</v>
+        <v>10.82</v>
       </c>
       <c r="M16" t="n">
-        <v>94</v>
-      </c>
-      <c r="N16" t="n">
-        <v>19.7</v>
+        <v>25.5</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P16" t="n">
-        <v>43.3</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1997,98 +1943,6 @@
         </is>
       </c>
       <c r="V16" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>GS</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>169.68</v>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Debit Put</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>30-60 DTE</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I17" t="n">
-        <v>30.6</v>
-      </c>
-      <c r="J17" t="n">
-        <v>34</v>
-      </c>
-      <c r="K17" t="n">
-        <v>36</v>
-      </c>
-      <c r="L17" t="n">
-        <v>6.21</v>
-      </c>
-      <c r="M17" t="n">
-        <v>48.8</v>
-      </c>
-      <c r="N17" t="n">
-        <v>42.5</v>
-      </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P17" t="n">
-        <v>51.4</v>
-      </c>
-      <c r="Q17" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R17" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S17" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T17" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U17" t="inlineStr"/>
-      <c r="V17" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Scan 03.04.2026 14:53 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,6 +32,9 @@
     </font>
     <font>
       <color rgb="00ef4444"/>
+    </font>
+    <font>
+      <color rgb="0022c55e"/>
     </font>
   </fonts>
   <fills count="3">
@@ -60,12 +63,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -431,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V16"/>
+  <dimension ref="A1:V17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -573,11 +577,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>QCOM</t>
+          <t>PGR</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>624.34</v>
+        <v>65.76000000000001</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -610,22 +614,22 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>74.09999999999999</v>
+        <v>82.2</v>
       </c>
       <c r="J2" t="n">
-        <v>64.90000000000001</v>
+        <v>60.5</v>
       </c>
       <c r="K2" t="n">
-        <v>94.2</v>
+        <v>90.7</v>
       </c>
       <c r="L2" t="n">
-        <v>5.39</v>
+        <v>5.02</v>
       </c>
       <c r="M2" t="n">
-        <v>56.1</v>
+        <v>55.6</v>
       </c>
       <c r="N2" t="n">
-        <v>60.6</v>
+        <v>99.7</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -633,7 +637,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>45.5</v>
+        <v>46.5</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -642,34 +646,38 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
           <t>Yes</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>No</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>PGR</t>
+          <t>PEP</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>624.34</v>
+        <v>65.76000000000001</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -702,22 +710,22 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>74.09999999999999</v>
+        <v>82.2</v>
       </c>
       <c r="J3" t="n">
-        <v>64.90000000000001</v>
+        <v>60.5</v>
       </c>
       <c r="K3" t="n">
-        <v>94.2</v>
+        <v>90.7</v>
       </c>
       <c r="L3" t="n">
-        <v>5.39</v>
+        <v>5.02</v>
       </c>
       <c r="M3" t="n">
-        <v>56.1</v>
+        <v>55.6</v>
       </c>
       <c r="N3" t="n">
-        <v>60.6</v>
+        <v>99.7</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -725,7 +733,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>31.4</v>
+        <v>46.5</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -734,38 +742,42 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
           <t>Yes</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>No</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TDG</t>
+          <t>CHTR</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>126.21</v>
+        <v>348.47</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -780,45 +792,48 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>56.3</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="J4" t="n">
-        <v>47</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="K4" t="n">
-        <v>3.5</v>
+        <v>80.2</v>
       </c>
       <c r="L4" t="n">
-        <v>10.82</v>
+        <v>10.08</v>
       </c>
       <c r="M4" t="n">
-        <v>93.8</v>
+        <v>91.7</v>
       </c>
       <c r="N4" t="n">
-        <v>19.4</v>
+        <v>56.7</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P4" t="n">
+        <v>38.5</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -828,7 +843,7 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -836,11 +851,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr">
         <is>
           <t>No</t>
@@ -850,15 +861,15 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SLB</t>
+          <t>CEG</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>126.21</v>
+        <v>348.47</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -873,45 +884,48 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>56.3</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="J5" t="n">
-        <v>47</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="K5" t="n">
-        <v>3.5</v>
+        <v>80.2</v>
       </c>
       <c r="L5" t="n">
-        <v>10.82</v>
+        <v>10.08</v>
       </c>
       <c r="M5" t="n">
-        <v>93.8</v>
+        <v>91.7</v>
       </c>
       <c r="N5" t="n">
-        <v>19.4</v>
+        <v>56.7</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P5" t="n">
+        <v>50</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -921,7 +935,7 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -929,11 +943,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr">
         <is>
           <t>No</t>
@@ -943,15 +953,15 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SNPS</t>
+          <t>ACN</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>126.21</v>
+        <v>348.47</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -966,42 +976,48 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>56.3</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="J6" t="n">
-        <v>47</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="K6" t="n">
-        <v>3.5</v>
+        <v>80.2</v>
       </c>
       <c r="L6" t="n">
-        <v>10.82</v>
+        <v>10.08</v>
       </c>
       <c r="M6" t="n">
-        <v>49.8</v>
+        <v>91.7</v>
+      </c>
+      <c r="N6" t="n">
+        <v>56.7</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P6" t="n">
+        <v>38.5</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -1011,7 +1027,7 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
@@ -1019,11 +1035,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U6" t="inlineStr"/>
       <c r="V6" t="inlineStr">
         <is>
           <t>No</t>
@@ -1033,15 +1045,15 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SPG</t>
+          <t>BMY</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>126.21</v>
+        <v>348.47</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -1056,45 +1068,48 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>56.3</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="J7" t="n">
-        <v>47</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="K7" t="n">
-        <v>3.5</v>
+        <v>80.2</v>
       </c>
       <c r="L7" t="n">
-        <v>10.82</v>
+        <v>10.08</v>
       </c>
       <c r="M7" t="n">
-        <v>93.8</v>
+        <v>91.7</v>
       </c>
       <c r="N7" t="n">
-        <v>19.4</v>
+        <v>56.7</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P7" t="n">
+        <v>38.5</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -1104,7 +1119,7 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
@@ -1112,11 +1127,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U7" t="inlineStr"/>
       <c r="V7" t="inlineStr">
         <is>
           <t>No</t>
@@ -1126,15 +1137,15 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SHW</t>
+          <t>TSLA</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>126.21</v>
+        <v>120.45</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -1149,67 +1160,66 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>56.3</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="J8" t="n">
-        <v>47</v>
+        <v>65.3</v>
       </c>
       <c r="K8" t="n">
-        <v>3.5</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="L8" t="n">
-        <v>10.82</v>
+        <v>6.01</v>
       </c>
       <c r="M8" t="n">
-        <v>93.8</v>
+        <v>57</v>
       </c>
       <c r="N8" t="n">
-        <v>19.4</v>
+        <v>22.9</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P8" t="n">
+        <v>52.5</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr">
         <is>
           <t>No</t>
@@ -1219,15 +1229,15 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>TGT</t>
+          <t>TXN</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>126.21</v>
+        <v>120.45</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -1242,67 +1252,66 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>56.3</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="J9" t="n">
-        <v>47</v>
+        <v>65.3</v>
       </c>
       <c r="K9" t="n">
-        <v>3.5</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="L9" t="n">
-        <v>10.82</v>
+        <v>6.01</v>
       </c>
       <c r="M9" t="n">
-        <v>93.8</v>
+        <v>57</v>
       </c>
       <c r="N9" t="n">
-        <v>19.4</v>
+        <v>22.9</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P9" t="n">
+        <v>53.5</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr">
         <is>
           <t>No</t>
@@ -1312,15 +1321,15 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SYK</t>
+          <t>TJX</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>126.21</v>
+        <v>120.45</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -1335,64 +1344,66 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>56.3</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="J10" t="n">
-        <v>47</v>
+        <v>65.3</v>
       </c>
       <c r="K10" t="n">
-        <v>3.5</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="L10" t="n">
-        <v>10.82</v>
+        <v>6.01</v>
       </c>
       <c r="M10" t="n">
-        <v>34.4</v>
+        <v>57</v>
+      </c>
+      <c r="N10" t="n">
+        <v>22.9</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P10" t="n">
+        <v>53.5</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U10" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr"/>
       <c r="V10" t="inlineStr">
         <is>
           <t>No</t>
@@ -1402,15 +1413,15 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SO</t>
+          <t>SRE</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>126.21</v>
+        <v>120.45</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -1425,67 +1436,66 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>56.3</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="J11" t="n">
-        <v>47</v>
+        <v>65.3</v>
       </c>
       <c r="K11" t="n">
-        <v>3.5</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="L11" t="n">
-        <v>10.82</v>
+        <v>6.01</v>
       </c>
       <c r="M11" t="n">
-        <v>93.8</v>
+        <v>57</v>
       </c>
       <c r="N11" t="n">
-        <v>19.4</v>
+        <v>22.9</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P11" t="n">
+        <v>52.5</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U11" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr"/>
       <c r="V11" t="inlineStr">
         <is>
           <t>No</t>
@@ -1495,15 +1505,15 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>PCAR</t>
+          <t>REGN</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>126.21</v>
+        <v>120.45</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -1518,67 +1528,66 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>56.3</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="J12" t="n">
-        <v>47</v>
+        <v>65.3</v>
       </c>
       <c r="K12" t="n">
-        <v>3.5</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="L12" t="n">
-        <v>10.82</v>
+        <v>6.01</v>
       </c>
       <c r="M12" t="n">
-        <v>93.8</v>
+        <v>57</v>
       </c>
       <c r="N12" t="n">
-        <v>19.4</v>
+        <v>22.9</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P12" t="n">
+        <v>53.5</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U12" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr"/>
       <c r="V12" t="inlineStr">
         <is>
           <t>No</t>
@@ -1588,15 +1597,15 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>SYY</t>
+          <t>TMUS</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>126.21</v>
+        <v>120.45</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -1611,64 +1620,66 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>56.3</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="J13" t="n">
-        <v>47</v>
+        <v>65.3</v>
       </c>
       <c r="K13" t="n">
-        <v>3.5</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="L13" t="n">
-        <v>10.82</v>
+        <v>6.01</v>
       </c>
       <c r="M13" t="n">
-        <v>33.7</v>
+        <v>57</v>
+      </c>
+      <c r="N13" t="n">
+        <v>22.9</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P13" t="n">
+        <v>53.5</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U13" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr"/>
       <c r="V13" t="inlineStr">
         <is>
           <t>No</t>
@@ -1678,15 +1689,15 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SRE</t>
+          <t>TDG</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>126.21</v>
+        <v>120.45</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1701,67 +1712,66 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>56.3</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="J14" t="n">
-        <v>47</v>
+        <v>65.3</v>
       </c>
       <c r="K14" t="n">
-        <v>3.5</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="L14" t="n">
-        <v>10.82</v>
+        <v>6.01</v>
       </c>
       <c r="M14" t="n">
-        <v>93.8</v>
+        <v>57</v>
       </c>
       <c r="N14" t="n">
-        <v>19.4</v>
+        <v>22.9</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P14" t="n">
+        <v>53.5</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U14" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr"/>
       <c r="V14" t="inlineStr">
         <is>
           <t>No</t>
@@ -1771,75 +1781,81 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SMCI</t>
+          <t>ANET</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>126.21</v>
+        <v>242.92</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>56.3</v>
+        <v>64</v>
       </c>
       <c r="J15" t="n">
-        <v>47</v>
+        <v>40.1</v>
       </c>
       <c r="K15" t="n">
-        <v>3.5</v>
+        <v>87</v>
       </c>
       <c r="L15" t="n">
-        <v>10.82</v>
+        <v>3.42</v>
       </c>
       <c r="M15" t="n">
-        <v>80.90000000000001</v>
+        <v>38.6</v>
+      </c>
+      <c r="N15" t="n">
+        <v>79.7</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P15" t="n">
+        <v>41.6</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
@@ -1847,11 +1863,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U15" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U15" t="inlineStr"/>
       <c r="V15" t="inlineStr">
         <is>
           <t>No</t>
@@ -1861,88 +1873,186 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>PFE</t>
+          <t>AAPL</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>126.21</v>
+        <v>318.34</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>63.7</v>
+      </c>
+      <c r="J16" t="n">
+        <v>60.8</v>
+      </c>
+      <c r="K16" t="n">
+        <v>80.2</v>
+      </c>
+      <c r="L16" t="n">
+        <v>6.78</v>
+      </c>
+      <c r="M16" t="n">
+        <v>76.09999999999999</v>
+      </c>
+      <c r="N16" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P16" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr"/>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>126.68</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>SELL</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>Debit Put</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="G17" t="inlineStr">
         <is>
           <t>30-60 DTE</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="H17" t="inlineStr">
         <is>
           <t>SQUEEZE</t>
         </is>
       </c>
-      <c r="I16" t="n">
-        <v>56.3</v>
-      </c>
-      <c r="J16" t="n">
-        <v>47</v>
-      </c>
-      <c r="K16" t="n">
+      <c r="I17" t="n">
+        <v>56.7</v>
+      </c>
+      <c r="J17" t="n">
+        <v>47.4</v>
+      </c>
+      <c r="K17" t="n">
         <v>3.5</v>
       </c>
-      <c r="L16" t="n">
-        <v>10.82</v>
-      </c>
-      <c r="M16" t="n">
-        <v>25.5</v>
-      </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="Q16" t="inlineStr">
+      <c r="L17" t="n">
+        <v>10.78</v>
+      </c>
+      <c r="M17" t="n">
+        <v>94</v>
+      </c>
+      <c r="N17" t="n">
+        <v>19.7</v>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P17" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="Q17" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
       </c>
-      <c r="R16" t="inlineStr">
+      <c r="R17" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="S16" t="inlineStr">
+      <c r="S17" t="inlineStr">
         <is>
           <t>red</t>
         </is>
       </c>
-      <c r="T16" t="inlineStr">
+      <c r="T17" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="U16" t="inlineStr">
+      <c r="U17" t="inlineStr">
         <is>
           <t>TTM Squeeze, Squeeze Expanding</t>
         </is>
       </c>
-      <c r="V16" t="inlineStr">
+      <c r="V17" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Scan 06.04.2026 14:57 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V17"/>
+  <dimension ref="A1:V14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -449,7 +449,7 @@
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="6" customWidth="1" min="10" max="10"/>
     <col width="6" customWidth="1" min="11" max="11"/>
-    <col width="7" customWidth="1" min="12" max="12"/>
+    <col width="6" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
     <col width="9" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
@@ -458,7 +458,7 @@
     <col width="15" customWidth="1" min="18" max="18"/>
     <col width="11" customWidth="1" min="19" max="19"/>
     <col width="11" customWidth="1" min="20" max="20"/>
-    <col width="25" customWidth="1" min="21" max="21"/>
+    <col width="13" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
@@ -577,11 +577,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>PGR</t>
+          <t>CPRT</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>65.76000000000001</v>
+        <v>161.3</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,30 +614,30 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>82.2</v>
+        <v>87.59999999999999</v>
       </c>
       <c r="J2" t="n">
-        <v>60.5</v>
+        <v>72.2</v>
       </c>
       <c r="K2" t="n">
-        <v>90.7</v>
+        <v>97.7</v>
       </c>
       <c r="L2" t="n">
-        <v>5.02</v>
+        <v>5.58</v>
       </c>
       <c r="M2" t="n">
-        <v>55.6</v>
+        <v>44.4</v>
       </c>
       <c r="N2" t="n">
-        <v>99.7</v>
+        <v>23.6</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>46.5</v>
+        <v>52</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -659,25 +659,21 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>PEP</t>
+          <t>TXN</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>65.76000000000001</v>
+        <v>161.3</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -710,22 +706,22 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>82.2</v>
+        <v>87.59999999999999</v>
       </c>
       <c r="J3" t="n">
-        <v>60.5</v>
+        <v>72.2</v>
       </c>
       <c r="K3" t="n">
-        <v>90.7</v>
+        <v>97.7</v>
       </c>
       <c r="L3" t="n">
-        <v>5.02</v>
+        <v>5.58</v>
       </c>
       <c r="M3" t="n">
-        <v>55.6</v>
+        <v>44.4</v>
       </c>
       <c r="N3" t="n">
-        <v>99.7</v>
+        <v>23.6</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -733,7 +729,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>46.5</v>
+        <v>44.2</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -755,25 +751,21 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U3" t="inlineStr"/>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CHTR</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>348.47</v>
+        <v>161.3</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -806,22 +798,22 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>69.40000000000001</v>
+        <v>87.59999999999999</v>
       </c>
       <c r="J4" t="n">
-        <v>64.59999999999999</v>
+        <v>72.2</v>
       </c>
       <c r="K4" t="n">
-        <v>80.2</v>
+        <v>97.7</v>
       </c>
       <c r="L4" t="n">
-        <v>10.08</v>
+        <v>5.58</v>
       </c>
       <c r="M4" t="n">
-        <v>91.7</v>
+        <v>44.4</v>
       </c>
       <c r="N4" t="n">
-        <v>56.7</v>
+        <v>23.6</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -829,7 +821,7 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>38.5</v>
+        <v>44.2</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -838,17 +830,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U4" t="inlineStr"/>
@@ -861,11 +853,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CEG</t>
+          <t>BIIB</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>348.47</v>
+        <v>161.3</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -898,30 +890,30 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>69.40000000000001</v>
+        <v>87.59999999999999</v>
       </c>
       <c r="J5" t="n">
-        <v>64.59999999999999</v>
+        <v>72.2</v>
       </c>
       <c r="K5" t="n">
-        <v>80.2</v>
+        <v>97.7</v>
       </c>
       <c r="L5" t="n">
-        <v>10.08</v>
+        <v>5.58</v>
       </c>
       <c r="M5" t="n">
-        <v>91.7</v>
+        <v>44.4</v>
       </c>
       <c r="N5" t="n">
-        <v>56.7</v>
+        <v>23.6</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>50</v>
+        <v>44.2</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -930,17 +922,17 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U5" t="inlineStr"/>
@@ -953,11 +945,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ACN</t>
+          <t>DASH</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>348.47</v>
+        <v>161.3</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -990,22 +982,22 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>69.40000000000001</v>
+        <v>87.59999999999999</v>
       </c>
       <c r="J6" t="n">
-        <v>64.59999999999999</v>
+        <v>72.2</v>
       </c>
       <c r="K6" t="n">
-        <v>80.2</v>
+        <v>97.7</v>
       </c>
       <c r="L6" t="n">
-        <v>10.08</v>
+        <v>5.58</v>
       </c>
       <c r="M6" t="n">
-        <v>91.7</v>
+        <v>44.4</v>
       </c>
       <c r="N6" t="n">
-        <v>56.7</v>
+        <v>23.6</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -1013,7 +1005,7 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>38.5</v>
+        <v>44.2</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1022,17 +1014,17 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
@@ -1045,11 +1037,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BMY</t>
+          <t>CDW</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>348.47</v>
+        <v>161.3</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1082,30 +1074,30 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>69.40000000000001</v>
+        <v>87.59999999999999</v>
       </c>
       <c r="J7" t="n">
-        <v>64.59999999999999</v>
+        <v>72.2</v>
       </c>
       <c r="K7" t="n">
-        <v>80.2</v>
+        <v>97.7</v>
       </c>
       <c r="L7" t="n">
-        <v>10.08</v>
+        <v>5.58</v>
       </c>
       <c r="M7" t="n">
-        <v>91.7</v>
+        <v>44.4</v>
       </c>
       <c r="N7" t="n">
-        <v>56.7</v>
+        <v>23.6</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>38.5</v>
+        <v>52</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1114,17 +1106,17 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U7" t="inlineStr"/>
@@ -1137,30 +1129,30 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>TSLA</t>
+          <t>ABBV</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>120.45</v>
+        <v>207.98</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1170,34 +1162,34 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>66.09999999999999</v>
+        <v>67.2</v>
       </c>
       <c r="J8" t="n">
-        <v>65.3</v>
+        <v>39.2</v>
       </c>
       <c r="K8" t="n">
-        <v>77.90000000000001</v>
+        <v>90</v>
       </c>
       <c r="L8" t="n">
-        <v>6.01</v>
+        <v>2.61</v>
       </c>
       <c r="M8" t="n">
-        <v>57</v>
+        <v>26.5</v>
       </c>
       <c r="N8" t="n">
-        <v>22.9</v>
+        <v>45.3</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>52.5</v>
+        <v>44.2</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1206,12 +1198,12 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
@@ -1229,30 +1221,30 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>TXN</t>
+          <t>ANSS</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>120.45</v>
+        <v>207.98</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1262,34 +1254,34 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>66.09999999999999</v>
+        <v>67.2</v>
       </c>
       <c r="J9" t="n">
-        <v>65.3</v>
+        <v>39.2</v>
       </c>
       <c r="K9" t="n">
-        <v>77.90000000000001</v>
+        <v>90</v>
       </c>
       <c r="L9" t="n">
-        <v>6.01</v>
+        <v>2.61</v>
       </c>
       <c r="M9" t="n">
-        <v>57</v>
+        <v>26.5</v>
       </c>
       <c r="N9" t="n">
-        <v>22.9</v>
+        <v>45.3</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>53.5</v>
+        <v>44.2</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1298,12 +1290,12 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
@@ -1321,30 +1313,30 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>TJX</t>
+          <t>APD</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>120.45</v>
+        <v>207.98</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1354,34 +1346,34 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>66.09999999999999</v>
+        <v>67.2</v>
       </c>
       <c r="J10" t="n">
-        <v>65.3</v>
+        <v>39.2</v>
       </c>
       <c r="K10" t="n">
-        <v>77.90000000000001</v>
+        <v>90</v>
       </c>
       <c r="L10" t="n">
-        <v>6.01</v>
+        <v>2.61</v>
       </c>
       <c r="M10" t="n">
-        <v>57</v>
+        <v>26.5</v>
       </c>
       <c r="N10" t="n">
-        <v>22.9</v>
+        <v>45.3</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>53.5</v>
+        <v>51.8</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1390,12 +1382,12 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -1413,30 +1405,30 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SRE</t>
+          <t>GILD</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>120.45</v>
+        <v>69.94</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1446,34 +1438,34 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>66.09999999999999</v>
+        <v>64.8</v>
       </c>
       <c r="J11" t="n">
+        <v>29.3</v>
+      </c>
+      <c r="K11" t="n">
+        <v>98</v>
+      </c>
+      <c r="L11" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="M11" t="n">
+        <v>57.4</v>
+      </c>
+      <c r="N11" t="n">
         <v>65.3</v>
       </c>
-      <c r="K11" t="n">
-        <v>77.90000000000001</v>
-      </c>
-      <c r="L11" t="n">
-        <v>6.01</v>
-      </c>
-      <c r="M11" t="n">
-        <v>57</v>
-      </c>
-      <c r="N11" t="n">
-        <v>22.9</v>
-      </c>
       <c r="O11" t="inlineStr">
         <is>
           <t>Bullish</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>52.5</v>
+        <v>53.1</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1487,12 +1479,12 @@
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U11" t="inlineStr"/>
@@ -1505,15 +1497,15 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>REGN</t>
+          <t>GD</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>120.45</v>
+        <v>126.75</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -1528,66 +1520,70 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>66.09999999999999</v>
+        <v>64.2</v>
       </c>
       <c r="J12" t="n">
-        <v>65.3</v>
+        <v>47.4</v>
       </c>
       <c r="K12" t="n">
-        <v>77.90000000000001</v>
+        <v>1.2</v>
       </c>
       <c r="L12" t="n">
-        <v>6.01</v>
+        <v>9.640000000000001</v>
       </c>
       <c r="M12" t="n">
-        <v>57</v>
+        <v>93.8</v>
       </c>
       <c r="N12" t="n">
-        <v>22.9</v>
+        <v>19.3</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>53.5</v>
+        <v>38.4</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U12" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
       <c r="V12" t="inlineStr">
         <is>
           <t>No</t>
@@ -1597,15 +1593,15 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TMUS</t>
+          <t>FICO</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>120.45</v>
+        <v>126.75</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -1620,66 +1616,70 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>66.09999999999999</v>
+        <v>64.2</v>
       </c>
       <c r="J13" t="n">
-        <v>65.3</v>
+        <v>47.4</v>
       </c>
       <c r="K13" t="n">
-        <v>77.90000000000001</v>
+        <v>1.2</v>
       </c>
       <c r="L13" t="n">
-        <v>6.01</v>
+        <v>9.640000000000001</v>
       </c>
       <c r="M13" t="n">
-        <v>57</v>
+        <v>93.8</v>
       </c>
       <c r="N13" t="n">
-        <v>22.9</v>
+        <v>19.3</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>53.5</v>
+        <v>38.4</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U13" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
       <c r="V13" t="inlineStr">
         <is>
           <t>No</t>
@@ -1689,11 +1689,11 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>TDG</t>
+          <t>AMP</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>120.45</v>
+        <v>349.06</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -1726,30 +1726,30 @@
         </is>
       </c>
       <c r="I14" t="n">
-        <v>66.09999999999999</v>
+        <v>61.5</v>
       </c>
       <c r="J14" t="n">
-        <v>65.3</v>
+        <v>64.7</v>
       </c>
       <c r="K14" t="n">
-        <v>77.90000000000001</v>
+        <v>76.7</v>
       </c>
       <c r="L14" t="n">
-        <v>6.01</v>
+        <v>9.01</v>
       </c>
       <c r="M14" t="n">
-        <v>57</v>
+        <v>92</v>
       </c>
       <c r="N14" t="n">
-        <v>22.9</v>
+        <v>58</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P14" t="n">
-        <v>53.5</v>
+        <v>44.2</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1758,301 +1758,21 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U14" t="inlineStr"/>
       <c r="V14" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>ANET</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>242.92</v>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I15" t="n">
-        <v>64</v>
-      </c>
-      <c r="J15" t="n">
-        <v>40.1</v>
-      </c>
-      <c r="K15" t="n">
-        <v>87</v>
-      </c>
-      <c r="L15" t="n">
-        <v>3.42</v>
-      </c>
-      <c r="M15" t="n">
-        <v>38.6</v>
-      </c>
-      <c r="N15" t="n">
-        <v>79.7</v>
-      </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P15" t="n">
-        <v>41.6</v>
-      </c>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R15" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="S15" t="inlineStr">
-        <is>
-          <t>maroon</t>
-        </is>
-      </c>
-      <c r="T15" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U15" t="inlineStr"/>
-      <c r="V15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>AAPL</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>318.34</v>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Credit Call</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I16" t="n">
-        <v>63.7</v>
-      </c>
-      <c r="J16" t="n">
-        <v>60.8</v>
-      </c>
-      <c r="K16" t="n">
-        <v>80.2</v>
-      </c>
-      <c r="L16" t="n">
-        <v>6.78</v>
-      </c>
-      <c r="M16" t="n">
-        <v>76.09999999999999</v>
-      </c>
-      <c r="N16" t="n">
-        <v>46.5</v>
-      </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P16" t="n">
-        <v>38.9</v>
-      </c>
-      <c r="Q16" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R16" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S16" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="T16" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U16" t="inlineStr"/>
-      <c r="V16" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>JPM</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>126.68</v>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Debit Put</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>30-60 DTE</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>SQUEEZE</t>
-        </is>
-      </c>
-      <c r="I17" t="n">
-        <v>56.7</v>
-      </c>
-      <c r="J17" t="n">
-        <v>47.4</v>
-      </c>
-      <c r="K17" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="L17" t="n">
-        <v>10.78</v>
-      </c>
-      <c r="M17" t="n">
-        <v>94</v>
-      </c>
-      <c r="N17" t="n">
-        <v>19.7</v>
-      </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P17" t="n">
-        <v>47.2</v>
-      </c>
-      <c r="Q17" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="R17" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S17" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T17" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U17" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
-      <c r="V17" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Scan 07.04.2026 15:19 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V14"/>
+  <dimension ref="A1:V26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -577,11 +577,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CPRT</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>161.3</v>
+        <v>72.55</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,30 +614,27 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>87.59999999999999</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="J2" t="n">
-        <v>72.2</v>
+        <v>62.9</v>
       </c>
       <c r="K2" t="n">
-        <v>97.7</v>
+        <v>87.2</v>
       </c>
       <c r="L2" t="n">
-        <v>5.58</v>
+        <v>6.19</v>
       </c>
       <c r="M2" t="n">
-        <v>44.4</v>
+        <v>60.5</v>
       </c>
       <c r="N2" t="n">
-        <v>23.6</v>
+        <v>55.1</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P2" t="n">
-        <v>52</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -669,11 +666,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>TXN</t>
+          <t>LMT</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>161.3</v>
+        <v>72.55</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -706,30 +703,27 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>87.59999999999999</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="J3" t="n">
-        <v>72.2</v>
+        <v>62.9</v>
       </c>
       <c r="K3" t="n">
-        <v>97.7</v>
+        <v>87.2</v>
       </c>
       <c r="L3" t="n">
-        <v>5.58</v>
+        <v>6.19</v>
       </c>
       <c r="M3" t="n">
-        <v>44.4</v>
+        <v>60.5</v>
       </c>
       <c r="N3" t="n">
-        <v>23.6</v>
+        <v>55.1</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P3" t="n">
-        <v>44.2</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -761,11 +755,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>MCD</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>161.3</v>
+        <v>72.55</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -798,30 +792,27 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>87.59999999999999</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="J4" t="n">
-        <v>72.2</v>
+        <v>62.9</v>
       </c>
       <c r="K4" t="n">
-        <v>97.7</v>
+        <v>87.2</v>
       </c>
       <c r="L4" t="n">
-        <v>5.58</v>
+        <v>6.19</v>
       </c>
       <c r="M4" t="n">
-        <v>44.4</v>
+        <v>60.5</v>
       </c>
       <c r="N4" t="n">
-        <v>23.6</v>
+        <v>55.1</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P4" t="n">
-        <v>44.2</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -853,11 +844,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BIIB</t>
+          <t>APP</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>161.3</v>
+        <v>64.13</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -886,34 +877,34 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>87.59999999999999</v>
+        <v>72.5</v>
       </c>
       <c r="J5" t="n">
-        <v>72.2</v>
+        <v>60.6</v>
       </c>
       <c r="K5" t="n">
-        <v>97.7</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="L5" t="n">
-        <v>5.58</v>
+        <v>4.69</v>
       </c>
       <c r="M5" t="n">
-        <v>44.4</v>
+        <v>55.4</v>
       </c>
       <c r="N5" t="n">
-        <v>23.6</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>44.2</v>
+        <v>38.2</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -945,11 +936,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>DASH</t>
+          <t>ASML</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>161.3</v>
+        <v>64.13</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -978,34 +969,34 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>87.59999999999999</v>
+        <v>72.5</v>
       </c>
       <c r="J6" t="n">
-        <v>72.2</v>
+        <v>60.6</v>
       </c>
       <c r="K6" t="n">
-        <v>97.7</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="L6" t="n">
-        <v>5.58</v>
+        <v>4.69</v>
       </c>
       <c r="M6" t="n">
-        <v>44.4</v>
+        <v>55.4</v>
       </c>
       <c r="N6" t="n">
-        <v>23.6</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P6" t="n">
-        <v>44.2</v>
+        <v>38.2</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1037,11 +1028,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CDW</t>
+          <t>XOM</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>161.3</v>
+        <v>64.13</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1070,34 +1061,34 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>87.59999999999999</v>
+        <v>72.5</v>
       </c>
       <c r="J7" t="n">
-        <v>72.2</v>
+        <v>60.6</v>
       </c>
       <c r="K7" t="n">
-        <v>97.7</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="L7" t="n">
-        <v>5.58</v>
+        <v>4.69</v>
       </c>
       <c r="M7" t="n">
-        <v>44.4</v>
+        <v>55.4</v>
       </c>
       <c r="N7" t="n">
-        <v>23.6</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>52</v>
+        <v>38.2</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1129,30 +1120,30 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ABBV</t>
+          <t>BIIB</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>207.98</v>
+        <v>64.13</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1162,34 +1153,31 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>67.2</v>
+        <v>72.5</v>
       </c>
       <c r="J8" t="n">
-        <v>39.2</v>
+        <v>60.6</v>
       </c>
       <c r="K8" t="n">
-        <v>90</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="L8" t="n">
-        <v>2.61</v>
+        <v>4.69</v>
       </c>
       <c r="M8" t="n">
-        <v>26.5</v>
-      </c>
-      <c r="N8" t="n">
-        <v>45.3</v>
+        <v>51.2</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>44.2</v>
+        <v>38.2</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1198,12 +1186,12 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
@@ -1221,30 +1209,30 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ANSS</t>
+          <t>ZTS</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>207.98</v>
+        <v>64.13</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1254,26 +1242,23 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>67.2</v>
+        <v>72.5</v>
       </c>
       <c r="J9" t="n">
-        <v>39.2</v>
+        <v>60.6</v>
       </c>
       <c r="K9" t="n">
-        <v>90</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="L9" t="n">
-        <v>2.61</v>
+        <v>4.69</v>
       </c>
       <c r="M9" t="n">
-        <v>26.5</v>
-      </c>
-      <c r="N9" t="n">
-        <v>45.3</v>
+        <v>41.3</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1281,7 +1266,7 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>44.2</v>
+        <v>46.5</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1290,12 +1275,12 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
@@ -1313,30 +1298,30 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>APD</t>
+          <t>XEL</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>207.98</v>
+        <v>64.13</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1346,34 +1331,31 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>67.2</v>
+        <v>72.5</v>
       </c>
       <c r="J10" t="n">
-        <v>39.2</v>
+        <v>60.6</v>
       </c>
       <c r="K10" t="n">
-        <v>90</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="L10" t="n">
-        <v>2.61</v>
+        <v>4.69</v>
       </c>
       <c r="M10" t="n">
-        <v>26.5</v>
-      </c>
-      <c r="N10" t="n">
-        <v>45.3</v>
+        <v>27.3</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>51.8</v>
+        <v>38.2</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1382,12 +1364,12 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -1405,81 +1387,81 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>GILD</t>
+          <t>APH</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>69.94</v>
+        <v>129.27</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>64.8</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="J11" t="n">
-        <v>29.3</v>
+        <v>49.2</v>
       </c>
       <c r="K11" t="n">
-        <v>98</v>
+        <v>1.2</v>
       </c>
       <c r="L11" t="n">
-        <v>5.7</v>
+        <v>9.73</v>
       </c>
       <c r="M11" t="n">
-        <v>57.4</v>
+        <v>94</v>
       </c>
       <c r="N11" t="n">
-        <v>65.3</v>
+        <v>19.7</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>53.1</v>
+        <v>43.9</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
@@ -1487,7 +1469,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U11" t="inlineStr"/>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
       <c r="V11" t="inlineStr">
         <is>
           <t>No</t>
@@ -1497,11 +1483,11 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>GD</t>
+          <t>BAC</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>126.75</v>
+        <v>129.27</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1534,30 +1520,30 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>64.2</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="J12" t="n">
-        <v>47.4</v>
+        <v>49.2</v>
       </c>
       <c r="K12" t="n">
         <v>1.2</v>
       </c>
       <c r="L12" t="n">
-        <v>9.640000000000001</v>
+        <v>9.73</v>
       </c>
       <c r="M12" t="n">
-        <v>93.8</v>
+        <v>94</v>
       </c>
       <c r="N12" t="n">
-        <v>19.3</v>
+        <v>19.7</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>38.4</v>
+        <v>57.2</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1593,11 +1579,11 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>FICO</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>126.75</v>
+        <v>129.27</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -1630,22 +1616,22 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>64.2</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="J13" t="n">
-        <v>47.4</v>
+        <v>49.2</v>
       </c>
       <c r="K13" t="n">
         <v>1.2</v>
       </c>
       <c r="L13" t="n">
-        <v>9.640000000000001</v>
+        <v>9.73</v>
       </c>
       <c r="M13" t="n">
-        <v>93.8</v>
+        <v>94</v>
       </c>
       <c r="N13" t="n">
-        <v>19.3</v>
+        <v>19.7</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1653,7 +1639,7 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>38.4</v>
+        <v>43.9</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1689,90 +1675,1235 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>AMP</t>
+          <t>BA</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>349.06</v>
+        <v>129.27</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>64.59999999999999</v>
+      </c>
+      <c r="J14" t="n">
+        <v>49.2</v>
+      </c>
+      <c r="K14" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="L14" t="n">
+        <v>9.73</v>
+      </c>
+      <c r="M14" t="n">
+        <v>94</v>
+      </c>
+      <c r="N14" t="n">
+        <v>19.7</v>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P14" t="n">
+        <v>57.2</v>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>201.88</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>63.8</v>
+      </c>
+      <c r="J15" t="n">
+        <v>33.7</v>
+      </c>
+      <c r="K15" t="n">
+        <v>89</v>
+      </c>
+      <c r="L15" t="n">
+        <v>2.71</v>
+      </c>
+      <c r="M15" t="n">
+        <v>26.3</v>
+      </c>
+      <c r="N15" t="n">
+        <v>44.5</v>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="P15" t="n">
+        <v>40.4</v>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>ADP</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>201.88</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>63.8</v>
+      </c>
+      <c r="J16" t="n">
+        <v>33.7</v>
+      </c>
+      <c r="K16" t="n">
+        <v>89</v>
+      </c>
+      <c r="L16" t="n">
+        <v>2.71</v>
+      </c>
+      <c r="M16" t="n">
+        <v>26.3</v>
+      </c>
+      <c r="N16" t="n">
+        <v>44.5</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P16" t="n">
+        <v>38.6</v>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>ACN</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>201.88</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>63.8</v>
+      </c>
+      <c r="J17" t="n">
+        <v>33.7</v>
+      </c>
+      <c r="K17" t="n">
+        <v>89</v>
+      </c>
+      <c r="L17" t="n">
+        <v>2.71</v>
+      </c>
+      <c r="M17" t="n">
+        <v>26.3</v>
+      </c>
+      <c r="N17" t="n">
+        <v>44.5</v>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P17" t="n">
+        <v>38.6</v>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>201.88</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>63.8</v>
+      </c>
+      <c r="J18" t="n">
+        <v>33.7</v>
+      </c>
+      <c r="K18" t="n">
+        <v>89</v>
+      </c>
+      <c r="L18" t="n">
+        <v>2.71</v>
+      </c>
+      <c r="M18" t="n">
+        <v>26.3</v>
+      </c>
+      <c r="N18" t="n">
+        <v>44.5</v>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="P18" t="n">
+        <v>40.4</v>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>AMGN</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>201.88</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>63.8</v>
+      </c>
+      <c r="J19" t="n">
+        <v>33.7</v>
+      </c>
+      <c r="K19" t="n">
+        <v>89</v>
+      </c>
+      <c r="L19" t="n">
+        <v>2.71</v>
+      </c>
+      <c r="M19" t="n">
+        <v>26.3</v>
+      </c>
+      <c r="N19" t="n">
+        <v>44.5</v>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="P19" t="n">
+        <v>40.4</v>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>ABT</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>201.88</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>63.8</v>
+      </c>
+      <c r="J20" t="n">
+        <v>33.7</v>
+      </c>
+      <c r="K20" t="n">
+        <v>89</v>
+      </c>
+      <c r="L20" t="n">
+        <v>2.71</v>
+      </c>
+      <c r="M20" t="n">
+        <v>26.3</v>
+      </c>
+      <c r="N20" t="n">
+        <v>44.5</v>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="P20" t="n">
+        <v>40.4</v>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>AMAT</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>201.88</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>63.8</v>
+      </c>
+      <c r="J21" t="n">
+        <v>33.7</v>
+      </c>
+      <c r="K21" t="n">
+        <v>89</v>
+      </c>
+      <c r="L21" t="n">
+        <v>2.71</v>
+      </c>
+      <c r="M21" t="n">
+        <v>26.3</v>
+      </c>
+      <c r="N21" t="n">
+        <v>44.5</v>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P21" t="n">
+        <v>38.6</v>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>201.88</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>63.8</v>
+      </c>
+      <c r="J22" t="n">
+        <v>33.7</v>
+      </c>
+      <c r="K22" t="n">
+        <v>89</v>
+      </c>
+      <c r="L22" t="n">
+        <v>2.71</v>
+      </c>
+      <c r="M22" t="n">
+        <v>26.3</v>
+      </c>
+      <c r="N22" t="n">
+        <v>44.5</v>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="P22" t="n">
+        <v>40.4</v>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>ADM</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>201.88</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>63.8</v>
+      </c>
+      <c r="J23" t="n">
+        <v>33.7</v>
+      </c>
+      <c r="K23" t="n">
+        <v>89</v>
+      </c>
+      <c r="L23" t="n">
+        <v>2.71</v>
+      </c>
+      <c r="M23" t="n">
+        <v>26.3</v>
+      </c>
+      <c r="N23" t="n">
+        <v>44.5</v>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P23" t="n">
+        <v>38.6</v>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>AIG</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>201.88</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>63.8</v>
+      </c>
+      <c r="J24" t="n">
+        <v>33.7</v>
+      </c>
+      <c r="K24" t="n">
+        <v>89</v>
+      </c>
+      <c r="L24" t="n">
+        <v>2.71</v>
+      </c>
+      <c r="M24" t="n">
+        <v>36.8</v>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P24" t="n">
+        <v>38.6</v>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>MMC</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>347.93</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>SELL</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F25" t="inlineStr">
         <is>
           <t>Credit Call</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="G25" t="inlineStr">
         <is>
           <t>7-21 DTE</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="H25" t="inlineStr">
         <is>
           <t>NEUTRAL</t>
         </is>
       </c>
-      <c r="I14" t="n">
-        <v>61.5</v>
-      </c>
-      <c r="J14" t="n">
-        <v>64.7</v>
-      </c>
-      <c r="K14" t="n">
+      <c r="I25" t="n">
+        <v>61.8</v>
+      </c>
+      <c r="J25" t="n">
+        <v>64.40000000000001</v>
+      </c>
+      <c r="K25" t="n">
         <v>76.7</v>
       </c>
-      <c r="L14" t="n">
-        <v>9.01</v>
-      </c>
-      <c r="M14" t="n">
-        <v>92</v>
-      </c>
-      <c r="N14" t="n">
-        <v>58</v>
-      </c>
-      <c r="O14" t="inlineStr">
+      <c r="L25" t="n">
+        <v>9.15</v>
+      </c>
+      <c r="M25" t="n">
+        <v>92.09999999999999</v>
+      </c>
+      <c r="N25" t="n">
+        <v>58.3</v>
+      </c>
+      <c r="O25" t="inlineStr">
         <is>
           <t>Bearish</t>
         </is>
       </c>
-      <c r="P14" t="n">
-        <v>44.2</v>
-      </c>
-      <c r="Q14" t="inlineStr">
+      <c r="P25" t="n">
+        <v>35.9</v>
+      </c>
+      <c r="Q25" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>
       </c>
-      <c r="R14" t="inlineStr">
+      <c r="R25" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="S14" t="inlineStr">
+      <c r="S25" t="inlineStr">
         <is>
           <t>green</t>
         </is>
       </c>
-      <c r="T14" t="inlineStr">
+      <c r="T25" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="U14" t="inlineStr"/>
-      <c r="V14" t="inlineStr">
+      <c r="U25" t="inlineStr"/>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>MDT</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>347.93</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>61.8</v>
+      </c>
+      <c r="J26" t="n">
+        <v>64.40000000000001</v>
+      </c>
+      <c r="K26" t="n">
+        <v>76.7</v>
+      </c>
+      <c r="L26" t="n">
+        <v>9.15</v>
+      </c>
+      <c r="M26" t="n">
+        <v>92.09999999999999</v>
+      </c>
+      <c r="N26" t="n">
+        <v>58.3</v>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P26" t="n">
+        <v>62.2</v>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr"/>
+      <c r="V26" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Scan 08.04.2026 15:19 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V26"/>
+  <dimension ref="A1:V39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -449,7 +449,7 @@
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="6" customWidth="1" min="10" max="10"/>
     <col width="6" customWidth="1" min="11" max="11"/>
-    <col width="6" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
     <col width="9" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
@@ -458,7 +458,7 @@
     <col width="15" customWidth="1" min="18" max="18"/>
     <col width="11" customWidth="1" min="19" max="19"/>
     <col width="11" customWidth="1" min="20" max="20"/>
-    <col width="13" customWidth="1" min="21" max="21"/>
+    <col width="19" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
@@ -577,11 +577,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>ZS</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>72.55</v>
+        <v>302.14</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,27 +614,30 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>80.59999999999999</v>
+        <v>79.90000000000001</v>
       </c>
       <c r="J2" t="n">
-        <v>62.9</v>
+        <v>60</v>
       </c>
       <c r="K2" t="n">
-        <v>87.2</v>
+        <v>94.2</v>
       </c>
       <c r="L2" t="n">
-        <v>6.19</v>
+        <v>4.52</v>
       </c>
       <c r="M2" t="n">
-        <v>60.5</v>
+        <v>45</v>
       </c>
       <c r="N2" t="n">
-        <v>55.1</v>
+        <v>100</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P2" t="n">
+        <v>50.3</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -643,34 +646,38 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>LMT</t>
+          <t>ODFL</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>72.55</v>
+        <v>302.14</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -703,27 +710,27 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>80.59999999999999</v>
+        <v>79.90000000000001</v>
       </c>
       <c r="J3" t="n">
-        <v>62.9</v>
+        <v>60</v>
       </c>
       <c r="K3" t="n">
-        <v>87.2</v>
+        <v>94.2</v>
       </c>
       <c r="L3" t="n">
-        <v>6.19</v>
+        <v>4.52</v>
       </c>
       <c r="M3" t="n">
-        <v>60.5</v>
-      </c>
-      <c r="N3" t="n">
-        <v>55.1</v>
+        <v>50</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P3" t="n">
+        <v>50.3</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -732,34 +739,38 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>MCD</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>72.55</v>
+        <v>302.14</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -792,27 +803,27 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>80.59999999999999</v>
+        <v>79.90000000000001</v>
       </c>
       <c r="J4" t="n">
-        <v>62.9</v>
+        <v>60</v>
       </c>
       <c r="K4" t="n">
-        <v>87.2</v>
+        <v>94.2</v>
       </c>
       <c r="L4" t="n">
-        <v>6.19</v>
+        <v>4.52</v>
       </c>
       <c r="M4" t="n">
-        <v>60.5</v>
-      </c>
-      <c r="N4" t="n">
-        <v>55.1</v>
+        <v>17.7</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P4" t="n">
+        <v>50.3</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -821,53 +832,57 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>APP</t>
+          <t>XLF</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>64.13</v>
+        <v>174.27</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -877,26 +892,23 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>72.5</v>
+        <v>76</v>
       </c>
       <c r="J5" t="n">
-        <v>60.6</v>
+        <v>40.1</v>
       </c>
       <c r="K5" t="n">
-        <v>75.59999999999999</v>
+        <v>93</v>
       </c>
       <c r="L5" t="n">
-        <v>4.69</v>
+        <v>3.01</v>
       </c>
       <c r="M5" t="n">
-        <v>55.4</v>
-      </c>
-      <c r="N5" t="n">
-        <v>97.40000000000001</v>
+        <v>21.1</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -904,7 +916,7 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>38.2</v>
+        <v>44.5</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -918,12 +930,12 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U5" t="inlineStr"/>
@@ -936,30 +948,30 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ASML</t>
+          <t>XLK</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>64.13</v>
+        <v>174.27</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -969,26 +981,23 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>72.5</v>
+        <v>76</v>
       </c>
       <c r="J6" t="n">
-        <v>60.6</v>
+        <v>40.1</v>
       </c>
       <c r="K6" t="n">
-        <v>75.59999999999999</v>
+        <v>93</v>
       </c>
       <c r="L6" t="n">
-        <v>4.69</v>
+        <v>3.01</v>
       </c>
       <c r="M6" t="n">
-        <v>55.4</v>
-      </c>
-      <c r="N6" t="n">
-        <v>97.40000000000001</v>
+        <v>28.8</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -996,7 +1005,7 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>38.2</v>
+        <v>44.5</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1010,12 +1019,12 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
@@ -1028,11 +1037,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>XOM</t>
+          <t>EXC</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>64.13</v>
+        <v>384.34</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1065,30 +1074,30 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>72.5</v>
+        <v>70.8</v>
       </c>
       <c r="J7" t="n">
-        <v>60.6</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="K7" t="n">
-        <v>75.59999999999999</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="L7" t="n">
-        <v>4.69</v>
+        <v>9.44</v>
       </c>
       <c r="M7" t="n">
-        <v>55.4</v>
+        <v>94.3</v>
       </c>
       <c r="N7" t="n">
-        <v>97.40000000000001</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>38.2</v>
+        <v>51</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1120,11 +1129,11 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>BIIB</t>
+          <t>FDX</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>64.13</v>
+        <v>384.34</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1157,27 +1166,30 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>72.5</v>
+        <v>70.8</v>
       </c>
       <c r="J8" t="n">
-        <v>60.6</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="K8" t="n">
-        <v>75.59999999999999</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="L8" t="n">
-        <v>4.69</v>
+        <v>9.44</v>
       </c>
       <c r="M8" t="n">
-        <v>51.2</v>
+        <v>94.3</v>
+      </c>
+      <c r="N8" t="n">
+        <v>67.59999999999999</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>38.2</v>
+        <v>55.5</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1209,11 +1221,11 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ZTS</t>
+          <t>GILD</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>64.13</v>
+        <v>384.34</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1246,27 +1258,30 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>72.5</v>
+        <v>70.8</v>
       </c>
       <c r="J9" t="n">
-        <v>60.6</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="K9" t="n">
-        <v>75.59999999999999</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="L9" t="n">
-        <v>4.69</v>
+        <v>9.44</v>
       </c>
       <c r="M9" t="n">
-        <v>41.3</v>
+        <v>94.3</v>
+      </c>
+      <c r="N9" t="n">
+        <v>67.59999999999999</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>46.5</v>
+        <v>51</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1298,11 +1313,11 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>XEL</t>
+          <t>F</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>64.13</v>
+        <v>384.34</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1335,27 +1350,30 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>72.5</v>
+        <v>70.8</v>
       </c>
       <c r="J10" t="n">
-        <v>60.6</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="K10" t="n">
-        <v>75.59999999999999</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="L10" t="n">
-        <v>4.69</v>
+        <v>9.44</v>
       </c>
       <c r="M10" t="n">
-        <v>27.3</v>
+        <v>94.3</v>
+      </c>
+      <c r="N10" t="n">
+        <v>67.59999999999999</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>38.2</v>
+        <v>55.5</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1387,15 +1405,15 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>APH</t>
+          <t>GE</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>129.27</v>
+        <v>384.34</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -1410,36 +1428,36 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>64.59999999999999</v>
+        <v>70.8</v>
       </c>
       <c r="J11" t="n">
-        <v>49.2</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="K11" t="n">
-        <v>1.2</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="L11" t="n">
-        <v>9.73</v>
+        <v>9.44</v>
       </c>
       <c r="M11" t="n">
-        <v>94</v>
+        <v>94.3</v>
       </c>
       <c r="N11" t="n">
-        <v>19.7</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1447,33 +1465,29 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>43.9</v>
+        <v>42.6</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U11" t="inlineStr">
-        <is>
-          <t>TTM Squeeze</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr"/>
       <c r="V11" t="inlineStr">
         <is>
           <t>No</t>
@@ -1483,15 +1497,15 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>BAC</t>
+          <t>GM</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>129.27</v>
+        <v>384.34</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -1506,36 +1520,36 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>64.59999999999999</v>
+        <v>70.8</v>
       </c>
       <c r="J12" t="n">
-        <v>49.2</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="K12" t="n">
-        <v>1.2</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="L12" t="n">
-        <v>9.73</v>
+        <v>9.44</v>
       </c>
       <c r="M12" t="n">
-        <v>94</v>
+        <v>94.3</v>
       </c>
       <c r="N12" t="n">
-        <v>19.7</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1543,33 +1557,29 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>57.2</v>
+        <v>43.7</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U12" t="inlineStr">
-        <is>
-          <t>TTM Squeeze</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr"/>
       <c r="V12" t="inlineStr">
         <is>
           <t>No</t>
@@ -1579,15 +1589,15 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>GD</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>129.27</v>
+        <v>384.34</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -1602,36 +1612,36 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>64.59999999999999</v>
+        <v>70.8</v>
       </c>
       <c r="J13" t="n">
-        <v>49.2</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="K13" t="n">
-        <v>1.2</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="L13" t="n">
-        <v>9.73</v>
+        <v>9.44</v>
       </c>
       <c r="M13" t="n">
-        <v>94</v>
+        <v>94.3</v>
       </c>
       <c r="N13" t="n">
-        <v>19.7</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1639,33 +1649,29 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>43.9</v>
+        <v>42.6</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U13" t="inlineStr">
-        <is>
-          <t>TTM Squeeze</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr"/>
       <c r="V13" t="inlineStr">
         <is>
           <t>No</t>
@@ -1675,15 +1681,15 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>BA</t>
+          <t>FICO</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>129.27</v>
+        <v>384.34</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1698,36 +1704,33 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>64.59999999999999</v>
+        <v>70.8</v>
       </c>
       <c r="J14" t="n">
-        <v>49.2</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="K14" t="n">
-        <v>1.2</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="L14" t="n">
-        <v>9.73</v>
+        <v>9.44</v>
       </c>
       <c r="M14" t="n">
-        <v>94</v>
-      </c>
-      <c r="N14" t="n">
-        <v>19.7</v>
+        <v>61.1</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1735,33 +1738,29 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>57.2</v>
+        <v>63.3</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U14" t="inlineStr">
-        <is>
-          <t>TTM Squeeze</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr"/>
       <c r="V14" t="inlineStr">
         <is>
           <t>No</t>
@@ -1771,30 +1770,30 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ADBE</t>
+          <t>GPN</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>201.88</v>
+        <v>384.34</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1804,34 +1803,34 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>63.8</v>
+        <v>70.8</v>
       </c>
       <c r="J15" t="n">
-        <v>33.7</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="K15" t="n">
-        <v>89</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="L15" t="n">
-        <v>2.71</v>
+        <v>9.44</v>
       </c>
       <c r="M15" t="n">
-        <v>26.3</v>
+        <v>94.3</v>
       </c>
       <c r="N15" t="n">
-        <v>44.5</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P15" t="n">
-        <v>40.4</v>
+        <v>55.5</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1840,12 +1839,12 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
@@ -1853,44 +1852,40 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U15" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U15" t="inlineStr"/>
       <c r="V15" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ADP</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>201.88</v>
+        <v>384.34</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1900,34 +1895,31 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>63.8</v>
+        <v>70.8</v>
       </c>
       <c r="J16" t="n">
-        <v>33.7</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="K16" t="n">
-        <v>89</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="L16" t="n">
-        <v>2.71</v>
+        <v>9.44</v>
       </c>
       <c r="M16" t="n">
-        <v>26.3</v>
-      </c>
-      <c r="N16" t="n">
-        <v>44.5</v>
+        <v>35.8</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>38.6</v>
+        <v>51</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1936,12 +1928,12 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
@@ -1949,25 +1941,21 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U16" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U16" t="inlineStr"/>
       <c r="V16" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ACN</t>
+          <t>AEP</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>201.88</v>
+        <v>209.59</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -2000,30 +1988,30 @@
         </is>
       </c>
       <c r="I17" t="n">
-        <v>63.8</v>
+        <v>65.5</v>
       </c>
       <c r="J17" t="n">
-        <v>33.7</v>
+        <v>42.8</v>
       </c>
       <c r="K17" t="n">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="L17" t="n">
-        <v>2.71</v>
+        <v>2.62</v>
       </c>
       <c r="M17" t="n">
         <v>26.3</v>
       </c>
       <c r="N17" t="n">
-        <v>44.5</v>
+        <v>52.1</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P17" t="n">
-        <v>38.6</v>
+        <v>63.3</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -2032,108 +2020,104 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U17" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr"/>
       <c r="V17" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>201.88</v>
+        <v>142.86</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>63.8</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="J18" t="n">
-        <v>33.7</v>
+        <v>56.9</v>
       </c>
       <c r="K18" t="n">
-        <v>89</v>
+        <v>2.3</v>
       </c>
       <c r="L18" t="n">
-        <v>2.71</v>
+        <v>10.21</v>
       </c>
       <c r="M18" t="n">
-        <v>26.3</v>
+        <v>101</v>
       </c>
       <c r="N18" t="n">
-        <v>44.5</v>
+        <v>30.7</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P18" t="n">
-        <v>40.4</v>
+        <v>24.7</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
@@ -2143,93 +2127,93 @@
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>Divergence</t>
+          <t>TTM Squeeze</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>BKNG</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>201.88</v>
+        <v>142.86</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>63.8</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="J19" t="n">
-        <v>33.7</v>
+        <v>56.9</v>
       </c>
       <c r="K19" t="n">
-        <v>89</v>
+        <v>2.3</v>
       </c>
       <c r="L19" t="n">
-        <v>2.71</v>
+        <v>10.21</v>
       </c>
       <c r="M19" t="n">
-        <v>26.3</v>
+        <v>101</v>
       </c>
       <c r="N19" t="n">
-        <v>44.5</v>
+        <v>30.7</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P19" t="n">
-        <v>40.4</v>
+        <v>24.7</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
@@ -2239,93 +2223,93 @@
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>Divergence</t>
+          <t>TTM Squeeze</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ABT</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>201.88</v>
+        <v>142.86</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I20" t="n">
-        <v>63.8</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="J20" t="n">
-        <v>33.7</v>
+        <v>56.9</v>
       </c>
       <c r="K20" t="n">
-        <v>89</v>
+        <v>2.3</v>
       </c>
       <c r="L20" t="n">
-        <v>2.71</v>
+        <v>10.21</v>
       </c>
       <c r="M20" t="n">
-        <v>26.3</v>
+        <v>101</v>
       </c>
       <c r="N20" t="n">
-        <v>44.5</v>
+        <v>30.7</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P20" t="n">
-        <v>40.4</v>
+        <v>24.7</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
@@ -2335,71 +2319,71 @@
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>Divergence</t>
+          <t>TTM Squeeze</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>AMAT</t>
+          <t>BLK</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>201.88</v>
+        <v>142.86</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>63.8</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="J21" t="n">
-        <v>33.7</v>
+        <v>56.9</v>
       </c>
       <c r="K21" t="n">
-        <v>89</v>
+        <v>2.3</v>
       </c>
       <c r="L21" t="n">
-        <v>2.71</v>
+        <v>10.21</v>
       </c>
       <c r="M21" t="n">
-        <v>26.3</v>
+        <v>101</v>
       </c>
       <c r="N21" t="n">
-        <v>44.5</v>
+        <v>30.7</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
@@ -2407,21 +2391,21 @@
         </is>
       </c>
       <c r="P21" t="n">
-        <v>38.6</v>
+        <v>24.7</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
@@ -2431,93 +2415,93 @@
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>Divergence</t>
+          <t>TTM Squeeze</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ALL</t>
+          <t>CCI</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>201.88</v>
+        <v>142.86</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I22" t="n">
-        <v>63.8</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="J22" t="n">
-        <v>33.7</v>
+        <v>56.9</v>
       </c>
       <c r="K22" t="n">
-        <v>89</v>
+        <v>2.3</v>
       </c>
       <c r="L22" t="n">
-        <v>2.71</v>
+        <v>10.21</v>
       </c>
       <c r="M22" t="n">
-        <v>26.3</v>
+        <v>101</v>
       </c>
       <c r="N22" t="n">
-        <v>44.5</v>
+        <v>30.7</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P22" t="n">
-        <v>40.4</v>
+        <v>24.7</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
@@ -2527,71 +2511,71 @@
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>Divergence</t>
+          <t>TTM Squeeze</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ADM</t>
+          <t>CDNS</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>201.88</v>
+        <v>142.86</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I23" t="n">
-        <v>63.8</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="J23" t="n">
-        <v>33.7</v>
+        <v>56.9</v>
       </c>
       <c r="K23" t="n">
-        <v>89</v>
+        <v>2.3</v>
       </c>
       <c r="L23" t="n">
-        <v>2.71</v>
+        <v>10.21</v>
       </c>
       <c r="M23" t="n">
-        <v>26.3</v>
+        <v>101</v>
       </c>
       <c r="N23" t="n">
-        <v>44.5</v>
+        <v>30.7</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -2599,21 +2583,21 @@
         </is>
       </c>
       <c r="P23" t="n">
-        <v>38.6</v>
+        <v>24.7</v>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
@@ -2623,68 +2607,71 @@
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>Divergence</t>
+          <t>TTM Squeeze</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>AIG</t>
+          <t>C</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>201.88</v>
+        <v>142.86</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I24" t="n">
-        <v>63.8</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="J24" t="n">
-        <v>33.7</v>
+        <v>56.9</v>
       </c>
       <c r="K24" t="n">
-        <v>89</v>
+        <v>2.3</v>
       </c>
       <c r="L24" t="n">
-        <v>2.71</v>
+        <v>10.21</v>
       </c>
       <c r="M24" t="n">
-        <v>36.8</v>
+        <v>101</v>
+      </c>
+      <c r="N24" t="n">
+        <v>30.7</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
@@ -2692,21 +2679,21 @@
         </is>
       </c>
       <c r="P24" t="n">
-        <v>38.6</v>
+        <v>24.7</v>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
@@ -2716,27 +2703,27 @@
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>Divergence</t>
+          <t>TTM Squeeze</t>
         </is>
       </c>
       <c r="V24" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>MMC</t>
+          <t>CAT</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>347.93</v>
+        <v>142.86</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -2751,36 +2738,36 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I25" t="n">
-        <v>61.8</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="J25" t="n">
-        <v>64.40000000000001</v>
+        <v>56.9</v>
       </c>
       <c r="K25" t="n">
-        <v>76.7</v>
+        <v>2.3</v>
       </c>
       <c r="L25" t="n">
-        <v>9.15</v>
+        <v>10.21</v>
       </c>
       <c r="M25" t="n">
-        <v>92.09999999999999</v>
+        <v>101</v>
       </c>
       <c r="N25" t="n">
-        <v>58.3</v>
+        <v>30.7</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
@@ -2788,29 +2775,33 @@
         </is>
       </c>
       <c r="P25" t="n">
-        <v>35.9</v>
+        <v>24.7</v>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U25" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
       <c r="V25" t="inlineStr">
         <is>
           <t>No</t>
@@ -2820,92 +2811,1314 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>MDT</t>
+          <t>BDX</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>347.93</v>
+        <v>142.86</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>65.40000000000001</v>
+      </c>
+      <c r="J26" t="n">
+        <v>56.9</v>
+      </c>
+      <c r="K26" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="L26" t="n">
+        <v>10.21</v>
+      </c>
+      <c r="M26" t="n">
+        <v>101</v>
+      </c>
+      <c r="N26" t="n">
+        <v>30.7</v>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P26" t="n">
+        <v>24.7</v>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>MCO</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>347.23</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Debit Call</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>61.3</v>
+      </c>
+      <c r="J27" t="n">
+        <v>56.1</v>
+      </c>
+      <c r="K27" t="n">
+        <v>18.6</v>
+      </c>
+      <c r="L27" t="n">
+        <v>8.960000000000001</v>
+      </c>
+      <c r="M27" t="n">
+        <v>88.8</v>
+      </c>
+      <c r="N27" t="n">
+        <v>24</v>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P27" t="n">
+        <v>54</v>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>MRK</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>347.23</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Debit Call</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>61.3</v>
+      </c>
+      <c r="J28" t="n">
+        <v>56.1</v>
+      </c>
+      <c r="K28" t="n">
+        <v>18.6</v>
+      </c>
+      <c r="L28" t="n">
+        <v>8.960000000000001</v>
+      </c>
+      <c r="M28" t="n">
+        <v>88.8</v>
+      </c>
+      <c r="N28" t="n">
+        <v>24</v>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P28" t="n">
+        <v>54</v>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>TDG</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>121.28</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="E29" t="inlineStr">
         <is>
           <t>SELL</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="F29" t="inlineStr">
         <is>
           <t>Credit Call</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
+      <c r="G29" t="inlineStr">
         <is>
           <t>7-21 DTE</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
+      <c r="H29" t="inlineStr">
         <is>
           <t>NEUTRAL</t>
         </is>
       </c>
-      <c r="I26" t="n">
-        <v>61.8</v>
-      </c>
-      <c r="J26" t="n">
+      <c r="I29" t="n">
+        <v>61.3</v>
+      </c>
+      <c r="J29" t="n">
+        <v>66</v>
+      </c>
+      <c r="K29" t="n">
+        <v>74.40000000000001</v>
+      </c>
+      <c r="L29" t="n">
+        <v>5.69</v>
+      </c>
+      <c r="M29" t="n">
+        <v>55.5</v>
+      </c>
+      <c r="N29" t="n">
+        <v>18.7</v>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P29" t="n">
+        <v>56.6</v>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr"/>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>URI</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>121.28</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>61.3</v>
+      </c>
+      <c r="J30" t="n">
+        <v>66</v>
+      </c>
+      <c r="K30" t="n">
+        <v>74.40000000000001</v>
+      </c>
+      <c r="L30" t="n">
+        <v>5.69</v>
+      </c>
+      <c r="M30" t="n">
+        <v>45.4</v>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P30" t="n">
+        <v>58.7</v>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr"/>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>VLO</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>121.28</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>61.3</v>
+      </c>
+      <c r="J31" t="n">
+        <v>66</v>
+      </c>
+      <c r="K31" t="n">
+        <v>74.40000000000001</v>
+      </c>
+      <c r="L31" t="n">
+        <v>5.69</v>
+      </c>
+      <c r="M31" t="n">
+        <v>55.5</v>
+      </c>
+      <c r="N31" t="n">
+        <v>18.7</v>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P31" t="n">
+        <v>58.7</v>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr"/>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>DDOG</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>123.57</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>53.2</v>
+      </c>
+      <c r="J32" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="K32" t="n">
+        <v>76</v>
+      </c>
+      <c r="L32" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="M32" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="N32" t="n">
+        <v>41.6</v>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>DXCM</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>123.57</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>53.2</v>
+      </c>
+      <c r="J33" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="K33" t="n">
+        <v>76</v>
+      </c>
+      <c r="L33" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="M33" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="N33" t="n">
+        <v>41.6</v>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P33" t="n">
+        <v>64.2</v>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>CTSH</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>123.57</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>53.2</v>
+      </c>
+      <c r="J34" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="K34" t="n">
+        <v>76</v>
+      </c>
+      <c r="L34" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="M34" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="N34" t="n">
+        <v>41.6</v>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>CPRT</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>123.57</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>53.2</v>
+      </c>
+      <c r="J35" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="K35" t="n">
+        <v>76</v>
+      </c>
+      <c r="L35" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="M35" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="N35" t="n">
+        <v>41.6</v>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>DLTR</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>123.57</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>53.2</v>
+      </c>
+      <c r="J36" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="K36" t="n">
+        <v>76</v>
+      </c>
+      <c r="L36" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="M36" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="N36" t="n">
+        <v>41.6</v>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P36" t="n">
+        <v>64.2</v>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>123.57</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>53.2</v>
+      </c>
+      <c r="J37" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="K37" t="n">
+        <v>76</v>
+      </c>
+      <c r="L37" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="M37" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="N37" t="n">
+        <v>41.6</v>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P37" t="n">
         <v>64.40000000000001</v>
       </c>
-      <c r="K26" t="n">
-        <v>76.7</v>
-      </c>
-      <c r="L26" t="n">
-        <v>9.15</v>
-      </c>
-      <c r="M26" t="n">
-        <v>92.09999999999999</v>
-      </c>
-      <c r="N26" t="n">
-        <v>58.3</v>
-      </c>
-      <c r="O26" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P26" t="n">
-        <v>62.2</v>
-      </c>
-      <c r="Q26" t="inlineStr">
+      <c r="Q37" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>
       </c>
-      <c r="R26" t="inlineStr">
+      <c r="R37" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="S26" t="inlineStr">
+      <c r="S37" t="inlineStr">
         <is>
           <t>green</t>
         </is>
       </c>
-      <c r="T26" t="inlineStr">
+      <c r="T37" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="U26" t="inlineStr"/>
-      <c r="V26" t="inlineStr">
-        <is>
-          <t>No</t>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V37" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>CDW</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>123.57</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>53.2</v>
+      </c>
+      <c r="J38" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="K38" t="n">
+        <v>76</v>
+      </c>
+      <c r="L38" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="M38" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="N38" t="n">
+        <v>41.6</v>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>123.57</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>53.2</v>
+      </c>
+      <c r="J39" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="K39" t="n">
+        <v>76</v>
+      </c>
+      <c r="L39" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="M39" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="N39" t="n">
+        <v>41.6</v>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan 10.04.2026 14:56 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V21"/>
+  <dimension ref="A1:V19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -445,7 +445,7 @@
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="6" customWidth="1" min="10" max="10"/>
     <col width="6" customWidth="1" min="11" max="11"/>
@@ -458,7 +458,7 @@
     <col width="15" customWidth="1" min="18" max="18"/>
     <col width="11" customWidth="1" min="19" max="19"/>
     <col width="11" customWidth="1" min="20" max="20"/>
-    <col width="13" customWidth="1" min="21" max="21"/>
+    <col width="25" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
@@ -577,11 +577,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CDW</t>
+          <t>LRCX</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>64.61</v>
+        <v>234.9</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -610,26 +610,26 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>73.5</v>
+        <v>74</v>
       </c>
       <c r="J2" t="n">
-        <v>62</v>
+        <v>62.6</v>
       </c>
       <c r="K2" t="n">
-        <v>75.59999999999999</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="L2" t="n">
         <v>4.71</v>
       </c>
       <c r="M2" t="n">
-        <v>55.2</v>
+        <v>46.8</v>
       </c>
       <c r="N2" t="n">
-        <v>96.5</v>
+        <v>26.4</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>64</v>
+        <v>71.7</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -669,11 +669,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>APP</t>
+          <t>MCK</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>64.61</v>
+        <v>234.9</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -702,26 +702,26 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>73.5</v>
+        <v>74</v>
       </c>
       <c r="J3" t="n">
-        <v>62</v>
+        <v>62.6</v>
       </c>
       <c r="K3" t="n">
-        <v>75.59999999999999</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="L3" t="n">
         <v>4.71</v>
       </c>
       <c r="M3" t="n">
-        <v>55.2</v>
+        <v>46.8</v>
       </c>
       <c r="N3" t="n">
-        <v>96.5</v>
+        <v>26.4</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -729,7 +729,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>64</v>
+        <v>71.7</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -761,11 +761,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BIIB</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>64.61</v>
+        <v>402.83</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -798,30 +798,30 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>73.5</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="J4" t="n">
-        <v>62</v>
+        <v>72.7</v>
       </c>
       <c r="K4" t="n">
-        <v>75.59999999999999</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="L4" t="n">
-        <v>4.71</v>
+        <v>9.6</v>
       </c>
       <c r="M4" t="n">
-        <v>55.2</v>
+        <v>99</v>
       </c>
       <c r="N4" t="n">
-        <v>96.5</v>
+        <v>87.59999999999999</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P4" t="n">
-        <v>45.7</v>
+        <v>29.1</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -853,11 +853,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>UPS</t>
+          <t>ADSK</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>64.61</v>
+        <v>402.83</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -890,27 +890,30 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>73.5</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="J5" t="n">
-        <v>62</v>
+        <v>72.7</v>
       </c>
       <c r="K5" t="n">
-        <v>75.59999999999999</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="L5" t="n">
-        <v>4.71</v>
+        <v>9.6</v>
       </c>
       <c r="M5" t="n">
-        <v>42.2</v>
+        <v>99</v>
+      </c>
+      <c r="N5" t="n">
+        <v>87.59999999999999</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>40.2</v>
+        <v>29.1</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -942,68 +945,68 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ASML</t>
+          <t>PGR</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>64.61</v>
+        <v>188.49</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>73.5</v>
+        <v>67</v>
       </c>
       <c r="J6" t="n">
-        <v>62</v>
+        <v>56.1</v>
       </c>
       <c r="K6" t="n">
-        <v>75.59999999999999</v>
+        <v>12.8</v>
       </c>
       <c r="L6" t="n">
-        <v>4.71</v>
+        <v>7.39</v>
       </c>
       <c r="M6" t="n">
-        <v>52.3</v>
+        <v>62.3</v>
+      </c>
+      <c r="N6" t="n">
+        <v>6.7</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Neutral</t>
-        </is>
-      </c>
-      <c r="P6" t="n">
-        <v>40.2</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -1013,15 +1016,19 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V6" t="inlineStr">
         <is>
           <t>No</t>
@@ -1031,71 +1038,68 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CPRT</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>64.61</v>
+        <v>188.49</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>73.5</v>
+        <v>67</v>
       </c>
       <c r="J7" t="n">
-        <v>62</v>
+        <v>56.1</v>
       </c>
       <c r="K7" t="n">
-        <v>75.59999999999999</v>
+        <v>12.8</v>
       </c>
       <c r="L7" t="n">
-        <v>4.71</v>
+        <v>7.39</v>
       </c>
       <c r="M7" t="n">
-        <v>55.2</v>
+        <v>62.3</v>
       </c>
       <c r="N7" t="n">
-        <v>96.5</v>
+        <v>6.7</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P7" t="n">
-        <v>64</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -1105,15 +1109,19 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U7" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V7" t="inlineStr">
         <is>
           <t>No</t>
@@ -1123,71 +1131,68 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ABNB</t>
+          <t>PFE</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>64.61</v>
+        <v>188.49</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>73.5</v>
+        <v>67</v>
       </c>
       <c r="J8" t="n">
-        <v>62</v>
+        <v>56.1</v>
       </c>
       <c r="K8" t="n">
-        <v>75.59999999999999</v>
+        <v>12.8</v>
       </c>
       <c r="L8" t="n">
-        <v>4.71</v>
+        <v>7.39</v>
       </c>
       <c r="M8" t="n">
-        <v>55.2</v>
+        <v>62.3</v>
       </c>
       <c r="N8" t="n">
-        <v>96.5</v>
+        <v>6.7</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Neutral</t>
-        </is>
-      </c>
-      <c r="P8" t="n">
-        <v>40.2</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
@@ -1197,15 +1202,19 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U8" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V8" t="inlineStr">
         <is>
           <t>No</t>
@@ -1215,59 +1224,59 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>WBA</t>
+          <t>NSC</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>392.91</v>
+        <v>188.49</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>72.09999999999999</v>
+        <v>67</v>
       </c>
       <c r="J9" t="n">
-        <v>71.5</v>
+        <v>56.1</v>
       </c>
       <c r="K9" t="n">
-        <v>77.90000000000001</v>
+        <v>12.8</v>
       </c>
       <c r="L9" t="n">
-        <v>9.460000000000001</v>
+        <v>7.39</v>
       </c>
       <c r="M9" t="n">
-        <v>96.2</v>
+        <v>62.3</v>
       </c>
       <c r="N9" t="n">
-        <v>75.7</v>
+        <v>6.7</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1275,11 +1284,11 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>62</v>
+        <v>63.3</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -1289,15 +1298,19 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U9" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V9" t="inlineStr">
         <is>
           <t>No</t>
@@ -1307,59 +1320,59 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>URI</t>
+          <t>OXY</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>392.91</v>
+        <v>188.49</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>72.09999999999999</v>
+        <v>67</v>
       </c>
       <c r="J10" t="n">
-        <v>71.5</v>
+        <v>56.1</v>
       </c>
       <c r="K10" t="n">
-        <v>77.90000000000001</v>
+        <v>12.8</v>
       </c>
       <c r="L10" t="n">
-        <v>9.460000000000001</v>
+        <v>7.39</v>
       </c>
       <c r="M10" t="n">
-        <v>96.2</v>
+        <v>62.3</v>
       </c>
       <c r="N10" t="n">
-        <v>75.7</v>
+        <v>6.7</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1367,11 +1380,11 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>62</v>
+        <v>55.7</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
@@ -1381,15 +1394,19 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U10" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V10" t="inlineStr">
         <is>
           <t>No</t>
@@ -1399,71 +1416,68 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>TT</t>
+          <t>PSA</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>392.91</v>
+        <v>188.49</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>72.09999999999999</v>
+        <v>67</v>
       </c>
       <c r="J11" t="n">
-        <v>71.5</v>
+        <v>56.1</v>
       </c>
       <c r="K11" t="n">
-        <v>77.90000000000001</v>
+        <v>12.8</v>
       </c>
       <c r="L11" t="n">
-        <v>9.460000000000001</v>
+        <v>7.39</v>
       </c>
       <c r="M11" t="n">
-        <v>96.2</v>
+        <v>62.3</v>
       </c>
       <c r="N11" t="n">
-        <v>75.7</v>
+        <v>6.7</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P11" t="n">
-        <v>62</v>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
@@ -1473,15 +1487,19 @@
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U11" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V11" t="inlineStr">
         <is>
           <t>No</t>
@@ -1491,71 +1509,71 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>VZ</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>392.91</v>
+        <v>188.49</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>72.09999999999999</v>
+        <v>67</v>
       </c>
       <c r="J12" t="n">
-        <v>71.5</v>
+        <v>56.1</v>
       </c>
       <c r="K12" t="n">
-        <v>77.90000000000001</v>
+        <v>12.8</v>
       </c>
       <c r="L12" t="n">
-        <v>9.460000000000001</v>
+        <v>7.39</v>
       </c>
       <c r="M12" t="n">
-        <v>96.2</v>
+        <v>62.3</v>
       </c>
       <c r="N12" t="n">
-        <v>75.7</v>
+        <v>6.7</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>62</v>
+        <v>51</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
@@ -1565,15 +1583,19 @@
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U12" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V12" t="inlineStr">
         <is>
           <t>No</t>
@@ -1583,71 +1605,71 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TXN</t>
+          <t>NKE</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>392.91</v>
+        <v>188.49</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>72.09999999999999</v>
+        <v>67</v>
       </c>
       <c r="J13" t="n">
-        <v>71.5</v>
+        <v>56.1</v>
       </c>
       <c r="K13" t="n">
-        <v>77.90000000000001</v>
+        <v>12.8</v>
       </c>
       <c r="L13" t="n">
-        <v>9.460000000000001</v>
+        <v>7.39</v>
       </c>
       <c r="M13" t="n">
-        <v>96.2</v>
+        <v>62.3</v>
       </c>
       <c r="N13" t="n">
-        <v>75.7</v>
+        <v>6.7</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>45.7</v>
+        <v>60.3</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
@@ -1657,15 +1679,19 @@
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U13" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V13" t="inlineStr">
         <is>
           <t>No</t>
@@ -1675,15 +1701,15 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>WMT</t>
+          <t>V</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>392.91</v>
+        <v>146.45</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1698,48 +1724,48 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>72.09999999999999</v>
+        <v>65.2</v>
       </c>
       <c r="J14" t="n">
-        <v>71.5</v>
+        <v>58.6</v>
       </c>
       <c r="K14" t="n">
-        <v>77.90000000000001</v>
+        <v>3.5</v>
       </c>
       <c r="L14" t="n">
-        <v>9.460000000000001</v>
+        <v>10.23</v>
       </c>
       <c r="M14" t="n">
-        <v>96.2</v>
+        <v>104.3</v>
       </c>
       <c r="N14" t="n">
-        <v>75.7</v>
+        <v>35.9</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P14" t="n">
-        <v>64</v>
+        <v>47.1</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
@@ -1757,7 +1783,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U14" t="inlineStr"/>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
       <c r="V14" t="inlineStr">
         <is>
           <t>No</t>
@@ -1767,11 +1797,11 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>HSY</t>
+          <t>UPS</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>142.88</v>
+        <v>146.45</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1804,22 +1834,22 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>65.09999999999999</v>
+        <v>65.2</v>
       </c>
       <c r="J15" t="n">
-        <v>56.9</v>
+        <v>58.6</v>
       </c>
       <c r="K15" t="n">
-        <v>2.3</v>
+        <v>3.5</v>
       </c>
       <c r="L15" t="n">
-        <v>10.24</v>
+        <v>10.23</v>
       </c>
       <c r="M15" t="n">
-        <v>101</v>
+        <v>104.3</v>
       </c>
       <c r="N15" t="n">
-        <v>30.7</v>
+        <v>35.9</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1827,7 +1857,7 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>40.5</v>
+        <v>47.1</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1841,7 +1871,7 @@
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
@@ -1863,11 +1893,11 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>URI</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>142.88</v>
+        <v>146.45</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -1900,22 +1930,22 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>65.09999999999999</v>
+        <v>65.2</v>
       </c>
       <c r="J16" t="n">
-        <v>56.9</v>
+        <v>58.6</v>
       </c>
       <c r="K16" t="n">
-        <v>2.3</v>
+        <v>3.5</v>
       </c>
       <c r="L16" t="n">
-        <v>10.24</v>
+        <v>10.23</v>
       </c>
       <c r="M16" t="n">
-        <v>101</v>
+        <v>104.3</v>
       </c>
       <c r="N16" t="n">
-        <v>30.7</v>
+        <v>35.9</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -1923,7 +1953,7 @@
         </is>
       </c>
       <c r="P16" t="n">
-        <v>40.5</v>
+        <v>47.1</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1937,7 +1967,7 @@
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
@@ -1959,59 +1989,59 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ANET</t>
+          <t>VLO</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>211.2</v>
+        <v>146.45</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>62.9</v>
+        <v>65.2</v>
       </c>
       <c r="J17" t="n">
-        <v>45.1</v>
+        <v>58.6</v>
       </c>
       <c r="K17" t="n">
-        <v>76</v>
+        <v>3.5</v>
       </c>
       <c r="L17" t="n">
-        <v>2.55</v>
+        <v>10.23</v>
       </c>
       <c r="M17" t="n">
-        <v>27</v>
+        <v>104.3</v>
       </c>
       <c r="N17" t="n">
-        <v>57.1</v>
+        <v>35.9</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -2019,11 +2049,11 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>36.4</v>
+        <v>49.7</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
@@ -2033,15 +2063,19 @@
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U17" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
       <c r="V17" t="inlineStr">
         <is>
           <t>No</t>
@@ -2051,71 +2085,71 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ADSK</t>
+          <t>TXN</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>211.2</v>
+        <v>146.45</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>62.9</v>
+        <v>65.2</v>
       </c>
       <c r="J18" t="n">
-        <v>45.1</v>
+        <v>58.6</v>
       </c>
       <c r="K18" t="n">
-        <v>76</v>
+        <v>3.5</v>
       </c>
       <c r="L18" t="n">
-        <v>2.55</v>
+        <v>10.23</v>
       </c>
       <c r="M18" t="n">
-        <v>27</v>
+        <v>104.3</v>
       </c>
       <c r="N18" t="n">
-        <v>57.1</v>
+        <v>35.9</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P18" t="n">
-        <v>51.8</v>
+        <v>47.1</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
@@ -2125,15 +2159,19 @@
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U18" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
       <c r="V18" t="inlineStr">
         <is>
           <t>No</t>
@@ -2143,71 +2181,71 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>TSN</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>211.2</v>
+        <v>146.45</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>62.9</v>
+        <v>65.2</v>
       </c>
       <c r="J19" t="n">
-        <v>45.1</v>
+        <v>58.6</v>
       </c>
       <c r="K19" t="n">
-        <v>76</v>
+        <v>3.5</v>
       </c>
       <c r="L19" t="n">
-        <v>2.55</v>
+        <v>10.23</v>
       </c>
       <c r="M19" t="n">
-        <v>27</v>
+        <v>104.3</v>
       </c>
       <c r="N19" t="n">
-        <v>57.1</v>
+        <v>35.9</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P19" t="n">
-        <v>67.2</v>
+        <v>47.1</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
@@ -2217,200 +2255,20 @@
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U19" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
       <c r="V19" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>AON</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>211.2</v>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I20" t="n">
-        <v>62.9</v>
-      </c>
-      <c r="J20" t="n">
-        <v>45.1</v>
-      </c>
-      <c r="K20" t="n">
-        <v>76</v>
-      </c>
-      <c r="L20" t="n">
-        <v>2.55</v>
-      </c>
-      <c r="M20" t="n">
-        <v>27</v>
-      </c>
-      <c r="N20" t="n">
-        <v>57.1</v>
-      </c>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P20" t="n">
-        <v>36.4</v>
-      </c>
-      <c r="Q20" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R20" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="S20" t="inlineStr">
-        <is>
-          <t>maroon</t>
-        </is>
-      </c>
-      <c r="T20" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U20" t="inlineStr"/>
-      <c r="V20" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>AMGN</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>211.2</v>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I21" t="n">
-        <v>62.9</v>
-      </c>
-      <c r="J21" t="n">
-        <v>45.1</v>
-      </c>
-      <c r="K21" t="n">
-        <v>76</v>
-      </c>
-      <c r="L21" t="n">
-        <v>2.55</v>
-      </c>
-      <c r="M21" t="n">
-        <v>27</v>
-      </c>
-      <c r="N21" t="n">
-        <v>57.1</v>
-      </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P21" t="n">
-        <v>31.3</v>
-      </c>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="S21" t="inlineStr">
-        <is>
-          <t>maroon</t>
-        </is>
-      </c>
-      <c r="T21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U21" t="inlineStr"/>
-      <c r="V21" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Scan 14.04.2026 15:20 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,6 +29,9 @@
       <b val="1"/>
       <color rgb="00f1f5f9"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <color rgb="0022c55e"/>
     </font>
     <font>
       <color rgb="00ef4444"/>
@@ -60,12 +63,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -431,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V8"/>
+  <dimension ref="A1:V4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -454,7 +458,7 @@
     <col width="15" customWidth="1" min="18" max="18"/>
     <col width="11" customWidth="1" min="19" max="19"/>
     <col width="11" customWidth="1" min="20" max="20"/>
-    <col width="25" customWidth="1" min="21" max="21"/>
+    <col width="13" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
@@ -573,11 +577,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>GILD</t>
+          <t>SYY</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>600.64</v>
+        <v>73.64</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -586,17 +590,17 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>BEARISH</t>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -610,22 +614,19 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>72.2</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="J2" t="n">
-        <v>62.2</v>
+        <v>37.9</v>
       </c>
       <c r="K2" t="n">
-        <v>90.7</v>
+        <v>93</v>
       </c>
       <c r="L2" t="n">
-        <v>6.04</v>
+        <v>3.01</v>
       </c>
       <c r="M2" t="n">
-        <v>62.5</v>
-      </c>
-      <c r="N2" t="n">
-        <v>68.8</v>
+        <v>30.7</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -633,7 +634,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>26.9</v>
+        <v>42.8</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -647,12 +648,12 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
@@ -665,18 +666,18 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>INTC</t>
+          <t>IDXX</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>600.64</v>
+        <v>582.0599999999999</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
@@ -688,36 +689,36 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>72.2</v>
+        <v>70.8</v>
       </c>
       <c r="J3" t="n">
-        <v>62.2</v>
+        <v>48.3</v>
       </c>
       <c r="K3" t="n">
-        <v>90.7</v>
+        <v>3</v>
       </c>
       <c r="L3" t="n">
-        <v>6.04</v>
+        <v>3</v>
       </c>
       <c r="M3" t="n">
-        <v>62.5</v>
+        <v>30.3</v>
       </c>
       <c r="N3" t="n">
-        <v>68.8</v>
+        <v>22.8</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -725,11 +726,11 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>26.9</v>
+        <v>42.3</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -739,7 +740,7 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -747,7 +748,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr"/>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
       <c r="V3" t="inlineStr">
         <is>
           <t>No</t>
@@ -757,11 +762,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>GPN</t>
+          <t>EL</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>600.64</v>
+        <v>75.01000000000001</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -770,17 +775,17 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>BEARISH</t>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -790,26 +795,26 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>72.2</v>
+        <v>70.3</v>
       </c>
       <c r="J4" t="n">
-        <v>62.2</v>
+        <v>41.9</v>
       </c>
       <c r="K4" t="n">
-        <v>90.7</v>
+        <v>78</v>
       </c>
       <c r="L4" t="n">
-        <v>6.04</v>
+        <v>4.6</v>
       </c>
       <c r="M4" t="n">
-        <v>62.5</v>
+        <v>57.3</v>
       </c>
       <c r="N4" t="n">
-        <v>68.8</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -817,7 +822,7 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>26.9</v>
+        <v>38.4</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -831,388 +836,16 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>HSY</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>600.64</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Credit Call</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I5" t="n">
-        <v>72.2</v>
-      </c>
-      <c r="J5" t="n">
-        <v>62.2</v>
-      </c>
-      <c r="K5" t="n">
-        <v>90.7</v>
-      </c>
-      <c r="L5" t="n">
-        <v>6.04</v>
-      </c>
-      <c r="M5" t="n">
-        <v>62.5</v>
-      </c>
-      <c r="N5" t="n">
-        <v>68.8</v>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P5" t="n">
-        <v>26.9</v>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>lime</t>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr"/>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>HD</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>600.64</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Credit Call</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I6" t="n">
-        <v>72.2</v>
-      </c>
-      <c r="J6" t="n">
-        <v>62.2</v>
-      </c>
-      <c r="K6" t="n">
-        <v>90.7</v>
-      </c>
-      <c r="L6" t="n">
-        <v>6.04</v>
-      </c>
-      <c r="M6" t="n">
-        <v>62.5</v>
-      </c>
-      <c r="N6" t="n">
-        <v>68.8</v>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P6" t="n">
-        <v>58</v>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>lime</t>
-        </is>
-      </c>
-      <c r="T6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr"/>
-      <c r="V6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>JNJ</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>600.64</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Credit Call</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I7" t="n">
-        <v>72.2</v>
-      </c>
-      <c r="J7" t="n">
-        <v>62.2</v>
-      </c>
-      <c r="K7" t="n">
-        <v>90.7</v>
-      </c>
-      <c r="L7" t="n">
-        <v>6.04</v>
-      </c>
-      <c r="M7" t="n">
-        <v>62.5</v>
-      </c>
-      <c r="N7" t="n">
-        <v>68.8</v>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P7" t="n">
-        <v>26.9</v>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="S7" t="inlineStr">
-        <is>
-          <t>lime</t>
-        </is>
-      </c>
-      <c r="T7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U7" t="inlineStr"/>
-      <c r="V7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>MAR</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>76.73</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Debit Put</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>30-60 DTE</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>SQUEEZE</t>
-        </is>
-      </c>
-      <c r="I8" t="n">
-        <v>51.6</v>
-      </c>
-      <c r="J8" t="n">
-        <v>43.2</v>
-      </c>
-      <c r="K8" t="n">
-        <v>18.6</v>
-      </c>
-      <c r="L8" t="n">
-        <v>7.42</v>
-      </c>
-      <c r="M8" t="n">
-        <v>64.2</v>
-      </c>
-      <c r="N8" t="n">
-        <v>8.4</v>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P8" t="n">
-        <v>59.1</v>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S8" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
-      <c r="V8" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Scan 15.04.2026 15:14 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -31,10 +31,10 @@
       <sz val="11"/>
     </font>
     <font>
-      <color rgb="0022c55e"/>
+      <color rgb="00ef4444"/>
     </font>
     <font>
-      <color rgb="00ef4444"/>
+      <color rgb="0022c55e"/>
     </font>
   </fonts>
   <fills count="3">
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V4"/>
+  <dimension ref="A1:V7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -458,7 +458,7 @@
     <col width="15" customWidth="1" min="18" max="18"/>
     <col width="11" customWidth="1" min="19" max="19"/>
     <col width="11" customWidth="1" min="20" max="20"/>
-    <col width="13" customWidth="1" min="21" max="21"/>
+    <col width="19" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
@@ -577,11 +577,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SYY</t>
+          <t>MU</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>73.64</v>
+        <v>452.87</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -590,17 +590,17 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>BULLISH</t>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -614,27 +614,30 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>72.09999999999999</v>
+        <v>77.09999999999999</v>
       </c>
       <c r="J2" t="n">
-        <v>37.9</v>
+        <v>62.2</v>
       </c>
       <c r="K2" t="n">
+        <v>82</v>
+      </c>
+      <c r="L2" t="n">
+        <v>5.77</v>
+      </c>
+      <c r="M2" t="n">
+        <v>77.2</v>
+      </c>
+      <c r="N2" t="n">
         <v>93</v>
       </c>
-      <c r="L2" t="n">
-        <v>3.01</v>
-      </c>
-      <c r="M2" t="n">
-        <v>30.7</v>
-      </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>42.8</v>
+        <v>67.8</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -648,12 +651,12 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
@@ -666,59 +669,59 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>IDXX</t>
+          <t>SYY</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>582.0599999999999</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>BEARISH</t>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>70.8</v>
+        <v>73.7</v>
       </c>
       <c r="J3" t="n">
-        <v>48.3</v>
+        <v>40.6</v>
       </c>
       <c r="K3" t="n">
-        <v>3</v>
+        <v>92</v>
       </c>
       <c r="L3" t="n">
-        <v>3</v>
+        <v>2.82</v>
       </c>
       <c r="M3" t="n">
-        <v>30.3</v>
+        <v>49.2</v>
       </c>
       <c r="N3" t="n">
-        <v>22.8</v>
+        <v>98</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -726,11 +729,11 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>42.3</v>
+        <v>44</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -745,14 +748,10 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>TTM Squeeze</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr"/>
       <c r="V3" t="inlineStr">
         <is>
           <t>No</t>
@@ -762,18 +761,18 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>EL</t>
+          <t>NKE</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>75.01000000000001</v>
+        <v>45.61</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
@@ -795,26 +794,26 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>70.3</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="J4" t="n">
-        <v>41.9</v>
+        <v>36.8</v>
       </c>
       <c r="K4" t="n">
-        <v>78</v>
+        <v>98</v>
       </c>
       <c r="L4" t="n">
-        <v>4.6</v>
+        <v>3.62</v>
       </c>
       <c r="M4" t="n">
-        <v>57.3</v>
+        <v>52.3</v>
       </c>
       <c r="N4" t="n">
-        <v>65.09999999999999</v>
+        <v>90.2</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -822,7 +821,7 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>38.4</v>
+        <v>32.3</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -846,6 +845,284 @@
       </c>
       <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>BSX</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>64.61</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>69</v>
+      </c>
+      <c r="J5" t="n">
+        <v>42</v>
+      </c>
+      <c r="K5" t="n">
+        <v>79</v>
+      </c>
+      <c r="L5" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="M5" t="n">
+        <v>41.8</v>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P5" t="n">
+        <v>29.2</v>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr"/>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>REGN</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>746.38</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>68.8</v>
+      </c>
+      <c r="J6" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="K6" t="n">
+        <v>13</v>
+      </c>
+      <c r="L6" t="n">
+        <v>2.53</v>
+      </c>
+      <c r="M6" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="N6" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P6" t="n">
+        <v>53.5</v>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>CHTR</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>221.12</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>52.3</v>
+      </c>
+      <c r="J7" t="n">
+        <v>50.7</v>
+      </c>
+      <c r="K7" t="n">
+        <v>16</v>
+      </c>
+      <c r="L7" t="n">
+        <v>3.97</v>
+      </c>
+      <c r="M7" t="n">
+        <v>59.8</v>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P7" t="n">
+        <v>44.8</v>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Scan 16.04.2026 15:47 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -458,7 +458,7 @@
     <col width="15" customWidth="1" min="18" max="18"/>
     <col width="11" customWidth="1" min="19" max="19"/>
     <col width="11" customWidth="1" min="20" max="20"/>
-    <col width="19" customWidth="1" min="21" max="21"/>
+    <col width="25" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
@@ -581,7 +581,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>452.87</v>
+        <v>459.77</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,22 +614,19 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>77.09999999999999</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="J2" t="n">
-        <v>62.2</v>
+        <v>63.8</v>
       </c>
       <c r="K2" t="n">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="L2" t="n">
-        <v>5.77</v>
+        <v>5.56</v>
       </c>
       <c r="M2" t="n">
-        <v>77.2</v>
-      </c>
-      <c r="N2" t="n">
-        <v>93</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -637,7 +634,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>67.8</v>
+        <v>68.5</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -669,11 +666,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SYY</t>
+          <t>NKE</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>74.40000000000001</v>
+        <v>46.38</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -706,22 +703,22 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>73.7</v>
+        <v>74.2</v>
       </c>
       <c r="J3" t="n">
-        <v>40.6</v>
+        <v>40.1</v>
       </c>
       <c r="K3" t="n">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="L3" t="n">
-        <v>2.82</v>
+        <v>3.44</v>
       </c>
       <c r="M3" t="n">
-        <v>49.2</v>
+        <v>52.7</v>
       </c>
       <c r="N3" t="n">
-        <v>98</v>
+        <v>91.3</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -729,7 +726,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>44</v>
+        <v>33.6</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -761,59 +758,59 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>NKE</t>
+          <t>MDT</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>45.61</v>
+        <v>86.42</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>71.40000000000001</v>
+        <v>73.7</v>
       </c>
       <c r="J4" t="n">
-        <v>36.8</v>
+        <v>40.9</v>
       </c>
       <c r="K4" t="n">
-        <v>98</v>
+        <v>6</v>
       </c>
       <c r="L4" t="n">
-        <v>3.62</v>
+        <v>1.86</v>
       </c>
       <c r="M4" t="n">
-        <v>52.3</v>
+        <v>18.9</v>
       </c>
       <c r="N4" t="n">
-        <v>90.2</v>
+        <v>60.3</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -821,7 +818,7 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>32.3</v>
+        <v>38.5</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -840,24 +837,28 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
           <t>Yes</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr"/>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t>No</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BSX</t>
+          <t>SYY</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>64.61</v>
+        <v>73.8</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -886,23 +887,23 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>69</v>
+        <v>72.8</v>
       </c>
       <c r="J5" t="n">
-        <v>42</v>
+        <v>38.7</v>
       </c>
       <c r="K5" t="n">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="L5" t="n">
-        <v>2.75</v>
+        <v>2.74</v>
       </c>
       <c r="M5" t="n">
-        <v>41.8</v>
+        <v>30</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -910,7 +911,7 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>29.2</v>
+        <v>43</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -942,67 +943,67 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>REGN</t>
+          <t>BSX</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>746.38</v>
+        <v>64.34999999999999</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>68.8</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="J6" t="n">
-        <v>45.5</v>
+        <v>41.2</v>
       </c>
       <c r="K6" t="n">
-        <v>13</v>
+        <v>76</v>
       </c>
       <c r="L6" t="n">
-        <v>2.53</v>
+        <v>2.71</v>
       </c>
       <c r="M6" t="n">
-        <v>27.3</v>
+        <v>34.2</v>
       </c>
       <c r="N6" t="n">
-        <v>8.199999999999999</v>
+        <v>45.2</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P6" t="n">
-        <v>53.5</v>
+        <v>28.8</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1011,24 +1012,20 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr"/>
       <c r="V6" t="inlineStr">
         <is>
           <t>No</t>
@@ -1042,7 +1039,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>221.12</v>
+        <v>228.57</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1075,19 +1072,19 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>52.3</v>
+        <v>54.1</v>
       </c>
       <c r="J7" t="n">
-        <v>50.7</v>
+        <v>56.9</v>
       </c>
       <c r="K7" t="n">
         <v>16</v>
       </c>
       <c r="L7" t="n">
-        <v>3.97</v>
+        <v>3.92</v>
       </c>
       <c r="M7" t="n">
-        <v>59.8</v>
+        <v>60.3</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1095,7 +1092,7 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>44.8</v>
+        <v>48.5</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1109,7 +1106,7 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">

</xml_diff>

<commit_message>
Scan 17.04.2026 15:04 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -31,10 +31,10 @@
       <sz val="11"/>
     </font>
     <font>
-      <color rgb="00ef4444"/>
+      <color rgb="0022c55e"/>
     </font>
     <font>
-      <color rgb="0022c55e"/>
+      <color rgb="00ef4444"/>
     </font>
   </fonts>
   <fills count="3">
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V7"/>
+  <dimension ref="A1:V10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -577,56 +577,56 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>BDX</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>459.77</v>
+        <v>159.25</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>BEARISH</t>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>74.40000000000001</v>
+        <v>80.7</v>
       </c>
       <c r="J2" t="n">
-        <v>63.8</v>
+        <v>52.7</v>
       </c>
       <c r="K2" t="n">
-        <v>81</v>
+        <v>3</v>
       </c>
       <c r="L2" t="n">
-        <v>5.56</v>
+        <v>1.98</v>
       </c>
       <c r="M2" t="n">
-        <v>72.59999999999999</v>
+        <v>36.1</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -634,11 +634,11 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>68.5</v>
+        <v>51.8</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -648,15 +648,19 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V2" t="inlineStr">
         <is>
           <t>No</t>
@@ -666,18 +670,18 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>NKE</t>
+          <t>SYY</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>46.38</v>
+        <v>75.76000000000001</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
@@ -703,22 +707,19 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>74.2</v>
+        <v>77.3</v>
       </c>
       <c r="J3" t="n">
-        <v>40.1</v>
+        <v>45.8</v>
       </c>
       <c r="K3" t="n">
-        <v>96</v>
+        <v>87</v>
       </c>
       <c r="L3" t="n">
-        <v>3.44</v>
+        <v>2.69</v>
       </c>
       <c r="M3" t="n">
-        <v>52.7</v>
-      </c>
-      <c r="N3" t="n">
-        <v>91.3</v>
+        <v>30.5</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -726,7 +727,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>33.6</v>
+        <v>46</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -758,11 +759,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>MDT</t>
+          <t>CMCSA</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>86.42</v>
+        <v>29.7</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -771,17 +772,17 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>BEARISH</t>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -791,34 +792,34 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>73.7</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="J4" t="n">
-        <v>40.9</v>
+        <v>60.8</v>
       </c>
       <c r="K4" t="n">
-        <v>6</v>
+        <v>31</v>
       </c>
       <c r="L4" t="n">
-        <v>1.86</v>
+        <v>2.27</v>
       </c>
       <c r="M4" t="n">
-        <v>18.9</v>
+        <v>25.1</v>
       </c>
       <c r="N4" t="n">
-        <v>60.3</v>
+        <v>69.5</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P4" t="n">
-        <v>38.5</v>
+        <v>54.6</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -840,32 +841,28 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SYY</t>
+          <t>NKE</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>73.8</v>
+        <v>46.15</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
@@ -891,19 +888,22 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>72.8</v>
+        <v>74.7</v>
       </c>
       <c r="J5" t="n">
-        <v>38.7</v>
+        <v>39.3</v>
       </c>
       <c r="K5" t="n">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="L5" t="n">
-        <v>2.74</v>
+        <v>3.31</v>
       </c>
       <c r="M5" t="n">
-        <v>30</v>
+        <v>52.4</v>
+      </c>
+      <c r="N5" t="n">
+        <v>90.5</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -911,7 +911,7 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>43</v>
+        <v>33.2</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -943,11 +943,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BSX</t>
+          <t>MU</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>64.34999999999999</v>
+        <v>459.92</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -956,17 +956,17 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>BULLISH</t>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -976,34 +976,31 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>68.90000000000001</v>
+        <v>73.7</v>
       </c>
       <c r="J6" t="n">
-        <v>41.2</v>
+        <v>63.9</v>
       </c>
       <c r="K6" t="n">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="L6" t="n">
-        <v>2.71</v>
+        <v>5.31</v>
       </c>
       <c r="M6" t="n">
-        <v>34.2</v>
-      </c>
-      <c r="N6" t="n">
-        <v>45.2</v>
+        <v>70.7</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P6" t="n">
-        <v>28.8</v>
+        <v>68.5</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1017,12 +1014,12 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
@@ -1035,11 +1032,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CHTR</t>
+          <t>IDXX</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>228.57</v>
+        <v>591.62</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1048,80 +1045,371 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Debit Call</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>72.3</v>
+      </c>
+      <c r="J7" t="n">
+        <v>52.7</v>
+      </c>
+      <c r="K7" t="n">
+        <v>10</v>
+      </c>
+      <c r="L7" t="n">
+        <v>2.92</v>
+      </c>
+      <c r="M7" t="n">
+        <v>29.7</v>
+      </c>
+      <c r="N7" t="n">
+        <v>22</v>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P7" t="n">
+        <v>44.2</v>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>FIRED</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>Squeeze Fired, Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>147.3</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Debit Call</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>71.7</v>
+      </c>
+      <c r="J8" t="n">
+        <v>52.2</v>
+      </c>
+      <c r="K8" t="n">
+        <v>8</v>
+      </c>
+      <c r="L8" t="n">
+        <v>1.77</v>
+      </c>
+      <c r="M8" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="N8" t="n">
+        <v>68.8</v>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P8" t="n">
+        <v>47</v>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>MDT</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>86.95</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
           <t>BEARISH</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>SELL</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>Debit Put</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>30-60 DTE</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>SQUEEZE</t>
         </is>
       </c>
-      <c r="I7" t="n">
-        <v>54.1</v>
-      </c>
-      <c r="J7" t="n">
-        <v>56.9</v>
-      </c>
-      <c r="K7" t="n">
-        <v>16</v>
-      </c>
-      <c r="L7" t="n">
-        <v>3.92</v>
-      </c>
-      <c r="M7" t="n">
-        <v>60.3</v>
-      </c>
-      <c r="O7" t="inlineStr">
+      <c r="I9" t="n">
+        <v>70.2</v>
+      </c>
+      <c r="J9" t="n">
+        <v>44.8</v>
+      </c>
+      <c r="K9" t="n">
+        <v>7</v>
+      </c>
+      <c r="L9" t="n">
+        <v>1.89</v>
+      </c>
+      <c r="M9" t="n">
+        <v>18.6</v>
+      </c>
+      <c r="N9" t="n">
+        <v>57.8</v>
+      </c>
+      <c r="O9" t="inlineStr">
         <is>
           <t>Bearish</t>
         </is>
       </c>
-      <c r="P7" t="n">
-        <v>48.5</v>
-      </c>
-      <c r="Q7" t="inlineStr">
+      <c r="P9" t="n">
+        <v>39.4</v>
+      </c>
+      <c r="Q9" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
       </c>
-      <c r="R7" t="inlineStr">
+      <c r="R9" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
       </c>
-      <c r="S7" t="inlineStr">
-        <is>
-          <t>lime</t>
-        </is>
-      </c>
-      <c r="T7" t="inlineStr">
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr">
+      <c r="U9" t="inlineStr">
         <is>
           <t>TTM Squeeze</t>
         </is>
       </c>
-      <c r="V7" t="inlineStr">
+      <c r="V9" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>LIN</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>489.13</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>57.3</v>
+      </c>
+      <c r="J10" t="n">
+        <v>46</v>
+      </c>
+      <c r="K10" t="n">
+        <v>11</v>
+      </c>
+      <c r="L10" t="n">
+        <v>1.98</v>
+      </c>
+      <c r="M10" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="N10" t="n">
+        <v>70.09999999999999</v>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P10" t="n">
+        <v>58.3</v>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan 20.04.2026 15:23 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V10"/>
+  <dimension ref="A1:V13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -577,15 +577,15 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BDX</t>
+          <t>SYY</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>159.25</v>
+        <v>76.66</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -600,45 +600,45 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>80.7</v>
+        <v>81.2</v>
       </c>
       <c r="J2" t="n">
-        <v>52.7</v>
+        <v>48.7</v>
       </c>
       <c r="K2" t="n">
-        <v>3</v>
+        <v>85</v>
       </c>
       <c r="L2" t="n">
-        <v>1.98</v>
+        <v>2.54</v>
       </c>
       <c r="M2" t="n">
-        <v>36.1</v>
+        <v>27.5</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>51.8</v>
+        <v>47.2</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -656,11 +656,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr">
         <is>
           <t>No</t>
@@ -670,15 +666,15 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SYY</t>
+          <t>CMCSA</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>75.76000000000001</v>
+        <v>30.02</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -693,41 +689,41 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>77.3</v>
+        <v>79.3</v>
       </c>
       <c r="J3" t="n">
-        <v>45.8</v>
+        <v>63.6</v>
       </c>
       <c r="K3" t="n">
-        <v>87</v>
+        <v>39</v>
       </c>
       <c r="L3" t="n">
-        <v>2.69</v>
+        <v>2.19</v>
       </c>
       <c r="M3" t="n">
-        <v>30.5</v>
+        <v>39.9</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P3" t="n">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -746,7 +742,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U3" t="inlineStr"/>
@@ -759,59 +755,59 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CMCSA</t>
+          <t>BAC</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>29.7</v>
+        <v>53.58</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>76.59999999999999</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="J4" t="n">
-        <v>60.8</v>
+        <v>65.7</v>
       </c>
       <c r="K4" t="n">
-        <v>31</v>
+        <v>98</v>
       </c>
       <c r="L4" t="n">
-        <v>2.27</v>
+        <v>2.18</v>
       </c>
       <c r="M4" t="n">
-        <v>25.1</v>
+        <v>22.7</v>
       </c>
       <c r="N4" t="n">
-        <v>69.5</v>
+        <v>56.3</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -819,7 +815,7 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>54.6</v>
+        <v>56.7</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -833,7 +829,7 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -851,59 +847,59 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>NKE</t>
+          <t>IDXX</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>46.15</v>
+        <v>582.22</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>74.7</v>
+        <v>76.2</v>
       </c>
       <c r="J5" t="n">
-        <v>39.3</v>
+        <v>49</v>
       </c>
       <c r="K5" t="n">
-        <v>95</v>
+        <v>11</v>
       </c>
       <c r="L5" t="n">
-        <v>3.31</v>
+        <v>2.8</v>
       </c>
       <c r="M5" t="n">
-        <v>52.4</v>
+        <v>29</v>
       </c>
       <c r="N5" t="n">
-        <v>90.5</v>
+        <v>21.1</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -911,11 +907,11 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>33.2</v>
+        <v>42.6</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>FIRED</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -930,10 +926,14 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>Squeeze Fired, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V5" t="inlineStr">
         <is>
           <t>No</t>
@@ -943,11 +943,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>FCX</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>459.92</v>
+        <v>70.34</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -980,19 +980,19 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>73.7</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="J6" t="n">
-        <v>63.9</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="K6" t="n">
-        <v>84</v>
+        <v>97</v>
       </c>
       <c r="L6" t="n">
-        <v>5.31</v>
+        <v>3.26</v>
       </c>
       <c r="M6" t="n">
-        <v>70.7</v>
+        <v>50.8</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -1000,7 +1000,7 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>68.5</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1032,71 +1032,71 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>IDXX</t>
+          <t>INTC</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>591.62</v>
+        <v>66.05</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>72.3</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="J7" t="n">
-        <v>52.7</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="K7" t="n">
-        <v>10</v>
+        <v>99</v>
       </c>
       <c r="L7" t="n">
-        <v>2.92</v>
+        <v>5.06</v>
       </c>
       <c r="M7" t="n">
-        <v>29.7</v>
+        <v>70.2</v>
       </c>
       <c r="N7" t="n">
-        <v>22</v>
+        <v>60.8</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>44.2</v>
+        <v>73.3</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>FIRED</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -1106,89 +1106,89 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
           <t>Yes</t>
-        </is>
-      </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>Squeeze Fired, Squeeze Expanding</t>
-        </is>
-      </c>
-      <c r="V7" t="inlineStr">
-        <is>
-          <t>No</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PG</t>
+          <t>MU</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>147.3</v>
+        <v>443.2</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>71.7</v>
+        <v>73.8</v>
       </c>
       <c r="J8" t="n">
-        <v>52.2</v>
+        <v>58.6</v>
       </c>
       <c r="K8" t="n">
-        <v>8</v>
+        <v>87</v>
       </c>
       <c r="L8" t="n">
-        <v>1.77</v>
+        <v>5.64</v>
       </c>
       <c r="M8" t="n">
-        <v>19.8</v>
+        <v>73</v>
       </c>
       <c r="N8" t="n">
-        <v>68.8</v>
+        <v>84.3</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>47</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1202,7 +1202,7 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
@@ -1212,12 +1212,12 @@
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>Squeeze Expanding</t>
+          <t>Divergence</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1228,7 +1228,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>86.95</v>
+        <v>86.67</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1261,22 +1261,22 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>70.2</v>
+        <v>72</v>
       </c>
       <c r="J9" t="n">
-        <v>44.8</v>
+        <v>43.7</v>
       </c>
       <c r="K9" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="L9" t="n">
-        <v>1.89</v>
+        <v>1.83</v>
       </c>
       <c r="M9" t="n">
-        <v>18.6</v>
+        <v>17.1</v>
       </c>
       <c r="N9" t="n">
-        <v>57.8</v>
+        <v>44.4</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1320,94 +1320,370 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>LIN</t>
+          <t>NKE</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>489.13</v>
+        <v>46.09</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>71.5</v>
+      </c>
+      <c r="J10" t="n">
+        <v>39</v>
+      </c>
+      <c r="K10" t="n">
+        <v>93</v>
+      </c>
+      <c r="L10" t="n">
+        <v>3.02</v>
+      </c>
+      <c r="M10" t="n">
+        <v>52.3</v>
+      </c>
+      <c r="N10" t="n">
+        <v>90.2</v>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P10" t="n">
+        <v>33.1</v>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr"/>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>CAT</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>795.3200000000001</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>70.90000000000001</v>
+      </c>
+      <c r="J11" t="n">
+        <v>64.7</v>
+      </c>
+      <c r="K11" t="n">
+        <v>86</v>
+      </c>
+      <c r="L11" t="n">
+        <v>2.86</v>
+      </c>
+      <c r="M11" t="n">
+        <v>37.9</v>
+      </c>
+      <c r="N11" t="n">
+        <v>71.2</v>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P11" t="n">
+        <v>72.59999999999999</v>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr"/>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>PCAR</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>127.91</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>70.90000000000001</v>
+      </c>
+      <c r="J12" t="n">
+        <v>65.3</v>
+      </c>
+      <c r="K12" t="n">
+        <v>88</v>
+      </c>
+      <c r="L12" t="n">
+        <v>2.22</v>
+      </c>
+      <c r="M12" t="n">
+        <v>25.6</v>
+      </c>
+      <c r="N12" t="n">
+        <v>58.1</v>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P12" t="n">
+        <v>65.09999999999999</v>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr"/>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>84.11</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="D13" s="3" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>SELL</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>Debit Put</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>30-60 DTE</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>SQUEEZE</t>
         </is>
       </c>
-      <c r="I10" t="n">
-        <v>57.3</v>
-      </c>
-      <c r="J10" t="n">
-        <v>46</v>
-      </c>
-      <c r="K10" t="n">
-        <v>11</v>
-      </c>
-      <c r="L10" t="n">
-        <v>1.98</v>
-      </c>
-      <c r="M10" t="n">
-        <v>18.9</v>
-      </c>
-      <c r="N10" t="n">
-        <v>70.09999999999999</v>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P10" t="n">
-        <v>58.3</v>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R10" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S10" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="T10" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U10" t="inlineStr">
-        <is>
-          <t>Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
-      <c r="V10" t="inlineStr">
+      <c r="I13" t="n">
+        <v>62.2</v>
+      </c>
+      <c r="J13" t="n">
+        <v>42.8</v>
+      </c>
+      <c r="K13" t="n">
+        <v>3</v>
+      </c>
+      <c r="L13" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="M13" t="n">
+        <v>23.3</v>
+      </c>
+      <c r="N13" t="n">
+        <v>61.6</v>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P13" t="n">
+        <v>46.9</v>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>

</xml_diff>

<commit_message>
Scan 21.04.2026 15:21 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -31,10 +31,10 @@
       <sz val="11"/>
     </font>
     <font>
-      <color rgb="0022c55e"/>
+      <color rgb="00ef4444"/>
     </font>
     <font>
-      <color rgb="00ef4444"/>
+      <color rgb="0022c55e"/>
     </font>
   </fonts>
   <fills count="3">
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V13"/>
+  <dimension ref="A1:V12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -577,11 +577,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SYY</t>
+          <t>EQR</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>76.66</v>
+        <v>62.56</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -590,17 +590,17 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>BULLISH</t>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -614,19 +614,22 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>81.2</v>
+        <v>81.09999999999999</v>
       </c>
       <c r="J2" t="n">
-        <v>48.7</v>
+        <v>60.3</v>
       </c>
       <c r="K2" t="n">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="L2" t="n">
-        <v>2.54</v>
+        <v>1.9</v>
       </c>
       <c r="M2" t="n">
-        <v>27.5</v>
+        <v>20.8</v>
+      </c>
+      <c r="N2" t="n">
+        <v>58.1</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -634,7 +637,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>47.2</v>
+        <v>54.8</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -648,12 +651,12 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
@@ -666,56 +669,59 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CMCSA</t>
+          <t>USB</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>30.02</v>
+        <v>57.12</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>BULLISH</t>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>79.3</v>
+        <v>77.7</v>
       </c>
       <c r="J3" t="n">
-        <v>63.6</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="K3" t="n">
-        <v>39</v>
+        <v>88</v>
       </c>
       <c r="L3" t="n">
-        <v>2.19</v>
+        <v>2.32</v>
       </c>
       <c r="M3" t="n">
-        <v>39.9</v>
+        <v>19.9</v>
+      </c>
+      <c r="N3" t="n">
+        <v>33.7</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -723,7 +729,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>56</v>
+        <v>61.9</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -737,7 +743,7 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -759,14 +765,14 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>53.58</v>
+        <v>54</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
@@ -792,22 +798,19 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>77.59999999999999</v>
+        <v>76.8</v>
       </c>
       <c r="J4" t="n">
-        <v>65.7</v>
+        <v>68.7</v>
       </c>
       <c r="K4" t="n">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="L4" t="n">
-        <v>2.18</v>
+        <v>2.07</v>
       </c>
       <c r="M4" t="n">
-        <v>22.7</v>
-      </c>
-      <c r="N4" t="n">
-        <v>56.3</v>
+        <v>25.1</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -815,7 +818,7 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>56.7</v>
+        <v>57.8</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -847,59 +850,56 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>IDXX</t>
+          <t>NKE</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>582.22</v>
+        <v>46.1</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>BEARISH</t>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>76.2</v>
+        <v>74</v>
       </c>
       <c r="J5" t="n">
-        <v>49</v>
+        <v>39.6</v>
       </c>
       <c r="K5" t="n">
-        <v>11</v>
+        <v>91</v>
       </c>
       <c r="L5" t="n">
-        <v>2.8</v>
+        <v>3.01</v>
       </c>
       <c r="M5" t="n">
-        <v>29</v>
-      </c>
-      <c r="N5" t="n">
-        <v>21.1</v>
+        <v>34.8</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -907,11 +907,11 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>42.6</v>
+        <v>33.1</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>FIRED</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -926,14 +926,10 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>Squeeze Fired, Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr">
         <is>
           <t>No</t>
@@ -943,18 +939,18 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>FCX</t>
+          <t>CAT</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>70.34</v>
+        <v>809.87</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
@@ -980,19 +976,19 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>75.90000000000001</v>
+        <v>73.8</v>
       </c>
       <c r="J6" t="n">
-        <v>70.59999999999999</v>
+        <v>67.7</v>
       </c>
       <c r="K6" t="n">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="L6" t="n">
-        <v>3.26</v>
+        <v>2.83</v>
       </c>
       <c r="M6" t="n">
-        <v>50.8</v>
+        <v>48.4</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -1000,7 +996,7 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>68.40000000000001</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1032,18 +1028,18 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>INTC</t>
+          <t>FCX</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>66.05</v>
+        <v>68.89</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
@@ -1069,22 +1065,22 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>74.09999999999999</v>
+        <v>73.7</v>
       </c>
       <c r="J7" t="n">
-        <v>71.09999999999999</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="K7" t="n">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="L7" t="n">
-        <v>5.06</v>
+        <v>3.32</v>
       </c>
       <c r="M7" t="n">
-        <v>70.2</v>
+        <v>50.1</v>
       </c>
       <c r="N7" t="n">
-        <v>60.8</v>
+        <v>54.3</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1092,7 +1088,7 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>73.3</v>
+        <v>66.3</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1114,32 +1110,28 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U7" t="inlineStr"/>
       <c r="V7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>AMGN</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>443.2</v>
+        <v>343.22</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
@@ -1151,36 +1143,33 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>73.8</v>
+        <v>70.7</v>
       </c>
       <c r="J8" t="n">
-        <v>58.6</v>
+        <v>41.1</v>
       </c>
       <c r="K8" t="n">
-        <v>87</v>
+        <v>5</v>
       </c>
       <c r="L8" t="n">
-        <v>5.64</v>
+        <v>2.29</v>
       </c>
       <c r="M8" t="n">
-        <v>73</v>
-      </c>
-      <c r="N8" t="n">
-        <v>84.3</v>
+        <v>38.3</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1188,31 +1177,31 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>65.59999999999999</v>
+        <v>51.3</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>Divergence</t>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
@@ -1224,18 +1213,18 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>MDT</t>
+          <t>INTC</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>86.67</v>
+        <v>67.13</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
@@ -1247,48 +1236,45 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>72</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="J9" t="n">
-        <v>43.7</v>
+        <v>71.8</v>
       </c>
       <c r="K9" t="n">
-        <v>4</v>
+        <v>98</v>
       </c>
       <c r="L9" t="n">
-        <v>1.83</v>
+        <v>4.9</v>
       </c>
       <c r="M9" t="n">
-        <v>17.1</v>
-      </c>
-      <c r="N9" t="n">
-        <v>44.4</v>
+        <v>72.8</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>39.4</v>
+        <v>75</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -1298,7 +1284,7 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
@@ -1306,11 +1292,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>TTM Squeeze</t>
-        </is>
-      </c>
+      <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr">
         <is>
           <t>No</t>
@@ -1320,11 +1302,11 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>NKE</t>
+          <t>PCAR</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>46.09</v>
+        <v>127.61</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1333,17 +1315,17 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>BULLISH</t>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1357,30 +1339,27 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>71.5</v>
+        <v>69.2</v>
       </c>
       <c r="J10" t="n">
-        <v>39</v>
+        <v>63.8</v>
       </c>
       <c r="K10" t="n">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="L10" t="n">
-        <v>3.02</v>
+        <v>2.18</v>
       </c>
       <c r="M10" t="n">
-        <v>52.3</v>
-      </c>
-      <c r="N10" t="n">
-        <v>90.2</v>
+        <v>34.2</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>33.1</v>
+        <v>64.8</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1394,12 +1373,12 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U10" t="inlineStr"/>
@@ -1412,18 +1391,18 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CAT</t>
+          <t>PG</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>795.3200000000001</v>
+        <v>142.55</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
@@ -1435,44 +1414,44 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>70.90000000000001</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="J11" t="n">
-        <v>64.7</v>
+        <v>41.7</v>
       </c>
       <c r="K11" t="n">
-        <v>86</v>
+        <v>10</v>
       </c>
       <c r="L11" t="n">
-        <v>2.86</v>
+        <v>1.86</v>
       </c>
       <c r="M11" t="n">
-        <v>37.9</v>
+        <v>19.8</v>
       </c>
       <c r="N11" t="n">
-        <v>71.2</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>72.59999999999999</v>
+        <v>42</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1486,7 +1465,7 @@
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
@@ -1494,7 +1473,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U11" t="inlineStr"/>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V11" t="inlineStr">
         <is>
           <t>No</t>
@@ -1504,18 +1487,18 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>PCAR</t>
+          <t>CL</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>127.91</v>
+        <v>82.27</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
@@ -1527,48 +1510,48 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>70.90000000000001</v>
+        <v>55.9</v>
       </c>
       <c r="J12" t="n">
-        <v>65.3</v>
+        <v>38.9</v>
       </c>
       <c r="K12" t="n">
-        <v>88</v>
+        <v>5</v>
       </c>
       <c r="L12" t="n">
-        <v>2.22</v>
+        <v>2.24</v>
       </c>
       <c r="M12" t="n">
-        <v>25.6</v>
+        <v>23.5</v>
       </c>
       <c r="N12" t="n">
-        <v>58.1</v>
+        <v>63.7</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>65.09999999999999</v>
+        <v>45</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
@@ -1578,7 +1561,7 @@
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
@@ -1586,104 +1569,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U12" t="inlineStr"/>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V12" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>CL</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>84.11</v>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Debit Put</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>30-60 DTE</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>SQUEEZE</t>
-        </is>
-      </c>
-      <c r="I13" t="n">
-        <v>62.2</v>
-      </c>
-      <c r="J13" t="n">
-        <v>42.8</v>
-      </c>
-      <c r="K13" t="n">
-        <v>3</v>
-      </c>
-      <c r="L13" t="n">
-        <v>2.15</v>
-      </c>
-      <c r="M13" t="n">
-        <v>23.3</v>
-      </c>
-      <c r="N13" t="n">
-        <v>61.6</v>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P13" t="n">
-        <v>46.9</v>
-      </c>
-      <c r="Q13" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="R13" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="S13" t="inlineStr">
-        <is>
-          <t>maroon</t>
-        </is>
-      </c>
-      <c r="T13" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U13" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
-      <c r="V13" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>

</xml_diff>

<commit_message>
Scan 22.04.2026 15:21 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V12"/>
+  <dimension ref="A1:V19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -577,15 +577,15 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>EQR</t>
+          <t>BDX</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>62.56</v>
+        <v>155.53</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -600,36 +600,36 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>81.09999999999999</v>
+        <v>80</v>
       </c>
       <c r="J2" t="n">
-        <v>60.3</v>
+        <v>43.8</v>
       </c>
       <c r="K2" t="n">
-        <v>92</v>
+        <v>6</v>
       </c>
       <c r="L2" t="n">
-        <v>1.9</v>
+        <v>1.91</v>
       </c>
       <c r="M2" t="n">
-        <v>20.8</v>
+        <v>18.2</v>
       </c>
       <c r="N2" t="n">
-        <v>58.1</v>
+        <v>5.4</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -637,11 +637,11 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>54.8</v>
+        <v>48.5</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -651,7 +651,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -659,7 +659,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr"/>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V2" t="inlineStr">
         <is>
           <t>No</t>
@@ -669,11 +673,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>USB</t>
+          <t>PSA</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>57.12</v>
+        <v>306.27</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -706,22 +710,19 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>77.7</v>
+        <v>77.2</v>
       </c>
       <c r="J3" t="n">
-        <v>66.40000000000001</v>
+        <v>63.6</v>
       </c>
       <c r="K3" t="n">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="L3" t="n">
-        <v>2.32</v>
+        <v>2.15</v>
       </c>
       <c r="M3" t="n">
-        <v>19.9</v>
-      </c>
-      <c r="N3" t="n">
-        <v>33.7</v>
+        <v>28.2</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -729,7 +730,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>61.9</v>
+        <v>58.5</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -761,11 +762,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BAC</t>
+          <t>SPG</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>54</v>
+        <v>204</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -798,19 +799,19 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>76.8</v>
+        <v>76.5</v>
       </c>
       <c r="J4" t="n">
-        <v>68.7</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="K4" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L4" t="n">
-        <v>2.07</v>
+        <v>1.68</v>
       </c>
       <c r="M4" t="n">
-        <v>25.1</v>
+        <v>26.8</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -818,7 +819,7 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>57.8</v>
+        <v>64</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -850,68 +851,71 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>NKE</t>
+          <t>AMGN</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>46.1</v>
+        <v>345.8</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>74</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="J5" t="n">
-        <v>39.6</v>
+        <v>43.3</v>
       </c>
       <c r="K5" t="n">
-        <v>91</v>
+        <v>6</v>
       </c>
       <c r="L5" t="n">
-        <v>3.01</v>
+        <v>2.13</v>
       </c>
       <c r="M5" t="n">
-        <v>34.8</v>
+        <v>20.1</v>
+      </c>
+      <c r="N5" t="n">
+        <v>15.7</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>33.1</v>
+        <v>52.4</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -926,10 +930,14 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V5" t="inlineStr">
         <is>
           <t>No</t>
@@ -939,30 +947,30 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CAT</t>
+          <t>NKE</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>809.87</v>
+        <v>46.11</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -976,27 +984,27 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>73.8</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="J6" t="n">
-        <v>67.7</v>
+        <v>39.6</v>
       </c>
       <c r="K6" t="n">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="L6" t="n">
-        <v>2.83</v>
+        <v>2.92</v>
       </c>
       <c r="M6" t="n">
-        <v>48.4</v>
+        <v>34.2</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P6" t="n">
-        <v>73.90000000000001</v>
+        <v>33.1</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1010,12 +1018,12 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
@@ -1028,11 +1036,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>FCX</t>
+          <t>MET</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>68.89</v>
+        <v>76.75</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1068,19 +1076,19 @@
         <v>73.7</v>
       </c>
       <c r="J7" t="n">
-        <v>65.09999999999999</v>
+        <v>62.2</v>
       </c>
       <c r="K7" t="n">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="L7" t="n">
-        <v>3.32</v>
+        <v>2.02</v>
       </c>
       <c r="M7" t="n">
-        <v>50.1</v>
+        <v>23.9</v>
       </c>
       <c r="N7" t="n">
-        <v>54.3</v>
+        <v>53.5</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1088,7 +1096,7 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>66.3</v>
+        <v>52.7</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1120,15 +1128,15 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>FCX</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>343.22</v>
+        <v>69.92</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -1143,33 +1151,33 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>70.7</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="J8" t="n">
-        <v>41.1</v>
+        <v>65.2</v>
       </c>
       <c r="K8" t="n">
-        <v>5</v>
+        <v>91</v>
       </c>
       <c r="L8" t="n">
-        <v>2.29</v>
+        <v>3.56</v>
       </c>
       <c r="M8" t="n">
-        <v>38.3</v>
+        <v>51.6</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1177,47 +1185,43 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>51.3</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>INTC</t>
+          <t>USB</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>67.13</v>
+        <v>56.86</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1250,19 +1254,19 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>70.09999999999999</v>
+        <v>72.5</v>
       </c>
       <c r="J9" t="n">
-        <v>71.8</v>
+        <v>64.8</v>
       </c>
       <c r="K9" t="n">
-        <v>98</v>
+        <v>84</v>
       </c>
       <c r="L9" t="n">
-        <v>4.9</v>
+        <v>2.18</v>
       </c>
       <c r="M9" t="n">
-        <v>72.8</v>
+        <v>28.2</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1270,7 +1274,7 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>75</v>
+        <v>61.3</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1302,11 +1306,11 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>PCAR</t>
+          <t>BAC</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>127.61</v>
+        <v>53.35</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1339,19 +1343,19 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>69.2</v>
+        <v>72.3</v>
       </c>
       <c r="J10" t="n">
-        <v>63.8</v>
+        <v>63.4</v>
       </c>
       <c r="K10" t="n">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="L10" t="n">
-        <v>2.18</v>
+        <v>2.11</v>
       </c>
       <c r="M10" t="n">
-        <v>34.2</v>
+        <v>25.4</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1359,7 +1363,7 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>64.8</v>
+        <v>56.1</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1391,15 +1395,15 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>PG</t>
+          <t>CAT</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>142.55</v>
+        <v>810.9400000000001</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -1414,44 +1418,44 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>64.09999999999999</v>
+        <v>71.5</v>
       </c>
       <c r="J11" t="n">
-        <v>41.7</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="K11" t="n">
-        <v>10</v>
+        <v>90</v>
       </c>
       <c r="L11" t="n">
-        <v>1.86</v>
+        <v>2.75</v>
       </c>
       <c r="M11" t="n">
-        <v>19.8</v>
+        <v>36.7</v>
       </c>
       <c r="N11" t="n">
-        <v>69.40000000000001</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>42</v>
+        <v>74</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1465,7 +1469,7 @@
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
@@ -1473,11 +1477,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U11" t="inlineStr">
-        <is>
-          <t>Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U11" t="inlineStr"/>
       <c r="V11" t="inlineStr">
         <is>
           <t>No</t>
@@ -1487,94 +1487,748 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>312.95</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>68.59999999999999</v>
+      </c>
+      <c r="J12" t="n">
+        <v>61.8</v>
+      </c>
+      <c r="K12" t="n">
+        <v>92</v>
+      </c>
+      <c r="L12" t="n">
+        <v>1.98</v>
+      </c>
+      <c r="M12" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="N12" t="n">
+        <v>49.3</v>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P12" t="n">
+        <v>56.3</v>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr"/>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>142.78</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>68.40000000000001</v>
+      </c>
+      <c r="J13" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="K13" t="n">
+        <v>12</v>
+      </c>
+      <c r="L13" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="M13" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="N13" t="n">
+        <v>69.59999999999999</v>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P13" t="n">
+        <v>42.3</v>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>PCAR</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>126.23</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>68.2</v>
+      </c>
+      <c r="J14" t="n">
+        <v>59.9</v>
+      </c>
+      <c r="K14" t="n">
+        <v>84</v>
+      </c>
+      <c r="L14" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="M14" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="N14" t="n">
+        <v>60.7</v>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P14" t="n">
+        <v>63.7</v>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr"/>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>INTC</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>66.23</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>67.2</v>
+      </c>
+      <c r="J15" t="n">
+        <v>70.8</v>
+      </c>
+      <c r="K15" t="n">
+        <v>96</v>
+      </c>
+      <c r="L15" t="n">
+        <v>4.99</v>
+      </c>
+      <c r="M15" t="n">
+        <v>69.8</v>
+      </c>
+      <c r="N15" t="n">
+        <v>60.1</v>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P15" t="n">
+        <v>73.59999999999999</v>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr"/>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>IDXX</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>579.22</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>66</v>
+      </c>
+      <c r="J16" t="n">
+        <v>48.3</v>
+      </c>
+      <c r="K16" t="n">
+        <v>13</v>
+      </c>
+      <c r="L16" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="M16" t="n">
+        <v>29.8</v>
+      </c>
+      <c r="N16" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P16" t="n">
+        <v>42.1</v>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>TMUS</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>186.22</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>63.6</v>
+      </c>
+      <c r="J17" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="K17" t="n">
+        <v>87</v>
+      </c>
+      <c r="L17" t="n">
+        <v>3.48</v>
+      </c>
+      <c r="M17" t="n">
+        <v>40.1</v>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P17" t="n">
+        <v>36.6</v>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>CL</t>
         </is>
       </c>
-      <c r="B12" t="n">
-        <v>82.27</v>
-      </c>
-      <c r="C12" t="inlineStr">
+      <c r="B18" t="n">
+        <v>82.12</v>
+      </c>
+      <c r="C18" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>SELL</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>Debit Put</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>30-60 DTE</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="H18" t="inlineStr">
         <is>
           <t>SQUEEZE</t>
         </is>
       </c>
-      <c r="I12" t="n">
-        <v>55.9</v>
-      </c>
-      <c r="J12" t="n">
-        <v>38.9</v>
-      </c>
-      <c r="K12" t="n">
-        <v>5</v>
-      </c>
-      <c r="L12" t="n">
-        <v>2.24</v>
-      </c>
-      <c r="M12" t="n">
-        <v>23.5</v>
-      </c>
-      <c r="N12" t="n">
-        <v>63.7</v>
-      </c>
-      <c r="O12" t="inlineStr">
+      <c r="I18" t="n">
+        <v>54.3</v>
+      </c>
+      <c r="J18" t="n">
+        <v>39.1</v>
+      </c>
+      <c r="K18" t="n">
+        <v>9</v>
+      </c>
+      <c r="L18" t="n">
+        <v>2.16</v>
+      </c>
+      <c r="M18" t="n">
+        <v>23.9</v>
+      </c>
+      <c r="N18" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="O18" t="inlineStr">
         <is>
           <t>Bearish</t>
         </is>
       </c>
-      <c r="P12" t="n">
-        <v>45</v>
-      </c>
-      <c r="Q12" t="inlineStr">
+      <c r="P18" t="n">
+        <v>44.8</v>
+      </c>
+      <c r="Q18" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
       </c>
-      <c r="R12" t="inlineStr">
+      <c r="R18" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
       </c>
-      <c r="S12" t="inlineStr">
+      <c r="S18" t="inlineStr">
         <is>
           <t>maroon</t>
         </is>
       </c>
-      <c r="T12" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U12" t="inlineStr">
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>324.55</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>52.4</v>
+      </c>
+      <c r="J19" t="n">
+        <v>45.2</v>
+      </c>
+      <c r="K19" t="n">
+        <v>16</v>
+      </c>
+      <c r="L19" t="n">
+        <v>1.87</v>
+      </c>
+      <c r="M19" t="n">
+        <v>20</v>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P19" t="n">
+        <v>57.6</v>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
         <is>
           <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
         </is>
       </c>
-      <c r="V12" t="inlineStr">
+      <c r="V19" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>

</xml_diff>

<commit_message>
Scan 24.04.2026 15:16 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V19"/>
+  <dimension ref="A1:V33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -577,15 +577,15 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BDX</t>
+          <t>INTC</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>155.53</v>
+        <v>82.73</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -600,48 +600,45 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>80</v>
+        <v>88.59999999999999</v>
       </c>
       <c r="J2" t="n">
-        <v>43.8</v>
+        <v>82.3</v>
       </c>
       <c r="K2" t="n">
-        <v>6</v>
+        <v>98</v>
       </c>
       <c r="L2" t="n">
-        <v>1.91</v>
+        <v>6.45</v>
       </c>
       <c r="M2" t="n">
-        <v>18.2</v>
-      </c>
-      <c r="N2" t="n">
-        <v>5.4</v>
+        <v>73.5</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>48.5</v>
+        <v>82.8</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -651,7 +648,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -659,11 +656,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr">
         <is>
           <t>No</t>
@@ -673,11 +666,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>PSA</t>
+          <t>BA</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>306.27</v>
+        <v>234.08</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -710,19 +703,19 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>77.2</v>
+        <v>84.2</v>
       </c>
       <c r="J3" t="n">
-        <v>63.6</v>
+        <v>64</v>
       </c>
       <c r="K3" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="L3" t="n">
-        <v>2.15</v>
+        <v>3.02</v>
       </c>
       <c r="M3" t="n">
-        <v>28.2</v>
+        <v>35</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -730,7 +723,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>58.5</v>
+        <v>56.5</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -762,11 +755,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SPG</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>204</v>
+        <v>711.6</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -799,19 +792,19 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>76.5</v>
+        <v>78.2</v>
       </c>
       <c r="J4" t="n">
-        <v>64.59999999999999</v>
+        <v>69.5</v>
       </c>
       <c r="K4" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="L4" t="n">
-        <v>1.68</v>
+        <v>1.08</v>
       </c>
       <c r="M4" t="n">
-        <v>26.8</v>
+        <v>15.6</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -819,7 +812,7 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>64</v>
+        <v>64.2</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -851,15 +844,15 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>IWM</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>345.8</v>
+        <v>276.11</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -874,36 +867,33 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>75.90000000000001</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="J5" t="n">
-        <v>43.3</v>
+        <v>69</v>
       </c>
       <c r="K5" t="n">
-        <v>6</v>
+        <v>99</v>
       </c>
       <c r="L5" t="n">
-        <v>2.13</v>
+        <v>1.66</v>
       </c>
       <c r="M5" t="n">
-        <v>20.1</v>
-      </c>
-      <c r="N5" t="n">
-        <v>15.7</v>
+        <v>22.9</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -911,11 +901,11 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>52.4</v>
+        <v>67.2</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -925,7 +915,7 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -933,11 +923,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr">
         <is>
           <t>No</t>
@@ -947,15 +933,15 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>NKE</t>
+          <t>LIN</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>46.11</v>
+        <v>508.36</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -970,45 +956,48 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>73.90000000000001</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="J6" t="n">
-        <v>39.6</v>
+        <v>59.7</v>
       </c>
       <c r="K6" t="n">
-        <v>89</v>
+        <v>3</v>
       </c>
       <c r="L6" t="n">
-        <v>2.92</v>
+        <v>1.79</v>
       </c>
       <c r="M6" t="n">
-        <v>34.2</v>
+        <v>18.7</v>
+      </c>
+      <c r="N6" t="n">
+        <v>69</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P6" t="n">
-        <v>33.1</v>
+        <v>64.3</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -1018,7 +1007,7 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
@@ -1026,7 +1015,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr"/>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V6" t="inlineStr">
         <is>
           <t>No</t>
@@ -1036,15 +1029,15 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>MET</t>
+          <t>BMY</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>76.75</v>
+        <v>58.4</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -1059,36 +1052,36 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>73.7</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="J7" t="n">
-        <v>62.2</v>
+        <v>47.5</v>
       </c>
       <c r="K7" t="n">
-        <v>98</v>
+        <v>7</v>
       </c>
       <c r="L7" t="n">
-        <v>2.02</v>
+        <v>2.1</v>
       </c>
       <c r="M7" t="n">
         <v>23.9</v>
       </c>
       <c r="N7" t="n">
-        <v>53.5</v>
+        <v>38.8</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1096,29 +1089,33 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>52.7</v>
+        <v>58.8</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U7" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V7" t="inlineStr">
         <is>
           <t>No</t>
@@ -1128,15 +1125,15 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>FCX</t>
+          <t>REGN</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>69.92</v>
+        <v>737.61</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -1151,33 +1148,33 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>72.90000000000001</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="J8" t="n">
-        <v>65.2</v>
+        <v>43.3</v>
       </c>
       <c r="K8" t="n">
-        <v>91</v>
+        <v>11</v>
       </c>
       <c r="L8" t="n">
-        <v>3.56</v>
+        <v>2.57</v>
       </c>
       <c r="M8" t="n">
-        <v>51.6</v>
+        <v>51.1</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1185,43 +1182,47 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>67.90000000000001</v>
+        <v>51.7</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U8" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>USB</t>
+          <t>PSA</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>56.86</v>
+        <v>310.34</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1254,16 +1255,16 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>72.5</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="J9" t="n">
-        <v>64.8</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="K9" t="n">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="L9" t="n">
-        <v>2.18</v>
+        <v>2.09</v>
       </c>
       <c r="M9" t="n">
         <v>28.2</v>
@@ -1274,7 +1275,7 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>61.3</v>
+        <v>60.2</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1306,11 +1307,11 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>BAC</t>
+          <t>DLR</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>53.35</v>
+        <v>206.71</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1346,16 +1347,16 @@
         <v>72.3</v>
       </c>
       <c r="J10" t="n">
-        <v>63.4</v>
+        <v>78.3</v>
       </c>
       <c r="K10" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="L10" t="n">
-        <v>2.11</v>
+        <v>2.16</v>
       </c>
       <c r="M10" t="n">
-        <v>25.4</v>
+        <v>32.5</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1363,7 +1364,7 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>56.1</v>
+        <v>73.5</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1395,15 +1396,15 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CAT</t>
+          <t>BDX</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>810.9400000000001</v>
+        <v>153.14</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -1418,66 +1419,70 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>71.5</v>
+        <v>72</v>
       </c>
       <c r="J11" t="n">
-        <v>68.09999999999999</v>
+        <v>38.5</v>
       </c>
       <c r="K11" t="n">
-        <v>90</v>
+        <v>8</v>
       </c>
       <c r="L11" t="n">
-        <v>2.75</v>
+        <v>1.94</v>
       </c>
       <c r="M11" t="n">
-        <v>36.7</v>
+        <v>17.4</v>
       </c>
       <c r="N11" t="n">
-        <v>67.09999999999999</v>
+        <v>3.5</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>74</v>
+        <v>46.5</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U11" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V11" t="inlineStr">
         <is>
           <t>No</t>
@@ -1487,11 +1492,11 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>JPM</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>312.95</v>
+        <v>418.45</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1524,22 +1529,19 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>68.59999999999999</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="J12" t="n">
-        <v>61.8</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="K12" t="n">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="L12" t="n">
-        <v>1.98</v>
+        <v>3.08</v>
       </c>
       <c r="M12" t="n">
-        <v>22.2</v>
-      </c>
-      <c r="N12" t="n">
-        <v>49.3</v>
+        <v>49.2</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1547,7 +1549,7 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>56.3</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1569,25 +1571,29 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U12" t="inlineStr"/>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>PG</t>
+          <t>BK</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>142.78</v>
+        <v>134.58</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -1602,44 +1608,44 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>68.40000000000001</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="J13" t="n">
-        <v>42.5</v>
+        <v>69.3</v>
       </c>
       <c r="K13" t="n">
-        <v>12</v>
+        <v>96</v>
       </c>
       <c r="L13" t="n">
-        <v>1.72</v>
+        <v>1.99</v>
       </c>
       <c r="M13" t="n">
-        <v>19.9</v>
+        <v>19.3</v>
       </c>
       <c r="N13" t="n">
-        <v>69.59999999999999</v>
+        <v>33.6</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>42.3</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1653,7 +1659,7 @@
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
@@ -1661,11 +1667,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U13" t="inlineStr">
-        <is>
-          <t>Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U13" t="inlineStr"/>
       <c r="V13" t="inlineStr">
         <is>
           <t>No</t>
@@ -1675,11 +1677,11 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>PCAR</t>
+          <t>MAR</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>126.23</v>
+        <v>367.35</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -1712,22 +1714,19 @@
         </is>
       </c>
       <c r="I14" t="n">
-        <v>68.2</v>
+        <v>71.3</v>
       </c>
       <c r="J14" t="n">
-        <v>59.9</v>
+        <v>62.2</v>
       </c>
       <c r="K14" t="n">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="L14" t="n">
-        <v>2.3</v>
+        <v>2.36</v>
       </c>
       <c r="M14" t="n">
-        <v>25.9</v>
-      </c>
-      <c r="N14" t="n">
-        <v>60.7</v>
+        <v>40.7</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1735,7 +1734,7 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>63.7</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1744,17 +1743,17 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U14" t="inlineStr"/>
@@ -1767,11 +1766,11 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>INTC</t>
+          <t>CDW</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>66.23</v>
+        <v>135.27</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1804,30 +1803,30 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>67.2</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="J15" t="n">
-        <v>70.8</v>
+        <v>60.4</v>
       </c>
       <c r="K15" t="n">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="L15" t="n">
-        <v>4.99</v>
+        <v>2.83</v>
       </c>
       <c r="M15" t="n">
-        <v>69.8</v>
+        <v>28.6</v>
       </c>
       <c r="N15" t="n">
-        <v>60.1</v>
+        <v>35.9</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P15" t="n">
-        <v>73.59999999999999</v>
+        <v>50.7</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1836,17 +1835,17 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U15" t="inlineStr"/>
@@ -1859,15 +1858,15 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>IDXX</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>579.22</v>
+        <v>187.77</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -1882,48 +1881,48 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>66</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="J16" t="n">
-        <v>48.3</v>
+        <v>64.7</v>
       </c>
       <c r="K16" t="n">
-        <v>13</v>
+        <v>98</v>
       </c>
       <c r="L16" t="n">
-        <v>2.99</v>
+        <v>2.45</v>
       </c>
       <c r="M16" t="n">
-        <v>29.8</v>
+        <v>26.9</v>
       </c>
       <c r="N16" t="n">
-        <v>22.2</v>
+        <v>46.3</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>42.1</v>
+        <v>63.3</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
@@ -1933,7 +1932,7 @@
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
@@ -1941,11 +1940,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U16" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U16" t="inlineStr"/>
       <c r="V16" t="inlineStr">
         <is>
           <t>No</t>
@@ -1955,68 +1950,71 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>TMUS</t>
+          <t>WBD</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>186.22</v>
+        <v>27.09</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>63.6</v>
+        <v>68.8</v>
       </c>
       <c r="J17" t="n">
-        <v>30.5</v>
+        <v>42.1</v>
       </c>
       <c r="K17" t="n">
-        <v>87</v>
+        <v>9</v>
       </c>
       <c r="L17" t="n">
-        <v>3.48</v>
+        <v>0.87</v>
       </c>
       <c r="M17" t="n">
-        <v>40.1</v>
+        <v>10.9</v>
+      </c>
+      <c r="N17" t="n">
+        <v>0.5</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P17" t="n">
-        <v>36.6</v>
+        <v>60.1</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
@@ -2031,32 +2029,32 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>Divergence</t>
+          <t>TTM Squeeze</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>APH</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>82.12</v>
+        <v>150.29</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -2071,48 +2069,45 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>54.3</v>
+        <v>68.7</v>
       </c>
       <c r="J18" t="n">
-        <v>39.1</v>
+        <v>62.9</v>
       </c>
       <c r="K18" t="n">
-        <v>9</v>
+        <v>97</v>
       </c>
       <c r="L18" t="n">
-        <v>2.16</v>
+        <v>2.97</v>
       </c>
       <c r="M18" t="n">
-        <v>23.9</v>
-      </c>
-      <c r="N18" t="n">
-        <v>66.7</v>
+        <v>52.6</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P18" t="n">
-        <v>44.8</v>
+        <v>60.5</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
@@ -2122,7 +2117,7 @@
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
@@ -2130,11 +2125,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U18" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U18" t="inlineStr"/>
       <c r="V18" t="inlineStr">
         <is>
           <t>No</t>
@@ -2144,93 +2135,1361 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>TT</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>485.45</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>68.59999999999999</v>
+      </c>
+      <c r="J19" t="n">
+        <v>68.90000000000001</v>
+      </c>
+      <c r="K19" t="n">
+        <v>88</v>
+      </c>
+      <c r="L19" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="M19" t="n">
+        <v>34.2</v>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P19" t="n">
+        <v>65.8</v>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr"/>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>SPG</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>202.9</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>68.3</v>
+      </c>
+      <c r="J20" t="n">
+        <v>60.7</v>
+      </c>
+      <c r="K20" t="n">
+        <v>94</v>
+      </c>
+      <c r="L20" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="M20" t="n">
+        <v>28</v>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P20" t="n">
+        <v>63</v>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr"/>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>MET</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>77.26000000000001</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>68.2</v>
+      </c>
+      <c r="J21" t="n">
+        <v>62.6</v>
+      </c>
+      <c r="K21" t="n">
+        <v>92</v>
+      </c>
+      <c r="L21" t="n">
+        <v>2.04</v>
+      </c>
+      <c r="M21" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="N21" t="n">
+        <v>50.9</v>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P21" t="n">
+        <v>53.5</v>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr"/>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>GOOG</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>336.22</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>67.90000000000001</v>
+      </c>
+      <c r="J22" t="n">
+        <v>65.59999999999999</v>
+      </c>
+      <c r="K22" t="n">
+        <v>97</v>
+      </c>
+      <c r="L22" t="n">
+        <v>1.99</v>
+      </c>
+      <c r="M22" t="n">
+        <v>35.5</v>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P22" t="n">
+        <v>63.3</v>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr"/>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>NKE</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>45.04</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>67.8</v>
+      </c>
+      <c r="J23" t="n">
+        <v>36.8</v>
+      </c>
+      <c r="K23" t="n">
+        <v>80</v>
+      </c>
+      <c r="L23" t="n">
+        <v>2.95</v>
+      </c>
+      <c r="M23" t="n">
+        <v>52.4</v>
+      </c>
+      <c r="N23" t="n">
+        <v>90.5</v>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P23" t="n">
+        <v>32.1</v>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr"/>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>LRCX</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>271.37</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>67.3</v>
+      </c>
+      <c r="J24" t="n">
+        <v>62.6</v>
+      </c>
+      <c r="K24" t="n">
+        <v>88</v>
+      </c>
+      <c r="L24" t="n">
+        <v>4.41</v>
+      </c>
+      <c r="M24" t="n">
+        <v>60</v>
+      </c>
+      <c r="N24" t="n">
+        <v>78.90000000000001</v>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P24" t="n">
+        <v>71.09999999999999</v>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr"/>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>337.51</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>67.2</v>
+      </c>
+      <c r="J25" t="n">
+        <v>64.8</v>
+      </c>
+      <c r="K25" t="n">
+        <v>96</v>
+      </c>
+      <c r="L25" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="M25" t="n">
+        <v>37.3</v>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P25" t="n">
+        <v>63.4</v>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr"/>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>26.2</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>65</v>
+      </c>
+      <c r="J26" t="n">
+        <v>43</v>
+      </c>
+      <c r="K26" t="n">
+        <v>78</v>
+      </c>
+      <c r="L26" t="n">
+        <v>2.57</v>
+      </c>
+      <c r="M26" t="n">
+        <v>26</v>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P26" t="n">
+        <v>48.9</v>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr"/>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>PCAR</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>126.01</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>64.90000000000001</v>
+      </c>
+      <c r="J27" t="n">
+        <v>57.9</v>
+      </c>
+      <c r="K27" t="n">
+        <v>81</v>
+      </c>
+      <c r="L27" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="M27" t="n">
+        <v>26</v>
+      </c>
+      <c r="N27" t="n">
+        <v>61.2</v>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P27" t="n">
+        <v>63.4</v>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr"/>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>FCX</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>61.54</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>64.2</v>
+      </c>
+      <c r="J28" t="n">
+        <v>45</v>
+      </c>
+      <c r="K28" t="n">
+        <v>85</v>
+      </c>
+      <c r="L28" t="n">
+        <v>5.31</v>
+      </c>
+      <c r="M28" t="n">
+        <v>52</v>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P28" t="n">
+        <v>56.2</v>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr"/>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>127.83</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>61.7</v>
+      </c>
+      <c r="J29" t="n">
+        <v>60.7</v>
+      </c>
+      <c r="K29" t="n">
+        <v>95</v>
+      </c>
+      <c r="L29" t="n">
+        <v>2.51</v>
+      </c>
+      <c r="M29" t="n">
+        <v>31.9</v>
+      </c>
+      <c r="N29" t="n">
+        <v>56.4</v>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P29" t="n">
+        <v>63.8</v>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr"/>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>52.21</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>61.2</v>
+      </c>
+      <c r="J30" t="n">
+        <v>54.4</v>
+      </c>
+      <c r="K30" t="n">
+        <v>92</v>
+      </c>
+      <c r="L30" t="n">
+        <v>2.07</v>
+      </c>
+      <c r="M30" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P30" t="n">
+        <v>53.2</v>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr"/>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>USB</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>55.97</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>60.5</v>
+      </c>
+      <c r="J31" t="n">
+        <v>57.6</v>
+      </c>
+      <c r="K31" t="n">
+        <v>71</v>
+      </c>
+      <c r="L31" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="M31" t="n">
+        <v>29.6</v>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P31" t="n">
+        <v>58.9</v>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr"/>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t>CB</t>
         </is>
       </c>
-      <c r="B19" t="n">
-        <v>324.55</v>
-      </c>
-      <c r="C19" t="inlineStr">
+      <c r="B32" t="n">
+        <v>328.7</v>
+      </c>
+      <c r="C32" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Debit Call</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>57.9</v>
+      </c>
+      <c r="J32" t="n">
+        <v>50.8</v>
+      </c>
+      <c r="K32" t="n">
+        <v>11</v>
+      </c>
+      <c r="L32" t="n">
+        <v>1.86</v>
+      </c>
+      <c r="M32" t="n">
+        <v>20.3</v>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P32" t="n">
+        <v>60.5</v>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>IDXX</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>557</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E33" t="inlineStr">
         <is>
           <t>SELL</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="F33" t="inlineStr">
         <is>
           <t>Debit Put</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="G33" t="inlineStr">
         <is>
           <t>30-60 DTE</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>SQUEEZE</t>
-        </is>
-      </c>
-      <c r="I19" t="n">
-        <v>52.4</v>
-      </c>
-      <c r="J19" t="n">
-        <v>45.2</v>
-      </c>
-      <c r="K19" t="n">
-        <v>16</v>
-      </c>
-      <c r="L19" t="n">
-        <v>1.87</v>
-      </c>
-      <c r="M19" t="n">
-        <v>20</v>
-      </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P19" t="n">
-        <v>57.6</v>
-      </c>
-      <c r="Q19" t="inlineStr">
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>53.8</v>
+      </c>
+      <c r="J33" t="n">
+        <v>40.8</v>
+      </c>
+      <c r="K33" t="n">
+        <v>23</v>
+      </c>
+      <c r="L33" t="n">
+        <v>3.05</v>
+      </c>
+      <c r="M33" t="n">
+        <v>27.6</v>
+      </c>
+      <c r="N33" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P33" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="Q33" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
       </c>
-      <c r="R19" t="inlineStr">
+      <c r="R33" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="S19" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="T19" t="inlineStr">
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="U19" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
-      <c r="V19" t="inlineStr">
-        <is>
-          <t>Yes</t>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan 27.04.2026 15:54 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,11 +435,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V33"/>
+  <dimension ref="A1:V46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
@@ -581,7 +581,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>82.73</v>
+        <v>83.48999999999999</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,19 +614,22 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>88.59999999999999</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="J2" t="n">
-        <v>82.3</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="K2" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="L2" t="n">
-        <v>6.45</v>
+        <v>6.26</v>
       </c>
       <c r="M2" t="n">
-        <v>73.5</v>
+        <v>92.8</v>
+      </c>
+      <c r="N2" t="n">
+        <v>98.09999999999999</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -634,7 +637,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>82.8</v>
+        <v>83.09999999999999</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -666,11 +669,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BA</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>234.08</v>
+        <v>156.38</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -703,19 +706,22 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>84.2</v>
+        <v>87</v>
       </c>
       <c r="J3" t="n">
-        <v>64</v>
+        <v>75.8</v>
       </c>
       <c r="K3" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="L3" t="n">
-        <v>3.02</v>
+        <v>5.64</v>
       </c>
       <c r="M3" t="n">
-        <v>35</v>
+        <v>65.90000000000001</v>
+      </c>
+      <c r="N3" t="n">
+        <v>65.2</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -723,7 +729,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>56.5</v>
+        <v>78.5</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -745,21 +751,25 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr"/>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>ADI</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>711.6</v>
+        <v>389.03</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -792,19 +802,22 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>78.2</v>
+        <v>86.3</v>
       </c>
       <c r="J4" t="n">
-        <v>69.5</v>
+        <v>68.7</v>
       </c>
       <c r="K4" t="n">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="L4" t="n">
-        <v>1.08</v>
+        <v>3.08</v>
       </c>
       <c r="M4" t="n">
-        <v>15.6</v>
+        <v>37.3</v>
+      </c>
+      <c r="N4" t="n">
+        <v>96.7</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -812,7 +825,7 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>64.2</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -844,56 +857,59 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>IWM</t>
+          <t>REGN</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>276.11</v>
+        <v>747.91</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>76.59999999999999</v>
+        <v>85.09999999999999</v>
       </c>
       <c r="J5" t="n">
-        <v>69</v>
+        <v>46.7</v>
       </c>
       <c r="K5" t="n">
-        <v>99</v>
+        <v>2</v>
       </c>
       <c r="L5" t="n">
-        <v>1.66</v>
+        <v>2.39</v>
       </c>
       <c r="M5" t="n">
-        <v>22.9</v>
+        <v>22.4</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0.1</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -901,21 +917,21 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>67.2</v>
+        <v>53.7</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -923,7 +939,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr"/>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
       <c r="V5" t="inlineStr">
         <is>
           <t>No</t>
@@ -933,59 +953,59 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>LIN</t>
+          <t>GFS</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>508.36</v>
+        <v>59.88</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>76.09999999999999</v>
+        <v>83.90000000000001</v>
       </c>
       <c r="J6" t="n">
-        <v>59.7</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="K6" t="n">
-        <v>3</v>
+        <v>99</v>
       </c>
       <c r="L6" t="n">
-        <v>1.79</v>
+        <v>4.91</v>
       </c>
       <c r="M6" t="n">
-        <v>18.7</v>
+        <v>56.4</v>
       </c>
       <c r="N6" t="n">
-        <v>69</v>
+        <v>64.7</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -993,11 +1013,11 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>64.3</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -1012,32 +1032,32 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
           <t>Yes</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
-      <c r="V6" t="inlineStr">
-        <is>
-          <t>No</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BMY</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>58.4</v>
+        <v>421.83</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -1052,70 +1072,63 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>73.90000000000001</v>
+        <v>82.2</v>
       </c>
       <c r="J7" t="n">
-        <v>47.5</v>
+        <v>61.6</v>
       </c>
       <c r="K7" t="n">
-        <v>7</v>
+        <v>90</v>
       </c>
       <c r="L7" t="n">
-        <v>2.1</v>
+        <v>2.57</v>
       </c>
       <c r="M7" t="n">
-        <v>23.9</v>
-      </c>
-      <c r="N7" t="n">
-        <v>38.8</v>
+        <v>38.6</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>58.8</v>
+        <v>48.1</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr"/>
       <c r="V7" t="inlineStr">
         <is>
           <t>No</t>
@@ -1125,15 +1138,15 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>REGN</t>
+          <t>UNH</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>737.61</v>
+        <v>349.99</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -1148,33 +1161,36 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>73.09999999999999</v>
+        <v>81.7</v>
       </c>
       <c r="J8" t="n">
-        <v>43.3</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="K8" t="n">
-        <v>11</v>
+        <v>89</v>
       </c>
       <c r="L8" t="n">
-        <v>2.57</v>
+        <v>2.84</v>
       </c>
       <c r="M8" t="n">
-        <v>51.1</v>
+        <v>40.3</v>
+      </c>
+      <c r="N8" t="n">
+        <v>37.8</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1182,47 +1198,43 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>51.7</v>
+        <v>59.3</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>PSA</t>
+          <t>MCHP</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>310.34</v>
+        <v>86.04000000000001</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1255,19 +1267,22 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>72.40000000000001</v>
+        <v>81</v>
       </c>
       <c r="J9" t="n">
-        <v>65.40000000000001</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="K9" t="n">
         <v>92</v>
       </c>
       <c r="L9" t="n">
-        <v>2.09</v>
+        <v>4.05</v>
       </c>
       <c r="M9" t="n">
-        <v>28.2</v>
+        <v>46.3</v>
+      </c>
+      <c r="N9" t="n">
+        <v>66</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1275,7 +1290,7 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>60.2</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1297,21 +1312,25 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U9" t="inlineStr"/>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>DLR</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>206.71</v>
+        <v>591.38</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1344,19 +1363,19 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>72.3</v>
+        <v>80</v>
       </c>
       <c r="J10" t="n">
-        <v>78.3</v>
+        <v>62</v>
       </c>
       <c r="K10" t="n">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="L10" t="n">
-        <v>2.16</v>
+        <v>2.8</v>
       </c>
       <c r="M10" t="n">
-        <v>32.5</v>
+        <v>29.5</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1364,7 +1383,7 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>73.5</v>
+        <v>56.2</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1396,30 +1415,30 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>BDX</t>
+          <t>LIN</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>153.14</v>
+        <v>508.29</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1433,30 +1452,27 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>72</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="J11" t="n">
-        <v>38.5</v>
+        <v>58.9</v>
       </c>
       <c r="K11" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="L11" t="n">
-        <v>1.94</v>
+        <v>1.74</v>
       </c>
       <c r="M11" t="n">
-        <v>17.4</v>
-      </c>
-      <c r="N11" t="n">
-        <v>3.5</v>
+        <v>24.9</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>46.5</v>
+        <v>63.8</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1465,12 +1481,12 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
@@ -1480,7 +1496,7 @@
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
+          <t>TTM Squeeze</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
@@ -1492,11 +1508,11 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>418.45</v>
+        <v>261.04</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1529,19 +1545,19 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>71.90000000000001</v>
+        <v>79.3</v>
       </c>
       <c r="J12" t="n">
-        <v>76.09999999999999</v>
+        <v>75.8</v>
       </c>
       <c r="K12" t="n">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="L12" t="n">
-        <v>3.08</v>
+        <v>2.46</v>
       </c>
       <c r="M12" t="n">
-        <v>49.2</v>
+        <v>40.8</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1549,7 +1565,7 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>68.40000000000001</v>
+        <v>64.5</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1571,25 +1587,21 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U12" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U12" t="inlineStr"/>
       <c r="V12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>BK</t>
+          <t>XLK</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>134.58</v>
+        <v>159.49</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -1622,22 +1634,19 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>71.40000000000001</v>
+        <v>78.7</v>
       </c>
       <c r="J13" t="n">
-        <v>69.3</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="K13" t="n">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="L13" t="n">
-        <v>1.99</v>
+        <v>1.85</v>
       </c>
       <c r="M13" t="n">
-        <v>19.3</v>
-      </c>
-      <c r="N13" t="n">
-        <v>33.6</v>
+        <v>28.1</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1645,7 +1654,7 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>72.90000000000001</v>
+        <v>69</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1677,11 +1686,11 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>ABNB</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>367.35</v>
+        <v>142.71</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -1714,19 +1723,19 @@
         </is>
       </c>
       <c r="I14" t="n">
-        <v>71.3</v>
+        <v>77.3</v>
       </c>
       <c r="J14" t="n">
-        <v>62.2</v>
+        <v>64.5</v>
       </c>
       <c r="K14" t="n">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="L14" t="n">
-        <v>2.36</v>
+        <v>3.03</v>
       </c>
       <c r="M14" t="n">
-        <v>40.7</v>
+        <v>52.4</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1734,7 +1743,7 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>65.90000000000001</v>
+        <v>60.5</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1743,17 +1752,17 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U14" t="inlineStr"/>
@@ -1766,11 +1775,11 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CDW</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>135.27</v>
+        <v>662.1900000000001</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1803,30 +1812,27 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>70.59999999999999</v>
+        <v>77.2</v>
       </c>
       <c r="J15" t="n">
-        <v>60.4</v>
+        <v>73.5</v>
       </c>
       <c r="K15" t="n">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="L15" t="n">
-        <v>2.83</v>
+        <v>1.45</v>
       </c>
       <c r="M15" t="n">
-        <v>28.6</v>
-      </c>
-      <c r="N15" t="n">
-        <v>35.9</v>
+        <v>20.7</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P15" t="n">
-        <v>50.7</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1835,17 +1841,17 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U15" t="inlineStr"/>
@@ -1858,11 +1864,11 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>187.77</v>
+        <v>713.1900000000001</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -1895,22 +1901,19 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>70.40000000000001</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="J16" t="n">
-        <v>64.7</v>
+        <v>69.7</v>
       </c>
       <c r="K16" t="n">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="L16" t="n">
-        <v>2.45</v>
+        <v>1.02</v>
       </c>
       <c r="M16" t="n">
-        <v>26.9</v>
-      </c>
-      <c r="N16" t="n">
-        <v>46.3</v>
+        <v>15.8</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -1918,7 +1921,7 @@
         </is>
       </c>
       <c r="P16" t="n">
-        <v>63.3</v>
+        <v>64.3</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1950,15 +1953,15 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>WBD</t>
+          <t>KLAC</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>27.09</v>
+        <v>1883.09</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -1973,36 +1976,33 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>68.8</v>
+        <v>74.3</v>
       </c>
       <c r="J17" t="n">
-        <v>42.1</v>
+        <v>68.7</v>
       </c>
       <c r="K17" t="n">
-        <v>9</v>
+        <v>97</v>
       </c>
       <c r="L17" t="n">
-        <v>0.87</v>
+        <v>3.47</v>
       </c>
       <c r="M17" t="n">
-        <v>10.9</v>
-      </c>
-      <c r="N17" t="n">
-        <v>0.5</v>
+        <v>54.4</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -2010,33 +2010,29 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>60.1</v>
+        <v>72.2</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U17" t="inlineStr">
-        <is>
-          <t>TTM Squeeze</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr"/>
       <c r="V17" t="inlineStr">
         <is>
           <t>No</t>
@@ -2046,11 +2042,11 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>APH</t>
+          <t>ETN</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>150.29</v>
+        <v>418.67</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -2083,19 +2079,19 @@
         </is>
       </c>
       <c r="I18" t="n">
-        <v>68.7</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="J18" t="n">
-        <v>62.9</v>
+        <v>67.7</v>
       </c>
       <c r="K18" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L18" t="n">
-        <v>2.97</v>
+        <v>2.77</v>
       </c>
       <c r="M18" t="n">
-        <v>52.6</v>
+        <v>42</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -2103,7 +2099,7 @@
         </is>
       </c>
       <c r="P18" t="n">
-        <v>60.5</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -2135,11 +2131,11 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>TT</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>485.45</v>
+        <v>210.68</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -2172,19 +2168,19 @@
         </is>
       </c>
       <c r="I19" t="n">
-        <v>68.59999999999999</v>
+        <v>73.5</v>
       </c>
       <c r="J19" t="n">
-        <v>68.90000000000001</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="K19" t="n">
-        <v>88</v>
+        <v>99</v>
       </c>
       <c r="L19" t="n">
-        <v>2.34</v>
+        <v>2.61</v>
       </c>
       <c r="M19" t="n">
-        <v>34.2</v>
+        <v>43.3</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -2192,7 +2188,7 @@
         </is>
       </c>
       <c r="P19" t="n">
-        <v>65.8</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -2224,11 +2220,11 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>SPG</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>202.9</v>
+        <v>350.24</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -2261,19 +2257,22 @@
         </is>
       </c>
       <c r="I20" t="n">
-        <v>68.3</v>
+        <v>73.2</v>
       </c>
       <c r="J20" t="n">
-        <v>60.7</v>
+        <v>71.7</v>
       </c>
       <c r="K20" t="n">
         <v>94</v>
       </c>
       <c r="L20" t="n">
-        <v>1.65</v>
+        <v>2.25</v>
       </c>
       <c r="M20" t="n">
-        <v>28</v>
+        <v>33.1</v>
+      </c>
+      <c r="N20" t="n">
+        <v>86.09999999999999</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -2281,7 +2280,7 @@
         </is>
       </c>
       <c r="P20" t="n">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
@@ -2313,11 +2312,11 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>MET</t>
+          <t>GOOG</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>77.26000000000001</v>
+        <v>348.3</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -2350,22 +2349,22 @@
         </is>
       </c>
       <c r="I21" t="n">
-        <v>68.2</v>
+        <v>72.2</v>
       </c>
       <c r="J21" t="n">
-        <v>62.6</v>
+        <v>72.5</v>
       </c>
       <c r="K21" t="n">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="L21" t="n">
-        <v>2.04</v>
+        <v>2.19</v>
       </c>
       <c r="M21" t="n">
-        <v>23.4</v>
+        <v>31.4</v>
       </c>
       <c r="N21" t="n">
-        <v>50.9</v>
+        <v>80.3</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
@@ -2373,7 +2372,7 @@
         </is>
       </c>
       <c r="P21" t="n">
-        <v>53.5</v>
+        <v>66.7</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
@@ -2405,11 +2404,11 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>GOOG</t>
+          <t>IWM</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>336.22</v>
+        <v>276.71</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -2442,19 +2441,22 @@
         </is>
       </c>
       <c r="I22" t="n">
-        <v>67.90000000000001</v>
+        <v>72.2</v>
       </c>
       <c r="J22" t="n">
-        <v>65.59999999999999</v>
+        <v>69.5</v>
       </c>
       <c r="K22" t="n">
         <v>97</v>
       </c>
       <c r="L22" t="n">
-        <v>1.99</v>
+        <v>1.57</v>
       </c>
       <c r="M22" t="n">
-        <v>35.5</v>
+        <v>21.4</v>
+      </c>
+      <c r="N22" t="n">
+        <v>72.40000000000001</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
@@ -2462,7 +2464,7 @@
         </is>
       </c>
       <c r="P22" t="n">
-        <v>63.3</v>
+        <v>67.5</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
@@ -2494,30 +2496,30 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>NKE</t>
+          <t>ANET</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>45.04</v>
+        <v>170.8</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2527,34 +2529,34 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I23" t="n">
-        <v>67.8</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="J23" t="n">
-        <v>36.8</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="K23" t="n">
-        <v>80</v>
+        <v>97</v>
       </c>
       <c r="L23" t="n">
-        <v>2.95</v>
+        <v>3.96</v>
       </c>
       <c r="M23" t="n">
-        <v>52.4</v>
+        <v>56.8</v>
       </c>
       <c r="N23" t="n">
-        <v>90.5</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P23" t="n">
-        <v>32.1</v>
+        <v>65.8</v>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
@@ -2568,29 +2570,33 @@
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
           <t>Yes</t>
-        </is>
-      </c>
-      <c r="U23" t="inlineStr"/>
-      <c r="V23" t="inlineStr">
-        <is>
-          <t>No</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>LRCX</t>
+          <t>BA</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>271.37</v>
+        <v>230.38</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -2619,26 +2625,26 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I24" t="n">
-        <v>67.3</v>
+        <v>72</v>
       </c>
       <c r="J24" t="n">
-        <v>62.6</v>
+        <v>59.9</v>
       </c>
       <c r="K24" t="n">
-        <v>88</v>
+        <v>71</v>
       </c>
       <c r="L24" t="n">
-        <v>4.41</v>
+        <v>3.04</v>
       </c>
       <c r="M24" t="n">
-        <v>60</v>
+        <v>37.2</v>
       </c>
       <c r="N24" t="n">
-        <v>78.90000000000001</v>
+        <v>71.3</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
@@ -2646,7 +2652,7 @@
         </is>
       </c>
       <c r="P24" t="n">
-        <v>71.09999999999999</v>
+        <v>55</v>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
@@ -2678,11 +2684,11 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>CAT</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>337.51</v>
+        <v>824.16</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -2715,19 +2721,22 @@
         </is>
       </c>
       <c r="I25" t="n">
-        <v>67.2</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="J25" t="n">
-        <v>64.8</v>
+        <v>67.7</v>
       </c>
       <c r="K25" t="n">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="L25" t="n">
-        <v>2.06</v>
+        <v>2.69</v>
       </c>
       <c r="M25" t="n">
-        <v>37.3</v>
+        <v>37</v>
+      </c>
+      <c r="N25" t="n">
+        <v>68.09999999999999</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
@@ -2735,7 +2744,7 @@
         </is>
       </c>
       <c r="P25" t="n">
-        <v>63.4</v>
+        <v>74.3</v>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
@@ -2767,30 +2776,30 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>META</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>26.2</v>
+        <v>674.55</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D26" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -2800,23 +2809,23 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I26" t="n">
-        <v>65</v>
+        <v>69.3</v>
       </c>
       <c r="J26" t="n">
-        <v>43</v>
+        <v>61.4</v>
       </c>
       <c r="K26" t="n">
-        <v>78</v>
+        <v>94</v>
       </c>
       <c r="L26" t="n">
-        <v>2.57</v>
+        <v>2.66</v>
       </c>
       <c r="M26" t="n">
-        <v>26</v>
+        <v>42.4</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
@@ -2824,7 +2833,7 @@
         </is>
       </c>
       <c r="P26" t="n">
-        <v>48.9</v>
+        <v>53.5</v>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
@@ -2833,12 +2842,12 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
@@ -2856,11 +2865,11 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>PCAR</t>
+          <t>HUM</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>126.01</v>
+        <v>219.28</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -2889,34 +2898,34 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I27" t="n">
-        <v>64.90000000000001</v>
+        <v>68.3</v>
       </c>
       <c r="J27" t="n">
-        <v>57.9</v>
+        <v>73.7</v>
       </c>
       <c r="K27" t="n">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="L27" t="n">
-        <v>2.35</v>
+        <v>3.12</v>
       </c>
       <c r="M27" t="n">
-        <v>26</v>
+        <v>35.7</v>
       </c>
       <c r="N27" t="n">
-        <v>61.2</v>
+        <v>24.6</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P27" t="n">
-        <v>63.4</v>
+        <v>51.2</v>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
@@ -2948,11 +2957,11 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>FCX</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>61.54</v>
+        <v>416.86</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -2985,19 +2994,22 @@
         </is>
       </c>
       <c r="I28" t="n">
-        <v>64.2</v>
+        <v>68.2</v>
       </c>
       <c r="J28" t="n">
-        <v>45</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="K28" t="n">
-        <v>85</v>
+        <v>97</v>
       </c>
       <c r="L28" t="n">
-        <v>5.31</v>
+        <v>2.94</v>
       </c>
       <c r="M28" t="n">
-        <v>52</v>
+        <v>42.6</v>
+      </c>
+      <c r="N28" t="n">
+        <v>45.9</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
@@ -3005,7 +3017,7 @@
         </is>
       </c>
       <c r="P28" t="n">
-        <v>56.2</v>
+        <v>67.2</v>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
@@ -3014,17 +3026,17 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U28" t="inlineStr"/>
@@ -3037,11 +3049,11 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>DLR</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>127.83</v>
+        <v>194.52</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -3074,22 +3086,19 @@
         </is>
       </c>
       <c r="I29" t="n">
-        <v>61.7</v>
+        <v>68.2</v>
       </c>
       <c r="J29" t="n">
-        <v>60.7</v>
+        <v>58</v>
       </c>
       <c r="K29" t="n">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="L29" t="n">
-        <v>2.51</v>
+        <v>2.45</v>
       </c>
       <c r="M29" t="n">
-        <v>31.9</v>
-      </c>
-      <c r="N29" t="n">
-        <v>56.4</v>
+        <v>35.3</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
@@ -3097,7 +3106,7 @@
         </is>
       </c>
       <c r="P29" t="n">
-        <v>63.8</v>
+        <v>63.7</v>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
@@ -3119,21 +3128,25 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U29" t="inlineStr"/>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V29" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>BAC</t>
+          <t>PSA</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>52.21</v>
+        <v>307.8</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -3166,19 +3179,19 @@
         </is>
       </c>
       <c r="I30" t="n">
-        <v>61.2</v>
+        <v>68.2</v>
       </c>
       <c r="J30" t="n">
-        <v>54.4</v>
+        <v>62.3</v>
       </c>
       <c r="K30" t="n">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="L30" t="n">
-        <v>2.07</v>
+        <v>2.03</v>
       </c>
       <c r="M30" t="n">
-        <v>25.4</v>
+        <v>29</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
@@ -3186,7 +3199,7 @@
         </is>
       </c>
       <c r="P30" t="n">
-        <v>53.2</v>
+        <v>59.2</v>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
@@ -3195,17 +3208,17 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U30" t="inlineStr"/>
@@ -3218,11 +3231,11 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>USB</t>
+          <t>APH</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>55.97</v>
+        <v>147.74</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -3251,23 +3264,26 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I31" t="n">
-        <v>60.5</v>
+        <v>66.5</v>
       </c>
       <c r="J31" t="n">
-        <v>57.6</v>
+        <v>58.6</v>
       </c>
       <c r="K31" t="n">
-        <v>71</v>
+        <v>95</v>
       </c>
       <c r="L31" t="n">
-        <v>2.15</v>
+        <v>3.13</v>
       </c>
       <c r="M31" t="n">
-        <v>29.6</v>
+        <v>42.1</v>
+      </c>
+      <c r="N31" t="n">
+        <v>48.6</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
@@ -3275,7 +3291,7 @@
         </is>
       </c>
       <c r="P31" t="n">
-        <v>58.9</v>
+        <v>58.6</v>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
@@ -3284,17 +3300,17 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U31" t="inlineStr"/>
@@ -3307,56 +3323,59 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>328.7</v>
+        <v>486.3</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D32" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I32" t="n">
-        <v>57.9</v>
+        <v>66.3</v>
       </c>
       <c r="J32" t="n">
-        <v>50.8</v>
+        <v>69.2</v>
       </c>
       <c r="K32" t="n">
-        <v>11</v>
+        <v>85</v>
       </c>
       <c r="L32" t="n">
-        <v>1.86</v>
+        <v>2.3</v>
       </c>
       <c r="M32" t="n">
-        <v>20.3</v>
+        <v>32.7</v>
+      </c>
+      <c r="N32" t="n">
+        <v>80</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
@@ -3364,21 +3383,21 @@
         </is>
       </c>
       <c r="P32" t="n">
-        <v>60.5</v>
+        <v>66</v>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T32" t="inlineStr">
@@ -3386,11 +3405,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U32" t="inlineStr">
-        <is>
-          <t>TTM Squeeze</t>
-        </is>
-      </c>
+      <c r="U32" t="inlineStr"/>
       <c r="V32" t="inlineStr">
         <is>
           <t>No</t>
@@ -3400,94 +3415,1271 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t>WBD</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>27.01</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>66</v>
+      </c>
+      <c r="J33" t="n">
+        <v>40.2</v>
+      </c>
+      <c r="K33" t="n">
+        <v>13</v>
+      </c>
+      <c r="L33" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="M33" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="N33" t="n">
+        <v>0</v>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P33" t="n">
+        <v>59.5</v>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>FIRED</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>Squeeze Fired, Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>MET</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>77.61</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>65.59999999999999</v>
+      </c>
+      <c r="J34" t="n">
+        <v>63.4</v>
+      </c>
+      <c r="K34" t="n">
+        <v>87</v>
+      </c>
+      <c r="L34" t="n">
+        <v>1.99</v>
+      </c>
+      <c r="M34" t="n">
+        <v>23.3</v>
+      </c>
+      <c r="N34" t="n">
+        <v>50.2</v>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P34" t="n">
+        <v>54.2</v>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr"/>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>MS</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>188.71</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>65.59999999999999</v>
+      </c>
+      <c r="J35" t="n">
+        <v>66</v>
+      </c>
+      <c r="K35" t="n">
+        <v>94</v>
+      </c>
+      <c r="L35" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="M35" t="n">
+        <v>26.8</v>
+      </c>
+      <c r="N35" t="n">
+        <v>46.1</v>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P35" t="n">
+        <v>63.8</v>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr"/>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>PCAR</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>127.68</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>64.59999999999999</v>
+      </c>
+      <c r="J36" t="n">
+        <v>62</v>
+      </c>
+      <c r="K36" t="n">
+        <v>72</v>
+      </c>
+      <c r="L36" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="M36" t="n">
+        <v>34.9</v>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P36" t="n">
+        <v>64.90000000000001</v>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr"/>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>CDW</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>133.61</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>63.9</v>
+      </c>
+      <c r="J37" t="n">
+        <v>57</v>
+      </c>
+      <c r="K37" t="n">
+        <v>85</v>
+      </c>
+      <c r="L37" t="n">
+        <v>2.91</v>
+      </c>
+      <c r="M37" t="n">
+        <v>45.7</v>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P37" t="n">
+        <v>49.4</v>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U37" t="inlineStr"/>
+      <c r="V37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>FDX</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>386.48</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>63.8</v>
+      </c>
+      <c r="J38" t="n">
+        <v>59.1</v>
+      </c>
+      <c r="K38" t="n">
+        <v>79</v>
+      </c>
+      <c r="L38" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="M38" t="n">
+        <v>29</v>
+      </c>
+      <c r="N38" t="n">
+        <v>67.90000000000001</v>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P38" t="n">
+        <v>68.90000000000001</v>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr"/>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>SPG</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>200.54</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>63.6</v>
+      </c>
+      <c r="J39" t="n">
+        <v>56</v>
+      </c>
+      <c r="K39" t="n">
+        <v>91</v>
+      </c>
+      <c r="L39" t="n">
+        <v>1.73</v>
+      </c>
+      <c r="M39" t="n">
+        <v>26.6</v>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P39" t="n">
+        <v>60.7</v>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U39" t="inlineStr"/>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>BK</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>133.95</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>63.2</v>
+      </c>
+      <c r="J40" t="n">
+        <v>67</v>
+      </c>
+      <c r="K40" t="n">
+        <v>93</v>
+      </c>
+      <c r="L40" t="n">
+        <v>1.92</v>
+      </c>
+      <c r="M40" t="n">
+        <v>26.8</v>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P40" t="n">
+        <v>71.8</v>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr"/>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>LRCX</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>261.4</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>63.2</v>
+      </c>
+      <c r="J41" t="n">
+        <v>57.2</v>
+      </c>
+      <c r="K41" t="n">
+        <v>81</v>
+      </c>
+      <c r="L41" t="n">
+        <v>4.61</v>
+      </c>
+      <c r="M41" t="n">
+        <v>63.6</v>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P41" t="n">
+        <v>67.7</v>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr"/>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>NKE</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>45.09</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>62.5</v>
+      </c>
+      <c r="J42" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="K42" t="n">
+        <v>74</v>
+      </c>
+      <c r="L42" t="n">
+        <v>2.85</v>
+      </c>
+      <c r="M42" t="n">
+        <v>35.9</v>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P42" t="n">
+        <v>32.6</v>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U42" t="inlineStr"/>
+      <c r="V42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>MAR</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>363.16</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>61.4</v>
+      </c>
+      <c r="J43" t="n">
+        <v>58.3</v>
+      </c>
+      <c r="K43" t="n">
+        <v>88</v>
+      </c>
+      <c r="L43" t="n">
+        <v>2.26</v>
+      </c>
+      <c r="M43" t="n">
+        <v>29.4</v>
+      </c>
+      <c r="N43" t="n">
+        <v>65.2</v>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P43" t="n">
+        <v>64.09999999999999</v>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U43" t="inlineStr"/>
+      <c r="V43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
           <t>IDXX</t>
         </is>
       </c>
-      <c r="B33" t="n">
-        <v>557</v>
-      </c>
-      <c r="C33" t="inlineStr">
+      <c r="B44" t="n">
+        <v>571.97</v>
+      </c>
+      <c r="C44" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D33" s="2" t="inlineStr">
+      <c r="D44" s="2" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E44" t="inlineStr">
         <is>
           <t>SELL</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="F44" t="inlineStr">
         <is>
           <t>Debit Put</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
+      <c r="G44" t="inlineStr">
         <is>
           <t>30-60 DTE</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I33" t="n">
-        <v>53.8</v>
-      </c>
-      <c r="J33" t="n">
-        <v>40.8</v>
-      </c>
-      <c r="K33" t="n">
-        <v>23</v>
-      </c>
-      <c r="L33" t="n">
-        <v>3.05</v>
-      </c>
-      <c r="M33" t="n">
-        <v>27.6</v>
-      </c>
-      <c r="N33" t="n">
-        <v>19.2</v>
-      </c>
-      <c r="O33" t="inlineStr">
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
+        <v>60.2</v>
+      </c>
+      <c r="J44" t="n">
+        <v>46.7</v>
+      </c>
+      <c r="K44" t="n">
+        <v>12</v>
+      </c>
+      <c r="L44" t="n">
+        <v>3.04</v>
+      </c>
+      <c r="M44" t="n">
+        <v>43.4</v>
+      </c>
+      <c r="O44" t="inlineStr">
         <is>
           <t>Bearish</t>
         </is>
       </c>
-      <c r="P33" t="n">
-        <v>38.9</v>
-      </c>
-      <c r="Q33" t="inlineStr">
+      <c r="P44" t="n">
+        <v>41.5</v>
+      </c>
+      <c r="Q44" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
       </c>
-      <c r="R33" t="inlineStr">
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
+      <c r="V44" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>328.83</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Debit Call</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I45" t="n">
+        <v>58</v>
+      </c>
+      <c r="J45" t="n">
+        <v>51.1</v>
+      </c>
+      <c r="K45" t="n">
+        <v>3</v>
+      </c>
+      <c r="L45" t="n">
+        <v>1.97</v>
+      </c>
+      <c r="M45" t="n">
+        <v>22.7</v>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P45" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="S33" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T33" t="inlineStr">
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>128.35</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I46" t="n">
+        <v>56.2</v>
+      </c>
+      <c r="J46" t="n">
+        <v>61.7</v>
+      </c>
+      <c r="K46" t="n">
+        <v>92</v>
+      </c>
+      <c r="L46" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="M46" t="n">
+        <v>34.3</v>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P46" t="n">
+        <v>64.2</v>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T46" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="U33" t="inlineStr">
-        <is>
-          <t>TTM Squeeze</t>
-        </is>
-      </c>
-      <c r="V33" t="inlineStr">
+      <c r="U46" t="inlineStr"/>
+      <c r="V46" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Scan 28.04.2026 16:12 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V46"/>
+  <dimension ref="A1:V51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -577,11 +577,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>INTC</t>
+          <t>TXN</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>83.48999999999999</v>
+        <v>266.77</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,22 +614,19 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>91.90000000000001</v>
+        <v>92.5</v>
       </c>
       <c r="J2" t="n">
-        <v>82.59999999999999</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="K2" t="n">
         <v>99</v>
       </c>
       <c r="L2" t="n">
-        <v>6.26</v>
+        <v>4.12</v>
       </c>
       <c r="M2" t="n">
-        <v>92.8</v>
-      </c>
-      <c r="N2" t="n">
-        <v>98.09999999999999</v>
+        <v>39.9</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -637,7 +634,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>83.09999999999999</v>
+        <v>71.8</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -669,11 +666,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>156.38</v>
+        <v>320.82</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -706,22 +703,22 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>87</v>
+        <v>89.8</v>
       </c>
       <c r="J3" t="n">
-        <v>75.8</v>
+        <v>72.3</v>
       </c>
       <c r="K3" t="n">
         <v>98</v>
       </c>
       <c r="L3" t="n">
-        <v>5.64</v>
+        <v>5.68</v>
       </c>
       <c r="M3" t="n">
-        <v>65.90000000000001</v>
+        <v>64.7</v>
       </c>
       <c r="N3" t="n">
-        <v>65.2</v>
+        <v>49.7</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -729,7 +726,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>78.5</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -765,11 +762,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ADI</t>
+          <t>INTC</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>389.03</v>
+        <v>82.39</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -802,22 +799,19 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>86.3</v>
+        <v>89.8</v>
       </c>
       <c r="J4" t="n">
-        <v>68.7</v>
+        <v>77.7</v>
       </c>
       <c r="K4" t="n">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="L4" t="n">
-        <v>3.08</v>
+        <v>6.18</v>
       </c>
       <c r="M4" t="n">
-        <v>37.3</v>
-      </c>
-      <c r="N4" t="n">
-        <v>96.7</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -825,7 +819,7 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>72.40000000000001</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -857,59 +851,56 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>REGN</t>
+          <t>SNPS</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>747.91</v>
+        <v>482.12</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>85.09999999999999</v>
+        <v>87.90000000000001</v>
       </c>
       <c r="J5" t="n">
-        <v>46.7</v>
+        <v>62.7</v>
       </c>
       <c r="K5" t="n">
-        <v>2</v>
+        <v>97</v>
       </c>
       <c r="L5" t="n">
-        <v>2.39</v>
+        <v>4.16</v>
       </c>
       <c r="M5" t="n">
-        <v>22.4</v>
-      </c>
-      <c r="N5" t="n">
-        <v>0.1</v>
+        <v>56.4</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -917,21 +908,21 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>53.7</v>
+        <v>54.7</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -941,23 +932,23 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>TTM Squeeze</t>
+          <t>Divergence</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>GFS</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>59.88</v>
+        <v>197.76</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -990,22 +981,22 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>83.90000000000001</v>
+        <v>87.90000000000001</v>
       </c>
       <c r="J6" t="n">
-        <v>73.09999999999999</v>
+        <v>62.5</v>
       </c>
       <c r="K6" t="n">
         <v>99</v>
       </c>
       <c r="L6" t="n">
-        <v>4.91</v>
+        <v>8.23</v>
       </c>
       <c r="M6" t="n">
-        <v>56.4</v>
+        <v>94.7</v>
       </c>
       <c r="N6" t="n">
-        <v>64.7</v>
+        <v>100</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -1013,7 +1004,7 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>72.40000000000001</v>
+        <v>64.2</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1022,17 +1013,17 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1049,11 +1040,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>421.83</v>
+        <v>93.03</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1086,27 +1077,27 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>82.2</v>
+        <v>87.5</v>
       </c>
       <c r="J7" t="n">
-        <v>61.6</v>
+        <v>74.8</v>
       </c>
       <c r="K7" t="n">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="L7" t="n">
-        <v>2.57</v>
+        <v>4.53</v>
       </c>
       <c r="M7" t="n">
-        <v>38.6</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>48.1</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1128,10 +1119,14 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr"/>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1142,7 +1137,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>349.99</v>
+        <v>367.3</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1175,22 +1170,22 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>81.7</v>
+        <v>82.8</v>
       </c>
       <c r="J8" t="n">
-        <v>76.40000000000001</v>
+        <v>84.7</v>
       </c>
       <c r="K8" t="n">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="L8" t="n">
-        <v>2.84</v>
+        <v>2.81</v>
       </c>
       <c r="M8" t="n">
-        <v>40.3</v>
+        <v>40.7</v>
       </c>
       <c r="N8" t="n">
-        <v>37.8</v>
+        <v>38.4</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1198,7 +1193,7 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>59.3</v>
+        <v>63</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1230,11 +1225,11 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>MCHP</t>
+          <t>ADI</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>86.04000000000001</v>
+        <v>383.49</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1270,19 +1265,19 @@
         <v>81</v>
       </c>
       <c r="J9" t="n">
-        <v>71.40000000000001</v>
+        <v>64.7</v>
       </c>
       <c r="K9" t="n">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="L9" t="n">
-        <v>4.05</v>
+        <v>3.13</v>
       </c>
       <c r="M9" t="n">
-        <v>46.3</v>
+        <v>37.7</v>
       </c>
       <c r="N9" t="n">
-        <v>66</v>
+        <v>98.5</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1290,7 +1285,7 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>65.59999999999999</v>
+        <v>70.2</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1299,38 +1294,34 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>591.38</v>
+        <v>209.69</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1363,19 +1354,22 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J10" t="n">
-        <v>62</v>
+        <v>66.3</v>
       </c>
       <c r="K10" t="n">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="L10" t="n">
-        <v>2.8</v>
+        <v>3.08</v>
       </c>
       <c r="M10" t="n">
-        <v>29.5</v>
+        <v>36.3</v>
+      </c>
+      <c r="N10" t="n">
+        <v>59.9</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1383,7 +1377,7 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>56.2</v>
+        <v>65.7</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1405,78 +1399,82 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U10" t="inlineStr"/>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>LIN</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>508.29</v>
+        <v>427.75</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>79.59999999999999</v>
+        <v>80.8</v>
       </c>
       <c r="J11" t="n">
-        <v>58.9</v>
+        <v>64.8</v>
       </c>
       <c r="K11" t="n">
-        <v>3</v>
+        <v>87</v>
       </c>
       <c r="L11" t="n">
-        <v>1.74</v>
+        <v>2.46</v>
       </c>
       <c r="M11" t="n">
-        <v>24.9</v>
+        <v>39.4</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>63.8</v>
+        <v>49.7</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
@@ -1491,14 +1489,10 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U11" t="inlineStr">
-        <is>
-          <t>TTM Squeeze</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr"/>
       <c r="V11" t="inlineStr">
         <is>
           <t>No</t>
@@ -1508,11 +1502,11 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>261.04</v>
+        <v>151.56</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1545,19 +1539,22 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>79.3</v>
+        <v>80</v>
       </c>
       <c r="J12" t="n">
-        <v>75.8</v>
+        <v>69.7</v>
       </c>
       <c r="K12" t="n">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="L12" t="n">
-        <v>2.46</v>
+        <v>6.05</v>
       </c>
       <c r="M12" t="n">
-        <v>40.8</v>
+        <v>67.09999999999999</v>
+      </c>
+      <c r="N12" t="n">
+        <v>67.59999999999999</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1565,7 +1562,7 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>64.5</v>
+        <v>75</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1574,34 +1571,38 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U12" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>XLK</t>
+          <t>GFS</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>159.49</v>
+        <v>58.82</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -1634,19 +1635,22 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>78.7</v>
+        <v>79.2</v>
       </c>
       <c r="J13" t="n">
-        <v>74.09999999999999</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="K13" t="n">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="L13" t="n">
-        <v>1.85</v>
+        <v>4.88</v>
       </c>
       <c r="M13" t="n">
-        <v>28.1</v>
+        <v>56.1</v>
+      </c>
+      <c r="N13" t="n">
+        <v>64</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1654,7 +1658,7 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>69</v>
+        <v>70.5</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1686,11 +1690,11 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ABNB</t>
+          <t>MU</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>142.71</v>
+        <v>495.15</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -1723,19 +1727,19 @@
         </is>
       </c>
       <c r="I14" t="n">
-        <v>77.3</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="J14" t="n">
-        <v>64.5</v>
+        <v>63.3</v>
       </c>
       <c r="K14" t="n">
-        <v>99</v>
+        <v>90</v>
       </c>
       <c r="L14" t="n">
-        <v>3.03</v>
+        <v>5.71</v>
       </c>
       <c r="M14" t="n">
-        <v>52.4</v>
+        <v>75.2</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1743,7 +1747,7 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>60.5</v>
+        <v>71.3</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1765,21 +1769,25 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U14" t="inlineStr"/>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>XLK</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>662.1900000000001</v>
+        <v>156.82</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1812,19 +1820,19 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>77.2</v>
+        <v>77.3</v>
       </c>
       <c r="J15" t="n">
-        <v>73.5</v>
+        <v>66.5</v>
       </c>
       <c r="K15" t="n">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="L15" t="n">
-        <v>1.45</v>
+        <v>2.03</v>
       </c>
       <c r="M15" t="n">
-        <v>20.7</v>
+        <v>29.2</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1832,7 +1840,7 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>66.40000000000001</v>
+        <v>65.5</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1854,21 +1862,25 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U15" t="inlineStr"/>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>713.1900000000001</v>
+        <v>595.66</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -1901,19 +1913,19 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>74.59999999999999</v>
+        <v>76.7</v>
       </c>
       <c r="J16" t="n">
-        <v>69.7</v>
+        <v>63.4</v>
       </c>
       <c r="K16" t="n">
-        <v>96</v>
+        <v>85</v>
       </c>
       <c r="L16" t="n">
-        <v>1.02</v>
+        <v>2.68</v>
       </c>
       <c r="M16" t="n">
-        <v>15.8</v>
+        <v>29.1</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -1921,7 +1933,7 @@
         </is>
       </c>
       <c r="P16" t="n">
-        <v>64.3</v>
+        <v>57</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1953,11 +1965,11 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>KLAC</t>
+          <t>MCHP</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>1883.09</v>
+        <v>84.81</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -1990,19 +2002,22 @@
         </is>
       </c>
       <c r="I17" t="n">
-        <v>74.3</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="J17" t="n">
-        <v>68.7</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="K17" t="n">
-        <v>97</v>
+        <v>88</v>
       </c>
       <c r="L17" t="n">
-        <v>3.47</v>
+        <v>4.05</v>
       </c>
       <c r="M17" t="n">
-        <v>54.4</v>
+        <v>46.3</v>
+      </c>
+      <c r="N17" t="n">
+        <v>65.90000000000001</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -2010,7 +2025,7 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>72.2</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -2042,11 +2057,11 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ETN</t>
+          <t>NXPI</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>418.67</v>
+        <v>229.11</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -2079,19 +2094,22 @@
         </is>
       </c>
       <c r="I18" t="n">
-        <v>73.59999999999999</v>
+        <v>75.40000000000001</v>
       </c>
       <c r="J18" t="n">
-        <v>67.7</v>
+        <v>61.5</v>
       </c>
       <c r="K18" t="n">
-        <v>98</v>
+        <v>81</v>
       </c>
       <c r="L18" t="n">
-        <v>2.77</v>
+        <v>3.63</v>
       </c>
       <c r="M18" t="n">
-        <v>42</v>
+        <v>35.4</v>
+      </c>
+      <c r="N18" t="n">
+        <v>58</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -2099,7 +2117,7 @@
         </is>
       </c>
       <c r="P18" t="n">
-        <v>66.59999999999999</v>
+        <v>55.1</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -2121,21 +2139,25 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U18" t="inlineStr"/>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>210.68</v>
+        <v>655.12</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -2168,19 +2190,22 @@
         </is>
       </c>
       <c r="I19" t="n">
-        <v>73.5</v>
+        <v>74.3</v>
       </c>
       <c r="J19" t="n">
-        <v>73.09999999999999</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="K19" t="n">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="L19" t="n">
-        <v>2.61</v>
+        <v>1.49</v>
       </c>
       <c r="M19" t="n">
-        <v>43.3</v>
+        <v>21.9</v>
+      </c>
+      <c r="N19" t="n">
+        <v>97.59999999999999</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -2188,7 +2213,7 @@
         </is>
       </c>
       <c r="P19" t="n">
-        <v>66.09999999999999</v>
+        <v>63.9</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -2220,11 +2245,11 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>350.24</v>
+        <v>260.18</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -2257,22 +2282,22 @@
         </is>
       </c>
       <c r="I20" t="n">
-        <v>73.2</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="J20" t="n">
-        <v>71.7</v>
+        <v>74.5</v>
       </c>
       <c r="K20" t="n">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="L20" t="n">
-        <v>2.25</v>
+        <v>2.37</v>
       </c>
       <c r="M20" t="n">
-        <v>33.1</v>
+        <v>33.4</v>
       </c>
       <c r="N20" t="n">
-        <v>86.09999999999999</v>
+        <v>56.7</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -2280,7 +2305,7 @@
         </is>
       </c>
       <c r="P20" t="n">
-        <v>67</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
@@ -2312,11 +2337,11 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>GOOG</t>
+          <t>KLAC</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>348.3</v>
+        <v>1831.57</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -2349,22 +2374,19 @@
         </is>
       </c>
       <c r="I21" t="n">
-        <v>72.2</v>
+        <v>71.7</v>
       </c>
       <c r="J21" t="n">
-        <v>72.5</v>
+        <v>62.3</v>
       </c>
       <c r="K21" t="n">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="L21" t="n">
-        <v>2.19</v>
+        <v>4.05</v>
       </c>
       <c r="M21" t="n">
-        <v>31.4</v>
-      </c>
-      <c r="N21" t="n">
-        <v>80.3</v>
+        <v>53.7</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
@@ -2372,7 +2394,7 @@
         </is>
       </c>
       <c r="P21" t="n">
-        <v>66.7</v>
+        <v>68.8</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
@@ -2381,17 +2403,17 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U21" t="inlineStr"/>
@@ -2404,11 +2426,11 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>IWM</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>276.71</v>
+        <v>348.98</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -2441,22 +2463,22 @@
         </is>
       </c>
       <c r="I22" t="n">
-        <v>72.2</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="J22" t="n">
-        <v>69.5</v>
+        <v>70.2</v>
       </c>
       <c r="K22" t="n">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="L22" t="n">
-        <v>1.57</v>
+        <v>2.24</v>
       </c>
       <c r="M22" t="n">
-        <v>21.4</v>
+        <v>33.2</v>
       </c>
       <c r="N22" t="n">
-        <v>72.40000000000001</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
@@ -2464,7 +2486,7 @@
         </is>
       </c>
       <c r="P22" t="n">
-        <v>67.5</v>
+        <v>66.7</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
@@ -2496,11 +2518,11 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ANET</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>170.8</v>
+        <v>710.27</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -2533,22 +2555,22 @@
         </is>
       </c>
       <c r="I23" t="n">
-        <v>72.09999999999999</v>
+        <v>71.3</v>
       </c>
       <c r="J23" t="n">
-        <v>66.59999999999999</v>
+        <v>66</v>
       </c>
       <c r="K23" t="n">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="L23" t="n">
-        <v>3.96</v>
+        <v>1.02</v>
       </c>
       <c r="M23" t="n">
-        <v>56.8</v>
+        <v>17.2</v>
       </c>
       <c r="N23" t="n">
-        <v>69.59999999999999</v>
+        <v>91.09999999999999</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -2556,7 +2578,7 @@
         </is>
       </c>
       <c r="P23" t="n">
-        <v>65.8</v>
+        <v>63.1</v>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
@@ -2578,25 +2600,21 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U23" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U23" t="inlineStr"/>
       <c r="V23" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>BA</t>
+          <t>HUM</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>230.38</v>
+        <v>230.29</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -2629,30 +2647,30 @@
         </is>
       </c>
       <c r="I24" t="n">
-        <v>72</v>
+        <v>71.2</v>
       </c>
       <c r="J24" t="n">
-        <v>59.9</v>
+        <v>78.7</v>
       </c>
       <c r="K24" t="n">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="L24" t="n">
-        <v>3.04</v>
+        <v>3.2</v>
       </c>
       <c r="M24" t="n">
-        <v>37.2</v>
+        <v>36.7</v>
       </c>
       <c r="N24" t="n">
-        <v>71.3</v>
+        <v>26.5</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P24" t="n">
-        <v>55</v>
+        <v>54.6</v>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
@@ -2684,11 +2702,11 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CAT</t>
+          <t>ANET</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>824.16</v>
+        <v>163</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -2721,22 +2739,19 @@
         </is>
       </c>
       <c r="I25" t="n">
-        <v>69.59999999999999</v>
+        <v>70.5</v>
       </c>
       <c r="J25" t="n">
-        <v>67.7</v>
+        <v>58.2</v>
       </c>
       <c r="K25" t="n">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="L25" t="n">
-        <v>2.69</v>
+        <v>4.43</v>
       </c>
       <c r="M25" t="n">
-        <v>37</v>
-      </c>
-      <c r="N25" t="n">
-        <v>68.09999999999999</v>
+        <v>64.2</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
@@ -2744,7 +2759,7 @@
         </is>
       </c>
       <c r="P25" t="n">
-        <v>74.3</v>
+        <v>61.2</v>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
@@ -2753,34 +2768,38 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U25" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V25" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>PSA</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>674.55</v>
+        <v>307.18</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -2809,23 +2828,26 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I26" t="n">
-        <v>69.3</v>
+        <v>70.2</v>
       </c>
       <c r="J26" t="n">
-        <v>61.4</v>
+        <v>60.9</v>
       </c>
       <c r="K26" t="n">
-        <v>94</v>
+        <v>76</v>
       </c>
       <c r="L26" t="n">
-        <v>2.66</v>
+        <v>2.33</v>
       </c>
       <c r="M26" t="n">
-        <v>42.4</v>
+        <v>27.3</v>
+      </c>
+      <c r="N26" t="n">
+        <v>96.40000000000001</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
@@ -2833,7 +2855,7 @@
         </is>
       </c>
       <c r="P26" t="n">
-        <v>53.5</v>
+        <v>58.9</v>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
@@ -2865,11 +2887,11 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>HUM</t>
+          <t>ABNB</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>219.28</v>
+        <v>140.27</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -2898,34 +2920,31 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I27" t="n">
-        <v>68.3</v>
+        <v>69.2</v>
       </c>
       <c r="J27" t="n">
-        <v>73.7</v>
+        <v>59.1</v>
       </c>
       <c r="K27" t="n">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="L27" t="n">
-        <v>3.12</v>
+        <v>3</v>
       </c>
       <c r="M27" t="n">
-        <v>35.7</v>
-      </c>
-      <c r="N27" t="n">
-        <v>24.6</v>
+        <v>49.6</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P27" t="n">
-        <v>51.2</v>
+        <v>58.1</v>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
@@ -2934,17 +2953,17 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U27" t="inlineStr"/>
@@ -2957,11 +2976,11 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>CSCO</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>416.86</v>
+        <v>86.94</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -2994,22 +3013,19 @@
         </is>
       </c>
       <c r="I28" t="n">
-        <v>68.2</v>
+        <v>69</v>
       </c>
       <c r="J28" t="n">
-        <v>73.40000000000001</v>
+        <v>60.5</v>
       </c>
       <c r="K28" t="n">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="L28" t="n">
-        <v>2.94</v>
+        <v>2.26</v>
       </c>
       <c r="M28" t="n">
-        <v>42.6</v>
-      </c>
-      <c r="N28" t="n">
-        <v>45.9</v>
+        <v>40.2</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
@@ -3017,7 +3033,7 @@
         </is>
       </c>
       <c r="P28" t="n">
-        <v>67.2</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
@@ -3026,17 +3042,17 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U28" t="inlineStr"/>
@@ -3049,11 +3065,11 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>DLR</t>
+          <t>GOOG</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>194.52</v>
+        <v>346.5</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -3086,19 +3102,19 @@
         </is>
       </c>
       <c r="I29" t="n">
-        <v>68.2</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="J29" t="n">
-        <v>58</v>
+        <v>70.2</v>
       </c>
       <c r="K29" t="n">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="L29" t="n">
-        <v>2.45</v>
+        <v>2.17</v>
       </c>
       <c r="M29" t="n">
-        <v>35.3</v>
+        <v>37.4</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
@@ -3106,7 +3122,7 @@
         </is>
       </c>
       <c r="P29" t="n">
-        <v>63.7</v>
+        <v>66.3</v>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
@@ -3115,83 +3131,79 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U29" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr"/>
       <c r="V29" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>PSA</t>
+          <t>PEP</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>307.8</v>
+        <v>157.41</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I30" t="n">
-        <v>68.2</v>
+        <v>68.3</v>
       </c>
       <c r="J30" t="n">
-        <v>62.3</v>
+        <v>53.5</v>
       </c>
       <c r="K30" t="n">
-        <v>87</v>
+        <v>2</v>
       </c>
       <c r="L30" t="n">
-        <v>2.03</v>
+        <v>1.91</v>
       </c>
       <c r="M30" t="n">
-        <v>29</v>
+        <v>23.2</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
@@ -3199,11 +3211,11 @@
         </is>
       </c>
       <c r="P30" t="n">
-        <v>59.2</v>
+        <v>54.9</v>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
@@ -3213,15 +3225,19 @@
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U30" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V30" t="inlineStr">
         <is>
           <t>No</t>
@@ -3231,11 +3247,11 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>APH</t>
+          <t>IWM</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>147.74</v>
+        <v>273.62</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -3268,22 +3284,19 @@
         </is>
       </c>
       <c r="I31" t="n">
-        <v>66.5</v>
+        <v>67</v>
       </c>
       <c r="J31" t="n">
-        <v>58.6</v>
+        <v>62.8</v>
       </c>
       <c r="K31" t="n">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="L31" t="n">
-        <v>3.13</v>
+        <v>1.58</v>
       </c>
       <c r="M31" t="n">
-        <v>42.1</v>
-      </c>
-      <c r="N31" t="n">
-        <v>48.6</v>
+        <v>22.5</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
@@ -3291,7 +3304,7 @@
         </is>
       </c>
       <c r="P31" t="n">
-        <v>58.6</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
@@ -3300,17 +3313,17 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U31" t="inlineStr"/>
@@ -3323,11 +3336,11 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>TT</t>
+          <t>ETN</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>486.3</v>
+        <v>411.33</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -3360,22 +3373,22 @@
         </is>
       </c>
       <c r="I32" t="n">
-        <v>66.3</v>
+        <v>66.7</v>
       </c>
       <c r="J32" t="n">
-        <v>69.2</v>
+        <v>61.8</v>
       </c>
       <c r="K32" t="n">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="L32" t="n">
-        <v>2.3</v>
+        <v>2.96</v>
       </c>
       <c r="M32" t="n">
-        <v>32.7</v>
+        <v>34.9</v>
       </c>
       <c r="N32" t="n">
-        <v>80</v>
+        <v>76.2</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
@@ -3383,7 +3396,7 @@
         </is>
       </c>
       <c r="P32" t="n">
-        <v>66</v>
+        <v>63.7</v>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
@@ -3392,17 +3405,17 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U32" t="inlineStr"/>
@@ -3415,15 +3428,15 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>WBD</t>
+          <t>BLK</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>27.01</v>
+        <v>1054.21</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -3438,36 +3451,36 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I33" t="n">
-        <v>66</v>
+        <v>66.5</v>
       </c>
       <c r="J33" t="n">
-        <v>40.2</v>
+        <v>59.6</v>
       </c>
       <c r="K33" t="n">
-        <v>13</v>
+        <v>80</v>
       </c>
       <c r="L33" t="n">
-        <v>0.82</v>
+        <v>2.34</v>
       </c>
       <c r="M33" t="n">
-        <v>10.4</v>
+        <v>27.7</v>
       </c>
       <c r="N33" t="n">
-        <v>0</v>
+        <v>61.1</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
@@ -3475,33 +3488,29 @@
         </is>
       </c>
       <c r="P33" t="n">
-        <v>59.5</v>
+        <v>52.3</v>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>FIRED</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U33" t="inlineStr">
-        <is>
-          <t>Squeeze Fired, Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr"/>
       <c r="V33" t="inlineStr">
         <is>
           <t>No</t>
@@ -3511,11 +3520,11 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>MET</t>
+          <t>APH</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>77.61</v>
+        <v>144.03</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -3548,22 +3557,19 @@
         </is>
       </c>
       <c r="I34" t="n">
-        <v>65.59999999999999</v>
+        <v>65.5</v>
       </c>
       <c r="J34" t="n">
-        <v>63.4</v>
+        <v>52.8</v>
       </c>
       <c r="K34" t="n">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="L34" t="n">
-        <v>1.99</v>
+        <v>3.37</v>
       </c>
       <c r="M34" t="n">
-        <v>23.3</v>
-      </c>
-      <c r="N34" t="n">
-        <v>50.2</v>
+        <v>54.7</v>
       </c>
       <c r="O34" t="inlineStr">
         <is>
@@ -3571,7 +3577,7 @@
         </is>
       </c>
       <c r="P34" t="n">
-        <v>54.2</v>
+        <v>55.9</v>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
@@ -3580,17 +3586,17 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U34" t="inlineStr"/>
@@ -3603,11 +3609,11 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>MET</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>188.71</v>
+        <v>78.87</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -3640,22 +3646,19 @@
         </is>
       </c>
       <c r="I35" t="n">
-        <v>65.59999999999999</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="J35" t="n">
-        <v>66</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="K35" t="n">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="L35" t="n">
-        <v>2.3</v>
+        <v>1.91</v>
       </c>
       <c r="M35" t="n">
-        <v>26.8</v>
-      </c>
-      <c r="N35" t="n">
-        <v>46.1</v>
+        <v>26.9</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
@@ -3663,7 +3666,7 @@
         </is>
       </c>
       <c r="P35" t="n">
-        <v>63.8</v>
+        <v>56.1</v>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
@@ -3695,11 +3698,11 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>PCAR</t>
+          <t>META</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>127.68</v>
+        <v>666.92</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -3728,23 +3731,23 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I36" t="n">
-        <v>64.59999999999999</v>
+        <v>65.2</v>
       </c>
       <c r="J36" t="n">
-        <v>62</v>
+        <v>57.9</v>
       </c>
       <c r="K36" t="n">
-        <v>72</v>
+        <v>90</v>
       </c>
       <c r="L36" t="n">
-        <v>2.38</v>
+        <v>2.59</v>
       </c>
       <c r="M36" t="n">
-        <v>34.9</v>
+        <v>43.9</v>
       </c>
       <c r="O36" t="inlineStr">
         <is>
@@ -3752,7 +3755,7 @@
         </is>
       </c>
       <c r="P36" t="n">
-        <v>64.90000000000001</v>
+        <v>52.6</v>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
@@ -3784,11 +3787,11 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CDW</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>133.61</v>
+        <v>189.55</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -3821,27 +3824,27 @@
         </is>
       </c>
       <c r="I37" t="n">
-        <v>63.9</v>
+        <v>63.4</v>
       </c>
       <c r="J37" t="n">
-        <v>57</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="K37" t="n">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="L37" t="n">
-        <v>2.91</v>
+        <v>2.29</v>
       </c>
       <c r="M37" t="n">
-        <v>45.7</v>
+        <v>31.1</v>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P37" t="n">
-        <v>49.4</v>
+        <v>64.2</v>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
@@ -3850,17 +3853,17 @@
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U37" t="inlineStr"/>
@@ -3873,11 +3876,11 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>FDX</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>386.48</v>
+        <v>396.41</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -3906,26 +3909,23 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I38" t="n">
-        <v>63.8</v>
+        <v>63.2</v>
       </c>
       <c r="J38" t="n">
-        <v>59.1</v>
+        <v>60.4</v>
       </c>
       <c r="K38" t="n">
-        <v>79</v>
+        <v>93</v>
       </c>
       <c r="L38" t="n">
-        <v>2.38</v>
+        <v>3.47</v>
       </c>
       <c r="M38" t="n">
-        <v>29</v>
-      </c>
-      <c r="N38" t="n">
-        <v>67.90000000000001</v>
+        <v>48.6</v>
       </c>
       <c r="O38" t="inlineStr">
         <is>
@@ -3933,7 +3933,7 @@
         </is>
       </c>
       <c r="P38" t="n">
-        <v>68.90000000000001</v>
+        <v>61.6</v>
       </c>
       <c r="Q38" t="inlineStr">
         <is>
@@ -3942,34 +3942,38 @@
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U38" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V38" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>SPG</t>
+          <t>CAT</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>200.54</v>
+        <v>815.13</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -3998,23 +4002,26 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I39" t="n">
-        <v>63.6</v>
+        <v>62.8</v>
       </c>
       <c r="J39" t="n">
-        <v>56</v>
+        <v>63.9</v>
       </c>
       <c r="K39" t="n">
-        <v>91</v>
+        <v>78</v>
       </c>
       <c r="L39" t="n">
-        <v>1.73</v>
+        <v>2.75</v>
       </c>
       <c r="M39" t="n">
-        <v>26.6</v>
+        <v>37.4</v>
+      </c>
+      <c r="N39" t="n">
+        <v>69.59999999999999</v>
       </c>
       <c r="O39" t="inlineStr">
         <is>
@@ -4022,7 +4029,7 @@
         </is>
       </c>
       <c r="P39" t="n">
-        <v>60.7</v>
+        <v>72.3</v>
       </c>
       <c r="Q39" t="inlineStr">
         <is>
@@ -4031,17 +4038,17 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U39" t="inlineStr"/>
@@ -4054,11 +4061,11 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>BK</t>
+          <t>DLR</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>133.95</v>
+        <v>192.9</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -4091,19 +4098,19 @@
         </is>
       </c>
       <c r="I40" t="n">
-        <v>63.2</v>
+        <v>61.5</v>
       </c>
       <c r="J40" t="n">
-        <v>67</v>
+        <v>54.3</v>
       </c>
       <c r="K40" t="n">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="L40" t="n">
-        <v>1.92</v>
+        <v>2.48</v>
       </c>
       <c r="M40" t="n">
-        <v>26.8</v>
+        <v>33.2</v>
       </c>
       <c r="O40" t="inlineStr">
         <is>
@@ -4111,7 +4118,7 @@
         </is>
       </c>
       <c r="P40" t="n">
-        <v>71.8</v>
+        <v>62.3</v>
       </c>
       <c r="Q40" t="inlineStr">
         <is>
@@ -4143,11 +4150,11 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>LRCX</t>
+          <t>PCAR</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>261.4</v>
+        <v>119.77</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -4176,23 +4183,26 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I41" t="n">
-        <v>63.2</v>
+        <v>60.7</v>
       </c>
       <c r="J41" t="n">
-        <v>57.2</v>
+        <v>43.2</v>
       </c>
       <c r="K41" t="n">
-        <v>81</v>
+        <v>56</v>
       </c>
       <c r="L41" t="n">
-        <v>4.61</v>
+        <v>3.22</v>
       </c>
       <c r="M41" t="n">
-        <v>63.6</v>
+        <v>31.1</v>
+      </c>
+      <c r="N41" t="n">
+        <v>100</v>
       </c>
       <c r="O41" t="inlineStr">
         <is>
@@ -4200,7 +4210,7 @@
         </is>
       </c>
       <c r="P41" t="n">
-        <v>67.7</v>
+        <v>54.5</v>
       </c>
       <c r="Q41" t="inlineStr">
         <is>
@@ -4222,40 +4232,44 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U41" t="inlineStr"/>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V41" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>NKE</t>
+          <t>BK</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>45.09</v>
+        <v>133.95</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D42" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -4265,31 +4279,34 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I42" t="n">
-        <v>62.5</v>
+        <v>59.9</v>
       </c>
       <c r="J42" t="n">
-        <v>37.5</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="K42" t="n">
-        <v>74</v>
+        <v>90</v>
       </c>
       <c r="L42" t="n">
-        <v>2.85</v>
+        <v>1.89</v>
       </c>
       <c r="M42" t="n">
-        <v>35.9</v>
+        <v>19.1</v>
+      </c>
+      <c r="N42" t="n">
+        <v>32.1</v>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P42" t="n">
-        <v>32.6</v>
+        <v>72.3</v>
       </c>
       <c r="Q42" t="inlineStr">
         <is>
@@ -4298,12 +4315,12 @@
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S42" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T42" t="inlineStr">
@@ -4321,11 +4338,11 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>363.16</v>
+        <v>479.44</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -4354,26 +4371,23 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I43" t="n">
-        <v>61.4</v>
+        <v>59.9</v>
       </c>
       <c r="J43" t="n">
-        <v>58.3</v>
+        <v>63.3</v>
       </c>
       <c r="K43" t="n">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="L43" t="n">
-        <v>2.26</v>
+        <v>2.3</v>
       </c>
       <c r="M43" t="n">
-        <v>29.4</v>
-      </c>
-      <c r="N43" t="n">
-        <v>65.2</v>
+        <v>34.7</v>
       </c>
       <c r="O43" t="inlineStr">
         <is>
@@ -4381,7 +4395,7 @@
         </is>
       </c>
       <c r="P43" t="n">
-        <v>64.09999999999999</v>
+        <v>63.5</v>
       </c>
       <c r="Q43" t="inlineStr">
         <is>
@@ -4390,17 +4404,17 @@
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U43" t="inlineStr"/>
@@ -4413,15 +4427,15 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>IDXX</t>
+          <t>LRCX</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>571.97</v>
+        <v>247.3</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -4436,67 +4450,66 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I44" t="n">
-        <v>60.2</v>
+        <v>58.7</v>
       </c>
       <c r="J44" t="n">
-        <v>46.7</v>
+        <v>49.6</v>
       </c>
       <c r="K44" t="n">
-        <v>12</v>
+        <v>75</v>
       </c>
       <c r="L44" t="n">
-        <v>3.04</v>
+        <v>5.11</v>
       </c>
       <c r="M44" t="n">
-        <v>43.4</v>
+        <v>61.9</v>
+      </c>
+      <c r="N44" t="n">
+        <v>82.90000000000001</v>
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P44" t="n">
-        <v>41.5</v>
+        <v>62.1</v>
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S44" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U44" t="inlineStr">
-        <is>
-          <t>TTM Squeeze</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U44" t="inlineStr"/>
       <c r="V44" t="inlineStr">
         <is>
           <t>No</t>
@@ -4506,56 +4519,59 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>FDX</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>328.83</v>
+        <v>386.22</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D45" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I45" t="n">
-        <v>58</v>
+        <v>57.1</v>
       </c>
       <c r="J45" t="n">
-        <v>51.1</v>
+        <v>58.8</v>
       </c>
       <c r="K45" t="n">
-        <v>3</v>
+        <v>69</v>
       </c>
       <c r="L45" t="n">
-        <v>1.97</v>
+        <v>2.31</v>
       </c>
       <c r="M45" t="n">
-        <v>22.7</v>
+        <v>29</v>
+      </c>
+      <c r="N45" t="n">
+        <v>68</v>
       </c>
       <c r="O45" t="inlineStr">
         <is>
@@ -4563,11 +4579,11 @@
         </is>
       </c>
       <c r="P45" t="n">
-        <v>60</v>
+        <v>68.7</v>
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R45" t="inlineStr">
@@ -4582,14 +4598,10 @@
       </c>
       <c r="T45" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U45" t="inlineStr">
-        <is>
-          <t>TTM Squeeze</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U45" t="inlineStr"/>
       <c r="V45" t="inlineStr">
         <is>
           <t>No</t>
@@ -4599,11 +4611,11 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>CDW</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>128.35</v>
+        <v>132.45</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -4632,31 +4644,31 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I46" t="n">
-        <v>56.2</v>
+        <v>56.7</v>
       </c>
       <c r="J46" t="n">
-        <v>61.7</v>
+        <v>54.7</v>
       </c>
       <c r="K46" t="n">
-        <v>92</v>
+        <v>77</v>
       </c>
       <c r="L46" t="n">
-        <v>2.34</v>
+        <v>2.94</v>
       </c>
       <c r="M46" t="n">
-        <v>34.3</v>
+        <v>47.8</v>
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P46" t="n">
-        <v>64.2</v>
+        <v>48.5</v>
       </c>
       <c r="Q46" t="inlineStr">
         <is>
@@ -4680,6 +4692,458 @@
       </c>
       <c r="U46" t="inlineStr"/>
       <c r="V46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>MAR</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>359.91</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I47" t="n">
+        <v>56.6</v>
+      </c>
+      <c r="J47" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="K47" t="n">
+        <v>82</v>
+      </c>
+      <c r="L47" t="n">
+        <v>2.37</v>
+      </c>
+      <c r="M47" t="n">
+        <v>37.1</v>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P47" t="n">
+        <v>62.7</v>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U47" t="inlineStr"/>
+      <c r="V47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>332.02</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Debit Call</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I48" t="n">
+        <v>55.8</v>
+      </c>
+      <c r="J48" t="n">
+        <v>54.8</v>
+      </c>
+      <c r="K48" t="n">
+        <v>5</v>
+      </c>
+      <c r="L48" t="n">
+        <v>2.02</v>
+      </c>
+      <c r="M48" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P48" t="n">
+        <v>61.7</v>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V48" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>228.96</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
+        <v>55.3</v>
+      </c>
+      <c r="J49" t="n">
+        <v>58.3</v>
+      </c>
+      <c r="K49" t="n">
+        <v>42</v>
+      </c>
+      <c r="L49" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="M49" t="n">
+        <v>37.1</v>
+      </c>
+      <c r="N49" t="n">
+        <v>70.8</v>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P49" t="n">
+        <v>54.4</v>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U49" t="inlineStr"/>
+      <c r="V49" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>128.51</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I50" t="n">
+        <v>53.4</v>
+      </c>
+      <c r="J50" t="n">
+        <v>61.2</v>
+      </c>
+      <c r="K50" t="n">
+        <v>88</v>
+      </c>
+      <c r="L50" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="M50" t="n">
+        <v>33.7</v>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P50" t="n">
+        <v>64.3</v>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U50" t="inlineStr"/>
+      <c r="V50" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>80.13</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I51" t="n">
+        <v>36.7</v>
+      </c>
+      <c r="J51" t="n">
+        <v>65.09999999999999</v>
+      </c>
+      <c r="K51" t="n">
+        <v>57</v>
+      </c>
+      <c r="L51" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="M51" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P51" t="n">
+        <v>64.90000000000001</v>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U51" t="inlineStr"/>
+      <c r="V51" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Scan 29.04.2026 16:00 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,9 +32,6 @@
     </font>
     <font>
       <color rgb="00ef4444"/>
-    </font>
-    <font>
-      <color rgb="0022c55e"/>
     </font>
   </fonts>
   <fills count="3">
@@ -63,13 +60,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -435,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V51"/>
+  <dimension ref="A1:V44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -448,7 +444,7 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="6" customWidth="1" min="10" max="10"/>
-    <col width="6" customWidth="1" min="11" max="11"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
     <col width="6" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
     <col width="9" customWidth="1" min="14" max="14"/>
@@ -577,11 +573,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>TXN</t>
+          <t>NXPI</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>266.77</v>
+        <v>288.25</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,19 +610,19 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>92.5</v>
+        <v>98.90000000000001</v>
       </c>
       <c r="J2" t="n">
-        <v>74.09999999999999</v>
+        <v>81.8</v>
       </c>
       <c r="K2" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L2" t="n">
-        <v>4.12</v>
+        <v>5.21</v>
       </c>
       <c r="M2" t="n">
-        <v>39.9</v>
+        <v>46.1</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -634,7 +630,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>71.8</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -666,11 +662,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>INTC</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>320.82</v>
+        <v>92.92</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -703,22 +699,22 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>89.8</v>
+        <v>94.2</v>
       </c>
       <c r="J3" t="n">
-        <v>72.3</v>
+        <v>85.8</v>
       </c>
       <c r="K3" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="L3" t="n">
-        <v>5.68</v>
+        <v>6.12</v>
       </c>
       <c r="M3" t="n">
-        <v>64.7</v>
+        <v>93.8</v>
       </c>
       <c r="N3" t="n">
-        <v>49.7</v>
+        <v>99.8</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -726,7 +722,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>69.40000000000001</v>
+        <v>85.59999999999999</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -748,25 +744,21 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U3" t="inlineStr"/>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>INTC</t>
+          <t>TXN</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>82.39</v>
+        <v>270.08</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -799,19 +791,19 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>89.8</v>
+        <v>90.09999999999999</v>
       </c>
       <c r="J4" t="n">
-        <v>77.7</v>
+        <v>74.2</v>
       </c>
       <c r="K4" t="n">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="L4" t="n">
-        <v>6.18</v>
+        <v>3.9</v>
       </c>
       <c r="M4" t="n">
-        <v>66.59999999999999</v>
+        <v>36.8</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -819,7 +811,7 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>82.59999999999999</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -851,11 +843,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SNPS</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>482.12</v>
+        <v>98.37</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -888,19 +880,19 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>87.90000000000001</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="J5" t="n">
-        <v>62.7</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="K5" t="n">
         <v>97</v>
       </c>
       <c r="L5" t="n">
-        <v>4.16</v>
+        <v>4.82</v>
       </c>
       <c r="M5" t="n">
-        <v>56.4</v>
+        <v>73.3</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -908,7 +900,7 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>54.7</v>
+        <v>78.3</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -944,11 +936,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>197.76</v>
+        <v>327.73</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -981,22 +973,22 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>87.90000000000001</v>
+        <v>87.09999999999999</v>
       </c>
       <c r="J6" t="n">
-        <v>62.5</v>
+        <v>74.5</v>
       </c>
       <c r="K6" t="n">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="L6" t="n">
-        <v>8.23</v>
+        <v>5.43</v>
       </c>
       <c r="M6" t="n">
-        <v>94.7</v>
+        <v>63.9</v>
       </c>
       <c r="N6" t="n">
-        <v>100</v>
+        <v>48.6</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -1004,7 +996,7 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>64.2</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1013,38 +1005,34 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr"/>
       <c r="V6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>93.03</v>
+        <v>198.29</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1077,19 +1065,22 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>87.5</v>
+        <v>82.2</v>
       </c>
       <c r="J7" t="n">
-        <v>74.8</v>
+        <v>62.7</v>
       </c>
       <c r="K7" t="n">
         <v>98</v>
       </c>
       <c r="L7" t="n">
-        <v>4.53</v>
+        <v>7.71</v>
       </c>
       <c r="M7" t="n">
-        <v>69.09999999999999</v>
+        <v>94.09999999999999</v>
+      </c>
+      <c r="N7" t="n">
+        <v>99.7</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1097,7 +1088,7 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>72.09999999999999</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1106,38 +1097,34 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr"/>
       <c r="V7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>UNH</t>
+          <t>NSC</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>367.3</v>
+        <v>312.83</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1166,26 +1153,23 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>82.8</v>
+        <v>81.09999999999999</v>
       </c>
       <c r="J8" t="n">
-        <v>84.7</v>
+        <v>61.8</v>
       </c>
       <c r="K8" t="n">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="L8" t="n">
-        <v>2.81</v>
+        <v>2.08</v>
       </c>
       <c r="M8" t="n">
-        <v>40.7</v>
-      </c>
-      <c r="N8" t="n">
-        <v>38.4</v>
+        <v>27.5</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1193,7 +1177,7 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1225,11 +1209,11 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ADI</t>
+          <t>SNPS</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>383.49</v>
+        <v>473.22</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1262,22 +1246,22 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>81</v>
+        <v>81.09999999999999</v>
       </c>
       <c r="J9" t="n">
-        <v>64.7</v>
+        <v>59.2</v>
       </c>
       <c r="K9" t="n">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="L9" t="n">
-        <v>3.13</v>
+        <v>4.02</v>
       </c>
       <c r="M9" t="n">
-        <v>37.7</v>
+        <v>50.8</v>
       </c>
       <c r="N9" t="n">
-        <v>98.5</v>
+        <v>23.7</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1285,7 +1269,7 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>70.2</v>
+        <v>53.3</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1294,17 +1278,17 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U9" t="inlineStr"/>
@@ -1317,11 +1301,11 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>GFS</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>209.69</v>
+        <v>63.03</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1354,22 +1338,22 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>81</v>
+        <v>80.5</v>
       </c>
       <c r="J10" t="n">
-        <v>66.3</v>
+        <v>76.3</v>
       </c>
       <c r="K10" t="n">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="L10" t="n">
-        <v>3.08</v>
+        <v>4.84</v>
       </c>
       <c r="M10" t="n">
-        <v>36.3</v>
+        <v>56.9</v>
       </c>
       <c r="N10" t="n">
-        <v>59.9</v>
+        <v>65.7</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1377,7 +1361,7 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>65.7</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1399,25 +1383,21 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U10" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U10" t="inlineStr"/>
       <c r="V10" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>MCHP</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>427.75</v>
+        <v>88.69</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1450,27 +1430,30 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>80.8</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="J11" t="n">
-        <v>64.8</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="K11" t="n">
         <v>87</v>
       </c>
       <c r="L11" t="n">
-        <v>2.46</v>
+        <v>4.22</v>
       </c>
       <c r="M11" t="n">
-        <v>39.4</v>
+        <v>48.3</v>
+      </c>
+      <c r="N11" t="n">
+        <v>71.7</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>49.7</v>
+        <v>69</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1502,11 +1485,11 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>UNH</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>151.56</v>
+        <v>368.17</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1539,22 +1522,19 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>80</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="J12" t="n">
-        <v>69.7</v>
+        <v>84.8</v>
       </c>
       <c r="K12" t="n">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="L12" t="n">
-        <v>6.05</v>
+        <v>2.69</v>
       </c>
       <c r="M12" t="n">
-        <v>67.09999999999999</v>
-      </c>
-      <c r="N12" t="n">
-        <v>67.59999999999999</v>
+        <v>29.3</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1562,7 +1542,7 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>75</v>
+        <v>63.1</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1571,38 +1551,34 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U12" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr"/>
       <c r="V12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>GFS</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>58.82</v>
+        <v>424.32</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -1635,30 +1611,27 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>79.2</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="J13" t="n">
-        <v>68.90000000000001</v>
+        <v>61.7</v>
       </c>
       <c r="K13" t="n">
-        <v>98</v>
+        <v>83</v>
       </c>
       <c r="L13" t="n">
-        <v>4.88</v>
+        <v>2.43</v>
       </c>
       <c r="M13" t="n">
-        <v>56.1</v>
-      </c>
-      <c r="N13" t="n">
-        <v>64</v>
+        <v>40.6</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>70.5</v>
+        <v>48.7</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1690,11 +1663,11 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>ADI</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>495.15</v>
+        <v>389.14</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -1727,19 +1700,22 @@
         </is>
       </c>
       <c r="I14" t="n">
-        <v>77.40000000000001</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="J14" t="n">
-        <v>63.3</v>
+        <v>66.7</v>
       </c>
       <c r="K14" t="n">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="L14" t="n">
-        <v>5.71</v>
+        <v>3.07</v>
       </c>
       <c r="M14" t="n">
-        <v>75.2</v>
+        <v>37.9</v>
+      </c>
+      <c r="N14" t="n">
+        <v>99</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1747,7 +1723,7 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>71.3</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1769,25 +1745,21 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U14" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U14" t="inlineStr"/>
       <c r="V14" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>XLK</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>156.82</v>
+        <v>210.71</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1820,19 +1792,22 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>77.3</v>
+        <v>76.2</v>
       </c>
       <c r="J15" t="n">
-        <v>66.5</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="K15" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="L15" t="n">
-        <v>2.03</v>
+        <v>2.87</v>
       </c>
       <c r="M15" t="n">
-        <v>29.2</v>
+        <v>35.3</v>
+      </c>
+      <c r="N15" t="n">
+        <v>55.3</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1840,7 +1815,7 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>65.5</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1862,25 +1837,21 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U15" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U15" t="inlineStr"/>
       <c r="V15" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>MU</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>595.66</v>
+        <v>519.66</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -1913,19 +1884,19 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>76.7</v>
+        <v>74</v>
       </c>
       <c r="J16" t="n">
-        <v>63.4</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="K16" t="n">
         <v>85</v>
       </c>
       <c r="L16" t="n">
-        <v>2.68</v>
+        <v>5.4</v>
       </c>
       <c r="M16" t="n">
-        <v>29.1</v>
+        <v>76.3</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -1933,7 +1904,7 @@
         </is>
       </c>
       <c r="P16" t="n">
-        <v>57</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1965,15 +1936,15 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>MCHP</t>
+          <t>CPRT</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>84.81</v>
+        <v>33.07</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -1988,48 +1959,48 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>75.90000000000001</v>
+        <v>73.5</v>
       </c>
       <c r="J17" t="n">
-        <v>67.90000000000001</v>
+        <v>42.2</v>
       </c>
       <c r="K17" t="n">
-        <v>88</v>
+        <v>12</v>
       </c>
       <c r="L17" t="n">
-        <v>4.05</v>
+        <v>2.06</v>
       </c>
       <c r="M17" t="n">
-        <v>46.3</v>
+        <v>19</v>
       </c>
       <c r="N17" t="n">
-        <v>65.90000000000001</v>
+        <v>14.6</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P17" t="n">
-        <v>64.09999999999999</v>
+        <v>31.6</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
@@ -2039,7 +2010,7 @@
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
@@ -2047,7 +2018,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U17" t="inlineStr"/>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V17" t="inlineStr">
         <is>
           <t>No</t>
@@ -2057,11 +2032,11 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>NXPI</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>229.11</v>
+        <v>154.37</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -2094,22 +2069,19 @@
         </is>
       </c>
       <c r="I18" t="n">
-        <v>75.40000000000001</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="J18" t="n">
-        <v>61.5</v>
+        <v>72.2</v>
       </c>
       <c r="K18" t="n">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="L18" t="n">
-        <v>3.63</v>
+        <v>5.65</v>
       </c>
       <c r="M18" t="n">
-        <v>35.4</v>
-      </c>
-      <c r="N18" t="n">
-        <v>58</v>
+        <v>80.3</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -2117,7 +2089,7 @@
         </is>
       </c>
       <c r="P18" t="n">
-        <v>55.1</v>
+        <v>77</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -2126,38 +2098,34 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U18" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr"/>
       <c r="V18" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>655.12</v>
+        <v>589.09</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -2190,22 +2158,22 @@
         </is>
       </c>
       <c r="I19" t="n">
-        <v>74.3</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="J19" t="n">
-        <v>67.40000000000001</v>
+        <v>59.8</v>
       </c>
       <c r="K19" t="n">
-        <v>95</v>
+        <v>83</v>
       </c>
       <c r="L19" t="n">
-        <v>1.49</v>
+        <v>2.64</v>
       </c>
       <c r="M19" t="n">
-        <v>21.9</v>
+        <v>27.3</v>
       </c>
       <c r="N19" t="n">
-        <v>97.59999999999999</v>
+        <v>44.7</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -2213,7 +2181,7 @@
         </is>
       </c>
       <c r="P19" t="n">
-        <v>63.9</v>
+        <v>55.7</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -2249,7 +2217,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>260.18</v>
+        <v>263.38</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -2282,22 +2250,19 @@
         </is>
       </c>
       <c r="I20" t="n">
-        <v>74.09999999999999</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="J20" t="n">
-        <v>74.5</v>
+        <v>75.7</v>
       </c>
       <c r="K20" t="n">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="L20" t="n">
-        <v>2.37</v>
+        <v>2.45</v>
       </c>
       <c r="M20" t="n">
-        <v>33.4</v>
-      </c>
-      <c r="N20" t="n">
-        <v>56.7</v>
+        <v>41.8</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -2305,7 +2270,7 @@
         </is>
       </c>
       <c r="P20" t="n">
-        <v>64.09999999999999</v>
+        <v>65.8</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
@@ -2337,11 +2302,11 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>KLAC</t>
+          <t>XLK</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1831.57</v>
+        <v>158.38</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -2374,19 +2339,19 @@
         </is>
       </c>
       <c r="I21" t="n">
-        <v>71.7</v>
+        <v>72.2</v>
       </c>
       <c r="J21" t="n">
-        <v>62.3</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="K21" t="n">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="L21" t="n">
-        <v>4.05</v>
+        <v>1.86</v>
       </c>
       <c r="M21" t="n">
-        <v>53.7</v>
+        <v>30.7</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
@@ -2394,7 +2359,7 @@
         </is>
       </c>
       <c r="P21" t="n">
-        <v>68.8</v>
+        <v>67.5</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
@@ -2403,17 +2368,17 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U21" t="inlineStr"/>
@@ -2430,7 +2395,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>348.98</v>
+        <v>351.07</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -2466,19 +2431,19 @@
         <v>71.40000000000001</v>
       </c>
       <c r="J22" t="n">
-        <v>70.2</v>
+        <v>71.7</v>
       </c>
       <c r="K22" t="n">
-        <v>92</v>
+        <v>85</v>
       </c>
       <c r="L22" t="n">
-        <v>2.24</v>
+        <v>2.37</v>
       </c>
       <c r="M22" t="n">
-        <v>33.2</v>
+        <v>32.9</v>
       </c>
       <c r="N22" t="n">
-        <v>86.40000000000001</v>
+        <v>85</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
@@ -2486,7 +2451,7 @@
         </is>
       </c>
       <c r="P22" t="n">
-        <v>66.7</v>
+        <v>67.2</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
@@ -2518,11 +2483,11 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>GOOG</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>710.27</v>
+        <v>348.7</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -2555,22 +2520,19 @@
         </is>
       </c>
       <c r="I23" t="n">
-        <v>71.3</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="J23" t="n">
-        <v>66</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="K23" t="n">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="L23" t="n">
-        <v>1.02</v>
+        <v>2.28</v>
       </c>
       <c r="M23" t="n">
-        <v>17.2</v>
-      </c>
-      <c r="N23" t="n">
-        <v>91.09999999999999</v>
+        <v>37.1</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -2578,7 +2540,7 @@
         </is>
       </c>
       <c r="P23" t="n">
-        <v>63.1</v>
+        <v>66.8</v>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
@@ -2610,11 +2572,11 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>HUM</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>230.29</v>
+        <v>659.28</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -2643,34 +2605,31 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I24" t="n">
-        <v>71.2</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="J24" t="n">
-        <v>78.7</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="K24" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="L24" t="n">
-        <v>3.2</v>
+        <v>1.38</v>
       </c>
       <c r="M24" t="n">
-        <v>36.7</v>
-      </c>
-      <c r="N24" t="n">
-        <v>26.5</v>
+        <v>21.2</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P24" t="n">
-        <v>54.6</v>
+        <v>65.3</v>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
@@ -2702,11 +2661,11 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>ANET</t>
+          <t>APH</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>163</v>
+        <v>152.25</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -2739,19 +2698,22 @@
         </is>
       </c>
       <c r="I25" t="n">
-        <v>70.5</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="J25" t="n">
-        <v>58.2</v>
+        <v>61.6</v>
       </c>
       <c r="K25" t="n">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="L25" t="n">
-        <v>4.43</v>
+        <v>3.74</v>
       </c>
       <c r="M25" t="n">
-        <v>64.2</v>
+        <v>45.8</v>
+      </c>
+      <c r="N25" t="n">
+        <v>55.1</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
@@ -2759,7 +2721,7 @@
         </is>
       </c>
       <c r="P25" t="n">
-        <v>61.2</v>
+        <v>61.4</v>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
@@ -2768,38 +2730,34 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U25" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr"/>
       <c r="V25" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>PSA</t>
+          <t>CSCO</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>307.18</v>
+        <v>88.68000000000001</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -2828,17 +2786,17 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I26" t="n">
-        <v>70.2</v>
+        <v>67.5</v>
       </c>
       <c r="J26" t="n">
-        <v>60.9</v>
+        <v>64.7</v>
       </c>
       <c r="K26" t="n">
-        <v>76</v>
+        <v>85</v>
       </c>
       <c r="L26" t="n">
         <v>2.33</v>
@@ -2847,7 +2805,7 @@
         <v>27.3</v>
       </c>
       <c r="N26" t="n">
-        <v>96.40000000000001</v>
+        <v>42.6</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
@@ -2855,7 +2813,7 @@
         </is>
       </c>
       <c r="P26" t="n">
-        <v>58.9</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
@@ -2887,11 +2845,11 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ABNB</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>140.27</v>
+        <v>710.02</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -2924,19 +2882,22 @@
         </is>
       </c>
       <c r="I27" t="n">
-        <v>69.2</v>
+        <v>66.2</v>
       </c>
       <c r="J27" t="n">
-        <v>59.1</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="K27" t="n">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="L27" t="n">
-        <v>3</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="M27" t="n">
-        <v>49.6</v>
+        <v>17.1</v>
+      </c>
+      <c r="N27" t="n">
+        <v>90.8</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -2944,7 +2905,7 @@
         </is>
       </c>
       <c r="P27" t="n">
-        <v>58.1</v>
+        <v>63</v>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
@@ -2953,17 +2914,17 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U27" t="inlineStr"/>
@@ -2976,11 +2937,11 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>ABNB</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>86.94</v>
+        <v>138.66</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -3013,19 +2974,22 @@
         </is>
       </c>
       <c r="I28" t="n">
-        <v>69</v>
+        <v>63.7</v>
       </c>
       <c r="J28" t="n">
-        <v>60.5</v>
+        <v>55.8</v>
       </c>
       <c r="K28" t="n">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="L28" t="n">
-        <v>2.26</v>
+        <v>3</v>
       </c>
       <c r="M28" t="n">
-        <v>40.2</v>
+        <v>33.9</v>
+      </c>
+      <c r="N28" t="n">
+        <v>66.7</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
@@ -3033,7 +2997,7 @@
         </is>
       </c>
       <c r="P28" t="n">
-        <v>65.59999999999999</v>
+        <v>56.7</v>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
@@ -3065,11 +3029,11 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>GOOG</t>
+          <t>ANET</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>346.5</v>
+        <v>163.54</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -3102,19 +3066,22 @@
         </is>
       </c>
       <c r="I29" t="n">
-        <v>68.90000000000001</v>
+        <v>62.3</v>
       </c>
       <c r="J29" t="n">
-        <v>70.2</v>
+        <v>58.6</v>
       </c>
       <c r="K29" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="L29" t="n">
-        <v>2.17</v>
+        <v>4.14</v>
       </c>
       <c r="M29" t="n">
-        <v>37.4</v>
+        <v>57.9</v>
+      </c>
+      <c r="N29" t="n">
+        <v>73.2</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
@@ -3122,7 +3089,7 @@
         </is>
       </c>
       <c r="P29" t="n">
-        <v>66.3</v>
+        <v>61.5</v>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
@@ -3131,17 +3098,17 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U29" t="inlineStr"/>
@@ -3154,78 +3121,78 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>PEP</t>
+          <t>BLK</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>157.41</v>
+        <v>1032.68</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D30" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I30" t="n">
-        <v>68.3</v>
+        <v>61.4</v>
       </c>
       <c r="J30" t="n">
-        <v>53.5</v>
+        <v>52.8</v>
       </c>
       <c r="K30" t="n">
-        <v>2</v>
+        <v>77</v>
       </c>
       <c r="L30" t="n">
-        <v>1.91</v>
+        <v>2.39</v>
       </c>
       <c r="M30" t="n">
-        <v>23.2</v>
+        <v>32.7</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P30" t="n">
-        <v>54.9</v>
+        <v>49.7</v>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
@@ -3233,11 +3200,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U30" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U30" t="inlineStr"/>
       <c r="V30" t="inlineStr">
         <is>
           <t>No</t>
@@ -3247,11 +3210,11 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>IWM</t>
+          <t>KLAC</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>273.62</v>
+        <v>1789.95</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -3280,23 +3243,23 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I31" t="n">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="J31" t="n">
-        <v>62.8</v>
+        <v>57.9</v>
       </c>
       <c r="K31" t="n">
-        <v>93</v>
+        <v>76</v>
       </c>
       <c r="L31" t="n">
-        <v>1.58</v>
+        <v>3.97</v>
       </c>
       <c r="M31" t="n">
-        <v>22.5</v>
+        <v>55.5</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
@@ -3304,7 +3267,7 @@
         </is>
       </c>
       <c r="P31" t="n">
-        <v>64.59999999999999</v>
+        <v>66.3</v>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
@@ -3336,11 +3299,11 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ETN</t>
+          <t>META</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>411.33</v>
+        <v>668.85</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -3373,22 +3336,19 @@
         </is>
       </c>
       <c r="I32" t="n">
-        <v>66.7</v>
+        <v>60.8</v>
       </c>
       <c r="J32" t="n">
-        <v>61.8</v>
+        <v>58.5</v>
       </c>
       <c r="K32" t="n">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="L32" t="n">
-        <v>2.96</v>
+        <v>2.44</v>
       </c>
       <c r="M32" t="n">
-        <v>34.9</v>
-      </c>
-      <c r="N32" t="n">
-        <v>76.2</v>
+        <v>43.3</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
@@ -3396,7 +3356,7 @@
         </is>
       </c>
       <c r="P32" t="n">
-        <v>63.7</v>
+        <v>52.8</v>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
@@ -3428,11 +3388,11 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>BLK</t>
+          <t>IWM</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>1054.21</v>
+        <v>271.56</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -3461,26 +3421,26 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I33" t="n">
-        <v>66.5</v>
+        <v>60.8</v>
       </c>
       <c r="J33" t="n">
-        <v>59.6</v>
+        <v>58.9</v>
       </c>
       <c r="K33" t="n">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="L33" t="n">
-        <v>2.34</v>
+        <v>1.54</v>
       </c>
       <c r="M33" t="n">
-        <v>27.7</v>
+        <v>22</v>
       </c>
       <c r="N33" t="n">
-        <v>61.1</v>
+        <v>78</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
@@ -3488,7 +3448,7 @@
         </is>
       </c>
       <c r="P33" t="n">
-        <v>52.3</v>
+        <v>62.8</v>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
@@ -3497,17 +3457,17 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U33" t="inlineStr"/>
@@ -3520,11 +3480,11 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>APH</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>144.03</v>
+        <v>186.02</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -3557,19 +3517,22 @@
         </is>
       </c>
       <c r="I34" t="n">
-        <v>65.5</v>
+        <v>60.2</v>
       </c>
       <c r="J34" t="n">
-        <v>52.8</v>
+        <v>59</v>
       </c>
       <c r="K34" t="n">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="L34" t="n">
-        <v>3.37</v>
+        <v>2.36</v>
       </c>
       <c r="M34" t="n">
-        <v>54.7</v>
+        <v>28.1</v>
+      </c>
+      <c r="N34" t="n">
+        <v>51</v>
       </c>
       <c r="O34" t="inlineStr">
         <is>
@@ -3577,7 +3540,7 @@
         </is>
       </c>
       <c r="P34" t="n">
-        <v>55.9</v>
+        <v>61.7</v>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
@@ -3609,11 +3572,11 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>MET</t>
+          <t>ETN</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>78.87</v>
+        <v>410.69</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -3646,19 +3609,22 @@
         </is>
       </c>
       <c r="I35" t="n">
-        <v>65.40000000000001</v>
+        <v>60.1</v>
       </c>
       <c r="J35" t="n">
-        <v>67.40000000000001</v>
+        <v>61.2</v>
       </c>
       <c r="K35" t="n">
         <v>83</v>
       </c>
       <c r="L35" t="n">
-        <v>1.91</v>
+        <v>2.87</v>
       </c>
       <c r="M35" t="n">
-        <v>26.9</v>
+        <v>34.8</v>
+      </c>
+      <c r="N35" t="n">
+        <v>75.90000000000001</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
@@ -3666,7 +3632,7 @@
         </is>
       </c>
       <c r="P35" t="n">
-        <v>56.1</v>
+        <v>63.5</v>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
@@ -3675,17 +3641,17 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U35" t="inlineStr"/>
@@ -3698,11 +3664,11 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>MET</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>666.92</v>
+        <v>78.34</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -3731,23 +3697,23 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I36" t="n">
-        <v>65.2</v>
+        <v>60</v>
       </c>
       <c r="J36" t="n">
-        <v>57.9</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="K36" t="n">
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="L36" t="n">
-        <v>2.59</v>
+        <v>1.86</v>
       </c>
       <c r="M36" t="n">
-        <v>43.9</v>
+        <v>29.2</v>
       </c>
       <c r="O36" t="inlineStr">
         <is>
@@ -3755,7 +3721,7 @@
         </is>
       </c>
       <c r="P36" t="n">
-        <v>52.6</v>
+        <v>55.3</v>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
@@ -3787,11 +3753,11 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>189.55</v>
+        <v>399.01</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -3824,19 +3790,22 @@
         </is>
       </c>
       <c r="I37" t="n">
-        <v>63.4</v>
+        <v>58</v>
       </c>
       <c r="J37" t="n">
-        <v>66.09999999999999</v>
+        <v>61.8</v>
       </c>
       <c r="K37" t="n">
         <v>91</v>
       </c>
       <c r="L37" t="n">
-        <v>2.29</v>
+        <v>3.18</v>
       </c>
       <c r="M37" t="n">
-        <v>31.1</v>
+        <v>44.9</v>
+      </c>
+      <c r="N37" t="n">
+        <v>52.6</v>
       </c>
       <c r="O37" t="inlineStr">
         <is>
@@ -3844,7 +3813,7 @@
         </is>
       </c>
       <c r="P37" t="n">
-        <v>64.2</v>
+        <v>62.3</v>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
@@ -3853,17 +3822,17 @@
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U37" t="inlineStr"/>
@@ -3876,11 +3845,11 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>CAT</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>396.41</v>
+        <v>811.16</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -3909,23 +3878,26 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I38" t="n">
-        <v>63.2</v>
+        <v>57.2</v>
       </c>
       <c r="J38" t="n">
-        <v>60.4</v>
+        <v>62.2</v>
       </c>
       <c r="K38" t="n">
-        <v>93</v>
+        <v>75</v>
       </c>
       <c r="L38" t="n">
-        <v>3.47</v>
+        <v>2.6</v>
       </c>
       <c r="M38" t="n">
-        <v>48.6</v>
+        <v>37.5</v>
+      </c>
+      <c r="N38" t="n">
+        <v>69.8</v>
       </c>
       <c r="O38" t="inlineStr">
         <is>
@@ -3933,7 +3905,7 @@
         </is>
       </c>
       <c r="P38" t="n">
-        <v>61.6</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="Q38" t="inlineStr">
         <is>
@@ -3955,25 +3927,21 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U38" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U38" t="inlineStr"/>
       <c r="V38" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CAT</t>
+          <t>BK</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>815.13</v>
+        <v>130.99</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -4002,26 +3970,23 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I39" t="n">
-        <v>62.8</v>
+        <v>54.7</v>
       </c>
       <c r="J39" t="n">
-        <v>63.9</v>
+        <v>57.1</v>
       </c>
       <c r="K39" t="n">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="L39" t="n">
-        <v>2.75</v>
+        <v>2.01</v>
       </c>
       <c r="M39" t="n">
-        <v>37.4</v>
-      </c>
-      <c r="N39" t="n">
-        <v>69.59999999999999</v>
+        <v>28.1</v>
       </c>
       <c r="O39" t="inlineStr">
         <is>
@@ -4029,7 +3994,7 @@
         </is>
       </c>
       <c r="P39" t="n">
-        <v>72.3</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="Q39" t="inlineStr">
         <is>
@@ -4038,17 +4003,17 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U39" t="inlineStr"/>
@@ -4061,11 +4026,11 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>DLR</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>192.9</v>
+        <v>480.92</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -4094,23 +4059,26 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I40" t="n">
-        <v>61.5</v>
+        <v>54</v>
       </c>
       <c r="J40" t="n">
-        <v>54.3</v>
+        <v>64.5</v>
       </c>
       <c r="K40" t="n">
-        <v>91</v>
+        <v>73</v>
       </c>
       <c r="L40" t="n">
-        <v>2.48</v>
+        <v>2.22</v>
       </c>
       <c r="M40" t="n">
-        <v>33.2</v>
+        <v>32.9</v>
+      </c>
+      <c r="N40" t="n">
+        <v>81</v>
       </c>
       <c r="O40" t="inlineStr">
         <is>
@@ -4118,7 +4086,7 @@
         </is>
       </c>
       <c r="P40" t="n">
-        <v>62.3</v>
+        <v>64</v>
       </c>
       <c r="Q40" t="inlineStr">
         <is>
@@ -4150,15 +4118,15 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>PCAR</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>119.77</v>
+        <v>324.31</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -4173,36 +4141,33 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I41" t="n">
-        <v>60.7</v>
+        <v>51.2</v>
       </c>
       <c r="J41" t="n">
-        <v>43.2</v>
+        <v>46.2</v>
       </c>
       <c r="K41" t="n">
-        <v>56</v>
+        <v>6</v>
       </c>
       <c r="L41" t="n">
-        <v>3.22</v>
+        <v>2.07</v>
       </c>
       <c r="M41" t="n">
-        <v>31.1</v>
-      </c>
-      <c r="N41" t="n">
-        <v>100</v>
+        <v>20.3</v>
       </c>
       <c r="O41" t="inlineStr">
         <is>
@@ -4210,11 +4175,11 @@
         </is>
       </c>
       <c r="P41" t="n">
-        <v>54.5</v>
+        <v>57.2</v>
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
@@ -4234,7 +4199,7 @@
       </c>
       <c r="U41" t="inlineStr">
         <is>
-          <t>Divergence</t>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V41" t="inlineStr">
@@ -4246,11 +4211,11 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>BK</t>
+          <t>DLR</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>133.95</v>
+        <v>193.08</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -4283,22 +4248,22 @@
         </is>
       </c>
       <c r="I42" t="n">
-        <v>59.9</v>
+        <v>50.7</v>
       </c>
       <c r="J42" t="n">
-        <v>67.09999999999999</v>
+        <v>54.4</v>
       </c>
       <c r="K42" t="n">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="L42" t="n">
-        <v>1.89</v>
+        <v>2.35</v>
       </c>
       <c r="M42" t="n">
-        <v>19.1</v>
+        <v>21.7</v>
       </c>
       <c r="N42" t="n">
-        <v>32.1</v>
+        <v>62.1</v>
       </c>
       <c r="O42" t="inlineStr">
         <is>
@@ -4306,7 +4271,7 @@
         </is>
       </c>
       <c r="P42" t="n">
-        <v>72.3</v>
+        <v>62.6</v>
       </c>
       <c r="Q42" t="inlineStr">
         <is>
@@ -4338,11 +4303,11 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>TT</t>
+          <t>C</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>479.44</v>
+        <v>126.84</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -4375,19 +4340,22 @@
         </is>
       </c>
       <c r="I43" t="n">
-        <v>59.9</v>
+        <v>44.3</v>
       </c>
       <c r="J43" t="n">
-        <v>63.3</v>
+        <v>56.9</v>
       </c>
       <c r="K43" t="n">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="L43" t="n">
-        <v>2.3</v>
+        <v>2.33</v>
       </c>
       <c r="M43" t="n">
-        <v>34.7</v>
+        <v>32.4</v>
+      </c>
+      <c r="N43" t="n">
+        <v>58.2</v>
       </c>
       <c r="O43" t="inlineStr">
         <is>
@@ -4395,7 +4363,7 @@
         </is>
       </c>
       <c r="P43" t="n">
-        <v>63.5</v>
+        <v>62.8</v>
       </c>
       <c r="Q43" t="inlineStr">
         <is>
@@ -4404,17 +4372,17 @@
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U43" t="inlineStr"/>
@@ -4427,15 +4395,15 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>LRCX</t>
+          <t>KO</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>247.3</v>
+        <v>78.79000000000001</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -4450,12 +4418,12 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -4464,22 +4432,19 @@
         </is>
       </c>
       <c r="I44" t="n">
-        <v>58.7</v>
+        <v>38.2</v>
       </c>
       <c r="J44" t="n">
-        <v>49.6</v>
+        <v>61.4</v>
       </c>
       <c r="K44" t="n">
-        <v>75</v>
+        <v>52</v>
       </c>
       <c r="L44" t="n">
-        <v>5.11</v>
+        <v>2.04</v>
       </c>
       <c r="M44" t="n">
-        <v>61.9</v>
-      </c>
-      <c r="N44" t="n">
-        <v>82.90000000000001</v>
+        <v>19.5</v>
       </c>
       <c r="O44" t="inlineStr">
         <is>
@@ -4487,663 +4452,34 @@
         </is>
       </c>
       <c r="P44" t="n">
-        <v>62.1</v>
+        <v>62.5</v>
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>FIRED</t>
         </is>
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S44" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U44" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>Squeeze Fired</t>
+        </is>
+      </c>
       <c r="V44" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>FDX</t>
-        </is>
-      </c>
-      <c r="B45" t="n">
-        <v>386.22</v>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D45" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>Credit Call</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I45" t="n">
-        <v>57.1</v>
-      </c>
-      <c r="J45" t="n">
-        <v>58.8</v>
-      </c>
-      <c r="K45" t="n">
-        <v>69</v>
-      </c>
-      <c r="L45" t="n">
-        <v>2.31</v>
-      </c>
-      <c r="M45" t="n">
-        <v>29</v>
-      </c>
-      <c r="N45" t="n">
-        <v>68</v>
-      </c>
-      <c r="O45" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P45" t="n">
-        <v>68.7</v>
-      </c>
-      <c r="Q45" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R45" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S45" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="T45" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U45" t="inlineStr"/>
-      <c r="V45" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>CDW</t>
-        </is>
-      </c>
-      <c r="B46" t="n">
-        <v>132.45</v>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>Credit Call</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I46" t="n">
-        <v>56.7</v>
-      </c>
-      <c r="J46" t="n">
-        <v>54.7</v>
-      </c>
-      <c r="K46" t="n">
-        <v>77</v>
-      </c>
-      <c r="L46" t="n">
-        <v>2.94</v>
-      </c>
-      <c r="M46" t="n">
-        <v>47.8</v>
-      </c>
-      <c r="O46" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P46" t="n">
-        <v>48.5</v>
-      </c>
-      <c r="Q46" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R46" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S46" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="T46" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U46" t="inlineStr"/>
-      <c r="V46" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>MAR</t>
-        </is>
-      </c>
-      <c r="B47" t="n">
-        <v>359.91</v>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>Credit Call</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I47" t="n">
-        <v>56.6</v>
-      </c>
-      <c r="J47" t="n">
-        <v>55.6</v>
-      </c>
-      <c r="K47" t="n">
-        <v>82</v>
-      </c>
-      <c r="L47" t="n">
-        <v>2.37</v>
-      </c>
-      <c r="M47" t="n">
-        <v>37.1</v>
-      </c>
-      <c r="O47" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P47" t="n">
-        <v>62.7</v>
-      </c>
-      <c r="Q47" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R47" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S47" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="T47" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U47" t="inlineStr"/>
-      <c r="V47" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>CB</t>
-        </is>
-      </c>
-      <c r="B48" t="n">
-        <v>332.02</v>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D48" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>Debit Call</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>30-60 DTE</t>
-        </is>
-      </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>SQUEEZE</t>
-        </is>
-      </c>
-      <c r="I48" t="n">
-        <v>55.8</v>
-      </c>
-      <c r="J48" t="n">
-        <v>54.8</v>
-      </c>
-      <c r="K48" t="n">
-        <v>5</v>
-      </c>
-      <c r="L48" t="n">
-        <v>2.02</v>
-      </c>
-      <c r="M48" t="n">
-        <v>22.9</v>
-      </c>
-      <c r="O48" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P48" t="n">
-        <v>61.7</v>
-      </c>
-      <c r="Q48" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="R48" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="S48" t="inlineStr">
-        <is>
-          <t>lime</t>
-        </is>
-      </c>
-      <c r="T48" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U48" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
-      <c r="V48" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>BA</t>
-        </is>
-      </c>
-      <c r="B49" t="n">
-        <v>228.96</v>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D49" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>Credit Call</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I49" t="n">
-        <v>55.3</v>
-      </c>
-      <c r="J49" t="n">
-        <v>58.3</v>
-      </c>
-      <c r="K49" t="n">
-        <v>42</v>
-      </c>
-      <c r="L49" t="n">
-        <v>2.9</v>
-      </c>
-      <c r="M49" t="n">
-        <v>37.1</v>
-      </c>
-      <c r="N49" t="n">
-        <v>70.8</v>
-      </c>
-      <c r="O49" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P49" t="n">
-        <v>54.4</v>
-      </c>
-      <c r="Q49" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R49" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="S49" t="inlineStr">
-        <is>
-          <t>lime</t>
-        </is>
-      </c>
-      <c r="T49" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U49" t="inlineStr"/>
-      <c r="V49" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="B50" t="n">
-        <v>128.51</v>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D50" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>Credit Call</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I50" t="n">
-        <v>53.4</v>
-      </c>
-      <c r="J50" t="n">
-        <v>61.2</v>
-      </c>
-      <c r="K50" t="n">
-        <v>88</v>
-      </c>
-      <c r="L50" t="n">
-        <v>2.38</v>
-      </c>
-      <c r="M50" t="n">
-        <v>33.7</v>
-      </c>
-      <c r="O50" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P50" t="n">
-        <v>64.3</v>
-      </c>
-      <c r="Q50" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R50" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S50" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="T50" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U50" t="inlineStr"/>
-      <c r="V50" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>KO</t>
-        </is>
-      </c>
-      <c r="B51" t="n">
-        <v>80.13</v>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D51" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>Debit Put</t>
-        </is>
-      </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>30-60 DTE</t>
-        </is>
-      </c>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I51" t="n">
-        <v>36.7</v>
-      </c>
-      <c r="J51" t="n">
-        <v>65.09999999999999</v>
-      </c>
-      <c r="K51" t="n">
-        <v>57</v>
-      </c>
-      <c r="L51" t="n">
-        <v>2.12</v>
-      </c>
-      <c r="M51" t="n">
-        <v>21.4</v>
-      </c>
-      <c r="O51" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P51" t="n">
-        <v>64.90000000000001</v>
-      </c>
-      <c r="Q51" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R51" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="S51" t="inlineStr">
-        <is>
-          <t>maroon</t>
-        </is>
-      </c>
-      <c r="T51" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U51" t="inlineStr"/>
-      <c r="V51" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Scan 30.04.2026 15:52 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,6 +32,9 @@
     </font>
     <font>
       <color rgb="00ef4444"/>
+    </font>
+    <font>
+      <color rgb="0022c55e"/>
     </font>
   </fonts>
   <fills count="3">
@@ -60,12 +63,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -431,11 +435,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V44"/>
+  <dimension ref="A1:V37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
@@ -577,7 +581,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>288.25</v>
+        <v>286.66</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -613,16 +617,16 @@
         <v>98.90000000000001</v>
       </c>
       <c r="J2" t="n">
-        <v>81.8</v>
+        <v>80</v>
       </c>
       <c r="K2" t="n">
         <v>100</v>
       </c>
       <c r="L2" t="n">
-        <v>5.21</v>
+        <v>5.15</v>
       </c>
       <c r="M2" t="n">
-        <v>46.1</v>
+        <v>44.5</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -630,7 +634,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>71.59999999999999</v>
+        <v>71.3</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -666,7 +670,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>92.92</v>
+        <v>93.54000000000001</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -699,22 +703,19 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>94.2</v>
+        <v>92.3</v>
       </c>
       <c r="J3" t="n">
-        <v>85.8</v>
+        <v>83.90000000000001</v>
       </c>
       <c r="K3" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L3" t="n">
-        <v>6.12</v>
+        <v>5.97</v>
       </c>
       <c r="M3" t="n">
-        <v>93.8</v>
-      </c>
-      <c r="N3" t="n">
-        <v>99.8</v>
+        <v>75</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -758,7 +759,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>270.08</v>
+        <v>276.96</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -791,19 +792,22 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>90.09999999999999</v>
+        <v>90</v>
       </c>
       <c r="J4" t="n">
-        <v>74.2</v>
+        <v>76.2</v>
       </c>
       <c r="K4" t="n">
         <v>99</v>
       </c>
       <c r="L4" t="n">
-        <v>3.9</v>
+        <v>3.85</v>
       </c>
       <c r="M4" t="n">
-        <v>36.8</v>
+        <v>62.8</v>
+      </c>
+      <c r="N4" t="n">
+        <v>98.8</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -811,7 +815,7 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>73.40000000000001</v>
+        <v>77</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -843,11 +847,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>98.37</v>
+        <v>374.95</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -880,19 +884,19 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>89.59999999999999</v>
+        <v>88.7</v>
       </c>
       <c r="J5" t="n">
-        <v>78.90000000000001</v>
+        <v>80.2</v>
       </c>
       <c r="K5" t="n">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="L5" t="n">
-        <v>4.82</v>
+        <v>2.93</v>
       </c>
       <c r="M5" t="n">
-        <v>73.3</v>
+        <v>32.5</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -900,7 +904,7 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>78.3</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -922,14 +926,10 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -940,7 +940,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>327.73</v>
+        <v>346.58</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -973,22 +973,22 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>87.09999999999999</v>
+        <v>87.59999999999999</v>
       </c>
       <c r="J6" t="n">
-        <v>74.5</v>
+        <v>77.8</v>
       </c>
       <c r="K6" t="n">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="L6" t="n">
-        <v>5.43</v>
+        <v>5.36</v>
       </c>
       <c r="M6" t="n">
-        <v>63.9</v>
+        <v>64.3</v>
       </c>
       <c r="N6" t="n">
-        <v>48.6</v>
+        <v>49.3</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -996,7 +996,7 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>71.40000000000001</v>
+        <v>77.2</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1028,11 +1028,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>GOOG</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>198.29</v>
+        <v>371.77</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1065,22 +1065,19 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>82.2</v>
+        <v>87.40000000000001</v>
       </c>
       <c r="J7" t="n">
-        <v>62.7</v>
+        <v>80.2</v>
       </c>
       <c r="K7" t="n">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="L7" t="n">
-        <v>7.71</v>
+        <v>2.86</v>
       </c>
       <c r="M7" t="n">
-        <v>94.09999999999999</v>
-      </c>
-      <c r="N7" t="n">
-        <v>99.7</v>
+        <v>31</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1088,7 +1085,7 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>64.40000000000001</v>
+        <v>71.2</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1097,17 +1094,17 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U7" t="inlineStr"/>
@@ -1120,11 +1117,11 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>NSC</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>312.83</v>
+        <v>100.16</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1153,31 +1150,31 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>81.09999999999999</v>
+        <v>84.59999999999999</v>
       </c>
       <c r="J8" t="n">
-        <v>61.8</v>
+        <v>80</v>
       </c>
       <c r="K8" t="n">
+        <v>96</v>
+      </c>
+      <c r="L8" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="M8" t="n">
+        <v>69.8</v>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P8" t="n">
         <v>79</v>
-      </c>
-      <c r="L8" t="n">
-        <v>2.08</v>
-      </c>
-      <c r="M8" t="n">
-        <v>27.5</v>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P8" t="n">
-        <v>61</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1209,11 +1206,11 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SNPS</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>473.22</v>
+        <v>212.49</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1246,22 +1243,19 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>81.09999999999999</v>
+        <v>82.5</v>
       </c>
       <c r="J9" t="n">
-        <v>59.2</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="K9" t="n">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="L9" t="n">
-        <v>4.02</v>
+        <v>7.14</v>
       </c>
       <c r="M9" t="n">
-        <v>50.8</v>
-      </c>
-      <c r="N9" t="n">
-        <v>23.7</v>
+        <v>85.2</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1269,7 +1263,7 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>53.3</v>
+        <v>69.5</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1301,11 +1295,11 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>GFS</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>63.03</v>
+        <v>257.83</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1334,26 +1328,23 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>80.5</v>
+        <v>78.3</v>
       </c>
       <c r="J10" t="n">
-        <v>76.3</v>
+        <v>67.8</v>
       </c>
       <c r="K10" t="n">
-        <v>98</v>
+        <v>80</v>
       </c>
       <c r="L10" t="n">
-        <v>4.84</v>
+        <v>3.08</v>
       </c>
       <c r="M10" t="n">
-        <v>56.9</v>
-      </c>
-      <c r="N10" t="n">
-        <v>65.7</v>
+        <v>30.1</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1361,7 +1352,7 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>77.59999999999999</v>
+        <v>63</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1370,34 +1361,38 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U10" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>MCHP</t>
+          <t>GFS</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>88.69</v>
+        <v>64.23999999999999</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1430,22 +1425,22 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>79.09999999999999</v>
+        <v>78.3</v>
       </c>
       <c r="J11" t="n">
-        <v>71.59999999999999</v>
+        <v>77.8</v>
       </c>
       <c r="K11" t="n">
-        <v>87</v>
+        <v>98</v>
       </c>
       <c r="L11" t="n">
-        <v>4.22</v>
+        <v>4.62</v>
       </c>
       <c r="M11" t="n">
-        <v>48.3</v>
+        <v>55.9</v>
       </c>
       <c r="N11" t="n">
-        <v>71.7</v>
+        <v>63.5</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1453,7 +1448,7 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>69</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1485,11 +1480,11 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>UNH</t>
+          <t>MCHP</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>368.17</v>
+        <v>91.73999999999999</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1522,19 +1517,22 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>78.90000000000001</v>
+        <v>77.8</v>
       </c>
       <c r="J12" t="n">
-        <v>84.8</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="K12" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="L12" t="n">
-        <v>2.69</v>
+        <v>4.07</v>
       </c>
       <c r="M12" t="n">
-        <v>29.3</v>
+        <v>49.8</v>
+      </c>
+      <c r="N12" t="n">
+        <v>75.90000000000001</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1542,7 +1540,7 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>63.1</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1574,11 +1572,11 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>UNH</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>424.32</v>
+        <v>368.49</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -1611,27 +1609,27 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>77.40000000000001</v>
+        <v>77.09999999999999</v>
       </c>
       <c r="J13" t="n">
-        <v>61.7</v>
+        <v>82.7</v>
       </c>
       <c r="K13" t="n">
         <v>83</v>
       </c>
       <c r="L13" t="n">
-        <v>2.43</v>
+        <v>2.63</v>
       </c>
       <c r="M13" t="n">
-        <v>40.6</v>
+        <v>27.4</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>48.7</v>
+        <v>63.2</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1663,11 +1661,11 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ADI</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>389.14</v>
+        <v>201.13</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -1700,22 +1698,22 @@
         </is>
       </c>
       <c r="I14" t="n">
-        <v>76.90000000000001</v>
+        <v>76.2</v>
       </c>
       <c r="J14" t="n">
-        <v>66.7</v>
+        <v>55.7</v>
       </c>
       <c r="K14" t="n">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="L14" t="n">
-        <v>3.07</v>
+        <v>3.5</v>
       </c>
       <c r="M14" t="n">
-        <v>37.9</v>
+        <v>37.6</v>
       </c>
       <c r="N14" t="n">
-        <v>99</v>
+        <v>66.5</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1723,7 +1721,7 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>72.40000000000001</v>
+        <v>60</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1732,34 +1730,38 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U14" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>SNPS</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>210.71</v>
+        <v>480.37</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1792,22 +1794,19 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>76.2</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="J15" t="n">
-        <v>67.40000000000001</v>
+        <v>61.9</v>
       </c>
       <c r="K15" t="n">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="L15" t="n">
-        <v>2.87</v>
+        <v>3.7</v>
       </c>
       <c r="M15" t="n">
-        <v>35.3</v>
-      </c>
-      <c r="N15" t="n">
-        <v>55.3</v>
+        <v>56.1</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1815,7 +1814,7 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>66.09999999999999</v>
+        <v>54.4</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1847,11 +1846,11 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>519.66</v>
+        <v>403.18</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -1884,27 +1883,30 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>74</v>
+        <v>75.5</v>
       </c>
       <c r="J16" t="n">
-        <v>68.59999999999999</v>
+        <v>48.8</v>
       </c>
       <c r="K16" t="n">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="L16" t="n">
-        <v>5.4</v>
+        <v>3.06</v>
       </c>
       <c r="M16" t="n">
-        <v>76.3</v>
+        <v>33.8</v>
+      </c>
+      <c r="N16" t="n">
+        <v>72.5</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>73.40000000000001</v>
+        <v>43.8</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1913,53 +1915,57 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U16" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CPRT</t>
+          <t>D</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>33.07</v>
+        <v>63.73</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1973,34 +1979,31 @@
         </is>
       </c>
       <c r="I17" t="n">
-        <v>73.5</v>
+        <v>74.7</v>
       </c>
       <c r="J17" t="n">
-        <v>42.2</v>
+        <v>58.6</v>
       </c>
       <c r="K17" t="n">
         <v>12</v>
       </c>
       <c r="L17" t="n">
-        <v>2.06</v>
+        <v>1.88</v>
       </c>
       <c r="M17" t="n">
-        <v>19</v>
-      </c>
-      <c r="N17" t="n">
-        <v>14.6</v>
+        <v>25.9</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P17" t="n">
-        <v>31.6</v>
+        <v>57</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
@@ -2010,7 +2013,7 @@
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
@@ -2020,7 +2023,7 @@
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
+          <t>Squeeze Expanding</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
@@ -2032,11 +2035,11 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>NSC</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>154.37</v>
+        <v>312.29</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -2065,23 +2068,26 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>73.40000000000001</v>
+        <v>74.3</v>
       </c>
       <c r="J18" t="n">
-        <v>72.2</v>
+        <v>61</v>
       </c>
       <c r="K18" t="n">
-        <v>90</v>
+        <v>76</v>
       </c>
       <c r="L18" t="n">
-        <v>5.65</v>
+        <v>1.97</v>
       </c>
       <c r="M18" t="n">
-        <v>80.3</v>
+        <v>26.6</v>
+      </c>
+      <c r="N18" t="n">
+        <v>91.09999999999999</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -2089,7 +2095,7 @@
         </is>
       </c>
       <c r="P18" t="n">
-        <v>77</v>
+        <v>60.6</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -2098,17 +2104,17 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U18" t="inlineStr"/>
@@ -2121,11 +2127,11 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>ADI</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>589.09</v>
+        <v>398.9</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -2158,22 +2164,22 @@
         </is>
       </c>
       <c r="I19" t="n">
-        <v>73.09999999999999</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="J19" t="n">
-        <v>59.8</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="K19" t="n">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L19" t="n">
-        <v>2.64</v>
+        <v>2.97</v>
       </c>
       <c r="M19" t="n">
-        <v>27.3</v>
+        <v>37.5</v>
       </c>
       <c r="N19" t="n">
-        <v>44.7</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -2181,7 +2187,7 @@
         </is>
       </c>
       <c r="P19" t="n">
-        <v>55.7</v>
+        <v>76.5</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -2213,11 +2219,11 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>263.38</v>
+        <v>164.18</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -2250,19 +2256,19 @@
         </is>
       </c>
       <c r="I20" t="n">
-        <v>72.90000000000001</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="J20" t="n">
-        <v>75.7</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="K20" t="n">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="L20" t="n">
-        <v>2.45</v>
+        <v>5.34</v>
       </c>
       <c r="M20" t="n">
-        <v>41.8</v>
+        <v>83</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -2270,7 +2276,7 @@
         </is>
       </c>
       <c r="P20" t="n">
-        <v>65.8</v>
+        <v>84.8</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
@@ -2302,11 +2308,11 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>XLK</t>
+          <t>MU</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>158.38</v>
+        <v>509.21</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -2335,23 +2341,26 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>72.2</v>
+        <v>71.2</v>
       </c>
       <c r="J21" t="n">
-        <v>69.59999999999999</v>
+        <v>65.2</v>
       </c>
       <c r="K21" t="n">
-        <v>94</v>
+        <v>76</v>
       </c>
       <c r="L21" t="n">
-        <v>1.86</v>
+        <v>5.64</v>
       </c>
       <c r="M21" t="n">
-        <v>30.7</v>
+        <v>74.2</v>
+      </c>
+      <c r="N21" t="n">
+        <v>86.8</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
@@ -2359,7 +2368,7 @@
         </is>
       </c>
       <c r="P21" t="n">
-        <v>67.5</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
@@ -2391,11 +2400,11 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>351.07</v>
+        <v>588.22</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -2428,22 +2437,19 @@
         </is>
       </c>
       <c r="I22" t="n">
-        <v>71.40000000000001</v>
+        <v>70.3</v>
       </c>
       <c r="J22" t="n">
-        <v>71.7</v>
+        <v>58.4</v>
       </c>
       <c r="K22" t="n">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="L22" t="n">
-        <v>2.37</v>
+        <v>2.59</v>
       </c>
       <c r="M22" t="n">
-        <v>32.9</v>
-      </c>
-      <c r="N22" t="n">
-        <v>85</v>
+        <v>30.5</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
@@ -2451,7 +2457,7 @@
         </is>
       </c>
       <c r="P22" t="n">
-        <v>67.2</v>
+        <v>55.5</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
@@ -2460,17 +2466,17 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U22" t="inlineStr"/>
@@ -2483,11 +2489,11 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>GOOG</t>
+          <t>CSCO</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>348.7</v>
+        <v>90.63</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -2520,19 +2526,19 @@
         </is>
       </c>
       <c r="I23" t="n">
-        <v>71.09999999999999</v>
+        <v>70</v>
       </c>
       <c r="J23" t="n">
-        <v>71.90000000000001</v>
+        <v>68.7</v>
       </c>
       <c r="K23" t="n">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="L23" t="n">
-        <v>2.28</v>
+        <v>2.31</v>
       </c>
       <c r="M23" t="n">
-        <v>37.1</v>
+        <v>38.1</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -2540,7 +2546,7 @@
         </is>
       </c>
       <c r="P23" t="n">
-        <v>66.8</v>
+        <v>72</v>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
@@ -2572,11 +2578,11 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>XLK</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>659.28</v>
+        <v>158.42</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -2609,19 +2615,19 @@
         </is>
       </c>
       <c r="I24" t="n">
-        <v>70.09999999999999</v>
+        <v>69.2</v>
       </c>
       <c r="J24" t="n">
-        <v>69.90000000000001</v>
+        <v>68.5</v>
       </c>
       <c r="K24" t="n">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="L24" t="n">
-        <v>1.38</v>
+        <v>1.85</v>
       </c>
       <c r="M24" t="n">
-        <v>21.2</v>
+        <v>27.8</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
@@ -2629,7 +2635,7 @@
         </is>
       </c>
       <c r="P24" t="n">
-        <v>65.3</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
@@ -2661,11 +2667,11 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>APH</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>152.25</v>
+        <v>662.9299999999999</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -2698,22 +2704,22 @@
         </is>
       </c>
       <c r="I25" t="n">
-        <v>69.09999999999999</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="J25" t="n">
-        <v>61.6</v>
+        <v>71.2</v>
       </c>
       <c r="K25" t="n">
         <v>91</v>
       </c>
       <c r="L25" t="n">
-        <v>3.74</v>
+        <v>1.35</v>
       </c>
       <c r="M25" t="n">
-        <v>45.8</v>
+        <v>21.1</v>
       </c>
       <c r="N25" t="n">
-        <v>55.1</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
@@ -2721,7 +2727,7 @@
         </is>
       </c>
       <c r="P25" t="n">
-        <v>61.4</v>
+        <v>66.7</v>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
@@ -2753,59 +2759,56 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>PEP</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>88.68000000000001</v>
+        <v>157.56</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I26" t="n">
-        <v>67.5</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="J26" t="n">
-        <v>64.7</v>
+        <v>54</v>
       </c>
       <c r="K26" t="n">
-        <v>85</v>
+        <v>4</v>
       </c>
       <c r="L26" t="n">
-        <v>2.33</v>
+        <v>1.99</v>
       </c>
       <c r="M26" t="n">
-        <v>27.3</v>
-      </c>
-      <c r="N26" t="n">
-        <v>42.6</v>
+        <v>22.5</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
@@ -2813,11 +2816,11 @@
         </is>
       </c>
       <c r="P26" t="n">
-        <v>69.59999999999999</v>
+        <v>55</v>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
@@ -2827,15 +2830,19 @@
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U26" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V26" t="inlineStr">
         <is>
           <t>No</t>
@@ -2849,7 +2856,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>710.02</v>
+        <v>714.38</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -2882,22 +2889,22 @@
         </is>
       </c>
       <c r="I27" t="n">
-        <v>66.2</v>
+        <v>65</v>
       </c>
       <c r="J27" t="n">
-        <v>65.59999999999999</v>
+        <v>68.7</v>
       </c>
       <c r="K27" t="n">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="L27" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.9</v>
       </c>
       <c r="M27" t="n">
-        <v>17.1</v>
+        <v>16.4</v>
       </c>
       <c r="N27" t="n">
-        <v>90.8</v>
+        <v>84.5</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -2905,7 +2912,7 @@
         </is>
       </c>
       <c r="P27" t="n">
-        <v>63</v>
+        <v>64.8</v>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
@@ -2937,11 +2944,11 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ABNB</t>
+          <t>MET</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>138.66</v>
+        <v>80.29000000000001</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -2970,26 +2977,23 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I28" t="n">
-        <v>63.7</v>
+        <v>64.2</v>
       </c>
       <c r="J28" t="n">
-        <v>55.8</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="K28" t="n">
-        <v>87</v>
+        <v>74</v>
       </c>
       <c r="L28" t="n">
-        <v>3</v>
+        <v>1.96</v>
       </c>
       <c r="M28" t="n">
-        <v>33.9</v>
-      </c>
-      <c r="N28" t="n">
-        <v>66.7</v>
+        <v>27.5</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
@@ -2997,7 +3001,7 @@
         </is>
       </c>
       <c r="P28" t="n">
-        <v>56.7</v>
+        <v>58.2</v>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
@@ -3006,17 +3010,17 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U28" t="inlineStr"/>
@@ -3029,11 +3033,11 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ANET</t>
+          <t>ETN</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>163.54</v>
+        <v>426.55</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -3062,26 +3066,26 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I29" t="n">
-        <v>62.3</v>
+        <v>63.3</v>
       </c>
       <c r="J29" t="n">
-        <v>58.6</v>
+        <v>68.2</v>
       </c>
       <c r="K29" t="n">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="L29" t="n">
-        <v>4.14</v>
+        <v>2.97</v>
       </c>
       <c r="M29" t="n">
-        <v>57.9</v>
+        <v>35.9</v>
       </c>
       <c r="N29" t="n">
-        <v>73.2</v>
+        <v>82.2</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
@@ -3089,7 +3093,7 @@
         </is>
       </c>
       <c r="P29" t="n">
-        <v>61.5</v>
+        <v>69.2</v>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
@@ -3098,17 +3102,17 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U29" t="inlineStr"/>
@@ -3121,11 +3125,11 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>BLK</t>
+          <t>ANET</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>1032.68</v>
+        <v>170.04</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -3154,31 +3158,31 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I30" t="n">
-        <v>61.4</v>
+        <v>59.7</v>
       </c>
       <c r="J30" t="n">
-        <v>52.8</v>
+        <v>63.6</v>
       </c>
       <c r="K30" t="n">
-        <v>77</v>
+        <v>91</v>
       </c>
       <c r="L30" t="n">
-        <v>2.39</v>
+        <v>3.92</v>
       </c>
       <c r="M30" t="n">
-        <v>32.7</v>
+        <v>62.5</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P30" t="n">
-        <v>49.7</v>
+        <v>65.3</v>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
@@ -3210,11 +3214,11 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>KLAC</t>
+          <t>IWM</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1789.95</v>
+        <v>275.78</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -3243,23 +3247,26 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I31" t="n">
-        <v>61</v>
+        <v>59.2</v>
       </c>
       <c r="J31" t="n">
-        <v>57.9</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="K31" t="n">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="L31" t="n">
-        <v>3.97</v>
+        <v>1.54</v>
       </c>
       <c r="M31" t="n">
-        <v>55.5</v>
+        <v>21.4</v>
+      </c>
+      <c r="N31" t="n">
+        <v>72.5</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
@@ -3267,7 +3274,7 @@
         </is>
       </c>
       <c r="P31" t="n">
-        <v>66.3</v>
+        <v>66.7</v>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
@@ -3276,17 +3283,17 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U31" t="inlineStr"/>
@@ -3299,11 +3306,11 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>668.85</v>
+        <v>188.6</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -3336,19 +3343,19 @@
         </is>
       </c>
       <c r="I32" t="n">
-        <v>60.8</v>
+        <v>58.8</v>
       </c>
       <c r="J32" t="n">
-        <v>58.5</v>
+        <v>62.7</v>
       </c>
       <c r="K32" t="n">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="L32" t="n">
-        <v>2.44</v>
+        <v>2.36</v>
       </c>
       <c r="M32" t="n">
-        <v>43.3</v>
+        <v>28.2</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
@@ -3356,7 +3363,7 @@
         </is>
       </c>
       <c r="P32" t="n">
-        <v>52.8</v>
+        <v>63.8</v>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
@@ -3388,11 +3395,11 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>IWM</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>271.56</v>
+        <v>412.49</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -3425,22 +3432,19 @@
         </is>
       </c>
       <c r="I33" t="n">
-        <v>60.8</v>
+        <v>57.5</v>
       </c>
       <c r="J33" t="n">
-        <v>58.9</v>
+        <v>66.5</v>
       </c>
       <c r="K33" t="n">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="L33" t="n">
-        <v>1.54</v>
+        <v>3.21</v>
       </c>
       <c r="M33" t="n">
-        <v>22</v>
-      </c>
-      <c r="N33" t="n">
-        <v>78</v>
+        <v>47.2</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
@@ -3448,7 +3452,7 @@
         </is>
       </c>
       <c r="P33" t="n">
-        <v>62.8</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
@@ -3457,17 +3461,17 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U33" t="inlineStr"/>
@@ -3480,11 +3484,11 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>BK</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>186.02</v>
+        <v>134.16</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -3517,22 +3521,22 @@
         </is>
       </c>
       <c r="I34" t="n">
-        <v>60.2</v>
+        <v>54</v>
       </c>
       <c r="J34" t="n">
-        <v>59</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="K34" t="n">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="L34" t="n">
-        <v>2.36</v>
+        <v>1.97</v>
       </c>
       <c r="M34" t="n">
-        <v>28.1</v>
+        <v>19.2</v>
       </c>
       <c r="N34" t="n">
-        <v>51</v>
+        <v>32.6</v>
       </c>
       <c r="O34" t="inlineStr">
         <is>
@@ -3540,7 +3544,7 @@
         </is>
       </c>
       <c r="P34" t="n">
-        <v>61.7</v>
+        <v>72.5</v>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
@@ -3572,15 +3576,15 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ETN</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>410.69</v>
+        <v>326.9</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -3595,36 +3599,33 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I35" t="n">
-        <v>60.1</v>
+        <v>53.1</v>
       </c>
       <c r="J35" t="n">
-        <v>61.2</v>
+        <v>49.1</v>
       </c>
       <c r="K35" t="n">
-        <v>83</v>
+        <v>6</v>
       </c>
       <c r="L35" t="n">
-        <v>2.87</v>
+        <v>2.07</v>
       </c>
       <c r="M35" t="n">
-        <v>34.8</v>
-      </c>
-      <c r="N35" t="n">
-        <v>75.90000000000001</v>
+        <v>21.2</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
@@ -3632,11 +3633,11 @@
         </is>
       </c>
       <c r="P35" t="n">
-        <v>63.5</v>
+        <v>59</v>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
@@ -3654,7 +3655,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U35" t="inlineStr"/>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V35" t="inlineStr">
         <is>
           <t>No</t>
@@ -3664,11 +3669,11 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>MET</t>
+          <t>DLR</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>78.34</v>
+        <v>199.15</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -3697,23 +3702,26 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I36" t="n">
-        <v>60</v>
+        <v>49.8</v>
       </c>
       <c r="J36" t="n">
-        <v>65.90000000000001</v>
+        <v>65</v>
       </c>
       <c r="K36" t="n">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="L36" t="n">
-        <v>1.86</v>
+        <v>2.29</v>
       </c>
       <c r="M36" t="n">
-        <v>29.2</v>
+        <v>22.1</v>
+      </c>
+      <c r="N36" t="n">
+        <v>64.59999999999999</v>
       </c>
       <c r="O36" t="inlineStr">
         <is>
@@ -3721,7 +3729,7 @@
         </is>
       </c>
       <c r="P36" t="n">
-        <v>55.3</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
@@ -3730,17 +3738,17 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U36" t="inlineStr"/>
@@ -3753,11 +3761,11 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>C</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>399.01</v>
+        <v>128.41</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -3786,26 +3794,26 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I37" t="n">
-        <v>58</v>
+        <v>40.9</v>
       </c>
       <c r="J37" t="n">
-        <v>61.8</v>
+        <v>60.3</v>
       </c>
       <c r="K37" t="n">
-        <v>91</v>
+        <v>68</v>
       </c>
       <c r="L37" t="n">
-        <v>3.18</v>
+        <v>2.24</v>
       </c>
       <c r="M37" t="n">
-        <v>44.9</v>
+        <v>32.1</v>
       </c>
       <c r="N37" t="n">
-        <v>52.6</v>
+        <v>57.2</v>
       </c>
       <c r="O37" t="inlineStr">
         <is>
@@ -3813,7 +3821,7 @@
         </is>
       </c>
       <c r="P37" t="n">
-        <v>62.3</v>
+        <v>64.2</v>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
@@ -3837,649 +3845,6 @@
       </c>
       <c r="U37" t="inlineStr"/>
       <c r="V37" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>CAT</t>
-        </is>
-      </c>
-      <c r="B38" t="n">
-        <v>811.16</v>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>Credit Call</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I38" t="n">
-        <v>57.2</v>
-      </c>
-      <c r="J38" t="n">
-        <v>62.2</v>
-      </c>
-      <c r="K38" t="n">
-        <v>75</v>
-      </c>
-      <c r="L38" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="M38" t="n">
-        <v>37.5</v>
-      </c>
-      <c r="N38" t="n">
-        <v>69.8</v>
-      </c>
-      <c r="O38" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P38" t="n">
-        <v>71.59999999999999</v>
-      </c>
-      <c r="Q38" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R38" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S38" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="T38" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U38" t="inlineStr"/>
-      <c r="V38" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>BK</t>
-        </is>
-      </c>
-      <c r="B39" t="n">
-        <v>130.99</v>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D39" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>Credit Call</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I39" t="n">
-        <v>54.7</v>
-      </c>
-      <c r="J39" t="n">
-        <v>57.1</v>
-      </c>
-      <c r="K39" t="n">
-        <v>87</v>
-      </c>
-      <c r="L39" t="n">
-        <v>2.01</v>
-      </c>
-      <c r="M39" t="n">
-        <v>28.1</v>
-      </c>
-      <c r="O39" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P39" t="n">
-        <v>67.59999999999999</v>
-      </c>
-      <c r="Q39" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R39" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S39" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="T39" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U39" t="inlineStr"/>
-      <c r="V39" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>TT</t>
-        </is>
-      </c>
-      <c r="B40" t="n">
-        <v>480.92</v>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D40" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>Credit Call</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I40" t="n">
-        <v>54</v>
-      </c>
-      <c r="J40" t="n">
-        <v>64.5</v>
-      </c>
-      <c r="K40" t="n">
-        <v>73</v>
-      </c>
-      <c r="L40" t="n">
-        <v>2.22</v>
-      </c>
-      <c r="M40" t="n">
-        <v>32.9</v>
-      </c>
-      <c r="N40" t="n">
-        <v>81</v>
-      </c>
-      <c r="O40" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P40" t="n">
-        <v>64</v>
-      </c>
-      <c r="Q40" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R40" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S40" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="T40" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U40" t="inlineStr"/>
-      <c r="V40" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>CB</t>
-        </is>
-      </c>
-      <c r="B41" t="n">
-        <v>324.31</v>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>Debit Put</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>30-60 DTE</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>SQUEEZE</t>
-        </is>
-      </c>
-      <c r="I41" t="n">
-        <v>51.2</v>
-      </c>
-      <c r="J41" t="n">
-        <v>46.2</v>
-      </c>
-      <c r="K41" t="n">
-        <v>6</v>
-      </c>
-      <c r="L41" t="n">
-        <v>2.07</v>
-      </c>
-      <c r="M41" t="n">
-        <v>20.3</v>
-      </c>
-      <c r="O41" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P41" t="n">
-        <v>57.2</v>
-      </c>
-      <c r="Q41" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="R41" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S41" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="T41" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U41" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
-      <c r="V41" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>DLR</t>
-        </is>
-      </c>
-      <c r="B42" t="n">
-        <v>193.08</v>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>Credit Call</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I42" t="n">
-        <v>50.7</v>
-      </c>
-      <c r="J42" t="n">
-        <v>54.4</v>
-      </c>
-      <c r="K42" t="n">
-        <v>88</v>
-      </c>
-      <c r="L42" t="n">
-        <v>2.35</v>
-      </c>
-      <c r="M42" t="n">
-        <v>21.7</v>
-      </c>
-      <c r="N42" t="n">
-        <v>62.1</v>
-      </c>
-      <c r="O42" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P42" t="n">
-        <v>62.6</v>
-      </c>
-      <c r="Q42" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R42" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S42" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="T42" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U42" t="inlineStr"/>
-      <c r="V42" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="B43" t="n">
-        <v>126.84</v>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>Credit Call</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I43" t="n">
-        <v>44.3</v>
-      </c>
-      <c r="J43" t="n">
-        <v>56.9</v>
-      </c>
-      <c r="K43" t="n">
-        <v>74</v>
-      </c>
-      <c r="L43" t="n">
-        <v>2.33</v>
-      </c>
-      <c r="M43" t="n">
-        <v>32.4</v>
-      </c>
-      <c r="N43" t="n">
-        <v>58.2</v>
-      </c>
-      <c r="O43" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P43" t="n">
-        <v>62.8</v>
-      </c>
-      <c r="Q43" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R43" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S43" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="T43" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U43" t="inlineStr"/>
-      <c r="V43" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>KO</t>
-        </is>
-      </c>
-      <c r="B44" t="n">
-        <v>78.79000000000001</v>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>Debit Put</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>30-60 DTE</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I44" t="n">
-        <v>38.2</v>
-      </c>
-      <c r="J44" t="n">
-        <v>61.4</v>
-      </c>
-      <c r="K44" t="n">
-        <v>52</v>
-      </c>
-      <c r="L44" t="n">
-        <v>2.04</v>
-      </c>
-      <c r="M44" t="n">
-        <v>19.5</v>
-      </c>
-      <c r="O44" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P44" t="n">
-        <v>62.5</v>
-      </c>
-      <c r="Q44" t="inlineStr">
-        <is>
-          <t>FIRED</t>
-        </is>
-      </c>
-      <c r="R44" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="S44" t="inlineStr">
-        <is>
-          <t>maroon</t>
-        </is>
-      </c>
-      <c r="T44" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U44" t="inlineStr">
-        <is>
-          <t>Squeeze Fired</t>
-        </is>
-      </c>
-      <c r="V44" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Scan 01.05.2026 15:05 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V37"/>
+  <dimension ref="A1:V35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -448,7 +448,7 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="6" customWidth="1" min="10" max="10"/>
-    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="6" customWidth="1" min="11" max="11"/>
     <col width="6" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
     <col width="9" customWidth="1" min="14" max="14"/>
@@ -577,11 +577,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>NXPI</t>
+          <t>GOOG</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>286.66</v>
+        <v>380.16</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,19 +614,19 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>98.90000000000001</v>
+        <v>93.3</v>
       </c>
       <c r="J2" t="n">
-        <v>80</v>
+        <v>80.7</v>
       </c>
       <c r="K2" t="n">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="L2" t="n">
-        <v>5.15</v>
+        <v>2.91</v>
       </c>
       <c r="M2" t="n">
-        <v>44.5</v>
+        <v>30.3</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -634,7 +634,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>71.3</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -666,11 +666,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>INTC</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>93.54000000000001</v>
+        <v>383.7</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -703,19 +703,19 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>92.3</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="J3" t="n">
-        <v>83.90000000000001</v>
+        <v>81.3</v>
       </c>
       <c r="K3" t="n">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="L3" t="n">
-        <v>5.97</v>
+        <v>2.96</v>
       </c>
       <c r="M3" t="n">
-        <v>75</v>
+        <v>31.5</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -723,7 +723,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>85.59999999999999</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -759,7 +759,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>276.96</v>
+        <v>280.06</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -792,22 +792,19 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>90</v>
+        <v>90.40000000000001</v>
       </c>
       <c r="J4" t="n">
-        <v>76.2</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="K4" t="n">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="L4" t="n">
-        <v>3.85</v>
+        <v>3.68</v>
       </c>
       <c r="M4" t="n">
-        <v>62.8</v>
-      </c>
-      <c r="N4" t="n">
-        <v>98.8</v>
+        <v>37.3</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -815,7 +812,7 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>77</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -847,11 +844,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>374.95</v>
+        <v>351.46</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -884,19 +881,22 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>88.7</v>
+        <v>84.8</v>
       </c>
       <c r="J5" t="n">
-        <v>80.2</v>
+        <v>77.3</v>
       </c>
       <c r="K5" t="n">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="L5" t="n">
-        <v>2.93</v>
+        <v>5.06</v>
       </c>
       <c r="M5" t="n">
-        <v>32.5</v>
+        <v>65.40000000000001</v>
+      </c>
+      <c r="N5" t="n">
+        <v>50.9</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -904,7 +904,7 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>71.59999999999999</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -936,11 +936,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>CDNS</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>346.58</v>
+        <v>335.98</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -973,22 +973,19 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>87.59999999999999</v>
+        <v>84</v>
       </c>
       <c r="J6" t="n">
-        <v>77.8</v>
+        <v>63.8</v>
       </c>
       <c r="K6" t="n">
         <v>96</v>
       </c>
       <c r="L6" t="n">
-        <v>5.36</v>
+        <v>4.05</v>
       </c>
       <c r="M6" t="n">
-        <v>64.3</v>
-      </c>
-      <c r="N6" t="n">
-        <v>49.3</v>
+        <v>45.9</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -996,7 +993,7 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>77.2</v>
+        <v>58.9</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1028,11 +1025,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>GOOG</t>
+          <t>URI</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>371.77</v>
+        <v>949.3</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1065,19 +1062,19 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>87.40000000000001</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="J7" t="n">
-        <v>80.2</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="K7" t="n">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="L7" t="n">
-        <v>2.86</v>
+        <v>3.65</v>
       </c>
       <c r="M7" t="n">
-        <v>31</v>
+        <v>31.6</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1085,7 +1082,7 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>71.2</v>
+        <v>59.6</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1121,7 +1118,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>100.16</v>
+        <v>101.98</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1154,19 +1151,19 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>84.59999999999999</v>
+        <v>81.7</v>
       </c>
       <c r="J8" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="K8" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="L8" t="n">
-        <v>4.4</v>
+        <v>4.2</v>
       </c>
       <c r="M8" t="n">
-        <v>69.8</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1174,7 +1171,7 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>79</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1206,11 +1203,11 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>212.49</v>
+        <v>268.87</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1239,23 +1236,23 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>82.5</v>
+        <v>81.2</v>
       </c>
       <c r="J9" t="n">
-        <v>67.09999999999999</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="K9" t="n">
-        <v>100</v>
+        <v>79</v>
       </c>
       <c r="L9" t="n">
-        <v>7.14</v>
+        <v>3.08</v>
       </c>
       <c r="M9" t="n">
-        <v>85.2</v>
+        <v>29.2</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1263,7 +1260,7 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>69.5</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1295,11 +1292,11 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>257.83</v>
+        <v>213.09</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1328,23 +1325,26 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>78.3</v>
+        <v>80.2</v>
       </c>
       <c r="J10" t="n">
-        <v>67.8</v>
+        <v>67.3</v>
       </c>
       <c r="K10" t="n">
-        <v>80</v>
+        <v>98</v>
       </c>
       <c r="L10" t="n">
-        <v>3.08</v>
+        <v>6.82</v>
       </c>
       <c r="M10" t="n">
-        <v>30.1</v>
+        <v>94.2</v>
+      </c>
+      <c r="N10" t="n">
+        <v>99.8</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1352,7 +1352,7 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>63</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1361,38 +1361,34 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U10" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr"/>
       <c r="V10" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>GFS</t>
+          <t>MCHP</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>64.23999999999999</v>
+        <v>93.06999999999999</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1425,22 +1421,19 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>78.3</v>
+        <v>75.40000000000001</v>
       </c>
       <c r="J11" t="n">
-        <v>77.8</v>
+        <v>75.5</v>
       </c>
       <c r="K11" t="n">
-        <v>98</v>
+        <v>85</v>
       </c>
       <c r="L11" t="n">
-        <v>4.62</v>
+        <v>3.81</v>
       </c>
       <c r="M11" t="n">
-        <v>55.9</v>
-      </c>
-      <c r="N11" t="n">
-        <v>63.5</v>
+        <v>56.3</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1448,7 +1441,7 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>78.40000000000001</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1480,11 +1473,11 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>MCHP</t>
+          <t>GFS</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>91.73999999999999</v>
+        <v>63.81</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1517,22 +1510,19 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>77.8</v>
+        <v>75</v>
       </c>
       <c r="J12" t="n">
-        <v>74.40000000000001</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="K12" t="n">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="L12" t="n">
-        <v>4.07</v>
+        <v>4.32</v>
       </c>
       <c r="M12" t="n">
-        <v>49.8</v>
-      </c>
-      <c r="N12" t="n">
-        <v>75.90000000000001</v>
+        <v>70.8</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1540,7 +1530,7 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>71.40000000000001</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1572,11 +1562,11 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>UNH</t>
+          <t>CSCO</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>368.49</v>
+        <v>92.34999999999999</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -1609,19 +1599,22 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>77.09999999999999</v>
+        <v>73.2</v>
       </c>
       <c r="J13" t="n">
-        <v>82.7</v>
+        <v>71.7</v>
       </c>
       <c r="K13" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="L13" t="n">
-        <v>2.63</v>
+        <v>2.33</v>
       </c>
       <c r="M13" t="n">
-        <v>27.4</v>
+        <v>27.3</v>
+      </c>
+      <c r="N13" t="n">
+        <v>42.7</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1629,7 +1622,7 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>63.2</v>
+        <v>73.5</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1661,11 +1654,11 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>201.13</v>
+        <v>414.06</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -1694,34 +1687,31 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>76.2</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="J14" t="n">
-        <v>55.7</v>
+        <v>54.3</v>
       </c>
       <c r="K14" t="n">
-        <v>92</v>
+        <v>79</v>
       </c>
       <c r="L14" t="n">
-        <v>3.5</v>
+        <v>2.92</v>
       </c>
       <c r="M14" t="n">
-        <v>37.6</v>
-      </c>
-      <c r="N14" t="n">
-        <v>66.5</v>
+        <v>27.2</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P14" t="n">
-        <v>60</v>
+        <v>46.2</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1743,14 +1733,10 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U14" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U14" t="inlineStr"/>
       <c r="V14" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -1761,7 +1747,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>480.37</v>
+        <v>487.48</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1794,19 +1780,22 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>75.59999999999999</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="J15" t="n">
-        <v>61.9</v>
+        <v>64</v>
       </c>
       <c r="K15" t="n">
-        <v>92</v>
+        <v>85</v>
       </c>
       <c r="L15" t="n">
-        <v>3.7</v>
+        <v>3.62</v>
       </c>
       <c r="M15" t="n">
-        <v>56.1</v>
+        <v>50.2</v>
+      </c>
+      <c r="N15" t="n">
+        <v>23.2</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1814,7 +1803,7 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>54.4</v>
+        <v>55.5</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1846,11 +1835,11 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>ADI</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>403.18</v>
+        <v>396.68</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -1883,31 +1872,31 @@
         </is>
       </c>
       <c r="I16" t="n">
+        <v>72.8</v>
+      </c>
+      <c r="J16" t="n">
+        <v>67</v>
+      </c>
+      <c r="K16" t="n">
+        <v>84</v>
+      </c>
+      <c r="L16" t="n">
+        <v>2.95</v>
+      </c>
+      <c r="M16" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="N16" t="n">
+        <v>100</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P16" t="n">
         <v>75.5</v>
       </c>
-      <c r="J16" t="n">
-        <v>48.8</v>
-      </c>
-      <c r="K16" t="n">
-        <v>81</v>
-      </c>
-      <c r="L16" t="n">
-        <v>3.06</v>
-      </c>
-      <c r="M16" t="n">
-        <v>33.8</v>
-      </c>
-      <c r="N16" t="n">
-        <v>72.5</v>
-      </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P16" t="n">
-        <v>43.8</v>
-      </c>
       <c r="Q16" t="inlineStr">
         <is>
           <t>OFF</t>
@@ -1915,38 +1904,34 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U16" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr"/>
       <c r="V16" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>PEP</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>63.73</v>
+        <v>159.29</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -1979,19 +1964,19 @@
         </is>
       </c>
       <c r="I17" t="n">
-        <v>74.7</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="J17" t="n">
-        <v>58.6</v>
+        <v>57.6</v>
       </c>
       <c r="K17" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="L17" t="n">
-        <v>1.88</v>
+        <v>1.85</v>
       </c>
       <c r="M17" t="n">
-        <v>25.9</v>
+        <v>21.2</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -1999,11 +1984,11 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>57</v>
+        <v>56.4</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
@@ -2018,12 +2003,12 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>Squeeze Expanding</t>
+          <t>TTM Squeeze, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
@@ -2035,11 +2020,11 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>NSC</t>
+          <t>UNH</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>312.29</v>
+        <v>368.92</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -2072,22 +2057,19 @@
         </is>
       </c>
       <c r="I18" t="n">
-        <v>74.3</v>
+        <v>71.7</v>
       </c>
       <c r="J18" t="n">
-        <v>61</v>
+        <v>83</v>
       </c>
       <c r="K18" t="n">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="L18" t="n">
-        <v>1.97</v>
+        <v>2.53</v>
       </c>
       <c r="M18" t="n">
-        <v>26.6</v>
-      </c>
-      <c r="N18" t="n">
-        <v>91.09999999999999</v>
+        <v>25.9</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -2095,7 +2077,7 @@
         </is>
       </c>
       <c r="P18" t="n">
-        <v>60.6</v>
+        <v>63.2</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -2127,11 +2109,11 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ADI</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>398.9</v>
+        <v>673</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -2164,22 +2146,22 @@
         </is>
       </c>
       <c r="I19" t="n">
-        <v>73.59999999999999</v>
+        <v>69.8</v>
       </c>
       <c r="J19" t="n">
-        <v>69.90000000000001</v>
+        <v>74.5</v>
       </c>
       <c r="K19" t="n">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="L19" t="n">
-        <v>2.97</v>
+        <v>1.37</v>
       </c>
       <c r="M19" t="n">
-        <v>37.5</v>
+        <v>21</v>
       </c>
       <c r="N19" t="n">
-        <v>97.40000000000001</v>
+        <v>91.40000000000001</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -2187,7 +2169,7 @@
         </is>
       </c>
       <c r="P19" t="n">
-        <v>76.5</v>
+        <v>68.7</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -2223,7 +2205,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>164.18</v>
+        <v>163.14</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -2256,19 +2238,22 @@
         </is>
       </c>
       <c r="I20" t="n">
-        <v>71.59999999999999</v>
+        <v>69.5</v>
       </c>
       <c r="J20" t="n">
-        <v>76.59999999999999</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="K20" t="n">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="L20" t="n">
-        <v>5.34</v>
+        <v>5.19</v>
       </c>
       <c r="M20" t="n">
-        <v>83</v>
+        <v>65.3</v>
+      </c>
+      <c r="N20" t="n">
+        <v>64</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -2276,7 +2261,7 @@
         </is>
       </c>
       <c r="P20" t="n">
-        <v>84.8</v>
+        <v>83.90000000000001</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
@@ -2285,17 +2270,17 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U20" t="inlineStr"/>
@@ -2308,11 +2293,11 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>XLK</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>509.21</v>
+        <v>161.04</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -2341,26 +2326,23 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>71.2</v>
+        <v>68.7</v>
       </c>
       <c r="J21" t="n">
-        <v>65.2</v>
+        <v>72.7</v>
       </c>
       <c r="K21" t="n">
-        <v>76</v>
+        <v>90</v>
       </c>
       <c r="L21" t="n">
-        <v>5.64</v>
+        <v>1.81</v>
       </c>
       <c r="M21" t="n">
-        <v>74.2</v>
-      </c>
-      <c r="N21" t="n">
-        <v>86.8</v>
+        <v>29.6</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
@@ -2368,7 +2350,7 @@
         </is>
       </c>
       <c r="P21" t="n">
-        <v>72.59999999999999</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
@@ -2400,56 +2382,56 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>LIN</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>588.22</v>
+        <v>517.09</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I22" t="n">
-        <v>70.3</v>
+        <v>68.5</v>
       </c>
       <c r="J22" t="n">
-        <v>58.4</v>
+        <v>62.5</v>
       </c>
       <c r="K22" t="n">
-        <v>81</v>
+        <v>9</v>
       </c>
       <c r="L22" t="n">
-        <v>2.59</v>
+        <v>1.92</v>
       </c>
       <c r="M22" t="n">
-        <v>30.5</v>
+        <v>25.2</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
@@ -2457,21 +2439,21 @@
         </is>
       </c>
       <c r="P22" t="n">
-        <v>55.5</v>
+        <v>66.5</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
@@ -2479,7 +2461,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U22" t="inlineStr"/>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V22" t="inlineStr">
         <is>
           <t>No</t>
@@ -2489,11 +2475,11 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>MU</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>90.63</v>
+        <v>526.28</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -2522,23 +2508,26 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I23" t="n">
-        <v>70</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="J23" t="n">
-        <v>68.7</v>
+        <v>69.5</v>
       </c>
       <c r="K23" t="n">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="L23" t="n">
-        <v>2.31</v>
+        <v>5.63</v>
       </c>
       <c r="M23" t="n">
-        <v>38.1</v>
+        <v>72.90000000000001</v>
+      </c>
+      <c r="N23" t="n">
+        <v>84.2</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -2546,7 +2535,7 @@
         </is>
       </c>
       <c r="P23" t="n">
-        <v>72</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
@@ -2578,11 +2567,11 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>XLK</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>158.42</v>
+        <v>722.36</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -2615,19 +2604,19 @@
         </is>
       </c>
       <c r="I24" t="n">
-        <v>69.2</v>
+        <v>67.7</v>
       </c>
       <c r="J24" t="n">
-        <v>68.5</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="K24" t="n">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="L24" t="n">
-        <v>1.85</v>
+        <v>0.97</v>
       </c>
       <c r="M24" t="n">
-        <v>27.8</v>
+        <v>14.1</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
@@ -2635,7 +2624,7 @@
         </is>
       </c>
       <c r="P24" t="n">
-        <v>67.59999999999999</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
@@ -2667,11 +2656,11 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>662.9299999999999</v>
+        <v>199.45</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -2704,22 +2693,19 @@
         </is>
       </c>
       <c r="I25" t="n">
-        <v>67.90000000000001</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="J25" t="n">
-        <v>71.2</v>
+        <v>54</v>
       </c>
       <c r="K25" t="n">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="L25" t="n">
-        <v>1.35</v>
+        <v>3.45</v>
       </c>
       <c r="M25" t="n">
-        <v>21.1</v>
-      </c>
-      <c r="N25" t="n">
-        <v>91.59999999999999</v>
+        <v>44.4</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
@@ -2727,7 +2713,7 @@
         </is>
       </c>
       <c r="P25" t="n">
-        <v>66.7</v>
+        <v>59</v>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
@@ -2736,17 +2722,17 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U25" t="inlineStr"/>
@@ -2759,56 +2745,59 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>PEP</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>157.56</v>
+        <v>592.45</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D26" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I26" t="n">
-        <v>65.40000000000001</v>
+        <v>67.5</v>
       </c>
       <c r="J26" t="n">
-        <v>54</v>
+        <v>60.6</v>
       </c>
       <c r="K26" t="n">
-        <v>4</v>
+        <v>80</v>
       </c>
       <c r="L26" t="n">
-        <v>1.99</v>
+        <v>2.49</v>
       </c>
       <c r="M26" t="n">
-        <v>22.5</v>
+        <v>27.2</v>
+      </c>
+      <c r="N26" t="n">
+        <v>44.6</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
@@ -2816,21 +2805,21 @@
         </is>
       </c>
       <c r="P26" t="n">
-        <v>55</v>
+        <v>56.4</v>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
@@ -2838,11 +2827,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U26" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U26" t="inlineStr"/>
       <c r="V26" t="inlineStr">
         <is>
           <t>No</t>
@@ -2852,11 +2837,11 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>ETN</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>714.38</v>
+        <v>424.56</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -2885,26 +2870,26 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I27" t="n">
-        <v>65</v>
+        <v>65.5</v>
       </c>
       <c r="J27" t="n">
-        <v>68.7</v>
+        <v>64.2</v>
       </c>
       <c r="K27" t="n">
-        <v>90</v>
+        <v>77</v>
       </c>
       <c r="L27" t="n">
-        <v>0.9</v>
+        <v>3.17</v>
       </c>
       <c r="M27" t="n">
-        <v>16.4</v>
+        <v>38.1</v>
       </c>
       <c r="N27" t="n">
-        <v>84.5</v>
+        <v>94.8</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -2912,7 +2897,7 @@
         </is>
       </c>
       <c r="P27" t="n">
-        <v>64.8</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
@@ -2944,11 +2929,11 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>MET</t>
+          <t>IWM</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>80.29000000000001</v>
+        <v>278.09</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -2977,23 +2962,26 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I28" t="n">
-        <v>64.2</v>
+        <v>60.2</v>
       </c>
       <c r="J28" t="n">
-        <v>71.40000000000001</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="K28" t="n">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="L28" t="n">
-        <v>1.96</v>
+        <v>1.55</v>
       </c>
       <c r="M28" t="n">
-        <v>27.5</v>
+        <v>21.8</v>
+      </c>
+      <c r="N28" t="n">
+        <v>76.40000000000001</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
@@ -3001,7 +2989,7 @@
         </is>
       </c>
       <c r="P28" t="n">
-        <v>58.2</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
@@ -3033,11 +3021,11 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ETN</t>
+          <t>ANET</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>426.55</v>
+        <v>174.82</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -3066,34 +3054,31 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I29" t="n">
-        <v>63.3</v>
+        <v>59.5</v>
       </c>
       <c r="J29" t="n">
+        <v>66.5</v>
+      </c>
+      <c r="K29" t="n">
+        <v>89</v>
+      </c>
+      <c r="L29" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="M29" t="n">
+        <v>61.6</v>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P29" t="n">
         <v>68.2</v>
-      </c>
-      <c r="K29" t="n">
-        <v>80</v>
-      </c>
-      <c r="L29" t="n">
-        <v>2.97</v>
-      </c>
-      <c r="M29" t="n">
-        <v>35.9</v>
-      </c>
-      <c r="N29" t="n">
-        <v>82.2</v>
-      </c>
-      <c r="O29" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P29" t="n">
-        <v>69.2</v>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
@@ -3125,56 +3110,59 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ANET</t>
+          <t>D</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>170.04</v>
+        <v>65.01000000000001</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I30" t="n">
-        <v>59.7</v>
+        <v>59.4</v>
       </c>
       <c r="J30" t="n">
-        <v>63.6</v>
+        <v>64.5</v>
       </c>
       <c r="K30" t="n">
-        <v>91</v>
+        <v>31</v>
       </c>
       <c r="L30" t="n">
-        <v>3.92</v>
+        <v>2.08</v>
       </c>
       <c r="M30" t="n">
-        <v>62.5</v>
+        <v>20.2</v>
+      </c>
+      <c r="N30" t="n">
+        <v>75.8</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
@@ -3182,7 +3170,7 @@
         </is>
       </c>
       <c r="P30" t="n">
-        <v>65.3</v>
+        <v>59.5</v>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
@@ -3191,17 +3179,17 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U30" t="inlineStr"/>
@@ -3214,11 +3202,11 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>IWM</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>275.78</v>
+        <v>191.79</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -3247,26 +3235,26 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I31" t="n">
-        <v>59.2</v>
+        <v>59.4</v>
       </c>
       <c r="J31" t="n">
-        <v>64.09999999999999</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="K31" t="n">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="L31" t="n">
-        <v>1.54</v>
+        <v>2.41</v>
       </c>
       <c r="M31" t="n">
-        <v>21.4</v>
+        <v>28</v>
       </c>
       <c r="N31" t="n">
-        <v>72.5</v>
+        <v>50.7</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
@@ -3274,7 +3262,7 @@
         </is>
       </c>
       <c r="P31" t="n">
-        <v>66.7</v>
+        <v>65.8</v>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
@@ -3306,11 +3294,11 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>188.6</v>
+        <v>419.9</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -3343,19 +3331,22 @@
         </is>
       </c>
       <c r="I32" t="n">
-        <v>58.8</v>
+        <v>58.4</v>
       </c>
       <c r="J32" t="n">
-        <v>62.7</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="K32" t="n">
         <v>88</v>
       </c>
       <c r="L32" t="n">
-        <v>2.36</v>
+        <v>3.02</v>
       </c>
       <c r="M32" t="n">
-        <v>28.2</v>
+        <v>44.6</v>
+      </c>
+      <c r="N32" t="n">
+        <v>51.8</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
@@ -3363,7 +3354,7 @@
         </is>
       </c>
       <c r="P32" t="n">
-        <v>63.8</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
@@ -3372,17 +3363,17 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U32" t="inlineStr"/>
@@ -3395,56 +3386,56 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>412.49</v>
+        <v>329.89</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I33" t="n">
-        <v>57.5</v>
+        <v>57.1</v>
       </c>
       <c r="J33" t="n">
-        <v>66.5</v>
+        <v>52.6</v>
       </c>
       <c r="K33" t="n">
-        <v>89</v>
+        <v>7</v>
       </c>
       <c r="L33" t="n">
-        <v>3.21</v>
+        <v>1.96</v>
       </c>
       <c r="M33" t="n">
-        <v>47.2</v>
+        <v>20.8</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
@@ -3452,11 +3443,11 @@
         </is>
       </c>
       <c r="P33" t="n">
-        <v>65.90000000000001</v>
+        <v>60.6</v>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
@@ -3471,10 +3462,14 @@
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U33" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V33" t="inlineStr">
         <is>
           <t>No</t>
@@ -3488,7 +3483,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>134.16</v>
+        <v>135.32</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -3517,26 +3512,26 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I34" t="n">
-        <v>54</v>
+        <v>54.2</v>
       </c>
       <c r="J34" t="n">
-        <v>64.90000000000001</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="K34" t="n">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="L34" t="n">
-        <v>1.97</v>
+        <v>2.02</v>
       </c>
       <c r="M34" t="n">
         <v>19.2</v>
       </c>
       <c r="N34" t="n">
-        <v>32.6</v>
+        <v>32.9</v>
       </c>
       <c r="O34" t="inlineStr">
         <is>
@@ -3544,7 +3539,7 @@
         </is>
       </c>
       <c r="P34" t="n">
-        <v>72.5</v>
+        <v>73.3</v>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
@@ -3576,15 +3571,15 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>DLR</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>326.9</v>
+        <v>200.28</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -3599,33 +3594,36 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I35" t="n">
-        <v>53.1</v>
+        <v>50.2</v>
       </c>
       <c r="J35" t="n">
-        <v>49.1</v>
+        <v>65.5</v>
       </c>
       <c r="K35" t="n">
-        <v>6</v>
+        <v>79</v>
       </c>
       <c r="L35" t="n">
-        <v>2.07</v>
+        <v>2.28</v>
       </c>
       <c r="M35" t="n">
-        <v>21.2</v>
+        <v>23.1</v>
+      </c>
+      <c r="N35" t="n">
+        <v>70.7</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
@@ -3633,11 +3631,11 @@
         </is>
       </c>
       <c r="P35" t="n">
-        <v>59</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
@@ -3655,196 +3653,8 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U35" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U35" t="inlineStr"/>
       <c r="V35" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>DLR</t>
-        </is>
-      </c>
-      <c r="B36" t="n">
-        <v>199.15</v>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D36" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>Credit Call</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I36" t="n">
-        <v>49.8</v>
-      </c>
-      <c r="J36" t="n">
-        <v>65</v>
-      </c>
-      <c r="K36" t="n">
-        <v>83</v>
-      </c>
-      <c r="L36" t="n">
-        <v>2.29</v>
-      </c>
-      <c r="M36" t="n">
-        <v>22.1</v>
-      </c>
-      <c r="N36" t="n">
-        <v>64.59999999999999</v>
-      </c>
-      <c r="O36" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P36" t="n">
-        <v>68.09999999999999</v>
-      </c>
-      <c r="Q36" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R36" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S36" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="T36" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U36" t="inlineStr"/>
-      <c r="V36" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="B37" t="n">
-        <v>128.41</v>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>Credit Call</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I37" t="n">
-        <v>40.9</v>
-      </c>
-      <c r="J37" t="n">
-        <v>60.3</v>
-      </c>
-      <c r="K37" t="n">
-        <v>68</v>
-      </c>
-      <c r="L37" t="n">
-        <v>2.24</v>
-      </c>
-      <c r="M37" t="n">
-        <v>32.1</v>
-      </c>
-      <c r="N37" t="n">
-        <v>57.2</v>
-      </c>
-      <c r="O37" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P37" t="n">
-        <v>64.2</v>
-      </c>
-      <c r="Q37" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R37" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S37" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="T37" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U37" t="inlineStr"/>
-      <c r="V37" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Scan 04.05.2026 16:07 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V35"/>
+  <dimension ref="A1:V33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -577,11 +577,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>GOOG</t>
+          <t>TXN</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>380.16</v>
+        <v>279.83</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,19 +614,19 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>93.3</v>
+        <v>88.8</v>
       </c>
       <c r="J2" t="n">
-        <v>80.7</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="K2" t="n">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="L2" t="n">
-        <v>2.91</v>
+        <v>3.57</v>
       </c>
       <c r="M2" t="n">
-        <v>30.3</v>
+        <v>39.9</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -634,7 +634,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>72.59999999999999</v>
+        <v>77</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -666,11 +666,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>INTC</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>383.7</v>
+        <v>97.28</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -703,19 +703,22 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>92.90000000000001</v>
+        <v>87.5</v>
       </c>
       <c r="J3" t="n">
-        <v>81.3</v>
+        <v>82.7</v>
       </c>
       <c r="K3" t="n">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="L3" t="n">
-        <v>2.96</v>
+        <v>5.72</v>
       </c>
       <c r="M3" t="n">
-        <v>31.5</v>
+        <v>94.59999999999999</v>
+      </c>
+      <c r="N3" t="n">
+        <v>97</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -723,7 +726,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>72.90000000000001</v>
+        <v>83.90000000000001</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -755,11 +758,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TXN</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>280.06</v>
+        <v>341.39</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -792,19 +795,22 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>90.40000000000001</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="J4" t="n">
-        <v>76.40000000000001</v>
+        <v>69.8</v>
       </c>
       <c r="K4" t="n">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="L4" t="n">
-        <v>3.68</v>
+        <v>5.57</v>
       </c>
       <c r="M4" t="n">
-        <v>37.3</v>
+        <v>67.40000000000001</v>
+      </c>
+      <c r="N4" t="n">
+        <v>53.8</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -812,7 +818,7 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>77.59999999999999</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -834,21 +840,25 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr"/>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>CDNS</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>351.46</v>
+        <v>348.63</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -881,22 +891,22 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>84.8</v>
+        <v>84.5</v>
       </c>
       <c r="J5" t="n">
-        <v>77.3</v>
+        <v>68</v>
       </c>
       <c r="K5" t="n">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="L5" t="n">
-        <v>5.06</v>
+        <v>3.78</v>
       </c>
       <c r="M5" t="n">
-        <v>65.40000000000001</v>
+        <v>48.6</v>
       </c>
       <c r="N5" t="n">
-        <v>50.9</v>
+        <v>80</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -904,7 +914,7 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>77.90000000000001</v>
+        <v>61.8</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -936,11 +946,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CDNS</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>335.98</v>
+        <v>102.31</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -973,19 +983,22 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="J6" t="n">
-        <v>63.8</v>
+        <v>79.8</v>
       </c>
       <c r="K6" t="n">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="L6" t="n">
-        <v>4.05</v>
+        <v>4.13</v>
       </c>
       <c r="M6" t="n">
-        <v>45.9</v>
+        <v>63.5</v>
+      </c>
+      <c r="N6" t="n">
+        <v>96.09999999999999</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -993,7 +1006,7 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>58.9</v>
+        <v>79</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1025,11 +1038,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>URI</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>949.3</v>
+        <v>270.55</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1058,23 +1071,23 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>82.09999999999999</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="J7" t="n">
-        <v>70.59999999999999</v>
+        <v>79.2</v>
       </c>
       <c r="K7" t="n">
-        <v>99</v>
+        <v>75</v>
       </c>
       <c r="L7" t="n">
-        <v>3.65</v>
+        <v>3.04</v>
       </c>
       <c r="M7" t="n">
-        <v>31.6</v>
+        <v>30.6</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1082,7 +1095,7 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>59.6</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1114,11 +1127,11 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>GFS</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>101.98</v>
+        <v>67.25</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1151,19 +1164,22 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>81.7</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="J8" t="n">
         <v>81</v>
       </c>
       <c r="K8" t="n">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="L8" t="n">
-        <v>4.2</v>
+        <v>4.5</v>
       </c>
       <c r="M8" t="n">
-        <v>69.09999999999999</v>
+        <v>56</v>
+      </c>
+      <c r="N8" t="n">
+        <v>63.8</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1171,7 +1187,7 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>79.59999999999999</v>
+        <v>80.09999999999999</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1203,11 +1219,11 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>URI</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>268.87</v>
+        <v>931.37</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1236,23 +1252,26 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>81.2</v>
+        <v>77.5</v>
       </c>
       <c r="J9" t="n">
-        <v>78.40000000000001</v>
+        <v>65.7</v>
       </c>
       <c r="K9" t="n">
-        <v>79</v>
+        <v>97</v>
       </c>
       <c r="L9" t="n">
-        <v>3.08</v>
+        <v>3.63</v>
       </c>
       <c r="M9" t="n">
-        <v>29.2</v>
+        <v>70.09999999999999</v>
+      </c>
+      <c r="N9" t="n">
+        <v>95.09999999999999</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1260,7 +1279,7 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>67.40000000000001</v>
+        <v>57.8</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1296,7 +1315,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>213.09</v>
+        <v>200.32</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1329,22 +1348,19 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>80.2</v>
+        <v>75.7</v>
       </c>
       <c r="J10" t="n">
-        <v>67.3</v>
+        <v>60.4</v>
       </c>
       <c r="K10" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="L10" t="n">
-        <v>6.82</v>
+        <v>7.32</v>
       </c>
       <c r="M10" t="n">
-        <v>94.2</v>
-      </c>
-      <c r="N10" t="n">
-        <v>99.8</v>
+        <v>81.40000000000001</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1352,7 +1368,7 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>69.59999999999999</v>
+        <v>64.8</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1361,23 +1377,27 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U10" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1388,7 +1408,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>93.06999999999999</v>
+        <v>94.73999999999999</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1424,16 +1444,19 @@
         <v>75.40000000000001</v>
       </c>
       <c r="J11" t="n">
-        <v>75.5</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="K11" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="L11" t="n">
-        <v>3.81</v>
+        <v>3.77</v>
       </c>
       <c r="M11" t="n">
-        <v>56.3</v>
+        <v>48.7</v>
+      </c>
+      <c r="N11" t="n">
+        <v>72.90000000000001</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1441,7 +1464,7 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>72.09999999999999</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1473,11 +1496,11 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>GFS</t>
+          <t>CSCO</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>63.81</v>
+        <v>92.53</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1506,23 +1529,26 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>75</v>
+        <v>72.2</v>
       </c>
       <c r="J12" t="n">
-        <v>75.09999999999999</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="K12" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="L12" t="n">
-        <v>4.32</v>
+        <v>2.29</v>
       </c>
       <c r="M12" t="n">
-        <v>70.8</v>
+        <v>26.8</v>
+      </c>
+      <c r="N12" t="n">
+        <v>41.3</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1530,7 +1556,7 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>78.09999999999999</v>
+        <v>73.7</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1562,11 +1588,11 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>ADI</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>92.34999999999999</v>
+        <v>393.93</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -1599,22 +1625,22 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>73.2</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="J13" t="n">
-        <v>71.7</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="K13" t="n">
         <v>82</v>
       </c>
       <c r="L13" t="n">
-        <v>2.33</v>
+        <v>2.88</v>
       </c>
       <c r="M13" t="n">
-        <v>27.3</v>
+        <v>38.5</v>
       </c>
       <c r="N13" t="n">
-        <v>42.7</v>
+        <v>100</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1622,7 +1648,7 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>73.5</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1631,17 +1657,17 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U13" t="inlineStr"/>
@@ -1654,11 +1680,11 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>SNPS</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>414.06</v>
+        <v>492.83</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -1687,31 +1713,34 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>72.90000000000001</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="J14" t="n">
-        <v>54.3</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="K14" t="n">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="L14" t="n">
-        <v>2.92</v>
+        <v>3.37</v>
       </c>
       <c r="M14" t="n">
-        <v>27.2</v>
+        <v>49.8</v>
+      </c>
+      <c r="N14" t="n">
+        <v>22.7</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P14" t="n">
-        <v>46.2</v>
+        <v>56.3</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1720,17 +1749,17 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U14" t="inlineStr"/>
@@ -1743,59 +1772,59 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SNPS</t>
+          <t>PEP</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>487.48</v>
+        <v>155.55</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>72.90000000000001</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="J15" t="n">
-        <v>64</v>
+        <v>48.7</v>
       </c>
       <c r="K15" t="n">
-        <v>85</v>
+        <v>6</v>
       </c>
       <c r="L15" t="n">
-        <v>3.62</v>
+        <v>1.97</v>
       </c>
       <c r="M15" t="n">
-        <v>50.2</v>
+        <v>19</v>
       </c>
       <c r="N15" t="n">
-        <v>23.2</v>
+        <v>23.1</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1803,21 +1832,21 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>55.5</v>
+        <v>53</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
@@ -1825,7 +1854,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U15" t="inlineStr"/>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
       <c r="V15" t="inlineStr">
         <is>
           <t>No</t>
@@ -1835,11 +1868,11 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ADI</t>
+          <t>XLK</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>396.68</v>
+        <v>161.31</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -1872,22 +1905,19 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>72.8</v>
+        <v>66.3</v>
       </c>
       <c r="J16" t="n">
-        <v>67</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="K16" t="n">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="L16" t="n">
-        <v>2.95</v>
+        <v>1.73</v>
       </c>
       <c r="M16" t="n">
-        <v>38.5</v>
-      </c>
-      <c r="N16" t="n">
-        <v>100</v>
+        <v>29.1</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -1895,7 +1925,7 @@
         </is>
       </c>
       <c r="P16" t="n">
-        <v>75.5</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1927,56 +1957,59 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>PEP</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>159.29</v>
+        <v>670.73</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>72.09999999999999</v>
+        <v>66</v>
       </c>
       <c r="J17" t="n">
-        <v>57.6</v>
+        <v>71.8</v>
       </c>
       <c r="K17" t="n">
-        <v>7</v>
+        <v>88</v>
       </c>
       <c r="L17" t="n">
-        <v>1.85</v>
+        <v>1.32</v>
       </c>
       <c r="M17" t="n">
-        <v>21.2</v>
+        <v>20.1</v>
+      </c>
+      <c r="N17" t="n">
+        <v>84.8</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -1984,11 +2017,11 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>56.4</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
@@ -2003,14 +2036,10 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U17" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr"/>
       <c r="V17" t="inlineStr">
         <is>
           <t>No</t>
@@ -2020,11 +2049,11 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>UNH</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>368.92</v>
+        <v>164.05</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -2053,23 +2082,26 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>71.7</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="J18" t="n">
-        <v>83</v>
+        <v>75.40000000000001</v>
       </c>
       <c r="K18" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="L18" t="n">
-        <v>2.53</v>
+        <v>4.87</v>
       </c>
       <c r="M18" t="n">
-        <v>25.9</v>
+        <v>64.40000000000001</v>
+      </c>
+      <c r="N18" t="n">
+        <v>62.1</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -2077,7 +2109,7 @@
         </is>
       </c>
       <c r="P18" t="n">
-        <v>63.2</v>
+        <v>84.3</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -2086,17 +2118,17 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U18" t="inlineStr"/>
@@ -2109,11 +2141,11 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>ORCL</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>673</v>
+        <v>181.43</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -2146,30 +2178,30 @@
         </is>
       </c>
       <c r="I19" t="n">
-        <v>69.8</v>
+        <v>65.2</v>
       </c>
       <c r="J19" t="n">
-        <v>74.5</v>
+        <v>62.4</v>
       </c>
       <c r="K19" t="n">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="L19" t="n">
-        <v>1.37</v>
+        <v>5.1</v>
       </c>
       <c r="M19" t="n">
-        <v>21</v>
+        <v>63.3</v>
       </c>
       <c r="N19" t="n">
-        <v>91.40000000000001</v>
+        <v>38.6</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P19" t="n">
-        <v>68.7</v>
+        <v>51.6</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -2201,11 +2233,11 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>UNH</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>163.14</v>
+        <v>368.59</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -2234,26 +2266,23 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I20" t="n">
-        <v>69.5</v>
+        <v>65.2</v>
       </c>
       <c r="J20" t="n">
-        <v>74.40000000000001</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="K20" t="n">
-        <v>87</v>
+        <v>76</v>
       </c>
       <c r="L20" t="n">
-        <v>5.19</v>
+        <v>2.4</v>
       </c>
       <c r="M20" t="n">
-        <v>65.3</v>
-      </c>
-      <c r="N20" t="n">
-        <v>64</v>
+        <v>29</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -2261,7 +2290,7 @@
         </is>
       </c>
       <c r="P20" t="n">
-        <v>83.90000000000001</v>
+        <v>63.1</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
@@ -2293,11 +2322,11 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>XLK</t>
+          <t>ETN</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>161.04</v>
+        <v>427.54</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -2326,23 +2355,26 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>68.7</v>
+        <v>62.8</v>
       </c>
       <c r="J21" t="n">
-        <v>72.7</v>
+        <v>65.7</v>
       </c>
       <c r="K21" t="n">
-        <v>90</v>
+        <v>68</v>
       </c>
       <c r="L21" t="n">
-        <v>1.81</v>
+        <v>3.04</v>
       </c>
       <c r="M21" t="n">
-        <v>29.6</v>
+        <v>37.7</v>
+      </c>
+      <c r="N21" t="n">
+        <v>92.5</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
@@ -2350,7 +2382,7 @@
         </is>
       </c>
       <c r="P21" t="n">
-        <v>70.59999999999999</v>
+        <v>69.5</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
@@ -2382,56 +2414,59 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>LIN</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>517.09</v>
+        <v>717.1900000000001</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I22" t="n">
-        <v>68.5</v>
+        <v>62.5</v>
       </c>
       <c r="J22" t="n">
-        <v>62.5</v>
+        <v>67.7</v>
       </c>
       <c r="K22" t="n">
-        <v>9</v>
+        <v>86</v>
       </c>
       <c r="L22" t="n">
-        <v>1.92</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="M22" t="n">
-        <v>25.2</v>
+        <v>15.8</v>
+      </c>
+      <c r="N22" t="n">
+        <v>79.2</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
@@ -2439,21 +2474,21 @@
         </is>
       </c>
       <c r="P22" t="n">
-        <v>66.5</v>
+        <v>64.2</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
@@ -2461,11 +2496,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U22" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U22" t="inlineStr"/>
       <c r="V22" t="inlineStr">
         <is>
           <t>No</t>
@@ -2475,11 +2506,11 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>526.28</v>
+        <v>584.01</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -2512,22 +2543,22 @@
         </is>
       </c>
       <c r="I23" t="n">
-        <v>68.40000000000001</v>
+        <v>61.7</v>
       </c>
       <c r="J23" t="n">
-        <v>69.5</v>
+        <v>55.7</v>
       </c>
       <c r="K23" t="n">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="L23" t="n">
-        <v>5.63</v>
+        <v>2.51</v>
       </c>
       <c r="M23" t="n">
-        <v>72.90000000000001</v>
+        <v>27.3</v>
       </c>
       <c r="N23" t="n">
-        <v>84.2</v>
+        <v>45</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -2535,7 +2566,7 @@
         </is>
       </c>
       <c r="P23" t="n">
-        <v>73.90000000000001</v>
+        <v>54.5</v>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
@@ -2544,17 +2575,17 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U23" t="inlineStr"/>
@@ -2567,11 +2598,11 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>ANET</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>722.36</v>
+        <v>173.26</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -2604,19 +2635,19 @@
         </is>
       </c>
       <c r="I24" t="n">
-        <v>67.7</v>
+        <v>57.8</v>
       </c>
       <c r="J24" t="n">
-        <v>72.40000000000001</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="K24" t="n">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="L24" t="n">
-        <v>0.97</v>
+        <v>3.82</v>
       </c>
       <c r="M24" t="n">
-        <v>14.1</v>
+        <v>61.1</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
@@ -2624,7 +2655,7 @@
         </is>
       </c>
       <c r="P24" t="n">
-        <v>66.59999999999999</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
@@ -2633,17 +2664,17 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U24" t="inlineStr"/>
@@ -2656,56 +2687,59 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>D</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>199.45</v>
+        <v>63.17</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I25" t="n">
-        <v>67.59999999999999</v>
+        <v>57.8</v>
       </c>
       <c r="J25" t="n">
-        <v>54</v>
+        <v>53.2</v>
       </c>
       <c r="K25" t="n">
-        <v>90</v>
+        <v>21</v>
       </c>
       <c r="L25" t="n">
-        <v>3.45</v>
+        <v>2.11</v>
       </c>
       <c r="M25" t="n">
-        <v>44.4</v>
+        <v>19</v>
+      </c>
+      <c r="N25" t="n">
+        <v>59.1</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
@@ -2713,11 +2747,11 @@
         </is>
       </c>
       <c r="P25" t="n">
-        <v>59</v>
+        <v>55.2</v>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
@@ -2732,10 +2766,14 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U25" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
       <c r="V25" t="inlineStr">
         <is>
           <t>No</t>
@@ -2745,30 +2783,30 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>LMT</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>592.45</v>
+        <v>522.22</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -2778,34 +2816,31 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I26" t="n">
-        <v>67.5</v>
+        <v>57.7</v>
       </c>
       <c r="J26" t="n">
-        <v>60.6</v>
+        <v>29.1</v>
       </c>
       <c r="K26" t="n">
-        <v>80</v>
+        <v>99</v>
       </c>
       <c r="L26" t="n">
-        <v>2.49</v>
+        <v>2.86</v>
       </c>
       <c r="M26" t="n">
-        <v>27.2</v>
-      </c>
-      <c r="N26" t="n">
-        <v>44.6</v>
+        <v>32.2</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P26" t="n">
-        <v>56.4</v>
+        <v>41.7</v>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
@@ -2819,12 +2854,12 @@
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U26" t="inlineStr"/>
@@ -2837,11 +2872,11 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ETN</t>
+          <t>IWM</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>424.56</v>
+        <v>277.29</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -2874,22 +2909,22 @@
         </is>
       </c>
       <c r="I27" t="n">
-        <v>65.5</v>
+        <v>56.7</v>
       </c>
       <c r="J27" t="n">
-        <v>64.2</v>
+        <v>63.7</v>
       </c>
       <c r="K27" t="n">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="L27" t="n">
-        <v>3.17</v>
+        <v>1.53</v>
       </c>
       <c r="M27" t="n">
-        <v>38.1</v>
+        <v>20.7</v>
       </c>
       <c r="N27" t="n">
-        <v>94.8</v>
+        <v>66.3</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -2897,7 +2932,7 @@
         </is>
       </c>
       <c r="P27" t="n">
-        <v>68.90000000000001</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
@@ -2906,17 +2941,17 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U27" t="inlineStr"/>
@@ -2929,59 +2964,59 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>IWM</t>
+          <t>TSN</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>278.09</v>
+        <v>66.12</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I28" t="n">
-        <v>60.2</v>
+        <v>55.2</v>
       </c>
       <c r="J28" t="n">
-        <v>66.40000000000001</v>
+        <v>60.5</v>
       </c>
       <c r="K28" t="n">
-        <v>82</v>
+        <v>8</v>
       </c>
       <c r="L28" t="n">
-        <v>1.55</v>
+        <v>2.53</v>
       </c>
       <c r="M28" t="n">
-        <v>21.8</v>
+        <v>22.2</v>
       </c>
       <c r="N28" t="n">
-        <v>76.40000000000001</v>
+        <v>49.3</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
@@ -2989,11 +3024,11 @@
         </is>
       </c>
       <c r="P28" t="n">
-        <v>68.09999999999999</v>
+        <v>62.9</v>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
@@ -3008,10 +3043,14 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U28" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V28" t="inlineStr">
         <is>
           <t>No</t>
@@ -3021,15 +3060,15 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ANET</t>
+          <t>LIN</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>174.82</v>
+        <v>494.29</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -3044,33 +3083,36 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I29" t="n">
-        <v>59.5</v>
+        <v>50.3</v>
       </c>
       <c r="J29" t="n">
-        <v>66.5</v>
+        <v>46.1</v>
       </c>
       <c r="K29" t="n">
-        <v>89</v>
+        <v>10</v>
       </c>
       <c r="L29" t="n">
-        <v>3.75</v>
+        <v>2.14</v>
       </c>
       <c r="M29" t="n">
-        <v>61.6</v>
+        <v>20.6</v>
+      </c>
+      <c r="N29" t="n">
+        <v>85.5</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
@@ -3078,67 +3120,71 @@
         </is>
       </c>
       <c r="P29" t="n">
-        <v>68.2</v>
+        <v>57.4</v>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U29" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V29" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>65.01000000000001</v>
+        <v>412.09</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D30" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -3147,22 +3193,22 @@
         </is>
       </c>
       <c r="I30" t="n">
-        <v>59.4</v>
+        <v>49.9</v>
       </c>
       <c r="J30" t="n">
-        <v>64.5</v>
+        <v>63.4</v>
       </c>
       <c r="K30" t="n">
-        <v>31</v>
+        <v>66</v>
       </c>
       <c r="L30" t="n">
-        <v>2.08</v>
+        <v>3.11</v>
       </c>
       <c r="M30" t="n">
-        <v>20.2</v>
+        <v>44.1</v>
       </c>
       <c r="N30" t="n">
-        <v>75.8</v>
+        <v>50.3</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
@@ -3170,7 +3216,7 @@
         </is>
       </c>
       <c r="P30" t="n">
-        <v>59.5</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
@@ -3179,17 +3225,17 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U30" t="inlineStr"/>
@@ -3206,7 +3252,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>191.79</v>
+        <v>188.4</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -3239,22 +3285,22 @@
         </is>
       </c>
       <c r="I31" t="n">
-        <v>59.4</v>
+        <v>48.3</v>
       </c>
       <c r="J31" t="n">
-        <v>67.09999999999999</v>
+        <v>61.5</v>
       </c>
       <c r="K31" t="n">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="L31" t="n">
-        <v>2.41</v>
+        <v>2.35</v>
       </c>
       <c r="M31" t="n">
-        <v>28</v>
+        <v>28.3</v>
       </c>
       <c r="N31" t="n">
-        <v>50.7</v>
+        <v>51.6</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
@@ -3262,7 +3308,7 @@
         </is>
       </c>
       <c r="P31" t="n">
-        <v>65.8</v>
+        <v>63.8</v>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
@@ -3271,17 +3317,17 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U31" t="inlineStr"/>
@@ -3294,11 +3340,11 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>DLR</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>419.9</v>
+        <v>198.81</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -3327,26 +3373,23 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I32" t="n">
-        <v>58.4</v>
+        <v>45.7</v>
       </c>
       <c r="J32" t="n">
-        <v>68.59999999999999</v>
+        <v>61.9</v>
       </c>
       <c r="K32" t="n">
-        <v>88</v>
+        <v>74</v>
       </c>
       <c r="L32" t="n">
-        <v>3.02</v>
+        <v>2.23</v>
       </c>
       <c r="M32" t="n">
-        <v>44.6</v>
-      </c>
-      <c r="N32" t="n">
-        <v>51.8</v>
+        <v>31.1</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
@@ -3354,7 +3397,7 @@
         </is>
       </c>
       <c r="P32" t="n">
-        <v>68.09999999999999</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
@@ -3363,17 +3406,17 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U32" t="inlineStr"/>
@@ -3386,56 +3429,59 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>BK</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>329.89</v>
+        <v>132.14</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D33" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I33" t="n">
-        <v>57.1</v>
+        <v>42.4</v>
       </c>
       <c r="J33" t="n">
-        <v>52.6</v>
+        <v>57.7</v>
       </c>
       <c r="K33" t="n">
-        <v>7</v>
+        <v>62</v>
       </c>
       <c r="L33" t="n">
-        <v>1.96</v>
+        <v>2.02</v>
       </c>
       <c r="M33" t="n">
-        <v>20.8</v>
+        <v>20</v>
+      </c>
+      <c r="N33" t="n">
+        <v>37.2</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
@@ -3443,21 +3489,21 @@
         </is>
       </c>
       <c r="P33" t="n">
-        <v>60.6</v>
+        <v>69.3</v>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T33" t="inlineStr">
@@ -3465,196 +3511,8 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U33" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U33" t="inlineStr"/>
       <c r="V33" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>BK</t>
-        </is>
-      </c>
-      <c r="B34" t="n">
-        <v>135.32</v>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>Credit Call</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I34" t="n">
-        <v>54.2</v>
-      </c>
-      <c r="J34" t="n">
-        <v>67.09999999999999</v>
-      </c>
-      <c r="K34" t="n">
-        <v>77</v>
-      </c>
-      <c r="L34" t="n">
-        <v>2.02</v>
-      </c>
-      <c r="M34" t="n">
-        <v>19.2</v>
-      </c>
-      <c r="N34" t="n">
-        <v>32.9</v>
-      </c>
-      <c r="O34" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P34" t="n">
-        <v>73.3</v>
-      </c>
-      <c r="Q34" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R34" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S34" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="T34" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U34" t="inlineStr"/>
-      <c r="V34" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>DLR</t>
-        </is>
-      </c>
-      <c r="B35" t="n">
-        <v>200.28</v>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>Credit Call</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I35" t="n">
-        <v>50.2</v>
-      </c>
-      <c r="J35" t="n">
-        <v>65.5</v>
-      </c>
-      <c r="K35" t="n">
-        <v>79</v>
-      </c>
-      <c r="L35" t="n">
-        <v>2.28</v>
-      </c>
-      <c r="M35" t="n">
-        <v>23.1</v>
-      </c>
-      <c r="N35" t="n">
-        <v>70.7</v>
-      </c>
-      <c r="O35" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P35" t="n">
-        <v>68.90000000000001</v>
-      </c>
-      <c r="Q35" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R35" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S35" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="T35" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U35" t="inlineStr"/>
-      <c r="V35" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Scan 05.05.2026 15:57 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V33"/>
+  <dimension ref="A1:V27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -448,7 +448,7 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="6" customWidth="1" min="10" max="10"/>
-    <col width="6" customWidth="1" min="11" max="11"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
     <col width="6" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
     <col width="9" customWidth="1" min="14" max="14"/>
@@ -577,11 +577,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>TXN</t>
+          <t>GD</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>279.83</v>
+        <v>347.86</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,19 +614,22 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>88.8</v>
+        <v>95.3</v>
       </c>
       <c r="J2" t="n">
-        <v>76.09999999999999</v>
+        <v>58.8</v>
       </c>
       <c r="K2" t="n">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="L2" t="n">
-        <v>3.57</v>
+        <v>2.77</v>
       </c>
       <c r="M2" t="n">
-        <v>39.9</v>
+        <v>30.9</v>
+      </c>
+      <c r="N2" t="n">
+        <v>99.2</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -634,7 +637,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>77</v>
+        <v>53.8</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -648,7 +651,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -670,7 +673,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>97.28</v>
+        <v>109.06</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -703,22 +706,22 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>87.5</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="J3" t="n">
-        <v>82.7</v>
+        <v>84.8</v>
       </c>
       <c r="K3" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L3" t="n">
-        <v>5.72</v>
+        <v>6.3</v>
       </c>
       <c r="M3" t="n">
-        <v>94.59999999999999</v>
+        <v>100.3</v>
       </c>
       <c r="N3" t="n">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -726,7 +729,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>83.90000000000001</v>
+        <v>88.5</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -758,11 +761,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>KDP</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>341.39</v>
+        <v>28.78</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -795,30 +798,27 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>85.90000000000001</v>
+        <v>89</v>
       </c>
       <c r="J4" t="n">
-        <v>69.8</v>
+        <v>61</v>
       </c>
       <c r="K4" t="n">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="L4" t="n">
-        <v>5.57</v>
+        <v>2.65</v>
       </c>
       <c r="M4" t="n">
-        <v>67.40000000000001</v>
-      </c>
-      <c r="N4" t="n">
-        <v>53.8</v>
+        <v>23.2</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P4" t="n">
-        <v>72.59999999999999</v>
+        <v>54.1</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -840,25 +840,21 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CDNS</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>348.63</v>
+        <v>101.93</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -891,22 +887,22 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>84.5</v>
+        <v>86</v>
       </c>
       <c r="J5" t="n">
-        <v>68</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="K5" t="n">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="L5" t="n">
-        <v>3.78</v>
+        <v>4.92</v>
       </c>
       <c r="M5" t="n">
-        <v>48.6</v>
+        <v>63.8</v>
       </c>
       <c r="N5" t="n">
-        <v>80</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -914,7 +910,7 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>61.8</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -936,21 +932,25 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr"/>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>TXN</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>102.31</v>
+        <v>279.62</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -983,22 +983,22 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>79</v>
+        <v>85.59999999999999</v>
       </c>
       <c r="J6" t="n">
-        <v>79.8</v>
+        <v>75.8</v>
       </c>
       <c r="K6" t="n">
         <v>93</v>
       </c>
       <c r="L6" t="n">
-        <v>4.13</v>
+        <v>3.35</v>
       </c>
       <c r="M6" t="n">
-        <v>63.5</v>
+        <v>63</v>
       </c>
       <c r="N6" t="n">
-        <v>96.09999999999999</v>
+        <v>99.2</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -1006,7 +1006,7 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>79</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1038,11 +1038,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>CDNS</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>270.55</v>
+        <v>351.19</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1071,23 +1071,26 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>78.40000000000001</v>
+        <v>82.2</v>
       </c>
       <c r="J7" t="n">
-        <v>79.2</v>
+        <v>68.8</v>
       </c>
       <c r="K7" t="n">
-        <v>75</v>
+        <v>98</v>
       </c>
       <c r="L7" t="n">
-        <v>3.04</v>
+        <v>3.54</v>
       </c>
       <c r="M7" t="n">
-        <v>30.6</v>
+        <v>48.2</v>
+      </c>
+      <c r="N7" t="n">
+        <v>78.8</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1095,7 +1098,7 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>67.90000000000001</v>
+        <v>62.4</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1127,11 +1130,11 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>GFS</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>67.25</v>
+        <v>355.24</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1164,22 +1167,22 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>77.90000000000001</v>
+        <v>81.7</v>
       </c>
       <c r="J8" t="n">
-        <v>81</v>
+        <v>72.5</v>
       </c>
       <c r="K8" t="n">
         <v>93</v>
       </c>
       <c r="L8" t="n">
-        <v>4.5</v>
+        <v>5.19</v>
       </c>
       <c r="M8" t="n">
-        <v>56</v>
+        <v>67.5</v>
       </c>
       <c r="N8" t="n">
-        <v>63.8</v>
+        <v>54</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1187,7 +1190,7 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>80.09999999999999</v>
+        <v>77</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1219,11 +1222,11 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>URI</t>
+          <t>GFS</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>931.37</v>
+        <v>69.92</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1256,22 +1259,22 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>77.5</v>
+        <v>80.7</v>
       </c>
       <c r="J9" t="n">
-        <v>65.7</v>
+        <v>83.3</v>
       </c>
       <c r="K9" t="n">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="L9" t="n">
-        <v>3.63</v>
+        <v>4.69</v>
       </c>
       <c r="M9" t="n">
-        <v>70.09999999999999</v>
+        <v>56.5</v>
       </c>
       <c r="N9" t="n">
-        <v>95.09999999999999</v>
+        <v>64.8</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1279,7 +1282,7 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>57.8</v>
+        <v>81.5</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1311,11 +1314,11 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>MCHP</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>200.32</v>
+        <v>98.28</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1348,19 +1351,22 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>75.7</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="J10" t="n">
-        <v>60.4</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="K10" t="n">
-        <v>95</v>
+        <v>84</v>
       </c>
       <c r="L10" t="n">
-        <v>7.32</v>
+        <v>3.73</v>
       </c>
       <c r="M10" t="n">
-        <v>81.40000000000001</v>
+        <v>48.9</v>
+      </c>
+      <c r="N10" t="n">
+        <v>73.40000000000001</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1368,7 +1374,7 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>64.8</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1377,38 +1383,34 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U10" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr"/>
       <c r="V10" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>MCHP</t>
+          <t>URI</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>94.73999999999999</v>
+        <v>938.4299999999999</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1441,22 +1443,22 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>75.40000000000001</v>
+        <v>73.7</v>
       </c>
       <c r="J11" t="n">
-        <v>76.90000000000001</v>
+        <v>66</v>
       </c>
       <c r="K11" t="n">
-        <v>84</v>
+        <v>95</v>
       </c>
       <c r="L11" t="n">
-        <v>3.77</v>
+        <v>3.5</v>
       </c>
       <c r="M11" t="n">
-        <v>48.7</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="N11" t="n">
-        <v>72.90000000000001</v>
+        <v>95.09999999999999</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1464,7 +1466,7 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>72.90000000000001</v>
+        <v>58.5</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1496,11 +1498,11 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>92.53</v>
+        <v>206.94</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1529,26 +1531,26 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>72.2</v>
+        <v>73</v>
       </c>
       <c r="J12" t="n">
-        <v>72.09999999999999</v>
+        <v>63.3</v>
       </c>
       <c r="K12" t="n">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="L12" t="n">
-        <v>2.29</v>
+        <v>6.94</v>
       </c>
       <c r="M12" t="n">
-        <v>26.8</v>
+        <v>95.5</v>
       </c>
       <c r="N12" t="n">
-        <v>41.3</v>
+        <v>99.8</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1556,7 +1558,7 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>73.7</v>
+        <v>67.3</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1565,17 +1567,17 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U12" t="inlineStr"/>
@@ -1588,11 +1590,11 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ADI</t>
+          <t>CSCO</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>393.93</v>
+        <v>93.73999999999999</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -1625,22 +1627,22 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>69.40000000000001</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="J13" t="n">
-        <v>65.09999999999999</v>
+        <v>74.2</v>
       </c>
       <c r="K13" t="n">
         <v>82</v>
       </c>
       <c r="L13" t="n">
-        <v>2.88</v>
+        <v>2.21</v>
       </c>
       <c r="M13" t="n">
-        <v>38.5</v>
+        <v>26.7</v>
       </c>
       <c r="N13" t="n">
-        <v>100</v>
+        <v>41.1</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1648,7 +1650,7 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>74.09999999999999</v>
+        <v>74.7</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1657,17 +1659,17 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U13" t="inlineStr"/>
@@ -1684,7 +1686,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>492.83</v>
+        <v>506.89</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -1713,26 +1715,26 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>69.09999999999999</v>
+        <v>69.3</v>
       </c>
       <c r="J14" t="n">
-        <v>65.40000000000001</v>
+        <v>68.8</v>
       </c>
       <c r="K14" t="n">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="L14" t="n">
-        <v>3.37</v>
+        <v>3.29</v>
       </c>
       <c r="M14" t="n">
-        <v>49.8</v>
+        <v>49.6</v>
       </c>
       <c r="N14" t="n">
-        <v>22.7</v>
+        <v>22.5</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1740,7 +1742,7 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>56.3</v>
+        <v>58.1</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1772,59 +1774,56 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>PEP</t>
+          <t>XLK</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>155.55</v>
+        <v>165.5</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>66.90000000000001</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="J15" t="n">
-        <v>48.7</v>
+        <v>77.2</v>
       </c>
       <c r="K15" t="n">
-        <v>6</v>
+        <v>87</v>
       </c>
       <c r="L15" t="n">
-        <v>1.97</v>
+        <v>1.78</v>
       </c>
       <c r="M15" t="n">
-        <v>19</v>
-      </c>
-      <c r="N15" t="n">
-        <v>23.1</v>
+        <v>28.9</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1832,21 +1831,21 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>53</v>
+        <v>73.2</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
@@ -1854,11 +1853,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U15" t="inlineStr">
-        <is>
-          <t>TTM Squeeze</t>
-        </is>
-      </c>
+      <c r="U15" t="inlineStr"/>
       <c r="V15" t="inlineStr">
         <is>
           <t>No</t>
@@ -1868,11 +1863,11 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>XLK</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>161.31</v>
+        <v>681.4</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -1905,19 +1900,19 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>66.3</v>
+        <v>67.3</v>
       </c>
       <c r="J16" t="n">
-        <v>71.90000000000001</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="K16" t="n">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="L16" t="n">
-        <v>1.73</v>
+        <v>1.33</v>
       </c>
       <c r="M16" t="n">
-        <v>29.1</v>
+        <v>19.9</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -1957,11 +1952,11 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>ADI</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>670.73</v>
+        <v>401.7</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -1990,26 +1985,26 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>66</v>
+        <v>66.8</v>
       </c>
       <c r="J17" t="n">
-        <v>71.8</v>
+        <v>68.8</v>
       </c>
       <c r="K17" t="n">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="L17" t="n">
-        <v>1.32</v>
+        <v>2.79</v>
       </c>
       <c r="M17" t="n">
-        <v>20.1</v>
+        <v>38.3</v>
       </c>
       <c r="N17" t="n">
-        <v>84.8</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -2017,7 +2012,7 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>67.40000000000001</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -2026,17 +2021,17 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U17" t="inlineStr"/>
@@ -2053,7 +2048,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>164.05</v>
+        <v>170.72</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -2086,22 +2081,22 @@
         </is>
       </c>
       <c r="I18" t="n">
-        <v>65.40000000000001</v>
+        <v>64</v>
       </c>
       <c r="J18" t="n">
-        <v>75.40000000000001</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="K18" t="n">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="L18" t="n">
-        <v>4.87</v>
+        <v>4.74</v>
       </c>
       <c r="M18" t="n">
-        <v>64.40000000000001</v>
+        <v>64.8</v>
       </c>
       <c r="N18" t="n">
-        <v>62.1</v>
+        <v>62.9</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -2109,7 +2104,7 @@
         </is>
       </c>
       <c r="P18" t="n">
-        <v>84.3</v>
+        <v>86</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -2118,17 +2113,17 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U18" t="inlineStr"/>
@@ -2145,7 +2140,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>181.43</v>
+        <v>183.15</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -2178,30 +2173,27 @@
         </is>
       </c>
       <c r="I19" t="n">
-        <v>65.2</v>
+        <v>63.3</v>
       </c>
       <c r="J19" t="n">
-        <v>62.4</v>
+        <v>63.4</v>
       </c>
       <c r="K19" t="n">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="L19" t="n">
-        <v>5.1</v>
+        <v>4.77</v>
       </c>
       <c r="M19" t="n">
-        <v>63.3</v>
-      </c>
-      <c r="N19" t="n">
-        <v>38.6</v>
+        <v>54.5</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P19" t="n">
-        <v>51.6</v>
+        <v>52.2</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -2233,15 +2225,15 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>UNH</t>
+          <t>PEP</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>368.59</v>
+        <v>154.66</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -2256,33 +2248,33 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I20" t="n">
-        <v>65.2</v>
+        <v>61.1</v>
       </c>
       <c r="J20" t="n">
-        <v>82.59999999999999</v>
+        <v>46.8</v>
       </c>
       <c r="K20" t="n">
-        <v>76</v>
+        <v>4</v>
       </c>
       <c r="L20" t="n">
-        <v>2.4</v>
+        <v>2.03</v>
       </c>
       <c r="M20" t="n">
-        <v>29</v>
+        <v>24.5</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -2290,11 +2282,11 @@
         </is>
       </c>
       <c r="P20" t="n">
-        <v>63.1</v>
+        <v>52</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
@@ -2304,7 +2296,7 @@
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
@@ -2312,7 +2304,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U20" t="inlineStr"/>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
       <c r="V20" t="inlineStr">
         <is>
           <t>No</t>
@@ -2322,11 +2318,11 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ETN</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>427.54</v>
+        <v>723.11</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -2355,26 +2351,26 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>62.8</v>
+        <v>60.8</v>
       </c>
       <c r="J21" t="n">
-        <v>65.7</v>
+        <v>71.2</v>
       </c>
       <c r="K21" t="n">
-        <v>68</v>
+        <v>81</v>
       </c>
       <c r="L21" t="n">
-        <v>3.04</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="M21" t="n">
-        <v>37.7</v>
+        <v>15.6</v>
       </c>
       <c r="N21" t="n">
-        <v>92.5</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
@@ -2382,7 +2378,7 @@
         </is>
       </c>
       <c r="P21" t="n">
-        <v>69.5</v>
+        <v>66.8</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
@@ -2391,17 +2387,17 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U21" t="inlineStr"/>
@@ -2414,59 +2410,59 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>AEP</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>717.1900000000001</v>
+        <v>136.95</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I22" t="n">
-        <v>62.5</v>
+        <v>58.1</v>
       </c>
       <c r="J22" t="n">
-        <v>67.7</v>
+        <v>59.2</v>
       </c>
       <c r="K22" t="n">
-        <v>86</v>
+        <v>14</v>
       </c>
       <c r="L22" t="n">
-        <v>0.9399999999999999</v>
+        <v>1.96</v>
       </c>
       <c r="M22" t="n">
-        <v>15.8</v>
+        <v>16</v>
       </c>
       <c r="N22" t="n">
-        <v>79.2</v>
+        <v>30.6</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
@@ -2474,21 +2470,21 @@
         </is>
       </c>
       <c r="P22" t="n">
-        <v>64.2</v>
+        <v>66.5</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
@@ -2496,7 +2492,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U22" t="inlineStr"/>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V22" t="inlineStr">
         <is>
           <t>No</t>
@@ -2506,30 +2506,30 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>LMT</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>584.01</v>
+        <v>510.76</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2539,34 +2539,31 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I23" t="n">
-        <v>61.7</v>
+        <v>56.1</v>
       </c>
       <c r="J23" t="n">
-        <v>55.7</v>
+        <v>24.9</v>
       </c>
       <c r="K23" t="n">
-        <v>75</v>
+        <v>99</v>
       </c>
       <c r="L23" t="n">
-        <v>2.51</v>
+        <v>2.79</v>
       </c>
       <c r="M23" t="n">
-        <v>27.3</v>
-      </c>
-      <c r="N23" t="n">
-        <v>45</v>
+        <v>32.2</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P23" t="n">
-        <v>54.5</v>
+        <v>39</v>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
@@ -2580,12 +2577,12 @@
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U23" t="inlineStr"/>
@@ -2602,7 +2599,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>173.26</v>
+        <v>173.58</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -2635,19 +2632,19 @@
         </is>
       </c>
       <c r="I24" t="n">
-        <v>57.8</v>
+        <v>55.3</v>
       </c>
       <c r="J24" t="n">
-        <v>65.59999999999999</v>
+        <v>65.8</v>
       </c>
       <c r="K24" t="n">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="L24" t="n">
-        <v>3.82</v>
+        <v>3.77</v>
       </c>
       <c r="M24" t="n">
-        <v>61.1</v>
+        <v>63.6</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
@@ -2687,35 +2684,35 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>IWM</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>63.17</v>
+        <v>282.06</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -2724,22 +2721,19 @@
         </is>
       </c>
       <c r="I25" t="n">
-        <v>57.8</v>
+        <v>54.6</v>
       </c>
       <c r="J25" t="n">
-        <v>53.2</v>
+        <v>68.8</v>
       </c>
       <c r="K25" t="n">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="L25" t="n">
-        <v>2.11</v>
+        <v>1.56</v>
       </c>
       <c r="M25" t="n">
-        <v>19</v>
-      </c>
-      <c r="N25" t="n">
-        <v>59.1</v>
+        <v>21.5</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
@@ -2747,21 +2741,21 @@
         </is>
       </c>
       <c r="P25" t="n">
-        <v>55.2</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
@@ -2769,11 +2763,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U25" t="inlineStr">
-        <is>
-          <t>TTM Squeeze</t>
-        </is>
-      </c>
+      <c r="U25" t="inlineStr"/>
       <c r="V25" t="inlineStr">
         <is>
           <t>No</t>
@@ -2783,68 +2773,68 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>LMT</t>
+          <t>LIN</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>522.22</v>
+        <v>500.39</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D26" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I26" t="n">
-        <v>57.7</v>
+        <v>52.2</v>
       </c>
       <c r="J26" t="n">
-        <v>29.1</v>
+        <v>50.7</v>
       </c>
       <c r="K26" t="n">
-        <v>99</v>
+        <v>7</v>
       </c>
       <c r="L26" t="n">
-        <v>2.86</v>
+        <v>2.12</v>
       </c>
       <c r="M26" t="n">
-        <v>32.2</v>
+        <v>24</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P26" t="n">
-        <v>41.7</v>
+        <v>60</v>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
@@ -2854,15 +2844,19 @@
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U26" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
       <c r="V26" t="inlineStr">
         <is>
           <t>No</t>
@@ -2872,11 +2866,11 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>IWM</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>277.29</v>
+        <v>427.64</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -2909,22 +2903,22 @@
         </is>
       </c>
       <c r="I27" t="n">
-        <v>56.7</v>
+        <v>50.6</v>
       </c>
       <c r="J27" t="n">
-        <v>63.7</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="K27" t="n">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="L27" t="n">
-        <v>1.53</v>
+        <v>3.02</v>
       </c>
       <c r="M27" t="n">
-        <v>20.7</v>
+        <v>42.9</v>
       </c>
       <c r="N27" t="n">
-        <v>66.3</v>
+        <v>46.7</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -2932,7 +2926,7 @@
         </is>
       </c>
       <c r="P27" t="n">
-        <v>66.40000000000001</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
@@ -2941,578 +2935,21 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U27" t="inlineStr"/>
       <c r="V27" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>TSN</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
-        <v>66.12</v>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D28" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>Debit Call</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>30-60 DTE</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>SQUEEZE</t>
-        </is>
-      </c>
-      <c r="I28" t="n">
-        <v>55.2</v>
-      </c>
-      <c r="J28" t="n">
-        <v>60.5</v>
-      </c>
-      <c r="K28" t="n">
-        <v>8</v>
-      </c>
-      <c r="L28" t="n">
-        <v>2.53</v>
-      </c>
-      <c r="M28" t="n">
-        <v>22.2</v>
-      </c>
-      <c r="N28" t="n">
-        <v>49.3</v>
-      </c>
-      <c r="O28" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P28" t="n">
-        <v>62.9</v>
-      </c>
-      <c r="Q28" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="R28" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="S28" t="inlineStr">
-        <is>
-          <t>lime</t>
-        </is>
-      </c>
-      <c r="T28" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U28" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
-      <c r="V28" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>LIN</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>494.29</v>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>Debit Put</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>30-60 DTE</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>SQUEEZE</t>
-        </is>
-      </c>
-      <c r="I29" t="n">
-        <v>50.3</v>
-      </c>
-      <c r="J29" t="n">
-        <v>46.1</v>
-      </c>
-      <c r="K29" t="n">
-        <v>10</v>
-      </c>
-      <c r="L29" t="n">
-        <v>2.14</v>
-      </c>
-      <c r="M29" t="n">
-        <v>20.6</v>
-      </c>
-      <c r="N29" t="n">
-        <v>85.5</v>
-      </c>
-      <c r="O29" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P29" t="n">
-        <v>57.4</v>
-      </c>
-      <c r="Q29" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="R29" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S29" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="T29" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U29" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
-      <c r="V29" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>AVGO</t>
-        </is>
-      </c>
-      <c r="B30" t="n">
-        <v>412.09</v>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>Credit Call</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I30" t="n">
-        <v>49.9</v>
-      </c>
-      <c r="J30" t="n">
-        <v>63.4</v>
-      </c>
-      <c r="K30" t="n">
-        <v>66</v>
-      </c>
-      <c r="L30" t="n">
-        <v>3.11</v>
-      </c>
-      <c r="M30" t="n">
-        <v>44.1</v>
-      </c>
-      <c r="N30" t="n">
-        <v>50.3</v>
-      </c>
-      <c r="O30" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P30" t="n">
-        <v>65.59999999999999</v>
-      </c>
-      <c r="Q30" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R30" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S30" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="T30" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U30" t="inlineStr"/>
-      <c r="V30" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>MS</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>188.4</v>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>Credit Call</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I31" t="n">
-        <v>48.3</v>
-      </c>
-      <c r="J31" t="n">
-        <v>61.5</v>
-      </c>
-      <c r="K31" t="n">
-        <v>63</v>
-      </c>
-      <c r="L31" t="n">
-        <v>2.35</v>
-      </c>
-      <c r="M31" t="n">
-        <v>28.3</v>
-      </c>
-      <c r="N31" t="n">
-        <v>51.6</v>
-      </c>
-      <c r="O31" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P31" t="n">
-        <v>63.8</v>
-      </c>
-      <c r="Q31" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R31" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S31" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="T31" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U31" t="inlineStr"/>
-      <c r="V31" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>DLR</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>198.81</v>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>Credit Call</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I32" t="n">
-        <v>45.7</v>
-      </c>
-      <c r="J32" t="n">
-        <v>61.9</v>
-      </c>
-      <c r="K32" t="n">
-        <v>74</v>
-      </c>
-      <c r="L32" t="n">
-        <v>2.23</v>
-      </c>
-      <c r="M32" t="n">
-        <v>31.1</v>
-      </c>
-      <c r="O32" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P32" t="n">
-        <v>67.09999999999999</v>
-      </c>
-      <c r="Q32" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R32" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S32" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="T32" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U32" t="inlineStr"/>
-      <c r="V32" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>BK</t>
-        </is>
-      </c>
-      <c r="B33" t="n">
-        <v>132.14</v>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>Credit Call</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I33" t="n">
-        <v>42.4</v>
-      </c>
-      <c r="J33" t="n">
-        <v>57.7</v>
-      </c>
-      <c r="K33" t="n">
-        <v>62</v>
-      </c>
-      <c r="L33" t="n">
-        <v>2.02</v>
-      </c>
-      <c r="M33" t="n">
-        <v>20</v>
-      </c>
-      <c r="N33" t="n">
-        <v>37.2</v>
-      </c>
-      <c r="O33" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P33" t="n">
-        <v>69.3</v>
-      </c>
-      <c r="Q33" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R33" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S33" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="T33" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U33" t="inlineStr"/>
-      <c r="V33" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Scan 06.05.2026 16:06 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V27"/>
+  <dimension ref="A1:V30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -577,11 +577,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>GD</t>
+          <t>INTC</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>347.86</v>
+        <v>111.15</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,19 +614,19 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>95.3</v>
+        <v>93.5</v>
       </c>
       <c r="J2" t="n">
-        <v>58.8</v>
+        <v>85.40000000000001</v>
       </c>
       <c r="K2" t="n">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="L2" t="n">
-        <v>2.77</v>
+        <v>6.19</v>
       </c>
       <c r="M2" t="n">
-        <v>30.9</v>
+        <v>99</v>
       </c>
       <c r="N2" t="n">
         <v>99.2</v>
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>53.8</v>
+        <v>88.8</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -651,7 +651,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -669,11 +669,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>INTC</t>
+          <t>GD</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>109.06</v>
+        <v>345.78</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -706,22 +706,22 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>94.40000000000001</v>
+        <v>92.09999999999999</v>
       </c>
       <c r="J3" t="n">
-        <v>84.8</v>
+        <v>56.7</v>
       </c>
       <c r="K3" t="n">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="L3" t="n">
-        <v>6.3</v>
+        <v>2.65</v>
       </c>
       <c r="M3" t="n">
-        <v>100.3</v>
+        <v>31</v>
       </c>
       <c r="N3" t="n">
-        <v>100</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -729,7 +729,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>88.5</v>
+        <v>53</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -761,11 +761,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>KDP</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>28.78</v>
+        <v>415.45</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -798,27 +798,27 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>89</v>
+        <v>90.40000000000001</v>
       </c>
       <c r="J4" t="n">
-        <v>61</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="K4" t="n">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="L4" t="n">
-        <v>2.65</v>
+        <v>6.36</v>
       </c>
       <c r="M4" t="n">
-        <v>23.2</v>
+        <v>65.2</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P4" t="n">
-        <v>54.1</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -850,11 +850,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>GFS</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>101.93</v>
+        <v>71.12</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -887,22 +887,22 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>86</v>
+        <v>90.3</v>
       </c>
       <c r="J5" t="n">
-        <v>78.90000000000001</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="K5" t="n">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="L5" t="n">
-        <v>4.92</v>
+        <v>5.34</v>
       </c>
       <c r="M5" t="n">
-        <v>63.8</v>
+        <v>62.1</v>
       </c>
       <c r="N5" t="n">
-        <v>96.90000000000001</v>
+        <v>76.7</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -910,7 +910,7 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>78.40000000000001</v>
+        <v>82</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -950,7 +950,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>279.62</v>
+        <v>288.89</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -983,22 +983,22 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>85.59999999999999</v>
+        <v>86.7</v>
       </c>
       <c r="J6" t="n">
-        <v>75.8</v>
+        <v>79.90000000000001</v>
       </c>
       <c r="K6" t="n">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="L6" t="n">
-        <v>3.35</v>
+        <v>3.36</v>
       </c>
       <c r="M6" t="n">
-        <v>63</v>
+        <v>62.8</v>
       </c>
       <c r="N6" t="n">
-        <v>99.2</v>
+        <v>98.59999999999999</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -1006,7 +1006,7 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>76.90000000000001</v>
+        <v>79.2</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1038,11 +1038,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CDNS</t>
+          <t>KDP</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>351.19</v>
+        <v>28.5</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1075,30 +1075,30 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>82.2</v>
+        <v>85.2</v>
       </c>
       <c r="J7" t="n">
-        <v>68.8</v>
+        <v>57.6</v>
       </c>
       <c r="K7" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="L7" t="n">
-        <v>3.54</v>
+        <v>2.8</v>
       </c>
       <c r="M7" t="n">
-        <v>48.2</v>
+        <v>31.3</v>
       </c>
       <c r="N7" t="n">
-        <v>78.8</v>
+        <v>57.7</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>62.4</v>
+        <v>52.8</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1107,17 +1107,17 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U7" t="inlineStr"/>
@@ -1130,11 +1130,11 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>355.24</v>
+        <v>103.67</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1167,22 +1167,19 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>81.7</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="J8" t="n">
-        <v>72.5</v>
+        <v>80.3</v>
       </c>
       <c r="K8" t="n">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="L8" t="n">
-        <v>5.19</v>
+        <v>4.73</v>
       </c>
       <c r="M8" t="n">
-        <v>67.5</v>
-      </c>
-      <c r="N8" t="n">
-        <v>54</v>
+        <v>59.1</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1190,7 +1187,7 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>77</v>
+        <v>80.09999999999999</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1222,59 +1219,56 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>GFS</t>
+          <t>JPM</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>69.92</v>
+        <v>315.93</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>80.7</v>
+        <v>79.90000000000001</v>
       </c>
       <c r="J9" t="n">
-        <v>83.3</v>
+        <v>60.6</v>
       </c>
       <c r="K9" t="n">
-        <v>92</v>
+        <v>2</v>
       </c>
       <c r="L9" t="n">
-        <v>4.69</v>
+        <v>1.79</v>
       </c>
       <c r="M9" t="n">
-        <v>56.5</v>
-      </c>
-      <c r="N9" t="n">
-        <v>64.8</v>
+        <v>23.3</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1282,21 +1276,21 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>81.5</v>
+        <v>57.5</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
@@ -1304,7 +1298,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U9" t="inlineStr"/>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V9" t="inlineStr">
         <is>
           <t>No</t>
@@ -1318,7 +1316,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>98.28</v>
+        <v>101.44</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1351,30 +1349,30 @@
         </is>
       </c>
       <c r="I10" t="n">
+        <v>78.59999999999999</v>
+      </c>
+      <c r="J10" t="n">
+        <v>81.7</v>
+      </c>
+      <c r="K10" t="n">
+        <v>92</v>
+      </c>
+      <c r="L10" t="n">
+        <v>3.67</v>
+      </c>
+      <c r="M10" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="N10" t="n">
+        <v>74.5</v>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P10" t="n">
         <v>76.09999999999999</v>
-      </c>
-      <c r="J10" t="n">
-        <v>79.59999999999999</v>
-      </c>
-      <c r="K10" t="n">
-        <v>84</v>
-      </c>
-      <c r="L10" t="n">
-        <v>3.73</v>
-      </c>
-      <c r="M10" t="n">
-        <v>48.9</v>
-      </c>
-      <c r="N10" t="n">
-        <v>73.40000000000001</v>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P10" t="n">
-        <v>74.59999999999999</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1406,11 +1404,11 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>URI</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>938.4299999999999</v>
+        <v>235.23</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1443,22 +1441,22 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>73.7</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="J11" t="n">
-        <v>66</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="K11" t="n">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="L11" t="n">
-        <v>3.5</v>
+        <v>6.85</v>
       </c>
       <c r="M11" t="n">
-        <v>70.09999999999999</v>
+        <v>100.3</v>
       </c>
       <c r="N11" t="n">
-        <v>95.09999999999999</v>
+        <v>100</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1466,7 +1464,7 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>58.5</v>
+        <v>72.8</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1498,11 +1496,11 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>CSCO</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>206.94</v>
+        <v>91.54000000000001</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1535,22 +1533,19 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>73</v>
+        <v>73.5</v>
       </c>
       <c r="J12" t="n">
-        <v>63.3</v>
+        <v>63.7</v>
       </c>
       <c r="K12" t="n">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="L12" t="n">
-        <v>6.94</v>
+        <v>2.49</v>
       </c>
       <c r="M12" t="n">
-        <v>95.5</v>
-      </c>
-      <c r="N12" t="n">
-        <v>99.8</v>
+        <v>38.5</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1558,7 +1553,7 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>67.3</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1580,21 +1575,25 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U12" t="inlineStr"/>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>ADI</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>93.73999999999999</v>
+        <v>414.63</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -1627,22 +1626,22 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>71.90000000000001</v>
+        <v>70.7</v>
       </c>
       <c r="J13" t="n">
-        <v>74.2</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="K13" t="n">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="L13" t="n">
-        <v>2.21</v>
+        <v>2.8</v>
       </c>
       <c r="M13" t="n">
-        <v>26.7</v>
+        <v>38.2</v>
       </c>
       <c r="N13" t="n">
-        <v>41.1</v>
+        <v>98.90000000000001</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1650,7 +1649,7 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>74.7</v>
+        <v>78.3</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1682,11 +1681,11 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SNPS</t>
+          <t>XLK</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>506.89</v>
+        <v>168.72</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -1715,26 +1714,23 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>69.3</v>
+        <v>70.7</v>
       </c>
       <c r="J14" t="n">
-        <v>68.8</v>
+        <v>79.90000000000001</v>
       </c>
       <c r="K14" t="n">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="L14" t="n">
-        <v>3.29</v>
+        <v>1.81</v>
       </c>
       <c r="M14" t="n">
-        <v>49.6</v>
-      </c>
-      <c r="N14" t="n">
-        <v>22.5</v>
+        <v>31.6</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1742,7 +1738,7 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>58.1</v>
+        <v>74.8</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1774,11 +1770,11 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>XLK</t>
+          <t>URI</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>165.5</v>
+        <v>950.09</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1811,19 +1807,19 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>68.90000000000001</v>
+        <v>70</v>
       </c>
       <c r="J15" t="n">
-        <v>77.2</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="K15" t="n">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="L15" t="n">
-        <v>1.78</v>
+        <v>3.27</v>
       </c>
       <c r="M15" t="n">
-        <v>28.9</v>
+        <v>32.3</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1831,7 +1827,7 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>73.2</v>
+        <v>59.6</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1863,11 +1859,11 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>ORCL</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>681.4</v>
+        <v>192.95</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -1896,23 +1892,23 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>67.3</v>
+        <v>69</v>
       </c>
       <c r="J16" t="n">
-        <v>76.40000000000001</v>
+        <v>68.2</v>
       </c>
       <c r="K16" t="n">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="L16" t="n">
-        <v>1.33</v>
+        <v>4.77</v>
       </c>
       <c r="M16" t="n">
-        <v>19.9</v>
+        <v>57.2</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -1920,7 +1916,7 @@
         </is>
       </c>
       <c r="P16" t="n">
-        <v>70.09999999999999</v>
+        <v>55.2</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1952,11 +1948,11 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ADI</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>401.7</v>
+        <v>692.16</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -1985,26 +1981,26 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>66.8</v>
+        <v>68.5</v>
       </c>
       <c r="J17" t="n">
-        <v>68.8</v>
+        <v>79.3</v>
       </c>
       <c r="K17" t="n">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="L17" t="n">
-        <v>2.79</v>
+        <v>1.36</v>
       </c>
       <c r="M17" t="n">
-        <v>38.3</v>
+        <v>20</v>
       </c>
       <c r="N17" t="n">
-        <v>99.90000000000001</v>
+        <v>83.5</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -2012,7 +2008,7 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>76.59999999999999</v>
+        <v>71.8</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -2021,17 +2017,17 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U17" t="inlineStr"/>
@@ -2048,7 +2044,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>170.72</v>
+        <v>169.63</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -2081,22 +2077,22 @@
         </is>
       </c>
       <c r="I18" t="n">
-        <v>64</v>
+        <v>66.3</v>
       </c>
       <c r="J18" t="n">
-        <v>77.90000000000001</v>
+        <v>77.5</v>
       </c>
       <c r="K18" t="n">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="L18" t="n">
-        <v>4.74</v>
+        <v>5.04</v>
       </c>
       <c r="M18" t="n">
-        <v>64.8</v>
+        <v>64.7</v>
       </c>
       <c r="N18" t="n">
-        <v>62.9</v>
+        <v>62.7</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -2104,7 +2100,7 @@
         </is>
       </c>
       <c r="P18" t="n">
-        <v>86</v>
+        <v>85.8</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -2113,17 +2109,17 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U18" t="inlineStr"/>
@@ -2136,11 +2132,11 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ORCL</t>
+          <t>SNPS</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>183.15</v>
+        <v>501.92</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -2169,31 +2165,34 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>63.3</v>
+        <v>65.7</v>
       </c>
       <c r="J19" t="n">
-        <v>63.4</v>
+        <v>67.5</v>
       </c>
       <c r="K19" t="n">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="L19" t="n">
-        <v>4.77</v>
+        <v>3.12</v>
       </c>
       <c r="M19" t="n">
-        <v>54.5</v>
+        <v>47.7</v>
+      </c>
+      <c r="N19" t="n">
+        <v>20.6</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P19" t="n">
-        <v>52.2</v>
+        <v>57.5</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -2225,15 +2224,15 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>PEP</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>154.66</v>
+        <v>731.73</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -2248,33 +2247,36 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I20" t="n">
-        <v>61.1</v>
+        <v>64.8</v>
       </c>
       <c r="J20" t="n">
-        <v>46.8</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="K20" t="n">
-        <v>4</v>
+        <v>79</v>
       </c>
       <c r="L20" t="n">
-        <v>2.03</v>
+        <v>0.99</v>
       </c>
       <c r="M20" t="n">
-        <v>24.5</v>
+        <v>15.7</v>
+      </c>
+      <c r="N20" t="n">
+        <v>78.3</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -2282,33 +2284,29 @@
         </is>
       </c>
       <c r="P20" t="n">
-        <v>52</v>
+        <v>68.7</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U20" t="inlineStr">
-        <is>
-          <t>TTM Squeeze</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr"/>
       <c r="V20" t="inlineStr">
         <is>
           <t>No</t>
@@ -2318,59 +2316,59 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>ASML</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>723.11</v>
+        <v>1532.8</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>60.8</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="J21" t="n">
-        <v>71.2</v>
+        <v>61.2</v>
       </c>
       <c r="K21" t="n">
-        <v>81</v>
+        <v>10</v>
       </c>
       <c r="L21" t="n">
-        <v>0.9399999999999999</v>
+        <v>3.88</v>
       </c>
       <c r="M21" t="n">
-        <v>15.6</v>
+        <v>52.4</v>
       </c>
       <c r="N21" t="n">
-        <v>77.90000000000001</v>
+        <v>95.40000000000001</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
@@ -2378,7 +2376,7 @@
         </is>
       </c>
       <c r="P21" t="n">
-        <v>66.8</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
@@ -2387,20 +2385,24 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U21" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V21" t="inlineStr">
         <is>
           <t>No</t>
@@ -2410,15 +2412,15 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>AEP</t>
+          <t>RTX</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>136.95</v>
+        <v>176.27</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
@@ -2433,36 +2435,36 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I22" t="n">
-        <v>58.1</v>
+        <v>61.9</v>
       </c>
       <c r="J22" t="n">
-        <v>59.2</v>
+        <v>36.5</v>
       </c>
       <c r="K22" t="n">
-        <v>14</v>
+        <v>98</v>
       </c>
       <c r="L22" t="n">
-        <v>1.96</v>
+        <v>2.56</v>
       </c>
       <c r="M22" t="n">
-        <v>16</v>
+        <v>27.1</v>
       </c>
       <c r="N22" t="n">
-        <v>30.6</v>
+        <v>78.8</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
@@ -2470,33 +2472,29 @@
         </is>
       </c>
       <c r="P22" t="n">
-        <v>66.5</v>
+        <v>43.8</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U22" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr"/>
       <c r="V22" t="inlineStr">
         <is>
           <t>No</t>
@@ -2506,30 +2504,30 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>LMT</t>
+          <t>ANET</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>510.76</v>
+        <v>145.43</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2543,27 +2541,30 @@
         </is>
       </c>
       <c r="I23" t="n">
-        <v>56.1</v>
+        <v>60.2</v>
       </c>
       <c r="J23" t="n">
-        <v>24.9</v>
+        <v>40.5</v>
       </c>
       <c r="K23" t="n">
-        <v>99</v>
+        <v>82</v>
       </c>
       <c r="L23" t="n">
-        <v>2.79</v>
+        <v>6.57</v>
       </c>
       <c r="M23" t="n">
-        <v>32.2</v>
+        <v>70.59999999999999</v>
+      </c>
+      <c r="N23" t="n">
+        <v>100</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P23" t="n">
-        <v>39</v>
+        <v>52.2</v>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
@@ -2577,33 +2578,37 @@
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U23" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ANET</t>
+          <t>PEP</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>173.58</v>
+        <v>155.16</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -2618,33 +2623,33 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I24" t="n">
-        <v>55.3</v>
+        <v>60.1</v>
       </c>
       <c r="J24" t="n">
-        <v>65.8</v>
+        <v>48.1</v>
       </c>
       <c r="K24" t="n">
-        <v>84</v>
+        <v>1</v>
       </c>
       <c r="L24" t="n">
-        <v>3.77</v>
+        <v>2.05</v>
       </c>
       <c r="M24" t="n">
-        <v>63.6</v>
+        <v>24.7</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
@@ -2652,11 +2657,11 @@
         </is>
       </c>
       <c r="P24" t="n">
-        <v>67.09999999999999</v>
+        <v>52.5</v>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
@@ -2666,7 +2671,7 @@
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
@@ -2674,7 +2679,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U24" t="inlineStr"/>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
       <c r="V24" t="inlineStr">
         <is>
           <t>No</t>
@@ -2684,30 +2693,30 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>IWM</t>
+          <t>ABT</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>282.06</v>
+        <v>86.86</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -2717,31 +2726,34 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I25" t="n">
-        <v>54.6</v>
+        <v>58.4</v>
       </c>
       <c r="J25" t="n">
-        <v>68.8</v>
+        <v>24.9</v>
       </c>
       <c r="K25" t="n">
-        <v>58</v>
+        <v>87</v>
       </c>
       <c r="L25" t="n">
-        <v>1.56</v>
+        <v>2.34</v>
       </c>
       <c r="M25" t="n">
-        <v>21.5</v>
+        <v>26.6</v>
+      </c>
+      <c r="N25" t="n">
+        <v>57.2</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P25" t="n">
-        <v>69.90000000000001</v>
+        <v>19.6</v>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
@@ -2750,12 +2762,12 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
@@ -2773,30 +2785,30 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>LIN</t>
+          <t>EMR</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>500.39</v>
+        <v>146.29</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -2810,19 +2822,19 @@
         </is>
       </c>
       <c r="I26" t="n">
-        <v>52.2</v>
+        <v>57.7</v>
       </c>
       <c r="J26" t="n">
-        <v>50.7</v>
+        <v>59.6</v>
       </c>
       <c r="K26" t="n">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="L26" t="n">
-        <v>2.12</v>
+        <v>3.12</v>
       </c>
       <c r="M26" t="n">
-        <v>24</v>
+        <v>34.7</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
@@ -2830,31 +2842,31 @@
         </is>
       </c>
       <c r="P26" t="n">
-        <v>60</v>
+        <v>55.8</v>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>TTM Squeeze</t>
+          <t>Squeeze Expanding</t>
         </is>
       </c>
       <c r="V26" t="inlineStr">
@@ -2866,92 +2878,374 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>COP</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>427.64</v>
+        <v>118.78</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>57.1</v>
+      </c>
+      <c r="J27" t="n">
+        <v>43.2</v>
+      </c>
+      <c r="K27" t="n">
+        <v>14</v>
+      </c>
+      <c r="L27" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="M27" t="n">
+        <v>34.3</v>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P27" t="n">
+        <v>57.8</v>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>LMT</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>507.89</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>56.1</v>
+      </c>
+      <c r="J28" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="K28" t="n">
+        <v>97</v>
+      </c>
+      <c r="L28" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="M28" t="n">
+        <v>32.2</v>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P28" t="n">
+        <v>38.6</v>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr"/>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>LIN</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>502.27</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="E29" t="inlineStr">
         <is>
           <t>SELL</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>Credit Call</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I27" t="n">
-        <v>50.6</v>
-      </c>
-      <c r="J27" t="n">
-        <v>69.40000000000001</v>
-      </c>
-      <c r="K27" t="n">
-        <v>63</v>
-      </c>
-      <c r="L27" t="n">
-        <v>3.02</v>
-      </c>
-      <c r="M27" t="n">
-        <v>42.9</v>
-      </c>
-      <c r="N27" t="n">
-        <v>46.7</v>
-      </c>
-      <c r="O27" t="inlineStr">
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>55</v>
+      </c>
+      <c r="J29" t="n">
+        <v>52</v>
+      </c>
+      <c r="K29" t="n">
+        <v>7</v>
+      </c>
+      <c r="L29" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="M29" t="n">
+        <v>20.1</v>
+      </c>
+      <c r="N29" t="n">
+        <v>81.2</v>
+      </c>
+      <c r="O29" t="inlineStr">
         <is>
           <t>Bullish</t>
         </is>
       </c>
-      <c r="P27" t="n">
-        <v>69.40000000000001</v>
-      </c>
-      <c r="Q27" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R27" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="S27" t="inlineStr">
-        <is>
-          <t>lime</t>
-        </is>
-      </c>
-      <c r="T27" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U27" t="inlineStr"/>
-      <c r="V27" t="inlineStr">
-        <is>
-          <t>No</t>
+      <c r="P29" t="n">
+        <v>60.9</v>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>AEP</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>133.85</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Debit Call</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>49.3</v>
+      </c>
+      <c r="J30" t="n">
+        <v>49.7</v>
+      </c>
+      <c r="K30" t="n">
+        <v>17</v>
+      </c>
+      <c r="L30" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="M30" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="N30" t="n">
+        <v>43.7</v>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P30" t="n">
+        <v>61.3</v>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan 07.05.2026 16:10 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,11 +435,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V30"/>
+  <dimension ref="A1:V29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
@@ -448,7 +448,7 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="6" customWidth="1" min="10" max="10"/>
-    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="6" customWidth="1" min="11" max="11"/>
     <col width="6" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
     <col width="9" customWidth="1" min="14" max="14"/>
@@ -577,11 +577,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>INTC</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>111.15</v>
+        <v>405.78</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,22 +614,22 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>93.5</v>
+        <v>91.3</v>
       </c>
       <c r="J2" t="n">
-        <v>85.40000000000001</v>
+        <v>75.2</v>
       </c>
       <c r="K2" t="n">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="L2" t="n">
-        <v>6.19</v>
+        <v>6.18</v>
       </c>
       <c r="M2" t="n">
-        <v>99</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="N2" t="n">
-        <v>99.2</v>
+        <v>77.7</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>88.8</v>
+        <v>82.3</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -669,11 +669,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>GD</t>
+          <t>NXPI</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>345.78</v>
+        <v>294.68</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -706,22 +706,22 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>92.09999999999999</v>
+        <v>89.7</v>
       </c>
       <c r="J3" t="n">
-        <v>56.7</v>
+        <v>74.8</v>
       </c>
       <c r="K3" t="n">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="L3" t="n">
-        <v>2.65</v>
+        <v>4.37</v>
       </c>
       <c r="M3" t="n">
-        <v>31</v>
+        <v>81.5</v>
       </c>
       <c r="N3" t="n">
-        <v>99.59999999999999</v>
+        <v>100</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -729,7 +729,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>53</v>
+        <v>72.5</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -751,21 +751,25 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr"/>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>TXN</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>415.45</v>
+        <v>283.57</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -798,19 +802,22 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>90.40000000000001</v>
+        <v>84.3</v>
       </c>
       <c r="J4" t="n">
-        <v>80.59999999999999</v>
+        <v>74</v>
       </c>
       <c r="K4" t="n">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="L4" t="n">
-        <v>6.36</v>
+        <v>3.48</v>
       </c>
       <c r="M4" t="n">
-        <v>65.2</v>
+        <v>63.6</v>
+      </c>
+      <c r="N4" t="n">
+        <v>100</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -818,7 +825,7 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>82.90000000000001</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -850,11 +857,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>GFS</t>
+          <t>KDP</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>71.12</v>
+        <v>28.51</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -887,30 +894,30 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>90.3</v>
+        <v>84</v>
       </c>
       <c r="J5" t="n">
-        <v>76.59999999999999</v>
+        <v>57.7</v>
       </c>
       <c r="K5" t="n">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="L5" t="n">
-        <v>5.34</v>
+        <v>2.83</v>
       </c>
       <c r="M5" t="n">
-        <v>62.1</v>
+        <v>31.2</v>
       </c>
       <c r="N5" t="n">
-        <v>76.7</v>
+        <v>57.5</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>82</v>
+        <v>52.8</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -919,38 +926,34 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>TXN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>288.89</v>
+        <v>101.38</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -983,22 +986,22 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>86.7</v>
+        <v>81.8</v>
       </c>
       <c r="J6" t="n">
-        <v>79.90000000000001</v>
+        <v>71.3</v>
       </c>
       <c r="K6" t="n">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="L6" t="n">
-        <v>3.36</v>
+        <v>5</v>
       </c>
       <c r="M6" t="n">
-        <v>62.8</v>
+        <v>65.7</v>
       </c>
       <c r="N6" t="n">
-        <v>98.59999999999999</v>
+        <v>100</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -1006,7 +1009,7 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>79.2</v>
+        <v>77.8</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1015,17 +1018,17 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
@@ -1038,11 +1041,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>KDP</t>
+          <t>MCHP</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>28.5</v>
+        <v>100.79</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1075,30 +1078,30 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>85.2</v>
+        <v>78.5</v>
       </c>
       <c r="J7" t="n">
-        <v>57.6</v>
+        <v>77.09999999999999</v>
       </c>
       <c r="K7" t="n">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="L7" t="n">
-        <v>2.8</v>
+        <v>3.8</v>
       </c>
       <c r="M7" t="n">
-        <v>31.3</v>
+        <v>50.4</v>
       </c>
       <c r="N7" t="n">
-        <v>57.7</v>
+        <v>78.2</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>52.8</v>
+        <v>75.8</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1107,17 +1110,17 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U7" t="inlineStr"/>
@@ -1130,11 +1133,11 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>CDNS</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>103.67</v>
+        <v>358.92</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1167,19 +1170,19 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>83.59999999999999</v>
+        <v>78.2</v>
       </c>
       <c r="J8" t="n">
-        <v>80.3</v>
+        <v>71.3</v>
       </c>
       <c r="K8" t="n">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="L8" t="n">
-        <v>4.73</v>
+        <v>3.18</v>
       </c>
       <c r="M8" t="n">
-        <v>59.1</v>
+        <v>45.4</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1187,7 +1190,7 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>80.09999999999999</v>
+        <v>63.9</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1219,56 +1222,56 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>JPM</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>315.93</v>
+        <v>214.01</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>79.90000000000001</v>
+        <v>77</v>
       </c>
       <c r="J9" t="n">
-        <v>60.6</v>
+        <v>60.2</v>
       </c>
       <c r="K9" t="n">
-        <v>2</v>
+        <v>91</v>
       </c>
       <c r="L9" t="n">
-        <v>1.79</v>
+        <v>8.25</v>
       </c>
       <c r="M9" t="n">
-        <v>23.3</v>
+        <v>73</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1276,11 +1279,11 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>57.5</v>
+        <v>69.5</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -1295,76 +1298,76 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
+          <t>Divergence</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>MCHP</t>
+          <t>JPM</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>101.44</v>
+        <v>310.28</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>78.59999999999999</v>
+        <v>74.8</v>
       </c>
       <c r="J10" t="n">
-        <v>81.7</v>
+        <v>53.4</v>
       </c>
       <c r="K10" t="n">
-        <v>92</v>
+        <v>3</v>
       </c>
       <c r="L10" t="n">
-        <v>3.67</v>
+        <v>1.91</v>
       </c>
       <c r="M10" t="n">
-        <v>49.1</v>
+        <v>23.5</v>
       </c>
       <c r="N10" t="n">
-        <v>74.5</v>
+        <v>58.1</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1372,21 +1375,21 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>76.09999999999999</v>
+        <v>54.8</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -1394,21 +1397,25 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U10" t="inlineStr"/>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>XLK</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>235.23</v>
+        <v>170.18</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1441,22 +1448,22 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>78.09999999999999</v>
+        <v>71.3</v>
       </c>
       <c r="J11" t="n">
-        <v>71.40000000000001</v>
+        <v>80.90000000000001</v>
       </c>
       <c r="K11" t="n">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="L11" t="n">
-        <v>6.85</v>
+        <v>1.82</v>
       </c>
       <c r="M11" t="n">
-        <v>100.3</v>
+        <v>25.9</v>
       </c>
       <c r="N11" t="n">
-        <v>100</v>
+        <v>92.7</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1464,7 +1471,7 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>72.8</v>
+        <v>75.5</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1496,11 +1503,11 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>URI</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>91.54000000000001</v>
+        <v>954.04</v>
       </c